<commit_message>
Add batch 2: 16 new prospects (40 total)
Letting agents, wedding venues, cosmetic clinics, pilates studios,
financial advisers, tutors, osteopaths and design & build firms across
Bristol, Cotswolds and London.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T25"/>
+  <dimension ref="A1:T41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2804,8 +2804,1496 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Lets Rent Bristol</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Letting agent</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>St Werburghs, Bristol BS2</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>https://letsrentbristol.co.uk</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>info@letsrentbristol.co.uk</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>0117 254 1133</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>Adil Ayub &amp; Usman Ayub</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr"/>
+      <c r="I26" s="3" t="inlineStr"/>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>Family-run since 2009; manages HMOs/student/corporate lets across 7 postcodes - recurring management fees make each landlord worth thousands over time</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L26" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M26" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N26" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O26" s="3" t="inlineStr">
+        <is>
+          <t>ARLA Propertymark, CMP badges; portal listings</t>
+        </is>
+      </c>
+      <c r="P26" s="3" t="inlineStr">
+        <is>
+          <t>Landlord acquisition dominated by bigger agencies and online agents (OpenRent) on search</t>
+        </is>
+      </c>
+      <c r="Q26" s="3" t="inlineStr">
+        <is>
+          <t>'Landlords ask Google and ChatGPT who to trust with their Bristol BTL - own that answer'</t>
+        </is>
+      </c>
+      <c r="R26" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S26" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T26" s="3" t="inlineStr">
+        <is>
+          <t>Single office, established book - upsell landlord-focused content</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Bristol Property Centre</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Letting &amp; estate agent</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Chandos Rd, Redland, Bristol BS6</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bristolpropertycentre.co.uk</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>info@bristolpropertycentre.co.uk</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>0117 907 3577</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>Alice Willmott (Head of Property Management)</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>uk.linkedin.com/company/bristol-property-centre</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr"/>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>Award-winning independent doing sales + lettings + student + commercial; Redland/BS6 is prime landlord territory</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L27" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M27" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N27" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O27" s="3" t="inlineStr">
+        <is>
+          <t>Award mentions; LinkedIn presence</t>
+        </is>
+      </c>
+      <c r="P27" s="3" t="inlineStr">
+        <is>
+          <t>Competes with national brands and Boardwalk-style digital independents for valuations</t>
+        </is>
+      </c>
+      <c r="Q27" s="3" t="inlineStr">
+        <is>
+          <t>Local-SEO audit of 'letting agent Redland/Bishopston' - show the gap vs OpenRent and corporates</t>
+        </is>
+      </c>
+      <c r="R27" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S27" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T27" s="3" t="inlineStr">
+        <is>
+          <t>Confirm director name via Companies House (07695593) before outreach</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Caswell House</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Wedding venue</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Brize Norton, Oxfordshire (Cotswolds)</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>https://caswellhouse.co.uk</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>kirsten@caswellhouse.co.uk</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>01993 701064</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Kirsten Jones (General Manager)</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr"/>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Exclusive-use 15th-century barn venue, 140 seated/200 evening; weddings worth £15-30k each - one booking pays for years of SEO</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>Bridebook/Guides for Brides listings; professional photography</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>Couples now ask ChatGPT for 'barn wedding venues Cotswolds' shortlists - directories get cited, venues don't</t>
+        </is>
+      </c>
+      <c r="Q28" s="2" t="inlineStr">
+        <is>
+          <t>'Get on the AI shortlist: couples ask ChatGPT before they open Bridebook'</t>
+        </is>
+      </c>
+      <c r="R28" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S28" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T28" s="2" t="inlineStr">
+        <is>
+          <t>Named GM with direct email - easiest warm route in batch 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Hyde House</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Wedding venue</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Stow-on-the-Wold, Gloucestershire</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>https://hyde-house.uk</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>hello@hyde-house.uk</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>01451 830354</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr"/>
+      <c r="H29" s="3" t="inlineStr"/>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/HydeHouse (via page)</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>Exclusive-use Victorian house + barn with 20 bedrooms; premium Cotswolds weddings; relies on directory listings for discovery</t>
+        </is>
+      </c>
+      <c r="K29" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L29" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M29" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N29" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O29" s="3" t="inlineStr">
+        <is>
+          <t>Bridebook/Coco Wedding Venues listings</t>
+        </is>
+      </c>
+      <c r="P29" s="3" t="inlineStr">
+        <is>
+          <t>Heavy dependence on paid directories that take commission or fees</t>
+        </is>
+      </c>
+      <c r="Q29" s="3" t="inlineStr">
+        <is>
+          <t>Reduce directory dependence: rank + get AI-recommended directly and keep the margin</t>
+        </is>
+      </c>
+      <c r="R29" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S29" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Clifton Cosmetics</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Cosmetic clinic (injectables)</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>The Body Centre, Alma Rd, Clifton, Bristol</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>https://cliftoncosmetics.co.uk</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr"/>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>Dr James Hesford (Founder)</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr"/>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/cliftoncosmetics</t>
+        </is>
+      </c>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>Doctor-led injectables clinic in affluent Clifton; repeat-treatment clients worth £1k+/year; local trust is the whole sales pitch</t>
+        </is>
+      </c>
+      <c r="K30" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L30" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M30" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N30" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O30" s="3" t="inlineStr">
+        <is>
+          <t>Facebook page; WhatClinic listing</t>
+        </is>
+      </c>
+      <c r="P30" s="3" t="inlineStr">
+        <is>
+          <t>Nurse-led and chain clinics outrank him; no clear local SEO presence</t>
+        </is>
+      </c>
+      <c r="Q30" s="3" t="inlineStr">
+        <is>
+          <t>'Patients Google the injector before they book - make Dr Hesford the name Bristol finds first'</t>
+        </is>
+      </c>
+      <c r="R30" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S30" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T30" s="3" t="inlineStr">
+        <is>
+          <t>Doctor-led = strong E-E-A-T story for AEO content</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Zafra Medical</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Cosmetic/anti-ageing clinic</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Litfield House, Clifton Down, Bristol BS8</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>https://www.zaframedical.co.uk</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr"/>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>Dr Jorge Zafra (Medical Director &amp; Owner)</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr"/>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/zaframedical</t>
+        </is>
+      </c>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>Owner-led anti-ageing clinic in prestige Litfield House medical centre; Vaser surgeon = high-ticket procedures</t>
+        </is>
+      </c>
+      <c r="K31" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L31" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M31" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N31" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O31" s="3" t="inlineStr">
+        <is>
+          <t>ConsultingRoom profile; Fresha booking</t>
+        </is>
+      </c>
+      <c r="P31" s="3" t="inlineStr">
+        <is>
+          <t>Squarespace-style site with weak local SEO; invisible for 'botox Bristol' money terms</t>
+        </is>
+      </c>
+      <c r="Q31" s="3" t="inlineStr">
+        <is>
+          <t>Free AI-visibility check for 'best aesthetic doctor Bristol' + one-page fix plan</t>
+        </is>
+      </c>
+      <c r="R31" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S31" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Yoganand Studio</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>Yoga &amp; reformer pilates studio</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Clifton Triangle, Bristol BS8</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>https://www.yoganand.co.uk</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr"/>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>Jade (Founder)</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>uk.linkedin.com/company/yoganand-studio</t>
+        </is>
+      </c>
+      <c r="I32" s="4" t="inlineStr">
+        <is>
+          <t>instagram.com/yoganandstudio</t>
+        </is>
+      </c>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>Boutique studio in prime Clifton Triangle; memberships = recurring revenue; reformer pilates demand exploding in Bristol</t>
+        </is>
+      </c>
+      <c r="K32" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M32" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N32" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O32" s="4" t="inlineStr">
+        <is>
+          <t>Active Instagram; ClassPass listing</t>
+        </is>
+      </c>
+      <c r="P32" s="4" t="inlineStr">
+        <is>
+          <t>Discovery happens on ClassPass (commission) rather than direct search</t>
+        </is>
+      </c>
+      <c r="Q32" s="4" t="inlineStr">
+        <is>
+          <t>'Fill classes without paying ClassPass commission - own the local reformer searches'</t>
+        </is>
+      </c>
+      <c r="R32" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S32" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T32" s="4" t="inlineStr">
+        <is>
+          <t>Smaller budget - fits entry £249 tier</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>The Reformer Space</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Reformer pilates studio</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Coldharbour Rd, Westbury Park, Bristol</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>https://thereformerspace.co.uk</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>info@thereformerspace.co.uk</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr"/>
+      <c r="G33" s="3" t="inlineStr"/>
+      <c r="H33" s="3" t="inlineStr"/>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com (The reformer space page)</t>
+        </is>
+      </c>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>New (2024) dedicated reformer/tower studio in affluent Westbury Park/Redland; needs to build visibility fast to fill classes</t>
+        </is>
+      </c>
+      <c r="K33" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L33" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M33" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N33" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O33" s="3" t="inlineStr">
+        <is>
+          <t>ClassPass/Wellhub listings</t>
+        </is>
+      </c>
+      <c r="P33" s="3" t="inlineStr">
+        <is>
+          <t>Brand-new domain with no authority; rivals (Soul Pilates, M.O) have head start</t>
+        </is>
+      </c>
+      <c r="Q33" s="3" t="inlineStr">
+        <is>
+          <t>Ground-floor pitch: build search presence now while the studio is new</t>
+        </is>
+      </c>
+      <c r="R33" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S33" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T33" s="3" t="inlineStr">
+        <is>
+          <t>New business - keen but validate budget early</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Frazer James Financial Advisers</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Financial adviser / wealth management</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Berkeley Square, Bristol BS8</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>https://frazerjames.co.uk</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>james@frazerjames.co.uk</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>0117 990 2602</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>James Mackay (Founder/MD)</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>uk.linkedin.com/company/frazer-james</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr"/>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>Award-winning IFA for professionals/business owners; client lifetime value tens of thousands; founder already writes content</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L34" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M34" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N34" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O34" s="3" t="inlineStr">
+        <is>
+          <t>VouchedFor profile; content marketing on site; awards</t>
+        </is>
+      </c>
+      <c r="P34" s="3" t="inlineStr">
+        <is>
+          <t>Content ranks for some terms but AI engines cite unbiased-looking directories instead of his articles</t>
+        </is>
+      </c>
+      <c r="Q34" s="3" t="inlineStr">
+        <is>
+          <t>'Your guides rank on Google - here's how to make ChatGPT cite them too'</t>
+        </is>
+      </c>
+      <c r="R34" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S34" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T34" s="3" t="inlineStr">
+        <is>
+          <t>Direct founder email; marketing-literate buyer</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Ifamax Wealth Management</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Wealth management</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Bristol (clients Bristol/Bath/London)</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ifamax.com</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>0117 332 2626</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>Max Tennant</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>uk.linkedin.com/company/ifamax-limited</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="inlineStr"/>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>Boutique firm targeting £400k+ investors; ultra-high client value; already runs keyword landing pages so believes in search</t>
+        </is>
+      </c>
+      <c r="K35" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M35" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N35" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O35" s="4" t="inlineStr">
+        <is>
+          <t>Multiple SEO landing pages (wealth management Bristol etc.) - active investment</t>
+        </is>
+      </c>
+      <c r="P35" s="4" t="inlineStr">
+        <is>
+          <t>Paying for SEO already; AEO/GEO layer missing; high-net-worth clients increasingly use AI research</t>
+        </is>
+      </c>
+      <c r="Q35" s="4" t="inlineStr">
+        <is>
+          <t>Agency-upgrade pitch: add AI-search visibility to an already-working SEO base</t>
+        </is>
+      </c>
+      <c r="R35" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S35" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T35" s="4" t="inlineStr">
+        <is>
+          <t>Likely has an agency - displacement/upsell only</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Kensington &amp; Chelsea Tutors</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Private tuition agency</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>Queens Gate Terrace, London SW7</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>https://www.kctutors.co.uk</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>learn@kctutors.co.uk</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>020 7584 7987</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>Nevil Chiles (MD &amp; Co-founder)</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr"/>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/KensingtonandChelseaTutors</t>
+        </is>
+      </c>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>Established 2002, serves ultra-wealthy SW London families; a single family client can be worth £10k+/year in tuition</t>
+        </is>
+      </c>
+      <c r="K36" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L36" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M36" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N36" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O36" s="3" t="inlineStr">
+        <is>
+          <t>Long-standing directory presence; celebrity client name-drops</t>
+        </is>
+      </c>
+      <c r="P36" s="3" t="inlineStr">
+        <is>
+          <t>Newer polished agencies (Keystone, Ivy) dominate search and AI recommendations</t>
+        </is>
+      </c>
+      <c r="Q36" s="3" t="inlineStr">
+        <is>
+          <t>'When parents ask ChatGPT for a Kensington tutor agency, Keystone comes up - not you'</t>
+        </is>
+      </c>
+      <c r="R36" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S36" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T36" s="3" t="inlineStr">
+        <is>
+          <t>Enquiries filter directly to MD Nevil - fast decision loop</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Ivy Education</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Private tuition &amp; education consultancy</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>London (Fulham office)</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ivyeducation.co.uk</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>020 7736 6977</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>Alastair Delafield (Founder &amp; CEO)</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>uk.linkedin.com/company/ivy-education</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr"/>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>Premium consultancy (tuition + school placement); wealthy international families; high fees per engagement</t>
+        </is>
+      </c>
+      <c r="K37" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L37" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M37" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N37" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O37" s="3" t="inlineStr">
+        <is>
+          <t>Award mentions; polished site; likely some agency spend</t>
+        </is>
+      </c>
+      <c r="P37" s="3" t="inlineStr">
+        <is>
+          <t>11+/school-admissions searches increasingly answered by AI Overviews citing content-rich competitors</t>
+        </is>
+      </c>
+      <c r="Q37" s="3" t="inlineStr">
+        <is>
+          <t>AEO content play: own the questions parents ask AI about London school entry</t>
+        </is>
+      </c>
+      <c r="R37" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S37" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Wimbledon Osteopathic Clinic</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>Osteopath</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Wimbledon/Raynes Park, London</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wimbledonosteopaths.co.uk</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>020 8946 6103</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>David Rowland (Principal)</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="inlineStr"/>
+      <c r="I38" s="4" t="inlineStr"/>
+      <c r="J38" s="4" t="inlineStr">
+        <is>
+          <t>39 years established in affluent Wimbledon; self-pay treatments with long courses; loyal base but ageing digital presence</t>
+        </is>
+      </c>
+      <c r="K38" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L38" s="4" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="M38" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N38" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O38" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P38" s="4" t="inlineStr">
+        <is>
+          <t>Dated website; younger clinics and physio chains capture all new-patient searches</t>
+        </is>
+      </c>
+      <c r="Q38" s="4" t="inlineStr">
+        <is>
+          <t>'Your reputation is 39 years strong - your Google presence isn't. Fix it for £249/month'</t>
+        </is>
+      </c>
+      <c r="R38" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S38" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T38" s="4" t="inlineStr">
+        <is>
+          <t>Classic modernisation candidate; confirm appetite to grow</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>West Dulwich Osteopaths</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>Osteopathy clinic</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>Park Hall Rd, West Dulwich, London SE21</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>https://westdulwichosteopaths.com</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>westdulwichosteopaths@gmail.com</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>07779 262055</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>Hollie Carter (Principal)</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr"/>
+      <c r="I39" s="4" t="inlineStr"/>
+      <c r="J39" s="4" t="inlineStr">
+        <is>
+          <t>7-practitioner clinic in affluent Dulwich Village catchment; still using a Gmail address and a legacy Weebly site - huge digital gap</t>
+        </is>
+      </c>
+      <c r="K39" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L39" s="4" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="M39" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N39" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O39" s="4" t="inlineStr">
+        <is>
+          <t>None - organic/word-of-mouth only</t>
+        </is>
+      </c>
+      <c r="P39" s="4" t="inlineStr">
+        <is>
+          <t>Multi-practitioner payroll but almost zero search visibility; losing new patients to marketed rivals</t>
+        </is>
+      </c>
+      <c r="Q39" s="4" t="inlineStr">
+        <is>
+          <t>'A 7-practitioner clinic running on word-of-mouth: here's what you're leaving on the table'</t>
+        </is>
+      </c>
+      <c r="R39" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S39" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T39" s="4" t="inlineStr">
+        <is>
+          <t>Gmail contact = no marketing infrastructure at all</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Excellence Living</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>Design &amp; build / home renovation</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Cheddar/Bristol &amp; North Somerset</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>https://excellenceliving.co.uk</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>hello@excellenceliving.co.uk</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>0117 212 0130</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Paul (Founder, 30+ yrs experience)</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/ExcellenceLivingLtd</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>Extensions/lofts/renovations worth £50-200k per job; already builds location landing pages (Bristol, Clevedon) so search-aware</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>Location landing pages; Facebook presence</t>
+        </is>
+      </c>
+      <c r="P40" s="2" t="inlineStr">
+        <is>
+          <t>Location pages exist but thin; AI engines recommend FMB directory results instead of firms</t>
+        </is>
+      </c>
+      <c r="Q40" s="2" t="inlineStr">
+        <is>
+          <t>'One extension job pays for 20 years of our fee - and your Clevedon page isn't even ranking'</t>
+        </is>
+      </c>
+      <c r="R40" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S40" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T40" s="2" t="inlineStr">
+        <is>
+          <t>High ticket + existing SEO intent = prime £249+ upsell</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Hallett Construction</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Builders / building contractor</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Hanham, Bristol BS15</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>https://hallettconstruction.co.uk</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>info@hallettconstruction.co.uk</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>0117 251 0179</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>Jason Hallett (Director)</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr"/>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/hallettconstruction.co.uk</t>
+        </is>
+      </c>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>FMB-member design &amp; build firm doing extensions with in-house planning service; already publishing postcode landing pages (BS40 etc.)</t>
+        </is>
+      </c>
+      <c r="K41" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L41" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M41" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N41" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O41" s="3" t="inlineStr">
+        <is>
+          <t>FMB membership; postcode landing pages = DIY SEO effort</t>
+        </is>
+      </c>
+      <c r="P41" s="3" t="inlineStr">
+        <is>
+          <t>DIY postcode pages show intent but lack authority to rank; no AEO strategy</t>
+        </is>
+      </c>
+      <c r="Q41" s="3" t="inlineStr">
+        <is>
+          <t>'You're already building postcode pages - let us make them actually rank and get cited by AI'</t>
+        </is>
+      </c>
+      <c r="R41" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S41" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T41" s="3" t="inlineStr">
+        <is>
+          <t>Owner-led; DIY SEO effort = proven willingness to invest</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T25"/>
+  <autoFilter ref="A1:T41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2816,7 +4304,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:B39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2836,7 +4324,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>24</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5">
@@ -2889,17 +4377,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Dentist / Orthodontics</t>
+          <t>Wedding venue</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Private dentist</t>
+          <t>Dentist / Orthodontics</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -2909,7 +4397,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Specialist dental/implant clinic</t>
+          <t>Private dentist</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -2919,7 +4407,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Law firm</t>
+          <t>Specialist dental/implant clinic</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -2929,7 +4417,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Boutique corporate law firm</t>
+          <t>Law firm</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -2939,7 +4427,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Cosmetic/aesthetics clinic</t>
+          <t>Boutique corporate law firm</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -2949,7 +4437,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Skin &amp; laser clinic</t>
+          <t>Cosmetic/aesthetics clinic</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -2959,7 +4447,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Mortgage broker</t>
+          <t>Skin &amp; laser clinic</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -2969,7 +4457,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Mortgage broker / financial adviser</t>
+          <t>Mortgage broker</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -2979,7 +4467,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Architects (RIBA chartered)</t>
+          <t>Mortgage broker / financial adviser</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -2989,7 +4477,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Recruitment agency (tech/startups)</t>
+          <t>Architects (RIBA chartered)</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -2999,7 +4487,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Recruitment agency (IT/data)</t>
+          <t>Recruitment agency (tech/startups)</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -3009,7 +4497,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Independent vet</t>
+          <t>Recruitment agency (IT/data)</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -3019,7 +4507,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Independent vet (24/7 emergency)</t>
+          <t>Independent vet</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -3029,10 +4517,160 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>Independent vet (24/7 emergency)</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>Interior design studio</t>
         </is>
       </c>
-      <c r="B24" t="n">
+      <c r="B25" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Letting agent</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Letting &amp; estate agent</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Cosmetic clinic (injectables)</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Cosmetic/anti-ageing clinic</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Yoga &amp; reformer pilates studio</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Reformer pilates studio</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Financial adviser / wealth management</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Wealth management</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Private tuition agency</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Private tuition &amp; education consultancy</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Osteopath</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Osteopathy clinic</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Design &amp; build / home renovation</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Builders / building contractor</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 3a: +15 prospects (55 total) - GPs, trades, caterers, care, nurseries, PT studios
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$56</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T41"/>
+  <dimension ref="A1:T56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -4292,8 +4292,1308 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Beard Medical Practice</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Private GP</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Litfield House, Clifton, Bristol BS8</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.beardmedical.com</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>0117 973 1323</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Dr John Beard &amp; Dr Henry Beard (Founders)</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr"/>
+      <c r="I42" s="2" t="inlineStr"/>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>Family-run private GP practice in Clifton; consultations + repeat memberships; self-pay healthcare demand booming as NHS waits grow</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>Established listing presence; little visible content marketing</t>
+        </is>
+      </c>
+      <c r="P42" s="2" t="inlineStr">
+        <is>
+          <t>Chains (Nuffield, HCA) and online GPs (DocTap) dominate 'private GP Bristol' searches</t>
+        </is>
+      </c>
+      <c r="Q42" s="2" t="inlineStr">
+        <is>
+          <t>'NHS waits are sending patients to Google - make sure Bristol finds the Beards first'</t>
+        </is>
+      </c>
+      <c r="R42" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S42" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T42" s="2" t="inlineStr">
+        <is>
+          <t>Family name practice = strong trust story for AEO content</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Broadgate GP</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Private GP</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>65 London Wall, City of London EC2</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>https://www.broadgategp.co.uk</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>doctor@broadgategp.co.uk</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>020 7638 4330</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr"/>
+      <c r="H43" s="3" t="inlineStr"/>
+      <c r="I43" s="3" t="inlineStr"/>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>Independent same-day private GP in the City since 2009; corporate workers self-pay £100+ per visit; high repeat and corporate-account value</t>
+        </is>
+      </c>
+      <c r="K43" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L43" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M43" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N43" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O43" s="3" t="inlineStr">
+        <is>
+          <t>Twitter/X presence; Doctify profile</t>
+        </is>
+      </c>
+      <c r="P43" s="3" t="inlineStr">
+        <is>
+          <t>DocTap's 11 clinics and hospital brands outrank a single-site independent</t>
+        </is>
+      </c>
+      <c r="Q43" s="3" t="inlineStr">
+        <is>
+          <t>'City workers ask ChatGPT where to get a same-day GP near Liverpool St - we checked who it names'</t>
+        </is>
+      </c>
+      <c r="R43" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S43" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Mayfield Clinic</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>Private GP</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Redland, Bristol (+ Oxford HQ)</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>https://www.mayfieldclinic.co.uk</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr"/>
+      <c r="G44" s="4" t="inlineStr"/>
+      <c r="H44" s="4" t="inlineStr"/>
+      <c r="I44" s="4" t="inlineStr"/>
+      <c r="J44" s="4" t="inlineStr">
+        <is>
+          <t>Growing private GP group already building 'nearby location' SEO pages (Keynsham, Bradley Stoke); blog answering patient questions = AEO-ready mindset</t>
+        </is>
+      </c>
+      <c r="K44" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L44" s="4" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M44" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N44" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O44" s="4" t="inlineStr">
+        <is>
+          <t>Location pages + patient-question blog posts = active SEO strategy</t>
+        </is>
+      </c>
+      <c r="P44" s="4" t="inlineStr">
+        <is>
+          <t>Content exists but thin authority; not cited by AI engines for Bristol private GP queries</t>
+        </is>
+      </c>
+      <c r="Q44" s="4" t="inlineStr">
+        <is>
+          <t>Upgrade pitch: turn their existing location/blog strategy into AI citations</t>
+        </is>
+      </c>
+      <c r="R44" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S44" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T44" s="4" t="inlineStr">
+        <is>
+          <t>May have in-house/agency SEO - qualify first</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>Nicola Roofing Ltd</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Roofer</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>Longwell Green, Bristol</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>https://www.nicolaroofing.co.uk</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>info@nicolaroofing.co.uk</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>0117 985 9882</t>
+        </is>
+      </c>
+      <c r="G45" s="3" t="inlineStr"/>
+      <c r="H45" s="3" t="inlineStr"/>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/Nicola-Roofing-Limited</t>
+        </is>
+      </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>30+ years established, covers Bristol &amp; Bath; re-roofs worth £5-15k; glowing reviews but weak digital presence</t>
+        </is>
+      </c>
+      <c r="K45" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L45" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M45" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N45" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O45" s="3" t="inlineStr">
+        <is>
+          <t>Yell/TrustATrader listings</t>
+        </is>
+      </c>
+      <c r="P45" s="3" t="inlineStr">
+        <is>
+          <t>Lead-gen platforms (Bark, TrustATrader) charge per lead for searches they could own</t>
+        </is>
+      </c>
+      <c r="Q45" s="3" t="inlineStr">
+        <is>
+          <t>'30 years of great roofs, invisible on Google - own "roofer Bristol" instead of renting it from Bark'</t>
+        </is>
+      </c>
+      <c r="R45" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S45" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T45" s="3" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>Westex Heating</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Plumbing &amp; heating / boilers</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>Queen Square, Bath</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>https://westexheating.co.uk</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>services@westexheating.com</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>01225 331 091</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr"/>
+      <c r="H46" s="3" t="inlineStr"/>
+      <c r="I46" s="3" t="inlineStr"/>
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>Bath-based Gas Safe firm; boiler installs £2.5-5k plus recurring service plans; affluent Bath housing stock</t>
+        </is>
+      </c>
+      <c r="K46" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L46" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M46" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N46" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O46" s="3" t="inlineStr">
+        <is>
+          <t>None visible beyond directories</t>
+        </is>
+      </c>
+      <c r="P46" s="3" t="inlineStr">
+        <is>
+          <t>British Gas and national installers (BOXT, Heatable) take the high-intent boiler searches</t>
+        </is>
+      </c>
+      <c r="Q46" s="3" t="inlineStr">
+        <is>
+          <t>'When a Bath boiler dies, the owner Googles once. Here's how to be the answer'</t>
+        </is>
+      </c>
+      <c r="R46" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S46" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T46" s="3" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Bristol Boiler Company</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing &amp; heating / boilers</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>Bristol</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>https://bristolboiler.co.uk</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>0117 939 6202</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr"/>
+      <c r="H47" s="4" t="inlineStr"/>
+      <c r="I47" s="4" t="inlineStr"/>
+      <c r="J47" s="4" t="inlineStr">
+        <is>
+          <t>Boiler installs + landlord gas certificates = recurring B2B revenue from letting agents/landlords; emergency repairs are high-intent searches</t>
+        </is>
+      </c>
+      <c r="K47" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L47" s="4" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="M47" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N47" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O47" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P47" s="4" t="inlineStr">
+        <is>
+          <t>Dated site losing emergency and landlord work to slicker rivals</t>
+        </is>
+      </c>
+      <c r="Q47" s="4" t="inlineStr">
+        <is>
+          <t>Quick-win pitch: emergency + landlord-certificate keywords they could own in months</t>
+        </is>
+      </c>
+      <c r="R47" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S47" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T47" s="4" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>Rygol Electrical</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Electrician</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Bristol</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>https://rygol.co.uk</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>0117 313 7644</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr"/>
+      <c r="H48" s="3" t="inlineStr"/>
+      <c r="I48" s="3" t="inlineStr"/>
+      <c r="J48" s="3" t="inlineStr">
+        <is>
+          <t>NICEIC contractor 20+ years; rewires worth £4-8k; also runs solar arm (solar.rygol.co.uk) - two service lines to market</t>
+        </is>
+      </c>
+      <c r="K48" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L48" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M48" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N48" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O48" s="3" t="inlineStr">
+        <is>
+          <t>Keyword landing pages (house rewiring Bristol) - some SEO effort</t>
+        </is>
+      </c>
+      <c r="P48" s="3" t="inlineStr">
+        <is>
+          <t>Split web presence (rygol.co.uk + solar subdomain) dilutes authority</t>
+        </is>
+      </c>
+      <c r="Q48" s="3" t="inlineStr">
+        <is>
+          <t>Consolidation + AEO pitch across both electrical and solar arms</t>
+        </is>
+      </c>
+      <c r="R48" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S48" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T48" s="3" t="inlineStr">
+        <is>
+          <t>One relationship, two revenue lines (electrical + solar)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>MJP Electrical Services</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Electrician</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Warmley, Bristol (covers Bath, S Wales, Glos, Swindon)</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mjpelectrical.com</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>info@mjpelectrical.com</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>0117 450 0124</t>
+        </is>
+      </c>
+      <c r="G49" s="3" t="inlineStr">
+        <is>
+          <t>Mark Parry (Founder/Director)</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr"/>
+      <c r="I49" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/MJPELECTRICALSW</t>
+        </is>
+      </c>
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>Family firm, 4.9-star rated, multi-region coverage; domestic + commercial; founder ex-British Gas senior engineer</t>
+        </is>
+      </c>
+      <c r="K49" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L49" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M49" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N49" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O49" s="3" t="inlineStr">
+        <is>
+          <t>Multiple regional Facebook pages; separate Bath site</t>
+        </is>
+      </c>
+      <c r="P49" s="3" t="inlineStr">
+        <is>
+          <t>Regional microsites (mjpelectricalbath.com) split domain authority - classic old-SEO setup</t>
+        </is>
+      </c>
+      <c r="Q49" s="3" t="inlineStr">
+        <is>
+          <t>'Your Bath site and main site are competing with each other on Google - here's the fix'</t>
+        </is>
+      </c>
+      <c r="R49" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S49" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T49" s="3" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Social Pantry</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Event &amp; wedding caterer</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>Battersea, London</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>https://socialpantry.co.uk</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr"/>
+      <c r="G50" s="4" t="inlineStr">
+        <is>
+          <t>Alex Head (Founder &amp; Owner)</t>
+        </is>
+      </c>
+      <c r="H50" s="4" t="inlineStr">
+        <is>
+          <t>uk.linkedin.com/in/alex-head-49744865</t>
+        </is>
+      </c>
+      <c r="I50" s="4" t="inlineStr"/>
+      <c r="J50" s="4" t="inlineStr">
+        <is>
+          <t>High-profile B Corp caterer; weddings/corporate events worth £5-50k; founder has strong press profile ripe for AEO citation leverage</t>
+        </is>
+      </c>
+      <c r="K50" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L50" s="4" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M50" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N50" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O50" s="4" t="inlineStr">
+        <is>
+          <t>PR agency coverage (Sainsbury's Mag, podcasts); £1.1M investment 2023</t>
+        </is>
+      </c>
+      <c r="P50" s="4" t="inlineStr">
+        <is>
+          <t>Press profile doesn't convert to AI-answer visibility for 'wedding caterer London' queries</t>
+        </is>
+      </c>
+      <c r="Q50" s="4" t="inlineStr">
+        <is>
+          <t>Turn press authority into AI citations; compete on answers not just aesthetics</t>
+        </is>
+      </c>
+      <c r="R50" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S50" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T50" s="4" t="inlineStr">
+        <is>
+          <t>Well-funded - bigger budget but may have agency already</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Kitchen Party</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>Event &amp; wedding caterer</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>Deptford, SE London</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>https://kitchen-party.co.uk</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr"/>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>Clem &amp; Joss (Co-founders, sisters)</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="inlineStr"/>
+      <c r="I51" s="4" t="inlineStr"/>
+      <c r="J51" s="4" t="inlineStr">
+        <is>
+          <t>Farm-to-fork caterer since 2015; weddings and corporate events; recommended-supplier listings at venues = referral-dependent</t>
+        </is>
+      </c>
+      <c r="K51" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L51" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M51" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N51" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O51" s="4" t="inlineStr">
+        <is>
+          <t>Venue recommended-supplier listings (Asylum Chapel)</t>
+        </is>
+      </c>
+      <c r="P51" s="4" t="inlineStr">
+        <is>
+          <t>Dependent on venue lists and word-of-mouth; near-zero search presence</t>
+        </is>
+      </c>
+      <c r="Q51" s="4" t="inlineStr">
+        <is>
+          <t>'Couples shortlist caterers on ChatGPT now - venue lists alone won't fill your calendar'</t>
+        </is>
+      </c>
+      <c r="R51" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S51" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T51" s="4" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>Featherbed Home Care</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Home care / live-in care</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>Keynsham, Bristol &amp; Bath</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>https://featherbedhomecare.co.uk</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>featherbedcare@gmail.com</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>0117 986 1948</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>Sally Carpenter (Manager)</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr"/>
+      <c r="I52" s="3" t="inlineStr"/>
+      <c r="J52" s="3" t="inlineStr">
+        <is>
+          <t>Family-owned since 1986; live-in care clients worth £50k+/year each; competes with nationals for the same searches</t>
+        </is>
+      </c>
+      <c r="K52" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L52" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M52" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N52" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O52" s="3" t="inlineStr">
+        <is>
+          <t>None - Gmail contact address signals zero marketing infrastructure</t>
+        </is>
+      </c>
+      <c r="P52" s="3" t="inlineStr">
+        <is>
+          <t>Agincare/Bluebird/Helping Hands dominate every care search; families ask AI who to trust</t>
+        </is>
+      </c>
+      <c r="Q52" s="3" t="inlineStr">
+        <is>
+          <t>'One live-in care client is worth £50k/year. Your Gmail address is costing you several'</t>
+        </is>
+      </c>
+      <c r="R52" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S52" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T52" s="3" t="inlineStr">
+        <is>
+          <t>Gmail tell again - same wedge as West Dulwich Osteopaths</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>Snapdragons Nurseries</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Private day nurseries</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>Redland/Horfield/Shirehampton Bristol + Bath &amp; Wiltshire</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>https://www.snapdragonsnursery.com</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>redland@snapdragonsnursery.com</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>0117 907 4032</t>
+        </is>
+      </c>
+      <c r="G53" s="3" t="inlineStr">
+        <is>
+          <t>Rosemary &amp; Paul Collard (Founders)</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>uk.linkedin.com/company/snapdragons-nurseries-limited</t>
+        </is>
+      </c>
+      <c r="I53" s="3" t="inlineStr"/>
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>Independent group since 1998 with Outstanding-rated settings; a nursery place is worth £12-15k/year and parents research obsessively</t>
+        </is>
+      </c>
+      <c r="K53" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L53" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M53" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N53" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O53" s="3" t="inlineStr">
+        <is>
+          <t>Established brand; council directory listings</t>
+        </is>
+      </c>
+      <c r="P53" s="3" t="inlineStr">
+        <is>
+          <t>Parents now ask ChatGPT 'best nursery near Redland' - chains (Kids Planet, Busy Bees) invest heavily in search</t>
+        </is>
+      </c>
+      <c r="Q53" s="3" t="inlineStr">
+        <is>
+          <t>'Your Outstanding rating should be the first thing AI tells parents - right now it isn't'</t>
+        </is>
+      </c>
+      <c r="R53" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S53" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T53" s="3" t="inlineStr">
+        <is>
+          <t>Multi-site independent = ideal mid-market client</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>Terra Hale</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Personal training studio</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>Chelsea &amp; Notting Hill, London</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>https://terrahale.com</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr"/>
+      <c r="G54" s="3" t="inlineStr"/>
+      <c r="H54" s="3" t="inlineStr"/>
+      <c r="I54" s="3" t="inlineStr"/>
+      <c r="J54" s="3" t="inlineStr">
+        <is>
+          <t>Private 1:1 longevity/PT studios in prime West London; clients pay £70-120/session on ongoing packages; 'longevity' positioning is search-trend gold</t>
+        </is>
+      </c>
+      <c r="K54" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L54" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M54" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N54" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O54" s="3" t="inlineStr">
+        <is>
+          <t>Location landing pages (personal training in Chelsea) - SEO aware</t>
+        </is>
+      </c>
+      <c r="P54" s="3" t="inlineStr">
+        <is>
+          <t>Longevity-fitness searches exploding; bigger brands (KX, Third Space) absorb the demand</t>
+        </is>
+      </c>
+      <c r="Q54" s="3" t="inlineStr">
+        <is>
+          <t>Own the emerging 'longevity training London' AI answers before the big clubs do</t>
+        </is>
+      </c>
+      <c r="R54" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S54" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T54" s="3" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>The Kensington Studio</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>Personal training studio</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>Kensington, London</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>https://thekensingtonstudio.com</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr"/>
+      <c r="G55" s="4" t="inlineStr"/>
+      <c r="H55" s="4" t="inlineStr"/>
+      <c r="I55" s="4" t="inlineStr"/>
+      <c r="J55" s="4" t="inlineStr">
+        <is>
+          <t>Exclusive private PT studio in ultra-affluent Kensington; high-ticket ongoing client relationships</t>
+        </is>
+      </c>
+      <c r="K55" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L55" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M55" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N55" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O55" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P55" s="4" t="inlineStr">
+        <is>
+          <t>Boutique studio invisible next to KX and Harbour Club in local searches</t>
+        </is>
+      </c>
+      <c r="Q55" s="4" t="inlineStr">
+        <is>
+          <t>Boutique-vs-big-club angle: be the AI answer for 'private personal trainer Kensington'</t>
+        </is>
+      </c>
+      <c r="R55" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S55" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T55" s="4" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>nmotion London</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>Personal training &amp; wellness studio</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>Chelsea, London</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>https://www.nmotionlondon.com</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr"/>
+      <c r="G56" s="4" t="inlineStr"/>
+      <c r="H56" s="4" t="inlineStr"/>
+      <c r="I56" s="4" t="inlineStr"/>
+      <c r="J56" s="4" t="inlineStr">
+        <is>
+          <t>Private fitness/wellbeing studio for professionals in Chelsea; tailored packages = high client lifetime value</t>
+        </is>
+      </c>
+      <c r="K56" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L56" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M56" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N56" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O56" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P56" s="4" t="inlineStr">
+        <is>
+          <t>Small brand fighting for visibility in London's most competitive fitness postcode</t>
+        </is>
+      </c>
+      <c r="Q56" s="4" t="inlineStr">
+        <is>
+          <t>Entry-tier pitch: £249/mo to start appearing in local + AI search results</t>
+        </is>
+      </c>
+      <c r="R56" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S56" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T56" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T41"/>
+  <autoFilter ref="A1:T56"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4304,7 +5604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B39"/>
+  <dimension ref="A1:B48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -4324,7 +5624,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>40</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5">
@@ -4347,17 +5647,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Physiotherapy clinic</t>
+          <t>Private GP</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Solar installer</t>
+          <t>Physiotherapy clinic</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -4367,7 +5667,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Chartered accountants</t>
+          <t>Solar installer</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -4377,7 +5677,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Wedding venue</t>
+          <t>Chartered accountants</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -4387,57 +5687,57 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Dentist / Orthodontics</t>
+          <t>Wedding venue</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Private dentist</t>
+          <t>Plumbing &amp; heating / boilers</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Specialist dental/implant clinic</t>
+          <t>Electrician</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Law firm</t>
+          <t>Event &amp; wedding caterer</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Boutique corporate law firm</t>
+          <t>Personal training studio</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Cosmetic/aesthetics clinic</t>
+          <t>Dentist / Orthodontics</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -4447,7 +5747,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Skin &amp; laser clinic</t>
+          <t>Private dentist</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -4457,7 +5757,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Mortgage broker</t>
+          <t>Specialist dental/implant clinic</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -4467,7 +5767,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Mortgage broker / financial adviser</t>
+          <t>Law firm</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -4477,7 +5777,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Architects (RIBA chartered)</t>
+          <t>Boutique corporate law firm</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -4487,7 +5787,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Recruitment agency (tech/startups)</t>
+          <t>Cosmetic/aesthetics clinic</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -4497,7 +5797,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Recruitment agency (IT/data)</t>
+          <t>Skin &amp; laser clinic</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -4507,7 +5807,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Independent vet</t>
+          <t>Mortgage broker</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -4517,7 +5817,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Independent vet (24/7 emergency)</t>
+          <t>Mortgage broker / financial adviser</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -4527,7 +5827,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Interior design studio</t>
+          <t>Architects (RIBA chartered)</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -4537,7 +5837,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Letting agent</t>
+          <t>Recruitment agency (tech/startups)</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -4547,7 +5847,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Letting &amp; estate agent</t>
+          <t>Recruitment agency (IT/data)</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -4557,7 +5857,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Cosmetic clinic (injectables)</t>
+          <t>Independent vet</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -4567,7 +5867,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Cosmetic/anti-ageing clinic</t>
+          <t>Independent vet (24/7 emergency)</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -4577,7 +5877,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Yoga &amp; reformer pilates studio</t>
+          <t>Interior design studio</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -4587,7 +5887,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Reformer pilates studio</t>
+          <t>Letting agent</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -4597,7 +5897,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Financial adviser / wealth management</t>
+          <t>Letting &amp; estate agent</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -4607,7 +5907,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Wealth management</t>
+          <t>Cosmetic clinic (injectables)</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -4617,7 +5917,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Private tuition agency</t>
+          <t>Cosmetic/anti-ageing clinic</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -4627,7 +5927,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Private tuition &amp; education consultancy</t>
+          <t>Yoga &amp; reformer pilates studio</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -4637,7 +5937,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Osteopath</t>
+          <t>Reformer pilates studio</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -4647,7 +5947,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Osteopathy clinic</t>
+          <t>Financial adviser / wealth management</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -4657,7 +5957,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Design &amp; build / home renovation</t>
+          <t>Wealth management</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -4667,10 +5967,100 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>Private tuition agency</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Private tuition &amp; education consultancy</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Osteopath</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Osteopathy clinic</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Design &amp; build / home renovation</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
           <t>Builders / building contractor</t>
         </is>
       </c>
-      <c r="B39" t="n">
+      <c r="B44" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Roofer</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Home care / live-in care</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Private day nurseries</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Personal training &amp; wellness studio</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 3b: +14 prospects (69 total) - family law, dentists, chiros, brokers, vets, consultants
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$70</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T56"/>
+  <dimension ref="A1:T70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -5592,8 +5592,1212 @@
       </c>
       <c r="T56" s="4" t="inlineStr"/>
     </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>Edwards Family Law</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Family law firm</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>Southampton Buildings, London WC2</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>https://www.edwardsfamilylaw.co.uk</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>contact@edwardsfamilylaw.co.uk</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>020 3983 1818</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="inlineStr">
+        <is>
+          <t>Kelly Edwards (Managing Partner)</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr"/>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/EdwardsFamilyLawLondon</t>
+        </is>
+      </c>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>Boutique divorce firm handling complex/high-net-worth cases worth £20k+ in fees each; Chambers-ranked but digitally quiet</t>
+        </is>
+      </c>
+      <c r="K57" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L57" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M57" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N57" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O57" s="3" t="inlineStr">
+        <is>
+          <t>Chambers UK profile; directory listings</t>
+        </is>
+      </c>
+      <c r="P57" s="3" t="inlineStr">
+        <is>
+          <t>HNW divorce clients research discreetly via search/AI - big firms and content-rich rivals get found first</t>
+        </is>
+      </c>
+      <c r="Q57" s="3" t="inlineStr">
+        <is>
+          <t>'People research divorce lawyers before telling anyone. Be the name Google and ChatGPT give them'</t>
+        </is>
+      </c>
+      <c r="R57" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S57" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T57" s="3" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>Peters May</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>Family law firm</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>Brook Street, Mayfair, London W1</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>https://www.petersmay.com</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>enquiries@petersmay.com</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>020 3036 0058</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>Juliette Peters &amp; Jessica May (Founders)</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr"/>
+      <c r="I58" s="3" t="inlineStr"/>
+      <c r="J58" s="3" t="inlineStr">
+        <is>
+          <t>Mayfair divorce boutique; ultra-high-value cases; two-founder firm with fast decision making</t>
+        </is>
+      </c>
+      <c r="K58" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L58" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M58" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N58" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O58" s="3" t="inlineStr">
+        <is>
+          <t>Chambers profile</t>
+        </is>
+      </c>
+      <c r="P58" s="3" t="inlineStr">
+        <is>
+          <t>Mayfair positioning but thin content vs Vardags/Stewarts who dominate HNW divorce searches</t>
+        </is>
+      </c>
+      <c r="Q58" s="3" t="inlineStr">
+        <is>
+          <t>AEO for the questions HNW spouses actually ask AI about UK divorce</t>
+        </is>
+      </c>
+      <c r="R58" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S58" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T58" s="3" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>Pickwick Estates</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>Dulwich Village &amp; Honor Oak, London SE22</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>https://www.pickwickestates.co.uk</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>adam.shea@pickwickestates.com</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr"/>
+      <c r="G59" s="3" t="inlineStr">
+        <is>
+          <t>Adam Shea (Director)</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="inlineStr"/>
+      <c r="I59" s="3" t="inlineStr"/>
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>Independent since 2002 in affluent Dulwich; premium family homes = high fees; dated .aspx website vs polished corporate rivals</t>
+        </is>
+      </c>
+      <c r="K59" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L59" s="3" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="M59" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N59" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O59" s="3" t="inlineStr">
+        <is>
+          <t>Portal listings only</t>
+        </is>
+      </c>
+      <c r="P59" s="3" t="inlineStr">
+        <is>
+          <t>Knight Frank/Foxtons/Pedder dominate Dulwich searches; dated site erodes valuation-lead credibility</t>
+        </is>
+      </c>
+      <c r="Q59" s="3" t="inlineStr">
+        <is>
+          <t>'Dulwich sellers shortlist agents online before calling - your website is costing you instructions'</t>
+        </is>
+      </c>
+      <c r="R59" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S59" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T59" s="3" t="inlineStr">
+        <is>
+          <t>Legacy .aspx site = instant credibility for a modernisation pitch</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Fulham Road Dental</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Private dentist</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>725 Fulham Rd, London SW6</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fulhamroaddental.com</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>enquiries@fulhamroaddental.com</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>020 4542 5555</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Dr George Cheetham</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr"/>
+      <c r="I60" s="2" t="inlineStr"/>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>Modern private practice selling implants + Invisalign in affluent SW6; every implant case £3k+; surrounded by chains (Perfect Smile, MyHealthcare)</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M60" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N60" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O60" s="2" t="inlineStr">
+        <is>
+          <t>Polished new site; likely some marketing spend</t>
+        </is>
+      </c>
+      <c r="P60" s="2" t="inlineStr">
+        <is>
+          <t>New-ish practice building patient base against established chains with bigger budgets</t>
+        </is>
+      </c>
+      <c r="Q60" s="2" t="inlineStr">
+        <is>
+          <t>AI-visibility race: be what ChatGPT recommends for 'Invisalign Fulham' before the chains lock it up</t>
+        </is>
+      </c>
+      <c r="R60" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S60" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T60" s="2" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>Natural Health Chiropractic</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>Chiropractor</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>Hampstead Village, London NW3</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>https://www.naturalhealthchiro.co.uk</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>020 7431 4882</t>
+        </is>
+      </c>
+      <c r="G61" s="4" t="inlineStr">
+        <is>
+          <t>Matt Murray (Chiropractor)</t>
+        </is>
+      </c>
+      <c r="H61" s="4" t="inlineStr"/>
+      <c r="I61" s="4" t="inlineStr"/>
+      <c r="J61" s="4" t="inlineStr">
+        <is>
+          <t>Solo/small chiropractic clinic in one of London's wealthiest villages; treatment courses worth £500-1500 per patient</t>
+        </is>
+      </c>
+      <c r="K61" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L61" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M61" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N61" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O61" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P61" s="4" t="inlineStr">
+        <is>
+          <t>Local visibility battle vs physio chains and osteopaths for the same back-pain searches</t>
+        </is>
+      </c>
+      <c r="Q61" s="4" t="inlineStr">
+        <is>
+          <t>'Hampstead residents ask AI who can fix their back - the answer should be you'</t>
+        </is>
+      </c>
+      <c r="R61" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S61" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T61" s="4" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t>Hampstead Chiropractic Clinic</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>Chiropractor</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>O2 Centre, Finchley Rd, London NW3</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>https://hampsteadchiropractic.co.uk</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="inlineStr"/>
+      <c r="G62" s="4" t="inlineStr"/>
+      <c r="H62" s="4" t="inlineStr"/>
+      <c r="I62" s="4" t="inlineStr">
+        <is>
+          <t>facebook.com/HCCgettreated</t>
+        </is>
+      </c>
+      <c r="J62" s="4" t="inlineStr">
+        <is>
+          <t>Established BCA-member clinic treating all ages in affluent NW3; located inside Virgin Active = footfall + referral potential</t>
+        </is>
+      </c>
+      <c r="K62" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L62" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M62" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N62" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O62" s="4" t="inlineStr">
+        <is>
+          <t>Facebook page; WhatClinic reviews</t>
+        </is>
+      </c>
+      <c r="P62" s="4" t="inlineStr">
+        <is>
+          <t>Generic clinic name + weak site = losing 'chiropractor near me' to newer rivals</t>
+        </is>
+      </c>
+      <c r="Q62" s="4" t="inlineStr">
+        <is>
+          <t>Quick local-SEO wins: reviews, GBP optimisation, then AEO layer</t>
+        </is>
+      </c>
+      <c r="R62" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S62" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T62" s="4" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>Rent A Home</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>Letting agent</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>Stoke Newington, London N16</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>https://www.rentahome-uk.com</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="inlineStr"/>
+      <c r="G63" s="4" t="inlineStr"/>
+      <c r="H63" s="4" t="inlineStr"/>
+      <c r="I63" s="4" t="inlineStr"/>
+      <c r="J63" s="4" t="inlineStr">
+        <is>
+          <t>Independent lettings/management since 1994 across N16/Hackney/Islington - dense landlord market with high management LTV</t>
+        </is>
+      </c>
+      <c r="K63" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L63" s="4" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="M63" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N63" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O63" s="4" t="inlineStr">
+        <is>
+          <t>Portal listings (OnTheMarket)</t>
+        </is>
+      </c>
+      <c r="P63" s="4" t="inlineStr">
+        <is>
+          <t>Dated site; landlords choosing agents via search find Dexters/Winkworth/OpenRent first</t>
+        </is>
+      </c>
+      <c r="Q63" s="4" t="inlineStr">
+        <is>
+          <t>'Hackney landlords are worth £1000s/year each in management fees - and they can't find you'</t>
+        </is>
+      </c>
+      <c r="R63" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S63" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T63" s="4" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>Steve Mears Independent Mortgage Services</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>Mortgage broker</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>Bristol</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>https://www.stevemears.com</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>info@stevemears.com</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>0117 973 4300</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>Steve Mears (Founder)</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr"/>
+      <c r="I64" s="3" t="inlineStr"/>
+      <c r="J64" s="3" t="inlineStr">
+        <is>
+          <t>One of Bristol's longest-established brokers (1995); whole-of-market; every case worth £500-2k in proc fees + repeat remortgages</t>
+        </is>
+      </c>
+      <c r="K64" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L64" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M64" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N64" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O64" s="3" t="inlineStr">
+        <is>
+          <t>Long-standing brand; directory presence</t>
+        </is>
+      </c>
+      <c r="P64" s="3" t="inlineStr">
+        <is>
+          <t>Online brokers (Habito, L&amp;C) and Clifton Private Finance's strong SEO squeeze the middle</t>
+        </is>
+      </c>
+      <c r="Q64" s="3" t="inlineStr">
+        <is>
+          <t>'Bristol homeowners ask ChatGPT whether to use a broker - the answer names your competitors'</t>
+        </is>
+      </c>
+      <c r="R64" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S64" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T64" s="3" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>Vesta Mortgages</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>Mortgage broker</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>Bristol</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>https://www.vestamortgages.co.uk</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>enquiries@vestamortgages.co.uk</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>0117 363 7575</t>
+        </is>
+      </c>
+      <c r="G65" s="3" t="inlineStr"/>
+      <c r="H65" s="3" t="inlineStr"/>
+      <c r="I65" s="3" t="inlineStr"/>
+      <c r="J65" s="3" t="inlineStr">
+        <is>
+          <t>Independent whole-of-market adviser in a hot property market; strong fit for local-intent search plays</t>
+        </is>
+      </c>
+      <c r="K65" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L65" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M65" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N65" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O65" s="3" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P65" s="3" t="inlineStr">
+        <is>
+          <t>Smaller brand fighting Clifton PF and Fox Davidson who both invest in SEO</t>
+        </is>
+      </c>
+      <c r="Q65" s="3" t="inlineStr">
+        <is>
+          <t>Underdog local-SEO pitch for specific niches (first-time buyer Bristol, BTL Bristol)</t>
+        </is>
+      </c>
+      <c r="R65" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S65" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T65" s="3" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>Mellow Financial</t>
+        </is>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>Mortgage &amp; insurance broker</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>Bristol</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>https://www.mellowfinancial.co.uk</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t>hello@mellowfinancial.co.uk</t>
+        </is>
+      </c>
+      <c r="F66" s="4" t="inlineStr">
+        <is>
+          <t>0117 251 0544</t>
+        </is>
+      </c>
+      <c r="G66" s="4" t="inlineStr"/>
+      <c r="H66" s="4" t="inlineStr"/>
+      <c r="I66" s="4" t="inlineStr"/>
+      <c r="J66" s="4" t="inlineStr">
+        <is>
+          <t>Young friendly-brand broker; protection cross-sales boost per-client value; brandable for content marketing</t>
+        </is>
+      </c>
+      <c r="K66" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L66" s="4" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M66" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N66" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O66" s="4" t="inlineStr">
+        <is>
+          <t>Modern brand suggests marketing awareness</t>
+        </is>
+      </c>
+      <c r="P66" s="4" t="inlineStr">
+        <is>
+          <t>New brand with little search authority in competitive market</t>
+        </is>
+      </c>
+      <c r="Q66" s="4" t="inlineStr">
+        <is>
+          <t>Entry-tier: £249/mo to build the search foundation while the brand is young</t>
+        </is>
+      </c>
+      <c r="R66" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S66" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T66" s="4" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>Holcombe Associates</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>Business consultancy</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>Dursley (serves Bristol/Glos/Somerset)</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>https://www.holcombeassociate.com</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>jwasdell@holcombeassociate.com</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>07796 195495</t>
+        </is>
+      </c>
+      <c r="G67" s="4" t="inlineStr">
+        <is>
+          <t>James Wadsell (Founder)</t>
+        </is>
+      </c>
+      <c r="H67" s="4" t="inlineStr"/>
+      <c r="I67" s="4" t="inlineStr"/>
+      <c r="J67" s="4" t="inlineStr">
+        <is>
+          <t>SME growth/exit consultancy; engagements worth £10k+; already builds county landing pages (Bristol, Somerset, Glos, Worcs) = SEO believer</t>
+        </is>
+      </c>
+      <c r="K67" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L67" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M67" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N67" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O67" s="4" t="inlineStr">
+        <is>
+          <t>County landing pages = active DIY SEO</t>
+        </is>
+      </c>
+      <c r="P67" s="4" t="inlineStr">
+        <is>
+          <t>Landing pages exist but thin; consultancy searches increasingly answered by AI</t>
+        </is>
+      </c>
+      <c r="Q67" s="4" t="inlineStr">
+        <is>
+          <t>'Your county pages show the intent - here's how to make them actually win clients'</t>
+        </is>
+      </c>
+      <c r="R67" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S67" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T67" s="4" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>Fernlea Vets</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>Independent vet</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>Hanham &amp; Kingswood, Bristol</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>https://fernleavets.co.uk</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>0117 967 7067</t>
+        </is>
+      </c>
+      <c r="G68" s="3" t="inlineStr"/>
+      <c r="H68" s="3" t="inlineStr"/>
+      <c r="I68" s="3" t="inlineStr"/>
+      <c r="J68" s="3" t="inlineStr">
+        <is>
+          <t>Privately run two-site practice since 1986 in a city where IVC (corporate HQ'd in Bristol!) owns most rivals; independence is a differentiator</t>
+        </is>
+      </c>
+      <c r="K68" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L68" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M68" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N68" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O68" s="3" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P68" s="3" t="inlineStr">
+        <is>
+          <t>Corporate groups dominate 'vet Bristol' searches with big budgets</t>
+        </is>
+      </c>
+      <c r="Q68" s="3" t="inlineStr">
+        <is>
+          <t>Independence story + AEO: be the answer to 'independent vet Bristol'</t>
+        </is>
+      </c>
+      <c r="R68" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S68" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T68" s="3" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>Avenue Veterinary Centre</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>Independent vet</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>Bristol</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>https://avenue-vets.com</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>enquiries@avenue-vets.com</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>0117 956 9038</t>
+        </is>
+      </c>
+      <c r="G69" s="3" t="inlineStr"/>
+      <c r="H69" s="3" t="inlineStr"/>
+      <c r="I69" s="3" t="inlineStr"/>
+      <c r="J69" s="3" t="inlineStr">
+        <is>
+          <t>Independent practice with 100+ years heritage; loyal client base but heritage doesn't rank on Google</t>
+        </is>
+      </c>
+      <c r="K69" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L69" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M69" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N69" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O69" s="3" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P69" s="3" t="inlineStr">
+        <is>
+          <t>Same corporate-vs-independent squeeze as Fernlea</t>
+        </is>
+      </c>
+      <c r="Q69" s="3" t="inlineStr">
+        <is>
+          <t>Heritage + independence content play for local and AI search</t>
+        </is>
+      </c>
+      <c r="R69" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S69" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T69" s="3" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t>Burnside Chartered Accountants</t>
+        </is>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>Chartered accountants</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>Queen Square, Bristol BS1</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>https://burnside.biz</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>0845 071 7676</t>
+        </is>
+      </c>
+      <c r="G70" s="4" t="inlineStr"/>
+      <c r="H70" s="4" t="inlineStr"/>
+      <c r="I70" s="4" t="inlineStr"/>
+      <c r="J70" s="4" t="inlineStr">
+        <is>
+          <t>Independent firm in prime Queen Square address serving Bristol SMEs; recurring-fee client model</t>
+        </is>
+      </c>
+      <c r="K70" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L70" s="4" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="M70" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N70" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O70" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P70" s="4" t="inlineStr">
+        <is>
+          <t>'.biz' domain and dated site vs cloud-first rivals chasing the same SME clients</t>
+        </is>
+      </c>
+      <c r="Q70" s="4" t="inlineStr">
+        <is>
+          <t>Modernisation pitch: site + local SEO before the online accountants take the market</t>
+        </is>
+      </c>
+      <c r="R70" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S70" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T70" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T56"/>
+  <autoFilter ref="A1:T70"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5604,7 +6808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B48"/>
+  <dimension ref="A1:B52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5624,7 +6828,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>55</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5">
@@ -5641,13 +6845,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Private GP</t>
+          <t>Mortgage broker</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -5657,37 +6861,37 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Physiotherapy clinic</t>
+          <t>Chartered accountants</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Solar installer</t>
+          <t>Independent vet</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Chartered accountants</t>
+          <t>Private GP</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Wedding venue</t>
+          <t>Private dentist</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -5697,7 +6901,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating / boilers</t>
+          <t>Physiotherapy clinic</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -5707,7 +6911,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Electrician</t>
+          <t>Solar installer</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -5717,7 +6921,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Event &amp; wedding caterer</t>
+          <t>Letting agent</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -5727,7 +6931,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Personal training studio</t>
+          <t>Wedding venue</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -5737,67 +6941,67 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Dentist / Orthodontics</t>
+          <t>Plumbing &amp; heating / boilers</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Private dentist</t>
+          <t>Electrician</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Specialist dental/implant clinic</t>
+          <t>Event &amp; wedding caterer</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Law firm</t>
+          <t>Personal training studio</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Boutique corporate law firm</t>
+          <t>Family law firm</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Cosmetic/aesthetics clinic</t>
+          <t>Chiropractor</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Skin &amp; laser clinic</t>
+          <t>Dentist / Orthodontics</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -5807,7 +7011,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Mortgage broker</t>
+          <t>Specialist dental/implant clinic</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -5817,7 +7021,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Mortgage broker / financial adviser</t>
+          <t>Law firm</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -5827,7 +7031,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Architects (RIBA chartered)</t>
+          <t>Boutique corporate law firm</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -5837,7 +7041,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Recruitment agency (tech/startups)</t>
+          <t>Cosmetic/aesthetics clinic</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -5847,7 +7051,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Recruitment agency (IT/data)</t>
+          <t>Skin &amp; laser clinic</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -5857,7 +7061,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Independent vet</t>
+          <t>Mortgage broker / financial adviser</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -5867,7 +7071,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Independent vet (24/7 emergency)</t>
+          <t>Architects (RIBA chartered)</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -5877,7 +7081,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Interior design studio</t>
+          <t>Recruitment agency (tech/startups)</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -5887,7 +7091,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Letting agent</t>
+          <t>Recruitment agency (IT/data)</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -5897,7 +7101,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Letting &amp; estate agent</t>
+          <t>Independent vet (24/7 emergency)</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -5907,7 +7111,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Cosmetic clinic (injectables)</t>
+          <t>Interior design studio</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -5917,7 +7121,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Cosmetic/anti-ageing clinic</t>
+          <t>Letting &amp; estate agent</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -5927,7 +7131,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Yoga &amp; reformer pilates studio</t>
+          <t>Cosmetic clinic (injectables)</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -5937,7 +7141,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Reformer pilates studio</t>
+          <t>Cosmetic/anti-ageing clinic</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -5947,7 +7151,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Financial adviser / wealth management</t>
+          <t>Yoga &amp; reformer pilates studio</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -5957,7 +7161,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Wealth management</t>
+          <t>Reformer pilates studio</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -5967,7 +7171,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Private tuition agency</t>
+          <t>Financial adviser / wealth management</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -5977,7 +7181,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Private tuition &amp; education consultancy</t>
+          <t>Wealth management</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -5987,7 +7191,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Osteopath</t>
+          <t>Private tuition agency</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -5997,7 +7201,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Osteopathy clinic</t>
+          <t>Private tuition &amp; education consultancy</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -6007,7 +7211,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Design &amp; build / home renovation</t>
+          <t>Osteopath</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -6017,7 +7221,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Builders / building contractor</t>
+          <t>Osteopathy clinic</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -6027,7 +7231,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Roofer</t>
+          <t>Design &amp; build / home renovation</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -6037,7 +7241,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Home care / live-in care</t>
+          <t>Builders / building contractor</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -6047,7 +7251,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Private day nurseries</t>
+          <t>Roofer</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -6057,10 +7261,50 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
+          <t>Home care / live-in care</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Private day nurseries</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
           <t>Personal training &amp; wellness studio</t>
         </is>
       </c>
-      <c r="B48" t="n">
+      <c r="B50" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Mortgage &amp; insurance broker</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Business consultancy</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 3c: +31 prospects - database complete at 100 rows
Interior design, landscaping, orthodontists, architects, gyms, physios,
aesthetics, solar, tutors, estate agents and law firms across Bath,
Richmond, Surrey, Cotswolds, Bristol and London. README batch log updated.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$101</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T70"/>
+  <dimension ref="A1:T101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -6796,8 +6796,2620 @@
       </c>
       <c r="T70" s="4" t="inlineStr"/>
     </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>Etons of Bath</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Interior designer (period homes)</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>Walcot Street, Bath</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>https://www.etonsofbath.com</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>sarah@etonsofbath.com</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>01225 639002</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>Sarah Latham (Founder)</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr"/>
+      <c r="I71" s="2" t="inlineStr"/>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>Specialist in Georgian/listed Bath properties - projects worth £50k+; showroom presence; already builds city landing pages (Bristol)</t>
+        </is>
+      </c>
+      <c r="K71" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L71" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M71" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N71" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O71" s="2" t="inlineStr">
+        <is>
+          <t>Location landing pages; showroom; established brand since 2009</t>
+        </is>
+      </c>
+      <c r="P71" s="2" t="inlineStr">
+        <is>
+          <t>Period-home niche is perfect AEO territory but AI engines don't yet cite them for it</t>
+        </is>
+      </c>
+      <c r="Q71" s="2" t="inlineStr">
+        <is>
+          <t>'Own the answer to "interior designer for Georgian homes" across Google and ChatGPT'</t>
+        </is>
+      </c>
+      <c r="R71" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S71" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T71" s="2" t="inlineStr">
+        <is>
+          <t>Founder email published - direct route</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Bluefish Landscaping</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>Landscape design &amp; build</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Farnham, Surrey (covers Weybridge/Guildford)</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bluefishlandscapes.co.uk</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>enquiries@bluefishlandscapes.co.uk</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>01252 321511</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>James Fish (Founder)</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr"/>
+      <c r="I72" s="2" t="inlineStr"/>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>Luxury gardens, pools and outdoor kitchens for Surrey estates - projects £50-500k; BALI member; one client pays for a decade of SEO</t>
+        </is>
+      </c>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L72" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M72" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N72" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O72" s="2" t="inlineStr">
+        <is>
+          <t>BALI membership; case-study content</t>
+        </is>
+      </c>
+      <c r="P72" s="2" t="inlineStr">
+        <is>
+          <t>Surrey's wealthiest postcodes research online; national design directories soak up the searches</t>
+        </is>
+      </c>
+      <c r="Q72" s="2" t="inlineStr">
+        <is>
+          <t>'One Weybridge garden project is worth 100x our fee - be the name Surrey finds'</t>
+        </is>
+      </c>
+      <c r="R72" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S72" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T72" s="2" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>Cobb Farr Estate Agents</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent (premium)</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>Bath (+ Bradford-on-Avon)</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cobbfarr.com</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F73" s="3" t="inlineStr"/>
+      <c r="G73" s="3" t="inlineStr">
+        <is>
+          <t>Philip Cobb (Co-founder &amp; MD)</t>
+        </is>
+      </c>
+      <c r="H73" s="3" t="inlineStr"/>
+      <c r="I73" s="3" t="inlineStr"/>
+      <c r="J73" s="3" t="inlineStr">
+        <is>
+          <t>Premium Bath independent since 1989; high-value Georgian stock = large fees per instruction</t>
+        </is>
+      </c>
+      <c r="K73" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L73" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M73" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N73" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O73" s="3" t="inlineStr">
+        <is>
+          <t>Portal listings; established brand</t>
+        </is>
+      </c>
+      <c r="P73" s="3" t="inlineStr">
+        <is>
+          <t>Knight Frank/Savills/Fine &amp; Country dominate premium Bath searches</t>
+        </is>
+      </c>
+      <c r="Q73" s="3" t="inlineStr">
+        <is>
+          <t>'Bath sellers of £1m+ homes shortlist 3 agents online - make sure you're one of them'</t>
+        </is>
+      </c>
+      <c r="R73" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S73" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T73" s="3" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>Nash &amp; Co Estate Agents</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>Bath</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>http://www.nashandcobath.co.uk</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>enquiries@nashandcobath.co.uk</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>01225 444 800</t>
+        </is>
+      </c>
+      <c r="G74" s="3" t="inlineStr"/>
+      <c r="H74" s="3" t="inlineStr"/>
+      <c r="I74" s="3" t="inlineStr"/>
+      <c r="J74" s="3" t="inlineStr">
+        <is>
+          <t>Independent Bath agency, 80+ years combined experience; dated website vs national rivals</t>
+        </is>
+      </c>
+      <c r="K74" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L74" s="3" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="M74" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N74" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O74" s="3" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P74" s="3" t="inlineStr">
+        <is>
+          <t>HTTP-only dated site actively hurts trust for valuation leads</t>
+        </is>
+      </c>
+      <c r="Q74" s="3" t="inlineStr">
+        <is>
+          <t>Website + local SEO rebuild pitch: table stakes to compete in Bath</t>
+        </is>
+      </c>
+      <c r="R74" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S74" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T74" s="3" t="inlineStr">
+        <is>
+          <t>Site still on http:// - instant credibility opener</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>@Home Estate Agents</t>
+        </is>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>Bath</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>https://www.athomebath.co.uk</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F75" s="4" t="inlineStr"/>
+      <c r="G75" s="4" t="inlineStr">
+        <is>
+          <t>Toby Knight (Founder)</t>
+        </is>
+      </c>
+      <c r="H75" s="4" t="inlineStr"/>
+      <c r="I75" s="4" t="inlineStr"/>
+      <c r="J75" s="4" t="inlineStr">
+        <is>
+          <t>Independent since 2013, founder with 33 years local experience; boutique service positioning</t>
+        </is>
+      </c>
+      <c r="K75" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L75" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M75" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N75" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O75" s="4" t="inlineStr">
+        <is>
+          <t>Rightmove profile</t>
+        </is>
+      </c>
+      <c r="P75" s="4" t="inlineStr">
+        <is>
+          <t>Small independent squeezed by corporates and Bath &amp; Rural boutiques alike</t>
+        </is>
+      </c>
+      <c r="Q75" s="4" t="inlineStr">
+        <is>
+          <t>Local-hero content play: founder's 33 years of Bath knowledge as AEO material</t>
+        </is>
+      </c>
+      <c r="R75" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S75" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T75" s="4" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>The Brace Orthodontic Practice</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>Orthodontist</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>Artillery Passage, London E1</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>https://www.thebrace.com</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>020 7247 5768</t>
+        </is>
+      </c>
+      <c r="G76" s="3" t="inlineStr"/>
+      <c r="H76" s="3" t="inlineStr"/>
+      <c r="I76" s="3" t="inlineStr"/>
+      <c r="J76" s="3" t="inlineStr">
+        <is>
+          <t>Specialist orthodontists near Liverpool St; Invisalign/braces cases £3-6k; City workers self-pay</t>
+        </is>
+      </c>
+      <c r="K76" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L76" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M76" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N76" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O76" s="3" t="inlineStr">
+        <is>
+          <t>Some review cultivation</t>
+        </is>
+      </c>
+      <c r="P76" s="3" t="inlineStr">
+        <is>
+          <t>Chain clinics and Harley St brands dominate 'Invisalign London' searches</t>
+        </is>
+      </c>
+      <c r="Q76" s="3" t="inlineStr">
+        <is>
+          <t>City-worker angle: own 'orthodontist near Liverpool Street' + AI answers</t>
+        </is>
+      </c>
+      <c r="R76" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S76" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T76" s="3" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>The London Orthodontic Group</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>Orthodontist</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>https://londonlovesbraces.com</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F77" s="3" t="inlineStr"/>
+      <c r="G77" s="3" t="inlineStr">
+        <is>
+          <t>Dr Richard Hennebry &amp; Dr Vivi Grigoriou-Hennebry (Owners)</t>
+        </is>
+      </c>
+      <c r="H77" s="3" t="inlineStr"/>
+      <c r="I77" s="3" t="inlineStr"/>
+      <c r="J77" s="3" t="inlineStr">
+        <is>
+          <t>Husband-and-wife US-trained specialists - rare credential in UK; high-value cases; memorable brand domain</t>
+        </is>
+      </c>
+      <c r="K77" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L77" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M77" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N77" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O77" s="3" t="inlineStr">
+        <is>
+          <t>Branded domain (londonlovesbraces) suggests marketing intent</t>
+        </is>
+      </c>
+      <c r="P77" s="3" t="inlineStr">
+        <is>
+          <t>US-trained differentiation invisible in search results and AI answers</t>
+        </is>
+      </c>
+      <c r="Q77" s="3" t="inlineStr">
+        <is>
+          <t>'You have the best credentials story in London orthodontics - nobody can find it'</t>
+        </is>
+      </c>
+      <c r="R77" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S77" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T77" s="3" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>TW10 Architects</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>Architects</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>Richmond, London TW10</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>https://find-an-architect.architecture.com/tw10-architects/richmond</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>via RIBA directory / website</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="inlineStr"/>
+      <c r="G78" s="3" t="inlineStr"/>
+      <c r="H78" s="3" t="inlineStr"/>
+      <c r="I78" s="3" t="inlineStr"/>
+      <c r="J78" s="3" t="inlineStr">
+        <is>
+          <t>RIBA practice, 15+ years, residential focus in affluent Richmond; extensions/refurbs worth £100k+</t>
+        </is>
+      </c>
+      <c r="K78" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L78" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M78" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N78" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O78" s="3" t="inlineStr">
+        <is>
+          <t>RIBA directory listing</t>
+        </is>
+      </c>
+      <c r="P78" s="3" t="inlineStr">
+        <is>
+          <t>Homeowners find architects via Houzz/directories that charge for leads</t>
+        </is>
+      </c>
+      <c r="Q78" s="3" t="inlineStr">
+        <is>
+          <t>'Richmond homeowners ask ChatGPT how to find an architect - be the named answer'</t>
+        </is>
+      </c>
+      <c r="R78" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S78" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T78" s="3" t="inlineStr">
+        <is>
+          <t>Get direct website/email before outreach</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t>Scenario Architecture</t>
+        </is>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>Architects</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>London &amp; Surrey</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>https://scenarioarchitecture.com</t>
+        </is>
+      </c>
+      <c r="E79" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F79" s="4" t="inlineStr"/>
+      <c r="G79" s="4" t="inlineStr">
+        <is>
+          <t>Ran Ankory &amp; Maya Carni (Founders)</t>
+        </is>
+      </c>
+      <c r="H79" s="4" t="inlineStr"/>
+      <c r="I79" s="4" t="inlineStr"/>
+      <c r="J79" s="4" t="inlineStr">
+        <is>
+          <t>RIBA practice with strong brand; already runs location landing pages ('architects Surrey') = active SEO spend</t>
+        </is>
+      </c>
+      <c r="K79" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L79" s="4" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M79" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N79" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O79" s="4" t="inlineStr">
+        <is>
+          <t>Location landing pages; polished site; likely agency</t>
+        </is>
+      </c>
+      <c r="P79" s="4" t="inlineStr">
+        <is>
+          <t>Paying for SEO but AEO/GEO layer missing in a design-literate market</t>
+        </is>
+      </c>
+      <c r="Q79" s="4" t="inlineStr">
+        <is>
+          <t>Agency-upgrade pitch: add AI-search visibility to existing SEO investment</t>
+        </is>
+      </c>
+      <c r="R79" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S79" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T79" s="4" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>Malcolm Jenkins Associates</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>Architects</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>Shepperton, Surrey</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>http://www.architectinguildford.co.uk</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="inlineStr">
+        <is>
+          <t>enquiries@malcolmjenkins.co.uk</t>
+        </is>
+      </c>
+      <c r="F80" s="4" t="inlineStr">
+        <is>
+          <t>01932 225344</t>
+        </is>
+      </c>
+      <c r="G80" s="4" t="inlineStr">
+        <is>
+          <t>Malcolm Jenkins (Principal)</t>
+        </is>
+      </c>
+      <c r="H80" s="4" t="inlineStr"/>
+      <c r="I80" s="4" t="inlineStr"/>
+      <c r="J80" s="4" t="inlineStr">
+        <is>
+          <t>Established Surrey practice with keyword domain but very dated site; residential project values high in TW/GU postcodes</t>
+        </is>
+      </c>
+      <c r="K80" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L80" s="4" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="M80" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N80" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O80" s="4" t="inlineStr">
+        <is>
+          <t>Keyword domain shows old SEO effort</t>
+        </is>
+      </c>
+      <c r="P80" s="4" t="inlineStr">
+        <is>
+          <t>1990s-era website undermines premium project credibility</t>
+        </is>
+      </c>
+      <c r="Q80" s="4" t="inlineStr">
+        <is>
+          <t>Modernise + rank: the domain has history, the site squanders it</t>
+        </is>
+      </c>
+      <c r="R80" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S80" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T80" s="4" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>Clair Strong Interior Design</t>
+        </is>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>Interior designer</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>Bath (+ London)</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>https://www.clairstrong.co.uk</t>
+        </is>
+      </c>
+      <c r="E81" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F81" s="4" t="inlineStr"/>
+      <c r="G81" s="4" t="inlineStr">
+        <is>
+          <t>Clair Strong (Founder)</t>
+        </is>
+      </c>
+      <c r="H81" s="4" t="inlineStr"/>
+      <c r="I81" s="4" t="inlineStr"/>
+      <c r="J81" s="4" t="inlineStr">
+        <is>
+          <t>Established 2006, Bath + London projects; residential and commercial; solo-led studio with strong portfolio</t>
+        </is>
+      </c>
+      <c r="K81" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L81" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M81" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N81" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O81" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P81" s="4" t="inlineStr">
+        <is>
+          <t>Etons of Bath and bigger studios out-market her in the same city</t>
+        </is>
+      </c>
+      <c r="Q81" s="4" t="inlineStr">
+        <is>
+          <t>Entry-tier local SEO: own 'interior designer Bath' long-tail queries</t>
+        </is>
+      </c>
+      <c r="R81" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S81" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T81" s="4" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t>Graduate Gardeners</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>Garden design &amp; landscaping</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>Bisley, Gloucestershire (Cotswolds)</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>https://www.graduategardeners.co.uk</t>
+        </is>
+      </c>
+      <c r="E82" s="3" t="inlineStr">
+        <is>
+          <t>office@graduategardeners.co.uk</t>
+        </is>
+      </c>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t>01452 770273</t>
+        </is>
+      </c>
+      <c r="G82" s="3" t="inlineStr"/>
+      <c r="H82" s="3" t="inlineStr"/>
+      <c r="I82" s="3" t="inlineStr"/>
+      <c r="J82" s="3" t="inlineStr">
+        <is>
+          <t>BALI award winners, 50+ years, serving Cotswolds wealth; garden builds worth £30-150k</t>
+        </is>
+      </c>
+      <c r="K82" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L82" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M82" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N82" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O82" s="3" t="inlineStr">
+        <is>
+          <t>BALI awards; established reputation</t>
+        </is>
+      </c>
+      <c r="P82" s="3" t="inlineStr">
+        <is>
+          <t>Award pedigree doesn't surface in AI answers for 'garden designer Cotswolds'</t>
+        </is>
+      </c>
+      <c r="Q82" s="3" t="inlineStr">
+        <is>
+          <t>Turn 50 years + BALI awards into the AI-cited Cotswolds authority</t>
+        </is>
+      </c>
+      <c r="R82" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S82" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T82" s="3" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>Hitchen Legal</t>
+        </is>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>Legal recruitment</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>https://www.hitchenlegal.com</t>
+        </is>
+      </c>
+      <c r="E83" s="4" t="inlineStr">
+        <is>
+          <t>kate@hitchenlegal.com</t>
+        </is>
+      </c>
+      <c r="F83" s="4" t="inlineStr"/>
+      <c r="G83" s="4" t="inlineStr">
+        <is>
+          <t>Kate Hitchen (Founder/Director)</t>
+        </is>
+      </c>
+      <c r="H83" s="4" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/katehitchen</t>
+        </is>
+      </c>
+      <c r="I83" s="4" t="inlineStr"/>
+      <c r="J83" s="4" t="inlineStr">
+        <is>
+          <t>Boutique legal search firm since 2013; placement fees £15-30k; founder active on LinkedIn</t>
+        </is>
+      </c>
+      <c r="K83" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L83" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M83" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N83" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O83" s="4" t="inlineStr">
+        <is>
+          <t>Founder LinkedIn activity</t>
+        </is>
+      </c>
+      <c r="P83" s="4" t="inlineStr">
+        <is>
+          <t>Law firms ask AI to name legal recruiters - big brands (Michael Page, Robert Walters) get cited</t>
+        </is>
+      </c>
+      <c r="Q83" s="4" t="inlineStr">
+        <is>
+          <t>Boutique-vs-giant AEO play in legal recruitment</t>
+        </is>
+      </c>
+      <c r="R83" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S83" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T83" s="4" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t>Workout Bristol</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>Independent gym &amp; health club</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>Harbourside + Ashton, Bristol</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>https://www.workoutbristol.co.uk</t>
+        </is>
+      </c>
+      <c r="E84" s="3" t="inlineStr">
+        <is>
+          <t>ashton@workoutbristol.co.uk</t>
+        </is>
+      </c>
+      <c r="F84" s="3" t="inlineStr"/>
+      <c r="G84" s="3" t="inlineStr"/>
+      <c r="H84" s="3" t="inlineStr"/>
+      <c r="I84" s="3" t="inlineStr"/>
+      <c r="J84" s="3" t="inlineStr">
+        <is>
+          <t>Bristol's longest-established independent club (1982), two sites, classes + PT; memberships = recurring revenue</t>
+        </is>
+      </c>
+      <c r="K84" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L84" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M84" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N84" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O84" s="3" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P84" s="3" t="inlineStr">
+        <is>
+          <t>PureGym/Anytime chains carpet-bomb 'gym Bristol' searches</t>
+        </is>
+      </c>
+      <c r="Q84" s="3" t="inlineStr">
+        <is>
+          <t>Independent-community angle vs chains; own 'independent gym Bristol'</t>
+        </is>
+      </c>
+      <c r="R84" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S84" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T84" s="3" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>Ministry of Fitness</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>Independent gym</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>Kingswood, Bristol</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>https://mofgym.co.uk</t>
+        </is>
+      </c>
+      <c r="E85" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F85" s="4" t="inlineStr"/>
+      <c r="G85" s="4" t="inlineStr"/>
+      <c r="H85" s="4" t="inlineStr"/>
+      <c r="I85" s="4" t="inlineStr"/>
+      <c r="J85" s="4" t="inlineStr">
+        <is>
+          <t>11,000 sq ft biggest independent gym in Bristol; four training areas; membership volume model</t>
+        </is>
+      </c>
+      <c r="K85" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L85" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M85" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N85" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O85" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P85" s="4" t="inlineStr">
+        <is>
+          <t>Budget chains undercut on price; needs differentiation in search</t>
+        </is>
+      </c>
+      <c r="Q85" s="4" t="inlineStr">
+        <is>
+          <t>Local-SEO + review engine to defend Kingswood catchment</t>
+        </is>
+      </c>
+      <c r="R85" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S85" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T85" s="4" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>Bristol Physiotherapy Clinic</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>Physiotherapy clinic</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>3 sites: Harbourside, Redland, Whiteladies Rd Bristol</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>https://bristolphysiotherapyclinic.co.uk</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="inlineStr">
+        <is>
+          <t>info@bristolphysiotherapyclinic.co.uk</t>
+        </is>
+      </c>
+      <c r="F86" s="3" t="inlineStr">
+        <is>
+          <t>0117 973 8319</t>
+        </is>
+      </c>
+      <c r="G86" s="3" t="inlineStr"/>
+      <c r="H86" s="3" t="inlineStr"/>
+      <c r="I86" s="3" t="inlineStr"/>
+      <c r="J86" s="3" t="inlineStr">
+        <is>
+          <t>Three-site evidence-based practice since 2007; self-pay + insurance work; sites inside gyms/clubs = referral flow</t>
+        </is>
+      </c>
+      <c r="K86" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L86" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M86" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N86" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O86" s="3" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P86" s="3" t="inlineStr">
+        <is>
+          <t>Multi-site practice with single-site search visibility</t>
+        </is>
+      </c>
+      <c r="Q86" s="3" t="inlineStr">
+        <is>
+          <t>Per-location Google/AI visibility: 3 sites should mean 3x the search presence</t>
+        </is>
+      </c>
+      <c r="R86" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S86" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T86" s="3" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t>McFerran Physio</t>
+        </is>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>Physiotherapy (sports)</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="inlineStr">
+        <is>
+          <t>Clifton Rugby Club, Bristol</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>https://mcferranphysio.co.uk</t>
+        </is>
+      </c>
+      <c r="E87" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F87" s="4" t="inlineStr"/>
+      <c r="G87" s="4" t="inlineStr">
+        <is>
+          <t>Alan McFerran (Founder)</t>
+        </is>
+      </c>
+      <c r="H87" s="4" t="inlineStr"/>
+      <c r="I87" s="4" t="inlineStr"/>
+      <c r="J87" s="4" t="inlineStr">
+        <is>
+          <t>Ex-Bristol City FC physio - elite-sport credibility; self-pay sports injury market in North Bristol</t>
+        </is>
+      </c>
+      <c r="K87" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L87" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M87" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N87" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O87" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P87" s="4" t="inlineStr">
+        <is>
+          <t>Pro-football story buried; generic rivals outrank him</t>
+        </is>
+      </c>
+      <c r="Q87" s="4" t="inlineStr">
+        <is>
+          <t>'11 years with Bristol City's players - make that the answer to "sports physio Bristol"'</t>
+        </is>
+      </c>
+      <c r="R87" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S87" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T87" s="4" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="3" t="inlineStr">
+        <is>
+          <t>Parkgate Estate Agents</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>Estate &amp; letting agent</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>Eton St, Richmond TW9</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>https://www.parkgate.co.uk</t>
+        </is>
+      </c>
+      <c r="E88" s="3" t="inlineStr">
+        <is>
+          <t>info@parkgate.co.uk</t>
+        </is>
+      </c>
+      <c r="F88" s="3" t="inlineStr">
+        <is>
+          <t>020 8940 2991</t>
+        </is>
+      </c>
+      <c r="G88" s="3" t="inlineStr"/>
+      <c r="H88" s="3" t="inlineStr"/>
+      <c r="I88" s="3" t="inlineStr"/>
+      <c r="J88" s="3" t="inlineStr">
+        <is>
+          <t>Truly independent Richmond agency since 1976; already builds service landing pages (letting agents Richmond, property managers Twickenham)</t>
+        </is>
+      </c>
+      <c r="K88" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L88" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M88" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N88" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O88" s="3" t="inlineStr">
+        <is>
+          <t>Service landing pages = active SEO</t>
+        </is>
+      </c>
+      <c r="P88" s="3" t="inlineStr">
+        <is>
+          <t>Foxtons/Savills/Hamptons saturate Richmond; AEO is the open flank</t>
+        </is>
+      </c>
+      <c r="Q88" s="3" t="inlineStr">
+        <is>
+          <t>Upgrade pitch: their landing pages + our AEO layer = AI-recommended independent</t>
+        </is>
+      </c>
+      <c r="R88" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S88" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T88" s="3" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>Antony Roberts</t>
+        </is>
+      </c>
+      <c r="B89" s="3" t="inlineStr">
+        <is>
+          <t>Estate &amp; letting agent</t>
+        </is>
+      </c>
+      <c r="C89" s="3" t="inlineStr">
+        <is>
+          <t>Richmond, Kew, East Sheen</t>
+        </is>
+      </c>
+      <c r="D89" s="3" t="inlineStr">
+        <is>
+          <t>https://www.antonyroberts.co.uk</t>
+        </is>
+      </c>
+      <c r="E89" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F89" s="3" t="inlineStr"/>
+      <c r="G89" s="3" t="inlineStr">
+        <is>
+          <t>Antony Roberts (Founder)</t>
+        </is>
+      </c>
+      <c r="H89" s="3" t="inlineStr"/>
+      <c r="I89" s="3" t="inlineStr"/>
+      <c r="J89" s="3" t="inlineStr">
+        <is>
+          <t>Leading independent in Richmond/Kew with founder-name brand and local landlord roots; premium stock</t>
+        </is>
+      </c>
+      <c r="K89" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L89" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M89" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N89" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O89" s="3" t="inlineStr">
+        <is>
+          <t>Established multi-office brand</t>
+        </is>
+      </c>
+      <c r="P89" s="3" t="inlineStr">
+        <is>
+          <t>Corporate agents dominate search for Richmond property despite AR's local standing</t>
+        </is>
+      </c>
+      <c r="Q89" s="3" t="inlineStr">
+        <is>
+          <t>'Richmond's leading independent should be Google's answer too'</t>
+        </is>
+      </c>
+      <c r="R89" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S89" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T89" s="3" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="4" t="inlineStr">
+        <is>
+          <t>Griffin Stevens</t>
+        </is>
+      </c>
+      <c r="B90" s="4" t="inlineStr">
+        <is>
+          <t>Estate &amp; letting agent</t>
+        </is>
+      </c>
+      <c r="C90" s="4" t="inlineStr">
+        <is>
+          <t>Twickenham</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>https://griffinstevens.co.uk</t>
+        </is>
+      </c>
+      <c r="E90" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F90" s="4" t="inlineStr"/>
+      <c r="G90" s="4" t="inlineStr"/>
+      <c r="H90" s="4" t="inlineStr"/>
+      <c r="I90" s="4" t="inlineStr"/>
+      <c r="J90" s="4" t="inlineStr">
+        <is>
+          <t>Independent sales + lettings in Twickenham's family-home market</t>
+        </is>
+      </c>
+      <c r="K90" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L90" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M90" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N90" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O90" s="4" t="inlineStr">
+        <is>
+          <t>Portal listings</t>
+        </is>
+      </c>
+      <c r="P90" s="4" t="inlineStr">
+        <is>
+          <t>Smaller brand in Foxtons territory</t>
+        </is>
+      </c>
+      <c r="Q90" s="4" t="inlineStr">
+        <is>
+          <t>Hyperlocal content: own Twickenham micro-neighbourhood searches</t>
+        </is>
+      </c>
+      <c r="R90" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S90" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T90" s="4" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="inlineStr">
+        <is>
+          <t>Jo &amp; Co Property Management</t>
+        </is>
+      </c>
+      <c r="B91" s="4" t="inlineStr">
+        <is>
+          <t>Letting agent / property management</t>
+        </is>
+      </c>
+      <c r="C91" s="4" t="inlineStr">
+        <is>
+          <t>Richmond &amp; Kingston, London</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>https://www.joandcoprop.com</t>
+        </is>
+      </c>
+      <c r="E91" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F91" s="4" t="inlineStr"/>
+      <c r="G91" s="4" t="inlineStr">
+        <is>
+          <t>Jo (Founder)</t>
+        </is>
+      </c>
+      <c r="H91" s="4" t="inlineStr"/>
+      <c r="I91" s="4" t="inlineStr"/>
+      <c r="J91" s="4" t="inlineStr">
+        <is>
+          <t>Modern management-focused agency across SW London suburbs; recurring management fees per landlord</t>
+        </is>
+      </c>
+      <c r="K91" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L91" s="4" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M91" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N91" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O91" s="4" t="inlineStr">
+        <is>
+          <t>Modern brand/site</t>
+        </is>
+      </c>
+      <c r="P91" s="4" t="inlineStr">
+        <is>
+          <t>Young brand lacking search authority vs Parkgate/Antony Roberts</t>
+        </is>
+      </c>
+      <c r="Q91" s="4" t="inlineStr">
+        <is>
+          <t>Landlord-focused content + local SEO from the ground up</t>
+        </is>
+      </c>
+      <c r="R91" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S91" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T91" s="4" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="3" t="inlineStr">
+        <is>
+          <t>Sharp Family Law</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>Family law firm</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>Bath (+ Bristol)</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sharpfamilylaw.com</t>
+        </is>
+      </c>
+      <c r="E92" s="3" t="inlineStr">
+        <is>
+          <t>info@sharpfamilylaw.com</t>
+        </is>
+      </c>
+      <c r="F92" s="3" t="inlineStr"/>
+      <c r="G92" s="3" t="inlineStr">
+        <is>
+          <t>Richard Sharp (Managing Partner)</t>
+        </is>
+      </c>
+      <c r="H92" s="3" t="inlineStr"/>
+      <c r="I92" s="3" t="inlineStr"/>
+      <c r="J92" s="3" t="inlineStr">
+        <is>
+          <t>Specialist divorce firm in Bath; complex/relocation cases worth £15k+ fees; named MP with direct email</t>
+        </is>
+      </c>
+      <c r="K92" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L92" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M92" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N92" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O92" s="3" t="inlineStr">
+        <is>
+          <t>Directory profiles</t>
+        </is>
+      </c>
+      <c r="P92" s="3" t="inlineStr">
+        <is>
+          <t>Regional giants (Thrings, Battens) and national brands crowd Bath family-law searches</t>
+        </is>
+      </c>
+      <c r="Q92" s="3" t="inlineStr">
+        <is>
+          <t>'Divorcing spouses in Bath research lawyers at midnight - be the answer they find'</t>
+        </is>
+      </c>
+      <c r="R92" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S92" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T92" s="3" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="4" t="inlineStr">
+        <is>
+          <t>Awdry Law</t>
+        </is>
+      </c>
+      <c r="B93" s="4" t="inlineStr">
+        <is>
+          <t>Law firm</t>
+        </is>
+      </c>
+      <c r="C93" s="4" t="inlineStr">
+        <is>
+          <t>Bath (+ Wiltshire offices)</t>
+        </is>
+      </c>
+      <c r="D93" s="4" t="inlineStr">
+        <is>
+          <t>https://awdry.law</t>
+        </is>
+      </c>
+      <c r="E93" s="4" t="inlineStr">
+        <is>
+          <t>info@awdry.law</t>
+        </is>
+      </c>
+      <c r="F93" s="4" t="inlineStr">
+        <is>
+          <t>01225 417111</t>
+        </is>
+      </c>
+      <c r="G93" s="4" t="inlineStr"/>
+      <c r="H93" s="4" t="inlineStr"/>
+      <c r="I93" s="4" t="inlineStr"/>
+      <c r="J93" s="4" t="inlineStr">
+        <is>
+          <t>Multi-office independent covering Bath/Wiltshire; conveyancing + private client = search-driven work</t>
+        </is>
+      </c>
+      <c r="K93" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L93" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M93" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N93" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O93" s="4" t="inlineStr">
+        <is>
+          <t>Modern .law domain rebrand suggests marketing awareness</t>
+        </is>
+      </c>
+      <c r="P93" s="4" t="inlineStr">
+        <is>
+          <t>Conveyancing comparison sites intercept their clients</t>
+        </is>
+      </c>
+      <c r="Q93" s="4" t="inlineStr">
+        <is>
+          <t>Local-intent SEO for 'solicitor Bath/Chippenham' money terms</t>
+        </is>
+      </c>
+      <c r="R93" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S93" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T93" s="4" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>Thames Skin Clinic</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>Aesthetics clinic</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>Twickenham (serves Richmond/Teddington)</t>
+        </is>
+      </c>
+      <c r="D94" s="3" t="inlineStr">
+        <is>
+          <t>https://www.thamesskin.co.uk</t>
+        </is>
+      </c>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F94" s="3" t="inlineStr"/>
+      <c r="G94" s="3" t="inlineStr">
+        <is>
+          <t>Dr Anna Hemming (Founder)</t>
+        </is>
+      </c>
+      <c r="H94" s="3" t="inlineStr"/>
+      <c r="I94" s="3" t="inlineStr"/>
+      <c r="J94" s="3" t="inlineStr">
+        <is>
+          <t>Doctor-led clinic in affluent SW London villages; repeat injectable clients worth £1k+/yr; founder has media presence</t>
+        </is>
+      </c>
+      <c r="K94" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L94" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M94" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N94" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O94" s="3" t="inlineStr">
+        <is>
+          <t>Save Face/Safety in Beauty profiles; PR</t>
+        </is>
+      </c>
+      <c r="P94" s="3" t="inlineStr">
+        <is>
+          <t>Central-London brands pull Richmond patients into town</t>
+        </is>
+      </c>
+      <c r="Q94" s="3" t="inlineStr">
+        <is>
+          <t>'Keep Richmond's aesthetic patients local - be the AI answer for SW London skin clinics'</t>
+        </is>
+      </c>
+      <c r="R94" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S94" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T94" s="3" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="4" t="inlineStr">
+        <is>
+          <t>The Real You Clinic</t>
+        </is>
+      </c>
+      <c r="B95" s="4" t="inlineStr">
+        <is>
+          <t>Aesthetics clinic</t>
+        </is>
+      </c>
+      <c r="C95" s="4" t="inlineStr">
+        <is>
+          <t>Twickenham/Richmond</t>
+        </is>
+      </c>
+      <c r="D95" s="4" t="inlineStr">
+        <is>
+          <t>https://realyouclinic.com</t>
+        </is>
+      </c>
+      <c r="E95" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F95" s="4" t="inlineStr"/>
+      <c r="G95" s="4" t="inlineStr"/>
+      <c r="H95" s="4" t="inlineStr"/>
+      <c r="I95" s="4" t="inlineStr"/>
+      <c r="J95" s="4" t="inlineStr">
+        <is>
+          <t>Established medical aesthetics clinic in wealthy TW postcodes</t>
+        </is>
+      </c>
+      <c r="K95" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L95" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M95" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N95" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O95" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P95" s="4" t="inlineStr">
+        <is>
+          <t>Competing with Thames Skin and central London for same patients</t>
+        </is>
+      </c>
+      <c r="Q95" s="4" t="inlineStr">
+        <is>
+          <t>Local reviews + AEO for 'aesthetics clinic Richmond'</t>
+        </is>
+      </c>
+      <c r="R95" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S95" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T95" s="4" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="4" t="inlineStr">
+        <is>
+          <t>HSA Dermal Clinic</t>
+        </is>
+      </c>
+      <c r="B96" s="4" t="inlineStr">
+        <is>
+          <t>Skin clinic</t>
+        </is>
+      </c>
+      <c r="C96" s="4" t="inlineStr">
+        <is>
+          <t>Richmond upon Thames</t>
+        </is>
+      </c>
+      <c r="D96" s="4" t="inlineStr">
+        <is>
+          <t>https://www.hsadermalclinic.co.uk</t>
+        </is>
+      </c>
+      <c r="E96" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F96" s="4" t="inlineStr"/>
+      <c r="G96" s="4" t="inlineStr"/>
+      <c r="H96" s="4" t="inlineStr"/>
+      <c r="I96" s="4" t="inlineStr"/>
+      <c r="J96" s="4" t="inlineStr">
+        <is>
+          <t>Advanced skin treatments in Richmond; Save Face accredited</t>
+        </is>
+      </c>
+      <c r="K96" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L96" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M96" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N96" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O96" s="4" t="inlineStr">
+        <is>
+          <t>Save Face accreditation</t>
+        </is>
+      </c>
+      <c r="P96" s="4" t="inlineStr">
+        <is>
+          <t>Weak differentiation in crowded local market</t>
+        </is>
+      </c>
+      <c r="Q96" s="4" t="inlineStr">
+        <is>
+          <t>Accreditation-led trust content for local + AI search</t>
+        </is>
+      </c>
+      <c r="R96" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S96" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T96" s="4" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="3" t="inlineStr">
+        <is>
+          <t>Solarsmith</t>
+        </is>
+      </c>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>Solar installer</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>Surrey, London &amp; South East</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>https://www.solarsmith.co.uk</t>
+        </is>
+      </c>
+      <c r="E97" s="3" t="inlineStr">
+        <is>
+          <t>team@solarsmith.co.uk</t>
+        </is>
+      </c>
+      <c r="F97" s="3" t="inlineStr">
+        <is>
+          <t>020 8050 2285</t>
+        </is>
+      </c>
+      <c r="G97" s="3" t="inlineStr"/>
+      <c r="H97" s="3" t="inlineStr"/>
+      <c r="I97" s="3" t="inlineStr"/>
+      <c r="J97" s="3" t="inlineStr">
+        <is>
+          <t>MCS installer covering Surrey's large-roof housing stock; installs £8-20k in wealthy postcodes</t>
+        </is>
+      </c>
+      <c r="K97" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L97" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M97" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N97" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O97" s="3" t="inlineStr">
+        <is>
+          <t>Bookable-online model suggests marketing awareness</t>
+        </is>
+      </c>
+      <c r="P97" s="3" t="inlineStr">
+        <is>
+          <t>Sunsave/EDF/Octopus muscling into domestic solar search</t>
+        </is>
+      </c>
+      <c r="Q97" s="3" t="inlineStr">
+        <is>
+          <t>'Surrey homeowners ask AI if solar is worth it - be the installer in the answer'</t>
+        </is>
+      </c>
+      <c r="R97" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S97" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T97" s="3" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="4" t="inlineStr">
+        <is>
+          <t>Surrey Solar Generation</t>
+        </is>
+      </c>
+      <c r="B98" s="4" t="inlineStr">
+        <is>
+          <t>Solar installer</t>
+        </is>
+      </c>
+      <c r="C98" s="4" t="inlineStr">
+        <is>
+          <t>Surrey (Leatherhead area)</t>
+        </is>
+      </c>
+      <c r="D98" s="4" t="inlineStr">
+        <is>
+          <t>http://discoversolar.co.uk/directory/mcs-installer/surrey/surrey-solar-generation-ltd/</t>
+        </is>
+      </c>
+      <c r="E98" s="4" t="inlineStr">
+        <is>
+          <t>info@surreysolargeneration.com</t>
+        </is>
+      </c>
+      <c r="F98" s="4" t="inlineStr">
+        <is>
+          <t>01372 457750</t>
+        </is>
+      </c>
+      <c r="G98" s="4" t="inlineStr">
+        <is>
+          <t>Simon Prichard (Director)</t>
+        </is>
+      </c>
+      <c r="H98" s="4" t="inlineStr"/>
+      <c r="I98" s="4" t="inlineStr"/>
+      <c r="J98" s="4" t="inlineStr">
+        <is>
+          <t>MCS-certified since 2011; long track record in affluent Surrey</t>
+        </is>
+      </c>
+      <c r="K98" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L98" s="4" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="M98" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N98" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O98" s="4" t="inlineStr">
+        <is>
+          <t>Directory listings only</t>
+        </is>
+      </c>
+      <c r="P98" s="4" t="inlineStr">
+        <is>
+          <t>Minimal web presence in a market being taken by national brands</t>
+        </is>
+      </c>
+      <c r="Q98" s="4" t="inlineStr">
+        <is>
+          <t>Ground-up local SEO: 14 years of installs as review/content ammunition</t>
+        </is>
+      </c>
+      <c r="R98" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S98" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T98" s="4" t="inlineStr">
+        <is>
+          <t>Confirm current website before outreach</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="4" t="inlineStr">
+        <is>
+          <t>Bristol Tuition</t>
+        </is>
+      </c>
+      <c r="B99" s="4" t="inlineStr">
+        <is>
+          <t>Private tuition agency</t>
+        </is>
+      </c>
+      <c r="C99" s="4" t="inlineStr">
+        <is>
+          <t>Bristol</t>
+        </is>
+      </c>
+      <c r="D99" s="4" t="inlineStr">
+        <is>
+          <t>https://bristoltuition.co.uk</t>
+        </is>
+      </c>
+      <c r="E99" s="4" t="inlineStr">
+        <is>
+          <t>enquiries@bristoltuition.co.uk</t>
+        </is>
+      </c>
+      <c r="F99" s="4" t="inlineStr">
+        <is>
+          <t>0117 457 6645</t>
+        </is>
+      </c>
+      <c r="G99" s="4" t="inlineStr"/>
+      <c r="H99" s="4" t="inlineStr"/>
+      <c r="I99" s="4" t="inlineStr"/>
+      <c r="J99" s="4" t="inlineStr">
+        <is>
+          <t>100+ registered tutors; 11+/GCSE demand from Bristol's grammar-adjacent families; per-family LTV high</t>
+        </is>
+      </c>
+      <c r="K99" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L99" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M99" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N99" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O99" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P99" s="4" t="inlineStr">
+        <is>
+          <t>National platforms (Tutorful, MyTutor) absorb local searches</t>
+        </is>
+      </c>
+      <c r="Q99" s="4" t="inlineStr">
+        <is>
+          <t>'Bristol parents ask ChatGPT how to find a tutor - the answer is a national platform, not you'</t>
+        </is>
+      </c>
+      <c r="R99" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S99" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T99" s="4" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="4" t="inlineStr">
+        <is>
+          <t>Greenhouse Learning</t>
+        </is>
+      </c>
+      <c r="B100" s="4" t="inlineStr">
+        <is>
+          <t>Tutoring company</t>
+        </is>
+      </c>
+      <c r="C100" s="4" t="inlineStr">
+        <is>
+          <t>Bristol</t>
+        </is>
+      </c>
+      <c r="D100" s="4" t="inlineStr">
+        <is>
+          <t>https://greenhouselearning.co.uk</t>
+        </is>
+      </c>
+      <c r="E100" s="4" t="inlineStr">
+        <is>
+          <t>rach@greenhouselearning.co.uk</t>
+        </is>
+      </c>
+      <c r="F100" s="4" t="inlineStr"/>
+      <c r="G100" s="4" t="inlineStr">
+        <is>
+          <t>Rachel (Founder)</t>
+        </is>
+      </c>
+      <c r="H100" s="4" t="inlineStr"/>
+      <c r="I100" s="4" t="inlineStr"/>
+      <c r="J100" s="4" t="inlineStr">
+        <is>
+          <t>Personalised 1:1 and small-group tutoring at home/school/centre across Bristol; named founder email</t>
+        </is>
+      </c>
+      <c r="K100" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L100" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M100" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N100" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O100" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P100" s="4" t="inlineStr">
+        <is>
+          <t>Same national-platform squeeze; SEN/personalisation niche underexploited in search</t>
+        </is>
+      </c>
+      <c r="Q100" s="4" t="inlineStr">
+        <is>
+          <t>Niche AEO: own 'SEN tutor Bristol' and personalised-tuition queries</t>
+        </is>
+      </c>
+      <c r="R100" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S100" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T100" s="4" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="4" t="inlineStr">
+        <is>
+          <t>3A Tutors</t>
+        </is>
+      </c>
+      <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t>Tutorial college &amp; exam centre</t>
+        </is>
+      </c>
+      <c r="C101" s="4" t="inlineStr">
+        <is>
+          <t>Bristol</t>
+        </is>
+      </c>
+      <c r="D101" s="4" t="inlineStr">
+        <is>
+          <t>https://www.3at.org.uk</t>
+        </is>
+      </c>
+      <c r="E101" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F101" s="4" t="inlineStr"/>
+      <c r="G101" s="4" t="inlineStr"/>
+      <c r="H101" s="4" t="inlineStr"/>
+      <c r="I101" s="4" t="inlineStr"/>
+      <c r="J101" s="4" t="inlineStr">
+        <is>
+          <t>Independent exam centre + tutorial college; private candidates (home-ed, retakes) pay hundreds per exam sitting</t>
+        </is>
+      </c>
+      <c r="K101" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L101" s="4" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="M101" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N101" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O101" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P101" s="4" t="inlineStr">
+        <is>
+          <t>Home-ed exam-centre searches are high-intent and poorly served locally</t>
+        </is>
+      </c>
+      <c r="Q101" s="4" t="inlineStr">
+        <is>
+          <t>'Own "sit GCSE privately Bristol" - a high-intent niche nobody optimises for'</t>
+        </is>
+      </c>
+      <c r="R101" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S101" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T101" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T70"/>
+  <autoFilter ref="A1:T101"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6808,7 +9420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B52"/>
+  <dimension ref="A1:B69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -6828,7 +9440,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>69</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5">
@@ -6845,23 +9457,23 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Mortgage broker</t>
+          <t>Solar installer</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Chartered accountants</t>
+          <t>Mortgage broker</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -6871,7 +9483,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Independent vet</t>
+          <t>Physiotherapy clinic</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -6881,7 +9493,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Private GP</t>
+          <t>Chartered accountants</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -6891,57 +9503,57 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Private dentist</t>
+          <t>Independent vet</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Physiotherapy clinic</t>
+          <t>Private GP</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Solar installer</t>
+          <t>Family law firm</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Letting agent</t>
+          <t>Architects</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Wedding venue</t>
+          <t>Estate &amp; letting agent</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating / boilers</t>
+          <t>Private dentist</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -6951,7 +9563,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Electrician</t>
+          <t>Law firm</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -6961,7 +9573,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Event &amp; wedding caterer</t>
+          <t>Letting agent</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -6971,7 +9583,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Personal training studio</t>
+          <t>Wedding venue</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -6981,7 +9593,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Family law firm</t>
+          <t>Private tuition agency</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -6991,7 +9603,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Chiropractor</t>
+          <t>Plumbing &amp; heating / boilers</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -7001,67 +9613,67 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Dentist / Orthodontics</t>
+          <t>Electrician</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Specialist dental/implant clinic</t>
+          <t>Event &amp; wedding caterer</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Law firm</t>
+          <t>Personal training studio</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Boutique corporate law firm</t>
+          <t>Chiropractor</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Cosmetic/aesthetics clinic</t>
+          <t>Orthodontist</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Skin &amp; laser clinic</t>
+          <t>Aesthetics clinic</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Mortgage broker / financial adviser</t>
+          <t>Dentist / Orthodontics</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -7071,7 +9683,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Architects (RIBA chartered)</t>
+          <t>Specialist dental/implant clinic</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -7081,7 +9693,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Recruitment agency (tech/startups)</t>
+          <t>Boutique corporate law firm</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -7091,7 +9703,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Recruitment agency (IT/data)</t>
+          <t>Cosmetic/aesthetics clinic</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -7101,7 +9713,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Independent vet (24/7 emergency)</t>
+          <t>Skin &amp; laser clinic</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -7111,7 +9723,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Interior design studio</t>
+          <t>Mortgage broker / financial adviser</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -7121,7 +9733,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Letting &amp; estate agent</t>
+          <t>Architects (RIBA chartered)</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -7131,7 +9743,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Cosmetic clinic (injectables)</t>
+          <t>Recruitment agency (tech/startups)</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -7141,7 +9753,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Cosmetic/anti-ageing clinic</t>
+          <t>Recruitment agency (IT/data)</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -7151,7 +9763,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Yoga &amp; reformer pilates studio</t>
+          <t>Independent vet (24/7 emergency)</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -7161,7 +9773,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Reformer pilates studio</t>
+          <t>Interior design studio</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -7171,7 +9783,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Financial adviser / wealth management</t>
+          <t>Letting &amp; estate agent</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -7181,7 +9793,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Wealth management</t>
+          <t>Cosmetic clinic (injectables)</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -7191,7 +9803,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Private tuition agency</t>
+          <t>Cosmetic/anti-ageing clinic</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -7201,7 +9813,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Private tuition &amp; education consultancy</t>
+          <t>Yoga &amp; reformer pilates studio</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -7211,7 +9823,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Osteopath</t>
+          <t>Reformer pilates studio</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -7221,7 +9833,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Osteopathy clinic</t>
+          <t>Financial adviser / wealth management</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -7231,7 +9843,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Design &amp; build / home renovation</t>
+          <t>Wealth management</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -7241,7 +9853,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Builders / building contractor</t>
+          <t>Private tuition &amp; education consultancy</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -7251,7 +9863,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Roofer</t>
+          <t>Osteopath</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -7261,7 +9873,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Home care / live-in care</t>
+          <t>Osteopathy clinic</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -7271,7 +9883,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Private day nurseries</t>
+          <t>Design &amp; build / home renovation</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -7281,7 +9893,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Personal training &amp; wellness studio</t>
+          <t>Builders / building contractor</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -7291,7 +9903,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Mortgage &amp; insurance broker</t>
+          <t>Roofer</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -7301,10 +9913,180 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
+          <t>Home care / live-in care</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Private day nurseries</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Personal training &amp; wellness studio</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Mortgage &amp; insurance broker</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>Business consultancy</t>
         </is>
       </c>
-      <c r="B52" t="n">
+      <c r="B56" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Interior designer (period homes)</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Landscape design &amp; build</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Estate agent (premium)</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Interior designer</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Garden design &amp; landscaping</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Legal recruitment</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Independent gym &amp; health club</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Independent gym</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Physiotherapy (sports)</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Letting agent / property management</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Skin clinic</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Tutoring company</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Tutorial college &amp; exam centre</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 4: +28 prospects (128 total) - Wimbledon/Chiswick agents, employment law, surveyors, Bath dentists, Surrey builders, SW London nurseries
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$129</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T101"/>
+  <dimension ref="A1:T129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -9408,8 +9408,2328 @@
       </c>
       <c r="T101" s="4" t="inlineStr"/>
     </row>
+    <row r="102">
+      <c r="A102" s="3" t="inlineStr">
+        <is>
+          <t>Elizabeth Wightwick</t>
+        </is>
+      </c>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>Estate &amp; letting agent</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>Wimbledon Village, London SW19</t>
+        </is>
+      </c>
+      <c r="D102" s="3" t="inlineStr">
+        <is>
+          <t>https://www.elizabeth-wightwick.co.uk</t>
+        </is>
+      </c>
+      <c r="E102" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F102" s="3" t="inlineStr"/>
+      <c r="G102" s="3" t="inlineStr">
+        <is>
+          <t>Elizabeth Wightwick (Founder)</t>
+        </is>
+      </c>
+      <c r="H102" s="3" t="inlineStr"/>
+      <c r="I102" s="3" t="inlineStr"/>
+      <c r="J102" s="3" t="inlineStr">
+        <is>
+          <t>Family-run independent in Wimbledon Village's premium market; instructions worth £10k+ in fees</t>
+        </is>
+      </c>
+      <c r="K102" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L102" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M102" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N102" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O102" s="3" t="inlineStr">
+        <is>
+          <t>Portal listings</t>
+        </is>
+      </c>
+      <c r="P102" s="3" t="inlineStr">
+        <is>
+          <t>Savills/Hamptons/Foxtons own Wimbledon search results</t>
+        </is>
+      </c>
+      <c r="Q102" s="3" t="inlineStr">
+        <is>
+          <t>'Village sellers want a village agent - make Google and ChatGPT agree'</t>
+        </is>
+      </c>
+      <c r="R102" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S102" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T102" s="3" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="4" t="inlineStr">
+        <is>
+          <t>C James &amp; Co</t>
+        </is>
+      </c>
+      <c r="B103" s="4" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C103" s="4" t="inlineStr">
+        <is>
+          <t>Wimbledon, London SW19</t>
+        </is>
+      </c>
+      <c r="D103" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cjames.co.uk</t>
+        </is>
+      </c>
+      <c r="E103" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F103" s="4" t="inlineStr"/>
+      <c r="G103" s="4" t="inlineStr">
+        <is>
+          <t>Suzanne (Founder)</t>
+        </is>
+      </c>
+      <c r="H103" s="4" t="inlineStr"/>
+      <c r="I103" s="4" t="inlineStr"/>
+      <c r="J103" s="4" t="inlineStr">
+        <is>
+          <t>Wimbledon's longest-established solely independent agent (1991); sales + lettings + management</t>
+        </is>
+      </c>
+      <c r="K103" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L103" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M103" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N103" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O103" s="4" t="inlineStr">
+        <is>
+          <t>Portal listings</t>
+        </is>
+      </c>
+      <c r="P103" s="4" t="inlineStr">
+        <is>
+          <t>30-year reputation invisible in modern search</t>
+        </is>
+      </c>
+      <c r="Q103" s="4" t="inlineStr">
+        <is>
+          <t>Heritage-into-authority content play</t>
+        </is>
+      </c>
+      <c r="R103" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S103" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T103" s="4" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="3" t="inlineStr">
+        <is>
+          <t>Andrew Nunn &amp; Associates</t>
+        </is>
+      </c>
+      <c r="B104" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>Chiswick / Bedford Park, London W4</t>
+        </is>
+      </c>
+      <c r="D104" s="3" t="inlineStr">
+        <is>
+          <t>https://www.andrewnunnassociates.co.uk</t>
+        </is>
+      </c>
+      <c r="E104" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F104" s="3" t="inlineStr"/>
+      <c r="G104" s="3" t="inlineStr">
+        <is>
+          <t>Andrew Nunn (Owner)</t>
+        </is>
+      </c>
+      <c r="H104" s="3" t="inlineStr"/>
+      <c r="I104" s="3" t="inlineStr"/>
+      <c r="J104" s="3" t="inlineStr">
+        <is>
+          <t>Owner-run independent in affluent Bedford Park conservation area; premium period stock</t>
+        </is>
+      </c>
+      <c r="K104" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L104" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M104" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N104" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O104" s="3" t="inlineStr">
+        <is>
+          <t>Local reputation</t>
+        </is>
+      </c>
+      <c r="P104" s="3" t="inlineStr">
+        <is>
+          <t>Corporate agents flood W4 searches; independents rely on word-of-mouth</t>
+        </is>
+      </c>
+      <c r="Q104" s="3" t="inlineStr">
+        <is>
+          <t>'Bedford Park owners ask AI who knows their conservation area best - be the answer'</t>
+        </is>
+      </c>
+      <c r="R104" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S104" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T104" s="3" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="3" t="inlineStr">
+        <is>
+          <t>BDBF LLP</t>
+        </is>
+      </c>
+      <c r="B105" s="3" t="inlineStr">
+        <is>
+          <t>Employment law firm</t>
+        </is>
+      </c>
+      <c r="C105" s="3" t="inlineStr">
+        <is>
+          <t>City of London</t>
+        </is>
+      </c>
+      <c r="D105" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bdbf.co.uk</t>
+        </is>
+      </c>
+      <c r="E105" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F105" s="3" t="inlineStr"/>
+      <c r="G105" s="3" t="inlineStr"/>
+      <c r="H105" s="3" t="inlineStr"/>
+      <c r="I105" s="3" t="inlineStr"/>
+      <c r="J105" s="3" t="inlineStr">
+        <is>
+          <t>Independent employment/partnership law boutique; exec severance cases worth £10-50k in fees; City catchment</t>
+        </is>
+      </c>
+      <c r="K105" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L105" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M105" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N105" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O105" s="3" t="inlineStr">
+        <is>
+          <t>Professional site; directory rankings</t>
+        </is>
+      </c>
+      <c r="P105" s="3" t="inlineStr">
+        <is>
+          <t>Executives research severance rights via AI before choosing lawyers - big firms get cited</t>
+        </is>
+      </c>
+      <c r="Q105" s="3" t="inlineStr">
+        <is>
+          <t>AEO for the questions executives ask AI about exit packages</t>
+        </is>
+      </c>
+      <c r="R105" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S105" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T105" s="3" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="3" t="inlineStr">
+        <is>
+          <t>Doyle Clayton</t>
+        </is>
+      </c>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>Employment law firm</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>London &amp; Reading</t>
+        </is>
+      </c>
+      <c r="D106" s="3" t="inlineStr">
+        <is>
+          <t>https://www.doyleclayton.co.uk</t>
+        </is>
+      </c>
+      <c r="E106" s="3" t="inlineStr">
+        <is>
+          <t>info@doyleclayton.co.uk</t>
+        </is>
+      </c>
+      <c r="F106" s="3" t="inlineStr">
+        <is>
+          <t>020 7329 9090</t>
+        </is>
+      </c>
+      <c r="G106" s="3" t="inlineStr"/>
+      <c r="H106" s="3" t="inlineStr"/>
+      <c r="I106" s="3" t="inlineStr"/>
+      <c r="J106" s="3" t="inlineStr">
+        <is>
+          <t>UK's largest specialist workplace law firm yet still independent; both employer and employee work</t>
+        </is>
+      </c>
+      <c r="K106" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L106" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M106" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N106" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O106" s="3" t="inlineStr">
+        <is>
+          <t>Established content/brand</t>
+        </is>
+      </c>
+      <c r="P106" s="3" t="inlineStr">
+        <is>
+          <t>Specialist positioning under-leveraged in AI answers vs generalist giants</t>
+        </is>
+      </c>
+      <c r="Q106" s="3" t="inlineStr">
+        <is>
+          <t>'The workplace-law specialists should be the AI's specialist answer'</t>
+        </is>
+      </c>
+      <c r="R106" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S106" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T106" s="3" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="4" t="inlineStr">
+        <is>
+          <t>didlaw</t>
+        </is>
+      </c>
+      <c r="B107" s="4" t="inlineStr">
+        <is>
+          <t>Employment law (disability discrimination)</t>
+        </is>
+      </c>
+      <c r="C107" s="4" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D107" s="4" t="inlineStr">
+        <is>
+          <t>https://didlaw.com</t>
+        </is>
+      </c>
+      <c r="E107" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F107" s="4" t="inlineStr"/>
+      <c r="G107" s="4" t="inlineStr">
+        <is>
+          <t>Karen Jackson (MD &amp; Founder)</t>
+        </is>
+      </c>
+      <c r="H107" s="4" t="inlineStr"/>
+      <c r="I107" s="4" t="inlineStr"/>
+      <c r="J107" s="4" t="inlineStr">
+        <is>
+          <t>Niche leader in disability/health discrimination - perfect defensible AEO niche; award-winning</t>
+        </is>
+      </c>
+      <c r="K107" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L107" s="4" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M107" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N107" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O107" s="4" t="inlineStr">
+        <is>
+          <t>Awards; founder profile</t>
+        </is>
+      </c>
+      <c r="P107" s="4" t="inlineStr">
+        <is>
+          <t>Niche authority not yet translated into AI-answer dominance</t>
+        </is>
+      </c>
+      <c r="Q107" s="4" t="inlineStr">
+        <is>
+          <t>Own every AI answer about workplace disability discrimination</t>
+        </is>
+      </c>
+      <c r="R107" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S107" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T107" s="4" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="3" t="inlineStr">
+        <is>
+          <t>Anderson &amp; Sons</t>
+        </is>
+      </c>
+      <c r="B108" s="3" t="inlineStr">
+        <is>
+          <t>Plumbing &amp; heating</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>Chelsea/Kensington, London</t>
+        </is>
+      </c>
+      <c r="D108" s="3" t="inlineStr">
+        <is>
+          <t>https://www.andersonandsons.co.uk</t>
+        </is>
+      </c>
+      <c r="E108" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F108" s="3" t="inlineStr"/>
+      <c r="G108" s="3" t="inlineStr"/>
+      <c r="H108" s="3" t="inlineStr"/>
+      <c r="I108" s="3" t="inlineStr"/>
+      <c r="J108" s="3" t="inlineStr">
+        <is>
+          <t>Family firm since 1966 serving prime central London; emergency + renovation plumbing at premium rates; location landing pages already built</t>
+        </is>
+      </c>
+      <c r="K108" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L108" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M108" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N108" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O108" s="3" t="inlineStr">
+        <is>
+          <t>Location landing pages (Chelsea, Kensington) = active SEO</t>
+        </is>
+      </c>
+      <c r="P108" s="3" t="inlineStr">
+        <is>
+          <t>Aggregators (AllService4U, Checkatrade) intercept emergency searches</t>
+        </is>
+      </c>
+      <c r="Q108" s="3" t="inlineStr">
+        <is>
+          <t>'55 years in Chelsea should beat any aggregator - in AI answers it doesn't yet'</t>
+        </is>
+      </c>
+      <c r="R108" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S108" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T108" s="3" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="4" t="inlineStr">
+        <is>
+          <t>Pippo Plumbers</t>
+        </is>
+      </c>
+      <c r="B109" s="4" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C109" s="4" t="inlineStr">
+        <is>
+          <t>Kensington &amp; Chelsea, London</t>
+        </is>
+      </c>
+      <c r="D109" s="4" t="inlineStr">
+        <is>
+          <t>https://pippoplumbers.co.uk</t>
+        </is>
+      </c>
+      <c r="E109" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F109" s="4" t="inlineStr"/>
+      <c r="G109" s="4" t="inlineStr"/>
+      <c r="H109" s="4" t="inlineStr"/>
+      <c r="I109" s="4" t="inlineStr"/>
+      <c r="J109" s="4" t="inlineStr">
+        <is>
+          <t>Growing K&amp;C plumbing firm since 2018; premium postcode = premium job values</t>
+        </is>
+      </c>
+      <c r="K109" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L109" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M109" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N109" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O109" s="4" t="inlineStr">
+        <is>
+          <t>Area landing pages</t>
+        </is>
+      </c>
+      <c r="P109" s="4" t="inlineStr">
+        <is>
+          <t>Young brand competing with 50-year incumbents and aggregators</t>
+        </is>
+      </c>
+      <c r="Q109" s="4" t="inlineStr">
+        <is>
+          <t>Ground-floor local SEO + review engine</t>
+        </is>
+      </c>
+      <c r="R109" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S109" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T109" s="4" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="4" t="inlineStr">
+        <is>
+          <t>The Pure Practice</t>
+        </is>
+      </c>
+      <c r="B110" s="4" t="inlineStr">
+        <is>
+          <t>Physiotherapy clinic</t>
+        </is>
+      </c>
+      <c r="C110" s="4" t="inlineStr">
+        <is>
+          <t>Central Bath</t>
+        </is>
+      </c>
+      <c r="D110" s="4" t="inlineStr">
+        <is>
+          <t>https://thepurepractice.co.uk</t>
+        </is>
+      </c>
+      <c r="E110" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F110" s="4" t="inlineStr"/>
+      <c r="G110" s="4" t="inlineStr">
+        <is>
+          <t>Sonja Bass (Founder)</t>
+        </is>
+      </c>
+      <c r="H110" s="4" t="inlineStr"/>
+      <c r="I110" s="4" t="inlineStr"/>
+      <c r="J110" s="4" t="inlineStr">
+        <is>
+          <t>Founder with 20+ years Bath experience; central clinic; self-pay physio in affluent city</t>
+        </is>
+      </c>
+      <c r="K110" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L110" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M110" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N110" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O110" s="4" t="inlineStr">
+        <is>
+          <t>Online booking</t>
+        </is>
+      </c>
+      <c r="P110" s="4" t="inlineStr">
+        <is>
+          <t>Hospital brands (Sulis, Ascenti) and Team Bath absorb physio searches</t>
+        </is>
+      </c>
+      <c r="Q110" s="4" t="inlineStr">
+        <is>
+          <t>'Bath's independent physio should be Bath's AI answer'</t>
+        </is>
+      </c>
+      <c r="R110" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S110" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T110" s="4" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="4" t="inlineStr">
+        <is>
+          <t>Hybrid Health Clinic</t>
+        </is>
+      </c>
+      <c r="B111" s="4" t="inlineStr">
+        <is>
+          <t>Sports physio &amp; massage</t>
+        </is>
+      </c>
+      <c r="C111" s="4" t="inlineStr">
+        <is>
+          <t>Milsom Street, Bath</t>
+        </is>
+      </c>
+      <c r="D111" s="4" t="inlineStr">
+        <is>
+          <t>https://www.hybridhealthphysio.com</t>
+        </is>
+      </c>
+      <c r="E111" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F111" s="4" t="inlineStr"/>
+      <c r="G111" s="4" t="inlineStr"/>
+      <c r="H111" s="4" t="inlineStr"/>
+      <c r="I111" s="4" t="inlineStr"/>
+      <c r="J111" s="4" t="inlineStr">
+        <is>
+          <t>Prime Milsom Street location; sports injury + massage; 20+ years experience</t>
+        </is>
+      </c>
+      <c r="K111" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L111" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M111" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N111" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O111" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P111" s="4" t="inlineStr">
+        <is>
+          <t>Same hospital-brand squeeze; thin differentiation online</t>
+        </is>
+      </c>
+      <c r="Q111" s="4" t="inlineStr">
+        <is>
+          <t>Local + AEO for 'sports physio Bath'</t>
+        </is>
+      </c>
+      <c r="R111" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S111" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T111" s="4" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="3" t="inlineStr">
+        <is>
+          <t>Arkenstone Wealth Management</t>
+        </is>
+      </c>
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t>Financial adviser / wealth management</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>Wimbledon Village, London SW19</t>
+        </is>
+      </c>
+      <c r="D112" s="3" t="inlineStr">
+        <is>
+          <t>https://www.arkenstonewealth.co.uk</t>
+        </is>
+      </c>
+      <c r="E112" s="3" t="inlineStr">
+        <is>
+          <t>advice@arkenstonewealth.co.uk</t>
+        </is>
+      </c>
+      <c r="F112" s="3" t="inlineStr">
+        <is>
+          <t>020 8323 8881</t>
+        </is>
+      </c>
+      <c r="G112" s="3" t="inlineStr"/>
+      <c r="H112" s="3" t="inlineStr"/>
+      <c r="I112" s="3" t="inlineStr"/>
+      <c r="J112" s="3" t="inlineStr">
+        <is>
+          <t>IFA practice in Wimbledon Village serving SW London professionals; client LTV in tens of thousands</t>
+        </is>
+      </c>
+      <c r="K112" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L112" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M112" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N112" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O112" s="3" t="inlineStr">
+        <is>
+          <t>Directory profiles (Unbiased)</t>
+        </is>
+      </c>
+      <c r="P112" s="3" t="inlineStr">
+        <is>
+          <t>Unbiased/VouchedFor intercept advice-seekers before they find local firms</t>
+        </is>
+      </c>
+      <c r="Q112" s="3" t="inlineStr">
+        <is>
+          <t>'Bypass the directories: be the direct AI answer for "IFA Wimbledon"'</t>
+        </is>
+      </c>
+      <c r="R112" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S112" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T112" s="3" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="3" t="inlineStr">
+        <is>
+          <t>Harding Chartered Surveyors</t>
+        </is>
+      </c>
+      <c r="B113" s="3" t="inlineStr">
+        <is>
+          <t>Chartered surveyors (party wall/building)</t>
+        </is>
+      </c>
+      <c r="C113" s="3" t="inlineStr">
+        <is>
+          <t>Piccadilly + offices across London</t>
+        </is>
+      </c>
+      <c r="D113" s="3" t="inlineStr">
+        <is>
+          <t>https://hardingsurveyors.co.uk</t>
+        </is>
+      </c>
+      <c r="E113" s="3" t="inlineStr">
+        <is>
+          <t>enquiries@hardingsurveyors.co.uk</t>
+        </is>
+      </c>
+      <c r="F113" s="3" t="inlineStr">
+        <is>
+          <t>020 7736 2383</t>
+        </is>
+      </c>
+      <c r="G113" s="3" t="inlineStr"/>
+      <c r="H113" s="3" t="inlineStr"/>
+      <c r="I113" s="3" t="inlineStr"/>
+      <c r="J113" s="3" t="inlineStr">
+        <is>
+          <t>RICS firm with party-wall specialism; London's renovation boom = constant high-intent searches; already builds location pages</t>
+        </is>
+      </c>
+      <c r="K113" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L113" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M113" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N113" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O113" s="3" t="inlineStr">
+        <is>
+          <t>Location pages (Piccadilly office etc.) = SEO investment</t>
+        </is>
+      </c>
+      <c r="P113" s="3" t="inlineStr">
+        <is>
+          <t>Party-wall queries increasingly answered by AI summaries citing content-rich rivals</t>
+        </is>
+      </c>
+      <c r="Q113" s="3" t="inlineStr">
+        <is>
+          <t>'Every London extension needs a party wall surveyor - own that AI answer'</t>
+        </is>
+      </c>
+      <c r="R113" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S113" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T113" s="3" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="3" t="inlineStr">
+        <is>
+          <t>Peter Barry Surveyors</t>
+        </is>
+      </c>
+      <c r="B114" s="3" t="inlineStr">
+        <is>
+          <t>Chartered surveyors</t>
+        </is>
+      </c>
+      <c r="C114" s="3" t="inlineStr">
+        <is>
+          <t>Fulham, SW London</t>
+        </is>
+      </c>
+      <c r="D114" s="3" t="inlineStr">
+        <is>
+          <t>https://www.peterbarry.co.uk</t>
+        </is>
+      </c>
+      <c r="E114" s="3" t="inlineStr">
+        <is>
+          <t>surveying@peterbarry.co.uk</t>
+        </is>
+      </c>
+      <c r="F114" s="3" t="inlineStr">
+        <is>
+          <t>020 7471 8932</t>
+        </is>
+      </c>
+      <c r="G114" s="3" t="inlineStr"/>
+      <c r="H114" s="3" t="inlineStr"/>
+      <c r="I114" s="3" t="inlineStr"/>
+      <c r="J114" s="3" t="inlineStr">
+        <is>
+          <t>Established SW London surveyors; party wall + building surveys tied to the extension boom</t>
+        </is>
+      </c>
+      <c r="K114" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L114" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M114" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N114" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O114" s="3" t="inlineStr">
+        <is>
+          <t>Office landing pages</t>
+        </is>
+      </c>
+      <c r="P114" s="3" t="inlineStr">
+        <is>
+          <t>Competing with Harding etc. for identical high-intent searches</t>
+        </is>
+      </c>
+      <c r="Q114" s="3" t="inlineStr">
+        <is>
+          <t>Local-borough AEO: own Wandsworth/Fulham survey queries</t>
+        </is>
+      </c>
+      <c r="R114" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S114" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T114" s="3" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="4" t="inlineStr">
+        <is>
+          <t>Tayross Associates</t>
+        </is>
+      </c>
+      <c r="B115" s="4" t="inlineStr">
+        <is>
+          <t>Chartered building surveyors</t>
+        </is>
+      </c>
+      <c r="C115" s="4" t="inlineStr">
+        <is>
+          <t>West London</t>
+        </is>
+      </c>
+      <c r="D115" s="4" t="inlineStr">
+        <is>
+          <t>https://www.tayross.com</t>
+        </is>
+      </c>
+      <c r="E115" s="4" t="inlineStr">
+        <is>
+          <t>carl@tayross.com</t>
+        </is>
+      </c>
+      <c r="F115" s="4" t="inlineStr">
+        <is>
+          <t>020 8426 1448</t>
+        </is>
+      </c>
+      <c r="G115" s="4" t="inlineStr">
+        <is>
+          <t>Carl (Principal)</t>
+        </is>
+      </c>
+      <c r="H115" s="4" t="inlineStr"/>
+      <c r="I115" s="4" t="inlineStr"/>
+      <c r="J115" s="4" t="inlineStr">
+        <is>
+          <t>RICS/CIOB consultancy - surveys, party wall, disputes; direct principal email</t>
+        </is>
+      </c>
+      <c r="K115" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L115" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M115" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N115" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O115" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P115" s="4" t="inlineStr">
+        <is>
+          <t>Small firm invisible next to bigger survey brands</t>
+        </is>
+      </c>
+      <c r="Q115" s="4" t="inlineStr">
+        <is>
+          <t>Niche content: boundary disputes + EWS1 as AEO wedges</t>
+        </is>
+      </c>
+      <c r="R115" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S115" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T115" s="4" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="4" t="inlineStr">
+        <is>
+          <t>MGN Events</t>
+        </is>
+      </c>
+      <c r="B116" s="4" t="inlineStr">
+        <is>
+          <t>Event management agency</t>
+        </is>
+      </c>
+      <c r="C116" s="4" t="inlineStr">
+        <is>
+          <t>London &amp; Surrey</t>
+        </is>
+      </c>
+      <c r="D116" s="4" t="inlineStr">
+        <is>
+          <t>https://www.mgnevents.co.uk</t>
+        </is>
+      </c>
+      <c r="E116" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F116" s="4" t="inlineStr"/>
+      <c r="G116" s="4" t="inlineStr"/>
+      <c r="H116" s="4" t="inlineStr"/>
+      <c r="I116" s="4" t="inlineStr"/>
+      <c r="J116" s="4" t="inlineStr">
+        <is>
+          <t>Award-winning creative agency for corporate + private events worth £20-200k each</t>
+        </is>
+      </c>
+      <c r="K116" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L116" s="4" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M116" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N116" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O116" s="4" t="inlineStr">
+        <is>
+          <t>Awards; polished site</t>
+        </is>
+      </c>
+      <c r="P116" s="4" t="inlineStr">
+        <is>
+          <t>Agency discovery moving to AI shortlists; referral-dependent</t>
+        </is>
+      </c>
+      <c r="Q116" s="4" t="inlineStr">
+        <is>
+          <t>'CMOs ask ChatGPT for event agency shortlists - get on them'</t>
+        </is>
+      </c>
+      <c r="R116" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S116" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T116" s="4" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="4" t="inlineStr">
+        <is>
+          <t>Eventify</t>
+        </is>
+      </c>
+      <c r="B117" s="4" t="inlineStr">
+        <is>
+          <t>Event management agency</t>
+        </is>
+      </c>
+      <c r="C117" s="4" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D117" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eventifyuk.com</t>
+        </is>
+      </c>
+      <c r="E117" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F117" s="4" t="inlineStr"/>
+      <c r="G117" s="4" t="inlineStr"/>
+      <c r="H117" s="4" t="inlineStr"/>
+      <c r="I117" s="4" t="inlineStr"/>
+      <c r="J117" s="4" t="inlineStr">
+        <is>
+          <t>Independent venue-finding + events agency; explicitly unbiased positioning = good content angle</t>
+        </is>
+      </c>
+      <c r="K117" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L117" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M117" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N117" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O117" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P117" s="4" t="inlineStr">
+        <is>
+          <t>Venue-finding is being eaten by AI directly - must become the cited source</t>
+        </is>
+      </c>
+      <c r="Q117" s="4" t="inlineStr">
+        <is>
+          <t>Position as the transparent venue-data source AI engines cite</t>
+        </is>
+      </c>
+      <c r="R117" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S117" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T117" s="4" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="3" t="inlineStr">
+        <is>
+          <t>Bristol Osteopaths</t>
+        </is>
+      </c>
+      <c r="B118" s="3" t="inlineStr">
+        <is>
+          <t>Osteopathy clinics</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="inlineStr">
+        <is>
+          <t>3 sites: Wells Rd, Queen Charlotte St, Sneyd Park Bristol</t>
+        </is>
+      </c>
+      <c r="D118" s="3" t="inlineStr">
+        <is>
+          <t>https://bristolosteopaths.com</t>
+        </is>
+      </c>
+      <c r="E118" s="3" t="inlineStr">
+        <is>
+          <t>wellsroad@bristolosteopaths.com</t>
+        </is>
+      </c>
+      <c r="F118" s="3" t="inlineStr">
+        <is>
+          <t>0117 971 0221</t>
+        </is>
+      </c>
+      <c r="G118" s="3" t="inlineStr"/>
+      <c r="H118" s="3" t="inlineStr"/>
+      <c r="I118" s="3" t="inlineStr"/>
+      <c r="J118" s="3" t="inlineStr">
+        <is>
+          <t>Three-site osteopathy group; multi-decade presence; self-pay treatment courses</t>
+        </is>
+      </c>
+      <c r="K118" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L118" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M118" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N118" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O118" s="3" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P118" s="3" t="inlineStr">
+        <is>
+          <t>Three locations but one weak web presence; physios and chiros take the same back-pain searches</t>
+        </is>
+      </c>
+      <c r="Q118" s="3" t="inlineStr">
+        <is>
+          <t>Per-site local SEO: 3 clinics should own 3 catchments</t>
+        </is>
+      </c>
+      <c r="R118" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S118" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T118" s="3" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="4" t="inlineStr">
+        <is>
+          <t>Chandos Clinic Osteopaths</t>
+        </is>
+      </c>
+      <c r="B119" s="4" t="inlineStr">
+        <is>
+          <t>Osteopathy clinic</t>
+        </is>
+      </c>
+      <c r="C119" s="4" t="inlineStr">
+        <is>
+          <t>Bristol</t>
+        </is>
+      </c>
+      <c r="D119" s="4" t="inlineStr">
+        <is>
+          <t>https://chandosclinic.co.uk</t>
+        </is>
+      </c>
+      <c r="E119" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F119" s="4" t="inlineStr">
+        <is>
+          <t>0117 974 5084</t>
+        </is>
+      </c>
+      <c r="G119" s="4" t="inlineStr"/>
+      <c r="H119" s="4" t="inlineStr"/>
+      <c r="I119" s="4" t="inlineStr"/>
+      <c r="J119" s="4" t="inlineStr">
+        <is>
+          <t>Established holistic clinic in Bristol; loyal patient base</t>
+        </is>
+      </c>
+      <c r="K119" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L119" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M119" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N119" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O119" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P119" s="4" t="inlineStr">
+        <is>
+          <t>Same local-visibility battle as peers</t>
+        </is>
+      </c>
+      <c r="Q119" s="4" t="inlineStr">
+        <is>
+          <t>Quick-win local SEO + reviews</t>
+        </is>
+      </c>
+      <c r="R119" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S119" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T119" s="4" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="3" t="inlineStr">
+        <is>
+          <t>Bath Spa Dentistry</t>
+        </is>
+      </c>
+      <c r="B120" s="3" t="inlineStr">
+        <is>
+          <t>Private dentist</t>
+        </is>
+      </c>
+      <c r="C120" s="3" t="inlineStr">
+        <is>
+          <t>James St West, Bath</t>
+        </is>
+      </c>
+      <c r="D120" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bathspadentistry.com</t>
+        </is>
+      </c>
+      <c r="E120" s="3" t="inlineStr">
+        <is>
+          <t>reception@bathspadentistry.com</t>
+        </is>
+      </c>
+      <c r="F120" s="3" t="inlineStr">
+        <is>
+          <t>01225 464346</t>
+        </is>
+      </c>
+      <c r="G120" s="3" t="inlineStr"/>
+      <c r="H120" s="3" t="inlineStr"/>
+      <c r="I120" s="3" t="inlineStr"/>
+      <c r="J120" s="3" t="inlineStr">
+        <is>
+          <t>Multi-award-winning private practice in Bath; cosmetic + implant work at Bath prices</t>
+        </is>
+      </c>
+      <c r="K120" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L120" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M120" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N120" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O120" s="3" t="inlineStr">
+        <is>
+          <t>Award wins promoted on site</t>
+        </is>
+      </c>
+      <c r="P120" s="3" t="inlineStr">
+        <is>
+          <t>Awards don't show up in AI answers; Bristol clinics pull Bath patients</t>
+        </is>
+      </c>
+      <c r="Q120" s="3" t="inlineStr">
+        <is>
+          <t>'Multi-award-winning should mean AI-recommended - let's close that gap'</t>
+        </is>
+      </c>
+      <c r="R120" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S120" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T120" s="3" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="3" t="inlineStr">
+        <is>
+          <t>Edgar Buildings Dental &amp; Implant Clinic</t>
+        </is>
+      </c>
+      <c r="B121" s="3" t="inlineStr">
+        <is>
+          <t>Private dentist / implants</t>
+        </is>
+      </c>
+      <c r="C121" s="3" t="inlineStr">
+        <is>
+          <t>Edgar Buildings, Bath</t>
+        </is>
+      </c>
+      <c r="D121" s="3" t="inlineStr">
+        <is>
+          <t>https://www.smileofconfidence.com</t>
+        </is>
+      </c>
+      <c r="E121" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F121" s="3" t="inlineStr"/>
+      <c r="G121" s="3" t="inlineStr"/>
+      <c r="H121" s="3" t="inlineStr"/>
+      <c r="I121" s="3" t="inlineStr"/>
+      <c r="J121" s="3" t="inlineStr">
+        <is>
+          <t>Implant-focused practice in prestige George St address; £3-10k cases</t>
+        </is>
+      </c>
+      <c r="K121" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L121" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M121" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N121" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O121" s="3" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P121" s="3" t="inlineStr">
+        <is>
+          <t>Implant searches in Bath poorly contested - winnable</t>
+        </is>
+      </c>
+      <c r="Q121" s="3" t="inlineStr">
+        <is>
+          <t>'Own "dental implants Bath" before anyone else wakes up'</t>
+        </is>
+      </c>
+      <c r="R121" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S121" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T121" s="3" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="4" t="inlineStr">
+        <is>
+          <t>Widcombe Dental Practice</t>
+        </is>
+      </c>
+      <c r="B122" s="4" t="inlineStr">
+        <is>
+          <t>Private dentist</t>
+        </is>
+      </c>
+      <c r="C122" s="4" t="inlineStr">
+        <is>
+          <t>Widcombe, Bath</t>
+        </is>
+      </c>
+      <c r="D122" s="4" t="inlineStr">
+        <is>
+          <t>https://widcombedentalpractice.co.uk</t>
+        </is>
+      </c>
+      <c r="E122" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F122" s="4" t="inlineStr">
+        <is>
+          <t>01225 317 681</t>
+        </is>
+      </c>
+      <c r="G122" s="4" t="inlineStr"/>
+      <c r="H122" s="4" t="inlineStr"/>
+      <c r="I122" s="4" t="inlineStr"/>
+      <c r="J122" s="4" t="inlineStr">
+        <is>
+          <t>Neighbourhood private practice in affluent Widcombe</t>
+        </is>
+      </c>
+      <c r="K122" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L122" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M122" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N122" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O122" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P122" s="4" t="inlineStr">
+        <is>
+          <t>Village practice with village-scale visibility</t>
+        </is>
+      </c>
+      <c r="Q122" s="4" t="inlineStr">
+        <is>
+          <t>Entry-tier local SEO package</t>
+        </is>
+      </c>
+      <c r="R122" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S122" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T122" s="4" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="4" t="inlineStr">
+        <is>
+          <t>Hogs Back Builders</t>
+        </is>
+      </c>
+      <c r="B123" s="4" t="inlineStr">
+        <is>
+          <t>Design &amp; build</t>
+        </is>
+      </c>
+      <c r="C123" s="4" t="inlineStr">
+        <is>
+          <t>Guildford, Surrey</t>
+        </is>
+      </c>
+      <c r="D123" s="4" t="inlineStr">
+        <is>
+          <t>https://www.hogsbackbuilders.co.uk</t>
+        </is>
+      </c>
+      <c r="E123" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F123" s="4" t="inlineStr"/>
+      <c r="G123" s="4" t="inlineStr"/>
+      <c r="H123" s="4" t="inlineStr"/>
+      <c r="I123" s="4" t="inlineStr"/>
+      <c r="J123" s="4" t="inlineStr">
+        <is>
+          <t>Bespoke design &amp; build across Surrey/Hampshire borders; project values £100k+</t>
+        </is>
+      </c>
+      <c r="K123" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L123" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M123" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N123" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O123" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P123" s="4" t="inlineStr">
+        <is>
+          <t>Checkatrade/MyBuilder soak up Surrey extension searches</t>
+        </is>
+      </c>
+      <c r="Q123" s="4" t="inlineStr">
+        <is>
+          <t>'One Guildford extension pays for 30 years of our fee'</t>
+        </is>
+      </c>
+      <c r="R123" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S123" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T123" s="4" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="4" t="inlineStr">
+        <is>
+          <t>Surrey Hills Build &amp; Design</t>
+        </is>
+      </c>
+      <c r="B124" s="4" t="inlineStr">
+        <is>
+          <t>Design &amp; build</t>
+        </is>
+      </c>
+      <c r="C124" s="4" t="inlineStr">
+        <is>
+          <t>Guildford &amp; Godalming, Surrey</t>
+        </is>
+      </c>
+      <c r="D124" s="4" t="inlineStr">
+        <is>
+          <t>http://www.surreyhillsbuild.co.uk</t>
+        </is>
+      </c>
+      <c r="E124" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F124" s="4" t="inlineStr"/>
+      <c r="G124" s="4" t="inlineStr">
+        <is>
+          <t>Trevor Steyne (MD)</t>
+        </is>
+      </c>
+      <c r="H124" s="4" t="inlineStr"/>
+      <c r="I124" s="4" t="inlineStr"/>
+      <c r="J124" s="4" t="inlineStr">
+        <is>
+          <t>MD with 30+ years craft background; affluent Surrey Hills catchment</t>
+        </is>
+      </c>
+      <c r="K124" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L124" s="4" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="M124" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N124" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O124" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P124" s="4" t="inlineStr">
+        <is>
+          <t>Dated site undersells premium work</t>
+        </is>
+      </c>
+      <c r="Q124" s="4" t="inlineStr">
+        <is>
+          <t>Site modernisation + local SEO bundle</t>
+        </is>
+      </c>
+      <c r="R124" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S124" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T124" s="4" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="3" t="inlineStr">
+        <is>
+          <t>Godman Construction</t>
+        </is>
+      </c>
+      <c r="B125" s="3" t="inlineStr">
+        <is>
+          <t>Builders / renovations</t>
+        </is>
+      </c>
+      <c r="C125" s="3" t="inlineStr">
+        <is>
+          <t>Guildford, Surrey</t>
+        </is>
+      </c>
+      <c r="D125" s="3" t="inlineStr">
+        <is>
+          <t>https://godmanconstruction.co.uk</t>
+        </is>
+      </c>
+      <c r="E125" s="3" t="inlineStr">
+        <is>
+          <t>info@godmanconstruction.co.uk</t>
+        </is>
+      </c>
+      <c r="F125" s="3" t="inlineStr">
+        <is>
+          <t>01483 494 651</t>
+        </is>
+      </c>
+      <c r="G125" s="3" t="inlineStr"/>
+      <c r="H125" s="3" t="inlineStr"/>
+      <c r="I125" s="3" t="inlineStr"/>
+      <c r="J125" s="3" t="inlineStr">
+        <is>
+          <t>Renovations, extensions and new builds across Surrey; already publishing location blog content</t>
+        </is>
+      </c>
+      <c r="K125" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L125" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M125" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N125" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O125" s="3" t="inlineStr">
+        <is>
+          <t>Location blog posts = DIY SEO</t>
+        </is>
+      </c>
+      <c r="P125" s="3" t="inlineStr">
+        <is>
+          <t>DIY content lacks authority to rank</t>
+        </is>
+      </c>
+      <c r="Q125" s="3" t="inlineStr">
+        <is>
+          <t>'You're writing the right pages - let's make them win'</t>
+        </is>
+      </c>
+      <c r="R125" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S125" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T125" s="3" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="4" t="inlineStr">
+        <is>
+          <t>CMD Recruitment</t>
+        </is>
+      </c>
+      <c r="B126" s="4" t="inlineStr">
+        <is>
+          <t>Recruitment agency</t>
+        </is>
+      </c>
+      <c r="C126" s="4" t="inlineStr">
+        <is>
+          <t>Bath (+ Wiltshire offices)</t>
+        </is>
+      </c>
+      <c r="D126" s="4" t="inlineStr">
+        <is>
+          <t>https://cmdrecruitment.com</t>
+        </is>
+      </c>
+      <c r="E126" s="4" t="inlineStr">
+        <is>
+          <t>Bath@cmdrecruitment.com</t>
+        </is>
+      </c>
+      <c r="F126" s="4" t="inlineStr">
+        <is>
+          <t>01225 800000</t>
+        </is>
+      </c>
+      <c r="G126" s="4" t="inlineStr"/>
+      <c r="H126" s="4" t="inlineStr"/>
+      <c r="I126" s="4" t="inlineStr"/>
+      <c r="J126" s="4" t="inlineStr">
+        <is>
+          <t>Independent multi-office agency since 2004; permanent/interim placements across Bath/Wiltshire</t>
+        </is>
+      </c>
+      <c r="K126" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L126" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M126" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N126" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O126" s="4" t="inlineStr">
+        <is>
+          <t>Multi-office landing pages</t>
+        </is>
+      </c>
+      <c r="P126" s="4" t="inlineStr">
+        <is>
+          <t>Reed/Indeed and nationals dominate; local independent invisible in AI answers</t>
+        </is>
+      </c>
+      <c r="Q126" s="4" t="inlineStr">
+        <is>
+          <t>'Bath employers ask AI for local recruiters - the answer is Reed. Fix that'</t>
+        </is>
+      </c>
+      <c r="R126" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S126" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T126" s="4" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="4" t="inlineStr">
+        <is>
+          <t>Juice Recruitment</t>
+        </is>
+      </c>
+      <c r="B127" s="4" t="inlineStr">
+        <is>
+          <t>Recruitment agency</t>
+        </is>
+      </c>
+      <c r="C127" s="4" t="inlineStr">
+        <is>
+          <t>Bath &amp; South West</t>
+        </is>
+      </c>
+      <c r="D127" s="4" t="inlineStr">
+        <is>
+          <t>https://juicerecruitment.com</t>
+        </is>
+      </c>
+      <c r="E127" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F127" s="4" t="inlineStr"/>
+      <c r="G127" s="4" t="inlineStr"/>
+      <c r="H127" s="4" t="inlineStr"/>
+      <c r="I127" s="4" t="inlineStr"/>
+      <c r="J127" s="4" t="inlineStr">
+        <is>
+          <t>Established SW independent with Bath specialism and location landing pages</t>
+        </is>
+      </c>
+      <c r="K127" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L127" s="4" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M127" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N127" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O127" s="4" t="inlineStr">
+        <is>
+          <t>Location landing pages</t>
+        </is>
+      </c>
+      <c r="P127" s="4" t="inlineStr">
+        <is>
+          <t>Same national-brand squeeze</t>
+        </is>
+      </c>
+      <c r="Q127" s="4" t="inlineStr">
+        <is>
+          <t>AEO layer on existing location-page strategy</t>
+        </is>
+      </c>
+      <c r="R127" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S127" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T127" s="4" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="3" t="inlineStr">
+        <is>
+          <t>Marmalade Schools</t>
+        </is>
+      </c>
+      <c r="B128" s="3" t="inlineStr">
+        <is>
+          <t>Private nursery schools</t>
+        </is>
+      </c>
+      <c r="C128" s="3" t="inlineStr">
+        <is>
+          <t>Fulham, Wandsworth Common &amp; Clapham South, London</t>
+        </is>
+      </c>
+      <c r="D128" s="3" t="inlineStr">
+        <is>
+          <t>https://www.marmaladeschools.co.uk</t>
+        </is>
+      </c>
+      <c r="E128" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F128" s="3" t="inlineStr"/>
+      <c r="G128" s="3" t="inlineStr">
+        <is>
+          <t>Rozzy Roberts (Founder)</t>
+        </is>
+      </c>
+      <c r="H128" s="3" t="inlineStr"/>
+      <c r="I128" s="3" t="inlineStr"/>
+      <c r="J128" s="3" t="inlineStr">
+        <is>
+          <t>Three-site independent nursery group founded by former teacher; nursery fees £15k+/year in SW London</t>
+        </is>
+      </c>
+      <c r="K128" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L128" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M128" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N128" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O128" s="3" t="inlineStr">
+        <is>
+          <t>Press mentions (Sotheby's journal, My Baba lists)</t>
+        </is>
+      </c>
+      <c r="P128" s="3" t="inlineStr">
+        <is>
+          <t>Parents shortlist via AI + listicles; corporate groups (Grandir, Dukes) spend big</t>
+        </is>
+      </c>
+      <c r="Q128" s="3" t="inlineStr">
+        <is>
+          <t>'SW London parents ask ChatGPT for nursery shortlists - be on all of them'</t>
+        </is>
+      </c>
+      <c r="R128" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S128" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T128" s="3" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="3" t="inlineStr">
+        <is>
+          <t>Parsons Green Nursery</t>
+        </is>
+      </c>
+      <c r="B129" s="3" t="inlineStr">
+        <is>
+          <t>Private day nursery</t>
+        </is>
+      </c>
+      <c r="C129" s="3" t="inlineStr">
+        <is>
+          <t>Fulham Road, London SW6</t>
+        </is>
+      </c>
+      <c r="D129" s="3" t="inlineStr">
+        <is>
+          <t>https://parsonsgreennursery.com</t>
+        </is>
+      </c>
+      <c r="E129" s="3" t="inlineStr">
+        <is>
+          <t>admissions@parsonsgreennursery.com</t>
+        </is>
+      </c>
+      <c r="F129" s="3" t="inlineStr">
+        <is>
+          <t>020 3943 4678</t>
+        </is>
+      </c>
+      <c r="G129" s="3" t="inlineStr"/>
+      <c r="H129" s="3" t="inlineStr"/>
+      <c r="I129" s="3" t="inlineStr"/>
+      <c r="J129" s="3" t="inlineStr">
+        <is>
+          <t>Ofsted Outstanding nursery in prime SW6; waitlist-driven but competition for premium families is fierce</t>
+        </is>
+      </c>
+      <c r="K129" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L129" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M129" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N129" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O129" s="3" t="inlineStr">
+        <is>
+          <t>Ofsted Outstanding badge</t>
+        </is>
+      </c>
+      <c r="P129" s="3" t="inlineStr">
+        <is>
+          <t>Outstanding rating under-marketed; chains outrank them</t>
+        </is>
+      </c>
+      <c r="Q129" s="3" t="inlineStr">
+        <is>
+          <t>'Outstanding-rated should be the first answer parents get - it isn't'</t>
+        </is>
+      </c>
+      <c r="R129" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S129" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T129" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T101"/>
+  <autoFilter ref="A1:T129"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -9420,7 +11740,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B69"/>
+  <dimension ref="A1:B85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -9440,7 +11760,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>100</v>
+        <v>128</v>
       </c>
     </row>
     <row r="5">
@@ -9457,13 +11777,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Solar installer</t>
+          <t>Private dentist</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -9473,37 +11793,37 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Mortgage broker</t>
+          <t>Physiotherapy clinic</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Physiotherapy clinic</t>
+          <t>Solar installer</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Chartered accountants</t>
+          <t>Estate &amp; letting agent</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Independent vet</t>
+          <t>Mortgage broker</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -9513,7 +11833,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Private GP</t>
+          <t>Chartered accountants</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -9523,7 +11843,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Family law firm</t>
+          <t>Independent vet</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -9533,7 +11853,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Architects</t>
+          <t>Private GP</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -9543,7 +11863,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Estate &amp; letting agent</t>
+          <t>Family law firm</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -9553,11 +11873,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Private dentist</t>
+          <t>Architects</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17">
@@ -9593,7 +11913,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Private tuition agency</t>
+          <t>Financial adviser / wealth management</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -9603,7 +11923,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating / boilers</t>
+          <t>Private tuition agency</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -9613,7 +11933,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Electrician</t>
+          <t>Osteopathy clinic</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -9623,7 +11943,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Event &amp; wedding caterer</t>
+          <t>Plumbing &amp; heating / boilers</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -9633,7 +11953,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Personal training studio</t>
+          <t>Electrician</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -9643,7 +11963,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Chiropractor</t>
+          <t>Event &amp; wedding caterer</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -9653,7 +11973,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Orthodontist</t>
+          <t>Personal training studio</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -9663,7 +11983,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Aesthetics clinic</t>
+          <t>Chiropractor</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -9673,67 +11993,67 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Dentist / Orthodontics</t>
+          <t>Orthodontist</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Specialist dental/implant clinic</t>
+          <t>Aesthetics clinic</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Boutique corporate law firm</t>
+          <t>Employment law firm</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Cosmetic/aesthetics clinic</t>
+          <t>Event management agency</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Skin &amp; laser clinic</t>
+          <t>Design &amp; build</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Mortgage broker / financial adviser</t>
+          <t>Recruitment agency</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Architects (RIBA chartered)</t>
+          <t>Dentist / Orthodontics</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -9743,7 +12063,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Recruitment agency (tech/startups)</t>
+          <t>Specialist dental/implant clinic</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -9753,7 +12073,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Recruitment agency (IT/data)</t>
+          <t>Boutique corporate law firm</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -9763,7 +12083,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Independent vet (24/7 emergency)</t>
+          <t>Cosmetic/aesthetics clinic</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -9773,7 +12093,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Interior design studio</t>
+          <t>Skin &amp; laser clinic</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -9783,7 +12103,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Letting &amp; estate agent</t>
+          <t>Mortgage broker / financial adviser</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -9793,7 +12113,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Cosmetic clinic (injectables)</t>
+          <t>Architects (RIBA chartered)</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -9803,7 +12123,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Cosmetic/anti-ageing clinic</t>
+          <t>Recruitment agency (tech/startups)</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -9813,7 +12133,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Yoga &amp; reformer pilates studio</t>
+          <t>Recruitment agency (IT/data)</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -9823,7 +12143,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Reformer pilates studio</t>
+          <t>Independent vet (24/7 emergency)</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -9833,7 +12153,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Financial adviser / wealth management</t>
+          <t>Interior design studio</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -9843,7 +12163,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Wealth management</t>
+          <t>Letting &amp; estate agent</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -9853,7 +12173,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Private tuition &amp; education consultancy</t>
+          <t>Cosmetic clinic (injectables)</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -9863,7 +12183,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Osteopath</t>
+          <t>Cosmetic/anti-ageing clinic</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -9873,7 +12193,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Osteopathy clinic</t>
+          <t>Yoga &amp; reformer pilates studio</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -9883,7 +12203,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Design &amp; build / home renovation</t>
+          <t>Reformer pilates studio</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -9893,7 +12213,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Builders / building contractor</t>
+          <t>Wealth management</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -9903,7 +12223,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Roofer</t>
+          <t>Private tuition &amp; education consultancy</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -9913,7 +12233,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Home care / live-in care</t>
+          <t>Osteopath</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -9923,7 +12243,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Private day nurseries</t>
+          <t>Design &amp; build / home renovation</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -9933,7 +12253,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Personal training &amp; wellness studio</t>
+          <t>Builders / building contractor</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -9943,7 +12263,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Mortgage &amp; insurance broker</t>
+          <t>Roofer</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -9953,7 +12273,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Business consultancy</t>
+          <t>Home care / live-in care</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -9963,7 +12283,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Interior designer (period homes)</t>
+          <t>Private day nurseries</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -9973,7 +12293,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Landscape design &amp; build</t>
+          <t>Personal training &amp; wellness studio</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -9983,7 +12303,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Estate agent (premium)</t>
+          <t>Mortgage &amp; insurance broker</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -9993,7 +12313,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Interior designer</t>
+          <t>Business consultancy</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -10003,7 +12323,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Garden design &amp; landscaping</t>
+          <t>Interior designer (period homes)</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -10013,7 +12333,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Legal recruitment</t>
+          <t>Landscape design &amp; build</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -10023,7 +12343,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Independent gym &amp; health club</t>
+          <t>Estate agent (premium)</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -10033,7 +12353,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Independent gym</t>
+          <t>Interior designer</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -10043,7 +12363,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Physiotherapy (sports)</t>
+          <t>Garden design &amp; landscaping</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -10053,7 +12373,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Letting agent / property management</t>
+          <t>Legal recruitment</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -10063,7 +12383,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Skin clinic</t>
+          <t>Independent gym &amp; health club</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -10073,7 +12393,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Tutoring company</t>
+          <t>Independent gym</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -10083,10 +12403,170 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
+          <t>Physiotherapy (sports)</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Letting agent / property management</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Skin clinic</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Tutoring company</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
           <t>Tutorial college &amp; exam centre</t>
         </is>
       </c>
-      <c r="B69" t="n">
+      <c r="B73" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Employment law (disability discrimination)</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Plumbing &amp; heating</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Sports physio &amp; massage</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Chartered surveyors (party wall/building)</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Chartered surveyors</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Chartered building surveyors</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Osteopathy clinics</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Private dentist / implants</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Builders / renovations</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Private nursery schools</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Private day nursery</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 5: +31 prospects (159 total) - Cheltenham, Oxford, Cotswolds, Kent, Guildford expansion
New geographies: Cheltenham, Oxford, Cotswolds (Tewkesbury/Broadway), Guildford/
Surrey, Kent, Hampshire. New niches: immigration law, conveyancing, IT/MSP
support, heritage sash-window restoration, live-in care.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$129</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$160</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T129"/>
+  <dimension ref="A1:T160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -11728,8 +11728,2636 @@
       </c>
       <c r="T129" s="3" t="inlineStr"/>
     </row>
+    <row r="130">
+      <c r="A130" s="3" t="inlineStr">
+        <is>
+          <t>Morgan Associates</t>
+        </is>
+      </c>
+      <c r="B130" s="3" t="inlineStr">
+        <is>
+          <t>Estate &amp; letting agent</t>
+        </is>
+      </c>
+      <c r="C130" s="3" t="inlineStr">
+        <is>
+          <t>Montpellier Exchange, Cheltenham</t>
+        </is>
+      </c>
+      <c r="D130" s="3" t="inlineStr">
+        <is>
+          <t>https://www.morgan-associates.co.uk</t>
+        </is>
+      </c>
+      <c r="E130" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F130" s="3" t="inlineStr">
+        <is>
+          <t>01242 354692</t>
+        </is>
+      </c>
+      <c r="G130" s="3" t="inlineStr"/>
+      <c r="H130" s="3" t="inlineStr"/>
+      <c r="I130" s="3" t="inlineStr"/>
+      <c r="J130" s="3" t="inlineStr">
+        <is>
+          <t>Independent agency in prestige Montpellier address covering Cheltenham/Cotswolds; premium instructions worth thousands in fees</t>
+        </is>
+      </c>
+      <c r="K130" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L130" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M130" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N130" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O130" s="3" t="inlineStr">
+        <is>
+          <t>Portal listings</t>
+        </is>
+      </c>
+      <c r="P130" s="3" t="inlineStr">
+        <is>
+          <t>Fine &amp; Country/Knight Frank corporate brands dominate Cheltenham premium search</t>
+        </is>
+      </c>
+      <c r="Q130" s="3" t="inlineStr">
+        <is>
+          <t>'Montpellier sellers shortlist online before calling - be on that shortlist'</t>
+        </is>
+      </c>
+      <c r="R130" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S130" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T130" s="3" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="3" t="inlineStr">
+        <is>
+          <t>Beyond Dental Cheltenham</t>
+        </is>
+      </c>
+      <c r="B131" s="3" t="inlineStr">
+        <is>
+          <t>Private dentist</t>
+        </is>
+      </c>
+      <c r="C131" s="3" t="inlineStr">
+        <is>
+          <t>Rodney Road, Cheltenham</t>
+        </is>
+      </c>
+      <c r="D131" s="3" t="inlineStr">
+        <is>
+          <t>https://beyond-dental.co.uk/cheltenham</t>
+        </is>
+      </c>
+      <c r="E131" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F131" s="3" t="inlineStr">
+        <is>
+          <t>01296 730260</t>
+        </is>
+      </c>
+      <c r="G131" s="3" t="inlineStr"/>
+      <c r="H131" s="3" t="inlineStr"/>
+      <c r="I131" s="3" t="inlineStr"/>
+      <c r="J131" s="3" t="inlineStr">
+        <is>
+          <t>Luxury private dental brand with multi-location model; implants/Invisalign cases £3-6k in wealthy Cheltenham</t>
+        </is>
+      </c>
+      <c r="K131" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L131" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M131" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N131" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O131" s="3" t="inlineStr">
+        <is>
+          <t>Multi-location brand site</t>
+        </is>
+      </c>
+      <c r="P131" s="3" t="inlineStr">
+        <is>
+          <t>Local Cheltenham searches split with Cheltenham &amp; Cotswold Dental, Pittville Lawn - AEO could tip the balance</t>
+        </is>
+      </c>
+      <c r="Q131" s="3" t="inlineStr">
+        <is>
+          <t>'Own the AI answer for "Invisalign Cheltenham" before your closest rival does'</t>
+        </is>
+      </c>
+      <c r="R131" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S131" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T131" s="3" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="3" t="inlineStr">
+        <is>
+          <t>Cheltenham &amp; Cotswold Dental</t>
+        </is>
+      </c>
+      <c r="B132" s="3" t="inlineStr">
+        <is>
+          <t>Private dentist</t>
+        </is>
+      </c>
+      <c r="C132" s="3" t="inlineStr">
+        <is>
+          <t>Cheltenham</t>
+        </is>
+      </c>
+      <c r="D132" s="3" t="inlineStr">
+        <is>
+          <t>https://cheltenhamandcotswolddental.com</t>
+        </is>
+      </c>
+      <c r="E132" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F132" s="3" t="inlineStr">
+        <is>
+          <t>01242 269 498</t>
+        </is>
+      </c>
+      <c r="G132" s="3" t="inlineStr">
+        <is>
+          <t>Dr Imran Nasser &amp; Dr Samantha Stewart (Principals)</t>
+        </is>
+      </c>
+      <c r="H132" s="3" t="inlineStr"/>
+      <c r="I132" s="3" t="inlineStr"/>
+      <c r="J132" s="3" t="inlineStr">
+        <is>
+          <t>Award-winning practice with named principals; also runs facial aesthetics arm = two revenue lines</t>
+        </is>
+      </c>
+      <c r="K132" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L132" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M132" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N132" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O132" s="3" t="inlineStr">
+        <is>
+          <t>Facial aesthetics cross-sell page; awards</t>
+        </is>
+      </c>
+      <c r="P132" s="3" t="inlineStr">
+        <is>
+          <t>Two service lines (dental + aesthetics) competing for the same searches without a unified strategy</t>
+        </is>
+      </c>
+      <c r="Q132" s="3" t="inlineStr">
+        <is>
+          <t>Consolidate dental + aesthetics AEO under one authority-building plan</t>
+        </is>
+      </c>
+      <c r="R132" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S132" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T132" s="3" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="3" t="inlineStr">
+        <is>
+          <t>JCP Estate Agents</t>
+        </is>
+      </c>
+      <c r="B133" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C133" s="3" t="inlineStr">
+        <is>
+          <t>Oxford (Jericho/Summertown/Marston/East Oxford)</t>
+        </is>
+      </c>
+      <c r="D133" s="3" t="inlineStr">
+        <is>
+          <t>https://www.jamescpenny.co.uk</t>
+        </is>
+      </c>
+      <c r="E133" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F133" s="3" t="inlineStr"/>
+      <c r="G133" s="3" t="inlineStr"/>
+      <c r="H133" s="3" t="inlineStr"/>
+      <c r="I133" s="3" t="inlineStr"/>
+      <c r="J133" s="3" t="inlineStr">
+        <is>
+          <t>Award-winning independent covering 'Prime Central Oxford' across 4 postcodes; academic-city premium market</t>
+        </is>
+      </c>
+      <c r="K133" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L133" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M133" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N133" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O133" s="3" t="inlineStr">
+        <is>
+          <t>Award mentions</t>
+        </is>
+      </c>
+      <c r="P133" s="3" t="inlineStr">
+        <is>
+          <t>Breckon &amp; Breckon and scottfraser also fight for the same Oxford postcodes</t>
+        </is>
+      </c>
+      <c r="Q133" s="3" t="inlineStr">
+        <is>
+          <t>'Oxford buyers/sellers now ask AI which agent knows Jericho best - claim it'</t>
+        </is>
+      </c>
+      <c r="R133" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S133" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T133" s="3" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="3" t="inlineStr">
+        <is>
+          <t>Breckon &amp; Breckon</t>
+        </is>
+      </c>
+      <c r="B134" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C134" s="3" t="inlineStr">
+        <is>
+          <t>Summertown, North Oxford</t>
+        </is>
+      </c>
+      <c r="D134" s="3" t="inlineStr">
+        <is>
+          <t>https://www.breckon.co.uk</t>
+        </is>
+      </c>
+      <c r="E134" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F134" s="3" t="inlineStr"/>
+      <c r="G134" s="3" t="inlineStr"/>
+      <c r="H134" s="3" t="inlineStr"/>
+      <c r="I134" s="3" t="inlineStr"/>
+      <c r="J134" s="3" t="inlineStr">
+        <is>
+          <t>Independent since 1947 covering Summertown/Wolvercote/Jericho; heritage brand with high-value North Oxford stock</t>
+        </is>
+      </c>
+      <c r="K134" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L134" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M134" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N134" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O134" s="3" t="inlineStr">
+        <is>
+          <t>Long-established brand</t>
+        </is>
+      </c>
+      <c r="P134" s="3" t="inlineStr">
+        <is>
+          <t>80 years of trust doesn't automatically appear in AI search answers</t>
+        </is>
+      </c>
+      <c r="Q134" s="3" t="inlineStr">
+        <is>
+          <t>Turn 'established 1947' into the AI-cited trust signal for North Oxford</t>
+        </is>
+      </c>
+      <c r="R134" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S134" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T134" s="3" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="4" t="inlineStr">
+        <is>
+          <t>Otus Mortgages</t>
+        </is>
+      </c>
+      <c r="B135" s="4" t="inlineStr">
+        <is>
+          <t>Mortgage broker</t>
+        </is>
+      </c>
+      <c r="C135" s="4" t="inlineStr">
+        <is>
+          <t>Oxford &amp; Warwick</t>
+        </is>
+      </c>
+      <c r="D135" s="4" t="inlineStr">
+        <is>
+          <t>https://otusoxford.co.uk</t>
+        </is>
+      </c>
+      <c r="E135" s="4" t="inlineStr">
+        <is>
+          <t>hello@otus.uk.com</t>
+        </is>
+      </c>
+      <c r="F135" s="4" t="inlineStr"/>
+      <c r="G135" s="4" t="inlineStr">
+        <is>
+          <t>Neil Yeoman (Director)</t>
+        </is>
+      </c>
+      <c r="H135" s="4" t="inlineStr"/>
+      <c r="I135" s="4" t="inlineStr"/>
+      <c r="J135" s="4" t="inlineStr">
+        <is>
+          <t>Independent whole-of-market broker; Oxford's academic/professional buyers = high-value cases</t>
+        </is>
+      </c>
+      <c r="K135" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L135" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M135" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N135" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O135" s="4" t="inlineStr">
+        <is>
+          <t>Two-site brand (Oxford/Warwick)</t>
+        </is>
+      </c>
+      <c r="P135" s="4" t="inlineStr">
+        <is>
+          <t>Oxford Mortgages and Bright Money compete for the same 'mortgage broker Oxford' searches</t>
+        </is>
+      </c>
+      <c r="Q135" s="4" t="inlineStr">
+        <is>
+          <t>Own the local-intent long tail before the other Oxford brokers do</t>
+        </is>
+      </c>
+      <c r="R135" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S135" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T135" s="4" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="3" t="inlineStr">
+        <is>
+          <t>Linbury Doctors</t>
+        </is>
+      </c>
+      <c r="B136" s="3" t="inlineStr">
+        <is>
+          <t>Private GP (membership model)</t>
+        </is>
+      </c>
+      <c r="C136" s="3" t="inlineStr">
+        <is>
+          <t>Cotswolds/Oxfordshire/Gloucestershire (Broadway HQ)</t>
+        </is>
+      </c>
+      <c r="D136" s="3" t="inlineStr">
+        <is>
+          <t>https://www.linburydoctors.co.uk</t>
+        </is>
+      </c>
+      <c r="E136" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F136" s="3" t="inlineStr">
+        <is>
+          <t>0333 050 7338</t>
+        </is>
+      </c>
+      <c r="G136" s="3" t="inlineStr">
+        <is>
+          <t>Dr Hala &amp; Dr Lucy (Medical Directors)</t>
+        </is>
+      </c>
+      <c r="H136" s="3" t="inlineStr"/>
+      <c r="I136" s="3" t="inlineStr"/>
+      <c r="J136" s="3" t="inlineStr">
+        <is>
+          <t>Membership-based private GP covering 6 counties; recurring membership fees = high LTV per patient</t>
+        </is>
+      </c>
+      <c r="K136" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L136" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M136" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N136" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O136" s="3" t="inlineStr">
+        <is>
+          <t>Multi-county location pages</t>
+        </is>
+      </c>
+      <c r="P136" s="3" t="inlineStr">
+        <is>
+          <t>Membership model needs constant new-patient acquisition across a huge rural catchment</t>
+        </is>
+      </c>
+      <c r="Q136" s="3" t="inlineStr">
+        <is>
+          <t>'Cotswold families ask AI for a private GP - be the membership they find first'</t>
+        </is>
+      </c>
+      <c r="R136" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S136" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T136" s="3" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="3" t="inlineStr">
+        <is>
+          <t>The Guildford Vet</t>
+        </is>
+      </c>
+      <c r="B137" s="3" t="inlineStr">
+        <is>
+          <t>Independent vet</t>
+        </is>
+      </c>
+      <c r="C137" s="3" t="inlineStr">
+        <is>
+          <t>Worplesdon Road, Guildford, Surrey</t>
+        </is>
+      </c>
+      <c r="D137" s="3" t="inlineStr">
+        <is>
+          <t>https://www.theguildfordvet.co.uk</t>
+        </is>
+      </c>
+      <c r="E137" s="3" t="inlineStr">
+        <is>
+          <t>info@theguildfordvet.co.uk</t>
+        </is>
+      </c>
+      <c r="F137" s="3" t="inlineStr">
+        <is>
+          <t>01483 610292</t>
+        </is>
+      </c>
+      <c r="G137" s="3" t="inlineStr">
+        <is>
+          <t>Rob, Amber, Chris &amp; Lucy (Founders); Christian Gray (Director)</t>
+        </is>
+      </c>
+      <c r="H137" s="3" t="inlineStr"/>
+      <c r="I137" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/theguildfordvet</t>
+        </is>
+      </c>
+      <c r="J137" s="3" t="inlineStr">
+        <is>
+          <t>Founded 2022, proudly independent in affluent Guildford; 24/7 emergency = highest-intent local searches</t>
+        </is>
+      </c>
+      <c r="K137" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L137" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M137" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N137" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O137" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence</t>
+        </is>
+      </c>
+      <c r="P137" s="3" t="inlineStr">
+        <is>
+          <t>Corporate vet groups (IVC, CVS) dominate Surrey vet searches with huge budgets</t>
+        </is>
+      </c>
+      <c r="Q137" s="3" t="inlineStr">
+        <is>
+          <t>'New, independent, and invisible on Google - let's fix that before the chains notice'</t>
+        </is>
+      </c>
+      <c r="R137" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S137" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T137" s="3" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="4" t="inlineStr">
+        <is>
+          <t>The Cape Veterinary Clinic</t>
+        </is>
+      </c>
+      <c r="B138" s="4" t="inlineStr">
+        <is>
+          <t>Independent vet</t>
+        </is>
+      </c>
+      <c r="C138" s="4" t="inlineStr">
+        <is>
+          <t>Guildford, Surrey</t>
+        </is>
+      </c>
+      <c r="D138" s="4" t="inlineStr">
+        <is>
+          <t>https://capevets.co.uk</t>
+        </is>
+      </c>
+      <c r="E138" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F138" s="4" t="inlineStr"/>
+      <c r="G138" s="4" t="inlineStr">
+        <is>
+          <t>Douglas Hall (Owner)</t>
+        </is>
+      </c>
+      <c r="H138" s="4" t="inlineStr"/>
+      <c r="I138" s="4" t="inlineStr"/>
+      <c r="J138" s="4" t="inlineStr">
+        <is>
+          <t>Family-run independent, increasingly rare model in Surrey; loyal client base</t>
+        </is>
+      </c>
+      <c r="K138" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L138" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M138" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N138" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O138" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P138" s="4" t="inlineStr">
+        <is>
+          <t>Independence story under-leveraged vs corporate-owned rivals</t>
+        </is>
+      </c>
+      <c r="Q138" s="4" t="inlineStr">
+        <is>
+          <t>Independence-as-differentiator AEO content</t>
+        </is>
+      </c>
+      <c r="R138" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S138" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T138" s="4" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="3" t="inlineStr">
+        <is>
+          <t>Cotswold Face &amp; Body Clinic</t>
+        </is>
+      </c>
+      <c r="B139" s="3" t="inlineStr">
+        <is>
+          <t>Aesthetics clinic</t>
+        </is>
+      </c>
+      <c r="C139" s="3" t="inlineStr">
+        <is>
+          <t>Cheltenham</t>
+        </is>
+      </c>
+      <c r="D139" s="3" t="inlineStr">
+        <is>
+          <t>https://cotswoldfabclinic.co.uk</t>
+        </is>
+      </c>
+      <c r="E139" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F139" s="3" t="inlineStr"/>
+      <c r="G139" s="3" t="inlineStr"/>
+      <c r="H139" s="3" t="inlineStr"/>
+      <c r="I139" s="3" t="inlineStr"/>
+      <c r="J139" s="3" t="inlineStr">
+        <is>
+          <t>Luxury clinic with Harley Street surgeon association; high-ticket surgical-adjacent consultations</t>
+        </is>
+      </c>
+      <c r="K139" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L139" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M139" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N139" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O139" s="3" t="inlineStr">
+        <is>
+          <t>Harley St association promoted</t>
+        </is>
+      </c>
+      <c r="P139" s="3" t="inlineStr">
+        <is>
+          <t>Association with prestige name not translating into local/AI search dominance</t>
+        </is>
+      </c>
+      <c r="Q139" s="3" t="inlineStr">
+        <is>
+          <t>Turn the Harley Street link into the AI-cited authority signal for Cotswold aesthetics</t>
+        </is>
+      </c>
+      <c r="R139" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S139" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T139" s="3" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="4" t="inlineStr">
+        <is>
+          <t>Iris Medical Aesthetics</t>
+        </is>
+      </c>
+      <c r="B140" s="4" t="inlineStr">
+        <is>
+          <t>Aesthetics clinic</t>
+        </is>
+      </c>
+      <c r="C140" s="4" t="inlineStr">
+        <is>
+          <t>Cheltenham</t>
+        </is>
+      </c>
+      <c r="D140" s="4" t="inlineStr">
+        <is>
+          <t>https://www.irismedicalaesthetics.com</t>
+        </is>
+      </c>
+      <c r="E140" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F140" s="4" t="inlineStr"/>
+      <c r="G140" s="4" t="inlineStr"/>
+      <c r="H140" s="4" t="inlineStr"/>
+      <c r="I140" s="4" t="inlineStr"/>
+      <c r="J140" s="4" t="inlineStr">
+        <is>
+          <t>Discreet boutique clinic in central Cheltenham; repeat injectable clients</t>
+        </is>
+      </c>
+      <c r="K140" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L140" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M140" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N140" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O140" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P140" s="4" t="inlineStr">
+        <is>
+          <t>Generic positioning in a market with several named-doctor rivals</t>
+        </is>
+      </c>
+      <c r="Q140" s="4" t="inlineStr">
+        <is>
+          <t>Local + AEO package to compete with named-practitioner clinics</t>
+        </is>
+      </c>
+      <c r="R140" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S140" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T140" s="4" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="3" t="inlineStr">
+        <is>
+          <t>Ashleigh Clarke Architects</t>
+        </is>
+      </c>
+      <c r="B141" s="3" t="inlineStr">
+        <is>
+          <t>Architects</t>
+        </is>
+      </c>
+      <c r="C141" s="3" t="inlineStr">
+        <is>
+          <t>Upper Rissington, Cheltenham/Cotswolds</t>
+        </is>
+      </c>
+      <c r="D141" s="3" t="inlineStr">
+        <is>
+          <t>https://ashleighclarkearchitects.com</t>
+        </is>
+      </c>
+      <c r="E141" s="3" t="inlineStr">
+        <is>
+          <t>info@ashleighclarkearchitects.com</t>
+        </is>
+      </c>
+      <c r="F141" s="3" t="inlineStr">
+        <is>
+          <t>01451 828 419</t>
+        </is>
+      </c>
+      <c r="G141" s="3" t="inlineStr">
+        <is>
+          <t>Ashleigh Clarke (Founder &amp; Lead Architect)</t>
+        </is>
+      </c>
+      <c r="H141" s="3" t="inlineStr"/>
+      <c r="I141" s="3" t="inlineStr"/>
+      <c r="J141" s="3" t="inlineStr">
+        <is>
+          <t>RIBA/ARB residential practice across the Cotswolds; project values £100k+; named founder with direct email</t>
+        </is>
+      </c>
+      <c r="K141" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L141" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M141" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N141" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O141" s="3" t="inlineStr">
+        <is>
+          <t>RIBA directory listing</t>
+        </is>
+      </c>
+      <c r="P141" s="3" t="inlineStr">
+        <is>
+          <t>Cotswold second-home owners search nationally; local firm needs to compete with London-based rivals</t>
+        </is>
+      </c>
+      <c r="Q141" s="3" t="inlineStr">
+        <is>
+          <t>'Cotswold clients ask AI for a local architect who knows the planning rules - be that answer'</t>
+        </is>
+      </c>
+      <c r="R141" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S141" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T141" s="3" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="3" t="inlineStr">
+        <is>
+          <t>Lewis Critchley Architects</t>
+        </is>
+      </c>
+      <c r="B142" s="3" t="inlineStr">
+        <is>
+          <t>Architects</t>
+        </is>
+      </c>
+      <c r="C142" s="3" t="inlineStr">
+        <is>
+          <t>Tewkesbury/Cheltenham, Cotswolds</t>
+        </is>
+      </c>
+      <c r="D142" s="3" t="inlineStr">
+        <is>
+          <t>https://lewiscritchleyarchitects.co.uk</t>
+        </is>
+      </c>
+      <c r="E142" s="3" t="inlineStr">
+        <is>
+          <t>lmc@lewiscritchleyarchitects.co.uk</t>
+        </is>
+      </c>
+      <c r="F142" s="3" t="inlineStr">
+        <is>
+          <t>01684 295473</t>
+        </is>
+      </c>
+      <c r="G142" s="3" t="inlineStr">
+        <is>
+          <t>Lewis Critchley (Founder)</t>
+        </is>
+      </c>
+      <c r="H142" s="3" t="inlineStr"/>
+      <c r="I142" s="3" t="inlineStr"/>
+      <c r="J142" s="3" t="inlineStr">
+        <is>
+          <t>RIBA chartered, established 2019; direct founder email; growing Cotswolds residential practice</t>
+        </is>
+      </c>
+      <c r="K142" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L142" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M142" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N142" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O142" s="3" t="inlineStr">
+        <is>
+          <t>Professional site</t>
+        </is>
+      </c>
+      <c r="P142" s="3" t="inlineStr">
+        <is>
+          <t>Young practice needs to build authority fast against established Cotswold firms</t>
+        </is>
+      </c>
+      <c r="Q142" s="3" t="inlineStr">
+        <is>
+          <t>Ground-floor local SEO + AEO while building reputation</t>
+        </is>
+      </c>
+      <c r="R142" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S142" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T142" s="3" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="4" t="inlineStr">
+        <is>
+          <t>Gray Architecture</t>
+        </is>
+      </c>
+      <c r="B143" s="4" t="inlineStr">
+        <is>
+          <t>Architects</t>
+        </is>
+      </c>
+      <c r="C143" s="4" t="inlineStr">
+        <is>
+          <t>Cheltenham/Cotswolds</t>
+        </is>
+      </c>
+      <c r="D143" s="4" t="inlineStr">
+        <is>
+          <t>https://grayarchitecture.co.uk</t>
+        </is>
+      </c>
+      <c r="E143" s="4" t="inlineStr">
+        <is>
+          <t>info@grayarchitecture.co.uk</t>
+        </is>
+      </c>
+      <c r="F143" s="4" t="inlineStr">
+        <is>
+          <t>07855 348 625</t>
+        </is>
+      </c>
+      <c r="G143" s="4" t="inlineStr">
+        <is>
+          <t>Chris Gray (Founder)</t>
+        </is>
+      </c>
+      <c r="H143" s="4" t="inlineStr"/>
+      <c r="I143" s="4" t="inlineStr"/>
+      <c r="J143" s="4" t="inlineStr">
+        <is>
+          <t>Established 2021, 15+ years experience; solo-led practice with direct founder contact</t>
+        </is>
+      </c>
+      <c r="K143" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L143" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M143" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N143" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O143" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P143" s="4" t="inlineStr">
+        <is>
+          <t>New practice with minimal search visibility</t>
+        </is>
+      </c>
+      <c r="Q143" s="4" t="inlineStr">
+        <is>
+          <t>Entry package: build local authority from a clean slate</t>
+        </is>
+      </c>
+      <c r="R143" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S143" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T143" s="4" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="3" t="inlineStr">
+        <is>
+          <t>Hawkes &amp; Son</t>
+        </is>
+      </c>
+      <c r="B144" s="3" t="inlineStr">
+        <is>
+          <t>Sash window restoration</t>
+        </is>
+      </c>
+      <c r="C144" s="3" t="inlineStr">
+        <is>
+          <t>Melksham (serves Bath)</t>
+        </is>
+      </c>
+      <c r="D144" s="3" t="inlineStr">
+        <is>
+          <t>http://www.hawkes-sash.co.uk</t>
+        </is>
+      </c>
+      <c r="E144" s="3" t="inlineStr">
+        <is>
+          <t>enquiries@hawkes-sash.co.uk</t>
+        </is>
+      </c>
+      <c r="F144" s="3" t="inlineStr">
+        <is>
+          <t>01225 791229</t>
+        </is>
+      </c>
+      <c r="G144" s="3" t="inlineStr">
+        <is>
+          <t>Michael Hawkes (Founder)</t>
+        </is>
+      </c>
+      <c r="H144" s="3" t="inlineStr"/>
+      <c r="I144" s="3" t="inlineStr"/>
+      <c r="J144" s="3" t="inlineStr">
+        <is>
+          <t>Heritage-joinery specialist for Bath's Georgian housing stock; restoration jobs £3-10k; highly defensible niche</t>
+        </is>
+      </c>
+      <c r="K144" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L144" s="3" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="M144" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N144" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O144" s="3" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P144" s="3" t="inlineStr">
+        <is>
+          <t>Dated site undersells a genuinely rare, high-value heritage-trade skill</t>
+        </is>
+      </c>
+      <c r="Q144" s="3" t="inlineStr">
+        <is>
+          <t>'Own "sash window restoration Bath" - a high-value niche almost nobody optimises for'</t>
+        </is>
+      </c>
+      <c r="R144" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S144" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T144" s="3" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="3" t="inlineStr">
+        <is>
+          <t>Clifton IT</t>
+        </is>
+      </c>
+      <c r="B145" s="3" t="inlineStr">
+        <is>
+          <t>IT support / MSP</t>
+        </is>
+      </c>
+      <c r="C145" s="3" t="inlineStr">
+        <is>
+          <t>Whiteladies Rd, Bristol</t>
+        </is>
+      </c>
+      <c r="D145" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cliftonit.co.uk</t>
+        </is>
+      </c>
+      <c r="E145" s="3" t="inlineStr">
+        <is>
+          <t>info@cliftonit.co.uk</t>
+        </is>
+      </c>
+      <c r="F145" s="3" t="inlineStr">
+        <is>
+          <t>01179 595143</t>
+        </is>
+      </c>
+      <c r="G145" s="3" t="inlineStr"/>
+      <c r="H145" s="3" t="inlineStr"/>
+      <c r="I145" s="3" t="inlineStr"/>
+      <c r="J145" s="3" t="inlineStr">
+        <is>
+          <t>MSP serving Bristol/Bath/Exeter/Plymouth SMEs; recurring monthly contracts = high LTV per client</t>
+        </is>
+      </c>
+      <c r="K145" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L145" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M145" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N145" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O145" s="3" t="inlineStr">
+        <is>
+          <t>Multi-region service pages</t>
+        </is>
+      </c>
+      <c r="P145" s="3" t="inlineStr">
+        <is>
+          <t>SMEs searching for IT support see nationals (Solutions4IT etc.) first</t>
+        </is>
+      </c>
+      <c r="Q145" s="3" t="inlineStr">
+        <is>
+          <t>'When a Bristol business Googles "IT support near me" at 9am on a bad day - be the answer'</t>
+        </is>
+      </c>
+      <c r="R145" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S145" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T145" s="3" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="3" t="inlineStr">
+        <is>
+          <t>Three Cherries</t>
+        </is>
+      </c>
+      <c r="B146" s="3" t="inlineStr">
+        <is>
+          <t>IT support / MSP</t>
+        </is>
+      </c>
+      <c r="C146" s="3" t="inlineStr">
+        <is>
+          <t>Bristol</t>
+        </is>
+      </c>
+      <c r="D146" s="3" t="inlineStr">
+        <is>
+          <t>https://www.threecherries.co.uk</t>
+        </is>
+      </c>
+      <c r="E146" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F146" s="3" t="inlineStr"/>
+      <c r="G146" s="3" t="inlineStr"/>
+      <c r="H146" s="3" t="inlineStr"/>
+      <c r="I146" s="3" t="inlineStr"/>
+      <c r="J146" s="3" t="inlineStr">
+        <is>
+          <t>Independent MSP since 1999 - one of the longest-standing in the region; SME contracts are sticky and high-value</t>
+        </is>
+      </c>
+      <c r="K146" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L146" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M146" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N146" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O146" s="3" t="inlineStr">
+        <is>
+          <t>25+ years trading</t>
+        </is>
+      </c>
+      <c r="P146" s="3" t="inlineStr">
+        <is>
+          <t>Longevity doesn't automatically win modern local/AI search</t>
+        </is>
+      </c>
+      <c r="Q146" s="3" t="inlineStr">
+        <is>
+          <t>'25 years of Bristol IT trust - let's make sure Google and AI both know it'</t>
+        </is>
+      </c>
+      <c r="R146" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S146" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T146" s="3" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="3" t="inlineStr">
+        <is>
+          <t>Alchemy 16</t>
+        </is>
+      </c>
+      <c r="B147" s="3" t="inlineStr">
+        <is>
+          <t>Personal training studio</t>
+        </is>
+      </c>
+      <c r="C147" s="3" t="inlineStr">
+        <is>
+          <t>Imperial Square, Cheltenham</t>
+        </is>
+      </c>
+      <c r="D147" s="3" t="inlineStr">
+        <is>
+          <t>https://www.alchemy16.com</t>
+        </is>
+      </c>
+      <c r="E147" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F147" s="3" t="inlineStr"/>
+      <c r="G147" s="3" t="inlineStr">
+        <is>
+          <t>Patrick (Founder)</t>
+        </is>
+      </c>
+      <c r="H147" s="3" t="inlineStr"/>
+      <c r="I147" s="3" t="inlineStr"/>
+      <c r="J147" s="3" t="inlineStr">
+        <is>
+          <t>Bespoke luxury 1:1 studio in a Grade II* listed building overlooking Imperial Gardens; premium ongoing PT packages</t>
+        </is>
+      </c>
+      <c r="K147" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L147" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M147" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N147" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O147" s="3" t="inlineStr">
+        <is>
+          <t>Polished brand/site</t>
+        </is>
+      </c>
+      <c r="P147" s="3" t="inlineStr">
+        <is>
+          <t>Boutique studio invisible next to gym chains in 'personal trainer Cheltenham' searches</t>
+        </is>
+      </c>
+      <c r="Q147" s="3" t="inlineStr">
+        <is>
+          <t>'Cheltenham's most exclusive PT studio should be Cheltenham's top AI answer'</t>
+        </is>
+      </c>
+      <c r="R147" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S147" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T147" s="3" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="4" t="inlineStr">
+        <is>
+          <t>Rob Ingram Fitness</t>
+        </is>
+      </c>
+      <c r="B148" s="4" t="inlineStr">
+        <is>
+          <t>Personal training (1:1)</t>
+        </is>
+      </c>
+      <c r="C148" s="4" t="inlineStr">
+        <is>
+          <t>Cheltenham</t>
+        </is>
+      </c>
+      <c r="D148" s="4" t="inlineStr">
+        <is>
+          <t>https://www.robingramfitness.com</t>
+        </is>
+      </c>
+      <c r="E148" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F148" s="4" t="inlineStr"/>
+      <c r="G148" s="4" t="inlineStr">
+        <is>
+          <t>Rob Ingram (Founder)</t>
+        </is>
+      </c>
+      <c r="H148" s="4" t="inlineStr"/>
+      <c r="I148" s="4" t="inlineStr"/>
+      <c r="J148" s="4" t="inlineStr">
+        <is>
+          <t>Cheltenham's only dedicated 1:1 PT gym - strong differentiation story; high per-client value from ongoing sessions</t>
+        </is>
+      </c>
+      <c r="K148" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L148" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M148" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N148" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O148" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P148" s="4" t="inlineStr">
+        <is>
+          <t>'Only 1:1 gym in Cheltenham' claim isn't surfaced in local search</t>
+        </is>
+      </c>
+      <c r="Q148" s="4" t="inlineStr">
+        <is>
+          <t>Own the 'private personal trainer Cheltenham' niche outright</t>
+        </is>
+      </c>
+      <c r="R148" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S148" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T148" s="4" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="4" t="inlineStr">
+        <is>
+          <t>Infinite Balance</t>
+        </is>
+      </c>
+      <c r="B149" s="4" t="inlineStr">
+        <is>
+          <t>Personal training &amp; nutrition coaching</t>
+        </is>
+      </c>
+      <c r="C149" s="4" t="inlineStr">
+        <is>
+          <t>Hatherley, Cheltenham</t>
+        </is>
+      </c>
+      <c r="D149" s="4" t="inlineStr">
+        <is>
+          <t>https://infinitebalance.co.uk</t>
+        </is>
+      </c>
+      <c r="E149" s="4" t="inlineStr">
+        <is>
+          <t>kirsty@infinitebalance.co.uk</t>
+        </is>
+      </c>
+      <c r="F149" s="4" t="inlineStr"/>
+      <c r="G149" s="4" t="inlineStr">
+        <is>
+          <t>Kirsty Ellson (Founder)</t>
+        </is>
+      </c>
+      <c r="H149" s="4" t="inlineStr"/>
+      <c r="I149" s="4" t="inlineStr"/>
+      <c r="J149" s="4" t="inlineStr">
+        <is>
+          <t>Solo-led PT + nutrition coaching; ongoing client relationships worth £150-300/month each</t>
+        </is>
+      </c>
+      <c r="K149" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L149" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M149" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N149" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O149" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P149" s="4" t="inlineStr">
+        <is>
+          <t>Solo practitioner competing with studio brands for visibility</t>
+        </is>
+      </c>
+      <c r="Q149" s="4" t="inlineStr">
+        <is>
+          <t>Entry-tier local SEO to build a client base efficiently</t>
+        </is>
+      </c>
+      <c r="R149" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S149" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T149" s="4" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="3" t="inlineStr">
+        <is>
+          <t>The Avenue Pre-Prep &amp; Nursery</t>
+        </is>
+      </c>
+      <c r="B150" s="3" t="inlineStr">
+        <is>
+          <t>Private nursery/pre-prep school</t>
+        </is>
+      </c>
+      <c r="C150" s="3" t="inlineStr">
+        <is>
+          <t>Highgate, London N6</t>
+        </is>
+      </c>
+      <c r="D150" s="3" t="inlineStr">
+        <is>
+          <t>https://avenuepreprep.co.uk</t>
+        </is>
+      </c>
+      <c r="E150" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F150" s="3" t="inlineStr">
+        <is>
+          <t>020 8348 6815</t>
+        </is>
+      </c>
+      <c r="G150" s="3" t="inlineStr"/>
+      <c r="H150" s="3" t="inlineStr"/>
+      <c r="I150" s="3" t="inlineStr"/>
+      <c r="J150" s="3" t="inlineStr">
+        <is>
+          <t>Independent pre-prep serving Highgate/Hampstead/Muswell Hill; fees £15-20k/year, waitlist-driven demand</t>
+        </is>
+      </c>
+      <c r="K150" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L150" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M150" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N150" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O150" s="3" t="inlineStr">
+        <is>
+          <t>Established local reputation</t>
+        </is>
+      </c>
+      <c r="P150" s="3" t="inlineStr">
+        <is>
+          <t>Competing with Channing, Highgate Junior School feeder nurseries for the same wealthy families</t>
+        </is>
+      </c>
+      <c r="Q150" s="3" t="inlineStr">
+        <is>
+          <t>'Highgate parents research nurseries on Google before they call - be the first result'</t>
+        </is>
+      </c>
+      <c r="R150" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S150" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T150" s="3" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="4" t="inlineStr">
+        <is>
+          <t>The Gower School</t>
+        </is>
+      </c>
+      <c r="B151" s="4" t="inlineStr">
+        <is>
+          <t>Independent nursery (Montessori)</t>
+        </is>
+      </c>
+      <c r="C151" s="4" t="inlineStr">
+        <is>
+          <t>Islington, North London</t>
+        </is>
+      </c>
+      <c r="D151" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thegowerschool.co.uk</t>
+        </is>
+      </c>
+      <c r="E151" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F151" s="4" t="inlineStr"/>
+      <c r="G151" s="4" t="inlineStr"/>
+      <c r="H151" s="4" t="inlineStr"/>
+      <c r="I151" s="4" t="inlineStr"/>
+      <c r="J151" s="4" t="inlineStr">
+        <is>
+          <t>Montessori nursery serving Islington/Angel/Camden/Highbury; premium early-years fees</t>
+        </is>
+      </c>
+      <c r="K151" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L151" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M151" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N151" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O151" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P151" s="4" t="inlineStr">
+        <is>
+          <t>Montessori niche under-marketed vs bigger nursery chains</t>
+        </is>
+      </c>
+      <c r="Q151" s="4" t="inlineStr">
+        <is>
+          <t>Own 'Montessori nursery Islington' AEO content</t>
+        </is>
+      </c>
+      <c r="R151" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S151" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T151" s="4" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="3" t="inlineStr">
+        <is>
+          <t>Independent People Homecare</t>
+        </is>
+      </c>
+      <c r="B152" s="3" t="inlineStr">
+        <is>
+          <t>Live-in care agency</t>
+        </is>
+      </c>
+      <c r="C152" s="3" t="inlineStr">
+        <is>
+          <t>Guildford (serves Surrey/Oxfordshire)</t>
+        </is>
+      </c>
+      <c r="D152" s="3" t="inlineStr">
+        <is>
+          <t>via Oxfordshire family info service listing</t>
+        </is>
+      </c>
+      <c r="E152" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F152" s="3" t="inlineStr">
+        <is>
+          <t>0330 053 5014</t>
+        </is>
+      </c>
+      <c r="G152" s="3" t="inlineStr"/>
+      <c r="H152" s="3" t="inlineStr"/>
+      <c r="I152" s="3" t="inlineStr"/>
+      <c r="J152" s="3" t="inlineStr">
+        <is>
+          <t>Live-in care across two wealthy counties; clients worth £50-80k/year each</t>
+        </is>
+      </c>
+      <c r="K152" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L152" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M152" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N152" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O152" s="3" t="inlineStr">
+        <is>
+          <t>Council directory listing</t>
+        </is>
+      </c>
+      <c r="P152" s="3" t="inlineStr">
+        <is>
+          <t>Bigger national brands (Agincare, Helping Hands) dominate the same searches</t>
+        </is>
+      </c>
+      <c r="Q152" s="3" t="inlineStr">
+        <is>
+          <t>'One live-in care client is worth £60k/year - and families are asking AI, not just Google'</t>
+        </is>
+      </c>
+      <c r="R152" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S152" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T152" s="3" t="inlineStr">
+        <is>
+          <t>Confirm website URL before outreach</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="3" t="inlineStr">
+        <is>
+          <t>Solton Manor</t>
+        </is>
+      </c>
+      <c r="B153" s="3" t="inlineStr">
+        <is>
+          <t>Wedding venue</t>
+        </is>
+      </c>
+      <c r="C153" s="3" t="inlineStr">
+        <is>
+          <t>East Langdon, Dover, Kent</t>
+        </is>
+      </c>
+      <c r="D153" s="3" t="inlineStr">
+        <is>
+          <t>https://www.soltonmanor.com</t>
+        </is>
+      </c>
+      <c r="E153" s="3" t="inlineStr">
+        <is>
+          <t>info@soltonmanor.com</t>
+        </is>
+      </c>
+      <c r="F153" s="3" t="inlineStr">
+        <is>
+          <t>01304 448 844</t>
+        </is>
+      </c>
+      <c r="G153" s="3" t="inlineStr"/>
+      <c r="H153" s="3" t="inlineStr"/>
+      <c r="I153" s="3" t="inlineStr"/>
+      <c r="J153" s="3" t="inlineStr">
+        <is>
+          <t>Grade II listed 9-acre manor/barn venue in Kent; weddings worth £15-30k each</t>
+        </is>
+      </c>
+      <c r="K153" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L153" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M153" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N153" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O153" s="3" t="inlineStr">
+        <is>
+          <t>Multiple directory listings (Guides for Brides, Bridebook, Married in Kent)</t>
+        </is>
+      </c>
+      <c r="P153" s="3" t="inlineStr">
+        <is>
+          <t>Heavy directory dependence; couples increasingly ask AI for shortlists directly</t>
+        </is>
+      </c>
+      <c r="Q153" s="3" t="inlineStr">
+        <is>
+          <t>'Reduce commission paid to wedding directories - own the AI-recommended shortlist instead'</t>
+        </is>
+      </c>
+      <c r="R153" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S153" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T153" s="3" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="3" t="inlineStr">
+        <is>
+          <t>The Oak Barn, Frame Farm</t>
+        </is>
+      </c>
+      <c r="B154" s="3" t="inlineStr">
+        <is>
+          <t>Wedding venue</t>
+        </is>
+      </c>
+      <c r="C154" s="3" t="inlineStr">
+        <is>
+          <t>Kent/Sussex border</t>
+        </is>
+      </c>
+      <c r="D154" s="3" t="inlineStr">
+        <is>
+          <t>https://www.the-oak-barn.co.uk</t>
+        </is>
+      </c>
+      <c r="E154" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F154" s="3" t="inlineStr"/>
+      <c r="G154" s="3" t="inlineStr">
+        <is>
+          <t>The Maw family (Owners)</t>
+        </is>
+      </c>
+      <c r="H154" s="3" t="inlineStr"/>
+      <c r="I154" s="3" t="inlineStr"/>
+      <c r="J154" s="3" t="inlineStr">
+        <is>
+          <t>Family-run barn venue in AONB; personalised-service positioning; high per-booking value</t>
+        </is>
+      </c>
+      <c r="K154" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L154" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M154" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N154" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O154" s="3" t="inlineStr">
+        <is>
+          <t>Directory listings</t>
+        </is>
+      </c>
+      <c r="P154" s="3" t="inlineStr">
+        <is>
+          <t>Family-run charm doesn't show up in generic 'barn wedding venue Kent' searches</t>
+        </is>
+      </c>
+      <c r="Q154" s="3" t="inlineStr">
+        <is>
+          <t>'Your family story is the differentiator - make it the AI-cited one'</t>
+        </is>
+      </c>
+      <c r="R154" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S154" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T154" s="3" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="4" t="inlineStr">
+        <is>
+          <t>Rivervale Barn</t>
+        </is>
+      </c>
+      <c r="B155" s="4" t="inlineStr">
+        <is>
+          <t>Wedding venue</t>
+        </is>
+      </c>
+      <c r="C155" s="4" t="inlineStr">
+        <is>
+          <t>Yateley, Hampshire</t>
+        </is>
+      </c>
+      <c r="D155" s="4" t="inlineStr">
+        <is>
+          <t>https://www.rivervalebarn.co.uk</t>
+        </is>
+      </c>
+      <c r="E155" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F155" s="4" t="inlineStr"/>
+      <c r="G155" s="4" t="inlineStr"/>
+      <c r="H155" s="4" t="inlineStr"/>
+      <c r="I155" s="4" t="inlineStr"/>
+      <c r="J155" s="4" t="inlineStr">
+        <is>
+          <t>Riverside barn venue in Hampshire; multiple barn options = flexible high-value bookings</t>
+        </is>
+      </c>
+      <c r="K155" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L155" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M155" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N155" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O155" s="4" t="inlineStr">
+        <is>
+          <t>Directory listings</t>
+        </is>
+      </c>
+      <c r="P155" s="4" t="inlineStr">
+        <is>
+          <t>Hampshire wedding-venue searches split across many similar barn venues</t>
+        </is>
+      </c>
+      <c r="Q155" s="4" t="inlineStr">
+        <is>
+          <t>Differentiate via riverside setting in AEO content</t>
+        </is>
+      </c>
+      <c r="R155" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S155" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T155" s="4" t="inlineStr">
+        <is>
+          <t>Verify site URL and contact before outreach</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="4" t="inlineStr">
+        <is>
+          <t>Watkins Solicitors</t>
+        </is>
+      </c>
+      <c r="B156" s="4" t="inlineStr">
+        <is>
+          <t>Law firm (conveyancing/family)</t>
+        </is>
+      </c>
+      <c r="C156" s="4" t="inlineStr">
+        <is>
+          <t>Bristol, Bath, Hereford, Evesham</t>
+        </is>
+      </c>
+      <c r="D156" s="4" t="inlineStr">
+        <is>
+          <t>https://www.watkinssolicitors.co.uk</t>
+        </is>
+      </c>
+      <c r="E156" s="4" t="inlineStr">
+        <is>
+          <t>info@watkinssolicitors.co.uk</t>
+        </is>
+      </c>
+      <c r="F156" s="4" t="inlineStr"/>
+      <c r="G156" s="4" t="inlineStr"/>
+      <c r="H156" s="4" t="inlineStr"/>
+      <c r="I156" s="4" t="inlineStr"/>
+      <c r="J156" s="4" t="inlineStr">
+        <is>
+          <t>Multi-office regional independent; conveyancing volume + family law = steady high-value pipeline</t>
+        </is>
+      </c>
+      <c r="K156" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L156" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M156" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N156" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O156" s="4" t="inlineStr">
+        <is>
+          <t>Multi-office site</t>
+        </is>
+      </c>
+      <c r="P156" s="4" t="inlineStr">
+        <is>
+          <t>Comparison sites (Compare My Move) intercept conveyancing searches before firms are found</t>
+        </is>
+      </c>
+      <c r="Q156" s="4" t="inlineStr">
+        <is>
+          <t>Local-office AEO: own 'conveyancing solicitor Bath' per branch</t>
+        </is>
+      </c>
+      <c r="R156" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S156" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T156" s="4" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="4" t="inlineStr">
+        <is>
+          <t>Battrick Clark Solicitors</t>
+        </is>
+      </c>
+      <c r="B157" s="4" t="inlineStr">
+        <is>
+          <t>Law firm</t>
+        </is>
+      </c>
+      <c r="C157" s="4" t="inlineStr">
+        <is>
+          <t>Whiteladies Rd, Clifton, Bristol</t>
+        </is>
+      </c>
+      <c r="D157" s="4" t="inlineStr">
+        <is>
+          <t>https://www.battrickclark.co.uk</t>
+        </is>
+      </c>
+      <c r="E157" s="4" t="inlineStr">
+        <is>
+          <t>info@battrickclark.co.uk</t>
+        </is>
+      </c>
+      <c r="F157" s="4" t="inlineStr">
+        <is>
+          <t>0117 973 1391</t>
+        </is>
+      </c>
+      <c r="G157" s="4" t="inlineStr"/>
+      <c r="H157" s="4" t="inlineStr"/>
+      <c r="I157" s="4" t="inlineStr"/>
+      <c r="J157" s="4" t="inlineStr">
+        <is>
+          <t>Established 1997, full-service firm on Bristol's professional strip; conveyancing + family + private client</t>
+        </is>
+      </c>
+      <c r="K157" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L157" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M157" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N157" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O157" s="4" t="inlineStr">
+        <is>
+          <t>Established brand</t>
+        </is>
+      </c>
+      <c r="P157" s="4" t="inlineStr">
+        <is>
+          <t>Generalist positioning competes with both boutiques and volume conveyancers</t>
+        </is>
+      </c>
+      <c r="Q157" s="4" t="inlineStr">
+        <is>
+          <t>Pick one high-value practice area to own in AI answers first</t>
+        </is>
+      </c>
+      <c r="R157" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S157" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T157" s="4" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="3" t="inlineStr">
+        <is>
+          <t>Danielle Cohen Immigration Law Solicitors</t>
+        </is>
+      </c>
+      <c r="B158" s="3" t="inlineStr">
+        <is>
+          <t>Immigration law firm</t>
+        </is>
+      </c>
+      <c r="C158" s="3" t="inlineStr">
+        <is>
+          <t>Camden, London NW1</t>
+        </is>
+      </c>
+      <c r="D158" s="3" t="inlineStr">
+        <is>
+          <t>https://daniellecohenimmigration.com</t>
+        </is>
+      </c>
+      <c r="E158" s="3" t="inlineStr">
+        <is>
+          <t>danielle.cohen@daniellecohen.co.uk</t>
+        </is>
+      </c>
+      <c r="F158" s="3" t="inlineStr">
+        <is>
+          <t>020 7267 4133</t>
+        </is>
+      </c>
+      <c r="G158" s="3" t="inlineStr">
+        <is>
+          <t>Danielle Cohen (Founder)</t>
+        </is>
+      </c>
+      <c r="H158" s="3" t="inlineStr"/>
+      <c r="I158" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/daniellecohensolicitors</t>
+        </is>
+      </c>
+      <c r="J158" s="3" t="inlineStr">
+        <is>
+          <t>20+ year specialist niche firm; visa/immigration cases worth £2-10k in fees; founder name = brand</t>
+        </is>
+      </c>
+      <c r="K158" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L158" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M158" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N158" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O158" s="3" t="inlineStr">
+        <is>
+          <t>YouTube channel; Facebook page - content-aware</t>
+        </is>
+      </c>
+      <c r="P158" s="3" t="inlineStr">
+        <is>
+          <t>Content exists but AI engines cite bigger immigration brands (IAS, Migrate) for generic queries</t>
+        </is>
+      </c>
+      <c r="Q158" s="3" t="inlineStr">
+        <is>
+          <t>Turn founder's 20-year expertise into the AI-cited answer for complex visa questions</t>
+        </is>
+      </c>
+      <c r="R158" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S158" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T158" s="3" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="3" t="inlineStr">
+        <is>
+          <t>Garth Coates Solicitors</t>
+        </is>
+      </c>
+      <c r="B159" s="3" t="inlineStr">
+        <is>
+          <t>Immigration law firm</t>
+        </is>
+      </c>
+      <c r="C159" s="3" t="inlineStr">
+        <is>
+          <t>Holborn, London WC1</t>
+        </is>
+      </c>
+      <c r="D159" s="3" t="inlineStr">
+        <is>
+          <t>https://garthcoates.com</t>
+        </is>
+      </c>
+      <c r="E159" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F159" s="3" t="inlineStr">
+        <is>
+          <t>020 7799 1600</t>
+        </is>
+      </c>
+      <c r="G159" s="3" t="inlineStr">
+        <is>
+          <t>Garth Coates (Founder)</t>
+        </is>
+      </c>
+      <c r="H159" s="3" t="inlineStr"/>
+      <c r="I159" s="3" t="inlineStr">
+        <is>
+          <t>instagram.com/garthcoatessol</t>
+        </is>
+      </c>
+      <c r="J159" s="3" t="inlineStr">
+        <is>
+          <t>Est. 2008 boutique immigration specialist; high-value work visa and citizenship cases</t>
+        </is>
+      </c>
+      <c r="K159" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L159" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M159" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N159" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O159" s="3" t="inlineStr">
+        <is>
+          <t>Instagram presence</t>
+        </is>
+      </c>
+      <c r="P159" s="3" t="inlineStr">
+        <is>
+          <t>Generic 'immigration solicitor London' searches won by volume firms with bigger ad spend</t>
+        </is>
+      </c>
+      <c r="Q159" s="3" t="inlineStr">
+        <is>
+          <t>AEO for specific high-value queries (Innovator visa, Global Talent) where boutiques can win</t>
+        </is>
+      </c>
+      <c r="R159" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S159" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T159" s="3" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="4" t="inlineStr">
+        <is>
+          <t>Vanessa Ganguin Immigration Law</t>
+        </is>
+      </c>
+      <c r="B160" s="4" t="inlineStr">
+        <is>
+          <t>Immigration law firm</t>
+        </is>
+      </c>
+      <c r="C160" s="4" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D160" s="4" t="inlineStr">
+        <is>
+          <t>https://vanessaganguin.com</t>
+        </is>
+      </c>
+      <c r="E160" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F160" s="4" t="inlineStr"/>
+      <c r="G160" s="4" t="inlineStr">
+        <is>
+          <t>Vanessa Ganguin (Founder)</t>
+        </is>
+      </c>
+      <c r="H160" s="4" t="inlineStr"/>
+      <c r="I160" s="4" t="inlineStr"/>
+      <c r="J160" s="4" t="inlineStr">
+        <is>
+          <t>Partner-led boutique with decades of experience; multi-city presence (also lists Bristol)</t>
+        </is>
+      </c>
+      <c r="K160" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L160" s="4" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M160" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N160" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O160" s="4" t="inlineStr">
+        <is>
+          <t>Multi-city professional site</t>
+        </is>
+      </c>
+      <c r="P160" s="4" t="inlineStr">
+        <is>
+          <t>Boutique quality buried under bigger firms' search spend</t>
+        </is>
+      </c>
+      <c r="Q160" s="4" t="inlineStr">
+        <is>
+          <t>Position as the boutique alternative in AI-generated shortlists</t>
+        </is>
+      </c>
+      <c r="R160" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S160" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T160" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T129"/>
+  <autoFilter ref="A1:T160"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11740,7 +14368,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B85"/>
+  <dimension ref="A1:B95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -11760,7 +14388,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>128</v>
+        <v>159</v>
       </c>
     </row>
     <row r="5">
@@ -11777,7 +14405,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
@@ -11787,93 +14415,93 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Physiotherapy clinic</t>
+          <t>Architects</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Solar installer</t>
+          <t>Independent vet</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Estate &amp; letting agent</t>
+          <t>Wedding venue</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Mortgage broker</t>
+          <t>Estate &amp; letting agent</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Chartered accountants</t>
+          <t>Mortgage broker</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Independent vet</t>
+          <t>Physiotherapy clinic</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Private GP</t>
+          <t>Solar installer</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Family law firm</t>
+          <t>Aesthetics clinic</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Architects</t>
+          <t>Law firm</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -11883,57 +14511,57 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Law firm</t>
+          <t>Chartered accountants</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Letting agent</t>
+          <t>Private GP</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Wedding venue</t>
+          <t>Personal training studio</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Financial adviser / wealth management</t>
+          <t>Family law firm</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Private tuition agency</t>
+          <t>Immigration law firm</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Osteopathy clinic</t>
+          <t>Letting agent</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -11943,7 +14571,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating / boilers</t>
+          <t>Financial adviser / wealth management</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -11953,7 +14581,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Electrician</t>
+          <t>Private tuition agency</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -11963,7 +14591,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Event &amp; wedding caterer</t>
+          <t>Osteopathy clinic</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -11973,7 +14601,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Personal training studio</t>
+          <t>Plumbing &amp; heating / boilers</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -11983,7 +14611,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Chiropractor</t>
+          <t>Electrician</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -11993,7 +14621,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Orthodontist</t>
+          <t>Event &amp; wedding caterer</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -12003,7 +14631,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Aesthetics clinic</t>
+          <t>Chiropractor</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -12013,7 +14641,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Employment law firm</t>
+          <t>Orthodontist</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -12023,7 +14651,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Event management agency</t>
+          <t>Employment law firm</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -12033,7 +14661,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Design &amp; build</t>
+          <t>Event management agency</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -12043,7 +14671,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Recruitment agency</t>
+          <t>Design &amp; build</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -12053,27 +14681,27 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Dentist / Orthodontics</t>
+          <t>Recruitment agency</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Specialist dental/implant clinic</t>
+          <t>IT support / MSP</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Boutique corporate law firm</t>
+          <t>Dentist / Orthodontics</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -12083,7 +14711,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Cosmetic/aesthetics clinic</t>
+          <t>Specialist dental/implant clinic</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -12093,7 +14721,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Skin &amp; laser clinic</t>
+          <t>Boutique corporate law firm</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -12103,7 +14731,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Mortgage broker / financial adviser</t>
+          <t>Cosmetic/aesthetics clinic</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -12113,7 +14741,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Architects (RIBA chartered)</t>
+          <t>Skin &amp; laser clinic</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -12123,7 +14751,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Recruitment agency (tech/startups)</t>
+          <t>Mortgage broker / financial adviser</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -12133,7 +14761,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Recruitment agency (IT/data)</t>
+          <t>Architects (RIBA chartered)</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -12143,7 +14771,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Independent vet (24/7 emergency)</t>
+          <t>Recruitment agency (tech/startups)</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -12153,7 +14781,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Interior design studio</t>
+          <t>Recruitment agency (IT/data)</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -12163,7 +14791,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Letting &amp; estate agent</t>
+          <t>Independent vet (24/7 emergency)</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -12173,7 +14801,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Cosmetic clinic (injectables)</t>
+          <t>Interior design studio</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -12183,7 +14811,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Cosmetic/anti-ageing clinic</t>
+          <t>Letting &amp; estate agent</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -12193,7 +14821,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Yoga &amp; reformer pilates studio</t>
+          <t>Cosmetic clinic (injectables)</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -12203,7 +14831,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Reformer pilates studio</t>
+          <t>Cosmetic/anti-ageing clinic</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -12213,7 +14841,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Wealth management</t>
+          <t>Yoga &amp; reformer pilates studio</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -12223,7 +14851,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Private tuition &amp; education consultancy</t>
+          <t>Reformer pilates studio</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -12233,7 +14861,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Osteopath</t>
+          <t>Wealth management</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -12243,7 +14871,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Design &amp; build / home renovation</t>
+          <t>Private tuition &amp; education consultancy</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -12253,7 +14881,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Builders / building contractor</t>
+          <t>Osteopath</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -12263,7 +14891,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Roofer</t>
+          <t>Design &amp; build / home renovation</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -12273,7 +14901,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Home care / live-in care</t>
+          <t>Builders / building contractor</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -12283,7 +14911,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Private day nurseries</t>
+          <t>Roofer</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -12293,7 +14921,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Personal training &amp; wellness studio</t>
+          <t>Home care / live-in care</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -12303,7 +14931,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Mortgage &amp; insurance broker</t>
+          <t>Private day nurseries</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -12313,7 +14941,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Business consultancy</t>
+          <t>Personal training &amp; wellness studio</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -12323,7 +14951,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Interior designer (period homes)</t>
+          <t>Mortgage &amp; insurance broker</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -12333,7 +14961,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Landscape design &amp; build</t>
+          <t>Business consultancy</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -12343,7 +14971,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Estate agent (premium)</t>
+          <t>Interior designer (period homes)</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -12353,7 +14981,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Interior designer</t>
+          <t>Landscape design &amp; build</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -12363,7 +14991,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Garden design &amp; landscaping</t>
+          <t>Estate agent (premium)</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -12373,7 +15001,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Legal recruitment</t>
+          <t>Interior designer</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -12383,7 +15011,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Independent gym &amp; health club</t>
+          <t>Garden design &amp; landscaping</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -12393,7 +15021,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Independent gym</t>
+          <t>Legal recruitment</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -12403,7 +15031,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Physiotherapy (sports)</t>
+          <t>Independent gym &amp; health club</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -12413,7 +15041,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Letting agent / property management</t>
+          <t>Independent gym</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -12423,7 +15051,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Skin clinic</t>
+          <t>Physiotherapy (sports)</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -12433,7 +15061,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Tutoring company</t>
+          <t>Letting agent / property management</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -12443,7 +15071,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Tutorial college &amp; exam centre</t>
+          <t>Skin clinic</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -12453,7 +15081,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Employment law (disability discrimination)</t>
+          <t>Tutoring company</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -12463,7 +15091,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating</t>
+          <t>Tutorial college &amp; exam centre</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -12473,7 +15101,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Employment law (disability discrimination)</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -12483,7 +15111,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Sports physio &amp; massage</t>
+          <t>Plumbing &amp; heating</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -12493,7 +15121,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Chartered surveyors (party wall/building)</t>
+          <t>Plumbing</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -12503,7 +15131,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Chartered surveyors</t>
+          <t>Sports physio &amp; massage</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -12513,7 +15141,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Chartered building surveyors</t>
+          <t>Chartered surveyors (party wall/building)</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -12523,7 +15151,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Osteopathy clinics</t>
+          <t>Chartered surveyors</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -12533,7 +15161,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Private dentist / implants</t>
+          <t>Chartered building surveyors</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -12543,7 +15171,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Builders / renovations</t>
+          <t>Osteopathy clinics</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -12553,7 +15181,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Private nursery schools</t>
+          <t>Private dentist / implants</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -12563,10 +15191,110 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
+          <t>Builders / renovations</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Private nursery schools</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
           <t>Private day nursery</t>
         </is>
       </c>
-      <c r="B85" t="n">
+      <c r="B87" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Private GP (membership model)</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Sash window restoration</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Personal training (1:1)</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Personal training &amp; nutrition coaching</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Private nursery/pre-prep school</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Independent nursery (Montessori)</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Live-in care agency</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Law firm (conveyancing/family)</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 6: +15 prospects (174 total) - Henley, Marlow, Blackheath, Notting Hill, Winchester
New geographies: Henley-on-Thames, Marlow, Beaconsfield, Blackheath, Notting
Hill, Winchester, Bicester, Chipping Norton.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$160</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$175</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T160"/>
+  <dimension ref="A1:T175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -14356,8 +14356,1292 @@
       </c>
       <c r="T160" s="4" t="inlineStr"/>
     </row>
+    <row r="161">
+      <c r="A161" s="3" t="inlineStr">
+        <is>
+          <t>Philip Booth Esq</t>
+        </is>
+      </c>
+      <c r="B161" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C161" s="3" t="inlineStr">
+        <is>
+          <t>Henley-on-Thames &amp; Marlow</t>
+        </is>
+      </c>
+      <c r="D161" s="3" t="inlineStr">
+        <is>
+          <t>https://www.philipboothesq.com</t>
+        </is>
+      </c>
+      <c r="E161" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F161" s="3" t="inlineStr"/>
+      <c r="G161" s="3" t="inlineStr">
+        <is>
+          <t>Phil Booth (Director, 37+ yrs experience)</t>
+        </is>
+      </c>
+      <c r="H161" s="3" t="inlineStr"/>
+      <c r="I161" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/PhilipBoothesq</t>
+        </is>
+      </c>
+      <c r="J161" s="3" t="inlineStr">
+        <is>
+          <t>Leading independent across two of the Thames Valley's wealthiest towns; premium riverside/village property fees</t>
+        </is>
+      </c>
+      <c r="K161" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L161" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M161" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N161" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O161" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence</t>
+        </is>
+      </c>
+      <c r="P161" s="3" t="inlineStr">
+        <is>
+          <t>Ballards and Stowhill compete for the same Henley/Marlow searches</t>
+        </is>
+      </c>
+      <c r="Q161" s="3" t="inlineStr">
+        <is>
+          <t>'Henley sellers ask AI who knows the river towns best - be that answer'</t>
+        </is>
+      </c>
+      <c r="R161" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S161" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T161" s="3" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="3" t="inlineStr">
+        <is>
+          <t>Ballards Estate Agents</t>
+        </is>
+      </c>
+      <c r="B162" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C162" s="3" t="inlineStr">
+        <is>
+          <t>Henley-on-Thames, Marlow, Twyford</t>
+        </is>
+      </c>
+      <c r="D162" s="3" t="inlineStr">
+        <is>
+          <t>https://ballards-uk.com</t>
+        </is>
+      </c>
+      <c r="E162" s="3" t="inlineStr">
+        <is>
+          <t>nicky@ballards-uk.com</t>
+        </is>
+      </c>
+      <c r="F162" s="3" t="inlineStr">
+        <is>
+          <t>01491 411 055</t>
+        </is>
+      </c>
+      <c r="G162" s="3" t="inlineStr">
+        <is>
+          <t>Chris (Founder, opened 1990)</t>
+        </is>
+      </c>
+      <c r="H162" s="3" t="inlineStr"/>
+      <c r="I162" s="3" t="inlineStr"/>
+      <c r="J162" s="3" t="inlineStr">
+        <is>
+          <t>Family-owned since 1990, award-winning, three-office Thames Valley coverage; instructions worth thousands each</t>
+        </is>
+      </c>
+      <c r="K162" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L162" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M162" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N162" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O162" s="3" t="inlineStr">
+        <is>
+          <t>Award mentions; multi-office presence</t>
+        </is>
+      </c>
+      <c r="P162" s="3" t="inlineStr">
+        <is>
+          <t>Three offices but fragmented digital visibility vs single-minded corporate rivals</t>
+        </is>
+      </c>
+      <c r="Q162" s="3" t="inlineStr">
+        <is>
+          <t>Per-office local SEO + unified AEO strategy across all three towns</t>
+        </is>
+      </c>
+      <c r="R162" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S162" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T162" s="3" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="3" t="inlineStr">
+        <is>
+          <t>Stowhill Estates Buckinghamshire</t>
+        </is>
+      </c>
+      <c r="B163" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent (premium)</t>
+        </is>
+      </c>
+      <c r="C163" s="3" t="inlineStr">
+        <is>
+          <t>Marlow, South Buckinghamshire</t>
+        </is>
+      </c>
+      <c r="D163" s="3" t="inlineStr">
+        <is>
+          <t>https://stowhillbucks.co.uk</t>
+        </is>
+      </c>
+      <c r="E163" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F163" s="3" t="inlineStr"/>
+      <c r="G163" s="3" t="inlineStr">
+        <is>
+          <t>David &amp; Sara (Founders, husband &amp; wife)</t>
+        </is>
+      </c>
+      <c r="H163" s="3" t="inlineStr"/>
+      <c r="I163" s="3" t="inlineStr"/>
+      <c r="J163" s="3" t="inlineStr">
+        <is>
+          <t>Boutique premium-only agency in one of the UK's wealthiest commuter belts; explicit premium positioning</t>
+        </is>
+      </c>
+      <c r="K163" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L163" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M163" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N163" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O163" s="3" t="inlineStr">
+        <is>
+          <t>Premium brand positioning</t>
+        </is>
+      </c>
+      <c r="P163" s="3" t="inlineStr">
+        <is>
+          <t>Niche premium focus not yet AI-search dominant vs bigger names</t>
+        </is>
+      </c>
+      <c r="Q163" s="3" t="inlineStr">
+        <is>
+          <t>'Premium-only' as the AEO hook: own that exact positioning in AI answers</t>
+        </is>
+      </c>
+      <c r="R163" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S163" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T163" s="3" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="3" t="inlineStr">
+        <is>
+          <t>Comber &amp; Company</t>
+        </is>
+      </c>
+      <c r="B164" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C164" s="3" t="inlineStr">
+        <is>
+          <t>Blackheath Village, London SE3</t>
+        </is>
+      </c>
+      <c r="D164" s="3" t="inlineStr">
+        <is>
+          <t>https://www.comberandco.co.uk</t>
+        </is>
+      </c>
+      <c r="E164" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F164" s="3" t="inlineStr">
+        <is>
+          <t>020 3641 5310</t>
+        </is>
+      </c>
+      <c r="G164" s="3" t="inlineStr">
+        <is>
+          <t>Jeremy Comber (Founder, since 1993)</t>
+        </is>
+      </c>
+      <c r="H164" s="3" t="inlineStr"/>
+      <c r="I164" s="3" t="inlineStr"/>
+      <c r="J164" s="3" t="inlineStr">
+        <is>
+          <t>Independent family firm in affluent Blackheath Village since 1993; sales+lettings+surveying under one roof</t>
+        </is>
+      </c>
+      <c r="K164" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L164" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M164" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N164" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O164" s="3" t="inlineStr">
+        <is>
+          <t>30+ years reputation</t>
+        </is>
+      </c>
+      <c r="P164" s="3" t="inlineStr">
+        <is>
+          <t>Winkworth/FJLord/Truepenny's all fight for the same Blackheath searches</t>
+        </is>
+      </c>
+      <c r="Q164" s="3" t="inlineStr">
+        <is>
+          <t>'32 years in Blackheath Village - make Google and ChatGPT say so too'</t>
+        </is>
+      </c>
+      <c r="R164" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S164" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T164" s="3" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="3" t="inlineStr">
+        <is>
+          <t>Rigby &amp; Marchant</t>
+        </is>
+      </c>
+      <c r="B165" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C165" s="3" t="inlineStr">
+        <is>
+          <t>Notting Hill, London W10/W11</t>
+        </is>
+      </c>
+      <c r="D165" s="3" t="inlineStr">
+        <is>
+          <t>https://rigbyandmarchant.co.uk</t>
+        </is>
+      </c>
+      <c r="E165" s="3" t="inlineStr">
+        <is>
+          <t>sales@rigbyandmarchant.co.uk</t>
+        </is>
+      </c>
+      <c r="F165" s="3" t="inlineStr">
+        <is>
+          <t>020 7221 7210</t>
+        </is>
+      </c>
+      <c r="G165" s="3" t="inlineStr">
+        <is>
+          <t>Keith Rigby, Matt Marchant &amp; Fraser Clark (Founders, 1996)</t>
+        </is>
+      </c>
+      <c r="H165" s="3" t="inlineStr"/>
+      <c r="I165" s="3" t="inlineStr"/>
+      <c r="J165" s="3" t="inlineStr">
+        <is>
+          <t>Independent since 1996 in one of London's priciest postcodes; instructions worth substantial fees each</t>
+        </is>
+      </c>
+      <c r="K165" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L165" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M165" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N165" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O165" s="3" t="inlineStr">
+        <is>
+          <t>Established local brand</t>
+        </is>
+      </c>
+      <c r="P165" s="3" t="inlineStr">
+        <is>
+          <t>Domus Nova and corporate giants (Knight Frank, Marsh &amp; Parsons) dominate W11 search</t>
+        </is>
+      </c>
+      <c r="Q165" s="3" t="inlineStr">
+        <is>
+          <t>'Notting Hill sellers now ask AI, not just Rightmove - own that answer'</t>
+        </is>
+      </c>
+      <c r="R165" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S165" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T165" s="3" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="4" t="inlineStr">
+        <is>
+          <t>St Cuthbert's Dental Surgery</t>
+        </is>
+      </c>
+      <c r="B166" s="4" t="inlineStr">
+        <is>
+          <t>Private dentist</t>
+        </is>
+      </c>
+      <c r="C166" s="4" t="inlineStr">
+        <is>
+          <t>Newburgh St, Winchester, Hampshire</t>
+        </is>
+      </c>
+      <c r="D166" s="4" t="inlineStr">
+        <is>
+          <t>https://www.stcuthbertsdentalsurgery.co.uk</t>
+        </is>
+      </c>
+      <c r="E166" s="4" t="inlineStr">
+        <is>
+          <t>info@stcuthbertsdentalsurgery.co.uk</t>
+        </is>
+      </c>
+      <c r="F166" s="4" t="inlineStr">
+        <is>
+          <t>01962 853135</t>
+        </is>
+      </c>
+      <c r="G166" s="4" t="inlineStr"/>
+      <c r="H166" s="4" t="inlineStr"/>
+      <c r="I166" s="4" t="inlineStr">
+        <is>
+          <t>facebook.com/StCuthbertsDentalSurgery</t>
+        </is>
+      </c>
+      <c r="J166" s="4" t="inlineStr">
+        <is>
+          <t>Private practice in Winchester city centre; senior team with long tenure; affluent cathedral-city catchment</t>
+        </is>
+      </c>
+      <c r="K166" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L166" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M166" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N166" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O166" s="4" t="inlineStr">
+        <is>
+          <t>Facebook page</t>
+        </is>
+      </c>
+      <c r="P166" s="4" t="inlineStr">
+        <is>
+          <t>Bupa and newer clinics (Solutions Dental) outspend on Winchester dental search</t>
+        </is>
+      </c>
+      <c r="Q166" s="4" t="inlineStr">
+        <is>
+          <t>'Winchester patients ask AI for a dentist near the cathedral - be the answer'</t>
+        </is>
+      </c>
+      <c r="R166" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S166" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T166" s="4" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="3" t="inlineStr">
+        <is>
+          <t>Solutions Dental Clinic</t>
+        </is>
+      </c>
+      <c r="B167" s="3" t="inlineStr">
+        <is>
+          <t>Private dentist / implants</t>
+        </is>
+      </c>
+      <c r="C167" s="3" t="inlineStr">
+        <is>
+          <t>Winchester, Hampshire</t>
+        </is>
+      </c>
+      <c r="D167" s="3" t="inlineStr">
+        <is>
+          <t>https://www.solutionsdentalclinic.co.uk</t>
+        </is>
+      </c>
+      <c r="E167" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F167" s="3" t="inlineStr">
+        <is>
+          <t>01962 864 655</t>
+        </is>
+      </c>
+      <c r="G167" s="3" t="inlineStr"/>
+      <c r="H167" s="3" t="inlineStr"/>
+      <c r="I167" s="3" t="inlineStr"/>
+      <c r="J167" s="3" t="inlineStr">
+        <is>
+          <t>Implant-focused private clinic in Winchester; £3-10k implant cases in a wealthy cathedral city</t>
+        </is>
+      </c>
+      <c r="K167" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L167" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M167" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N167" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O167" s="3" t="inlineStr">
+        <is>
+          <t>Dedicated implants landing page</t>
+        </is>
+      </c>
+      <c r="P167" s="3" t="inlineStr">
+        <is>
+          <t>Implant searches contested locally but AI-answer visibility still open</t>
+        </is>
+      </c>
+      <c r="Q167" s="3" t="inlineStr">
+        <is>
+          <t>'Own "dental implants Winchester" - a high-value niche with room at the top'</t>
+        </is>
+      </c>
+      <c r="R167" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S167" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T167" s="3" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="3" t="inlineStr">
+        <is>
+          <t>YK Design</t>
+        </is>
+      </c>
+      <c r="B168" s="3" t="inlineStr">
+        <is>
+          <t>Architect &amp; interior designer</t>
+        </is>
+      </c>
+      <c r="C168" s="3" t="inlineStr">
+        <is>
+          <t>Henley-on-Thames</t>
+        </is>
+      </c>
+      <c r="D168" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ykdesign.co.uk</t>
+        </is>
+      </c>
+      <c r="E168" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F168" s="3" t="inlineStr"/>
+      <c r="G168" s="3" t="inlineStr">
+        <is>
+          <t>Yasemin Kirkpatrick (Founder, RIBA, est. 2005)</t>
+        </is>
+      </c>
+      <c r="H168" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/yasemin-kirkpatrick-93533369</t>
+        </is>
+      </c>
+      <c r="I168" s="3" t="inlineStr"/>
+      <c r="J168" s="3" t="inlineStr">
+        <is>
+          <t>20-year practice combining architecture + interiors for Thames Valley homes; project values £100k-1m+</t>
+        </is>
+      </c>
+      <c r="K168" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L168" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M168" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N168" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O168" s="3" t="inlineStr">
+        <is>
+          <t>Professional portfolio site</t>
+        </is>
+      </c>
+      <c r="P168" s="3" t="inlineStr">
+        <is>
+          <t>Combined architecture+interiors offering underexploited in local AI search</t>
+        </is>
+      </c>
+      <c r="Q168" s="3" t="inlineStr">
+        <is>
+          <t>'One Henley client is worth years of our fee - be the AI's Henley architect'</t>
+        </is>
+      </c>
+      <c r="R168" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S168" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T168" s="3" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="3" t="inlineStr">
+        <is>
+          <t>Trace Architects</t>
+        </is>
+      </c>
+      <c r="B169" s="3" t="inlineStr">
+        <is>
+          <t>Architects</t>
+        </is>
+      </c>
+      <c r="C169" s="3" t="inlineStr">
+        <is>
+          <t>London &amp; Henley-on-Thames</t>
+        </is>
+      </c>
+      <c r="D169" s="3" t="inlineStr">
+        <is>
+          <t>https://tracearchitects.format.com</t>
+        </is>
+      </c>
+      <c r="E169" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F169" s="3" t="inlineStr"/>
+      <c r="G169" s="3" t="inlineStr">
+        <is>
+          <t>Giles Lovegrove &amp; Kristian Rapallini (Founders)</t>
+        </is>
+      </c>
+      <c r="H169" s="3" t="inlineStr"/>
+      <c r="I169" s="3" t="inlineStr"/>
+      <c r="J169" s="3" t="inlineStr">
+        <is>
+          <t>Two-studio practice (London + Henley) for high-end residential; decades of combined experience at leading firms</t>
+        </is>
+      </c>
+      <c r="K169" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L169" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M169" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N169" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O169" s="3" t="inlineStr">
+        <is>
+          <t>Portfolio site referencing prior firm pedigree</t>
+        </is>
+      </c>
+      <c r="P169" s="3" t="inlineStr">
+        <is>
+          <t>Pedigree from previous firms not yet built into their own AI-search authority</t>
+        </is>
+      </c>
+      <c r="Q169" s="3" t="inlineStr">
+        <is>
+          <t>Turn founders' prior-firm credentials into the new practice's AEO content</t>
+        </is>
+      </c>
+      <c r="R169" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S169" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T169" s="3" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="4" t="inlineStr">
+        <is>
+          <t>Francis Associates</t>
+        </is>
+      </c>
+      <c r="B170" s="4" t="inlineStr">
+        <is>
+          <t>Architects / project management</t>
+        </is>
+      </c>
+      <c r="C170" s="4" t="inlineStr">
+        <is>
+          <t>Medmenham, Buckinghamshire</t>
+        </is>
+      </c>
+      <c r="D170" s="4" t="inlineStr">
+        <is>
+          <t>https://www.francis-associates.co.uk</t>
+        </is>
+      </c>
+      <c r="E170" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F170" s="4" t="inlineStr"/>
+      <c r="G170" s="4" t="inlineStr">
+        <is>
+          <t>Julian Francis FRICS (Founder, est. 1988)</t>
+        </is>
+      </c>
+      <c r="H170" s="4" t="inlineStr"/>
+      <c r="I170" s="4" t="inlineStr"/>
+      <c r="J170" s="4" t="inlineStr">
+        <is>
+          <t>Established 1988, RICS-qualified; project management + architecture for Thames Valley estates</t>
+        </is>
+      </c>
+      <c r="K170" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L170" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M170" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N170" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O170" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P170" s="4" t="inlineStr">
+        <is>
+          <t>37 years of trust not converted into digital-era search visibility</t>
+        </is>
+      </c>
+      <c r="Q170" s="4" t="inlineStr">
+        <is>
+          <t>Heritage-into-authority AEO play for high-value estate projects</t>
+        </is>
+      </c>
+      <c r="R170" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S170" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T170" s="4" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="3" t="inlineStr">
+        <is>
+          <t>Austyn Smith Associates</t>
+        </is>
+      </c>
+      <c r="B171" s="3" t="inlineStr">
+        <is>
+          <t>IFA / wealth management</t>
+        </is>
+      </c>
+      <c r="C171" s="3" t="inlineStr">
+        <is>
+          <t>Henley-on-Thames, Beaconsfield, High Wycombe, Marlow</t>
+        </is>
+      </c>
+      <c r="D171" s="3" t="inlineStr">
+        <is>
+          <t>https://austynsmith.com</t>
+        </is>
+      </c>
+      <c r="E171" s="3" t="inlineStr">
+        <is>
+          <t>info@austynsmith.com</t>
+        </is>
+      </c>
+      <c r="F171" s="3" t="inlineStr">
+        <is>
+          <t>01494 578 100</t>
+        </is>
+      </c>
+      <c r="G171" s="3" t="inlineStr">
+        <is>
+          <t>Austyn (Founder, 25+ years)</t>
+        </is>
+      </c>
+      <c r="H171" s="3" t="inlineStr"/>
+      <c r="I171" s="3" t="inlineStr"/>
+      <c r="J171" s="3" t="inlineStr">
+        <is>
+          <t>25-year independent IFA across 4 wealthy Bucks/Oxon towns; already builds per-town landing pages</t>
+        </is>
+      </c>
+      <c r="K171" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L171" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M171" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N171" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O171" s="3" t="inlineStr">
+        <is>
+          <t>Per-town SEO landing pages = active investment</t>
+        </is>
+      </c>
+      <c r="P171" s="3" t="inlineStr">
+        <is>
+          <t>Landing pages exist across 4 towns but none dominate AI answers yet</t>
+        </is>
+      </c>
+      <c r="Q171" s="3" t="inlineStr">
+        <is>
+          <t>AEO layer across all 4 existing town pages - multiply an existing strategy</t>
+        </is>
+      </c>
+      <c r="R171" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S171" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T171" s="3" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="3" t="inlineStr">
+        <is>
+          <t>The Guildford Private General Practice</t>
+        </is>
+      </c>
+      <c r="B172" s="3" t="inlineStr">
+        <is>
+          <t>Private GP</t>
+        </is>
+      </c>
+      <c r="C172" s="3" t="inlineStr">
+        <is>
+          <t>Central Guildford, Surrey</t>
+        </is>
+      </c>
+      <c r="D172" s="3" t="inlineStr">
+        <is>
+          <t>https://www.thegpgp.co.uk</t>
+        </is>
+      </c>
+      <c r="E172" s="3" t="inlineStr">
+        <is>
+          <t>enquiries@thegpgp.co.uk</t>
+        </is>
+      </c>
+      <c r="F172" s="3" t="inlineStr">
+        <is>
+          <t>01483 826367</t>
+        </is>
+      </c>
+      <c r="G172" s="3" t="inlineStr">
+        <is>
+          <t>Dr Selby, Dr Ballance, Dr Hendley (Partners)</t>
+        </is>
+      </c>
+      <c r="H172" s="3" t="inlineStr"/>
+      <c r="I172" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/thegpgp</t>
+        </is>
+      </c>
+      <c r="J172" s="3" t="inlineStr">
+        <is>
+          <t>Established 2013, three named GP partners with 15-20 years' experience each; self-pay consultations in wealthy Guildford</t>
+        </is>
+      </c>
+      <c r="K172" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L172" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M172" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N172" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O172" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence</t>
+        </is>
+      </c>
+      <c r="P172" s="3" t="inlineStr">
+        <is>
+          <t>Circle Health/Mount Alvernia hospital brand competes for the same Guildford private-GP searches</t>
+        </is>
+      </c>
+      <c r="Q172" s="3" t="inlineStr">
+        <is>
+          <t>'Guildford professionals ask AI for a private GP - beat the hospital brand to the answer'</t>
+        </is>
+      </c>
+      <c r="R172" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S172" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T172" s="3" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="3" t="inlineStr">
+        <is>
+          <t>Manor Farm Barn (Tythe)</t>
+        </is>
+      </c>
+      <c r="B173" s="3" t="inlineStr">
+        <is>
+          <t>Wedding venue</t>
+        </is>
+      </c>
+      <c r="C173" s="3" t="inlineStr">
+        <is>
+          <t>Bicester, Oxfordshire</t>
+        </is>
+      </c>
+      <c r="D173" s="3" t="inlineStr">
+        <is>
+          <t>https://www.manorfarmtythebarn.co.uk</t>
+        </is>
+      </c>
+      <c r="E173" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F173" s="3" t="inlineStr"/>
+      <c r="G173" s="3" t="inlineStr"/>
+      <c r="H173" s="3" t="inlineStr"/>
+      <c r="I173" s="3" t="inlineStr"/>
+      <c r="J173" s="3" t="inlineStr">
+        <is>
+          <t>16th-century barn venue near Bicester; Oxfordshire weddings worth £15-25k each</t>
+        </is>
+      </c>
+      <c r="K173" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L173" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M173" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N173" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O173" s="3" t="inlineStr">
+        <is>
+          <t>Dedicated wedding microsite</t>
+        </is>
+      </c>
+      <c r="P173" s="3" t="inlineStr">
+        <is>
+          <t>Directory-dependent discovery same as other venues in the database</t>
+        </is>
+      </c>
+      <c r="Q173" s="3" t="inlineStr">
+        <is>
+          <t>'Own the AI-recommended shortlist for Oxfordshire barn weddings'</t>
+        </is>
+      </c>
+      <c r="R173" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S173" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T173" s="3" t="inlineStr"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="4" t="inlineStr">
+        <is>
+          <t>Dovecote Events</t>
+        </is>
+      </c>
+      <c r="B174" s="4" t="inlineStr">
+        <is>
+          <t>Wedding venue</t>
+        </is>
+      </c>
+      <c r="C174" s="4" t="inlineStr">
+        <is>
+          <t>Rural Oxfordshire (Cotswolds edge)</t>
+        </is>
+      </c>
+      <c r="D174" s="4" t="inlineStr">
+        <is>
+          <t>https://www.dovecoteevents.uk</t>
+        </is>
+      </c>
+      <c r="E174" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F174" s="4" t="inlineStr"/>
+      <c r="G174" s="4" t="inlineStr"/>
+      <c r="H174" s="4" t="inlineStr"/>
+      <c r="I174" s="4" t="inlineStr"/>
+      <c r="J174" s="4" t="inlineStr">
+        <is>
+          <t>Grade II listed barn on the Cotswolds/Oxfordshire border; exclusive-use bookings</t>
+        </is>
+      </c>
+      <c r="K174" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L174" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M174" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N174" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O174" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P174" s="4" t="inlineStr">
+        <is>
+          <t>Listed-building charm undersold in generic wedding-venue search</t>
+        </is>
+      </c>
+      <c r="Q174" s="4" t="inlineStr">
+        <is>
+          <t>Grade II heritage story as AEO differentiator</t>
+        </is>
+      </c>
+      <c r="R174" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S174" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T174" s="4" t="inlineStr"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="3" t="inlineStr">
+        <is>
+          <t>Cornwell Manor</t>
+        </is>
+      </c>
+      <c r="B175" s="3" t="inlineStr">
+        <is>
+          <t>Wedding venue</t>
+        </is>
+      </c>
+      <c r="C175" s="3" t="inlineStr">
+        <is>
+          <t>Chipping Norton, Oxfordshire/Gloucestershire border</t>
+        </is>
+      </c>
+      <c r="D175" s="3" t="inlineStr">
+        <is>
+          <t>https://cornwellmanor.com</t>
+        </is>
+      </c>
+      <c r="E175" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F175" s="3" t="inlineStr"/>
+      <c r="G175" s="3" t="inlineStr"/>
+      <c r="H175" s="3" t="inlineStr"/>
+      <c r="I175" s="3" t="inlineStr"/>
+      <c r="J175" s="3" t="inlineStr">
+        <is>
+          <t>2,000-acre estate venue; ultra-premium Cotswolds weddings worth £30k+</t>
+        </is>
+      </c>
+      <c r="K175" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L175" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M175" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N175" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O175" s="3" t="inlineStr">
+        <is>
+          <t>Polished estate branding</t>
+        </is>
+      </c>
+      <c r="P175" s="3" t="inlineStr">
+        <is>
+          <t>Ultra-premium positioning needs to win the highest-value AI-search queries specifically</t>
+        </is>
+      </c>
+      <c r="Q175" s="3" t="inlineStr">
+        <is>
+          <t>Target 'luxury Cotswolds wedding venue' AEO exclusively - don't compete on volume terms</t>
+        </is>
+      </c>
+      <c r="R175" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S175" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T175" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T160"/>
+  <autoFilter ref="A1:T175"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -14368,7 +15652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B95"/>
+  <dimension ref="A1:B98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -14388,7 +15672,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>159</v>
+        <v>174</v>
       </c>
     </row>
     <row r="5">
@@ -14405,43 +15689,43 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Private dentist</t>
+          <t>Wedding venue</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Architects</t>
+          <t>Private dentist</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Independent vet</t>
+          <t>Architects</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Wedding venue</t>
+          <t>Independent vet</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -14491,7 +15775,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Aesthetics clinic</t>
+          <t>Private GP</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -14501,17 +15785,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Law firm</t>
+          <t>Aesthetics clinic</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Chartered accountants</t>
+          <t>Law firm</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -14521,7 +15805,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Private GP</t>
+          <t>Chartered accountants</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -14641,7 +15925,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Orthodontist</t>
+          <t>Estate agent (premium)</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -14651,7 +15935,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Employment law firm</t>
+          <t>Orthodontist</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -14661,7 +15945,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Event management agency</t>
+          <t>Employment law firm</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -14671,7 +15955,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Design &amp; build</t>
+          <t>Event management agency</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -14681,7 +15965,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Recruitment agency</t>
+          <t>Private dentist / implants</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -14691,7 +15975,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>IT support / MSP</t>
+          <t>Design &amp; build</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -14701,27 +15985,27 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Dentist / Orthodontics</t>
+          <t>Recruitment agency</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Specialist dental/implant clinic</t>
+          <t>IT support / MSP</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Boutique corporate law firm</t>
+          <t>Dentist / Orthodontics</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -14731,7 +16015,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Cosmetic/aesthetics clinic</t>
+          <t>Specialist dental/implant clinic</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -14741,7 +16025,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Skin &amp; laser clinic</t>
+          <t>Boutique corporate law firm</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -14751,7 +16035,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Mortgage broker / financial adviser</t>
+          <t>Cosmetic/aesthetics clinic</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -14761,7 +16045,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Architects (RIBA chartered)</t>
+          <t>Skin &amp; laser clinic</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -14771,7 +16055,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Recruitment agency (tech/startups)</t>
+          <t>Mortgage broker / financial adviser</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -14781,7 +16065,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Recruitment agency (IT/data)</t>
+          <t>Architects (RIBA chartered)</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -14791,7 +16075,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Independent vet (24/7 emergency)</t>
+          <t>Recruitment agency (tech/startups)</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -14801,7 +16085,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Interior design studio</t>
+          <t>Recruitment agency (IT/data)</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -14811,7 +16095,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Letting &amp; estate agent</t>
+          <t>Independent vet (24/7 emergency)</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -14821,7 +16105,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Cosmetic clinic (injectables)</t>
+          <t>Interior design studio</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -14831,7 +16115,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Cosmetic/anti-ageing clinic</t>
+          <t>Letting &amp; estate agent</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -14841,7 +16125,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Yoga &amp; reformer pilates studio</t>
+          <t>Cosmetic clinic (injectables)</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -14851,7 +16135,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Reformer pilates studio</t>
+          <t>Cosmetic/anti-ageing clinic</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -14861,7 +16145,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Wealth management</t>
+          <t>Yoga &amp; reformer pilates studio</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -14871,7 +16155,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Private tuition &amp; education consultancy</t>
+          <t>Reformer pilates studio</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -14881,7 +16165,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Osteopath</t>
+          <t>Wealth management</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -14891,7 +16175,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Design &amp; build / home renovation</t>
+          <t>Private tuition &amp; education consultancy</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -14901,7 +16185,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Builders / building contractor</t>
+          <t>Osteopath</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -14911,7 +16195,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Roofer</t>
+          <t>Design &amp; build / home renovation</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -14921,7 +16205,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Home care / live-in care</t>
+          <t>Builders / building contractor</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -14931,7 +16215,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Private day nurseries</t>
+          <t>Roofer</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -14941,7 +16225,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Personal training &amp; wellness studio</t>
+          <t>Home care / live-in care</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -14951,7 +16235,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Mortgage &amp; insurance broker</t>
+          <t>Private day nurseries</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -14961,7 +16245,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Business consultancy</t>
+          <t>Personal training &amp; wellness studio</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -14971,7 +16255,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Interior designer (period homes)</t>
+          <t>Mortgage &amp; insurance broker</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -14981,7 +16265,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Landscape design &amp; build</t>
+          <t>Business consultancy</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -14991,7 +16275,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Estate agent (premium)</t>
+          <t>Interior designer (period homes)</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -15001,7 +16285,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Interior designer</t>
+          <t>Landscape design &amp; build</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -15011,7 +16295,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Garden design &amp; landscaping</t>
+          <t>Interior designer</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -15021,7 +16305,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Legal recruitment</t>
+          <t>Garden design &amp; landscaping</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -15031,7 +16315,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Independent gym &amp; health club</t>
+          <t>Legal recruitment</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -15041,7 +16325,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Independent gym</t>
+          <t>Independent gym &amp; health club</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -15051,7 +16335,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Physiotherapy (sports)</t>
+          <t>Independent gym</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -15061,7 +16345,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Letting agent / property management</t>
+          <t>Physiotherapy (sports)</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -15071,7 +16355,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Skin clinic</t>
+          <t>Letting agent / property management</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -15081,7 +16365,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Tutoring company</t>
+          <t>Skin clinic</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -15091,7 +16375,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Tutorial college &amp; exam centre</t>
+          <t>Tutoring company</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -15101,7 +16385,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Employment law (disability discrimination)</t>
+          <t>Tutorial college &amp; exam centre</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -15111,7 +16395,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating</t>
+          <t>Employment law (disability discrimination)</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -15121,7 +16405,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Plumbing &amp; heating</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -15131,7 +16415,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Sports physio &amp; massage</t>
+          <t>Plumbing</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -15141,7 +16425,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Chartered surveyors (party wall/building)</t>
+          <t>Sports physio &amp; massage</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -15151,7 +16435,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Chartered surveyors</t>
+          <t>Chartered surveyors (party wall/building)</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -15161,7 +16445,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Chartered building surveyors</t>
+          <t>Chartered surveyors</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -15171,7 +16455,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Osteopathy clinics</t>
+          <t>Chartered building surveyors</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -15181,7 +16465,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Private dentist / implants</t>
+          <t>Osteopathy clinics</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -15295,6 +16579,36 @@
         </is>
       </c>
       <c r="B95" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Architect &amp; interior designer</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Architects / project management</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>IFA / wealth management</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 7: +12 prospects (186 total) - Tunbridge Wells, Sevenoaks, St Albans
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$175</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$187</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T175"/>
+  <dimension ref="A1:T187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -15640,8 +15640,1036 @@
       </c>
       <c r="T175" s="3" t="inlineStr"/>
     </row>
+    <row r="176">
+      <c r="A176" s="3" t="inlineStr">
+        <is>
+          <t>Kings Estates</t>
+        </is>
+      </c>
+      <c r="B176" s="3" t="inlineStr">
+        <is>
+          <t>Estate &amp; letting agent</t>
+        </is>
+      </c>
+      <c r="C176" s="3" t="inlineStr">
+        <is>
+          <t>Tunbridge Wells, Kent</t>
+        </is>
+      </c>
+      <c r="D176" s="3" t="inlineStr">
+        <is>
+          <t>https://www.kings-estates.co.uk</t>
+        </is>
+      </c>
+      <c r="E176" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F176" s="3" t="inlineStr">
+        <is>
+          <t>01892 533367</t>
+        </is>
+      </c>
+      <c r="G176" s="3" t="inlineStr">
+        <is>
+          <t>Mike Heath (lettings) &amp; Gemma Collins (sales) - siblings, since 1985</t>
+        </is>
+      </c>
+      <c r="H176" s="3" t="inlineStr"/>
+      <c r="I176" s="3" t="inlineStr"/>
+      <c r="J176" s="3" t="inlineStr">
+        <is>
+          <t>Owner-led independent since 1985; sibling founders handle every client personally; premium marketing for Tunbridge Wells/Kent/Sussex homes</t>
+        </is>
+      </c>
+      <c r="K176" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L176" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M176" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N176" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O176" s="3" t="inlineStr">
+        <is>
+          <t>Area-guide content pages (Tunbridge Wells guide) = active SEO effort</t>
+        </is>
+      </c>
+      <c r="P176" s="3" t="inlineStr">
+        <is>
+          <t>Content exists but competes with Savills/Hamptons/Fine &amp; Country's bigger budgets</t>
+        </is>
+      </c>
+      <c r="Q176" s="3" t="inlineStr">
+        <is>
+          <t>'You built the area guides - let's make AI cite them, not just Google index them'</t>
+        </is>
+      </c>
+      <c r="R176" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S176" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T176" s="3" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="3" t="inlineStr">
+        <is>
+          <t>Druce &amp; Partners</t>
+        </is>
+      </c>
+      <c r="B177" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C177" s="3" t="inlineStr">
+        <is>
+          <t>St Albans, Hertfordshire</t>
+        </is>
+      </c>
+      <c r="D177" s="3" t="inlineStr">
+        <is>
+          <t>https://druce-partners.co.uk</t>
+        </is>
+      </c>
+      <c r="E177" s="3" t="inlineStr">
+        <is>
+          <t>sales@druce-partners.co.uk</t>
+        </is>
+      </c>
+      <c r="F177" s="3" t="inlineStr">
+        <is>
+          <t>01727 855 232</t>
+        </is>
+      </c>
+      <c r="G177" s="3" t="inlineStr">
+        <is>
+          <t>Darryl Druce (Founder, est. 1988)</t>
+        </is>
+      </c>
+      <c r="H177" s="3" t="inlineStr"/>
+      <c r="I177" s="3" t="inlineStr"/>
+      <c r="J177" s="3" t="inlineStr">
+        <is>
+          <t>Independent family firm since 1988; 50+ years combined local experience; premium St Albans period-home fees</t>
+        </is>
+      </c>
+      <c r="K177" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L177" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M177" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N177" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O177" s="3" t="inlineStr">
+        <is>
+          <t>Long-established brand</t>
+        </is>
+      </c>
+      <c r="P177" s="3" t="inlineStr">
+        <is>
+          <t>Cassidy &amp; Tate and Heartwood Homes both fight for the same St Albans premium searches</t>
+        </is>
+      </c>
+      <c r="Q177" s="3" t="inlineStr">
+        <is>
+          <t>'St Albans buyers now ask AI before Rightmove - be the answer they get'</t>
+        </is>
+      </c>
+      <c r="R177" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S177" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T177" s="3" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="3" t="inlineStr">
+        <is>
+          <t>Woodbury Park Dental Surgery</t>
+        </is>
+      </c>
+      <c r="B178" s="3" t="inlineStr">
+        <is>
+          <t>Private dentist</t>
+        </is>
+      </c>
+      <c r="C178" s="3" t="inlineStr">
+        <is>
+          <t>Tunbridge Wells, Kent</t>
+        </is>
+      </c>
+      <c r="D178" s="3" t="inlineStr">
+        <is>
+          <t>https://woodburyparkdentalsurgery.com</t>
+        </is>
+      </c>
+      <c r="E178" s="3" t="inlineStr">
+        <is>
+          <t>info@woodburyparkdentalsurgery.com</t>
+        </is>
+      </c>
+      <c r="F178" s="3" t="inlineStr">
+        <is>
+          <t>01892 522297</t>
+        </is>
+      </c>
+      <c r="G178" s="3" t="inlineStr">
+        <is>
+          <t>Dr Alanna Gardiner (Principal)</t>
+        </is>
+      </c>
+      <c r="H178" s="3" t="inlineStr"/>
+      <c r="I178" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/WoodburyParkDentalSurgery</t>
+        </is>
+      </c>
+      <c r="J178" s="3" t="inlineStr">
+        <is>
+          <t>Independent, non-corporate, family-run practice - explicit differentiation from chains; named principal dentist</t>
+        </is>
+      </c>
+      <c r="K178" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L178" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M178" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N178" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O178" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence</t>
+        </is>
+      </c>
+      <c r="P178" s="3" t="inlineStr">
+        <is>
+          <t>'Non-corporate' story not yet leveraged as an AI-search differentiator vs Bupa/mydentist</t>
+        </is>
+      </c>
+      <c r="Q178" s="3" t="inlineStr">
+        <is>
+          <t>'Own the AI answer for "independent dentist Tunbridge Wells" - it's your exact positioning'</t>
+        </is>
+      </c>
+      <c r="R178" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S178" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T178" s="3" t="inlineStr"/>
+    </row>
+    <row r="179">
+      <c r="A179" s="3" t="inlineStr">
+        <is>
+          <t>The Dental Box</t>
+        </is>
+      </c>
+      <c r="B179" s="3" t="inlineStr">
+        <is>
+          <t>Private dentist</t>
+        </is>
+      </c>
+      <c r="C179" s="3" t="inlineStr">
+        <is>
+          <t>Southborough, Tunbridge Wells</t>
+        </is>
+      </c>
+      <c r="D179" s="3" t="inlineStr">
+        <is>
+          <t>https://www.thedentalbox.co.uk</t>
+        </is>
+      </c>
+      <c r="E179" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F179" s="3" t="inlineStr"/>
+      <c r="G179" s="3" t="inlineStr"/>
+      <c r="H179" s="3" t="inlineStr"/>
+      <c r="I179" s="3" t="inlineStr"/>
+      <c r="J179" s="3" t="inlineStr">
+        <is>
+          <t>Private-only practice in a newly regenerated civic centre; no NHS dilution means fully self-pay client base</t>
+        </is>
+      </c>
+      <c r="K179" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L179" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M179" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N179" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O179" s="3" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P179" s="3" t="inlineStr">
+        <is>
+          <t>Private-only positioning is a strong differentiator currently invisible in local search</t>
+        </is>
+      </c>
+      <c r="Q179" s="3" t="inlineStr">
+        <is>
+          <t>'Private-only' AEO content: own the self-pay dental searches in Southborough/TW</t>
+        </is>
+      </c>
+      <c r="R179" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S179" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T179" s="3" t="inlineStr"/>
+    </row>
+    <row r="180">
+      <c r="A180" s="4" t="inlineStr">
+        <is>
+          <t>Lewis &amp; Co Accountants &amp; Tax Advisors</t>
+        </is>
+      </c>
+      <c r="B180" s="4" t="inlineStr">
+        <is>
+          <t>Chartered accountants</t>
+        </is>
+      </c>
+      <c r="C180" s="4" t="inlineStr">
+        <is>
+          <t>Southborough, Tunbridge Wells, Kent</t>
+        </is>
+      </c>
+      <c r="D180" s="4" t="inlineStr">
+        <is>
+          <t>https://www.lewisandco.biz</t>
+        </is>
+      </c>
+      <c r="E180" s="4" t="inlineStr">
+        <is>
+          <t>info@lewisandco.biz</t>
+        </is>
+      </c>
+      <c r="F180" s="4" t="inlineStr">
+        <is>
+          <t>01892 513 515</t>
+        </is>
+      </c>
+      <c r="G180" s="4" t="inlineStr">
+        <is>
+          <t>Barney Lewis (Principal &amp; MD, FCA)</t>
+        </is>
+      </c>
+      <c r="H180" s="4" t="inlineStr"/>
+      <c r="I180" s="4" t="inlineStr">
+        <is>
+          <t>facebook.com/LewisandCoAccountantsandTaxAdvisors</t>
+        </is>
+      </c>
+      <c r="J180" s="4" t="inlineStr">
+        <is>
+          <t>Independent since 1986, serving Kent/Sussex SMEs; recurring-fee clients across decades of trading</t>
+        </is>
+      </c>
+      <c r="K180" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L180" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M180" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N180" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O180" s="4" t="inlineStr">
+        <is>
+          <t>Facebook presence</t>
+        </is>
+      </c>
+      <c r="P180" s="4" t="inlineStr">
+        <is>
+          <t>Perrys and S&amp;W (150-year-old firm) dominate Tunbridge Wells accountant searches with scale</t>
+        </is>
+      </c>
+      <c r="Q180" s="4" t="inlineStr">
+        <is>
+          <t>'The small firm that's big on personal service' - own that exact AEO positioning</t>
+        </is>
+      </c>
+      <c r="R180" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S180" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T180" s="4" t="inlineStr"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="4" t="inlineStr">
+        <is>
+          <t>Gilberts Chartered Accountants</t>
+        </is>
+      </c>
+      <c r="B181" s="4" t="inlineStr">
+        <is>
+          <t>Chartered accountants</t>
+        </is>
+      </c>
+      <c r="C181" s="4" t="inlineStr">
+        <is>
+          <t>St Albans, Hertfordshire</t>
+        </is>
+      </c>
+      <c r="D181" s="4" t="inlineStr">
+        <is>
+          <t>https://gilberts.uk.com</t>
+        </is>
+      </c>
+      <c r="E181" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F181" s="4" t="inlineStr"/>
+      <c r="G181" s="4" t="inlineStr"/>
+      <c r="H181" s="4" t="inlineStr"/>
+      <c r="I181" s="4" t="inlineStr"/>
+      <c r="J181" s="4" t="inlineStr">
+        <is>
+          <t>Medium-sized independent firm with roots to 1921; serves St Albans SMEs and private clients</t>
+        </is>
+      </c>
+      <c r="K181" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L181" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M181" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N181" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O181" s="4" t="inlineStr">
+        <is>
+          <t>Century-old heritage promoted</t>
+        </is>
+      </c>
+      <c r="P181" s="4" t="inlineStr">
+        <is>
+          <t>Heritage brand not translated into modern local/AI search dominance</t>
+        </is>
+      </c>
+      <c r="Q181" s="4" t="inlineStr">
+        <is>
+          <t>'103 years in St Albans - let's make AI say so when clients ask for an accountant'</t>
+        </is>
+      </c>
+      <c r="R181" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S181" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T181" s="4" t="inlineStr"/>
+    </row>
+    <row r="182">
+      <c r="A182" s="3" t="inlineStr">
+        <is>
+          <t>Culverden Vets</t>
+        </is>
+      </c>
+      <c r="B182" s="3" t="inlineStr">
+        <is>
+          <t>Independent vet</t>
+        </is>
+      </c>
+      <c r="C182" s="3" t="inlineStr">
+        <is>
+          <t>Tunbridge Wells, Wadhurst &amp; Crowborough, Kent</t>
+        </is>
+      </c>
+      <c r="D182" s="3" t="inlineStr">
+        <is>
+          <t>https://culverden.co.uk</t>
+        </is>
+      </c>
+      <c r="E182" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F182" s="3" t="inlineStr"/>
+      <c r="G182" s="3" t="inlineStr"/>
+      <c r="H182" s="3" t="inlineStr"/>
+      <c r="I182" s="3" t="inlineStr"/>
+      <c r="J182" s="3" t="inlineStr">
+        <is>
+          <t>One of Kent &amp; Sussex's longest-running independent vets, 3 sites; loyal multi-generation client base</t>
+        </is>
+      </c>
+      <c r="K182" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L182" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M182" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N182" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O182" s="3" t="inlineStr">
+        <is>
+          <t>Multi-site established brand</t>
+        </is>
+      </c>
+      <c r="P182" s="3" t="inlineStr">
+        <is>
+          <t>Corporate groups (IVC, CVS) and Vets Now dominate local + emergency vet search</t>
+        </is>
+      </c>
+      <c r="Q182" s="3" t="inlineStr">
+        <is>
+          <t>'3 sites, decades of trust - none of it shows up when pet owners ask AI'</t>
+        </is>
+      </c>
+      <c r="R182" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S182" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T182" s="3" t="inlineStr"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="3" t="inlineStr">
+        <is>
+          <t>Carewell Vets</t>
+        </is>
+      </c>
+      <c r="B183" s="3" t="inlineStr">
+        <is>
+          <t>Independent vet</t>
+        </is>
+      </c>
+      <c r="C183" s="3" t="inlineStr">
+        <is>
+          <t>Kent &amp; Surrey (Edenbridge area)</t>
+        </is>
+      </c>
+      <c r="D183" s="3" t="inlineStr">
+        <is>
+          <t>https://carewellvets.co.uk</t>
+        </is>
+      </c>
+      <c r="E183" s="3" t="inlineStr">
+        <is>
+          <t>reception@carewellvets.co.uk</t>
+        </is>
+      </c>
+      <c r="F183" s="3" t="inlineStr">
+        <is>
+          <t>01342 612103</t>
+        </is>
+      </c>
+      <c r="G183" s="3" t="inlineStr"/>
+      <c r="H183" s="3" t="inlineStr"/>
+      <c r="I183" s="3" t="inlineStr"/>
+      <c r="J183" s="3" t="inlineStr">
+        <is>
+          <t>Explicitly '100% independent', family-run across the Kent/Surrey border; strong differentiation story</t>
+        </is>
+      </c>
+      <c r="K183" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L183" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M183" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N183" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O183" s="3" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P183" s="3" t="inlineStr">
+        <is>
+          <t>'100% independent' claim isn't yet an AI-search asset</t>
+        </is>
+      </c>
+      <c r="Q183" s="3" t="inlineStr">
+        <is>
+          <t>Own the AI answer for '100% independent vet Kent/Surrey' - it's their own tagline</t>
+        </is>
+      </c>
+      <c r="R183" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S183" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T183" s="3" t="inlineStr"/>
+    </row>
+    <row r="184">
+      <c r="A184" s="3" t="inlineStr">
+        <is>
+          <t>Sevenoaks Physiotherapy</t>
+        </is>
+      </c>
+      <c r="B184" s="3" t="inlineStr">
+        <is>
+          <t>Physiotherapy clinic</t>
+        </is>
+      </c>
+      <c r="C184" s="3" t="inlineStr">
+        <is>
+          <t>Manor Clinic, Sevenoaks, Kent</t>
+        </is>
+      </c>
+      <c r="D184" s="3" t="inlineStr">
+        <is>
+          <t>https://sevenoaksphysiotherapy.co.uk</t>
+        </is>
+      </c>
+      <c r="E184" s="3" t="inlineStr">
+        <is>
+          <t>info@7oaksphysio.co.uk</t>
+        </is>
+      </c>
+      <c r="F184" s="3" t="inlineStr">
+        <is>
+          <t>01732 464 400</t>
+        </is>
+      </c>
+      <c r="G184" s="3" t="inlineStr"/>
+      <c r="H184" s="3" t="inlineStr"/>
+      <c r="I184" s="3" t="inlineStr"/>
+      <c r="J184" s="3" t="inlineStr">
+        <is>
+          <t>30 practitioners under one roof in affluent Sevenoaks; self-pay physio + multiple specialisms = high patient LTV</t>
+        </is>
+      </c>
+      <c r="K184" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L184" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M184" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N184" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O184" s="3" t="inlineStr">
+        <is>
+          <t>Multi-practitioner scale</t>
+        </is>
+      </c>
+      <c r="P184" s="3" t="inlineStr">
+        <is>
+          <t>Scale not reflected in 'physio Sevenoaks' search visibility vs newer boutique rivals</t>
+        </is>
+      </c>
+      <c r="Q184" s="3" t="inlineStr">
+        <is>
+          <t>'30 practitioners deserve to dominate the search, not just the waiting room'</t>
+        </is>
+      </c>
+      <c r="R184" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S184" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T184" s="3" t="inlineStr"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="3" t="inlineStr">
+        <is>
+          <t>Orchard Clinic</t>
+        </is>
+      </c>
+      <c r="B185" s="3" t="inlineStr">
+        <is>
+          <t>Physiotherapy &amp; clinical Pilates</t>
+        </is>
+      </c>
+      <c r="C185" s="3" t="inlineStr">
+        <is>
+          <t>St Albans, Hertfordshire</t>
+        </is>
+      </c>
+      <c r="D185" s="3" t="inlineStr">
+        <is>
+          <t>https://www.orchardphysio.co.uk</t>
+        </is>
+      </c>
+      <c r="E185" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F185" s="3" t="inlineStr">
+        <is>
+          <t>01727 855 414</t>
+        </is>
+      </c>
+      <c r="G185" s="3" t="inlineStr">
+        <is>
+          <t>Paul Carnell (Clinic Director &amp; Head Physiotherapist)</t>
+        </is>
+      </c>
+      <c r="H185" s="3" t="inlineStr"/>
+      <c r="I185" s="3" t="inlineStr"/>
+      <c r="J185" s="3" t="inlineStr">
+        <is>
+          <t>Established 1987, named director; St Albans' longest-running physio brand</t>
+        </is>
+      </c>
+      <c r="K185" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L185" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M185" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N185" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O185" s="3" t="inlineStr">
+        <is>
+          <t>40 years trading</t>
+        </is>
+      </c>
+      <c r="P185" s="3" t="inlineStr">
+        <is>
+          <t>Heritage brand losing 'physio St Albans' searches to newer entrants (Redrock, Ann Physiocare)</t>
+        </is>
+      </c>
+      <c r="Q185" s="3" t="inlineStr">
+        <is>
+          <t>'Founded 1987 - make that longevity the AI's answer, not just a footnote'</t>
+        </is>
+      </c>
+      <c r="R185" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S185" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T185" s="3" t="inlineStr"/>
+    </row>
+    <row r="186">
+      <c r="A186" s="4" t="inlineStr">
+        <is>
+          <t>Simon Knight Architects</t>
+        </is>
+      </c>
+      <c r="B186" s="4" t="inlineStr">
+        <is>
+          <t>Architects</t>
+        </is>
+      </c>
+      <c r="C186" s="4" t="inlineStr">
+        <is>
+          <t>St Albans, Hertfordshire</t>
+        </is>
+      </c>
+      <c r="D186" s="4" t="inlineStr">
+        <is>
+          <t>https://simonknightarchitects.com</t>
+        </is>
+      </c>
+      <c r="E186" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F186" s="4" t="inlineStr"/>
+      <c r="G186" s="4" t="inlineStr">
+        <is>
+          <t>Simon Knight (Founder, 15+ years)</t>
+        </is>
+      </c>
+      <c r="H186" s="4" t="inlineStr"/>
+      <c r="I186" s="4" t="inlineStr"/>
+      <c r="J186" s="4" t="inlineStr">
+        <is>
+          <t>RIBA chartered practice in historic St Albans; residential + larger projects across Herts</t>
+        </is>
+      </c>
+      <c r="K186" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L186" s="4" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M186" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N186" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O186" s="4" t="inlineStr">
+        <is>
+          <t>Professional portfolio site</t>
+        </is>
+      </c>
+      <c r="P186" s="4" t="inlineStr">
+        <is>
+          <t>Competing with London-based AURA and Scenario for the same Herts clients</t>
+        </is>
+      </c>
+      <c r="Q186" s="4" t="inlineStr">
+        <is>
+          <t>'St Albans' own architect vs London firms parachuting in - own that local-first AEO angle'</t>
+        </is>
+      </c>
+      <c r="R186" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S186" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T186" s="4" t="inlineStr"/>
+    </row>
+    <row r="187">
+      <c r="A187" s="4" t="inlineStr">
+        <is>
+          <t>Seth White Architects</t>
+        </is>
+      </c>
+      <c r="B187" s="4" t="inlineStr">
+        <is>
+          <t>Architects</t>
+        </is>
+      </c>
+      <c r="C187" s="4" t="inlineStr">
+        <is>
+          <t>St Albans, Hertfordshire</t>
+        </is>
+      </c>
+      <c r="D187" s="4" t="inlineStr">
+        <is>
+          <t>via RIBA directory listing</t>
+        </is>
+      </c>
+      <c r="E187" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F187" s="4" t="inlineStr"/>
+      <c r="G187" s="4" t="inlineStr">
+        <is>
+          <t>Seth White (Founder)</t>
+        </is>
+      </c>
+      <c r="H187" s="4" t="inlineStr"/>
+      <c r="I187" s="4" t="inlineStr"/>
+      <c r="J187" s="4" t="inlineStr">
+        <is>
+          <t>Design-led RIBA practice for St Albans new builds/extensions/refurbs; residential project values £100k+</t>
+        </is>
+      </c>
+      <c r="K187" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L187" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M187" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N187" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O187" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P187" s="4" t="inlineStr">
+        <is>
+          <t>Small practice needs differentiated content to compete for Herts residential work</t>
+        </is>
+      </c>
+      <c r="Q187" s="4" t="inlineStr">
+        <is>
+          <t>Local-first AEO content targeting St Albans conservation-area planning queries</t>
+        </is>
+      </c>
+      <c r="R187" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S187" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T187" s="4" t="inlineStr">
+        <is>
+          <t>Confirm live website URL before outreach</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T175"/>
+  <autoFilter ref="A1:T187"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -15652,7 +16680,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B98"/>
+  <dimension ref="A1:B99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -15672,7 +16700,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>174</v>
+        <v>186</v>
       </c>
     </row>
     <row r="5">
@@ -15689,37 +16717,37 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Wedding venue</t>
+          <t>Private dentist</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Private dentist</t>
+          <t>Architects</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Architects</t>
+          <t>Wedding venue</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10">
@@ -15729,7 +16757,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11">
@@ -15739,33 +16767,33 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Mortgage broker</t>
+          <t>Physiotherapy clinic</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Physiotherapy clinic</t>
+          <t>Chartered accountants</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Solar installer</t>
+          <t>Mortgage broker</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -15775,7 +16803,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Private GP</t>
+          <t>Solar installer</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -15785,7 +16813,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Aesthetics clinic</t>
+          <t>Private GP</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -15795,17 +16823,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Law firm</t>
+          <t>Aesthetics clinic</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Chartered accountants</t>
+          <t>Law firm</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -16609,6 +17637,16 @@
         </is>
       </c>
       <c r="B98" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Physiotherapy &amp; clinical Pilates</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 8: +11 prospects (197 total) - Cobham, Virginia Water, Beaconsfield, Weybridge
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$187</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$198</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T187"/>
+  <dimension ref="A1:T198"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -16668,8 +16668,960 @@
         </is>
       </c>
     </row>
+    <row r="188">
+      <c r="A188" s="3" t="inlineStr">
+        <is>
+          <t>Davies Property Partners</t>
+        </is>
+      </c>
+      <c r="B188" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C188" s="3" t="inlineStr">
+        <is>
+          <t>Cobham, Surrey</t>
+        </is>
+      </c>
+      <c r="D188" s="3" t="inlineStr">
+        <is>
+          <t>https://daviespropertypartners.co.uk</t>
+        </is>
+      </c>
+      <c r="E188" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F188" s="3" t="inlineStr">
+        <is>
+          <t>01932 588 288</t>
+        </is>
+      </c>
+      <c r="G188" s="3" t="inlineStr">
+        <is>
+          <t>Gareth &amp; Claire Davies (2nd generation, since 2021); founded by Ian Davies 2002</t>
+        </is>
+      </c>
+      <c r="H188" s="3" t="inlineStr"/>
+      <c r="I188" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/daviespropertypartners</t>
+        </is>
+      </c>
+      <c r="J188" s="3" t="inlineStr">
+        <is>
+          <t>Family-owned since 2002, recent generational handover to siblings; premium Cobham/Surrey stock, high fees per instruction</t>
+        </is>
+      </c>
+      <c r="K188" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L188" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M188" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N188" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O188" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence; 20+ years trading</t>
+        </is>
+      </c>
+      <c r="P188" s="3" t="inlineStr">
+        <is>
+          <t>New generation running the business - a natural moment to modernise marketing</t>
+        </is>
+      </c>
+      <c r="Q188" s="3" t="inlineStr">
+        <is>
+          <t>'New leadership, same trust - let's make sure your digital presence matches your reputation'</t>
+        </is>
+      </c>
+      <c r="R188" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S188" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T188" s="3" t="inlineStr"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="3" t="inlineStr">
+        <is>
+          <t>Buckinghams</t>
+        </is>
+      </c>
+      <c r="B189" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C189" s="3" t="inlineStr">
+        <is>
+          <t>Virginia Water, Surrey</t>
+        </is>
+      </c>
+      <c r="D189" s="3" t="inlineStr">
+        <is>
+          <t>https://www.buckinghams.com</t>
+        </is>
+      </c>
+      <c r="E189" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F189" s="3" t="inlineStr">
+        <is>
+          <t>01344 933898</t>
+        </is>
+      </c>
+      <c r="G189" s="3" t="inlineStr">
+        <is>
+          <t>Wyatt family (Owners, since 1991)</t>
+        </is>
+      </c>
+      <c r="H189" s="3" t="inlineStr"/>
+      <c r="I189" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/BuckinghamsEstateAgents</t>
+        </is>
+      </c>
+      <c r="J189" s="3" t="inlineStr">
+        <is>
+          <t>Independent since 1991 in one of the UK's wealthiest villages (Virginia Water); very high average property values</t>
+        </is>
+      </c>
+      <c r="K189" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L189" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M189" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N189" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O189" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence; 30+ years trading</t>
+        </is>
+      </c>
+      <c r="P189" s="3" t="inlineStr">
+        <is>
+          <t>Savills/Knight Frank corporate offices also based in Virginia Water compete for the same ultra-high-value stock</t>
+        </is>
+      </c>
+      <c r="Q189" s="3" t="inlineStr">
+        <is>
+          <t>'Virginia Water sellers ask AI before Rightmove now - be the independent name it gives'</t>
+        </is>
+      </c>
+      <c r="R189" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S189" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T189" s="3" t="inlineStr"/>
+    </row>
+    <row r="190">
+      <c r="A190" s="3" t="inlineStr">
+        <is>
+          <t>Peter Scott Estate Agents</t>
+        </is>
+      </c>
+      <c r="B190" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C190" s="3" t="inlineStr">
+        <is>
+          <t>Chalfont St Giles (serves Beaconsfield/Gerrards Cross)</t>
+        </is>
+      </c>
+      <c r="D190" s="3" t="inlineStr">
+        <is>
+          <t>https://www.peterscottproperty.co.uk</t>
+        </is>
+      </c>
+      <c r="E190" s="3" t="inlineStr">
+        <is>
+          <t>peter@peterscottproperty.co.uk</t>
+        </is>
+      </c>
+      <c r="F190" s="3" t="inlineStr">
+        <is>
+          <t>01494 870 633</t>
+        </is>
+      </c>
+      <c r="G190" s="3" t="inlineStr">
+        <is>
+          <t>Peter Scott (Founder, est. 1982)</t>
+        </is>
+      </c>
+      <c r="H190" s="3" t="inlineStr"/>
+      <c r="I190" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/peterscottproperty</t>
+        </is>
+      </c>
+      <c r="J190" s="3" t="inlineStr">
+        <is>
+          <t>Independent since 1982 across South Bucks' wealthiest villages; long-term repeat clients (sold same client 10 homes)</t>
+        </is>
+      </c>
+      <c r="K190" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L190" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M190" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N190" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O190" s="3" t="inlineStr">
+        <is>
+          <t>YouTube channel; Facebook presence</t>
+        </is>
+      </c>
+      <c r="P190" s="3" t="inlineStr">
+        <is>
+          <t>40+ years of repeat-client trust not converted into modern digital dominance</t>
+        </is>
+      </c>
+      <c r="Q190" s="3" t="inlineStr">
+        <is>
+          <t>'You've sold one client 10 houses - let's make sure the next one finds you on Google first'</t>
+        </is>
+      </c>
+      <c r="R190" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S190" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T190" s="3" t="inlineStr"/>
+    </row>
+    <row r="191">
+      <c r="A191" s="3" t="inlineStr">
+        <is>
+          <t>Weybridge Dental Care</t>
+        </is>
+      </c>
+      <c r="B191" s="3" t="inlineStr">
+        <is>
+          <t>Private dentist</t>
+        </is>
+      </c>
+      <c r="C191" s="3" t="inlineStr">
+        <is>
+          <t>Weybridge High St, Surrey</t>
+        </is>
+      </c>
+      <c r="D191" s="3" t="inlineStr">
+        <is>
+          <t>https://weybridge-dental-care.co.uk</t>
+        </is>
+      </c>
+      <c r="E191" s="3" t="inlineStr">
+        <is>
+          <t>weybridgedentalcare@gmail.com</t>
+        </is>
+      </c>
+      <c r="F191" s="3" t="inlineStr">
+        <is>
+          <t>01932 842 838</t>
+        </is>
+      </c>
+      <c r="G191" s="3" t="inlineStr">
+        <is>
+          <t>Rashi Soin (Principal Dentist &amp; Owner)</t>
+        </is>
+      </c>
+      <c r="H191" s="3" t="inlineStr"/>
+      <c r="I191" s="3" t="inlineStr"/>
+      <c r="J191" s="3" t="inlineStr">
+        <is>
+          <t>20+ year established practice in affluent Weybridge; named owner-principal; general + cosmetic private work</t>
+        </is>
+      </c>
+      <c r="K191" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L191" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M191" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N191" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O191" s="3" t="inlineStr">
+        <is>
+          <t>Gmail contact address - low marketing infrastructure</t>
+        </is>
+      </c>
+      <c r="P191" s="3" t="inlineStr">
+        <is>
+          <t>Bupa Dental Care Weybridge and MyoDental compete for the same high-value searches</t>
+        </is>
+      </c>
+      <c r="Q191" s="3" t="inlineStr">
+        <is>
+          <t>'20 years of trust in Weybridge deserves better than a Gmail inbox - let's fix the whole funnel'</t>
+        </is>
+      </c>
+      <c r="R191" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S191" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T191" s="3" t="inlineStr">
+        <is>
+          <t>Gmail tell - same infrastructure-gap wedge as other rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="3" t="inlineStr">
+        <is>
+          <t>The Specialist Dental Practice</t>
+        </is>
+      </c>
+      <c r="B192" s="3" t="inlineStr">
+        <is>
+          <t>Private dentist</t>
+        </is>
+      </c>
+      <c r="C192" s="3" t="inlineStr">
+        <is>
+          <t>Weybridge, Surrey</t>
+        </is>
+      </c>
+      <c r="D192" s="3" t="inlineStr">
+        <is>
+          <t>https://thespecialistdentalpractice.com</t>
+        </is>
+      </c>
+      <c r="E192" s="3" t="inlineStr">
+        <is>
+          <t>info@weybridgedentist.co.uk</t>
+        </is>
+      </c>
+      <c r="F192" s="3" t="inlineStr">
+        <is>
+          <t>01932 857 585</t>
+        </is>
+      </c>
+      <c r="G192" s="3" t="inlineStr"/>
+      <c r="H192" s="3" t="inlineStr"/>
+      <c r="I192" s="3" t="inlineStr"/>
+      <c r="J192" s="3" t="inlineStr">
+        <is>
+          <t>Specialist-branded practice in wealthy Weybridge; positioning suggests referral/specialist work at premium fees</t>
+        </is>
+      </c>
+      <c r="K192" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L192" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M192" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N192" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O192" s="3" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P192" s="3" t="inlineStr">
+        <is>
+          <t>'Specialist' branding underexploited in local search - genuinely differentiated in NLP terms</t>
+        </is>
+      </c>
+      <c r="Q192" s="3" t="inlineStr">
+        <is>
+          <t>Own 'specialist dentist Weybridge' - the branding practically writes the AEO content</t>
+        </is>
+      </c>
+      <c r="R192" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S192" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T192" s="3" t="inlineStr"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="4" t="inlineStr">
+        <is>
+          <t>MyoDental</t>
+        </is>
+      </c>
+      <c r="B193" s="4" t="inlineStr">
+        <is>
+          <t>Private dentist</t>
+        </is>
+      </c>
+      <c r="C193" s="4" t="inlineStr">
+        <is>
+          <t>Weybridge, Surrey</t>
+        </is>
+      </c>
+      <c r="D193" s="4" t="inlineStr">
+        <is>
+          <t>https://myodental.co.uk/surrey</t>
+        </is>
+      </c>
+      <c r="E193" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F193" s="4" t="inlineStr"/>
+      <c r="G193" s="4" t="inlineStr"/>
+      <c r="H193" s="4" t="inlineStr"/>
+      <c r="I193" s="4" t="inlineStr"/>
+      <c r="J193" s="4" t="inlineStr">
+        <is>
+          <t>Serving Surrey since 2008; accepting new private patients; competitive £80 check-up pricing suggests volume model</t>
+        </is>
+      </c>
+      <c r="K193" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L193" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M193" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N193" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O193" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P193" s="4" t="inlineStr">
+        <is>
+          <t>Volume private model needs constant new-patient search visibility to sustain growth</t>
+        </is>
+      </c>
+      <c r="Q193" s="4" t="inlineStr">
+        <is>
+          <t>Local-intent SEO to keep the new-patient pipeline full</t>
+        </is>
+      </c>
+      <c r="R193" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S193" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T193" s="4" t="inlineStr"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="3" t="inlineStr">
+        <is>
+          <t>Weybridge Vets</t>
+        </is>
+      </c>
+      <c r="B194" s="3" t="inlineStr">
+        <is>
+          <t>Independent vet</t>
+        </is>
+      </c>
+      <c r="C194" s="3" t="inlineStr">
+        <is>
+          <t>York Road, Weybridge, Surrey</t>
+        </is>
+      </c>
+      <c r="D194" s="3" t="inlineStr">
+        <is>
+          <t>https://www.weybridgevets.co.uk</t>
+        </is>
+      </c>
+      <c r="E194" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F194" s="3" t="inlineStr">
+        <is>
+          <t>01932 855 856</t>
+        </is>
+      </c>
+      <c r="G194" s="3" t="inlineStr"/>
+      <c r="H194" s="3" t="inlineStr"/>
+      <c r="I194" s="3" t="inlineStr"/>
+      <c r="J194" s="3" t="inlineStr">
+        <is>
+          <t>Explicitly independent 'family vets for family pets' serving Weybridge/Leatherhead/Cobham - three wealthy towns from one site</t>
+        </is>
+      </c>
+      <c r="K194" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L194" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M194" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N194" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O194" s="3" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P194" s="3" t="inlineStr">
+        <is>
+          <t>Multi-town catchment but single-location search visibility</t>
+        </is>
+      </c>
+      <c r="Q194" s="3" t="inlineStr">
+        <is>
+          <t>'Family vets for family pets' - turn that tagline into the AI-cited answer across 3 towns</t>
+        </is>
+      </c>
+      <c r="R194" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S194" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T194" s="3" t="inlineStr"/>
+    </row>
+    <row r="195">
+      <c r="A195" s="3" t="inlineStr">
+        <is>
+          <t>Concept Eight Architects</t>
+        </is>
+      </c>
+      <c r="B195" s="3" t="inlineStr">
+        <is>
+          <t>Architects</t>
+        </is>
+      </c>
+      <c r="C195" s="3" t="inlineStr">
+        <is>
+          <t>Weybridge, Surrey</t>
+        </is>
+      </c>
+      <c r="D195" s="3" t="inlineStr">
+        <is>
+          <t>via RIBA directory listing</t>
+        </is>
+      </c>
+      <c r="E195" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F195" s="3" t="inlineStr"/>
+      <c r="G195" s="3" t="inlineStr"/>
+      <c r="H195" s="3" t="inlineStr"/>
+      <c r="I195" s="3" t="inlineStr"/>
+      <c r="J195" s="3" t="inlineStr">
+        <is>
+          <t>RIBA chartered since 2006, based in Weybridge; residential specialism in one of Surrey's wealthiest commuter towns</t>
+        </is>
+      </c>
+      <c r="K195" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L195" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M195" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N195" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O195" s="3" t="inlineStr">
+        <is>
+          <t>RIBA chartered practice</t>
+        </is>
+      </c>
+      <c r="P195" s="3" t="inlineStr">
+        <is>
+          <t>Established credentials not converted into local AI-search dominance</t>
+        </is>
+      </c>
+      <c r="Q195" s="3" t="inlineStr">
+        <is>
+          <t>Own 'architect Weybridge/Cobham' - direct geographic match to their office</t>
+        </is>
+      </c>
+      <c r="R195" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S195" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T195" s="3" t="inlineStr">
+        <is>
+          <t>Confirm live website before outreach</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="3" t="inlineStr">
+        <is>
+          <t>Dr Cat Aesthetics</t>
+        </is>
+      </c>
+      <c r="B196" s="3" t="inlineStr">
+        <is>
+          <t>Aesthetics clinic</t>
+        </is>
+      </c>
+      <c r="C196" s="3" t="inlineStr">
+        <is>
+          <t>Weybridge, Surrey</t>
+        </is>
+      </c>
+      <c r="D196" s="3" t="inlineStr">
+        <is>
+          <t>https://drcataesthetics.com</t>
+        </is>
+      </c>
+      <c r="E196" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F196" s="3" t="inlineStr"/>
+      <c r="G196" s="3" t="inlineStr">
+        <is>
+          <t>Dr Cat (Founder, practising NHS GP)</t>
+        </is>
+      </c>
+      <c r="H196" s="3" t="inlineStr"/>
+      <c r="I196" s="3" t="inlineStr"/>
+      <c r="J196" s="3" t="inlineStr">
+        <is>
+          <t>Doctor-led (practising GP) aesthetics clinic; strong trust credential; repeat injectable clients in wealthy Weybridge</t>
+        </is>
+      </c>
+      <c r="K196" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L196" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M196" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N196" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O196" s="3" t="inlineStr">
+        <is>
+          <t>Professional site</t>
+        </is>
+      </c>
+      <c r="P196" s="3" t="inlineStr">
+        <is>
+          <t>GP credential is a strong differentiator not yet leveraged for AI-search trust signals</t>
+        </is>
+      </c>
+      <c r="Q196" s="3" t="inlineStr">
+        <is>
+          <t>'A real GP doing your Botox' - own that credibility angle in AEO content</t>
+        </is>
+      </c>
+      <c r="R196" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S196" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T196" s="3" t="inlineStr"/>
+    </row>
+    <row r="197">
+      <c r="A197" s="3" t="inlineStr">
+        <is>
+          <t>The Norup Clinic</t>
+        </is>
+      </c>
+      <c r="B197" s="3" t="inlineStr">
+        <is>
+          <t>Aesthetics &amp; skin clinic</t>
+        </is>
+      </c>
+      <c r="C197" s="3" t="inlineStr">
+        <is>
+          <t>Esher, Surrey (serves Cobham/Weybridge/Walton)</t>
+        </is>
+      </c>
+      <c r="D197" s="3" t="inlineStr">
+        <is>
+          <t>https://www.thenorupclinic.co.uk</t>
+        </is>
+      </c>
+      <c r="E197" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F197" s="3" t="inlineStr"/>
+      <c r="G197" s="3" t="inlineStr">
+        <is>
+          <t>Dr Mette Norup (Founder)</t>
+        </is>
+      </c>
+      <c r="H197" s="3" t="inlineStr"/>
+      <c r="I197" s="3" t="inlineStr"/>
+      <c r="J197" s="3" t="inlineStr">
+        <is>
+          <t>Named-doctor clinic covering 4 wealthy Surrey towns from one base; high-value repeat skin/aesthetic clients</t>
+        </is>
+      </c>
+      <c r="K197" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L197" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M197" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N197" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O197" s="3" t="inlineStr">
+        <is>
+          <t>Multi-town service area</t>
+        </is>
+      </c>
+      <c r="P197" s="3" t="inlineStr">
+        <is>
+          <t>Single clinic serving 4 towns needs 4x the local search presence it currently has</t>
+        </is>
+      </c>
+      <c r="Q197" s="3" t="inlineStr">
+        <is>
+          <t>Per-town local SEO + AEO to match the multi-town service claim</t>
+        </is>
+      </c>
+      <c r="R197" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S197" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T197" s="3" t="inlineStr"/>
+    </row>
+    <row r="198">
+      <c r="A198" s="4" t="inlineStr">
+        <is>
+          <t>Light Touch Clinic</t>
+        </is>
+      </c>
+      <c r="B198" s="4" t="inlineStr">
+        <is>
+          <t>Aesthetics clinic</t>
+        </is>
+      </c>
+      <c r="C198" s="4" t="inlineStr">
+        <is>
+          <t>Weybridge, Surrey</t>
+        </is>
+      </c>
+      <c r="D198" s="4" t="inlineStr">
+        <is>
+          <t>https://lighttouchclinic.co.uk</t>
+        </is>
+      </c>
+      <c r="E198" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F198" s="4" t="inlineStr"/>
+      <c r="G198" s="4" t="inlineStr">
+        <is>
+          <t>Dr Natalie Geary (Medical Lead)</t>
+        </is>
+      </c>
+      <c r="H198" s="4" t="inlineStr"/>
+      <c r="I198" s="4" t="inlineStr"/>
+      <c r="J198" s="4" t="inlineStr">
+        <is>
+          <t>Award-winning medical team; doctor-led positioning in a competitive Surrey aesthetics market</t>
+        </is>
+      </c>
+      <c r="K198" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L198" s="4" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M198" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N198" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O198" s="4" t="inlineStr">
+        <is>
+          <t>Awards promoted</t>
+        </is>
+      </c>
+      <c r="P198" s="4" t="inlineStr">
+        <is>
+          <t>Awards don't automatically appear in AI-search answers</t>
+        </is>
+      </c>
+      <c r="Q198" s="4" t="inlineStr">
+        <is>
+          <t>Turn award-winning status into the AI-cited trust signal for Weybridge aesthetics</t>
+        </is>
+      </c>
+      <c r="R198" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S198" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T198" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T187"/>
+  <autoFilter ref="A1:T198"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16680,7 +17632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B99"/>
+  <dimension ref="A1:B100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -16700,7 +17652,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>186</v>
+        <v>197</v>
       </c>
     </row>
     <row r="5">
@@ -16717,7 +17669,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7">
@@ -16727,7 +17679,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8">
@@ -16737,13 +17689,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Wedding venue</t>
+          <t>Independent vet</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -16753,11 +17705,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Independent vet</t>
+          <t>Wedding venue</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11">
@@ -16773,17 +17725,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Physiotherapy clinic</t>
+          <t>Aesthetics clinic</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Chartered accountants</t>
+          <t>Physiotherapy clinic</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -16793,17 +17745,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Mortgage broker</t>
+          <t>Chartered accountants</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Solar installer</t>
+          <t>Mortgage broker</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -16813,7 +17765,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Private GP</t>
+          <t>Solar installer</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -16823,7 +17775,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Aesthetics clinic</t>
+          <t>Private GP</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -17647,6 +18599,16 @@
         </is>
       </c>
       <c r="B99" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Aesthetics &amp; skin clinic</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 9: +9 prospects (206 total) - Guildford/Weybridge finance & trades, Wiltshire venues
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$198</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$207</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T198"/>
+  <dimension ref="A1:T207"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -17620,8 +17620,760 @@
       </c>
       <c r="T198" s="4" t="inlineStr"/>
     </row>
+    <row r="199">
+      <c r="A199" s="4" t="inlineStr">
+        <is>
+          <t>The Recruitment Consultancy</t>
+        </is>
+      </c>
+      <c r="B199" s="4" t="inlineStr">
+        <is>
+          <t>Recruitment agency</t>
+        </is>
+      </c>
+      <c r="C199" s="4" t="inlineStr">
+        <is>
+          <t>Guildford (+ Worthing)</t>
+        </is>
+      </c>
+      <c r="D199" s="4" t="inlineStr">
+        <is>
+          <t>https://therecruitmentconsultancy.com</t>
+        </is>
+      </c>
+      <c r="E199" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F199" s="4" t="inlineStr">
+        <is>
+          <t>01483 456465</t>
+        </is>
+      </c>
+      <c r="G199" s="4" t="inlineStr">
+        <is>
+          <t>Sharon Ellis (Managing Director)</t>
+        </is>
+      </c>
+      <c r="H199" s="4" t="inlineStr"/>
+      <c r="I199" s="4" t="inlineStr"/>
+      <c r="J199" s="4" t="inlineStr">
+        <is>
+          <t>Independent since 1997, 2 offices across Surrey/Sussex; placement fees + repeat SME client relationships</t>
+        </is>
+      </c>
+      <c r="K199" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L199" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M199" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N199" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O199" s="4" t="inlineStr">
+        <is>
+          <t>Established 2-office brand</t>
+        </is>
+      </c>
+      <c r="P199" s="4" t="inlineStr">
+        <is>
+          <t>Michael Page/Robert Half corporate brands dominate Guildford recruitment search</t>
+        </is>
+      </c>
+      <c r="Q199" s="4" t="inlineStr">
+        <is>
+          <t>'Guildford SMEs ask AI for a recruiter who knows the local market - be that answer'</t>
+        </is>
+      </c>
+      <c r="R199" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S199" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T199" s="4" t="inlineStr"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="3" t="inlineStr">
+        <is>
+          <t>Price Ferguson Wealth Management</t>
+        </is>
+      </c>
+      <c r="B200" s="3" t="inlineStr">
+        <is>
+          <t>Wealth management / IFA</t>
+        </is>
+      </c>
+      <c r="C200" s="3" t="inlineStr">
+        <is>
+          <t>Guildford (+ Farnham)</t>
+        </is>
+      </c>
+      <c r="D200" s="3" t="inlineStr">
+        <is>
+          <t>https://priceferguson.com</t>
+        </is>
+      </c>
+      <c r="E200" s="3" t="inlineStr">
+        <is>
+          <t>info@priceferguson.com</t>
+        </is>
+      </c>
+      <c r="F200" s="3" t="inlineStr">
+        <is>
+          <t>01483 456 477</t>
+        </is>
+      </c>
+      <c r="G200" s="3" t="inlineStr">
+        <is>
+          <t>Michael Price (Founder, est. 1997)</t>
+        </is>
+      </c>
+      <c r="H200" s="3" t="inlineStr"/>
+      <c r="I200" s="3" t="inlineStr"/>
+      <c r="J200" s="3" t="inlineStr">
+        <is>
+          <t>Established 1997, multi-office Surrey wealth manager; client AUM relationships worth tens of thousands in fees</t>
+        </is>
+      </c>
+      <c r="K200" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L200" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M200" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N200" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O200" s="3" t="inlineStr">
+        <is>
+          <t>Multi-office landing pages</t>
+        </is>
+      </c>
+      <c r="P200" s="3" t="inlineStr">
+        <is>
+          <t>Rathbones/HFMC/Chapters all compete for the same affluent Guildford searches</t>
+        </is>
+      </c>
+      <c r="Q200" s="3" t="inlineStr">
+        <is>
+          <t>'27 years managing Guildford's wealth - let's make sure AI knows it'</t>
+        </is>
+      </c>
+      <c r="R200" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S200" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T200" s="3" t="inlineStr"/>
+    </row>
+    <row r="201">
+      <c r="A201" s="3" t="inlineStr">
+        <is>
+          <t>Pembroke Consulting</t>
+        </is>
+      </c>
+      <c r="B201" s="3" t="inlineStr">
+        <is>
+          <t>IFA / financial planning</t>
+        </is>
+      </c>
+      <c r="C201" s="3" t="inlineStr">
+        <is>
+          <t>Weybridge, Surrey</t>
+        </is>
+      </c>
+      <c r="D201" s="3" t="inlineStr">
+        <is>
+          <t>https://www.pembroke.uk.net</t>
+        </is>
+      </c>
+      <c r="E201" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F201" s="3" t="inlineStr"/>
+      <c r="G201" s="3" t="inlineStr">
+        <is>
+          <t>Tony Jaume (Founder, est. 1996)</t>
+        </is>
+      </c>
+      <c r="H201" s="3" t="inlineStr"/>
+      <c r="I201" s="3" t="inlineStr"/>
+      <c r="J201" s="3" t="inlineStr">
+        <is>
+          <t>Independent since 1996 in wealthy Weybridge; long-tenured founder-adviser relationships</t>
+        </is>
+      </c>
+      <c r="K201" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L201" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M201" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N201" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O201" s="3" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P201" s="3" t="inlineStr">
+        <is>
+          <t>Nearly 30 years of trust invisible in modern local/AI search</t>
+        </is>
+      </c>
+      <c r="Q201" s="3" t="inlineStr">
+        <is>
+          <t>Turn three decades of Weybridge trust into the AI-cited local IFA answer</t>
+        </is>
+      </c>
+      <c r="R201" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S201" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T201" s="3" t="inlineStr"/>
+    </row>
+    <row r="202">
+      <c r="A202" s="3" t="inlineStr">
+        <is>
+          <t>Rosan Helmsley</t>
+        </is>
+      </c>
+      <c r="B202" s="3" t="inlineStr">
+        <is>
+          <t>Wealth management &amp; employee benefits</t>
+        </is>
+      </c>
+      <c r="C202" s="3" t="inlineStr">
+        <is>
+          <t>Guildford, Surrey</t>
+        </is>
+      </c>
+      <c r="D202" s="3" t="inlineStr">
+        <is>
+          <t>https://www.rosan-ifa.com</t>
+        </is>
+      </c>
+      <c r="E202" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F202" s="3" t="inlineStr"/>
+      <c r="G202" s="3" t="inlineStr"/>
+      <c r="H202" s="3" t="inlineStr"/>
+      <c r="I202" s="3" t="inlineStr"/>
+      <c r="J202" s="3" t="inlineStr">
+        <is>
+          <t>Independent since 2001; advisers average 20+ years' experience; corporate benefits arm = B2B revenue line too</t>
+        </is>
+      </c>
+      <c r="K202" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L202" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M202" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N202" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O202" s="3" t="inlineStr">
+        <is>
+          <t>Professional site</t>
+        </is>
+      </c>
+      <c r="P202" s="3" t="inlineStr">
+        <is>
+          <t>Two service lines (personal wealth + corporate benefits) competing for attention without unified AEO strategy</t>
+        </is>
+      </c>
+      <c r="Q202" s="3" t="inlineStr">
+        <is>
+          <t>Split content strategy: separate AEO tracks for personal wealth vs corporate benefits searches</t>
+        </is>
+      </c>
+      <c r="R202" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S202" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T202" s="3" t="inlineStr"/>
+    </row>
+    <row r="203">
+      <c r="A203" s="4" t="inlineStr">
+        <is>
+          <t>RH Electrical Services</t>
+        </is>
+      </c>
+      <c r="B203" s="4" t="inlineStr">
+        <is>
+          <t>Electrician</t>
+        </is>
+      </c>
+      <c r="C203" s="4" t="inlineStr">
+        <is>
+          <t>Weybridge (serves Surrey/SW London)</t>
+        </is>
+      </c>
+      <c r="D203" s="4" t="inlineStr">
+        <is>
+          <t>https://www.rh-electrical.co.uk</t>
+        </is>
+      </c>
+      <c r="E203" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F203" s="4" t="inlineStr"/>
+      <c r="G203" s="4" t="inlineStr">
+        <is>
+          <t>Andy Hedges (Owner, NICEIC since 2007)</t>
+        </is>
+      </c>
+      <c r="H203" s="4" t="inlineStr"/>
+      <c r="I203" s="4" t="inlineStr"/>
+      <c r="J203" s="4" t="inlineStr">
+        <is>
+          <t>Established 1976 - nearly 50 years trading; NICEIC member; rewires/consumer units in premium Surrey homes</t>
+        </is>
+      </c>
+      <c r="K203" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L203" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M203" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N203" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O203" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P203" s="4" t="inlineStr">
+        <is>
+          <t>Half a century of trust doesn't show up in 'electrician Weybridge' searches</t>
+        </is>
+      </c>
+      <c r="Q203" s="4" t="inlineStr">
+        <is>
+          <t>'49 years wiring Weybridge homes - time AI knew it too'</t>
+        </is>
+      </c>
+      <c r="R203" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S203" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T203" s="4" t="inlineStr"/>
+    </row>
+    <row r="204">
+      <c r="A204" s="3" t="inlineStr">
+        <is>
+          <t>Surrey Roofing Specialists</t>
+        </is>
+      </c>
+      <c r="B204" s="3" t="inlineStr">
+        <is>
+          <t>Roofer</t>
+        </is>
+      </c>
+      <c r="C204" s="3" t="inlineStr">
+        <is>
+          <t>Addlestone (serves Weybridge/Esher/Cobham/Guildford)</t>
+        </is>
+      </c>
+      <c r="D204" s="3" t="inlineStr">
+        <is>
+          <t>https://www.surreyroofingspecialists.co.uk</t>
+        </is>
+      </c>
+      <c r="E204" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F204" s="3" t="inlineStr">
+        <is>
+          <t>07946 640262</t>
+        </is>
+      </c>
+      <c r="G204" s="3" t="inlineStr">
+        <is>
+          <t>Carl (Director)</t>
+        </is>
+      </c>
+      <c r="H204" s="3" t="inlineStr"/>
+      <c r="I204" s="3" t="inlineStr"/>
+      <c r="J204" s="3" t="inlineStr">
+        <is>
+          <t>Covers 10+ wealthy Surrey/SW London towns from one base; roof jobs £5-20k in premium housing stock</t>
+        </is>
+      </c>
+      <c r="K204" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L204" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M204" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N204" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O204" s="3" t="inlineStr">
+        <is>
+          <t>CORC membership (Confederation of Roofing Contractors)</t>
+        </is>
+      </c>
+      <c r="P204" s="3" t="inlineStr">
+        <is>
+          <t>Wide catchment but thin per-town search visibility - opportunity to dominate several towns at once</t>
+        </is>
+      </c>
+      <c r="Q204" s="3" t="inlineStr">
+        <is>
+          <t>Multi-town local SEO campaign covering the whole Surrey Roofing Specialists service area</t>
+        </is>
+      </c>
+      <c r="R204" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S204" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T204" s="3" t="inlineStr"/>
+    </row>
+    <row r="205">
+      <c r="A205" s="3" t="inlineStr">
+        <is>
+          <t>Barford Park Barn</t>
+        </is>
+      </c>
+      <c r="B205" s="3" t="inlineStr">
+        <is>
+          <t>Wedding venue</t>
+        </is>
+      </c>
+      <c r="C205" s="3" t="inlineStr">
+        <is>
+          <t>Downton, near Salisbury, Wiltshire</t>
+        </is>
+      </c>
+      <c r="D205" s="3" t="inlineStr">
+        <is>
+          <t>https://barfordparkweddings.co.uk</t>
+        </is>
+      </c>
+      <c r="E205" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F205" s="3" t="inlineStr"/>
+      <c r="G205" s="3" t="inlineStr"/>
+      <c r="H205" s="3" t="inlineStr"/>
+      <c r="I205" s="3" t="inlineStr"/>
+      <c r="J205" s="3" t="inlineStr">
+        <is>
+          <t>300-acre family farm wedding venue, seats 150-200; Wiltshire weddings worth £15-25k each</t>
+        </is>
+      </c>
+      <c r="K205" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L205" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M205" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N205" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O205" s="3" t="inlineStr">
+        <is>
+          <t>Multiple directory listings (Guides for Brides, Bridebook, Confetti)</t>
+        </is>
+      </c>
+      <c r="P205" s="3" t="inlineStr">
+        <is>
+          <t>Heavy directory dependence - same commission-middleman pattern as other venues</t>
+        </is>
+      </c>
+      <c r="Q205" s="3" t="inlineStr">
+        <is>
+          <t>'Own the AI-recommended shortlist for South Wiltshire barn weddings directly'</t>
+        </is>
+      </c>
+      <c r="R205" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S205" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T205" s="3" t="inlineStr"/>
+    </row>
+    <row r="206">
+      <c r="A206" s="3" t="inlineStr">
+        <is>
+          <t>Manor Estate</t>
+        </is>
+      </c>
+      <c r="B206" s="3" t="inlineStr">
+        <is>
+          <t>Wedding venue</t>
+        </is>
+      </c>
+      <c r="C206" s="3" t="inlineStr">
+        <is>
+          <t>Wiltshire</t>
+        </is>
+      </c>
+      <c r="D206" s="3" t="inlineStr">
+        <is>
+          <t>https://manorestate.co.uk</t>
+        </is>
+      </c>
+      <c r="E206" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F206" s="3" t="inlineStr"/>
+      <c r="G206" s="3" t="inlineStr"/>
+      <c r="H206" s="3" t="inlineStr"/>
+      <c r="I206" s="3" t="inlineStr"/>
+      <c r="J206" s="3" t="inlineStr">
+        <is>
+          <t>Grade II* listed manor house + barn, privately owned; premium exclusive-use weddings</t>
+        </is>
+      </c>
+      <c r="K206" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L206" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M206" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N206" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O206" s="3" t="inlineStr">
+        <is>
+          <t>Polished dedicated wedding site</t>
+        </is>
+      </c>
+      <c r="P206" s="3" t="inlineStr">
+        <is>
+          <t>Grade II* listing not leveraged as an AI-search authority/trust signal</t>
+        </is>
+      </c>
+      <c r="Q206" s="3" t="inlineStr">
+        <is>
+          <t>Heritage-listing content as the AEO differentiator vs generic barn venues</t>
+        </is>
+      </c>
+      <c r="R206" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S206" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T206" s="3" t="inlineStr"/>
+    </row>
+    <row r="207">
+      <c r="A207" s="4" t="inlineStr">
+        <is>
+          <t>Wellington Barn</t>
+        </is>
+      </c>
+      <c r="B207" s="4" t="inlineStr">
+        <is>
+          <t>Wedding venue</t>
+        </is>
+      </c>
+      <c r="C207" s="4" t="inlineStr">
+        <is>
+          <t>Wiltshire</t>
+        </is>
+      </c>
+      <c r="D207" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wellingtonbarn.co.uk</t>
+        </is>
+      </c>
+      <c r="E207" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F207" s="4" t="inlineStr"/>
+      <c r="G207" s="4" t="inlineStr"/>
+      <c r="H207" s="4" t="inlineStr"/>
+      <c r="I207" s="4" t="inlineStr"/>
+      <c r="J207" s="4" t="inlineStr">
+        <is>
+          <t>'Wiltshire's original authentic barn venue' - strong positioning claim; countryside views</t>
+        </is>
+      </c>
+      <c r="K207" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L207" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M207" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N207" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O207" s="4" t="inlineStr">
+        <is>
+          <t>Branded positioning ('original authentic')</t>
+        </is>
+      </c>
+      <c r="P207" s="4" t="inlineStr">
+        <is>
+          <t>Positioning claim not yet the AI-cited answer for 'original barn venue Wiltshire'</t>
+        </is>
+      </c>
+      <c r="Q207" s="4" t="inlineStr">
+        <is>
+          <t>Own the 'original authentic barn' AEO positioning outright</t>
+        </is>
+      </c>
+      <c r="R207" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S207" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T207" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T198"/>
+  <autoFilter ref="A1:T207"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -17632,7 +18384,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B100"/>
+  <dimension ref="A1:B103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -17652,7 +18404,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>197</v>
+        <v>206</v>
       </c>
     </row>
     <row r="5">
@@ -17685,27 +18437,27 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Architects</t>
+          <t>Wedding venue</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Independent vet</t>
+          <t>Architects</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Wedding venue</t>
+          <t>Independent vet</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -17795,7 +18547,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Personal training studio</t>
+          <t>Electrician</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -17805,7 +18557,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Family law firm</t>
+          <t>Personal training studio</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -17815,7 +18567,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Immigration law firm</t>
+          <t>Family law firm</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -17825,27 +18577,27 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Letting agent</t>
+          <t>Recruitment agency</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Financial adviser / wealth management</t>
+          <t>Immigration law firm</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Private tuition agency</t>
+          <t>Letting agent</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -17855,7 +18607,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Osteopathy clinic</t>
+          <t>Financial adviser / wealth management</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -17865,7 +18617,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating / boilers</t>
+          <t>Private tuition agency</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -17875,7 +18627,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Electrician</t>
+          <t>Osteopathy clinic</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -17885,7 +18637,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Event &amp; wedding caterer</t>
+          <t>Roofer</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -17895,7 +18647,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Chiropractor</t>
+          <t>Plumbing &amp; heating / boilers</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -17905,7 +18657,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Estate agent (premium)</t>
+          <t>Event &amp; wedding caterer</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -17915,7 +18667,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Orthodontist</t>
+          <t>Chiropractor</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -17925,7 +18677,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Employment law firm</t>
+          <t>Estate agent (premium)</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -17935,7 +18687,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Event management agency</t>
+          <t>Orthodontist</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -17945,7 +18697,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Private dentist / implants</t>
+          <t>Employment law firm</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -17955,7 +18707,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Design &amp; build</t>
+          <t>Event management agency</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -17965,7 +18717,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Recruitment agency</t>
+          <t>Private dentist / implants</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -17975,7 +18727,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>IT support / MSP</t>
+          <t>Design &amp; build</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -17985,17 +18737,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Dentist / Orthodontics</t>
+          <t>IT support / MSP</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Specialist dental/implant clinic</t>
+          <t>Dentist / Orthodontics</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -18005,7 +18757,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Boutique corporate law firm</t>
+          <t>Specialist dental/implant clinic</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -18015,7 +18767,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Cosmetic/aesthetics clinic</t>
+          <t>Boutique corporate law firm</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -18025,7 +18777,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Skin &amp; laser clinic</t>
+          <t>Cosmetic/aesthetics clinic</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -18035,7 +18787,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Mortgage broker / financial adviser</t>
+          <t>Skin &amp; laser clinic</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -18045,7 +18797,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Architects (RIBA chartered)</t>
+          <t>Mortgage broker / financial adviser</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -18055,7 +18807,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Recruitment agency (tech/startups)</t>
+          <t>Architects (RIBA chartered)</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -18065,7 +18817,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Recruitment agency (IT/data)</t>
+          <t>Recruitment agency (tech/startups)</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -18075,7 +18827,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Independent vet (24/7 emergency)</t>
+          <t>Recruitment agency (IT/data)</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -18085,7 +18837,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Interior design studio</t>
+          <t>Independent vet (24/7 emergency)</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -18095,7 +18847,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Letting &amp; estate agent</t>
+          <t>Interior design studio</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -18105,7 +18857,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Cosmetic clinic (injectables)</t>
+          <t>Letting &amp; estate agent</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -18115,7 +18867,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Cosmetic/anti-ageing clinic</t>
+          <t>Cosmetic clinic (injectables)</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -18125,7 +18877,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Yoga &amp; reformer pilates studio</t>
+          <t>Cosmetic/anti-ageing clinic</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -18135,7 +18887,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Reformer pilates studio</t>
+          <t>Yoga &amp; reformer pilates studio</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -18145,7 +18897,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Wealth management</t>
+          <t>Reformer pilates studio</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -18155,7 +18907,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Private tuition &amp; education consultancy</t>
+          <t>Wealth management</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -18165,7 +18917,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Osteopath</t>
+          <t>Private tuition &amp; education consultancy</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -18175,7 +18927,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Design &amp; build / home renovation</t>
+          <t>Osteopath</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -18185,7 +18937,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Builders / building contractor</t>
+          <t>Design &amp; build / home renovation</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -18195,7 +18947,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Roofer</t>
+          <t>Builders / building contractor</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -18609,6 +19361,36 @@
         </is>
       </c>
       <c r="B100" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Wealth management / IFA</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>IFA / financial planning</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Wealth management &amp; employee benefits</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 10: +8 prospects (214 total) - Guildford, Reigate, Wandsworth, Ealing estate agents
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$207</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$215</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T207"/>
+  <dimension ref="A1:T215"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -18372,8 +18372,684 @@
       </c>
       <c r="T207" s="4" t="inlineStr"/>
     </row>
+    <row r="208">
+      <c r="A208" s="3" t="inlineStr">
+        <is>
+          <t>Cavender Estate Agent</t>
+        </is>
+      </c>
+      <c r="B208" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C208" s="3" t="inlineStr">
+        <is>
+          <t>Guildford &amp; Godalming, Surrey</t>
+        </is>
+      </c>
+      <c r="D208" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cavenders.co.uk</t>
+        </is>
+      </c>
+      <c r="E208" s="3" t="inlineStr">
+        <is>
+          <t>info@cavenders.co.uk</t>
+        </is>
+      </c>
+      <c r="F208" s="3" t="inlineStr">
+        <is>
+          <t>01483 457 728</t>
+        </is>
+      </c>
+      <c r="G208" s="3" t="inlineStr"/>
+      <c r="H208" s="3" t="inlineStr"/>
+      <c r="I208" s="3" t="inlineStr"/>
+      <c r="J208" s="3" t="inlineStr">
+        <is>
+          <t>Truly independent since 2012 across two Surrey towns; residential sales/lettings for professional-family stock</t>
+        </is>
+      </c>
+      <c r="K208" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L208" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M208" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N208" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O208" s="3" t="inlineStr">
+        <is>
+          <t>Two-office presence</t>
+        </is>
+      </c>
+      <c r="P208" s="3" t="inlineStr">
+        <is>
+          <t>Bourne/Curchods/Clarke Gammon corporate-scale rivals dominate Guildford search</t>
+        </is>
+      </c>
+      <c r="Q208" s="3" t="inlineStr">
+        <is>
+          <t>'Guildford's genuinely independent agent should win the AI answer, not the network brands'</t>
+        </is>
+      </c>
+      <c r="R208" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S208" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T208" s="3" t="inlineStr"/>
+    </row>
+    <row r="209">
+      <c r="A209" s="3" t="inlineStr">
+        <is>
+          <t>Ralph James</t>
+        </is>
+      </c>
+      <c r="B209" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C209" s="3" t="inlineStr">
+        <is>
+          <t>Reigate, Redhill, Dorking, Banstead, Surrey</t>
+        </is>
+      </c>
+      <c r="D209" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ralphjames.co.uk</t>
+        </is>
+      </c>
+      <c r="E209" s="3" t="inlineStr">
+        <is>
+          <t>reigate@ralphjames.co.uk</t>
+        </is>
+      </c>
+      <c r="F209" s="3" t="inlineStr">
+        <is>
+          <t>01737 333 677</t>
+        </is>
+      </c>
+      <c r="G209" s="3" t="inlineStr">
+        <is>
+          <t>Thomas Cullum Cina &amp; Paul Cooney (Senior management)</t>
+        </is>
+      </c>
+      <c r="H209" s="3" t="inlineStr"/>
+      <c r="I209" s="3" t="inlineStr"/>
+      <c r="J209" s="3" t="inlineStr">
+        <is>
+          <t>Independent since 2015, 4-office growth in premium Surrey towns; outperforming rivals in Redhill/Reigate per their own claim</t>
+        </is>
+      </c>
+      <c r="K209" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L209" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M209" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N209" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O209" s="3" t="inlineStr">
+        <is>
+          <t>Per-office landing pages; growth-stage marketing awareness</t>
+        </is>
+      </c>
+      <c r="P209" s="3" t="inlineStr">
+        <is>
+          <t>Rapid 4-office growth needs matching search-visibility growth across all locations</t>
+        </is>
+      </c>
+      <c r="Q209" s="3" t="inlineStr">
+        <is>
+          <t>'You outperform rivals locally - let's make sure AI says so across all 4 towns'</t>
+        </is>
+      </c>
+      <c r="R209" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S209" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T209" s="3" t="inlineStr"/>
+    </row>
+    <row r="210">
+      <c r="A210" s="3" t="inlineStr">
+        <is>
+          <t>White &amp; Sons</t>
+        </is>
+      </c>
+      <c r="B210" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C210" s="3" t="inlineStr">
+        <is>
+          <t>Dorking, Reigate, Horley, Oxted, Leatherhead</t>
+        </is>
+      </c>
+      <c r="D210" s="3" t="inlineStr">
+        <is>
+          <t>https://www.whiteandsons.co.uk</t>
+        </is>
+      </c>
+      <c r="E210" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F210" s="3" t="inlineStr"/>
+      <c r="G210" s="3" t="inlineStr"/>
+      <c r="H210" s="3" t="inlineStr"/>
+      <c r="I210" s="3" t="inlineStr"/>
+      <c r="J210" s="3" t="inlineStr">
+        <is>
+          <t>Established 1817 - over 200 years trading; 5-office coverage of Surrey's wealthiest towns</t>
+        </is>
+      </c>
+      <c r="K210" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L210" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M210" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N210" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O210" s="3" t="inlineStr">
+        <is>
+          <t>Multi-office; 'cutting edge technology' self-description</t>
+        </is>
+      </c>
+      <c r="P210" s="3" t="inlineStr">
+        <is>
+          <t>200 years of heritage vastly under-leveraged as an AI-search trust signal</t>
+        </is>
+      </c>
+      <c r="Q210" s="3" t="inlineStr">
+        <is>
+          <t>'207 years in Surrey property - the AI answer should reflect that, not just Rightmove'</t>
+        </is>
+      </c>
+      <c r="R210" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S210" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T210" s="3" t="inlineStr"/>
+    </row>
+    <row r="211">
+      <c r="A211" s="3" t="inlineStr">
+        <is>
+          <t>Rochford Stokes</t>
+        </is>
+      </c>
+      <c r="B211" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C211" s="3" t="inlineStr">
+        <is>
+          <t>Battersea/Clapham/Wandsworth/Balham, London</t>
+        </is>
+      </c>
+      <c r="D211" s="3" t="inlineStr">
+        <is>
+          <t>https://www.rochfordstokes.com</t>
+        </is>
+      </c>
+      <c r="E211" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F211" s="3" t="inlineStr"/>
+      <c r="G211" s="3" t="inlineStr">
+        <is>
+          <t>Founders with 35+ years combined experience each (est. 2006)</t>
+        </is>
+      </c>
+      <c r="H211" s="3" t="inlineStr"/>
+      <c r="I211" s="3" t="inlineStr"/>
+      <c r="J211" s="3" t="inlineStr">
+        <is>
+          <t>Founder-run since 2006 across SW11/SW4 postcodes; high property values, repeat-client relationships</t>
+        </is>
+      </c>
+      <c r="K211" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L211" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M211" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N211" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O211" s="3" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P211" s="3" t="inlineStr">
+        <is>
+          <t>Marsh &amp; Parsons/Jacksons corporate-scale rivals dominate the same postcodes</t>
+        </is>
+      </c>
+      <c r="Q211" s="3" t="inlineStr">
+        <is>
+          <t>35 years' combined experience as the AEO trust signal vs bigger network brands</t>
+        </is>
+      </c>
+      <c r="R211" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S211" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T211" s="3" t="inlineStr"/>
+    </row>
+    <row r="212">
+      <c r="A212" s="3" t="inlineStr">
+        <is>
+          <t>C. Scott &amp; Co</t>
+        </is>
+      </c>
+      <c r="B212" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C212" s="3" t="inlineStr">
+        <is>
+          <t>Wandsworth Common, London SW18</t>
+        </is>
+      </c>
+      <c r="D212" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cscottandco.com</t>
+        </is>
+      </c>
+      <c r="E212" s="3" t="inlineStr">
+        <is>
+          <t>carrie@cscottandco.com</t>
+        </is>
+      </c>
+      <c r="F212" s="3" t="inlineStr"/>
+      <c r="G212" s="3" t="inlineStr">
+        <is>
+          <t>Carrie Scott (Founder)</t>
+        </is>
+      </c>
+      <c r="H212" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/carriescottcscottandco</t>
+        </is>
+      </c>
+      <c r="I212" s="3" t="inlineStr">
+        <is>
+          <t>instagram.com/c.scottandco_estateagents</t>
+        </is>
+      </c>
+      <c r="J212" s="3" t="inlineStr">
+        <is>
+          <t>Award-winning independent, 25+ years serving Wandsworth/Balham/Earlsfield/Streatham/Tooting</t>
+        </is>
+      </c>
+      <c r="K212" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L212" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M212" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N212" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O212" s="3" t="inlineStr">
+        <is>
+          <t>Active Instagram presence; awards</t>
+        </is>
+      </c>
+      <c r="P212" s="3" t="inlineStr">
+        <is>
+          <t>Award-winning but competing with Jacksons/Porters/Realm for the same dense SW London postcodes</t>
+        </is>
+      </c>
+      <c r="Q212" s="3" t="inlineStr">
+        <is>
+          <t>'25 years and an award - now make sure ChatGPT recommends you over the corporate chains'</t>
+        </is>
+      </c>
+      <c r="R212" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S212" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T212" s="3" t="inlineStr"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="4" t="inlineStr">
+        <is>
+          <t>Porters Estate Agents</t>
+        </is>
+      </c>
+      <c r="B213" s="4" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C213" s="4" t="inlineStr">
+        <is>
+          <t>Balham, London SW17</t>
+        </is>
+      </c>
+      <c r="D213" s="4" t="inlineStr">
+        <is>
+          <t>https://portersbalham.com</t>
+        </is>
+      </c>
+      <c r="E213" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F213" s="4" t="inlineStr"/>
+      <c r="G213" s="4" t="inlineStr"/>
+      <c r="H213" s="4" t="inlineStr"/>
+      <c r="I213" s="4" t="inlineStr"/>
+      <c r="J213" s="4" t="inlineStr">
+        <is>
+          <t>Family-owned, 40 years trading, 100+ years combined team experience in Balham/Wandsworth</t>
+        </is>
+      </c>
+      <c r="K213" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L213" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M213" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N213" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O213" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P213" s="4" t="inlineStr">
+        <is>
+          <t>Longevity claim buried; newer branded independents (C.Scott, Patrick Henry) out-market them digitally</t>
+        </is>
+      </c>
+      <c r="Q213" s="4" t="inlineStr">
+        <is>
+          <t>Turn '100 years combined experience' into the AI-cited local-expert answer</t>
+        </is>
+      </c>
+      <c r="R213" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S213" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T213" s="4" t="inlineStr"/>
+    </row>
+    <row r="214">
+      <c r="A214" s="4" t="inlineStr">
+        <is>
+          <t>Colin Bibra Estate Agents</t>
+        </is>
+      </c>
+      <c r="B214" s="4" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C214" s="4" t="inlineStr">
+        <is>
+          <t>Ealing, London W5</t>
+        </is>
+      </c>
+      <c r="D214" s="4" t="inlineStr">
+        <is>
+          <t>https://www.colinbibra.com</t>
+        </is>
+      </c>
+      <c r="E214" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F214" s="4" t="inlineStr">
+        <is>
+          <t>020 8566 3333</t>
+        </is>
+      </c>
+      <c r="G214" s="4" t="inlineStr">
+        <is>
+          <t>Colin Bibra (Founder, est. 1988)</t>
+        </is>
+      </c>
+      <c r="H214" s="4" t="inlineStr"/>
+      <c r="I214" s="4" t="inlineStr"/>
+      <c r="J214" s="4" t="inlineStr">
+        <is>
+          <t>Independent since 1988, founder's namesake brand; 35+ years in Ealing's premium property market</t>
+        </is>
+      </c>
+      <c r="K214" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L214" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M214" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N214" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O214" s="4" t="inlineStr">
+        <is>
+          <t>Established namesake brand</t>
+        </is>
+      </c>
+      <c r="P214" s="4" t="inlineStr">
+        <is>
+          <t>Corporate brands (Savills, haart) and Grimshaw/Robertson Smith &amp; Kempson compete for Ealing search visibility</t>
+        </is>
+      </c>
+      <c r="Q214" s="4" t="inlineStr">
+        <is>
+          <t>'The Ealing agent named after its founder - make AI say his name when clients search'</t>
+        </is>
+      </c>
+      <c r="R214" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S214" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T214" s="4" t="inlineStr"/>
+    </row>
+    <row r="215">
+      <c r="A215" s="4" t="inlineStr">
+        <is>
+          <t>Grimshaw and Co</t>
+        </is>
+      </c>
+      <c r="B215" s="4" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C215" s="4" t="inlineStr">
+        <is>
+          <t>Ealing, London W5</t>
+        </is>
+      </c>
+      <c r="D215" s="4" t="inlineStr">
+        <is>
+          <t>https://www.grimshawhomes.co.uk</t>
+        </is>
+      </c>
+      <c r="E215" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F215" s="4" t="inlineStr"/>
+      <c r="G215" s="4" t="inlineStr"/>
+      <c r="H215" s="4" t="inlineStr"/>
+      <c r="I215" s="4" t="inlineStr"/>
+      <c r="J215" s="4" t="inlineStr">
+        <is>
+          <t>Independent 50+ years in Ealing; deep local market knowledge, residential sales specialism</t>
+        </is>
+      </c>
+      <c r="K215" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L215" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M215" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N215" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O215" s="4" t="inlineStr">
+        <is>
+          <t>Half-century heritage promoted</t>
+        </is>
+      </c>
+      <c r="P215" s="4" t="inlineStr">
+        <is>
+          <t>50 years untranslated into digital-era search dominance</t>
+        </is>
+      </c>
+      <c r="Q215" s="4" t="inlineStr">
+        <is>
+          <t>'50 years knowing Ealing - it's time Google and AI knew it as well as your clients do'</t>
+        </is>
+      </c>
+      <c r="R215" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S215" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T215" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T207"/>
+  <autoFilter ref="A1:T215"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -18404,7 +19080,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>206</v>
+        <v>214</v>
       </c>
     </row>
     <row r="5">
@@ -18421,7 +19097,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
Batch 11: +6 prospects (220 total) - Balham/Chiswick dentists, SW London architects
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$215</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$221</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T215"/>
+  <dimension ref="A1:T221"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -19048,8 +19048,528 @@
       </c>
       <c r="T215" s="4" t="inlineStr"/>
     </row>
+    <row r="216">
+      <c r="A216" s="3" t="inlineStr">
+        <is>
+          <t>Balham Gateway Dental Practice</t>
+        </is>
+      </c>
+      <c r="B216" s="3" t="inlineStr">
+        <is>
+          <t>Private dentist / implants</t>
+        </is>
+      </c>
+      <c r="C216" s="3" t="inlineStr">
+        <is>
+          <t>Balham High Rd, London SW12</t>
+        </is>
+      </c>
+      <c r="D216" s="3" t="inlineStr">
+        <is>
+          <t>https://www.balhamgatewaydental.com</t>
+        </is>
+      </c>
+      <c r="E216" s="3" t="inlineStr">
+        <is>
+          <t>balham-gateway-dental@dentallymail.co.uk</t>
+        </is>
+      </c>
+      <c r="F216" s="3" t="inlineStr">
+        <is>
+          <t>020 8673 7887</t>
+        </is>
+      </c>
+      <c r="G216" s="3" t="inlineStr">
+        <is>
+          <t>Dr Panos Angelopoulos (Principal, acquired 2021)</t>
+        </is>
+      </c>
+      <c r="H216" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/panos-angelopoulos-78647a41</t>
+        </is>
+      </c>
+      <c r="I216" s="3" t="inlineStr"/>
+      <c r="J216" s="3" t="inlineStr">
+        <is>
+          <t>Independent since 1950s, new owner-principal with implant/oral surgery specialism; Invisalign provider since 2015</t>
+        </is>
+      </c>
+      <c r="K216" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L216" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M216" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N216" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O216" s="3" t="inlineStr">
+        <is>
+          <t>Doctify profile</t>
+        </is>
+      </c>
+      <c r="P216" s="3" t="inlineStr">
+        <is>
+          <t>70-year heritage + new specialist owner not yet converted into AI-search visibility</t>
+        </is>
+      </c>
+      <c r="Q216" s="3" t="inlineStr">
+        <is>
+          <t>'70 years in Balham, new implant expertise - let's make sure Google and AI both know both halves of the story'</t>
+        </is>
+      </c>
+      <c r="R216" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S216" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T216" s="3" t="inlineStr"/>
+    </row>
+    <row r="217">
+      <c r="A217" s="3" t="inlineStr">
+        <is>
+          <t>Chiswick Dental</t>
+        </is>
+      </c>
+      <c r="B217" s="3" t="inlineStr">
+        <is>
+          <t>Private dentist / implants</t>
+        </is>
+      </c>
+      <c r="C217" s="3" t="inlineStr">
+        <is>
+          <t>Chiswick High Road, London W4</t>
+        </is>
+      </c>
+      <c r="D217" s="3" t="inlineStr">
+        <is>
+          <t>https://www.chiswickdental.co.uk</t>
+        </is>
+      </c>
+      <c r="E217" s="3" t="inlineStr">
+        <is>
+          <t>info@chiswickdental.co.uk</t>
+        </is>
+      </c>
+      <c r="F217" s="3" t="inlineStr">
+        <is>
+          <t>020 8994 6202</t>
+        </is>
+      </c>
+      <c r="G217" s="3" t="inlineStr">
+        <is>
+          <t>Dr Gajen Pathmanathan (Principal, Implant &amp; Cosmetic Dentist)</t>
+        </is>
+      </c>
+      <c r="H217" s="3" t="inlineStr"/>
+      <c r="I217" s="3" t="inlineStr"/>
+      <c r="J217" s="3" t="inlineStr">
+        <is>
+          <t>Named implant/cosmetic specialist principal on Chiswick's main high street; premium W4 client base</t>
+        </is>
+      </c>
+      <c r="K217" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L217" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M217" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N217" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O217" s="3" t="inlineStr">
+        <is>
+          <t>Detailed referral/fees pages - marketing-aware</t>
+        </is>
+      </c>
+      <c r="P217" s="3" t="inlineStr">
+        <is>
+          <t>Referral infrastructure built but AI-answer visibility for 'implants Chiswick' still open</t>
+        </is>
+      </c>
+      <c r="Q217" s="3" t="inlineStr">
+        <is>
+          <t>'You built the referral pages - let's make sure ChatGPT recommends you to patients too'</t>
+        </is>
+      </c>
+      <c r="R217" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S217" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T217" s="3" t="inlineStr"/>
+    </row>
+    <row r="218">
+      <c r="A218" s="4" t="inlineStr">
+        <is>
+          <t>Juliet Moss &amp; Associates Physiotherapy</t>
+        </is>
+      </c>
+      <c r="B218" s="4" t="inlineStr">
+        <is>
+          <t>Physiotherapy clinic</t>
+        </is>
+      </c>
+      <c r="C218" s="4" t="inlineStr">
+        <is>
+          <t>Thurleigh Rd, Balham, London SW12</t>
+        </is>
+      </c>
+      <c r="D218" s="4" t="inlineStr">
+        <is>
+          <t>https://www.julietmossphysio.co.uk</t>
+        </is>
+      </c>
+      <c r="E218" s="4" t="inlineStr">
+        <is>
+          <t>info@julietmossphysio.co.uk</t>
+        </is>
+      </c>
+      <c r="F218" s="4" t="inlineStr">
+        <is>
+          <t>020 8675 5633</t>
+        </is>
+      </c>
+      <c r="G218" s="4" t="inlineStr">
+        <is>
+          <t>Juliet Moss (Founder)</t>
+        </is>
+      </c>
+      <c r="H218" s="4" t="inlineStr"/>
+      <c r="I218" s="4" t="inlineStr"/>
+      <c r="J218" s="4" t="inlineStr">
+        <is>
+          <t>Established practice serving Clapham/Balham/Wandsworth; insurance + self-pay mix in dense affluent SW postcodes</t>
+        </is>
+      </c>
+      <c r="K218" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L218" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M218" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N218" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O218" s="4" t="inlineStr">
+        <is>
+          <t>BUPA/CSP directory listings</t>
+        </is>
+      </c>
+      <c r="P218" s="4" t="inlineStr">
+        <is>
+          <t>Excellence Physiotherapy and reCentre Health compete for the same dense-postcode searches</t>
+        </is>
+      </c>
+      <c r="Q218" s="4" t="inlineStr">
+        <is>
+          <t>'Own the AI answer for physio across Clapham, Balham AND Wandsworth - not just one'</t>
+        </is>
+      </c>
+      <c r="R218" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S218" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T218" s="4" t="inlineStr"/>
+    </row>
+    <row r="219">
+      <c r="A219" s="3" t="inlineStr">
+        <is>
+          <t>Armstrong Simmonds Architects</t>
+        </is>
+      </c>
+      <c r="B219" s="3" t="inlineStr">
+        <is>
+          <t>Architects</t>
+        </is>
+      </c>
+      <c r="C219" s="3" t="inlineStr">
+        <is>
+          <t>Battersea, London SW11</t>
+        </is>
+      </c>
+      <c r="D219" s="3" t="inlineStr">
+        <is>
+          <t>https://www.as-architects.co.uk</t>
+        </is>
+      </c>
+      <c r="E219" s="3" t="inlineStr">
+        <is>
+          <t>projects@as-architects.co.uk</t>
+        </is>
+      </c>
+      <c r="F219" s="3" t="inlineStr">
+        <is>
+          <t>020 7228 1324</t>
+        </is>
+      </c>
+      <c r="G219" s="3" t="inlineStr">
+        <is>
+          <t>John Armstrong (Founder, est. 2010)</t>
+        </is>
+      </c>
+      <c r="H219" s="3" t="inlineStr"/>
+      <c r="I219" s="3" t="inlineStr"/>
+      <c r="J219" s="3" t="inlineStr">
+        <is>
+          <t>RIBA practice with dedicated per-borough landing pages (Wandsworth/Clapham/Battersea) - genuine SEO investment</t>
+        </is>
+      </c>
+      <c r="K219" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L219" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M219" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N219" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O219" s="3" t="inlineStr">
+        <is>
+          <t>Per-area landing pages = active SEO strategy</t>
+        </is>
+      </c>
+      <c r="P219" s="3" t="inlineStr">
+        <is>
+          <t>Landing pages exist across 3+ areas but AI-answer citations still open</t>
+        </is>
+      </c>
+      <c r="Q219" s="3" t="inlineStr">
+        <is>
+          <t>'You've built the SEO pages for 3 boroughs - add the AEO layer to make AI cite them too'</t>
+        </is>
+      </c>
+      <c r="R219" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S219" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T219" s="3" t="inlineStr"/>
+    </row>
+    <row r="220">
+      <c r="A220" s="4" t="inlineStr">
+        <is>
+          <t>Quartet Architecture</t>
+        </is>
+      </c>
+      <c r="B220" s="4" t="inlineStr">
+        <is>
+          <t>Architects</t>
+        </is>
+      </c>
+      <c r="C220" s="4" t="inlineStr">
+        <is>
+          <t>Wandsworth, London</t>
+        </is>
+      </c>
+      <c r="D220" s="4" t="inlineStr">
+        <is>
+          <t>https://www.quartetarchitecture.com</t>
+        </is>
+      </c>
+      <c r="E220" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F220" s="4" t="inlineStr"/>
+      <c r="G220" s="4" t="inlineStr"/>
+      <c r="H220" s="4" t="inlineStr"/>
+      <c r="I220" s="4" t="inlineStr"/>
+      <c r="J220" s="4" t="inlineStr">
+        <is>
+          <t>RIBA-chartered, 20+ years delivering bespoke residences in Wandsworth; high project values</t>
+        </is>
+      </c>
+      <c r="K220" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L220" s="4" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M220" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N220" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O220" s="4" t="inlineStr">
+        <is>
+          <t>Professional portfolio site</t>
+        </is>
+      </c>
+      <c r="P220" s="4" t="inlineStr">
+        <is>
+          <t>20 years' delivery record not translated into modern local AI-search authority</t>
+        </is>
+      </c>
+      <c r="Q220" s="4" t="inlineStr">
+        <is>
+          <t>Portfolio-driven AEO content: let 20 years of projects answer AI queries directly</t>
+        </is>
+      </c>
+      <c r="R220" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S220" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T220" s="4" t="inlineStr"/>
+    </row>
+    <row r="221">
+      <c r="A221" s="4" t="inlineStr">
+        <is>
+          <t>Browning Architects</t>
+        </is>
+      </c>
+      <c r="B221" s="4" t="inlineStr">
+        <is>
+          <t>Architects</t>
+        </is>
+      </c>
+      <c r="C221" s="4" t="inlineStr">
+        <is>
+          <t>Earlsfield, Wandsworth, London</t>
+        </is>
+      </c>
+      <c r="D221" s="4" t="inlineStr">
+        <is>
+          <t>via RIBA directory listing</t>
+        </is>
+      </c>
+      <c r="E221" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F221" s="4" t="inlineStr"/>
+      <c r="G221" s="4" t="inlineStr"/>
+      <c r="H221" s="4" t="inlineStr"/>
+      <c r="I221" s="4" t="inlineStr"/>
+      <c r="J221" s="4" t="inlineStr">
+        <is>
+          <t>Award-winning SW London practice, deep council/planning relationships in Wandsworth</t>
+        </is>
+      </c>
+      <c r="K221" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L221" s="4" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M221" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N221" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O221" s="4" t="inlineStr">
+        <is>
+          <t>Awards; planning-department relationships</t>
+        </is>
+      </c>
+      <c r="P221" s="4" t="inlineStr">
+        <is>
+          <t>Planning expertise is a strong differentiator invisible in generic architect searches</t>
+        </is>
+      </c>
+      <c r="Q221" s="4" t="inlineStr">
+        <is>
+          <t>'We know Wandsworth planning inside out' - own that exact AEO angle</t>
+        </is>
+      </c>
+      <c r="R221" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S221" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T221" s="4" t="inlineStr">
+        <is>
+          <t>Confirm live site before outreach</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T215"/>
+  <autoFilter ref="A1:T221"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -19080,7 +19600,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>214</v>
+        <v>220</v>
       </c>
     </row>
     <row r="5">
@@ -19103,31 +19623,31 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Private dentist</t>
+          <t>Architects</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Wedding venue</t>
+          <t>Private dentist</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Architects</t>
+          <t>Wedding venue</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10">
@@ -19143,7 +19663,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Estate &amp; letting agent</t>
+          <t>Physiotherapy clinic</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -19153,7 +19673,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Aesthetics clinic</t>
+          <t>Estate &amp; letting agent</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -19163,11 +19683,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Physiotherapy clinic</t>
+          <t>Aesthetics clinic</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
@@ -19213,17 +19733,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Law firm</t>
+          <t>Private dentist / implants</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Electrician</t>
+          <t>Law firm</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -19233,7 +19753,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Personal training studio</t>
+          <t>Electrician</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -19243,7 +19763,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Family law firm</t>
+          <t>Personal training studio</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -19253,7 +19773,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Recruitment agency</t>
+          <t>Family law firm</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -19263,7 +19783,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Immigration law firm</t>
+          <t>Recruitment agency</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -19273,17 +19793,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Letting agent</t>
+          <t>Immigration law firm</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Financial adviser / wealth management</t>
+          <t>Letting agent</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -19293,7 +19813,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Private tuition agency</t>
+          <t>Financial adviser / wealth management</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -19303,7 +19823,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Osteopathy clinic</t>
+          <t>Private tuition agency</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -19313,7 +19833,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Roofer</t>
+          <t>Osteopathy clinic</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -19323,7 +19843,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating / boilers</t>
+          <t>Roofer</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -19333,7 +19853,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Event &amp; wedding caterer</t>
+          <t>Plumbing &amp; heating / boilers</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -19343,7 +19863,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Chiropractor</t>
+          <t>Event &amp; wedding caterer</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -19353,7 +19873,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Estate agent (premium)</t>
+          <t>Chiropractor</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -19363,7 +19883,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Orthodontist</t>
+          <t>Estate agent (premium)</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -19373,7 +19893,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Employment law firm</t>
+          <t>Orthodontist</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -19383,7 +19903,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Event management agency</t>
+          <t>Employment law firm</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -19393,7 +19913,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Private dentist / implants</t>
+          <t>Event management agency</t>
         </is>
       </c>
       <c r="B36" t="n">

</xml_diff>

<commit_message>
Batch 12: +8 prospects (228 total) - opticians, Kent, North Somerset, dermatology
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$221</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$229</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T221"/>
+  <dimension ref="A1:T229"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -19568,8 +19568,692 @@
         </is>
       </c>
     </row>
+    <row r="222">
+      <c r="A222" s="3" t="inlineStr">
+        <is>
+          <t>Auerbach &amp; Steele</t>
+        </is>
+      </c>
+      <c r="B222" s="3" t="inlineStr">
+        <is>
+          <t>Independent optician</t>
+        </is>
+      </c>
+      <c r="C222" s="3" t="inlineStr">
+        <is>
+          <t>King's Road, Chelsea, London SW3</t>
+        </is>
+      </c>
+      <c r="D222" s="3" t="inlineStr">
+        <is>
+          <t>https://www.auerbach-steele.com</t>
+        </is>
+      </c>
+      <c r="E222" s="3" t="inlineStr">
+        <is>
+          <t>info@auerbach-steele.com</t>
+        </is>
+      </c>
+      <c r="F222" s="3" t="inlineStr">
+        <is>
+          <t>020 7349 0001</t>
+        </is>
+      </c>
+      <c r="G222" s="3" t="inlineStr">
+        <is>
+          <t>Gail Steele (Founder, est. 1996)</t>
+        </is>
+      </c>
+      <c r="H222" s="3" t="inlineStr"/>
+      <c r="I222" s="3" t="inlineStr"/>
+      <c r="J222" s="3" t="inlineStr">
+        <is>
+          <t>Premium design-led eyewear on King's Road since 1996; repeat prescription clients worth £300-1000+ per visit</t>
+        </is>
+      </c>
+      <c r="K222" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L222" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M222" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N222" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O222" s="3" t="inlineStr">
+        <is>
+          <t>Design-led branding; 28 years trading</t>
+        </is>
+      </c>
+      <c r="P222" s="3" t="inlineStr">
+        <is>
+          <t>Independent eyewear boutiques increasingly squeezed by Specsavers/Vision Express search dominance</t>
+        </is>
+      </c>
+      <c r="Q222" s="3" t="inlineStr">
+        <is>
+          <t>'Chelsea's design-literate opticians deserve to beat the chains in AI answers too'</t>
+        </is>
+      </c>
+      <c r="R222" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S222" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T222" s="3" t="inlineStr"/>
+    </row>
+    <row r="223">
+      <c r="A223" s="4" t="inlineStr">
+        <is>
+          <t>CULT VISION</t>
+        </is>
+      </c>
+      <c r="B223" s="4" t="inlineStr">
+        <is>
+          <t>Independent optician</t>
+        </is>
+      </c>
+      <c r="C223" s="4" t="inlineStr">
+        <is>
+          <t>Clerkenwell, London EC1</t>
+        </is>
+      </c>
+      <c r="D223" s="4" t="inlineStr">
+        <is>
+          <t>https://cultvision.com</t>
+        </is>
+      </c>
+      <c r="E223" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F223" s="4" t="inlineStr"/>
+      <c r="G223" s="4" t="inlineStr">
+        <is>
+          <t>Panos (Founder, 20+ years)</t>
+        </is>
+      </c>
+      <c r="H223" s="4" t="inlineStr"/>
+      <c r="I223" s="4" t="inlineStr"/>
+      <c r="J223" s="4" t="inlineStr">
+        <is>
+          <t>Curated independent-designer eyewear boutique; strong niche positioning against mass-market chains</t>
+        </is>
+      </c>
+      <c r="K223" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L223" s="4" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M223" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N223" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O223" s="4" t="inlineStr">
+        <is>
+          <t>Curated-brand positioning</t>
+        </is>
+      </c>
+      <c r="P223" s="4" t="inlineStr">
+        <is>
+          <t>Niche 'independent designer eyewear' story not yet the AI-cited Clerkenwell answer</t>
+        </is>
+      </c>
+      <c r="Q223" s="4" t="inlineStr">
+        <is>
+          <t>Own the AI answer for 'independent eyewear designer London' - genuinely defensible niche</t>
+        </is>
+      </c>
+      <c r="R223" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S223" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T223" s="4" t="inlineStr"/>
+    </row>
+    <row r="224">
+      <c r="A224" s="4" t="inlineStr">
+        <is>
+          <t>Aristone Optical</t>
+        </is>
+      </c>
+      <c r="B224" s="4" t="inlineStr">
+        <is>
+          <t>Independent optician</t>
+        </is>
+      </c>
+      <c r="C224" s="4" t="inlineStr">
+        <is>
+          <t>Fulham, London SW6</t>
+        </is>
+      </c>
+      <c r="D224" s="4" t="inlineStr">
+        <is>
+          <t>https://www.aristoneopticians.com</t>
+        </is>
+      </c>
+      <c r="E224" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F224" s="4" t="inlineStr"/>
+      <c r="G224" s="4" t="inlineStr"/>
+      <c r="H224" s="4" t="inlineStr"/>
+      <c r="I224" s="4" t="inlineStr"/>
+      <c r="J224" s="4" t="inlineStr">
+        <is>
+          <t>Family-run for 70 years - one of West London's most established independents; multi-generation trust</t>
+        </is>
+      </c>
+      <c r="K224" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L224" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M224" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N224" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O224" s="4" t="inlineStr">
+        <is>
+          <t>70-year heritage promoted</t>
+        </is>
+      </c>
+      <c r="P224" s="4" t="inlineStr">
+        <is>
+          <t>Heritage brand invisible against Specsavers/Boots Opticians in modern local search</t>
+        </is>
+      </c>
+      <c r="Q224" s="4" t="inlineStr">
+        <is>
+          <t>'70 years of Fulham trust - let's make AI recommend you, not just the high-street chains'</t>
+        </is>
+      </c>
+      <c r="R224" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S224" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T224" s="4" t="inlineStr"/>
+    </row>
+    <row r="225">
+      <c r="A225" s="3" t="inlineStr">
+        <is>
+          <t>Charles Bainbridge Estate Agents</t>
+        </is>
+      </c>
+      <c r="B225" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C225" s="3" t="inlineStr">
+        <is>
+          <t>Canterbury, Kent</t>
+        </is>
+      </c>
+      <c r="D225" s="3" t="inlineStr">
+        <is>
+          <t>https://www.charlesbainbridge.com</t>
+        </is>
+      </c>
+      <c r="E225" s="3" t="inlineStr">
+        <is>
+          <t>charlie@charlesbainbridge.com</t>
+        </is>
+      </c>
+      <c r="F225" s="3" t="inlineStr">
+        <is>
+          <t>01227 780 227</t>
+        </is>
+      </c>
+      <c r="G225" s="3" t="inlineStr">
+        <is>
+          <t>Andrea Dann (Founding team)</t>
+        </is>
+      </c>
+      <c r="H225" s="3" t="inlineStr"/>
+      <c r="I225" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/charlesbainbridgeea</t>
+        </is>
+      </c>
+      <c r="J225" s="3" t="inlineStr">
+        <is>
+          <t>Proudly independent family-run agency in Canterbury's premium period-home market; strong local reputation for integrity</t>
+        </is>
+      </c>
+      <c r="K225" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L225" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M225" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N225" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O225" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence</t>
+        </is>
+      </c>
+      <c r="P225" s="3" t="inlineStr">
+        <is>
+          <t>Wards/Fine &amp; Country corporate-scale rivals dominate Canterbury searches</t>
+        </is>
+      </c>
+      <c r="Q225" s="3" t="inlineStr">
+        <is>
+          <t>'Canterbury sellers value integrity - make sure AI recommends the independent, not just the network brand'</t>
+        </is>
+      </c>
+      <c r="R225" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S225" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T225" s="3" t="inlineStr"/>
+    </row>
+    <row r="226">
+      <c r="A226" s="3" t="inlineStr">
+        <is>
+          <t>Simon Miller &amp; Company</t>
+        </is>
+      </c>
+      <c r="B226" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C226" s="3" t="inlineStr">
+        <is>
+          <t>Maidstone &amp; the Weald, Kent</t>
+        </is>
+      </c>
+      <c r="D226" s="3" t="inlineStr">
+        <is>
+          <t>https://simonmiller.co.uk</t>
+        </is>
+      </c>
+      <c r="E226" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F226" s="3" t="inlineStr">
+        <is>
+          <t>01622 691 255</t>
+        </is>
+      </c>
+      <c r="G226" s="3" t="inlineStr"/>
+      <c r="H226" s="3" t="inlineStr"/>
+      <c r="I226" s="3" t="inlineStr"/>
+      <c r="J226" s="3" t="inlineStr">
+        <is>
+          <t>Truly independent, multi-office coverage of Maidstone/Malling/the Weald; strong local-knowledge positioning</t>
+        </is>
+      </c>
+      <c r="K226" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L226" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M226" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N226" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O226" s="3" t="inlineStr">
+        <is>
+          <t>Multi-office network</t>
+        </is>
+      </c>
+      <c r="P226" s="3" t="inlineStr">
+        <is>
+          <t>Independent claim not converted into AI-search dominance vs Wards/Foundation</t>
+        </is>
+      </c>
+      <c r="Q226" s="3" t="inlineStr">
+        <is>
+          <t>'Truly independent' as the exact AEO positioning to own in Kent property search</t>
+        </is>
+      </c>
+      <c r="R226" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S226" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T226" s="3" t="inlineStr"/>
+    </row>
+    <row r="227">
+      <c r="A227" s="3" t="inlineStr">
+        <is>
+          <t>Heritage Estate Agents</t>
+        </is>
+      </c>
+      <c r="B227" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C227" s="3" t="inlineStr">
+        <is>
+          <t>Portishead, Nailsea, Clevedon, Yatton (North Somerset)</t>
+        </is>
+      </c>
+      <c r="D227" s="3" t="inlineStr">
+        <is>
+          <t>https://heritage4homes.co.uk</t>
+        </is>
+      </c>
+      <c r="E227" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F227" s="3" t="inlineStr">
+        <is>
+          <t>01275 840 610</t>
+        </is>
+      </c>
+      <c r="G227" s="3" t="inlineStr"/>
+      <c r="H227" s="3" t="inlineStr"/>
+      <c r="I227" s="3" t="inlineStr"/>
+      <c r="J227" s="3" t="inlineStr">
+        <is>
+          <t>North Somerset's largest independent, 5-town coverage; steady commuter-belt Bristol demand</t>
+        </is>
+      </c>
+      <c r="K227" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L227" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M227" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N227" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O227" s="3" t="inlineStr">
+        <is>
+          <t>Multi-office coverage</t>
+        </is>
+      </c>
+      <c r="P227" s="3" t="inlineStr">
+        <is>
+          <t>Largest independent claim not leveraged as AI-search trust signal across all 5 towns</t>
+        </is>
+      </c>
+      <c r="Q227" s="3" t="inlineStr">
+        <is>
+          <t>'Largest independent in North Somerset - own that claim in every AI answer, not just the tagline'</t>
+        </is>
+      </c>
+      <c r="R227" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S227" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T227" s="3" t="inlineStr"/>
+    </row>
+    <row r="228">
+      <c r="A228" s="4" t="inlineStr">
+        <is>
+          <t>Westcoast Properties</t>
+        </is>
+      </c>
+      <c r="B228" s="4" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C228" s="4" t="inlineStr">
+        <is>
+          <t>Weston-super-Mare, Portishead, Nailsea, Patchway (North Somerset/Bristol)</t>
+        </is>
+      </c>
+      <c r="D228" s="4" t="inlineStr">
+        <is>
+          <t>https://www.westcoast-properties.co.uk</t>
+        </is>
+      </c>
+      <c r="E228" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F228" s="4" t="inlineStr"/>
+      <c r="G228" s="4" t="inlineStr"/>
+      <c r="H228" s="4" t="inlineStr"/>
+      <c r="I228" s="4" t="inlineStr"/>
+      <c r="J228" s="4" t="inlineStr">
+        <is>
+          <t>Independent since 1995, 4-office North Somerset/North Bristol coverage; 30 years trading</t>
+        </is>
+      </c>
+      <c r="K228" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L228" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M228" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N228" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O228" s="4" t="inlineStr">
+        <is>
+          <t>Multi-office established brand</t>
+        </is>
+      </c>
+      <c r="P228" s="4" t="inlineStr">
+        <is>
+          <t>30-year trading history under-leveraged for search trust vs Heritage/Connells</t>
+        </is>
+      </c>
+      <c r="Q228" s="4" t="inlineStr">
+        <is>
+          <t>Turn 3 decades of trading into the AI-cited local-authority answer</t>
+        </is>
+      </c>
+      <c r="R228" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S228" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T228" s="4" t="inlineStr"/>
+    </row>
+    <row r="229">
+      <c r="A229" s="3" t="inlineStr">
+        <is>
+          <t>London Dermatology Centre</t>
+        </is>
+      </c>
+      <c r="B229" s="3" t="inlineStr">
+        <is>
+          <t>Dermatology clinic</t>
+        </is>
+      </c>
+      <c r="C229" s="3" t="inlineStr">
+        <is>
+          <t>Wimpole Street, London W1</t>
+        </is>
+      </c>
+      <c r="D229" s="3" t="inlineStr">
+        <is>
+          <t>https://www.london-dermatology-centre.co.uk</t>
+        </is>
+      </c>
+      <c r="E229" s="3" t="inlineStr">
+        <is>
+          <t>reception@the-dermatology-centre.co.uk</t>
+        </is>
+      </c>
+      <c r="F229" s="3" t="inlineStr">
+        <is>
+          <t>020 7467 3720</t>
+        </is>
+      </c>
+      <c r="G229" s="3" t="inlineStr">
+        <is>
+          <t>Dr Sunil Chopra (Founder &amp; Clinical Director, est. 2005)</t>
+        </is>
+      </c>
+      <c r="H229" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/drsunilchopra</t>
+        </is>
+      </c>
+      <c r="I229" s="3" t="inlineStr"/>
+      <c r="J229" s="3" t="inlineStr">
+        <is>
+          <t>20-year-established consultant dermatology clinic; skin cancer/acne/rosacea cases worth £200-500+ per consultation with repeat visits</t>
+        </is>
+      </c>
+      <c r="K229" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L229" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M229" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N229" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O229" s="3" t="inlineStr">
+        <is>
+          <t>Doctify reviews; established brand</t>
+        </is>
+      </c>
+      <c r="P229" s="3" t="inlineStr">
+        <is>
+          <t>Newer, more aggressively-marketed dermatology brands (Skin55, Eudelo) may be winning AI-search share from established players</t>
+        </is>
+      </c>
+      <c r="Q229" s="3" t="inlineStr">
+        <is>
+          <t>'20 years of consultant-level expertise - make sure that outranks newer, flashier competitors in AI answers too'</t>
+        </is>
+      </c>
+      <c r="R229" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S229" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T229" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T221"/>
+  <autoFilter ref="A1:T229"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -19580,7 +20264,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B103"/>
+  <dimension ref="A1:B105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -19600,7 +20284,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>220</v>
+        <v>228</v>
       </c>
     </row>
     <row r="5">
@@ -19617,7 +20301,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7">
@@ -19803,17 +20487,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Letting agent</t>
+          <t>Independent optician</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Financial adviser / wealth management</t>
+          <t>Letting agent</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -19823,7 +20507,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Private tuition agency</t>
+          <t>Financial adviser / wealth management</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -19833,7 +20517,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Osteopathy clinic</t>
+          <t>Private tuition agency</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -19843,7 +20527,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Roofer</t>
+          <t>Osteopathy clinic</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -19853,7 +20537,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating / boilers</t>
+          <t>Roofer</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -19863,7 +20547,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Event &amp; wedding caterer</t>
+          <t>Plumbing &amp; heating / boilers</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -19873,7 +20557,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Chiropractor</t>
+          <t>Event &amp; wedding caterer</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -19883,7 +20567,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Estate agent (premium)</t>
+          <t>Chiropractor</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -19893,7 +20577,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Orthodontist</t>
+          <t>Estate agent (premium)</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -19903,7 +20587,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Employment law firm</t>
+          <t>Orthodontist</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -19913,7 +20597,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Event management agency</t>
+          <t>Employment law firm</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -19923,7 +20607,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Design &amp; build</t>
+          <t>Event management agency</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -19933,7 +20617,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>IT support / MSP</t>
+          <t>Design &amp; build</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -19943,17 +20627,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Dentist / Orthodontics</t>
+          <t>IT support / MSP</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Specialist dental/implant clinic</t>
+          <t>Dentist / Orthodontics</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -19963,7 +20647,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Boutique corporate law firm</t>
+          <t>Specialist dental/implant clinic</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -19973,7 +20657,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Cosmetic/aesthetics clinic</t>
+          <t>Boutique corporate law firm</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -19983,7 +20667,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Skin &amp; laser clinic</t>
+          <t>Cosmetic/aesthetics clinic</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -19993,7 +20677,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Mortgage broker / financial adviser</t>
+          <t>Skin &amp; laser clinic</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -20003,7 +20687,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Architects (RIBA chartered)</t>
+          <t>Mortgage broker / financial adviser</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -20013,7 +20697,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Recruitment agency (tech/startups)</t>
+          <t>Architects (RIBA chartered)</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -20023,7 +20707,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Recruitment agency (IT/data)</t>
+          <t>Recruitment agency (tech/startups)</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -20033,7 +20717,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Independent vet (24/7 emergency)</t>
+          <t>Recruitment agency (IT/data)</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -20043,7 +20727,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Interior design studio</t>
+          <t>Independent vet (24/7 emergency)</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -20053,7 +20737,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Letting &amp; estate agent</t>
+          <t>Interior design studio</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -20063,7 +20747,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Cosmetic clinic (injectables)</t>
+          <t>Letting &amp; estate agent</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -20073,7 +20757,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Cosmetic/anti-ageing clinic</t>
+          <t>Cosmetic clinic (injectables)</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -20083,7 +20767,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Yoga &amp; reformer pilates studio</t>
+          <t>Cosmetic/anti-ageing clinic</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -20093,7 +20777,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Reformer pilates studio</t>
+          <t>Yoga &amp; reformer pilates studio</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -20103,7 +20787,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Wealth management</t>
+          <t>Reformer pilates studio</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -20113,7 +20797,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Private tuition &amp; education consultancy</t>
+          <t>Wealth management</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -20123,7 +20807,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Osteopath</t>
+          <t>Private tuition &amp; education consultancy</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -20133,7 +20817,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Design &amp; build / home renovation</t>
+          <t>Osteopath</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -20143,7 +20827,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Builders / building contractor</t>
+          <t>Design &amp; build / home renovation</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -20153,7 +20837,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Home care / live-in care</t>
+          <t>Builders / building contractor</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -20163,7 +20847,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Private day nurseries</t>
+          <t>Home care / live-in care</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -20173,7 +20857,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Personal training &amp; wellness studio</t>
+          <t>Private day nurseries</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -20183,7 +20867,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Mortgage &amp; insurance broker</t>
+          <t>Personal training &amp; wellness studio</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -20193,7 +20877,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Business consultancy</t>
+          <t>Mortgage &amp; insurance broker</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -20203,7 +20887,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Interior designer (period homes)</t>
+          <t>Business consultancy</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -20213,7 +20897,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Landscape design &amp; build</t>
+          <t>Interior designer (period homes)</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -20223,7 +20907,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Interior designer</t>
+          <t>Landscape design &amp; build</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -20233,7 +20917,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Garden design &amp; landscaping</t>
+          <t>Interior designer</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -20243,7 +20927,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Legal recruitment</t>
+          <t>Garden design &amp; landscaping</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -20253,7 +20937,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Independent gym &amp; health club</t>
+          <t>Legal recruitment</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -20263,7 +20947,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Independent gym</t>
+          <t>Independent gym &amp; health club</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -20273,7 +20957,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Physiotherapy (sports)</t>
+          <t>Independent gym</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -20283,7 +20967,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Letting agent / property management</t>
+          <t>Physiotherapy (sports)</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -20293,7 +20977,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Skin clinic</t>
+          <t>Letting agent / property management</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -20303,7 +20987,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Tutoring company</t>
+          <t>Skin clinic</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -20313,7 +20997,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Tutorial college &amp; exam centre</t>
+          <t>Tutoring company</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -20323,7 +21007,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Employment law (disability discrimination)</t>
+          <t>Tutorial college &amp; exam centre</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -20333,7 +21017,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating</t>
+          <t>Employment law (disability discrimination)</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -20343,7 +21027,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Plumbing &amp; heating</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -20353,7 +21037,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Sports physio &amp; massage</t>
+          <t>Plumbing</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -20363,7 +21047,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Chartered surveyors (party wall/building)</t>
+          <t>Sports physio &amp; massage</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -20373,7 +21057,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Chartered surveyors</t>
+          <t>Chartered surveyors (party wall/building)</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -20383,7 +21067,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Chartered building surveyors</t>
+          <t>Chartered surveyors</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -20393,7 +21077,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Osteopathy clinics</t>
+          <t>Chartered building surveyors</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -20403,7 +21087,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Builders / renovations</t>
+          <t>Osteopathy clinics</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -20413,7 +21097,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Private nursery schools</t>
+          <t>Builders / renovations</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -20423,7 +21107,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Private day nursery</t>
+          <t>Private nursery schools</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -20433,7 +21117,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Private GP (membership model)</t>
+          <t>Private day nursery</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -20443,7 +21127,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Sash window restoration</t>
+          <t>Private GP (membership model)</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -20453,7 +21137,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Personal training (1:1)</t>
+          <t>Sash window restoration</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -20463,7 +21147,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Personal training &amp; nutrition coaching</t>
+          <t>Personal training (1:1)</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -20473,7 +21157,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Private nursery/pre-prep school</t>
+          <t>Personal training &amp; nutrition coaching</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -20483,7 +21167,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Independent nursery (Montessori)</t>
+          <t>Private nursery/pre-prep school</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -20493,7 +21177,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Live-in care agency</t>
+          <t>Independent nursery (Montessori)</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -20503,7 +21187,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Law firm (conveyancing/family)</t>
+          <t>Live-in care agency</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -20513,7 +21197,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Architect &amp; interior designer</t>
+          <t>Law firm (conveyancing/family)</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -20523,7 +21207,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Architects / project management</t>
+          <t>Architect &amp; interior designer</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -20533,7 +21217,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>IFA / wealth management</t>
+          <t>Architects / project management</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -20543,7 +21227,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Physiotherapy &amp; clinical Pilates</t>
+          <t>IFA / wealth management</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -20553,7 +21237,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Aesthetics &amp; skin clinic</t>
+          <t>Physiotherapy &amp; clinical Pilates</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -20563,7 +21247,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Wealth management / IFA</t>
+          <t>Aesthetics &amp; skin clinic</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -20573,7 +21257,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>IFA / financial planning</t>
+          <t>Wealth management / IFA</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -20583,10 +21267,30 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
+          <t>IFA / financial planning</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
           <t>Wealth management &amp; employee benefits</t>
         </is>
       </c>
-      <c r="B103" t="n">
+      <c r="B104" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Dermatology clinic</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 13: +7 prospects (235 total) - Primrose Hill, St John's Wood, South Kensington, Surrey pilates
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$229</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$236</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T229"/>
+  <dimension ref="A1:T236"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -20252,8 +20252,616 @@
       </c>
       <c r="T229" s="3" t="inlineStr"/>
     </row>
+    <row r="230">
+      <c r="A230" s="3" t="inlineStr">
+        <is>
+          <t>Jeremy Bass Estate Agents</t>
+        </is>
+      </c>
+      <c r="B230" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C230" s="3" t="inlineStr">
+        <is>
+          <t>Primrose Hill, London NW1</t>
+        </is>
+      </c>
+      <c r="D230" s="3" t="inlineStr">
+        <is>
+          <t>https://www.jeremybass.co.uk</t>
+        </is>
+      </c>
+      <c r="E230" s="3" t="inlineStr">
+        <is>
+          <t>info@jeremybass.co.uk</t>
+        </is>
+      </c>
+      <c r="F230" s="3" t="inlineStr">
+        <is>
+          <t>020 7722 8686</t>
+        </is>
+      </c>
+      <c r="G230" s="3" t="inlineStr">
+        <is>
+          <t>Jeremy Bass (Founder &amp; Director, est. 2000)</t>
+        </is>
+      </c>
+      <c r="H230" s="3" t="inlineStr"/>
+      <c r="I230" s="3" t="inlineStr"/>
+      <c r="J230" s="3" t="inlineStr">
+        <is>
+          <t>Independent since 2000 in ultra-premium Primrose Hill village; founder personally known in the area for 30+ years</t>
+        </is>
+      </c>
+      <c r="K230" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L230" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M230" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N230" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O230" s="3" t="inlineStr">
+        <is>
+          <t>Local press interviews (I Love Primrose Hill blog)</t>
+        </is>
+      </c>
+      <c r="P230" s="3" t="inlineStr">
+        <is>
+          <t>Corporate giants (John D Wood, Knight Frank) also operate in Primrose Hill and outspend on digital</t>
+        </is>
+      </c>
+      <c r="Q230" s="3" t="inlineStr">
+        <is>
+          <t>'Primrose Hill's own agent for 25 years - make sure AI says his name, not just the corporates'</t>
+        </is>
+      </c>
+      <c r="R230" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S230" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T230" s="3" t="inlineStr"/>
+    </row>
+    <row r="231">
+      <c r="A231" s="3" t="inlineStr">
+        <is>
+          <t>Laurence Leigh</t>
+        </is>
+      </c>
+      <c r="B231" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C231" s="3" t="inlineStr">
+        <is>
+          <t>St John's Wood, Maida Vale, Regent's Park, Primrose Hill, Hampstead</t>
+        </is>
+      </c>
+      <c r="D231" s="3" t="inlineStr">
+        <is>
+          <t>https://laurenceleigh.com</t>
+        </is>
+      </c>
+      <c r="E231" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F231" s="3" t="inlineStr"/>
+      <c r="G231" s="3" t="inlineStr"/>
+      <c r="H231" s="3" t="inlineStr"/>
+      <c r="I231" s="3" t="inlineStr"/>
+      <c r="J231" s="3" t="inlineStr">
+        <is>
+          <t>Independent, 50+ years combined team experience across 5 of London's wealthiest villages</t>
+        </is>
+      </c>
+      <c r="K231" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L231" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M231" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N231" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O231" s="3" t="inlineStr">
+        <is>
+          <t>Multi-village coverage claim</t>
+        </is>
+      </c>
+      <c r="P231" s="3" t="inlineStr">
+        <is>
+          <t>Broad coverage claim not matched by dominant per-village search visibility</t>
+        </is>
+      </c>
+      <c r="Q231" s="3" t="inlineStr">
+        <is>
+          <t>Per-village AEO content to actually own all 5 areas claimed</t>
+        </is>
+      </c>
+      <c r="R231" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S231" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T231" s="3" t="inlineStr"/>
+    </row>
+    <row r="232">
+      <c r="A232" s="3" t="inlineStr">
+        <is>
+          <t>McKee &amp; Co</t>
+        </is>
+      </c>
+      <c r="B232" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C232" s="3" t="inlineStr">
+        <is>
+          <t>South Kensington, London SW7</t>
+        </is>
+      </c>
+      <c r="D232" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mckee.co.uk</t>
+        </is>
+      </c>
+      <c r="E232" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F232" s="3" t="inlineStr">
+        <is>
+          <t>020 8022 7161</t>
+        </is>
+      </c>
+      <c r="G232" s="3" t="inlineStr">
+        <is>
+          <t>David McKee (2nd generation, family firm since 1979)</t>
+        </is>
+      </c>
+      <c r="H232" s="3" t="inlineStr"/>
+      <c r="I232" s="3" t="inlineStr"/>
+      <c r="J232" s="3" t="inlineStr">
+        <is>
+          <t>45+ year independent niche agency in Prime Central London; family firm with deep multi-generation local knowledge</t>
+        </is>
+      </c>
+      <c r="K232" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L232" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M232" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N232" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O232" s="3" t="inlineStr">
+        <is>
+          <t>Area-guide content (South Kensington/Kensington guides)</t>
+        </is>
+      </c>
+      <c r="P232" s="3" t="inlineStr">
+        <is>
+          <t>Area guides exist but Knight Frank/Strutt &amp; Parker corporate scale dominates PCL search</t>
+        </is>
+      </c>
+      <c r="Q232" s="3" t="inlineStr">
+        <is>
+          <t>'Second-generation local knowledge vs corporate scale - AEO is the equaliser'</t>
+        </is>
+      </c>
+      <c r="R232" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S232" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T232" s="3" t="inlineStr"/>
+    </row>
+    <row r="233">
+      <c r="A233" s="4" t="inlineStr">
+        <is>
+          <t>Pilates Hub Weybridge</t>
+        </is>
+      </c>
+      <c r="B233" s="4" t="inlineStr">
+        <is>
+          <t>Pilates studio</t>
+        </is>
+      </c>
+      <c r="C233" s="4" t="inlineStr">
+        <is>
+          <t>Queens Rd, Weybridge, Surrey</t>
+        </is>
+      </c>
+      <c r="D233" s="4" t="inlineStr">
+        <is>
+          <t>https://www.pilateshubweybridge.co.uk</t>
+        </is>
+      </c>
+      <c r="E233" s="4" t="inlineStr">
+        <is>
+          <t>info@pilateshubweybridge.co.uk</t>
+        </is>
+      </c>
+      <c r="F233" s="4" t="inlineStr">
+        <is>
+          <t>07961 740302</t>
+        </is>
+      </c>
+      <c r="G233" s="4" t="inlineStr">
+        <is>
+          <t>Sara Noon (Founder &amp; Director)</t>
+        </is>
+      </c>
+      <c r="H233" s="4" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/sara-noon-61066253</t>
+        </is>
+      </c>
+      <c r="I233" s="4" t="inlineStr">
+        <is>
+          <t>instagram.com/pilates_hub_weybridge</t>
+        </is>
+      </c>
+      <c r="J233" s="4" t="inlineStr">
+        <is>
+          <t>Founder-led boutique studio in affluent Weybridge; memberships + 1:1 sessions = strong recurring revenue per client</t>
+        </is>
+      </c>
+      <c r="K233" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L233" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M233" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N233" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O233" s="4" t="inlineStr">
+        <is>
+          <t>Active Instagram; Mindbody/Wellhub listings</t>
+        </is>
+      </c>
+      <c r="P233" s="4" t="inlineStr">
+        <is>
+          <t>Discovery via booking platforms (Mindbody) means paying commission on the studio's own clients</t>
+        </is>
+      </c>
+      <c r="Q233" s="4" t="inlineStr">
+        <is>
+          <t>'Stop paying Mindbody for leads you could own directly via local + AI search'</t>
+        </is>
+      </c>
+      <c r="R233" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S233" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T233" s="4" t="inlineStr"/>
+    </row>
+    <row r="234">
+      <c r="A234" s="4" t="inlineStr">
+        <is>
+          <t>Guildford Pilates Place</t>
+        </is>
+      </c>
+      <c r="B234" s="4" t="inlineStr">
+        <is>
+          <t>Pilates studio</t>
+        </is>
+      </c>
+      <c r="C234" s="4" t="inlineStr">
+        <is>
+          <t>High Street, Guildford, Surrey</t>
+        </is>
+      </c>
+      <c r="D234" s="4" t="inlineStr">
+        <is>
+          <t>https://guildfordpilatesplace.co.uk</t>
+        </is>
+      </c>
+      <c r="E234" s="4" t="inlineStr">
+        <is>
+          <t>pilates@guildfordpilatesplace.co.uk</t>
+        </is>
+      </c>
+      <c r="F234" s="4" t="inlineStr">
+        <is>
+          <t>01483 506 113</t>
+        </is>
+      </c>
+      <c r="G234" s="4" t="inlineStr"/>
+      <c r="H234" s="4" t="inlineStr"/>
+      <c r="I234" s="4" t="inlineStr">
+        <is>
+          <t>instagram.com/guildfordpilates</t>
+        </is>
+      </c>
+      <c r="J234" s="4" t="inlineStr">
+        <is>
+          <t>Guildford's original dedicated Pilates studio since 2010 - first-mover positioning in the town centre</t>
+        </is>
+      </c>
+      <c r="K234" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L234" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M234" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N234" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O234" s="4" t="inlineStr">
+        <is>
+          <t>Instagram presence; Mindbody listing</t>
+        </is>
+      </c>
+      <c r="P234" s="4" t="inlineStr">
+        <is>
+          <t>'Original' claim undefended in local search against newer entrants (HiP Studio, The Pilates Movement)</t>
+        </is>
+      </c>
+      <c r="Q234" s="4" t="inlineStr">
+        <is>
+          <t>'Guildford's original Pilates studio' - own that exact AEO positioning before newer rivals claim it</t>
+        </is>
+      </c>
+      <c r="R234" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S234" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T234" s="4" t="inlineStr"/>
+    </row>
+    <row r="235">
+      <c r="A235" s="4" t="inlineStr">
+        <is>
+          <t>HiP Studio</t>
+        </is>
+      </c>
+      <c r="B235" s="4" t="inlineStr">
+        <is>
+          <t>Pilates studio</t>
+        </is>
+      </c>
+      <c r="C235" s="4" t="inlineStr">
+        <is>
+          <t>Shalford, Guildford, Surrey</t>
+        </is>
+      </c>
+      <c r="D235" s="4" t="inlineStr">
+        <is>
+          <t>https://www.hipstudio.co.uk</t>
+        </is>
+      </c>
+      <c r="E235" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F235" s="4" t="inlineStr"/>
+      <c r="G235" s="4" t="inlineStr"/>
+      <c r="H235" s="4" t="inlineStr"/>
+      <c r="I235" s="4" t="inlineStr"/>
+      <c r="J235" s="4" t="inlineStr">
+        <is>
+          <t>Boutique reformer studio with premium STOTT equipment in Shalford village near Guildford</t>
+        </is>
+      </c>
+      <c r="K235" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L235" s="4" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M235" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N235" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O235" s="4" t="inlineStr">
+        <is>
+          <t>Premium equipment branding</t>
+        </is>
+      </c>
+      <c r="P235" s="4" t="inlineStr">
+        <is>
+          <t>Boutique/premium positioning invisible against bigger Guildford studios in search</t>
+        </is>
+      </c>
+      <c r="Q235" s="4" t="inlineStr">
+        <is>
+          <t>Own 'STOTT reformer Guildford' - equipment-brand AEO niche nobody else claims</t>
+        </is>
+      </c>
+      <c r="R235" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S235" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T235" s="4" t="inlineStr"/>
+    </row>
+    <row r="236">
+      <c r="A236" s="3" t="inlineStr">
+        <is>
+          <t>The Pilates Movement</t>
+        </is>
+      </c>
+      <c r="B236" s="3" t="inlineStr">
+        <is>
+          <t>Pilates studio (multi-site)</t>
+        </is>
+      </c>
+      <c r="C236" s="3" t="inlineStr">
+        <is>
+          <t>4 studios across Surrey incl. Guildford</t>
+        </is>
+      </c>
+      <c r="D236" s="3" t="inlineStr">
+        <is>
+          <t>https://thepilatesmovementstudio.co.uk</t>
+        </is>
+      </c>
+      <c r="E236" s="3" t="inlineStr">
+        <is>
+          <t>guildford@thepilatesmovementstudio.co.uk</t>
+        </is>
+      </c>
+      <c r="F236" s="3" t="inlineStr">
+        <is>
+          <t>01483 399 149</t>
+        </is>
+      </c>
+      <c r="G236" s="3" t="inlineStr">
+        <is>
+          <t>Jeff &amp; Jane (Founders, husband &amp; wife)</t>
+        </is>
+      </c>
+      <c r="H236" s="3" t="inlineStr"/>
+      <c r="I236" s="3" t="inlineStr"/>
+      <c r="J236" s="3" t="inlineStr">
+        <is>
+          <t>4-studio Surrey group; couple-founded; multi-site scale gives real cross-sell/membership revenue</t>
+        </is>
+      </c>
+      <c r="K236" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L236" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M236" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N236" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O236" s="3" t="inlineStr">
+        <is>
+          <t>Per-studio booking pages = active marketing</t>
+        </is>
+      </c>
+      <c r="P236" s="3" t="inlineStr">
+        <is>
+          <t>4 studios but not yet 4x the search dominance in each catchment</t>
+        </is>
+      </c>
+      <c r="Q236" s="3" t="inlineStr">
+        <is>
+          <t>Per-studio local SEO + AEO push to match the scale they've already built</t>
+        </is>
+      </c>
+      <c r="R236" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S236" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T236" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T229"/>
+  <autoFilter ref="A1:T236"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -20264,7 +20872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B105"/>
+  <dimension ref="A1:B107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -20284,7 +20892,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>228</v>
+        <v>235</v>
       </c>
     </row>
     <row r="5">
@@ -20301,7 +20909,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7">
@@ -20497,17 +21105,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Letting agent</t>
+          <t>Pilates studio</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Financial adviser / wealth management</t>
+          <t>Letting agent</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -20517,7 +21125,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Private tuition agency</t>
+          <t>Financial adviser / wealth management</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -20527,7 +21135,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Osteopathy clinic</t>
+          <t>Private tuition agency</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -20537,7 +21145,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Roofer</t>
+          <t>Osteopathy clinic</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -20547,7 +21155,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating / boilers</t>
+          <t>Roofer</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -20557,7 +21165,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Event &amp; wedding caterer</t>
+          <t>Plumbing &amp; heating / boilers</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -20567,7 +21175,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Chiropractor</t>
+          <t>Event &amp; wedding caterer</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -20577,7 +21185,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Estate agent (premium)</t>
+          <t>Chiropractor</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -20587,7 +21195,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Orthodontist</t>
+          <t>Estate agent (premium)</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -20597,7 +21205,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Employment law firm</t>
+          <t>Orthodontist</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -20607,7 +21215,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Event management agency</t>
+          <t>Employment law firm</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -20617,7 +21225,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Design &amp; build</t>
+          <t>Event management agency</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -20627,7 +21235,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>IT support / MSP</t>
+          <t>Design &amp; build</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -20637,17 +21245,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Dentist / Orthodontics</t>
+          <t>IT support / MSP</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Specialist dental/implant clinic</t>
+          <t>Dentist / Orthodontics</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -20657,7 +21265,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Boutique corporate law firm</t>
+          <t>Specialist dental/implant clinic</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -20667,7 +21275,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Cosmetic/aesthetics clinic</t>
+          <t>Boutique corporate law firm</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -20677,7 +21285,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Skin &amp; laser clinic</t>
+          <t>Cosmetic/aesthetics clinic</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -20687,7 +21295,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Mortgage broker / financial adviser</t>
+          <t>Skin &amp; laser clinic</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -20697,7 +21305,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Architects (RIBA chartered)</t>
+          <t>Mortgage broker / financial adviser</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -20707,7 +21315,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Recruitment agency (tech/startups)</t>
+          <t>Architects (RIBA chartered)</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -20717,7 +21325,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Recruitment agency (IT/data)</t>
+          <t>Recruitment agency (tech/startups)</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -20727,7 +21335,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Independent vet (24/7 emergency)</t>
+          <t>Recruitment agency (IT/data)</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -20737,7 +21345,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Interior design studio</t>
+          <t>Independent vet (24/7 emergency)</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -20747,7 +21355,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Letting &amp; estate agent</t>
+          <t>Interior design studio</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -20757,7 +21365,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Cosmetic clinic (injectables)</t>
+          <t>Letting &amp; estate agent</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -20767,7 +21375,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Cosmetic/anti-ageing clinic</t>
+          <t>Cosmetic clinic (injectables)</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -20777,7 +21385,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Yoga &amp; reformer pilates studio</t>
+          <t>Cosmetic/anti-ageing clinic</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -20787,7 +21395,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Reformer pilates studio</t>
+          <t>Yoga &amp; reformer pilates studio</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -20797,7 +21405,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Wealth management</t>
+          <t>Reformer pilates studio</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -20807,7 +21415,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Private tuition &amp; education consultancy</t>
+          <t>Wealth management</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -20817,7 +21425,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Osteopath</t>
+          <t>Private tuition &amp; education consultancy</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -20827,7 +21435,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Design &amp; build / home renovation</t>
+          <t>Osteopath</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -20837,7 +21445,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Builders / building contractor</t>
+          <t>Design &amp; build / home renovation</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -20847,7 +21455,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Home care / live-in care</t>
+          <t>Builders / building contractor</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -20857,7 +21465,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Private day nurseries</t>
+          <t>Home care / live-in care</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -20867,7 +21475,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Personal training &amp; wellness studio</t>
+          <t>Private day nurseries</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -20877,7 +21485,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Mortgage &amp; insurance broker</t>
+          <t>Personal training &amp; wellness studio</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -20887,7 +21495,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Business consultancy</t>
+          <t>Mortgage &amp; insurance broker</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -20897,7 +21505,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Interior designer (period homes)</t>
+          <t>Business consultancy</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -20907,7 +21515,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Landscape design &amp; build</t>
+          <t>Interior designer (period homes)</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -20917,7 +21525,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Interior designer</t>
+          <t>Landscape design &amp; build</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -20927,7 +21535,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Garden design &amp; landscaping</t>
+          <t>Interior designer</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -20937,7 +21545,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Legal recruitment</t>
+          <t>Garden design &amp; landscaping</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -20947,7 +21555,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Independent gym &amp; health club</t>
+          <t>Legal recruitment</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -20957,7 +21565,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Independent gym</t>
+          <t>Independent gym &amp; health club</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -20967,7 +21575,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Physiotherapy (sports)</t>
+          <t>Independent gym</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -20977,7 +21585,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Letting agent / property management</t>
+          <t>Physiotherapy (sports)</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -20987,7 +21595,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Skin clinic</t>
+          <t>Letting agent / property management</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -20997,7 +21605,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Tutoring company</t>
+          <t>Skin clinic</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -21007,7 +21615,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Tutorial college &amp; exam centre</t>
+          <t>Tutoring company</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -21017,7 +21625,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Employment law (disability discrimination)</t>
+          <t>Tutorial college &amp; exam centre</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -21027,7 +21635,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating</t>
+          <t>Employment law (disability discrimination)</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -21037,7 +21645,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Plumbing &amp; heating</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -21047,7 +21655,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Sports physio &amp; massage</t>
+          <t>Plumbing</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -21057,7 +21665,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Chartered surveyors (party wall/building)</t>
+          <t>Sports physio &amp; massage</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -21067,7 +21675,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Chartered surveyors</t>
+          <t>Chartered surveyors (party wall/building)</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -21077,7 +21685,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Chartered building surveyors</t>
+          <t>Chartered surveyors</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -21087,7 +21695,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Osteopathy clinics</t>
+          <t>Chartered building surveyors</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -21097,7 +21705,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Builders / renovations</t>
+          <t>Osteopathy clinics</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -21107,7 +21715,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Private nursery schools</t>
+          <t>Builders / renovations</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -21117,7 +21725,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Private day nursery</t>
+          <t>Private nursery schools</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -21127,7 +21735,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Private GP (membership model)</t>
+          <t>Private day nursery</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -21137,7 +21745,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Sash window restoration</t>
+          <t>Private GP (membership model)</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -21147,7 +21755,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Personal training (1:1)</t>
+          <t>Sash window restoration</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -21157,7 +21765,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Personal training &amp; nutrition coaching</t>
+          <t>Personal training (1:1)</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -21167,7 +21775,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Private nursery/pre-prep school</t>
+          <t>Personal training &amp; nutrition coaching</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -21177,7 +21785,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Independent nursery (Montessori)</t>
+          <t>Private nursery/pre-prep school</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -21187,7 +21795,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Live-in care agency</t>
+          <t>Independent nursery (Montessori)</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -21197,7 +21805,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Law firm (conveyancing/family)</t>
+          <t>Live-in care agency</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -21207,7 +21815,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Architect &amp; interior designer</t>
+          <t>Law firm (conveyancing/family)</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -21217,7 +21825,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Architects / project management</t>
+          <t>Architect &amp; interior designer</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -21227,7 +21835,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>IFA / wealth management</t>
+          <t>Architects / project management</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -21237,7 +21845,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Physiotherapy &amp; clinical Pilates</t>
+          <t>IFA / wealth management</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -21247,7 +21855,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Aesthetics &amp; skin clinic</t>
+          <t>Physiotherapy &amp; clinical Pilates</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -21257,7 +21865,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Wealth management / IFA</t>
+          <t>Aesthetics &amp; skin clinic</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -21267,7 +21875,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>IFA / financial planning</t>
+          <t>Wealth management / IFA</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -21277,7 +21885,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Wealth management &amp; employee benefits</t>
+          <t>IFA / financial planning</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -21287,10 +21895,30 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
+          <t>Wealth management &amp; employee benefits</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
           <t>Dermatology clinic</t>
         </is>
       </c>
-      <c r="B105" t="n">
+      <c r="B106" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Pilates studio (multi-site)</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 14: +6 prospects (241 total) - Guildford nursery/IT, East London probate, Surrey consulting
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$236</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$242</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T236"/>
+  <dimension ref="A1:T242"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -20860,8 +20860,520 @@
       </c>
       <c r="T236" s="3" t="inlineStr"/>
     </row>
+    <row r="237">
+      <c r="A237" s="3" t="inlineStr">
+        <is>
+          <t>Christopher Robin Day Nurseries</t>
+        </is>
+      </c>
+      <c r="B237" s="3" t="inlineStr">
+        <is>
+          <t>Private nursery (Montessori, multi-site)</t>
+        </is>
+      </c>
+      <c r="C237" s="3" t="inlineStr">
+        <is>
+          <t>Guildford, Cranleigh &amp; Woking, Surrey</t>
+        </is>
+      </c>
+      <c r="D237" s="3" t="inlineStr">
+        <is>
+          <t>https://www.daynurseriessurrey.co.uk</t>
+        </is>
+      </c>
+      <c r="E237" s="3" t="inlineStr">
+        <is>
+          <t>admin@christopherrobin.co.uk</t>
+        </is>
+      </c>
+      <c r="F237" s="3" t="inlineStr">
+        <is>
+          <t>01483 339 406</t>
+        </is>
+      </c>
+      <c r="G237" s="3" t="inlineStr"/>
+      <c r="H237" s="3" t="inlineStr"/>
+      <c r="I237" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/christopherrobinnurseries</t>
+        </is>
+      </c>
+      <c r="J237" s="3" t="inlineStr">
+        <is>
+          <t>Family-run Montessori group, 30+ years, 4+ sites across Surrey; nursery fees £15k+/year per child with sibling/multi-year retention</t>
+        </is>
+      </c>
+      <c r="K237" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L237" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M237" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N237" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O237" s="3" t="inlineStr">
+        <is>
+          <t>Facebook page; per-site listings</t>
+        </is>
+      </c>
+      <c r="P237" s="3" t="inlineStr">
+        <is>
+          <t>Corporate nursery chains (Bright Horizons, N Family, Grandir) heavily outspend on search in the same towns</t>
+        </is>
+      </c>
+      <c r="Q237" s="3" t="inlineStr">
+        <is>
+          <t>'30 years family-run Montessori vs corporate chains - own the AI answer for "independent nursery Guildford"'</t>
+        </is>
+      </c>
+      <c r="R237" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S237" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T237" s="3" t="inlineStr"/>
+    </row>
+    <row r="238">
+      <c r="A238" s="3" t="inlineStr">
+        <is>
+          <t>Ramsac</t>
+        </is>
+      </c>
+      <c r="B238" s="3" t="inlineStr">
+        <is>
+          <t>IT support / MSP</t>
+        </is>
+      </c>
+      <c r="C238" s="3" t="inlineStr">
+        <is>
+          <t>Guildford (Old Portsmouth Rd)</t>
+        </is>
+      </c>
+      <c r="D238" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ramsac.com</t>
+        </is>
+      </c>
+      <c r="E238" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F238" s="3" t="inlineStr">
+        <is>
+          <t>01483 412 040</t>
+        </is>
+      </c>
+      <c r="G238" s="3" t="inlineStr"/>
+      <c r="H238" s="3" t="inlineStr"/>
+      <c r="I238" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/ramsac.ltd</t>
+        </is>
+      </c>
+      <c r="J238" s="3" t="inlineStr">
+        <is>
+          <t>Award-winning Surrey MSP with cybersecurity specialism; recurring SME contracts = high client LTV</t>
+        </is>
+      </c>
+      <c r="K238" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L238" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M238" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N238" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O238" s="3" t="inlineStr">
+        <is>
+          <t>Award-winning brand; thought-leadership positioning</t>
+        </is>
+      </c>
+      <c r="P238" s="3" t="inlineStr">
+        <is>
+          <t>Award-winning status not automatically an AI-search citation advantage over Akita/Wessex IT</t>
+        </is>
+      </c>
+      <c r="Q238" s="3" t="inlineStr">
+        <is>
+          <t>'Award-winning Guildford IT support - make sure that's what AI says when SMEs ask'</t>
+        </is>
+      </c>
+      <c r="R238" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S238" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T238" s="3" t="inlineStr"/>
+    </row>
+    <row r="239">
+      <c r="A239" s="4" t="inlineStr">
+        <is>
+          <t>LP Networks</t>
+        </is>
+      </c>
+      <c r="B239" s="4" t="inlineStr">
+        <is>
+          <t>IT support / MSP</t>
+        </is>
+      </c>
+      <c r="C239" s="4" t="inlineStr">
+        <is>
+          <t>Woking (serves Surrey: Reigate/Redhill/Guildford/Morden)</t>
+        </is>
+      </c>
+      <c r="D239" s="4" t="inlineStr">
+        <is>
+          <t>https://lpnetworks.com</t>
+        </is>
+      </c>
+      <c r="E239" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F239" s="4" t="inlineStr"/>
+      <c r="G239" s="4" t="inlineStr"/>
+      <c r="H239" s="4" t="inlineStr"/>
+      <c r="I239" s="4" t="inlineStr"/>
+      <c r="J239" s="4" t="inlineStr">
+        <is>
+          <t>Fixed-price MSP model across 5+ Surrey towns; recurring monthly contracts</t>
+        </is>
+      </c>
+      <c r="K239" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L239" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M239" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N239" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O239" s="4" t="inlineStr">
+        <is>
+          <t>Fixed-price packaging = marketing-aware</t>
+        </is>
+      </c>
+      <c r="P239" s="4" t="inlineStr">
+        <is>
+          <t>Multi-town coverage but generic 'IT support Surrey' searches won by bigger regional players</t>
+        </is>
+      </c>
+      <c r="Q239" s="4" t="inlineStr">
+        <is>
+          <t>Per-town local SEO to match the fixed-price, multi-town service promise</t>
+        </is>
+      </c>
+      <c r="R239" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S239" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T239" s="4" t="inlineStr"/>
+    </row>
+    <row r="240">
+      <c r="A240" s="4" t="inlineStr">
+        <is>
+          <t>Wessex IT</t>
+        </is>
+      </c>
+      <c r="B240" s="4" t="inlineStr">
+        <is>
+          <t>IT support / MSP</t>
+        </is>
+      </c>
+      <c r="C240" s="4" t="inlineStr">
+        <is>
+          <t>Guildford, Surrey</t>
+        </is>
+      </c>
+      <c r="D240" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wessexit.com</t>
+        </is>
+      </c>
+      <c r="E240" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F240" s="4" t="inlineStr"/>
+      <c r="G240" s="4" t="inlineStr"/>
+      <c r="H240" s="4" t="inlineStr"/>
+      <c r="I240" s="4" t="inlineStr"/>
+      <c r="J240" s="4" t="inlineStr">
+        <is>
+          <t>Supports 250+ Guildford-area businesses; established SME-focused MSP</t>
+        </is>
+      </c>
+      <c r="K240" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L240" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M240" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N240" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O240" s="4" t="inlineStr">
+        <is>
+          <t>250+ client claim promoted</t>
+        </is>
+      </c>
+      <c r="P240" s="4" t="inlineStr">
+        <is>
+          <t>Client-base size claim not leveraged as an AI-search trust signal</t>
+        </is>
+      </c>
+      <c r="Q240" s="4" t="inlineStr">
+        <is>
+          <t>'250+ Surrey businesses trust us' - turn that into the AEO-cited proof point</t>
+        </is>
+      </c>
+      <c r="R240" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S240" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T240" s="4" t="inlineStr"/>
+    </row>
+    <row r="241">
+      <c r="A241" s="4" t="inlineStr">
+        <is>
+          <t>Huggins Lewis Foskett Solicitors</t>
+        </is>
+      </c>
+      <c r="B241" s="4" t="inlineStr">
+        <is>
+          <t>Law firm (wills &amp; probate)</t>
+        </is>
+      </c>
+      <c r="C241" s="4" t="inlineStr">
+        <is>
+          <t>South Woodford, East London</t>
+        </is>
+      </c>
+      <c r="D241" s="4" t="inlineStr">
+        <is>
+          <t>https://www.hugginslaw.co.uk</t>
+        </is>
+      </c>
+      <c r="E241" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F241" s="4" t="inlineStr">
+        <is>
+          <t>020 8989 3000</t>
+        </is>
+      </c>
+      <c r="G241" s="4" t="inlineStr">
+        <is>
+          <t>Simon Huggins (Partner, Head of Wills &amp; Probate)</t>
+        </is>
+      </c>
+      <c r="H241" s="4" t="inlineStr"/>
+      <c r="I241" s="4" t="inlineStr"/>
+      <c r="J241" s="4" t="inlineStr">
+        <is>
+          <t>Long-established East London firm; contentious probate specialism = high-value, high-stress client searches</t>
+        </is>
+      </c>
+      <c r="K241" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L241" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M241" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N241" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O241" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P241" s="4" t="inlineStr">
+        <is>
+          <t>Contentious probate searches are high-intent but dominated by London-wide specialist brands (Osbornes, Russell-Cooke)</t>
+        </is>
+      </c>
+      <c r="Q241" s="4" t="inlineStr">
+        <is>
+          <t>'When families fight over an estate, they Google fast - be the East London name that comes up'</t>
+        </is>
+      </c>
+      <c r="R241" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S241" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T241" s="4" t="inlineStr"/>
+    </row>
+    <row r="242">
+      <c r="A242" s="4" t="inlineStr">
+        <is>
+          <t>Waymont Consulting</t>
+        </is>
+      </c>
+      <c r="B242" s="4" t="inlineStr">
+        <is>
+          <t>Business/technical consultancy</t>
+        </is>
+      </c>
+      <c r="C242" s="4" t="inlineStr">
+        <is>
+          <t>Surrey Research Park, Guildford</t>
+        </is>
+      </c>
+      <c r="D242" s="4" t="inlineStr">
+        <is>
+          <t>https://surrey-research-park.com/company/waymont-consulting</t>
+        </is>
+      </c>
+      <c r="E242" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F242" s="4" t="inlineStr"/>
+      <c r="G242" s="4" t="inlineStr">
+        <is>
+          <t>Dave Waymont (Founder, est. 2000)</t>
+        </is>
+      </c>
+      <c r="H242" s="4" t="inlineStr"/>
+      <c r="I242" s="4" t="inlineStr"/>
+      <c r="J242" s="4" t="inlineStr">
+        <is>
+          <t>25-year technical/business consultancy based at Surrey Research Park; established B2B relationships</t>
+        </is>
+      </c>
+      <c r="K242" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L242" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M242" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N242" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O242" s="4" t="inlineStr">
+        <is>
+          <t>Research Park location = credibility signal</t>
+        </is>
+      </c>
+      <c r="P242" s="4" t="inlineStr">
+        <is>
+          <t>Prestigious location not converted into search-driven new client acquisition</t>
+        </is>
+      </c>
+      <c r="Q242" s="4" t="inlineStr">
+        <is>
+          <t>Location + longevity as the AEO trust signal for Surrey SME consultancy searches</t>
+        </is>
+      </c>
+      <c r="R242" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S242" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T242" s="4" t="inlineStr">
+        <is>
+          <t>Confirm direct website/contact before outreach</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T236"/>
+  <autoFilter ref="A1:T242"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -20872,7 +21384,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B107"/>
+  <dimension ref="A1:B110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -20892,7 +21404,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>235</v>
+        <v>241</v>
       </c>
     </row>
     <row r="5">
@@ -20995,17 +21507,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Mortgage broker</t>
+          <t>IT support / MSP</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Solar installer</t>
+          <t>Mortgage broker</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -21015,7 +21527,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Private GP</t>
+          <t>Solar installer</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -21025,7 +21537,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Private dentist / implants</t>
+          <t>Private GP</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -21035,17 +21547,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Law firm</t>
+          <t>Private dentist / implants</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Electrician</t>
+          <t>Law firm</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -21055,7 +21567,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Personal training studio</t>
+          <t>Electrician</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -21065,7 +21577,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Family law firm</t>
+          <t>Personal training studio</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -21075,7 +21587,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Recruitment agency</t>
+          <t>Family law firm</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -21085,7 +21597,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Immigration law firm</t>
+          <t>Recruitment agency</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -21095,7 +21607,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Independent optician</t>
+          <t>Immigration law firm</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -21105,7 +21617,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Pilates studio</t>
+          <t>Independent optician</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -21115,17 +21627,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Letting agent</t>
+          <t>Pilates studio</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Financial adviser / wealth management</t>
+          <t>Letting agent</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -21135,7 +21647,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Private tuition agency</t>
+          <t>Financial adviser / wealth management</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -21145,7 +21657,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Osteopathy clinic</t>
+          <t>Private tuition agency</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -21155,7 +21667,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Roofer</t>
+          <t>Osteopathy clinic</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -21165,7 +21677,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating / boilers</t>
+          <t>Roofer</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -21175,7 +21687,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Event &amp; wedding caterer</t>
+          <t>Plumbing &amp; heating / boilers</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -21185,7 +21697,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Chiropractor</t>
+          <t>Event &amp; wedding caterer</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -21195,7 +21707,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Estate agent (premium)</t>
+          <t>Chiropractor</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -21205,7 +21717,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Orthodontist</t>
+          <t>Estate agent (premium)</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -21215,7 +21727,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Employment law firm</t>
+          <t>Orthodontist</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -21225,7 +21737,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Event management agency</t>
+          <t>Employment law firm</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -21235,7 +21747,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Design &amp; build</t>
+          <t>Event management agency</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -21245,7 +21757,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>IT support / MSP</t>
+          <t>Design &amp; build</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -21919,6 +22431,36 @@
         </is>
       </c>
       <c r="B107" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Private nursery (Montessori, multi-site)</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Law firm (wills &amp; probate)</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Business/technical consultancy</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 15: +4 prospects (245 total) - West Sussex (Horsham/Haywards Heath)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$242</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$246</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T242"/>
+  <dimension ref="A1:T246"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -21372,8 +21372,376 @@
         </is>
       </c>
     </row>
+    <row r="243">
+      <c r="A243" s="2" t="inlineStr">
+        <is>
+          <t>Brock Taylor</t>
+        </is>
+      </c>
+      <c r="B243" s="2" t="inlineStr">
+        <is>
+          <t>Estate &amp; letting agent</t>
+        </is>
+      </c>
+      <c r="C243" s="2" t="inlineStr">
+        <is>
+          <t>Horsham &amp; Haywards Heath, West Sussex</t>
+        </is>
+      </c>
+      <c r="D243" s="2" t="inlineStr">
+        <is>
+          <t>https://brocktaylor.co.uk</t>
+        </is>
+      </c>
+      <c r="E243" s="2" t="inlineStr">
+        <is>
+          <t>horshamsales@brocktaylor.co.uk</t>
+        </is>
+      </c>
+      <c r="F243" s="2" t="inlineStr">
+        <is>
+          <t>01403 272 022</t>
+        </is>
+      </c>
+      <c r="G243" s="2" t="inlineStr">
+        <is>
+          <t>Peter &amp; Lucy Maskell (Owners, since 2007); founded 1992</t>
+        </is>
+      </c>
+      <c r="H243" s="2" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/brock-taylor</t>
+        </is>
+      </c>
+      <c r="I243" s="2" t="inlineStr">
+        <is>
+          <t>instagram.com/brocktaylor.estate.agents</t>
+        </is>
+      </c>
+      <c r="J243" s="2" t="inlineStr">
+        <is>
+          <t>'Best Agent in West Sussex' 12 years running; 2-office independent with award pedigree and active social presence</t>
+        </is>
+      </c>
+      <c r="K243" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L243" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M243" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N243" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O243" s="2" t="inlineStr">
+        <is>
+          <t>Instagram/YouTube presence; 12 consecutive award wins</t>
+        </is>
+      </c>
+      <c r="P243" s="2" t="inlineStr">
+        <is>
+          <t>Award-winning status not fully converted into AI-search citation dominance</t>
+        </is>
+      </c>
+      <c r="Q243" s="2" t="inlineStr">
+        <is>
+          <t>'12 years as West Sussex's best agent - make AI say so, not just the award ceremony'</t>
+        </is>
+      </c>
+      <c r="R243" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S243" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T243" s="2" t="inlineStr">
+        <is>
+          <t>Strong existing marketing awareness = easy upsell conversation</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="3" t="inlineStr">
+        <is>
+          <t>Clark &amp; Company</t>
+        </is>
+      </c>
+      <c r="B244" s="3" t="inlineStr">
+        <is>
+          <t>Chartered accountants</t>
+        </is>
+      </c>
+      <c r="C244" s="3" t="inlineStr">
+        <is>
+          <t>Haywards Heath, West Sussex</t>
+        </is>
+      </c>
+      <c r="D244" s="3" t="inlineStr">
+        <is>
+          <t>https://clarkandcompany.co.uk</t>
+        </is>
+      </c>
+      <c r="E244" s="3" t="inlineStr">
+        <is>
+          <t>mclark2302@aol.com</t>
+        </is>
+      </c>
+      <c r="F244" s="3" t="inlineStr">
+        <is>
+          <t>01444 416 376</t>
+        </is>
+      </c>
+      <c r="G244" s="3" t="inlineStr">
+        <is>
+          <t>Mitch Clark (Founder &amp; Managing Partner, 2nd generation)</t>
+        </is>
+      </c>
+      <c r="H244" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/clark-&amp;-co</t>
+        </is>
+      </c>
+      <c r="I244" s="3" t="inlineStr"/>
+      <c r="J244" s="3" t="inlineStr">
+        <is>
+          <t>Second-generation family accountancy firm covering Haywards Heath to Brighton/Crawley/Oxted - wide recurring-fee catchment</t>
+        </is>
+      </c>
+      <c r="K244" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L244" s="3" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="M244" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N244" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O244" s="3" t="inlineStr">
+        <is>
+          <t>AOL email address - low marketing infrastructure</t>
+        </is>
+      </c>
+      <c r="P244" s="3" t="inlineStr">
+        <is>
+          <t>Wide geographic coverage undermined by dated digital presence (AOL email is the tell)</t>
+        </is>
+      </c>
+      <c r="Q244" s="3" t="inlineStr">
+        <is>
+          <t>'You cover 12 towns but your email address is stuck in 2005 - let's fix the whole funnel'</t>
+        </is>
+      </c>
+      <c r="R244" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S244" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T244" s="3" t="inlineStr">
+        <is>
+          <t>AOL email = same infrastructure-gap wedge as Gmail-contact prospects elsewhere in the database</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="4" t="inlineStr">
+        <is>
+          <t>Rose Chapman Architects</t>
+        </is>
+      </c>
+      <c r="B245" s="4" t="inlineStr">
+        <is>
+          <t>Architects &amp; interior design</t>
+        </is>
+      </c>
+      <c r="C245" s="4" t="inlineStr">
+        <is>
+          <t>Haywards Heath, West Sussex</t>
+        </is>
+      </c>
+      <c r="D245" s="4" t="inlineStr">
+        <is>
+          <t>https://rosechapmanarchitects.com</t>
+        </is>
+      </c>
+      <c r="E245" s="4" t="inlineStr">
+        <is>
+          <t>nicholas@rosechapmanarchitects.com</t>
+        </is>
+      </c>
+      <c r="F245" s="4" t="inlineStr">
+        <is>
+          <t>07429 074995</t>
+        </is>
+      </c>
+      <c r="G245" s="4" t="inlineStr">
+        <is>
+          <t>Rose Chapman / Nicholas (Founders)</t>
+        </is>
+      </c>
+      <c r="H245" s="4" t="inlineStr"/>
+      <c r="I245" s="4" t="inlineStr"/>
+      <c r="J245" s="4" t="inlineStr">
+        <is>
+          <t>Combined architecture + interior design studio covering listed buildings across Sussex/Brighton/London; young practice building reputation</t>
+        </is>
+      </c>
+      <c r="K245" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L245" s="4" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M245" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N245" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O245" s="4" t="inlineStr">
+        <is>
+          <t>Active journal/blog content</t>
+        </is>
+      </c>
+      <c r="P245" s="4" t="inlineStr">
+        <is>
+          <t>New practice (2022) needs to build search authority fast in a competitive Sussex market</t>
+        </is>
+      </c>
+      <c r="Q245" s="4" t="inlineStr">
+        <is>
+          <t>Ground-floor AEO investment while the practice is still establishing its market position</t>
+        </is>
+      </c>
+      <c r="R245" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S245" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T245" s="4" t="inlineStr"/>
+    </row>
+    <row r="246">
+      <c r="A246" s="4" t="inlineStr">
+        <is>
+          <t>DHP Dental Healthcare Practice</t>
+        </is>
+      </c>
+      <c r="B246" s="4" t="inlineStr">
+        <is>
+          <t>Private/NHS dentist</t>
+        </is>
+      </c>
+      <c r="C246" s="4" t="inlineStr">
+        <is>
+          <t>North Heath Lane, Horsham, Sussex</t>
+        </is>
+      </c>
+      <c r="D246" s="4" t="inlineStr">
+        <is>
+          <t>https://dhp.dental</t>
+        </is>
+      </c>
+      <c r="E246" s="4" t="inlineStr">
+        <is>
+          <t>info@dhp.dental</t>
+        </is>
+      </c>
+      <c r="F246" s="4" t="inlineStr">
+        <is>
+          <t>01403 259 717</t>
+        </is>
+      </c>
+      <c r="G246" s="4" t="inlineStr"/>
+      <c r="H246" s="4" t="inlineStr"/>
+      <c r="I246" s="4" t="inlineStr"/>
+      <c r="J246" s="4" t="inlineStr">
+        <is>
+          <t>Modern family dental practice in Horsham; mixed private/NHS model with upsell potential to cosmetic/implant work</t>
+        </is>
+      </c>
+      <c r="K246" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L246" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M246" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N246" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O246" s="4" t="inlineStr">
+        <is>
+          <t>Rebranded domain (dhp.dental) suggests marketing awareness</t>
+        </is>
+      </c>
+      <c r="P246" s="4" t="inlineStr">
+        <is>
+          <t>New domain/brand needs search authority built from scratch</t>
+        </is>
+      </c>
+      <c r="Q246" s="4" t="inlineStr">
+        <is>
+          <t>Early-mover AEO advantage while rebrand is still fresh</t>
+        </is>
+      </c>
+      <c r="R246" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S246" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T246" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T242"/>
+  <autoFilter ref="A1:T246"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -21384,7 +21752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B110"/>
+  <dimension ref="A1:B112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -21404,7 +21772,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="5">
@@ -21467,17 +21835,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Physiotherapy clinic</t>
+          <t>Estate &amp; letting agent</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Estate &amp; letting agent</t>
+          <t>Physiotherapy clinic</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -21487,7 +21855,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Aesthetics clinic</t>
+          <t>Chartered accountants</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -21497,11 +21865,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Chartered accountants</t>
+          <t>Aesthetics clinic</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15">
@@ -22461,6 +22829,26 @@
         </is>
       </c>
       <c r="B110" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Architects &amp; interior design</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Private/NHS dentist</t>
+        </is>
+      </c>
+      <c r="B112" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 16: +8 prospects (253 total) - kitchen/bathroom design, removals, funeral directors, chiropractors
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$246</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$254</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T246"/>
+  <dimension ref="A1:T254"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -21740,8 +21740,700 @@
       </c>
       <c r="T246" s="4" t="inlineStr"/>
     </row>
+    <row r="247">
+      <c r="A247" s="3" t="inlineStr">
+        <is>
+          <t>Bath Kitchen Company</t>
+        </is>
+      </c>
+      <c r="B247" s="3" t="inlineStr">
+        <is>
+          <t>Kitchen &amp; bathroom design</t>
+        </is>
+      </c>
+      <c r="C247" s="3" t="inlineStr">
+        <is>
+          <t>Bath, Somerset</t>
+        </is>
+      </c>
+      <c r="D247" s="3" t="inlineStr">
+        <is>
+          <t>https://bathkitchencompany.co.uk</t>
+        </is>
+      </c>
+      <c r="E247" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F247" s="3" t="inlineStr"/>
+      <c r="G247" s="3" t="inlineStr">
+        <is>
+          <t>James Horsfall (Owner)</t>
+        </is>
+      </c>
+      <c r="H247" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/james-horsfall-6b71a711</t>
+        </is>
+      </c>
+      <c r="I247" s="3" t="inlineStr"/>
+      <c r="J247" s="3" t="inlineStr">
+        <is>
+          <t>Independent handmade-kitchen specialist, 30+ years trading in Bath; bespoke kitchen projects worth £20-80k each</t>
+        </is>
+      </c>
+      <c r="K247" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L247" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M247" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N247" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O247" s="3" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P247" s="3" t="inlineStr">
+        <is>
+          <t>National kitchen chains (Wren, Magnet) outspend on 'kitchen design Bath' search terms</t>
+        </is>
+      </c>
+      <c r="Q247" s="3" t="inlineStr">
+        <is>
+          <t>'A £40k bespoke kitchen deserves a bespoke marketing plan, not just a showroom visit'</t>
+        </is>
+      </c>
+      <c r="R247" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S247" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T247" s="3" t="inlineStr"/>
+    </row>
+    <row r="248">
+      <c r="A248" s="4" t="inlineStr">
+        <is>
+          <t>Somerset Kitchens Design Studio</t>
+        </is>
+      </c>
+      <c r="B248" s="4" t="inlineStr">
+        <is>
+          <t>Kitchen &amp; bathroom design</t>
+        </is>
+      </c>
+      <c r="C248" s="4" t="inlineStr">
+        <is>
+          <t>Wrington (serves Bristol/Bath)</t>
+        </is>
+      </c>
+      <c r="D248" s="4" t="inlineStr">
+        <is>
+          <t>https://www.somersetkitchendesignstudio.co.uk</t>
+        </is>
+      </c>
+      <c r="E248" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F248" s="4" t="inlineStr"/>
+      <c r="G248" s="4" t="inlineStr"/>
+      <c r="H248" s="4" t="inlineStr"/>
+      <c r="I248" s="4" t="inlineStr"/>
+      <c r="J248" s="4" t="inlineStr">
+        <is>
+          <t>Family-run bespoke kitchen/bathroom designer serving Bristol and Bath from one Somerset base</t>
+        </is>
+      </c>
+      <c r="K248" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L248" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M248" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N248" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O248" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P248" s="4" t="inlineStr">
+        <is>
+          <t>Two-city catchment but single-location search visibility limits reach</t>
+        </is>
+      </c>
+      <c r="Q248" s="4" t="inlineStr">
+        <is>
+          <t>Own both 'kitchen designer Bristol' and 'kitchen designer Bath' from one business</t>
+        </is>
+      </c>
+      <c r="R248" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S248" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T248" s="4" t="inlineStr"/>
+    </row>
+    <row r="249">
+      <c r="A249" s="3" t="inlineStr">
+        <is>
+          <t>BK11 (Bathroom &amp; Kitchen 11)</t>
+        </is>
+      </c>
+      <c r="B249" s="3" t="inlineStr">
+        <is>
+          <t>Kitchen &amp; bathroom design</t>
+        </is>
+      </c>
+      <c r="C249" s="3" t="inlineStr">
+        <is>
+          <t>Long Ditton, Surrey (serves Esher/Cobham/Surbiton)</t>
+        </is>
+      </c>
+      <c r="D249" s="3" t="inlineStr">
+        <is>
+          <t>https://bathroomandkitcheneleven.co.uk</t>
+        </is>
+      </c>
+      <c r="E249" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F249" s="3" t="inlineStr"/>
+      <c r="G249" s="3" t="inlineStr">
+        <is>
+          <t>Ben (Managing Director)</t>
+        </is>
+      </c>
+      <c r="H249" s="3" t="inlineStr"/>
+      <c r="I249" s="3" t="inlineStr"/>
+      <c r="J249" s="3" t="inlineStr">
+        <is>
+          <t>Award-winning luxury bathroom/kitchen showroom in the heart of wealthy Surrey; projects £30-100k+</t>
+        </is>
+      </c>
+      <c r="K249" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L249" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M249" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N249" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O249" s="3" t="inlineStr">
+        <is>
+          <t>Award-winning branding</t>
+        </is>
+      </c>
+      <c r="P249" s="3" t="inlineStr">
+        <is>
+          <t>Awards not converted into AI-search dominance for Esher/Cobham searches</t>
+        </is>
+      </c>
+      <c r="Q249" s="3" t="inlineStr">
+        <is>
+          <t>'Award-winning Surrey design should be the AI's answer, not just the showroom's trophy cabinet'</t>
+        </is>
+      </c>
+      <c r="R249" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S249" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T249" s="3" t="inlineStr"/>
+    </row>
+    <row r="250">
+      <c r="A250" s="4" t="inlineStr">
+        <is>
+          <t>AJM Removals Bristol</t>
+        </is>
+      </c>
+      <c r="B250" s="4" t="inlineStr">
+        <is>
+          <t>Removals company</t>
+        </is>
+      </c>
+      <c r="C250" s="4" t="inlineStr">
+        <is>
+          <t>Fishponds Rd, Bristol</t>
+        </is>
+      </c>
+      <c r="D250" s="4" t="inlineStr">
+        <is>
+          <t>https://ajm-removals-bristol.co.uk</t>
+        </is>
+      </c>
+      <c r="E250" s="4" t="inlineStr">
+        <is>
+          <t>contact@ajmremovals.co.uk</t>
+        </is>
+      </c>
+      <c r="F250" s="4" t="inlineStr">
+        <is>
+          <t>0117 251 0113</t>
+        </is>
+      </c>
+      <c r="G250" s="4" t="inlineStr">
+        <is>
+          <t>Artjom "AJ" (Founder, est. 2011)</t>
+        </is>
+      </c>
+      <c r="H250" s="4" t="inlineStr"/>
+      <c r="I250" s="4" t="inlineStr"/>
+      <c r="J250" s="4" t="inlineStr">
+        <is>
+          <t>Owner personally oversees every move since 2011; £1m public liability insurance signals a serious, insured operation worth more than budget rivals</t>
+        </is>
+      </c>
+      <c r="K250" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L250" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M250" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N250" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O250" s="4" t="inlineStr">
+        <is>
+          <t>Insurance credentials promoted</t>
+        </is>
+      </c>
+      <c r="P250" s="4" t="inlineStr">
+        <is>
+          <t>Man-and-van budget competitors and national brands (Bishop's Move) both crowd 'removals Bristol' search</t>
+        </is>
+      </c>
+      <c r="Q250" s="4" t="inlineStr">
+        <is>
+          <t>'Fully insured, owner-managed removals vs a stranger with a van - own that trust gap in AI answers'</t>
+        </is>
+      </c>
+      <c r="R250" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S250" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T250" s="4" t="inlineStr"/>
+    </row>
+    <row r="251">
+      <c r="A251" s="3" t="inlineStr">
+        <is>
+          <t>Clarkson's Independent Funeral Directors</t>
+        </is>
+      </c>
+      <c r="B251" s="3" t="inlineStr">
+        <is>
+          <t>Funeral directors</t>
+        </is>
+      </c>
+      <c r="C251" s="3" t="inlineStr">
+        <is>
+          <t>Bath, Frome &amp; Saltford (Bristol)</t>
+        </is>
+      </c>
+      <c r="D251" s="3" t="inlineStr">
+        <is>
+          <t>https://www.clarksonsfuneraldirectors.co.uk</t>
+        </is>
+      </c>
+      <c r="E251" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F251" s="3" t="inlineStr">
+        <is>
+          <t>01225 426 822</t>
+        </is>
+      </c>
+      <c r="G251" s="3" t="inlineStr">
+        <is>
+          <t>Carol Spalding &amp; Sophie May (mother &amp; daughter, Owners)</t>
+        </is>
+      </c>
+      <c r="H251" s="3" t="inlineStr"/>
+      <c r="I251" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/ClarksonsBathFromeSaltford</t>
+        </is>
+      </c>
+      <c r="J251" s="3" t="inlineStr">
+        <is>
+          <t>Family-run across 3 sites; funerals are high-emotion, high-value, once-only decisions researched urgently online</t>
+        </is>
+      </c>
+      <c r="K251" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L251" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M251" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N251" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O251" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence; multi-site coverage</t>
+        </is>
+      </c>
+      <c r="P251" s="3" t="inlineStr">
+        <is>
+          <t>Corporate funeral groups (Dignity, Co-op Funeralcare) dominate search visibility despite worse reputations</t>
+        </is>
+      </c>
+      <c r="Q251" s="3" t="inlineStr">
+        <is>
+          <t>'Grieving families search fast and trust local - be the independent name Google and AI recommend over the corporates'</t>
+        </is>
+      </c>
+      <c r="R251" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S251" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T251" s="3" t="inlineStr"/>
+    </row>
+    <row r="252">
+      <c r="A252" s="4" t="inlineStr">
+        <is>
+          <t>Hebden Pople Independent Funerals</t>
+        </is>
+      </c>
+      <c r="B252" s="4" t="inlineStr">
+        <is>
+          <t>Funeral directors</t>
+        </is>
+      </c>
+      <c r="C252" s="4" t="inlineStr">
+        <is>
+          <t>Stockwood, South Bristol</t>
+        </is>
+      </c>
+      <c r="D252" s="4" t="inlineStr">
+        <is>
+          <t>https://hebdenpople.co.uk</t>
+        </is>
+      </c>
+      <c r="E252" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F252" s="4" t="inlineStr">
+        <is>
+          <t>01275 563 422</t>
+        </is>
+      </c>
+      <c r="G252" s="4" t="inlineStr"/>
+      <c r="H252" s="4" t="inlineStr"/>
+      <c r="I252" s="4" t="inlineStr"/>
+      <c r="J252" s="4" t="inlineStr">
+        <is>
+          <t>Family-run independent serving Bristol/Bath/South Gloucestershire; approachable positioning differentiates from corporate chains</t>
+        </is>
+      </c>
+      <c r="K252" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L252" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M252" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N252" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O252" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P252" s="4" t="inlineStr">
+        <is>
+          <t>Same corporate-chain search dominance problem as Clarkson's</t>
+        </is>
+      </c>
+      <c r="Q252" s="4" t="inlineStr">
+        <is>
+          <t>'Approachable, independent, local' - own that AEO positioning against Dignity/Co-op</t>
+        </is>
+      </c>
+      <c r="R252" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S252" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T252" s="4" t="inlineStr"/>
+    </row>
+    <row r="253">
+      <c r="A253" s="3" t="inlineStr">
+        <is>
+          <t>Guildford Chiropractic Centre</t>
+        </is>
+      </c>
+      <c r="B253" s="3" t="inlineStr">
+        <is>
+          <t>Chiropractor</t>
+        </is>
+      </c>
+      <c r="C253" s="3" t="inlineStr">
+        <is>
+          <t>Guildford, Surrey</t>
+        </is>
+      </c>
+      <c r="D253" s="3" t="inlineStr">
+        <is>
+          <t>https://www.guildfordchiropractic.co.uk</t>
+        </is>
+      </c>
+      <c r="E253" s="3" t="inlineStr">
+        <is>
+          <t>info@guildfordchiropractic.co.uk</t>
+        </is>
+      </c>
+      <c r="F253" s="3" t="inlineStr">
+        <is>
+          <t>01483 562 830</t>
+        </is>
+      </c>
+      <c r="G253" s="3" t="inlineStr">
+        <is>
+          <t>Founded by Donald &amp; Elizabeth Bennett, 1953 (multi-generation family)</t>
+        </is>
+      </c>
+      <c r="H253" s="3" t="inlineStr"/>
+      <c r="I253" s="3" t="inlineStr"/>
+      <c r="J253" s="3" t="inlineStr">
+        <is>
+          <t>70+ years trading, multi-generational chiropractic family - genuinely rare heritage in a competitive Surrey market</t>
+        </is>
+      </c>
+      <c r="K253" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L253" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M253" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N253" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O253" s="3" t="inlineStr">
+        <is>
+          <t>70-year heritage</t>
+        </is>
+      </c>
+      <c r="P253" s="3" t="inlineStr">
+        <is>
+          <t>Decades of trust invisible against newer, better-marketed rivals (Health in Motion, GW Osteopathy)</t>
+        </is>
+      </c>
+      <c r="Q253" s="3" t="inlineStr">
+        <is>
+          <t>'70 years and three generations of Bennetts - the AI answer should reflect that, not just Google Maps'</t>
+        </is>
+      </c>
+      <c r="R253" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S253" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T253" s="3" t="inlineStr"/>
+    </row>
+    <row r="254">
+      <c r="A254" s="4" t="inlineStr">
+        <is>
+          <t>Health In Motion</t>
+        </is>
+      </c>
+      <c r="B254" s="4" t="inlineStr">
+        <is>
+          <t>Osteopathy clinic</t>
+        </is>
+      </c>
+      <c r="C254" s="4" t="inlineStr">
+        <is>
+          <t>Guildford &amp; Surbiton, Surrey</t>
+        </is>
+      </c>
+      <c r="D254" s="4" t="inlineStr">
+        <is>
+          <t>https://healthinmotiononline.co.uk</t>
+        </is>
+      </c>
+      <c r="E254" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F254" s="4" t="inlineStr">
+        <is>
+          <t>01483 310 440</t>
+        </is>
+      </c>
+      <c r="G254" s="4" t="inlineStr">
+        <is>
+          <t>Dominic Malone (Founder, 10+ years)</t>
+        </is>
+      </c>
+      <c r="H254" s="4" t="inlineStr"/>
+      <c r="I254" s="4" t="inlineStr"/>
+      <c r="J254" s="4" t="inlineStr">
+        <is>
+          <t>Two-town osteopathy/wellness practice; founder-led with over a decade of trading</t>
+        </is>
+      </c>
+      <c r="K254" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L254" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M254" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N254" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O254" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P254" s="4" t="inlineStr">
+        <is>
+          <t>Two-town coverage undermined by single-location search visibility</t>
+        </is>
+      </c>
+      <c r="Q254" s="4" t="inlineStr">
+        <is>
+          <t>Own both Guildford AND Surbiton osteopathy searches from one founder-led brand</t>
+        </is>
+      </c>
+      <c r="R254" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S254" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T254" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T246"/>
+  <autoFilter ref="A1:T254"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -21752,7 +22444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B112"/>
+  <dimension ref="A1:B115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -21772,7 +22464,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>245</v>
+        <v>253</v>
       </c>
     </row>
     <row r="5">
@@ -21935,7 +22627,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Electrician</t>
+          <t>Osteopathy clinic</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -21945,7 +22637,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Personal training studio</t>
+          <t>Electrician</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -21955,7 +22647,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Family law firm</t>
+          <t>Personal training studio</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -21965,7 +22657,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Recruitment agency</t>
+          <t>Family law firm</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -21975,7 +22667,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Immigration law firm</t>
+          <t>Chiropractor</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -21985,7 +22677,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Independent optician</t>
+          <t>Recruitment agency</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -21995,7 +22687,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Pilates studio</t>
+          <t>Immigration law firm</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -22005,37 +22697,37 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Letting agent</t>
+          <t>Independent optician</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Financial adviser / wealth management</t>
+          <t>Pilates studio</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Private tuition agency</t>
+          <t>Kitchen &amp; bathroom design</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Osteopathy clinic</t>
+          <t>Letting agent</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -22045,7 +22737,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Roofer</t>
+          <t>Financial adviser / wealth management</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -22055,7 +22747,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating / boilers</t>
+          <t>Private tuition agency</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -22065,7 +22757,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Event &amp; wedding caterer</t>
+          <t>Roofer</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -22075,7 +22767,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Chiropractor</t>
+          <t>Plumbing &amp; heating / boilers</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -22085,7 +22777,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Estate agent (premium)</t>
+          <t>Event &amp; wedding caterer</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -22095,7 +22787,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Orthodontist</t>
+          <t>Estate agent (premium)</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -22105,7 +22797,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Employment law firm</t>
+          <t>Orthodontist</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -22115,7 +22807,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Event management agency</t>
+          <t>Employment law firm</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -22125,7 +22817,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Design &amp; build</t>
+          <t>Event management agency</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -22135,27 +22827,27 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Dentist / Orthodontics</t>
+          <t>Design &amp; build</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Specialist dental/implant clinic</t>
+          <t>Funeral directors</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Boutique corporate law firm</t>
+          <t>Dentist / Orthodontics</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -22165,7 +22857,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Cosmetic/aesthetics clinic</t>
+          <t>Specialist dental/implant clinic</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -22175,7 +22867,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Skin &amp; laser clinic</t>
+          <t>Boutique corporate law firm</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -22185,7 +22877,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Mortgage broker / financial adviser</t>
+          <t>Cosmetic/aesthetics clinic</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -22195,7 +22887,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Architects (RIBA chartered)</t>
+          <t>Skin &amp; laser clinic</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -22205,7 +22897,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Recruitment agency (tech/startups)</t>
+          <t>Mortgage broker / financial adviser</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -22215,7 +22907,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Recruitment agency (IT/data)</t>
+          <t>Architects (RIBA chartered)</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -22225,7 +22917,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Independent vet (24/7 emergency)</t>
+          <t>Recruitment agency (tech/startups)</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -22235,7 +22927,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Interior design studio</t>
+          <t>Recruitment agency (IT/data)</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -22245,7 +22937,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Letting &amp; estate agent</t>
+          <t>Independent vet (24/7 emergency)</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -22255,7 +22947,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Cosmetic clinic (injectables)</t>
+          <t>Interior design studio</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -22265,7 +22957,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Cosmetic/anti-ageing clinic</t>
+          <t>Letting &amp; estate agent</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -22275,7 +22967,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Yoga &amp; reformer pilates studio</t>
+          <t>Cosmetic clinic (injectables)</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -22285,7 +22977,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Reformer pilates studio</t>
+          <t>Cosmetic/anti-ageing clinic</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -22295,7 +22987,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Wealth management</t>
+          <t>Yoga &amp; reformer pilates studio</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -22305,7 +22997,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Private tuition &amp; education consultancy</t>
+          <t>Reformer pilates studio</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -22315,7 +23007,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Osteopath</t>
+          <t>Wealth management</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -22325,7 +23017,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Design &amp; build / home renovation</t>
+          <t>Private tuition &amp; education consultancy</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -22335,7 +23027,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Builders / building contractor</t>
+          <t>Osteopath</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -22345,7 +23037,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Home care / live-in care</t>
+          <t>Design &amp; build / home renovation</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -22355,7 +23047,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Private day nurseries</t>
+          <t>Builders / building contractor</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -22365,7 +23057,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Personal training &amp; wellness studio</t>
+          <t>Home care / live-in care</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -22375,7 +23067,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Mortgage &amp; insurance broker</t>
+          <t>Private day nurseries</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -22385,7 +23077,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Business consultancy</t>
+          <t>Personal training &amp; wellness studio</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -22395,7 +23087,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Interior designer (period homes)</t>
+          <t>Mortgage &amp; insurance broker</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -22405,7 +23097,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Landscape design &amp; build</t>
+          <t>Business consultancy</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -22415,7 +23107,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Interior designer</t>
+          <t>Interior designer (period homes)</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -22425,7 +23117,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Garden design &amp; landscaping</t>
+          <t>Landscape design &amp; build</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -22435,7 +23127,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Legal recruitment</t>
+          <t>Interior designer</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -22445,7 +23137,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Independent gym &amp; health club</t>
+          <t>Garden design &amp; landscaping</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -22455,7 +23147,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Independent gym</t>
+          <t>Legal recruitment</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -22465,7 +23157,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Physiotherapy (sports)</t>
+          <t>Independent gym &amp; health club</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -22475,7 +23167,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Letting agent / property management</t>
+          <t>Independent gym</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -22485,7 +23177,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Skin clinic</t>
+          <t>Physiotherapy (sports)</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -22495,7 +23187,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Tutoring company</t>
+          <t>Letting agent / property management</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -22505,7 +23197,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Tutorial college &amp; exam centre</t>
+          <t>Skin clinic</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -22515,7 +23207,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Employment law (disability discrimination)</t>
+          <t>Tutoring company</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -22525,7 +23217,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating</t>
+          <t>Tutorial college &amp; exam centre</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -22535,7 +23227,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Employment law (disability discrimination)</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -22545,7 +23237,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Sports physio &amp; massage</t>
+          <t>Plumbing &amp; heating</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -22555,7 +23247,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Chartered surveyors (party wall/building)</t>
+          <t>Plumbing</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -22565,7 +23257,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Chartered surveyors</t>
+          <t>Sports physio &amp; massage</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -22575,7 +23267,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Chartered building surveyors</t>
+          <t>Chartered surveyors (party wall/building)</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -22585,7 +23277,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Osteopathy clinics</t>
+          <t>Chartered surveyors</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -22595,7 +23287,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Builders / renovations</t>
+          <t>Chartered building surveyors</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -22605,7 +23297,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Private nursery schools</t>
+          <t>Osteopathy clinics</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -22615,7 +23307,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Private day nursery</t>
+          <t>Builders / renovations</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -22625,7 +23317,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Private GP (membership model)</t>
+          <t>Private nursery schools</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -22635,7 +23327,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Sash window restoration</t>
+          <t>Private day nursery</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -22645,7 +23337,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Personal training (1:1)</t>
+          <t>Private GP (membership model)</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -22655,7 +23347,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Personal training &amp; nutrition coaching</t>
+          <t>Sash window restoration</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -22665,7 +23357,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Private nursery/pre-prep school</t>
+          <t>Personal training (1:1)</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -22675,7 +23367,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Independent nursery (Montessori)</t>
+          <t>Personal training &amp; nutrition coaching</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -22685,7 +23377,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Live-in care agency</t>
+          <t>Private nursery/pre-prep school</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -22695,7 +23387,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Law firm (conveyancing/family)</t>
+          <t>Independent nursery (Montessori)</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -22705,7 +23397,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Architect &amp; interior designer</t>
+          <t>Live-in care agency</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -22715,7 +23407,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Architects / project management</t>
+          <t>Law firm (conveyancing/family)</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -22725,7 +23417,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>IFA / wealth management</t>
+          <t>Architect &amp; interior designer</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -22735,7 +23427,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Physiotherapy &amp; clinical Pilates</t>
+          <t>Architects / project management</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -22745,7 +23437,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Aesthetics &amp; skin clinic</t>
+          <t>IFA / wealth management</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -22755,7 +23447,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Wealth management / IFA</t>
+          <t>Physiotherapy &amp; clinical Pilates</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -22765,7 +23457,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>IFA / financial planning</t>
+          <t>Aesthetics &amp; skin clinic</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -22775,7 +23467,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Wealth management &amp; employee benefits</t>
+          <t>Wealth management / IFA</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -22785,7 +23477,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Dermatology clinic</t>
+          <t>IFA / financial planning</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -22795,7 +23487,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Pilates studio (multi-site)</t>
+          <t>Wealth management &amp; employee benefits</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -22805,7 +23497,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Private nursery (Montessori, multi-site)</t>
+          <t>Dermatology clinic</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -22815,7 +23507,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Law firm (wills &amp; probate)</t>
+          <t>Pilates studio (multi-site)</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -22825,7 +23517,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Business/technical consultancy</t>
+          <t>Private nursery (Montessori, multi-site)</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -22835,7 +23527,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Architects &amp; interior design</t>
+          <t>Law firm (wills &amp; probate)</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -22845,10 +23537,40 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
+          <t>Business/technical consultancy</t>
+        </is>
+      </c>
+      <c r="B112" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Architects &amp; interior design</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
           <t>Private/NHS dentist</t>
         </is>
       </c>
-      <c r="B112" t="n">
+      <c r="B114" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Removals company</t>
+        </is>
+      </c>
+      <c r="B115" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 17: +7 prospects (260 total) - garden rooms, paving, Somerset/Devon venues, Kent IFA
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$254</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$261</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T254"/>
+  <dimension ref="A1:T261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -22432,8 +22432,604 @@
       </c>
       <c r="T254" s="4" t="inlineStr"/>
     </row>
+    <row r="255">
+      <c r="A255" s="4" t="inlineStr">
+        <is>
+          <t>Little Green Rooms</t>
+        </is>
+      </c>
+      <c r="B255" s="4" t="inlineStr">
+        <is>
+          <t>Garden rooms / outbuildings</t>
+        </is>
+      </c>
+      <c r="C255" s="4" t="inlineStr">
+        <is>
+          <t>Gloucester Road, Bishopston, Bristol</t>
+        </is>
+      </c>
+      <c r="D255" s="4" t="inlineStr">
+        <is>
+          <t>https://littlegreenrooms.co.uk</t>
+        </is>
+      </c>
+      <c r="E255" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F255" s="4" t="inlineStr"/>
+      <c r="G255" s="4" t="inlineStr">
+        <is>
+          <t>Jack (Founder, launched during lockdown)</t>
+        </is>
+      </c>
+      <c r="H255" s="4" t="inlineStr">
+        <is>
+          <t>instagram.com/little_green_rooms</t>
+        </is>
+      </c>
+      <c r="I255" s="4" t="inlineStr"/>
+      <c r="J255" s="4" t="inlineStr">
+        <is>
+          <t>Sustainability-led garden room maker with a Bristol showroom; work-from-home boom drove strong demand, projects £15-40k</t>
+        </is>
+      </c>
+      <c r="K255" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L255" s="4" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M255" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N255" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O255" s="4" t="inlineStr">
+        <is>
+          <t>Instagram presence; showroom</t>
+        </is>
+      </c>
+      <c r="P255" s="4" t="inlineStr">
+        <is>
+          <t>National garden-room brands (Crane, Cabin Master) outspend on generic search terms</t>
+        </is>
+      </c>
+      <c r="Q255" s="4" t="inlineStr">
+        <is>
+          <t>'Sustainable, Bristol-made garden rooms deserve to beat national brands in local search'</t>
+        </is>
+      </c>
+      <c r="R255" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S255" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T255" s="4" t="inlineStr"/>
+    </row>
+    <row r="256">
+      <c r="A256" s="3" t="inlineStr">
+        <is>
+          <t>Garden Rooms by Drumbeat</t>
+        </is>
+      </c>
+      <c r="B256" s="3" t="inlineStr">
+        <is>
+          <t>Garden rooms / outbuildings</t>
+        </is>
+      </c>
+      <c r="C256" s="3" t="inlineStr">
+        <is>
+          <t>Surrey &amp; South East</t>
+        </is>
+      </c>
+      <c r="D256" s="3" t="inlineStr">
+        <is>
+          <t>https://gardenroomsbydrumbeat.co.uk</t>
+        </is>
+      </c>
+      <c r="E256" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F256" s="3" t="inlineStr">
+        <is>
+          <t>01483 768 273</t>
+        </is>
+      </c>
+      <c r="G256" s="3" t="inlineStr"/>
+      <c r="H256" s="3" t="inlineStr"/>
+      <c r="I256" s="3" t="inlineStr"/>
+      <c r="J256" s="3" t="inlineStr">
+        <is>
+          <t>30 years' design &amp; build experience in Surrey's wealthy commuter belt; premium garden offices/studios</t>
+        </is>
+      </c>
+      <c r="K256" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L256" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M256" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N256" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O256" s="3" t="inlineStr">
+        <is>
+          <t>30-year heritage promoted</t>
+        </is>
+      </c>
+      <c r="P256" s="3" t="inlineStr">
+        <is>
+          <t>Three decades of trust not converted into AI-search dominance vs newer brands</t>
+        </is>
+      </c>
+      <c r="Q256" s="3" t="inlineStr">
+        <is>
+          <t>'30 years building Surrey's garden rooms - make sure AI still recommends the original'</t>
+        </is>
+      </c>
+      <c r="R256" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S256" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T256" s="3" t="inlineStr"/>
+    </row>
+    <row r="257">
+      <c r="A257" s="4" t="inlineStr">
+        <is>
+          <t>S&amp;D Paving &amp; Landscaping</t>
+        </is>
+      </c>
+      <c r="B257" s="4" t="inlineStr">
+        <is>
+          <t>Driveways &amp; landscaping</t>
+        </is>
+      </c>
+      <c r="C257" s="4" t="inlineStr">
+        <is>
+          <t>Epsom, Surrey</t>
+        </is>
+      </c>
+      <c r="D257" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sanddpaving.co.uk</t>
+        </is>
+      </c>
+      <c r="E257" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F257" s="4" t="inlineStr"/>
+      <c r="G257" s="4" t="inlineStr"/>
+      <c r="H257" s="4" t="inlineStr"/>
+      <c r="I257" s="4" t="inlineStr"/>
+      <c r="J257" s="4" t="inlineStr">
+        <is>
+          <t>Established 2008, FSB/Tobermore/Bradstone accredited; driveway/patio jobs £5-20k in premium Surrey postcodes</t>
+        </is>
+      </c>
+      <c r="K257" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L257" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M257" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N257" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O257" s="4" t="inlineStr">
+        <is>
+          <t>Trade accreditations</t>
+        </is>
+      </c>
+      <c r="P257" s="4" t="inlineStr">
+        <is>
+          <t>Checkatrade/MyBuilder intercept driveway searches before firms are found directly</t>
+        </is>
+      </c>
+      <c r="Q257" s="4" t="inlineStr">
+        <is>
+          <t>'Stop paying Checkatrade for leads to your own jobs - own "driveways Epsom" outright'</t>
+        </is>
+      </c>
+      <c r="R257" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S257" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T257" s="4" t="inlineStr"/>
+    </row>
+    <row r="258">
+      <c r="A258" s="2" t="inlineStr">
+        <is>
+          <t>Midelney Manor</t>
+        </is>
+      </c>
+      <c r="B258" s="2" t="inlineStr">
+        <is>
+          <t>Wedding venue</t>
+        </is>
+      </c>
+      <c r="C258" s="2" t="inlineStr">
+        <is>
+          <t>Langport, Somerset</t>
+        </is>
+      </c>
+      <c r="D258" s="2" t="inlineStr">
+        <is>
+          <t>https://www.midelneymanor.co.uk</t>
+        </is>
+      </c>
+      <c r="E258" s="2" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F258" s="2" t="inlineStr">
+        <is>
+          <t>01458 252 377</t>
+        </is>
+      </c>
+      <c r="G258" s="2" t="inlineStr">
+        <is>
+          <t>Alice &amp; Jeremy (Family owners, 500-year family estate)</t>
+        </is>
+      </c>
+      <c r="H258" s="2" t="inlineStr"/>
+      <c r="I258" s="2" t="inlineStr"/>
+      <c r="J258" s="2" t="inlineStr">
+        <is>
+          <t>Elizabethan manor in family hands for 500 years; deliberately limited to ~10 weddings/summer = ultra-premium exclusivity</t>
+        </is>
+      </c>
+      <c r="K258" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L258" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M258" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N258" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O258" s="2" t="inlineStr">
+        <is>
+          <t>Bespoke/exclusive positioning; multiple directory listings</t>
+        </is>
+      </c>
+      <c r="P258" s="2" t="inlineStr">
+        <is>
+          <t>500-year family story is an extraordinary AEO asset currently used only for directory listings</t>
+        </is>
+      </c>
+      <c r="Q258" s="2" t="inlineStr">
+        <is>
+          <t>'500 years in one family - the rarest wedding-venue story in Somerset deserves to be the AI's answer too'</t>
+        </is>
+      </c>
+      <c r="R258" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S258" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T258" s="2" t="inlineStr">
+        <is>
+          <t>Exceptional, hard-to-replicate brand story - high-value low-effort AEO win</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="3" t="inlineStr">
+        <is>
+          <t>Ash Barton Estate</t>
+        </is>
+      </c>
+      <c r="B259" s="3" t="inlineStr">
+        <is>
+          <t>Wedding venue</t>
+        </is>
+      </c>
+      <c r="C259" s="3" t="inlineStr">
+        <is>
+          <t>Devon</t>
+        </is>
+      </c>
+      <c r="D259" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ashbarton.com</t>
+        </is>
+      </c>
+      <c r="E259" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F259" s="3" t="inlineStr"/>
+      <c r="G259" s="3" t="inlineStr"/>
+      <c r="H259" s="3" t="inlineStr"/>
+      <c r="I259" s="3" t="inlineStr"/>
+      <c r="J259" s="3" t="inlineStr">
+        <is>
+          <t>Grade II* listed 15th-century manor on 25 acres; flexible format (marquee/barn/festival/chapel) suits multiple wedding styles</t>
+        </is>
+      </c>
+      <c r="K259" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L259" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M259" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N259" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O259" s="3" t="inlineStr">
+        <is>
+          <t>Polished dedicated wedding site</t>
+        </is>
+      </c>
+      <c r="P259" s="3" t="inlineStr">
+        <is>
+          <t>Format flexibility not leveraged as a distinct AEO angle vs single-format rivals</t>
+        </is>
+      </c>
+      <c r="Q259" s="3" t="inlineStr">
+        <is>
+          <t>'One venue, four wedding styles' - own that flexibility positioning in AI answers</t>
+        </is>
+      </c>
+      <c r="R259" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S259" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T259" s="3" t="inlineStr"/>
+    </row>
+    <row r="260">
+      <c r="A260" s="3" t="inlineStr">
+        <is>
+          <t>Huntsham Court</t>
+        </is>
+      </c>
+      <c r="B260" s="3" t="inlineStr">
+        <is>
+          <t>Wedding &amp; event venue</t>
+        </is>
+      </c>
+      <c r="C260" s="3" t="inlineStr">
+        <is>
+          <t>Devon (Exmoor border)</t>
+        </is>
+      </c>
+      <c r="D260" s="3" t="inlineStr">
+        <is>
+          <t>https://www.huntshamcourt.co.uk</t>
+        </is>
+      </c>
+      <c r="E260" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F260" s="3" t="inlineStr"/>
+      <c r="G260" s="3" t="inlineStr"/>
+      <c r="H260" s="3" t="inlineStr"/>
+      <c r="I260" s="3" t="inlineStr"/>
+      <c r="J260" s="3" t="inlineStr">
+        <is>
+          <t>Award-winning private-hire estate sleeping 100 across 42 bedrooms; ultra-high-value multi-day event bookings</t>
+        </is>
+      </c>
+      <c r="K260" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L260" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M260" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N260" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O260" s="3" t="inlineStr">
+        <is>
+          <t>Award-winning branding</t>
+        </is>
+      </c>
+      <c r="P260" s="3" t="inlineStr">
+        <is>
+          <t>Scale (100 guests, 42 bedrooms) undersold as the AEO differentiator vs smaller venues</t>
+        </is>
+      </c>
+      <c r="Q260" s="3" t="inlineStr">
+        <is>
+          <t>Target 'large wedding venue Devon' AEO specifically - most rivals can't match the capacity</t>
+        </is>
+      </c>
+      <c r="R260" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S260" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T260" s="3" t="inlineStr"/>
+    </row>
+    <row r="261">
+      <c r="A261" s="3" t="inlineStr">
+        <is>
+          <t>AV Trinity</t>
+        </is>
+      </c>
+      <c r="B261" s="3" t="inlineStr">
+        <is>
+          <t>IFA &amp; mortgage broker</t>
+        </is>
+      </c>
+      <c r="C261" s="3" t="inlineStr">
+        <is>
+          <t>Tunbridge Wells, Kent</t>
+        </is>
+      </c>
+      <c r="D261" s="3" t="inlineStr">
+        <is>
+          <t>https://www.avtrinity.com</t>
+        </is>
+      </c>
+      <c r="E261" s="3" t="inlineStr">
+        <is>
+          <t>info@avtrinity.com</t>
+        </is>
+      </c>
+      <c r="F261" s="3" t="inlineStr">
+        <is>
+          <t>01892 612 500</t>
+        </is>
+      </c>
+      <c r="G261" s="3" t="inlineStr">
+        <is>
+          <t>Karen Vidler (Co-founder, est. 1986)</t>
+        </is>
+      </c>
+      <c r="H261" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/AVTrinity</t>
+        </is>
+      </c>
+      <c r="I261" s="3" t="inlineStr"/>
+      <c r="J261" s="3" t="inlineStr">
+        <is>
+          <t>Independent since 1986 - nearly 40 years serving Kent/Sussex; combined IFA + mortgage broker = higher per-client value</t>
+        </is>
+      </c>
+      <c r="K261" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L261" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M261" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N261" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O261" s="3" t="inlineStr">
+        <is>
+          <t>Community page; Facebook presence</t>
+        </is>
+      </c>
+      <c r="P261" s="3" t="inlineStr">
+        <is>
+          <t>40 years of trust competing with newer, more search-savvy brokers for the same Kent/Sussex clients</t>
+        </is>
+      </c>
+      <c r="Q261" s="3" t="inlineStr">
+        <is>
+          <t>'40 years of independent advice in Tunbridge Wells - the AI answer should say so, not just Unbiased.co.uk'</t>
+        </is>
+      </c>
+      <c r="R261" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S261" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T261" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T254"/>
+  <autoFilter ref="A1:T261"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -22444,7 +23040,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B115"/>
+  <dimension ref="A1:B119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -22464,7 +23060,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>253</v>
+        <v>260</v>
       </c>
     </row>
     <row r="5">
@@ -22487,7 +23083,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Architects</t>
+          <t>Wedding venue</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -22497,21 +23093,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Private dentist</t>
+          <t>Architects</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Wedding venue</t>
+          <t>Private dentist</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10">
@@ -22847,17 +23443,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Dentist / Orthodontics</t>
+          <t>Garden rooms / outbuildings</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Specialist dental/implant clinic</t>
+          <t>Dentist / Orthodontics</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -22867,7 +23463,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Boutique corporate law firm</t>
+          <t>Specialist dental/implant clinic</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -22877,7 +23473,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Cosmetic/aesthetics clinic</t>
+          <t>Boutique corporate law firm</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -22887,7 +23483,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Skin &amp; laser clinic</t>
+          <t>Cosmetic/aesthetics clinic</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -22897,7 +23493,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Mortgage broker / financial adviser</t>
+          <t>Skin &amp; laser clinic</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -22907,7 +23503,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Architects (RIBA chartered)</t>
+          <t>Mortgage broker / financial adviser</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -22917,7 +23513,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Recruitment agency (tech/startups)</t>
+          <t>Architects (RIBA chartered)</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -22927,7 +23523,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Recruitment agency (IT/data)</t>
+          <t>Recruitment agency (tech/startups)</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -22937,7 +23533,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Independent vet (24/7 emergency)</t>
+          <t>Recruitment agency (IT/data)</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -22947,7 +23543,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Interior design studio</t>
+          <t>Independent vet (24/7 emergency)</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -22957,7 +23553,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Letting &amp; estate agent</t>
+          <t>Interior design studio</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -22967,7 +23563,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Cosmetic clinic (injectables)</t>
+          <t>Letting &amp; estate agent</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -22977,7 +23573,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Cosmetic/anti-ageing clinic</t>
+          <t>Cosmetic clinic (injectables)</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -22987,7 +23583,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Yoga &amp; reformer pilates studio</t>
+          <t>Cosmetic/anti-ageing clinic</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -22997,7 +23593,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Reformer pilates studio</t>
+          <t>Yoga &amp; reformer pilates studio</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -23007,7 +23603,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Wealth management</t>
+          <t>Reformer pilates studio</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -23017,7 +23613,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Private tuition &amp; education consultancy</t>
+          <t>Wealth management</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -23027,7 +23623,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Osteopath</t>
+          <t>Private tuition &amp; education consultancy</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -23037,7 +23633,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Design &amp; build / home renovation</t>
+          <t>Osteopath</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -23047,7 +23643,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Builders / building contractor</t>
+          <t>Design &amp; build / home renovation</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -23057,7 +23653,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Home care / live-in care</t>
+          <t>Builders / building contractor</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -23067,7 +23663,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Private day nurseries</t>
+          <t>Home care / live-in care</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -23077,7 +23673,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Personal training &amp; wellness studio</t>
+          <t>Private day nurseries</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -23087,7 +23683,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Mortgage &amp; insurance broker</t>
+          <t>Personal training &amp; wellness studio</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -23097,7 +23693,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Business consultancy</t>
+          <t>Mortgage &amp; insurance broker</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -23107,7 +23703,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Interior designer (period homes)</t>
+          <t>Business consultancy</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -23117,7 +23713,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Landscape design &amp; build</t>
+          <t>Interior designer (period homes)</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -23127,7 +23723,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Interior designer</t>
+          <t>Landscape design &amp; build</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -23137,7 +23733,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Garden design &amp; landscaping</t>
+          <t>Interior designer</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -23147,7 +23743,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Legal recruitment</t>
+          <t>Garden design &amp; landscaping</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -23157,7 +23753,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Independent gym &amp; health club</t>
+          <t>Legal recruitment</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -23167,7 +23763,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Independent gym</t>
+          <t>Independent gym &amp; health club</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -23177,7 +23773,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Physiotherapy (sports)</t>
+          <t>Independent gym</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -23187,7 +23783,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Letting agent / property management</t>
+          <t>Physiotherapy (sports)</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -23197,7 +23793,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Skin clinic</t>
+          <t>Letting agent / property management</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -23207,7 +23803,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Tutoring company</t>
+          <t>Skin clinic</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -23217,7 +23813,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Tutorial college &amp; exam centre</t>
+          <t>Tutoring company</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -23227,7 +23823,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Employment law (disability discrimination)</t>
+          <t>Tutorial college &amp; exam centre</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -23237,7 +23833,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating</t>
+          <t>Employment law (disability discrimination)</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -23247,7 +23843,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Plumbing &amp; heating</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -23257,7 +23853,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Sports physio &amp; massage</t>
+          <t>Plumbing</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -23267,7 +23863,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Chartered surveyors (party wall/building)</t>
+          <t>Sports physio &amp; massage</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -23277,7 +23873,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Chartered surveyors</t>
+          <t>Chartered surveyors (party wall/building)</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -23287,7 +23883,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Chartered building surveyors</t>
+          <t>Chartered surveyors</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -23297,7 +23893,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Osteopathy clinics</t>
+          <t>Chartered building surveyors</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -23307,7 +23903,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Builders / renovations</t>
+          <t>Osteopathy clinics</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -23317,7 +23913,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Private nursery schools</t>
+          <t>Builders / renovations</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -23327,7 +23923,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Private day nursery</t>
+          <t>Private nursery schools</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -23337,7 +23933,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Private GP (membership model)</t>
+          <t>Private day nursery</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -23347,7 +23943,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Sash window restoration</t>
+          <t>Private GP (membership model)</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -23357,7 +23953,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Personal training (1:1)</t>
+          <t>Sash window restoration</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -23367,7 +23963,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Personal training &amp; nutrition coaching</t>
+          <t>Personal training (1:1)</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -23377,7 +23973,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Private nursery/pre-prep school</t>
+          <t>Personal training &amp; nutrition coaching</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -23387,7 +23983,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Independent nursery (Montessori)</t>
+          <t>Private nursery/pre-prep school</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -23397,7 +23993,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Live-in care agency</t>
+          <t>Independent nursery (Montessori)</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -23407,7 +24003,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Law firm (conveyancing/family)</t>
+          <t>Live-in care agency</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -23417,7 +24013,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Architect &amp; interior designer</t>
+          <t>Law firm (conveyancing/family)</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -23427,7 +24023,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Architects / project management</t>
+          <t>Architect &amp; interior designer</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -23437,7 +24033,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>IFA / wealth management</t>
+          <t>Architects / project management</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -23447,7 +24043,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Physiotherapy &amp; clinical Pilates</t>
+          <t>IFA / wealth management</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -23457,7 +24053,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Aesthetics &amp; skin clinic</t>
+          <t>Physiotherapy &amp; clinical Pilates</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -23467,7 +24063,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Wealth management / IFA</t>
+          <t>Aesthetics &amp; skin clinic</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -23477,7 +24073,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>IFA / financial planning</t>
+          <t>Wealth management / IFA</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -23487,7 +24083,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Wealth management &amp; employee benefits</t>
+          <t>IFA / financial planning</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -23497,7 +24093,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Dermatology clinic</t>
+          <t>Wealth management &amp; employee benefits</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -23507,7 +24103,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Pilates studio (multi-site)</t>
+          <t>Dermatology clinic</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -23517,7 +24113,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Private nursery (Montessori, multi-site)</t>
+          <t>Pilates studio (multi-site)</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -23527,7 +24123,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Law firm (wills &amp; probate)</t>
+          <t>Private nursery (Montessori, multi-site)</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -23537,7 +24133,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Business/technical consultancy</t>
+          <t>Law firm (wills &amp; probate)</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -23547,7 +24143,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Architects &amp; interior design</t>
+          <t>Business/technical consultancy</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -23557,7 +24153,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Private/NHS dentist</t>
+          <t>Architects &amp; interior design</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -23567,10 +24163,50 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
+          <t>Private/NHS dentist</t>
+        </is>
+      </c>
+      <c r="B115" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
           <t>Removals company</t>
         </is>
       </c>
-      <c r="B115" t="n">
+      <c r="B116" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Driveways &amp; landscaping</t>
+        </is>
+      </c>
+      <c r="B117" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Wedding &amp; event venue</t>
+        </is>
+      </c>
+      <c r="B118" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>IFA &amp; mortgage broker</t>
+        </is>
+      </c>
+      <c r="B119" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 18: +5 prospects (265 total) - Sevenoaks/Tunbridge Wells GP, aesthetics, vets, PT
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$261</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$266</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T261"/>
+  <dimension ref="A1:T266"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -23028,8 +23028,444 @@
       </c>
       <c r="T261" s="3" t="inlineStr"/>
     </row>
+    <row r="262">
+      <c r="A262" s="3" t="inlineStr">
+        <is>
+          <t>The Private GP Clinic</t>
+        </is>
+      </c>
+      <c r="B262" s="3" t="inlineStr">
+        <is>
+          <t>Private GP</t>
+        </is>
+      </c>
+      <c r="C262" s="3" t="inlineStr">
+        <is>
+          <t>Underriver, Sevenoaks, Kent</t>
+        </is>
+      </c>
+      <c r="D262" s="3" t="inlineStr">
+        <is>
+          <t>https://www.theprivategpclinic.co.uk</t>
+        </is>
+      </c>
+      <c r="E262" s="3" t="inlineStr">
+        <is>
+          <t>info@theprivategpclinic.co.uk</t>
+        </is>
+      </c>
+      <c r="F262" s="3" t="inlineStr">
+        <is>
+          <t>01732 835 212</t>
+        </is>
+      </c>
+      <c r="G262" s="3" t="inlineStr"/>
+      <c r="H262" s="3" t="inlineStr"/>
+      <c r="I262" s="3" t="inlineStr"/>
+      <c r="J262" s="3" t="inlineStr">
+        <is>
+          <t>Independent private GP in rural Sevenoaks catchment; self-pay consultations with Saturday availability = strong convenience differentiator</t>
+        </is>
+      </c>
+      <c r="K262" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L262" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M262" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N262" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O262" s="3" t="inlineStr">
+        <is>
+          <t>Weekend opening hours promoted</t>
+        </is>
+      </c>
+      <c r="P262" s="3" t="inlineStr">
+        <is>
+          <t>KIMS Hospital and Nuffield Health private-GP brands dominate Kent private-GP search with hospital-scale marketing</t>
+        </is>
+      </c>
+      <c r="Q262" s="3" t="inlineStr">
+        <is>
+          <t>'Saturday appointments, no hospital wait - own that convenience story in AI answers'</t>
+        </is>
+      </c>
+      <c r="R262" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S262" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T262" s="3" t="inlineStr"/>
+    </row>
+    <row r="263">
+      <c r="A263" s="3" t="inlineStr">
+        <is>
+          <t>Dr Anita Aesthetics</t>
+        </is>
+      </c>
+      <c r="B263" s="3" t="inlineStr">
+        <is>
+          <t>Aesthetics clinic</t>
+        </is>
+      </c>
+      <c r="C263" s="3" t="inlineStr">
+        <is>
+          <t>Mount Ephraim Rd, Tunbridge Wells (serves Sevenoaks)</t>
+        </is>
+      </c>
+      <c r="D263" s="3" t="inlineStr">
+        <is>
+          <t>https://www.dranitaaesthetics.com</t>
+        </is>
+      </c>
+      <c r="E263" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F263" s="3" t="inlineStr"/>
+      <c r="G263" s="3" t="inlineStr">
+        <is>
+          <t>Dr Anita Madi (Founder, GMC public health specialist)</t>
+        </is>
+      </c>
+      <c r="H263" s="3" t="inlineStr"/>
+      <c r="I263" s="3" t="inlineStr"/>
+      <c r="J263" s="3" t="inlineStr">
+        <is>
+          <t>Doctor-led, GMC-registered aesthetic doctor serving two wealthy Kent towns from one clinic; genuine medical credential differentiator</t>
+        </is>
+      </c>
+      <c r="K263" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L263" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M263" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N263" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O263" s="3" t="inlineStr">
+        <is>
+          <t>Dual-town service pages (Tunbridge Wells + Sevenoaks)</t>
+        </is>
+      </c>
+      <c r="P263" s="3" t="inlineStr">
+        <is>
+          <t>Dual-town SEO pages exist but AI-answer citations still open for either town</t>
+        </is>
+      </c>
+      <c r="Q263" s="3" t="inlineStr">
+        <is>
+          <t>'A GMC-registered doctor doing your Botox' - the exact trust signal AEO content should carry</t>
+        </is>
+      </c>
+      <c r="R263" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S263" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T263" s="3" t="inlineStr"/>
+    </row>
+    <row r="264">
+      <c r="A264" s="4" t="inlineStr">
+        <is>
+          <t>Priory Lodge Vets</t>
+        </is>
+      </c>
+      <c r="B264" s="4" t="inlineStr">
+        <is>
+          <t>Independent vet</t>
+        </is>
+      </c>
+      <c r="C264" s="4" t="inlineStr">
+        <is>
+          <t>Pembury Road, Tonbridge, Kent</t>
+        </is>
+      </c>
+      <c r="D264" s="4" t="inlineStr">
+        <is>
+          <t>https://www.plvet.co.uk</t>
+        </is>
+      </c>
+      <c r="E264" s="4" t="inlineStr">
+        <is>
+          <t>info@plvet.co.uk</t>
+        </is>
+      </c>
+      <c r="F264" s="4" t="inlineStr">
+        <is>
+          <t>01732 353 668</t>
+        </is>
+      </c>
+      <c r="G264" s="4" t="inlineStr"/>
+      <c r="H264" s="4" t="inlineStr"/>
+      <c r="I264" s="4" t="inlineStr">
+        <is>
+          <t>facebook.com/p/Priory-Lodge-Vets-100057128660958</t>
+        </is>
+      </c>
+      <c r="J264" s="4" t="inlineStr">
+        <is>
+          <t>Firmly independent small-animal practice in Tonbridge; explicit independence positioning vs corporate rivals</t>
+        </is>
+      </c>
+      <c r="K264" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L264" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M264" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N264" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O264" s="4" t="inlineStr">
+        <is>
+          <t>Facebook presence</t>
+        </is>
+      </c>
+      <c r="P264" s="4" t="inlineStr">
+        <is>
+          <t>'Firmly independent' claim not yet the AI-cited answer against corporate vet groups</t>
+        </is>
+      </c>
+      <c r="Q264" s="4" t="inlineStr">
+        <is>
+          <t>Own 'independent vet Tonbridge' - their own positioning statement as the AEO target</t>
+        </is>
+      </c>
+      <c r="R264" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S264" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T264" s="4" t="inlineStr"/>
+    </row>
+    <row r="265">
+      <c r="A265" s="4" t="inlineStr">
+        <is>
+          <t>Hollow Rock Fitness</t>
+        </is>
+      </c>
+      <c r="B265" s="4" t="inlineStr">
+        <is>
+          <t>Personal training gym</t>
+        </is>
+      </c>
+      <c r="C265" s="4" t="inlineStr">
+        <is>
+          <t>London Road, Riverhead, Sevenoaks</t>
+        </is>
+      </c>
+      <c r="D265" s="4" t="inlineStr">
+        <is>
+          <t>https://www.hollowrockfitness.com</t>
+        </is>
+      </c>
+      <c r="E265" s="4" t="inlineStr">
+        <is>
+          <t>JFARMER101@ICLOUD.COM</t>
+        </is>
+      </c>
+      <c r="F265" s="4" t="inlineStr">
+        <is>
+          <t>07887 711664</t>
+        </is>
+      </c>
+      <c r="G265" s="4" t="inlineStr">
+        <is>
+          <t>James Farmer (Founder, 24+ years training experience)</t>
+        </is>
+      </c>
+      <c r="H265" s="4" t="inlineStr"/>
+      <c r="I265" s="4" t="inlineStr">
+        <is>
+          <t>instagram.com/hollowrockfitness</t>
+        </is>
+      </c>
+      <c r="J265" s="4" t="inlineStr">
+        <is>
+          <t>Founder-led PT gym with nearly a quarter-century of coaching experience; ongoing client packages in affluent Sevenoaks</t>
+        </is>
+      </c>
+      <c r="K265" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L265" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M265" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N265" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O265" s="4" t="inlineStr">
+        <is>
+          <t>ClassPass/Fresha booking listings</t>
+        </is>
+      </c>
+      <c r="P265" s="4" t="inlineStr">
+        <is>
+          <t>Booking-platform discovery means paying commission on clients the gym could own directly</t>
+        </is>
+      </c>
+      <c r="Q265" s="4" t="inlineStr">
+        <is>
+          <t>'24 years of coaching experience - stop renting your leads from ClassPass, own the search instead'</t>
+        </is>
+      </c>
+      <c r="R265" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S265" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T265" s="4" t="inlineStr">
+        <is>
+          <t>Personal iCloud email - confirm before outreach, may prefer phone contact</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="4" t="inlineStr">
+        <is>
+          <t>Thrive Personal Training</t>
+        </is>
+      </c>
+      <c r="B266" s="4" t="inlineStr">
+        <is>
+          <t>Personal training gym</t>
+        </is>
+      </c>
+      <c r="C266" s="4" t="inlineStr">
+        <is>
+          <t>Tunbridge Wells, Kent</t>
+        </is>
+      </c>
+      <c r="D266" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thrive-personaltraining.co.uk</t>
+        </is>
+      </c>
+      <c r="E266" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F266" s="4" t="inlineStr"/>
+      <c r="G266" s="4" t="inlineStr">
+        <is>
+          <t>Luke French (Owner)</t>
+        </is>
+      </c>
+      <c r="H266" s="4" t="inlineStr"/>
+      <c r="I266" s="4" t="inlineStr"/>
+      <c r="J266" s="4" t="inlineStr">
+        <is>
+          <t>Owner-led, second Tunbridge Wells location opened - proven growth and reinvestment in the local market</t>
+        </is>
+      </c>
+      <c r="K266" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L266" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M266" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N266" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O266" s="4" t="inlineStr">
+        <is>
+          <t>Two-site expansion</t>
+        </is>
+      </c>
+      <c r="P266" s="4" t="inlineStr">
+        <is>
+          <t>Second-site growth not matched by dominant local search share</t>
+        </is>
+      </c>
+      <c r="Q266" s="4" t="inlineStr">
+        <is>
+          <t>'You've proven the model works twice - now make sure AI recommends both locations'</t>
+        </is>
+      </c>
+      <c r="R266" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S266" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T266" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T261"/>
+  <autoFilter ref="A1:T266"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -23040,7 +23476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B119"/>
+  <dimension ref="A1:B120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -23060,7 +23496,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>260</v>
+        <v>265</v>
       </c>
     </row>
     <row r="5">
@@ -23117,7 +23553,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11">
@@ -23133,17 +23569,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Physiotherapy clinic</t>
+          <t>Aesthetics clinic</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Chartered accountants</t>
+          <t>Physiotherapy clinic</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -23153,7 +23589,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Aesthetics clinic</t>
+          <t>Chartered accountants</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -23163,7 +23599,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>IT support / MSP</t>
+          <t>Private GP</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -23173,17 +23609,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Mortgage broker</t>
+          <t>IT support / MSP</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Solar installer</t>
+          <t>Mortgage broker</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -23193,7 +23629,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Private GP</t>
+          <t>Solar installer</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -23453,17 +23889,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Dentist / Orthodontics</t>
+          <t>Personal training gym</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Specialist dental/implant clinic</t>
+          <t>Dentist / Orthodontics</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -23473,7 +23909,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Boutique corporate law firm</t>
+          <t>Specialist dental/implant clinic</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -23483,7 +23919,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Cosmetic/aesthetics clinic</t>
+          <t>Boutique corporate law firm</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -23493,7 +23929,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Skin &amp; laser clinic</t>
+          <t>Cosmetic/aesthetics clinic</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -23503,7 +23939,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Mortgage broker / financial adviser</t>
+          <t>Skin &amp; laser clinic</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -23513,7 +23949,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Architects (RIBA chartered)</t>
+          <t>Mortgage broker / financial adviser</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -23523,7 +23959,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Recruitment agency (tech/startups)</t>
+          <t>Architects (RIBA chartered)</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -23533,7 +23969,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Recruitment agency (IT/data)</t>
+          <t>Recruitment agency (tech/startups)</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -23543,7 +23979,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Independent vet (24/7 emergency)</t>
+          <t>Recruitment agency (IT/data)</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -23553,7 +23989,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Interior design studio</t>
+          <t>Independent vet (24/7 emergency)</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -23563,7 +23999,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Letting &amp; estate agent</t>
+          <t>Interior design studio</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -23573,7 +24009,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Cosmetic clinic (injectables)</t>
+          <t>Letting &amp; estate agent</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -23583,7 +24019,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Cosmetic/anti-ageing clinic</t>
+          <t>Cosmetic clinic (injectables)</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -23593,7 +24029,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Yoga &amp; reformer pilates studio</t>
+          <t>Cosmetic/anti-ageing clinic</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -23603,7 +24039,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Reformer pilates studio</t>
+          <t>Yoga &amp; reformer pilates studio</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -23613,7 +24049,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Wealth management</t>
+          <t>Reformer pilates studio</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -23623,7 +24059,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Private tuition &amp; education consultancy</t>
+          <t>Wealth management</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -23633,7 +24069,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Osteopath</t>
+          <t>Private tuition &amp; education consultancy</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -23643,7 +24079,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Design &amp; build / home renovation</t>
+          <t>Osteopath</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -23653,7 +24089,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Builders / building contractor</t>
+          <t>Design &amp; build / home renovation</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -23663,7 +24099,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Home care / live-in care</t>
+          <t>Builders / building contractor</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -23673,7 +24109,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Private day nurseries</t>
+          <t>Home care / live-in care</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -23683,7 +24119,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Personal training &amp; wellness studio</t>
+          <t>Private day nurseries</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -23693,7 +24129,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Mortgage &amp; insurance broker</t>
+          <t>Personal training &amp; wellness studio</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -23703,7 +24139,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Business consultancy</t>
+          <t>Mortgage &amp; insurance broker</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -23713,7 +24149,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Interior designer (period homes)</t>
+          <t>Business consultancy</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -23723,7 +24159,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Landscape design &amp; build</t>
+          <t>Interior designer (period homes)</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -23733,7 +24169,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Interior designer</t>
+          <t>Landscape design &amp; build</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -23743,7 +24179,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Garden design &amp; landscaping</t>
+          <t>Interior designer</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -23753,7 +24189,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Legal recruitment</t>
+          <t>Garden design &amp; landscaping</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -23763,7 +24199,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Independent gym &amp; health club</t>
+          <t>Legal recruitment</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -23773,7 +24209,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Independent gym</t>
+          <t>Independent gym &amp; health club</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -23783,7 +24219,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Physiotherapy (sports)</t>
+          <t>Independent gym</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -23793,7 +24229,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Letting agent / property management</t>
+          <t>Physiotherapy (sports)</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -23803,7 +24239,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Skin clinic</t>
+          <t>Letting agent / property management</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -23813,7 +24249,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Tutoring company</t>
+          <t>Skin clinic</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -23823,7 +24259,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Tutorial college &amp; exam centre</t>
+          <t>Tutoring company</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -23833,7 +24269,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Employment law (disability discrimination)</t>
+          <t>Tutorial college &amp; exam centre</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -23843,7 +24279,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating</t>
+          <t>Employment law (disability discrimination)</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -23853,7 +24289,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Plumbing &amp; heating</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -23863,7 +24299,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Sports physio &amp; massage</t>
+          <t>Plumbing</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -23873,7 +24309,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Chartered surveyors (party wall/building)</t>
+          <t>Sports physio &amp; massage</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -23883,7 +24319,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Chartered surveyors</t>
+          <t>Chartered surveyors (party wall/building)</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -23893,7 +24329,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Chartered building surveyors</t>
+          <t>Chartered surveyors</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -23903,7 +24339,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Osteopathy clinics</t>
+          <t>Chartered building surveyors</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -23913,7 +24349,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Builders / renovations</t>
+          <t>Osteopathy clinics</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -23923,7 +24359,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Private nursery schools</t>
+          <t>Builders / renovations</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -23933,7 +24369,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Private day nursery</t>
+          <t>Private nursery schools</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -23943,7 +24379,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Private GP (membership model)</t>
+          <t>Private day nursery</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -23953,7 +24389,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Sash window restoration</t>
+          <t>Private GP (membership model)</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -23963,7 +24399,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Personal training (1:1)</t>
+          <t>Sash window restoration</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -23973,7 +24409,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Personal training &amp; nutrition coaching</t>
+          <t>Personal training (1:1)</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -23983,7 +24419,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Private nursery/pre-prep school</t>
+          <t>Personal training &amp; nutrition coaching</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -23993,7 +24429,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Independent nursery (Montessori)</t>
+          <t>Private nursery/pre-prep school</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -24003,7 +24439,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Live-in care agency</t>
+          <t>Independent nursery (Montessori)</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -24013,7 +24449,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Law firm (conveyancing/family)</t>
+          <t>Live-in care agency</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -24023,7 +24459,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Architect &amp; interior designer</t>
+          <t>Law firm (conveyancing/family)</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -24033,7 +24469,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Architects / project management</t>
+          <t>Architect &amp; interior designer</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -24043,7 +24479,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>IFA / wealth management</t>
+          <t>Architects / project management</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -24053,7 +24489,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Physiotherapy &amp; clinical Pilates</t>
+          <t>IFA / wealth management</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -24063,7 +24499,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Aesthetics &amp; skin clinic</t>
+          <t>Physiotherapy &amp; clinical Pilates</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -24073,7 +24509,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Wealth management / IFA</t>
+          <t>Aesthetics &amp; skin clinic</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -24083,7 +24519,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>IFA / financial planning</t>
+          <t>Wealth management / IFA</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -24093,7 +24529,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Wealth management &amp; employee benefits</t>
+          <t>IFA / financial planning</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -24103,7 +24539,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Dermatology clinic</t>
+          <t>Wealth management &amp; employee benefits</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -24113,7 +24549,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Pilates studio (multi-site)</t>
+          <t>Dermatology clinic</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -24123,7 +24559,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Private nursery (Montessori, multi-site)</t>
+          <t>Pilates studio (multi-site)</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -24133,7 +24569,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Law firm (wills &amp; probate)</t>
+          <t>Private nursery (Montessori, multi-site)</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -24143,7 +24579,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Business/technical consultancy</t>
+          <t>Law firm (wills &amp; probate)</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -24153,7 +24589,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Architects &amp; interior design</t>
+          <t>Business/technical consultancy</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -24163,7 +24599,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Private/NHS dentist</t>
+          <t>Architects &amp; interior design</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -24173,7 +24609,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Removals company</t>
+          <t>Private/NHS dentist</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -24183,7 +24619,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Driveways &amp; landscaping</t>
+          <t>Removals company</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -24193,7 +24629,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Wedding &amp; event venue</t>
+          <t>Driveways &amp; landscaping</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -24203,10 +24639,20 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
+          <t>Wedding &amp; event venue</t>
+        </is>
+      </c>
+      <c r="B119" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
           <t>IFA &amp; mortgage broker</t>
         </is>
       </c>
-      <c r="B119" t="n">
+      <c r="B120" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 19: +4 prospects (269 total) - Cotswolds towns, Marlborough, wedding films, Bristol litigation
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$266</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$270</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T266"/>
+  <dimension ref="A1:T270"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -23464,8 +23464,364 @@
       </c>
       <c r="T266" s="4" t="inlineStr"/>
     </row>
+    <row r="267">
+      <c r="A267" s="3" t="inlineStr">
+        <is>
+          <t>Tayler and Fletcher</t>
+        </is>
+      </c>
+      <c r="B267" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent &amp; chartered surveyors</t>
+        </is>
+      </c>
+      <c r="C267" s="3" t="inlineStr">
+        <is>
+          <t>Stow-on-the-Wold, Bourton-on-the-Water, Chipping Norton</t>
+        </is>
+      </c>
+      <c r="D267" s="3" t="inlineStr">
+        <is>
+          <t>https://www.taylerandfletcher.co.uk</t>
+        </is>
+      </c>
+      <c r="E267" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F267" s="3" t="inlineStr">
+        <is>
+          <t>01451 798 056</t>
+        </is>
+      </c>
+      <c r="G267" s="3" t="inlineStr"/>
+      <c r="H267" s="3" t="inlineStr"/>
+      <c r="I267" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/TaylerandFletcher</t>
+        </is>
+      </c>
+      <c r="J267" s="3" t="inlineStr">
+        <is>
+          <t>Leading independent covering the Cotswolds' most tourist-famous villages; residential + rural/agricultural property = high average fees</t>
+        </is>
+      </c>
+      <c r="K267" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L267" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M267" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N267" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O267" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence; 3-office coverage</t>
+        </is>
+      </c>
+      <c r="P267" s="3" t="inlineStr">
+        <is>
+          <t>Corporate premium brands (Knight Frank, Savills) also target Stow/Bourton for second-home buyers</t>
+        </is>
+      </c>
+      <c r="Q267" s="3" t="inlineStr">
+        <is>
+          <t>'Cotswolds second-home buyers research online for months - be the independent name AI recommends'</t>
+        </is>
+      </c>
+      <c r="R267" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S267" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T267" s="3" t="inlineStr"/>
+    </row>
+    <row r="268">
+      <c r="A268" s="3" t="inlineStr">
+        <is>
+          <t>Birkmyre Property Consultants</t>
+        </is>
+      </c>
+      <c r="B268" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C268" s="3" t="inlineStr">
+        <is>
+          <t>Marlborough, Wiltshire</t>
+        </is>
+      </c>
+      <c r="D268" s="3" t="inlineStr">
+        <is>
+          <t>https://www.birkmyrepc.co.uk</t>
+        </is>
+      </c>
+      <c r="E268" s="3" t="inlineStr">
+        <is>
+          <t>info@birkmyrepc.co.uk</t>
+        </is>
+      </c>
+      <c r="F268" s="3" t="inlineStr">
+        <is>
+          <t>01672 516 619</t>
+        </is>
+      </c>
+      <c r="G268" s="3" t="inlineStr">
+        <is>
+          <t>Dominic Birkmyre (Founder, MRICS, est. 2009)</t>
+        </is>
+      </c>
+      <c r="H268" s="3" t="inlineStr"/>
+      <c r="I268" s="3" t="inlineStr"/>
+      <c r="J268" s="3" t="inlineStr">
+        <is>
+          <t>RICS-qualified founder with 25 years' experience; village/country property specialism across Wiltshire/Hampshire/Berkshire</t>
+        </is>
+      </c>
+      <c r="K268" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L268" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M268" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N268" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O268" s="3" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P268" s="3" t="inlineStr">
+        <is>
+          <t>Fine &amp; Country and Winkworth national brands dominate Marlborough search visibility</t>
+        </is>
+      </c>
+      <c r="Q268" s="3" t="inlineStr">
+        <is>
+          <t>'RICS-qualified, 25 years of country property expertise - the AI answer should say so'</t>
+        </is>
+      </c>
+      <c r="R268" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S268" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T268" s="3" t="inlineStr"/>
+    </row>
+    <row r="269">
+      <c r="A269" s="4" t="inlineStr">
+        <is>
+          <t>Wedding Films London</t>
+        </is>
+      </c>
+      <c r="B269" s="4" t="inlineStr">
+        <is>
+          <t>Wedding photography &amp; videography</t>
+        </is>
+      </c>
+      <c r="C269" s="4" t="inlineStr">
+        <is>
+          <t>South London (serves London/Surrey/Kent/Herts/Essex)</t>
+        </is>
+      </c>
+      <c r="D269" s="4" t="inlineStr">
+        <is>
+          <t>https://weddingfilmslondon.co.uk</t>
+        </is>
+      </c>
+      <c r="E269" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F269" s="4" t="inlineStr"/>
+      <c r="G269" s="4" t="inlineStr">
+        <is>
+          <t>Founder &amp; Kate (husband-and-wife team, est. 2008)</t>
+        </is>
+      </c>
+      <c r="H269" s="4" t="inlineStr">
+        <is>
+          <t>facebook.com/wedding.films.london</t>
+        </is>
+      </c>
+      <c r="I269" s="4" t="inlineStr"/>
+      <c r="J269" s="4" t="inlineStr">
+        <is>
+          <t>Award-winning team, 300+ weddings filmed since 2008; premium packages £2-5k+ per wedding across a huge catchment</t>
+        </is>
+      </c>
+      <c r="K269" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L269" s="4" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M269" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N269" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O269" s="4" t="inlineStr">
+        <is>
+          <t>Award-winning branding; wide-area coverage</t>
+        </is>
+      </c>
+      <c r="P269" s="4" t="inlineStr">
+        <is>
+          <t>Wide catchment claim not matched by per-county search dominance</t>
+        </is>
+      </c>
+      <c r="Q269" s="4" t="inlineStr">
+        <is>
+          <t>Per-county AEO content to actually own the whole claimed coverage area</t>
+        </is>
+      </c>
+      <c r="R269" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S269" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T269" s="4" t="inlineStr"/>
+    </row>
+    <row r="270">
+      <c r="A270" s="3" t="inlineStr">
+        <is>
+          <t>Estate Legal</t>
+        </is>
+      </c>
+      <c r="B270" s="3" t="inlineStr">
+        <is>
+          <t>Commercial property litigation law firm</t>
+        </is>
+      </c>
+      <c r="C270" s="3" t="inlineStr">
+        <is>
+          <t>Whiteladies Road, Clifton, Bristol (+ London)</t>
+        </is>
+      </c>
+      <c r="D270" s="3" t="inlineStr">
+        <is>
+          <t>https://estatelegal.co.uk</t>
+        </is>
+      </c>
+      <c r="E270" s="3" t="inlineStr">
+        <is>
+          <t>amyrudrum@estatelegal.co.uk</t>
+        </is>
+      </c>
+      <c r="F270" s="3" t="inlineStr">
+        <is>
+          <t>07825 336 680</t>
+        </is>
+      </c>
+      <c r="G270" s="3" t="inlineStr">
+        <is>
+          <t>Bonnie Martin &amp; Amy Rudrum (Founders, ex-national-firm partners)</t>
+        </is>
+      </c>
+      <c r="H270" s="3" t="inlineStr"/>
+      <c r="I270" s="3" t="inlineStr"/>
+      <c r="J270" s="3" t="inlineStr">
+        <is>
+          <t>Boutique property litigation specialists with 50+ years combined experience; niche expertise (Pubs Code, rent review) = high-value instructions</t>
+        </is>
+      </c>
+      <c r="K270" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L270" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M270" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N270" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O270" s="3" t="inlineStr">
+        <is>
+          <t>Detailed niche-service SEO pages (Pubs Code, dilapidations, rent review)</t>
+        </is>
+      </c>
+      <c r="P270" s="3" t="inlineStr">
+        <is>
+          <t>Deep niche content exists but AI-answer citations for these specific legal queries still open</t>
+        </is>
+      </c>
+      <c r="Q270" s="3" t="inlineStr">
+        <is>
+          <t>'You've written the definitive pages on Pubs Code disputes - let's make AI cite them, not just index them'</t>
+        </is>
+      </c>
+      <c r="R270" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S270" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T270" s="3" t="inlineStr">
+        <is>
+          <t>Sophisticated, marketing-literate founders - lead with AEO specifics, not basics</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T266"/>
+  <autoFilter ref="A1:T270"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -23476,7 +23832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B120"/>
+  <dimension ref="A1:B123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -23496,7 +23852,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>265</v>
+        <v>269</v>
       </c>
     </row>
     <row r="5">
@@ -23513,7 +23869,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7">
@@ -24653,6 +25009,36 @@
         </is>
       </c>
       <c r="B120" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Estate agent &amp; chartered surveyors</t>
+        </is>
+      </c>
+      <c r="B121" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Wedding photography &amp; videography</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Commercial property litigation law firm</t>
+        </is>
+      </c>
+      <c r="B123" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 20: +7 prospects (276 total) - Whitstable, Bristol architects, Sussex solar, recruitment
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$270</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$277</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T270"/>
+  <dimension ref="A1:T277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -23820,8 +23820,620 @@
         </is>
       </c>
     </row>
+    <row r="271">
+      <c r="A271" s="3" t="inlineStr">
+        <is>
+          <t>Spiller Brooks Estate Agents</t>
+        </is>
+      </c>
+      <c r="B271" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C271" s="3" t="inlineStr">
+        <is>
+          <t>Whitstable, Kent</t>
+        </is>
+      </c>
+      <c r="D271" s="3" t="inlineStr">
+        <is>
+          <t>https://spillerbrooks.co.uk</t>
+        </is>
+      </c>
+      <c r="E271" s="3" t="inlineStr">
+        <is>
+          <t>info@spillerbrooks.co.uk</t>
+        </is>
+      </c>
+      <c r="F271" s="3" t="inlineStr">
+        <is>
+          <t>01227 272 155</t>
+        </is>
+      </c>
+      <c r="G271" s="3" t="inlineStr">
+        <is>
+          <t>Nikki Spiller (Owner, 17+ years experience)</t>
+        </is>
+      </c>
+      <c r="H271" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/SpillerbrooksEstateAgents</t>
+        </is>
+      </c>
+      <c r="I271" s="3" t="inlineStr"/>
+      <c r="J271" s="3" t="inlineStr">
+        <is>
+          <t>Truly independent, rebranded from Mark Smith Estate Agents; named 'one of the best in the UK'; coastal Kent premium market</t>
+        </is>
+      </c>
+      <c r="K271" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L271" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M271" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N271" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O271" s="3" t="inlineStr">
+        <is>
+          <t>National award recognition; Facebook presence</t>
+        </is>
+      </c>
+      <c r="P271" s="3" t="inlineStr">
+        <is>
+          <t>National award status not converted into local/AI-search dominance for Whitstable searches</t>
+        </is>
+      </c>
+      <c r="Q271" s="3" t="inlineStr">
+        <is>
+          <t>'Named one of the UK's best agents - make sure that's what AI says for "estate agent Whitstable"'</t>
+        </is>
+      </c>
+      <c r="R271" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S271" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T271" s="3" t="inlineStr"/>
+    </row>
+    <row r="272">
+      <c r="A272" s="4" t="inlineStr">
+        <is>
+          <t>County Estate Agents</t>
+        </is>
+      </c>
+      <c r="B272" s="4" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C272" s="4" t="inlineStr">
+        <is>
+          <t>Whitstable (serves Tankerton/Herne Bay/Faversham/Canterbury)</t>
+        </is>
+      </c>
+      <c r="D272" s="4" t="inlineStr">
+        <is>
+          <t>https://www.countyestateagents.co.uk</t>
+        </is>
+      </c>
+      <c r="E272" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F272" s="4" t="inlineStr"/>
+      <c r="G272" s="4" t="inlineStr"/>
+      <c r="H272" s="4" t="inlineStr"/>
+      <c r="I272" s="4" t="inlineStr"/>
+      <c r="J272" s="4" t="inlineStr">
+        <is>
+          <t>Long-established independent covering 4 East Kent coastal/market towns; residential, coastal and commercial property</t>
+        </is>
+      </c>
+      <c r="K272" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L272" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M272" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N272" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O272" s="4" t="inlineStr">
+        <is>
+          <t>Multi-town coverage</t>
+        </is>
+      </c>
+      <c r="P272" s="4" t="inlineStr">
+        <is>
+          <t>Wide catchment but single-brand search visibility thin per town</t>
+        </is>
+      </c>
+      <c r="Q272" s="4" t="inlineStr">
+        <is>
+          <t>Per-town AEO content to actually own all 4 claimed markets</t>
+        </is>
+      </c>
+      <c r="R272" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S272" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T272" s="4" t="inlineStr"/>
+    </row>
+    <row r="273">
+      <c r="A273" s="4" t="inlineStr">
+        <is>
+          <t>Breadings</t>
+        </is>
+      </c>
+      <c r="B273" s="4" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C273" s="4" t="inlineStr">
+        <is>
+          <t>Whitstable/East Kent</t>
+        </is>
+      </c>
+      <c r="D273" s="4" t="inlineStr">
+        <is>
+          <t>via directory listing</t>
+        </is>
+      </c>
+      <c r="E273" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F273" s="4" t="inlineStr"/>
+      <c r="G273" s="4" t="inlineStr"/>
+      <c r="H273" s="4" t="inlineStr"/>
+      <c r="I273" s="4" t="inlineStr"/>
+      <c r="J273" s="4" t="inlineStr">
+        <is>
+          <t>Private independent trading 70+ years - genuinely rare longevity in East Kent property market</t>
+        </is>
+      </c>
+      <c r="K273" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L273" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M273" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N273" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O273" s="4" t="inlineStr">
+        <is>
+          <t>70-year heritage</t>
+        </is>
+      </c>
+      <c r="P273" s="4" t="inlineStr">
+        <is>
+          <t>Decades of trust untranslated into modern AI-search visibility</t>
+        </is>
+      </c>
+      <c r="Q273" s="4" t="inlineStr">
+        <is>
+          <t>'70 years of Kentish property trust deserves to be the AI's answer too'</t>
+        </is>
+      </c>
+      <c r="R273" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S273" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T273" s="4" t="inlineStr">
+        <is>
+          <t>Confirm live website before outreach</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="4" t="inlineStr">
+        <is>
+          <t>Clifton Architects</t>
+        </is>
+      </c>
+      <c r="B274" s="4" t="inlineStr">
+        <is>
+          <t>Architects</t>
+        </is>
+      </c>
+      <c r="C274" s="4" t="inlineStr">
+        <is>
+          <t>Cliftonwood, Bristol</t>
+        </is>
+      </c>
+      <c r="D274" s="4" t="inlineStr">
+        <is>
+          <t>http://www.cliftonarchitects.com</t>
+        </is>
+      </c>
+      <c r="E274" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F274" s="4" t="inlineStr"/>
+      <c r="G274" s="4" t="inlineStr">
+        <is>
+          <t>Amanda Webb (Founder, 30+ years experience)</t>
+        </is>
+      </c>
+      <c r="H274" s="4" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/amanda-webb-052b455a</t>
+        </is>
+      </c>
+      <c r="I274" s="4" t="inlineStr"/>
+      <c r="J274" s="4" t="inlineStr">
+        <is>
+          <t>Founder with 20 years at a prior Bristol practice before establishing her own; deep local residential experience</t>
+        </is>
+      </c>
+      <c r="K274" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L274" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M274" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N274" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O274" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P274" s="4" t="inlineStr">
+        <is>
+          <t>30 years of Bristol residential expertise invisible in modern search</t>
+        </is>
+      </c>
+      <c r="Q274" s="4" t="inlineStr">
+        <is>
+          <t>Portfolio-driven AEO content leveraging three decades of local project history</t>
+        </is>
+      </c>
+      <c r="R274" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S274" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T274" s="4" t="inlineStr"/>
+    </row>
+    <row r="275">
+      <c r="A275" s="3" t="inlineStr">
+        <is>
+          <t>Sussex Solar</t>
+        </is>
+      </c>
+      <c r="B275" s="3" t="inlineStr">
+        <is>
+          <t>Solar installer</t>
+        </is>
+      </c>
+      <c r="C275" s="3" t="inlineStr">
+        <is>
+          <t>Horsham, West Sussex (serves Sussex/Surrey/Kent/Hampshire)</t>
+        </is>
+      </c>
+      <c r="D275" s="3" t="inlineStr">
+        <is>
+          <t>https://sussexsolar.com</t>
+        </is>
+      </c>
+      <c r="E275" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F275" s="3" t="inlineStr">
+        <is>
+          <t>01403 371 000</t>
+        </is>
+      </c>
+      <c r="G275" s="3" t="inlineStr">
+        <is>
+          <t>Andy Baxter (Founder, est. 2005)</t>
+        </is>
+      </c>
+      <c r="H275" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/p/Sussex-Solar-Ltd-100043388126281</t>
+        </is>
+      </c>
+      <c r="I275" s="3" t="inlineStr"/>
+      <c r="J275" s="3" t="inlineStr">
+        <is>
+          <t>Family-owned since 2005, MCS-certified across 4 counties; solar installs £8-20k each in a booming demand market</t>
+        </is>
+      </c>
+      <c r="K275" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L275" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M275" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N275" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O275" s="3" t="inlineStr">
+        <is>
+          <t>20-year trading history; Facebook page</t>
+        </is>
+      </c>
+      <c r="P275" s="3" t="inlineStr">
+        <is>
+          <t>National lead-gen platforms (Sunsave, Solar Guide) intercept searches across all 4 counties</t>
+        </is>
+      </c>
+      <c r="Q275" s="3" t="inlineStr">
+        <is>
+          <t>'Stop paying national lead-gen sites for leads in your own 4-county patch'</t>
+        </is>
+      </c>
+      <c r="R275" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S275" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T275" s="3" t="inlineStr"/>
+    </row>
+    <row r="276">
+      <c r="A276" s="3" t="inlineStr">
+        <is>
+          <t>i2i Recruitment</t>
+        </is>
+      </c>
+      <c r="B276" s="3" t="inlineStr">
+        <is>
+          <t>Recruitment agency</t>
+        </is>
+      </c>
+      <c r="C276" s="3" t="inlineStr">
+        <is>
+          <t>Cheltenham (South West)</t>
+        </is>
+      </c>
+      <c r="D276" s="3" t="inlineStr">
+        <is>
+          <t>https://i2irecruitment.co.uk</t>
+        </is>
+      </c>
+      <c r="E276" s="3" t="inlineStr">
+        <is>
+          <t>richard@i2irecruitment.co.uk</t>
+        </is>
+      </c>
+      <c r="F276" s="3" t="inlineStr">
+        <is>
+          <t>01242 771 021</t>
+        </is>
+      </c>
+      <c r="G276" s="3" t="inlineStr">
+        <is>
+          <t>Charlie (Founder); Richard Ogden-Metherell (CEO)</t>
+        </is>
+      </c>
+      <c r="H276" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/i2i-recruitment</t>
+        </is>
+      </c>
+      <c r="I276" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/i2irecruitment.co.uk</t>
+        </is>
+      </c>
+      <c r="J276" s="3" t="inlineStr">
+        <is>
+          <t>Certified B Corp independent recruiter with a personal, relationship-led positioning; placement fees + repeat SME clients</t>
+        </is>
+      </c>
+      <c r="K276" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L276" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M276" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N276" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O276" s="3" t="inlineStr">
+        <is>
+          <t>B Corp certification; active socials</t>
+        </is>
+      </c>
+      <c r="P276" s="3" t="inlineStr">
+        <is>
+          <t>B Corp status is a strong ethical differentiator not yet leveraged in AI-search answers</t>
+        </is>
+      </c>
+      <c r="Q276" s="3" t="inlineStr">
+        <is>
+          <t>'B Corp-certified recruitment - own the AI answer for "ethical recruiter Cheltenham"'</t>
+        </is>
+      </c>
+      <c r="R276" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S276" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T276" s="3" t="inlineStr"/>
+    </row>
+    <row r="277">
+      <c r="A277" s="4" t="inlineStr">
+        <is>
+          <t>The Burford Recruitment Company</t>
+        </is>
+      </c>
+      <c r="B277" s="4" t="inlineStr">
+        <is>
+          <t>Recruitment agency (boutique)</t>
+        </is>
+      </c>
+      <c r="C277" s="4" t="inlineStr">
+        <is>
+          <t>Burford, West Oxfordshire (Cotswolds)</t>
+        </is>
+      </c>
+      <c r="D277" s="4" t="inlineStr">
+        <is>
+          <t>https://www.burfordrecruitment.co.uk</t>
+        </is>
+      </c>
+      <c r="E277" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F277" s="4" t="inlineStr"/>
+      <c r="G277" s="4" t="inlineStr"/>
+      <c r="H277" s="4" t="inlineStr"/>
+      <c r="I277" s="4" t="inlineStr"/>
+      <c r="J277" s="4" t="inlineStr">
+        <is>
+          <t>Award-winning boutique agency est. 2016 covering office/professional/creative/finance roles across the Cotswolds</t>
+        </is>
+      </c>
+      <c r="K277" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L277" s="4" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M277" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N277" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O277" s="4" t="inlineStr">
+        <is>
+          <t>Award-winning branding</t>
+        </is>
+      </c>
+      <c r="P277" s="4" t="inlineStr">
+        <is>
+          <t>Boutique positioning in a rural catchment with less digital competition than cities - genuinely winnable</t>
+        </is>
+      </c>
+      <c r="Q277" s="4" t="inlineStr">
+        <is>
+          <t>Own 'recruitment agency Cotswolds' outright - thin competition for this exact query</t>
+        </is>
+      </c>
+      <c r="R277" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S277" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T277" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T270"/>
+  <autoFilter ref="A1:T277"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -23832,7 +24444,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B123"/>
+  <dimension ref="A1:B124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -23852,7 +24464,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>269</v>
+        <v>276</v>
       </c>
     </row>
     <row r="5">
@@ -23869,23 +24481,23 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Wedding venue</t>
+          <t>Architects</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Architects</t>
+          <t>Wedding venue</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -23955,7 +24567,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Private GP</t>
+          <t>Solar installer</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -23965,7 +24577,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>IT support / MSP</t>
+          <t>Private GP</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -23975,17 +24587,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Mortgage broker</t>
+          <t>IT support / MSP</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Solar installer</t>
+          <t>Mortgage broker</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -24005,17 +24617,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Law firm</t>
+          <t>Recruitment agency</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Osteopathy clinic</t>
+          <t>Law firm</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -24025,7 +24637,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Electrician</t>
+          <t>Osteopathy clinic</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -24035,7 +24647,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Personal training studio</t>
+          <t>Electrician</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -24045,7 +24657,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Family law firm</t>
+          <t>Personal training studio</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -24055,7 +24667,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Chiropractor</t>
+          <t>Family law firm</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -24065,7 +24677,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Recruitment agency</t>
+          <t>Chiropractor</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -25039,6 +25651,16 @@
         </is>
       </c>
       <c r="B123" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Recruitment agency (boutique)</t>
+        </is>
+      </c>
+      <c r="B124" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 21: +6 prospects (282 total) - home AV, soft furnishings, wine merchant, school consultancy
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$277</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$283</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T277"/>
+  <dimension ref="A1:T283"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -24432,8 +24432,532 @@
       </c>
       <c r="T277" s="4" t="inlineStr"/>
     </row>
+    <row r="278">
+      <c r="A278" s="3" t="inlineStr">
+        <is>
+          <t>Airwave AV</t>
+        </is>
+      </c>
+      <c r="B278" s="3" t="inlineStr">
+        <is>
+          <t>Home cinema &amp; smart home installer</t>
+        </is>
+      </c>
+      <c r="C278" s="3" t="inlineStr">
+        <is>
+          <t>Surrey &amp; Greater London</t>
+        </is>
+      </c>
+      <c r="D278" s="3" t="inlineStr">
+        <is>
+          <t>https://airwaveav.co.uk</t>
+        </is>
+      </c>
+      <c r="E278" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F278" s="3" t="inlineStr">
+        <is>
+          <t>020 8243 8547</t>
+        </is>
+      </c>
+      <c r="G278" s="3" t="inlineStr"/>
+      <c r="H278" s="3" t="inlineStr"/>
+      <c r="I278" s="3" t="inlineStr"/>
+      <c r="J278" s="3" t="inlineStr">
+        <is>
+          <t>Control4 smart-home specialist for premium Surrey/London homes; installs £10-50k+ per project with ongoing service contracts</t>
+        </is>
+      </c>
+      <c r="K278" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L278" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M278" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N278" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O278" s="3" t="inlineStr">
+        <is>
+          <t>Control4 dealer accreditation</t>
+        </is>
+      </c>
+      <c r="P278" s="3" t="inlineStr">
+        <is>
+          <t>Multiple similar-positioned rivals (Vertex AV, Lighthouse, New Wave AV) compete for identical high-net-worth clients</t>
+        </is>
+      </c>
+      <c r="Q278" s="3" t="inlineStr">
+        <is>
+          <t>'Own the AI answer for "Control4 installer Surrey" before the next AV firm does'</t>
+        </is>
+      </c>
+      <c r="R278" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S278" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T278" s="3" t="inlineStr"/>
+    </row>
+    <row r="279">
+      <c r="A279" s="4" t="inlineStr">
+        <is>
+          <t>Lighthouse</t>
+        </is>
+      </c>
+      <c r="B279" s="4" t="inlineStr">
+        <is>
+          <t>Home cinema installer</t>
+        </is>
+      </c>
+      <c r="C279" s="4" t="inlineStr">
+        <is>
+          <t>Thames Ditton, Surrey (serves London/South East)</t>
+        </is>
+      </c>
+      <c r="D279" s="4" t="inlineStr">
+        <is>
+          <t>https://www.lighthouse-ltd.co.uk</t>
+        </is>
+      </c>
+      <c r="E279" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F279" s="4" t="inlineStr">
+        <is>
+          <t>020 3696 5257</t>
+        </is>
+      </c>
+      <c r="G279" s="4" t="inlineStr"/>
+      <c r="H279" s="4" t="inlineStr"/>
+      <c r="I279" s="4" t="inlineStr"/>
+      <c r="J279" s="4" t="inlineStr">
+        <is>
+          <t>Luxury bespoke home cinema specialist in wealthy Surrey; project values easily £20-100k for full builds</t>
+        </is>
+      </c>
+      <c r="K279" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L279" s="4" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M279" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N279" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O279" s="4" t="inlineStr">
+        <is>
+          <t>Luxury brand positioning</t>
+        </is>
+      </c>
+      <c r="P279" s="4" t="inlineStr">
+        <is>
+          <t>Crowded 'home cinema installer London/Surrey' niche with many similarly-positioned rivals</t>
+        </is>
+      </c>
+      <c r="Q279" s="4" t="inlineStr">
+        <is>
+          <t>Differentiate via AEO on bespoke/luxury build specifics vs generic AV installers</t>
+        </is>
+      </c>
+      <c r="R279" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S279" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T279" s="4" t="inlineStr"/>
+    </row>
+    <row r="280">
+      <c r="A280" s="4" t="inlineStr">
+        <is>
+          <t>Ionaida</t>
+        </is>
+      </c>
+      <c r="B280" s="4" t="inlineStr">
+        <is>
+          <t>Curtains, blinds &amp; upholstery</t>
+        </is>
+      </c>
+      <c r="C280" s="4" t="inlineStr">
+        <is>
+          <t>North Somerset &amp; Bristol</t>
+        </is>
+      </c>
+      <c r="D280" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ionaida.com</t>
+        </is>
+      </c>
+      <c r="E280" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F280" s="4" t="inlineStr"/>
+      <c r="G280" s="4" t="inlineStr">
+        <is>
+          <t>Rebecca Fawcett (Founder)</t>
+        </is>
+      </c>
+      <c r="H280" s="4" t="inlineStr"/>
+      <c r="I280" s="4" t="inlineStr"/>
+      <c r="J280" s="4" t="inlineStr">
+        <is>
+          <t>Solo interior specialist with strong retail/design pedigree (ex-Bentalls, Monkwell Fabrics); bespoke curtain projects £2-10k per home</t>
+        </is>
+      </c>
+      <c r="K280" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L280" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M280" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N280" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O280" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P280" s="4" t="inlineStr">
+        <is>
+          <t>National made-to-measure chains (Hillarys, Style Studio) outspend on generic curtain-search terms</t>
+        </is>
+      </c>
+      <c r="Q280" s="4" t="inlineStr">
+        <is>
+          <t>'A design pedigree from Bentalls and Monkwell deserves better than losing to national chains on Google'</t>
+        </is>
+      </c>
+      <c r="R280" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S280" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T280" s="4" t="inlineStr"/>
+    </row>
+    <row r="281">
+      <c r="A281" s="4" t="inlineStr">
+        <is>
+          <t>Curtain Flair</t>
+        </is>
+      </c>
+      <c r="B281" s="4" t="inlineStr">
+        <is>
+          <t>Bespoke curtains &amp; soft furnishings</t>
+        </is>
+      </c>
+      <c r="C281" s="4" t="inlineStr">
+        <is>
+          <t>Bristol &amp; Bath</t>
+        </is>
+      </c>
+      <c r="D281" s="4" t="inlineStr">
+        <is>
+          <t>https://www.curtainflairltd.com</t>
+        </is>
+      </c>
+      <c r="E281" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F281" s="4" t="inlineStr">
+        <is>
+          <t>0117 986 7277</t>
+        </is>
+      </c>
+      <c r="G281" s="4" t="inlineStr">
+        <is>
+          <t>Alison (Principal)</t>
+        </is>
+      </c>
+      <c r="H281" s="4" t="inlineStr">
+        <is>
+          <t>facebook.com/curtainflairltd</t>
+        </is>
+      </c>
+      <c r="I281" s="4" t="inlineStr"/>
+      <c r="J281" s="4" t="inlineStr">
+        <is>
+          <t>Independent since 2003, hand-making in-house across Bristol/Bath; premium made-to-measure projects</t>
+        </is>
+      </c>
+      <c r="K281" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L281" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M281" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N281" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O281" s="4" t="inlineStr">
+        <is>
+          <t>Facebook presence</t>
+        </is>
+      </c>
+      <c r="P281" s="4" t="inlineStr">
+        <is>
+          <t>20+ years of craftsmanship not converted into search-driven client acquisition</t>
+        </is>
+      </c>
+      <c r="Q281" s="4" t="inlineStr">
+        <is>
+          <t>'20 years of hand-made curtains vs a national chain's factory line - own that story in AI answers'</t>
+        </is>
+      </c>
+      <c r="R281" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S281" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T281" s="4" t="inlineStr"/>
+    </row>
+    <row r="282">
+      <c r="A282" s="3" t="inlineStr">
+        <is>
+          <t>Averys of Bristol</t>
+        </is>
+      </c>
+      <c r="B282" s="3" t="inlineStr">
+        <is>
+          <t>Wine merchant</t>
+        </is>
+      </c>
+      <c r="C282" s="3" t="inlineStr">
+        <is>
+          <t>Culver Street, Bristol</t>
+        </is>
+      </c>
+      <c r="D282" s="3" t="inlineStr">
+        <is>
+          <t>via directory/press coverage</t>
+        </is>
+      </c>
+      <c r="E282" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F282" s="3" t="inlineStr"/>
+      <c r="G282" s="3" t="inlineStr">
+        <is>
+          <t>Mimi Avery (5th generation owner)</t>
+        </is>
+      </c>
+      <c r="H282" s="3" t="inlineStr"/>
+      <c r="I282" s="3" t="inlineStr"/>
+      <c r="J282" s="3" t="inlineStr">
+        <is>
+          <t>227-year-old family wine merchant with historic vaulted cellar; extraordinary heritage story, high-value repeat/gifting clients</t>
+        </is>
+      </c>
+      <c r="K282" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L282" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M282" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N282" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O282" s="3" t="inlineStr">
+        <is>
+          <t>Historic brand; press coverage</t>
+        </is>
+      </c>
+      <c r="P282" s="3" t="inlineStr">
+        <is>
+          <t>227 years of history is an exceptional, almost un-copyable AEO asset currently underused for search</t>
+        </is>
+      </c>
+      <c r="Q282" s="3" t="inlineStr">
+        <is>
+          <t>'227 years and five generations - the rarest wine-merchant story in Bristol should be AI's answer too'</t>
+        </is>
+      </c>
+      <c r="R282" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S282" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T282" s="3" t="inlineStr">
+        <is>
+          <t>Confirm current live website before outreach - one of the most compelling heritage stories in the database</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="3" t="inlineStr">
+        <is>
+          <t>Janie Richardson School Search &amp; Placement</t>
+        </is>
+      </c>
+      <c r="B283" s="3" t="inlineStr">
+        <is>
+          <t>Education consultancy (school placement)</t>
+        </is>
+      </c>
+      <c r="C283" s="3" t="inlineStr">
+        <is>
+          <t>Fulham, London SW6</t>
+        </is>
+      </c>
+      <c r="D283" s="3" t="inlineStr">
+        <is>
+          <t>https://jrschoolsearch.com</t>
+        </is>
+      </c>
+      <c r="E283" s="3" t="inlineStr">
+        <is>
+          <t>janie@jrschoolsearch.co.uk</t>
+        </is>
+      </c>
+      <c r="F283" s="3" t="inlineStr">
+        <is>
+          <t>020 7731 0695</t>
+        </is>
+      </c>
+      <c r="G283" s="3" t="inlineStr">
+        <is>
+          <t>Janie Richardson (Founder)</t>
+        </is>
+      </c>
+      <c r="H283" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/janie-richardson-95557737</t>
+        </is>
+      </c>
+      <c r="I283" s="3" t="inlineStr"/>
+      <c r="J283" s="3" t="inlineStr">
+        <is>
+          <t>Independent school-search consultant for relocating/international families; fees run into thousands per placement</t>
+        </is>
+      </c>
+      <c r="K283" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L283" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M283" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N283" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O283" s="3" t="inlineStr">
+        <is>
+          <t>Professional site; LinkedIn presence</t>
+        </is>
+      </c>
+      <c r="P283" s="3" t="inlineStr">
+        <is>
+          <t>Bigger consultancies (William Clarence, Keystone) outspend on 'school consultant London' search</t>
+        </is>
+      </c>
+      <c r="Q283" s="3" t="inlineStr">
+        <is>
+          <t>'Discreet, personal school placement vs a big consultancy brand - own that AEO positioning'</t>
+        </is>
+      </c>
+      <c r="R283" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S283" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T283" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T277"/>
+  <autoFilter ref="A1:T283"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -24444,7 +24968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B124"/>
+  <dimension ref="A1:B130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -24464,7 +24988,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>276</v>
+        <v>282</v>
       </c>
     </row>
     <row r="5">
@@ -25661,6 +26185,66 @@
         </is>
       </c>
       <c r="B124" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Home cinema &amp; smart home installer</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Home cinema installer</t>
+        </is>
+      </c>
+      <c r="B126" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Curtains, blinds &amp; upholstery</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Bespoke curtains &amp; soft furnishings</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Wine merchant</t>
+        </is>
+      </c>
+      <c r="B129" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Education consultancy (school placement)</t>
+        </is>
+      </c>
+      <c r="B130" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 22: +6 prospects (288 total) - Epsom/Ashtead agents, Surrey tutoring, Cotswolds caterers
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$283</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$289</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T283"/>
+  <dimension ref="A1:T289"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -24956,8 +24956,528 @@
       </c>
       <c r="T283" s="3" t="inlineStr"/>
     </row>
+    <row r="284">
+      <c r="A284" s="3" t="inlineStr">
+        <is>
+          <t>V&amp;H Homes</t>
+        </is>
+      </c>
+      <c r="B284" s="3" t="inlineStr">
+        <is>
+          <t>Estate &amp; letting agent</t>
+        </is>
+      </c>
+      <c r="C284" s="3" t="inlineStr">
+        <is>
+          <t>Ashtead (serves Epsom/Fetcham), Surrey</t>
+        </is>
+      </c>
+      <c r="D284" s="3" t="inlineStr">
+        <is>
+          <t>https://vhhomes.co.uk</t>
+        </is>
+      </c>
+      <c r="E284" s="3" t="inlineStr">
+        <is>
+          <t>sales@vhhomes.co.uk</t>
+        </is>
+      </c>
+      <c r="F284" s="3" t="inlineStr">
+        <is>
+          <t>01372 221 678</t>
+        </is>
+      </c>
+      <c r="G284" s="3" t="inlineStr">
+        <is>
+          <t>Paul Aboud (Founder, est. 2009)</t>
+        </is>
+      </c>
+      <c r="H284" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/VHHomes.EstateAgents</t>
+        </is>
+      </c>
+      <c r="I284" s="3" t="inlineStr"/>
+      <c r="J284" s="3" t="inlineStr">
+        <is>
+          <t>Family-run, 16 years established, leading agent in Ashtead; premium Surrey commuter-belt property fees</t>
+        </is>
+      </c>
+      <c r="K284" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L284" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M284" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N284" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O284" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence</t>
+        </is>
+      </c>
+      <c r="P284" s="3" t="inlineStr">
+        <is>
+          <t>Cairds/Davies Property Partners compete for the same Epsom/Ashtead/Leatherhead searches</t>
+        </is>
+      </c>
+      <c r="Q284" s="3" t="inlineStr">
+        <is>
+          <t>'Leading agent in Ashtead - make AI say so, not just the local reputation'</t>
+        </is>
+      </c>
+      <c r="R284" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S284" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T284" s="3" t="inlineStr"/>
+    </row>
+    <row r="285">
+      <c r="A285" s="4" t="inlineStr">
+        <is>
+          <t>Cairds Estate Agents</t>
+        </is>
+      </c>
+      <c r="B285" s="4" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C285" s="4" t="inlineStr">
+        <is>
+          <t>Epsom &amp; Ashtead, Surrey</t>
+        </is>
+      </c>
+      <c r="D285" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cairds.co.uk</t>
+        </is>
+      </c>
+      <c r="E285" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F285" s="4" t="inlineStr"/>
+      <c r="G285" s="4" t="inlineStr"/>
+      <c r="H285" s="4" t="inlineStr"/>
+      <c r="I285" s="4" t="inlineStr"/>
+      <c r="J285" s="4" t="inlineStr">
+        <is>
+          <t>Independent local business, 40+ years' experience in Epsom/Ashtead property market</t>
+        </is>
+      </c>
+      <c r="K285" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L285" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M285" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N285" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O285" s="4" t="inlineStr">
+        <is>
+          <t>40-year heritage</t>
+        </is>
+      </c>
+      <c r="P285" s="4" t="inlineStr">
+        <is>
+          <t>Four decades of trust untranslated into modern AI-search dominance</t>
+        </is>
+      </c>
+      <c r="Q285" s="4" t="inlineStr">
+        <is>
+          <t>'40 years in Epsom deserves to be the AI's answer, not just word-of-mouth'</t>
+        </is>
+      </c>
+      <c r="R285" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S285" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T285" s="4" t="inlineStr"/>
+    </row>
+    <row r="286">
+      <c r="A286" s="4" t="inlineStr">
+        <is>
+          <t>Jackie Quinn Estate Agents</t>
+        </is>
+      </c>
+      <c r="B286" s="4" t="inlineStr">
+        <is>
+          <t>Letting agent</t>
+        </is>
+      </c>
+      <c r="C286" s="4" t="inlineStr">
+        <is>
+          <t>Ashtead/Epsom/Leatherhead/Dorking/Clapham/Balham</t>
+        </is>
+      </c>
+      <c r="D286" s="4" t="inlineStr">
+        <is>
+          <t>https://www.jackiequinn.co.uk</t>
+        </is>
+      </c>
+      <c r="E286" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F286" s="4" t="inlineStr"/>
+      <c r="G286" s="4" t="inlineStr">
+        <is>
+          <t>Jackie Quinn (Founder)</t>
+        </is>
+      </c>
+      <c r="H286" s="4" t="inlineStr"/>
+      <c r="I286" s="4" t="inlineStr"/>
+      <c r="J286" s="4" t="inlineStr">
+        <is>
+          <t>Wide-catchment independent letting specialist spanning Surrey and South London; landlord management fees recur</t>
+        </is>
+      </c>
+      <c r="K286" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L286" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M286" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N286" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O286" s="4" t="inlineStr">
+        <is>
+          <t>Multi-area coverage</t>
+        </is>
+      </c>
+      <c r="P286" s="4" t="inlineStr">
+        <is>
+          <t>Broad geographic claim not matched by per-area search dominance</t>
+        </is>
+      </c>
+      <c r="Q286" s="4" t="inlineStr">
+        <is>
+          <t>Per-town landlord-focused AEO content across the whole claimed footprint</t>
+        </is>
+      </c>
+      <c r="R286" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S286" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T286" s="4" t="inlineStr"/>
+    </row>
+    <row r="287">
+      <c r="A287" s="4" t="inlineStr">
+        <is>
+          <t>Elite Tuition Collective</t>
+        </is>
+      </c>
+      <c r="B287" s="4" t="inlineStr">
+        <is>
+          <t>Private tuition agency</t>
+        </is>
+      </c>
+      <c r="C287" s="4" t="inlineStr">
+        <is>
+          <t>Chertsey, Surrey (serves Staines/Weybridge/Egham/Virginia Water)</t>
+        </is>
+      </c>
+      <c r="D287" s="4" t="inlineStr">
+        <is>
+          <t>https://elitetuitioncollective.com</t>
+        </is>
+      </c>
+      <c r="E287" s="4" t="inlineStr">
+        <is>
+          <t>info@elitetuitioncollective.com</t>
+        </is>
+      </c>
+      <c r="F287" s="4" t="inlineStr">
+        <is>
+          <t>07843 934 949</t>
+        </is>
+      </c>
+      <c r="G287" s="4" t="inlineStr">
+        <is>
+          <t>Lauren Bowles (Founder, ex-primary teacher)</t>
+        </is>
+      </c>
+      <c r="H287" s="4" t="inlineStr"/>
+      <c r="I287" s="4" t="inlineStr"/>
+      <c r="J287" s="4" t="inlineStr">
+        <is>
+          <t>Founder-led, teacher-credentialed tutoring group across 5 wealthy Surrey towns; per-family tuition spend can run thousands/year</t>
+        </is>
+      </c>
+      <c r="K287" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L287" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M287" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N287" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O287" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P287" s="4" t="inlineStr">
+        <is>
+          <t>National tutoring platforms (MyTutor, Tutorful) absorb the same local searches</t>
+        </is>
+      </c>
+      <c r="Q287" s="4" t="inlineStr">
+        <is>
+          <t>'A qualified teacher's tuition agency vs an anonymous national platform - own that trust gap'</t>
+        </is>
+      </c>
+      <c r="R287" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S287" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T287" s="4" t="inlineStr"/>
+    </row>
+    <row r="288">
+      <c r="A288" s="3" t="inlineStr">
+        <is>
+          <t>The Cotswold Caterer</t>
+        </is>
+      </c>
+      <c r="B288" s="3" t="inlineStr">
+        <is>
+          <t>Wedding &amp; event caterer</t>
+        </is>
+      </c>
+      <c r="C288" s="3" t="inlineStr">
+        <is>
+          <t>Quedgeley, Gloucester (serves Cotswolds/Gloucestershire)</t>
+        </is>
+      </c>
+      <c r="D288" s="3" t="inlineStr">
+        <is>
+          <t>https://thecotswoldcaterer.co.uk</t>
+        </is>
+      </c>
+      <c r="E288" s="3" t="inlineStr">
+        <is>
+          <t>hello@thecotswoldcaterer.co.uk</t>
+        </is>
+      </c>
+      <c r="F288" s="3" t="inlineStr">
+        <is>
+          <t>01452 905 106</t>
+        </is>
+      </c>
+      <c r="G288" s="3" t="inlineStr"/>
+      <c r="H288" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/thecotswoldcaterergloucestershire</t>
+        </is>
+      </c>
+      <c r="I288" s="3" t="inlineStr"/>
+      <c r="J288" s="3" t="inlineStr">
+        <is>
+          <t>Family business with 15+ years catering experience across weddings/corporate/funerals - three revenue lines from one kitchen</t>
+        </is>
+      </c>
+      <c r="K288" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L288" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M288" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N288" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O288" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence; dedicated event-type landing pages</t>
+        </is>
+      </c>
+      <c r="P288" s="3" t="inlineStr">
+        <is>
+          <t>Landing pages exist per event type but AI-answer citations for 'wedding caterer Cotswolds' still open</t>
+        </is>
+      </c>
+      <c r="Q288" s="3" t="inlineStr">
+        <is>
+          <t>'You built pages for weddings, corporate AND funerals - let's make AI cite all three'</t>
+        </is>
+      </c>
+      <c r="R288" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S288" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T288" s="3" t="inlineStr"/>
+    </row>
+    <row r="289">
+      <c r="A289" s="4" t="inlineStr">
+        <is>
+          <t>Bennett &amp; Friends</t>
+        </is>
+      </c>
+      <c r="B289" s="4" t="inlineStr">
+        <is>
+          <t>Wedding &amp; event caterer</t>
+        </is>
+      </c>
+      <c r="C289" s="4" t="inlineStr">
+        <is>
+          <t>Rural Cotswolds (Gloucestershire/Oxfordshire)</t>
+        </is>
+      </c>
+      <c r="D289" s="4" t="inlineStr">
+        <is>
+          <t>https://bennettandfriends.co.uk</t>
+        </is>
+      </c>
+      <c r="E289" s="4" t="inlineStr">
+        <is>
+          <t>sam@bennettandfriends.co.uk</t>
+        </is>
+      </c>
+      <c r="F289" s="4" t="inlineStr">
+        <is>
+          <t>01386 575 840</t>
+        </is>
+      </c>
+      <c r="G289" s="4" t="inlineStr">
+        <is>
+          <t>Sam (Founder)</t>
+        </is>
+      </c>
+      <c r="H289" s="4" t="inlineStr"/>
+      <c r="I289" s="4" t="inlineStr"/>
+      <c r="J289" s="4" t="inlineStr">
+        <is>
+          <t>Friendly, flexible independent caterer serving the wider Cotswolds; repeat venue partnerships drive referral business</t>
+        </is>
+      </c>
+      <c r="K289" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L289" s="4" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M289" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N289" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O289" s="4" t="inlineStr">
+        <is>
+          <t>Venue-partner relationships</t>
+        </is>
+      </c>
+      <c r="P289" s="4" t="inlineStr">
+        <is>
+          <t>Referral-dependent growth model vulnerable if venue partnerships shift; direct search presence would diversify</t>
+        </is>
+      </c>
+      <c r="Q289" s="4" t="inlineStr">
+        <is>
+          <t>'Stop relying only on venue referrals - build a direct search presence as backup income'</t>
+        </is>
+      </c>
+      <c r="R289" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S289" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T289" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T283"/>
+  <autoFilter ref="A1:T289"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -24968,7 +25488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B130"/>
+  <dimension ref="A1:B131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -24988,7 +25508,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>282</v>
+        <v>288</v>
       </c>
     </row>
     <row r="5">
@@ -25005,7 +25525,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7">
@@ -25055,7 +25575,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12">
@@ -25161,7 +25681,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Osteopathy clinic</t>
+          <t>Letting agent</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -25171,7 +25691,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Electrician</t>
+          <t>Private tuition agency</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -25181,7 +25701,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Personal training studio</t>
+          <t>Osteopathy clinic</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -25191,7 +25711,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Family law firm</t>
+          <t>Electrician</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -25201,7 +25721,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Chiropractor</t>
+          <t>Personal training studio</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -25211,7 +25731,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Immigration law firm</t>
+          <t>Family law firm</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -25221,7 +25741,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Independent optician</t>
+          <t>Chiropractor</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -25231,7 +25751,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Pilates studio</t>
+          <t>Immigration law firm</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -25241,7 +25761,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Kitchen &amp; bathroom design</t>
+          <t>Independent optician</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -25251,27 +25771,27 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Letting agent</t>
+          <t>Pilates studio</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Financial adviser / wealth management</t>
+          <t>Kitchen &amp; bathroom design</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Private tuition agency</t>
+          <t>Financial adviser / wealth management</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -25391,17 +25911,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Dentist / Orthodontics</t>
+          <t>Wedding &amp; event caterer</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Specialist dental/implant clinic</t>
+          <t>Dentist / Orthodontics</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -25411,7 +25931,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Boutique corporate law firm</t>
+          <t>Specialist dental/implant clinic</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -25421,7 +25941,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Cosmetic/aesthetics clinic</t>
+          <t>Boutique corporate law firm</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -25431,7 +25951,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Skin &amp; laser clinic</t>
+          <t>Cosmetic/aesthetics clinic</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -25441,7 +25961,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Mortgage broker / financial adviser</t>
+          <t>Skin &amp; laser clinic</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -25451,7 +25971,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Architects (RIBA chartered)</t>
+          <t>Mortgage broker / financial adviser</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -25461,7 +25981,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Recruitment agency (tech/startups)</t>
+          <t>Architects (RIBA chartered)</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -25471,7 +25991,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Recruitment agency (IT/data)</t>
+          <t>Recruitment agency (tech/startups)</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -25481,7 +26001,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Independent vet (24/7 emergency)</t>
+          <t>Recruitment agency (IT/data)</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -25491,7 +26011,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Interior design studio</t>
+          <t>Independent vet (24/7 emergency)</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -25501,7 +26021,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Letting &amp; estate agent</t>
+          <t>Interior design studio</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -25511,7 +26031,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Cosmetic clinic (injectables)</t>
+          <t>Letting &amp; estate agent</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -25521,7 +26041,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Cosmetic/anti-ageing clinic</t>
+          <t>Cosmetic clinic (injectables)</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -25531,7 +26051,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Yoga &amp; reformer pilates studio</t>
+          <t>Cosmetic/anti-ageing clinic</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -25541,7 +26061,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Reformer pilates studio</t>
+          <t>Yoga &amp; reformer pilates studio</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -25551,7 +26071,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Wealth management</t>
+          <t>Reformer pilates studio</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -25561,7 +26081,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Private tuition &amp; education consultancy</t>
+          <t>Wealth management</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -25571,7 +26091,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Osteopath</t>
+          <t>Private tuition &amp; education consultancy</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -25581,7 +26101,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Design &amp; build / home renovation</t>
+          <t>Osteopath</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -25591,7 +26111,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Builders / building contractor</t>
+          <t>Design &amp; build / home renovation</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -25601,7 +26121,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Home care / live-in care</t>
+          <t>Builders / building contractor</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -25611,7 +26131,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Private day nurseries</t>
+          <t>Home care / live-in care</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -25621,7 +26141,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Personal training &amp; wellness studio</t>
+          <t>Private day nurseries</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -25631,7 +26151,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Mortgage &amp; insurance broker</t>
+          <t>Personal training &amp; wellness studio</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -25641,7 +26161,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Business consultancy</t>
+          <t>Mortgage &amp; insurance broker</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -25651,7 +26171,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Interior designer (period homes)</t>
+          <t>Business consultancy</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -25661,7 +26181,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Landscape design &amp; build</t>
+          <t>Interior designer (period homes)</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -25671,7 +26191,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Interior designer</t>
+          <t>Landscape design &amp; build</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -25681,7 +26201,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Garden design &amp; landscaping</t>
+          <t>Interior designer</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -25691,7 +26211,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Legal recruitment</t>
+          <t>Garden design &amp; landscaping</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -25701,7 +26221,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Independent gym &amp; health club</t>
+          <t>Legal recruitment</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -25711,7 +26231,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Independent gym</t>
+          <t>Independent gym &amp; health club</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -25721,7 +26241,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Physiotherapy (sports)</t>
+          <t>Independent gym</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -25731,7 +26251,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Letting agent / property management</t>
+          <t>Physiotherapy (sports)</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -25741,7 +26261,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Skin clinic</t>
+          <t>Letting agent / property management</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -25751,7 +26271,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Tutoring company</t>
+          <t>Skin clinic</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -25761,7 +26281,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Tutorial college &amp; exam centre</t>
+          <t>Tutoring company</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -25771,7 +26291,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Employment law (disability discrimination)</t>
+          <t>Tutorial college &amp; exam centre</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -25781,7 +26301,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating</t>
+          <t>Employment law (disability discrimination)</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -25791,7 +26311,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Plumbing &amp; heating</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -25801,7 +26321,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Sports physio &amp; massage</t>
+          <t>Plumbing</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -25811,7 +26331,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Chartered surveyors (party wall/building)</t>
+          <t>Sports physio &amp; massage</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -25821,7 +26341,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Chartered surveyors</t>
+          <t>Chartered surveyors (party wall/building)</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -25831,7 +26351,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Chartered building surveyors</t>
+          <t>Chartered surveyors</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -25841,7 +26361,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Osteopathy clinics</t>
+          <t>Chartered building surveyors</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -25851,7 +26371,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Builders / renovations</t>
+          <t>Osteopathy clinics</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -25861,7 +26381,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Private nursery schools</t>
+          <t>Builders / renovations</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -25871,7 +26391,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Private day nursery</t>
+          <t>Private nursery schools</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -25881,7 +26401,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Private GP (membership model)</t>
+          <t>Private day nursery</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -25891,7 +26411,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Sash window restoration</t>
+          <t>Private GP (membership model)</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -25901,7 +26421,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Personal training (1:1)</t>
+          <t>Sash window restoration</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -25911,7 +26431,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Personal training &amp; nutrition coaching</t>
+          <t>Personal training (1:1)</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -25921,7 +26441,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Private nursery/pre-prep school</t>
+          <t>Personal training &amp; nutrition coaching</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -25931,7 +26451,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Independent nursery (Montessori)</t>
+          <t>Private nursery/pre-prep school</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -25941,7 +26461,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Live-in care agency</t>
+          <t>Independent nursery (Montessori)</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -25951,7 +26471,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Law firm (conveyancing/family)</t>
+          <t>Live-in care agency</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -25961,7 +26481,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Architect &amp; interior designer</t>
+          <t>Law firm (conveyancing/family)</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -25971,7 +26491,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Architects / project management</t>
+          <t>Architect &amp; interior designer</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -25981,7 +26501,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>IFA / wealth management</t>
+          <t>Architects / project management</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -25991,7 +26511,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Physiotherapy &amp; clinical Pilates</t>
+          <t>IFA / wealth management</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -26001,7 +26521,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Aesthetics &amp; skin clinic</t>
+          <t>Physiotherapy &amp; clinical Pilates</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -26011,7 +26531,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Wealth management / IFA</t>
+          <t>Aesthetics &amp; skin clinic</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -26021,7 +26541,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>IFA / financial planning</t>
+          <t>Wealth management / IFA</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -26031,7 +26551,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Wealth management &amp; employee benefits</t>
+          <t>IFA / financial planning</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -26041,7 +26561,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Dermatology clinic</t>
+          <t>Wealth management &amp; employee benefits</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -26051,7 +26571,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Pilates studio (multi-site)</t>
+          <t>Dermatology clinic</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -26061,7 +26581,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Private nursery (Montessori, multi-site)</t>
+          <t>Pilates studio (multi-site)</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -26071,7 +26591,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Law firm (wills &amp; probate)</t>
+          <t>Private nursery (Montessori, multi-site)</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -26081,7 +26601,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Business/technical consultancy</t>
+          <t>Law firm (wills &amp; probate)</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -26091,7 +26611,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Architects &amp; interior design</t>
+          <t>Business/technical consultancy</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -26101,7 +26621,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Private/NHS dentist</t>
+          <t>Architects &amp; interior design</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -26111,7 +26631,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Removals company</t>
+          <t>Private/NHS dentist</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -26121,7 +26641,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Driveways &amp; landscaping</t>
+          <t>Removals company</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -26131,7 +26651,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Wedding &amp; event venue</t>
+          <t>Driveways &amp; landscaping</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -26141,7 +26661,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>IFA &amp; mortgage broker</t>
+          <t>Wedding &amp; event venue</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -26151,7 +26671,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Estate agent &amp; chartered surveyors</t>
+          <t>IFA &amp; mortgage broker</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -26161,7 +26681,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Wedding photography &amp; videography</t>
+          <t>Estate agent &amp; chartered surveyors</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -26171,7 +26691,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Commercial property litigation law firm</t>
+          <t>Wedding photography &amp; videography</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -26181,7 +26701,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Recruitment agency (boutique)</t>
+          <t>Commercial property litigation law firm</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -26191,7 +26711,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Home cinema &amp; smart home installer</t>
+          <t>Recruitment agency (boutique)</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -26201,7 +26721,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Home cinema installer</t>
+          <t>Home cinema &amp; smart home installer</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -26211,7 +26731,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Curtains, blinds &amp; upholstery</t>
+          <t>Home cinema installer</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -26221,7 +26741,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Bespoke curtains &amp; soft furnishings</t>
+          <t>Curtains, blinds &amp; upholstery</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -26231,7 +26751,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Wine merchant</t>
+          <t>Bespoke curtains &amp; soft furnishings</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -26241,10 +26761,20 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
+          <t>Wine merchant</t>
+        </is>
+      </c>
+      <c r="B130" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
           <t>Education consultancy (school placement)</t>
         </is>
       </c>
-      <c r="B130" t="n">
+      <c r="B131" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 23: +7 prospects (295 total) - Twickenham/Teddington agents, dentists, IFA, architects
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$289</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$296</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T289"/>
+  <dimension ref="A1:T296"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -25476,8 +25476,612 @@
       </c>
       <c r="T289" s="4" t="inlineStr"/>
     </row>
+    <row r="290">
+      <c r="A290" s="2" t="inlineStr">
+        <is>
+          <t>Milestone &amp; Collis</t>
+        </is>
+      </c>
+      <c r="B290" s="2" t="inlineStr">
+        <is>
+          <t>Estate agent &amp; surveyors</t>
+        </is>
+      </c>
+      <c r="C290" s="2" t="inlineStr">
+        <is>
+          <t>Church Street, Twickenham (+ Teddington)</t>
+        </is>
+      </c>
+      <c r="D290" s="2" t="inlineStr">
+        <is>
+          <t>https://www.milestone-collis.com</t>
+        </is>
+      </c>
+      <c r="E290" s="2" t="inlineStr">
+        <is>
+          <t>Sales@milestone-collis.com</t>
+        </is>
+      </c>
+      <c r="F290" s="2" t="inlineStr">
+        <is>
+          <t>020 8892 1313</t>
+        </is>
+      </c>
+      <c r="G290" s="2" t="inlineStr">
+        <is>
+          <t>Est. 1890; current principals B. Dinnage &amp; D. Dunlop lineage</t>
+        </is>
+      </c>
+      <c r="H290" s="2" t="inlineStr">
+        <is>
+          <t>instagram.com/milestone.collis</t>
+        </is>
+      </c>
+      <c r="I290" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/milestonecollis</t>
+        </is>
+      </c>
+      <c r="J290" s="2" t="inlineStr">
+        <is>
+          <t>135-year-old independent firm - extraordinary heritage in Twickenham/Teddington property; surveying arm adds a second revenue line</t>
+        </is>
+      </c>
+      <c r="K290" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L290" s="2" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M290" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N290" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O290" s="2" t="inlineStr">
+        <is>
+          <t>Instagram/Facebook presence</t>
+        </is>
+      </c>
+      <c r="P290" s="2" t="inlineStr">
+        <is>
+          <t>135 years of trust is an exceptional AEO asset currently underused against modern digital-first rivals</t>
+        </is>
+      </c>
+      <c r="Q290" s="2" t="inlineStr">
+        <is>
+          <t>'135 years in Twickenham - the longest-established name should be AI's answer too'</t>
+        </is>
+      </c>
+      <c r="R290" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S290" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T290" s="2" t="inlineStr">
+        <is>
+          <t>Rare, hard-to-replicate heritage story - high-value AEO opportunity</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="4" t="inlineStr">
+        <is>
+          <t>Websters Estate Agents</t>
+        </is>
+      </c>
+      <c r="B291" s="4" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C291" s="4" t="inlineStr">
+        <is>
+          <t>Twickenham &amp; Teddington, London</t>
+        </is>
+      </c>
+      <c r="D291" s="4" t="inlineStr">
+        <is>
+          <t>https://www.mywebsters.co.uk</t>
+        </is>
+      </c>
+      <c r="E291" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F291" s="4" t="inlineStr">
+        <is>
+          <t>020 8892 3343</t>
+        </is>
+      </c>
+      <c r="G291" s="4" t="inlineStr"/>
+      <c r="H291" s="4" t="inlineStr"/>
+      <c r="I291" s="4" t="inlineStr"/>
+      <c r="J291" s="4" t="inlineStr">
+        <is>
+          <t>Two-office independent covering 9+ SW London postcodes (Twickenham, St Margaret's, Whitton, Hampton, etc.)</t>
+        </is>
+      </c>
+      <c r="K291" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L291" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M291" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N291" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O291" s="4" t="inlineStr">
+        <is>
+          <t>Two-office coverage</t>
+        </is>
+      </c>
+      <c r="P291" s="4" t="inlineStr">
+        <is>
+          <t>Wide postcode claim not matched by per-area search dominance</t>
+        </is>
+      </c>
+      <c r="Q291" s="4" t="inlineStr">
+        <is>
+          <t>Per-postcode AEO content to actually own the 9 areas claimed</t>
+        </is>
+      </c>
+      <c r="R291" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S291" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T291" s="4" t="inlineStr"/>
+    </row>
+    <row r="292">
+      <c r="A292" s="4" t="inlineStr">
+        <is>
+          <t>Devenports Estate Agents</t>
+        </is>
+      </c>
+      <c r="B292" s="4" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C292" s="4" t="inlineStr">
+        <is>
+          <t>Twickenham &amp; Hampton, London</t>
+        </is>
+      </c>
+      <c r="D292" s="4" t="inlineStr">
+        <is>
+          <t>https://devenports.co.uk</t>
+        </is>
+      </c>
+      <c r="E292" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F292" s="4" t="inlineStr"/>
+      <c r="G292" s="4" t="inlineStr"/>
+      <c r="H292" s="4" t="inlineStr"/>
+      <c r="I292" s="4" t="inlineStr"/>
+      <c r="J292" s="4" t="inlineStr">
+        <is>
+          <t>Independent covering Twickenham/Hampton; sales and lettings for premium riverside property</t>
+        </is>
+      </c>
+      <c r="K292" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L292" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M292" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N292" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O292" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P292" s="4" t="inlineStr">
+        <is>
+          <t>Corporate brands (Dexters, Hamptons) dominate Twickenham search visibility</t>
+        </is>
+      </c>
+      <c r="Q292" s="4" t="inlineStr">
+        <is>
+          <t>Local-first AEO positioning vs the corporate-brand search dominance</t>
+        </is>
+      </c>
+      <c r="R292" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S292" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T292" s="4" t="inlineStr"/>
+    </row>
+    <row r="293">
+      <c r="A293" s="3" t="inlineStr">
+        <is>
+          <t>Lebanon Park Dental Group</t>
+        </is>
+      </c>
+      <c r="B293" s="3" t="inlineStr">
+        <is>
+          <t>Private dentist</t>
+        </is>
+      </c>
+      <c r="C293" s="3" t="inlineStr">
+        <is>
+          <t>Richmond Road, Twickenham</t>
+        </is>
+      </c>
+      <c r="D293" s="3" t="inlineStr">
+        <is>
+          <t>https://www.lebanonparkdental.co.uk</t>
+        </is>
+      </c>
+      <c r="E293" s="3" t="inlineStr">
+        <is>
+          <t>info@lebanonparkdental.co.uk</t>
+        </is>
+      </c>
+      <c r="F293" s="3" t="inlineStr">
+        <is>
+          <t>020 8892 3803</t>
+        </is>
+      </c>
+      <c r="G293" s="3" t="inlineStr"/>
+      <c r="H293" s="3" t="inlineStr"/>
+      <c r="I293" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/lebanonparkdentalgroup</t>
+        </is>
+      </c>
+      <c r="J293" s="3" t="inlineStr">
+        <is>
+          <t>Private practice offering implants/Invisalign/hygiene in premium Twickenham; group model with named team page</t>
+        </is>
+      </c>
+      <c r="K293" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L293" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M293" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N293" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O293" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence; BUPA finder listing</t>
+        </is>
+      </c>
+      <c r="P293" s="3" t="inlineStr">
+        <is>
+          <t>Perfect Smile/Complete Smile chains outspend on 'dental implants Twickenham' search</t>
+        </is>
+      </c>
+      <c r="Q293" s="3" t="inlineStr">
+        <is>
+          <t>'Own "dental implants Twickenham" before the multi-site chains lock it up'</t>
+        </is>
+      </c>
+      <c r="R293" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S293" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T293" s="3" t="inlineStr"/>
+    </row>
+    <row r="294">
+      <c r="A294" s="3" t="inlineStr">
+        <is>
+          <t>The Complete Smile Twickenham</t>
+        </is>
+      </c>
+      <c r="B294" s="3" t="inlineStr">
+        <is>
+          <t>Private dentist / implants</t>
+        </is>
+      </c>
+      <c r="C294" s="3" t="inlineStr">
+        <is>
+          <t>Twickenham, London</t>
+        </is>
+      </c>
+      <c r="D294" s="3" t="inlineStr">
+        <is>
+          <t>https://www.thecompletesmile.co.uk</t>
+        </is>
+      </c>
+      <c r="E294" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F294" s="3" t="inlineStr"/>
+      <c r="G294" s="3" t="inlineStr"/>
+      <c r="H294" s="3" t="inlineStr"/>
+      <c r="I294" s="3" t="inlineStr"/>
+      <c r="J294" s="3" t="inlineStr">
+        <is>
+          <t>10,000+ implants placed - genuinely exceptional volume claim; serves Twickenham/Richmond</t>
+        </is>
+      </c>
+      <c r="K294" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L294" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M294" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N294" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O294" s="3" t="inlineStr">
+        <is>
+          <t>Volume-of-implants claim promoted</t>
+        </is>
+      </c>
+      <c r="P294" s="3" t="inlineStr">
+        <is>
+          <t>Extraordinary track record (10,000+ implants) not yet the AI-cited proof point</t>
+        </is>
+      </c>
+      <c r="Q294" s="3" t="inlineStr">
+        <is>
+          <t>'10,000 implants placed - make that the number AI quotes back to patients'</t>
+        </is>
+      </c>
+      <c r="R294" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S294" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T294" s="3" t="inlineStr"/>
+    </row>
+    <row r="295">
+      <c r="A295" s="3" t="inlineStr">
+        <is>
+          <t>Globe IFA</t>
+        </is>
+      </c>
+      <c r="B295" s="3" t="inlineStr">
+        <is>
+          <t>Independent financial adviser</t>
+        </is>
+      </c>
+      <c r="C295" s="3" t="inlineStr">
+        <is>
+          <t>St Margarets, Twickenham</t>
+        </is>
+      </c>
+      <c r="D295" s="3" t="inlineStr">
+        <is>
+          <t>https://globeifa.co.uk</t>
+        </is>
+      </c>
+      <c r="E295" s="3" t="inlineStr">
+        <is>
+          <t>garry@globeifa.co.uk</t>
+        </is>
+      </c>
+      <c r="F295" s="3" t="inlineStr">
+        <is>
+          <t>020 8891 0711</t>
+        </is>
+      </c>
+      <c r="G295" s="3" t="inlineStr">
+        <is>
+          <t>Garry Haywood (Founder, est. 1994)</t>
+        </is>
+      </c>
+      <c r="H295" s="3" t="inlineStr"/>
+      <c r="I295" s="3" t="inlineStr"/>
+      <c r="J295" s="3" t="inlineStr">
+        <is>
+          <t>30-year independent IFA in wealthy SW London; multi-adviser team with detailed fee transparency content</t>
+        </is>
+      </c>
+      <c r="K295" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L295" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M295" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N295" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O295" s="3" t="inlineStr">
+        <is>
+          <t>Transparent-fees content = marketing-aware</t>
+        </is>
+      </c>
+      <c r="P295" s="3" t="inlineStr">
+        <is>
+          <t>30 years of trust and transparent-fee positioning not yet the AI-cited local answer</t>
+        </is>
+      </c>
+      <c r="Q295" s="3" t="inlineStr">
+        <is>
+          <t>'30 years, transparent fees - the exact story AI should tell when Twickenham residents ask for an IFA'</t>
+        </is>
+      </c>
+      <c r="R295" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S295" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T295" s="3" t="inlineStr"/>
+    </row>
+    <row r="296">
+      <c r="A296" s="4" t="inlineStr">
+        <is>
+          <t>Marguerite Murdoch Architects</t>
+        </is>
+      </c>
+      <c r="B296" s="4" t="inlineStr">
+        <is>
+          <t>Architects</t>
+        </is>
+      </c>
+      <c r="C296" s="4" t="inlineStr">
+        <is>
+          <t>Teddington, London</t>
+        </is>
+      </c>
+      <c r="D296" s="4" t="inlineStr">
+        <is>
+          <t>https://mmurdocharchitects.co.uk</t>
+        </is>
+      </c>
+      <c r="E296" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F296" s="4" t="inlineStr"/>
+      <c r="G296" s="4" t="inlineStr">
+        <is>
+          <t>Marguerite Murdoch (Founder, est. 2006)</t>
+        </is>
+      </c>
+      <c r="H296" s="4" t="inlineStr"/>
+      <c r="I296" s="4" t="inlineStr"/>
+      <c r="J296" s="4" t="inlineStr">
+        <is>
+          <t>Founder-led practice, nearly 20 years in Teddington/Richmond residential architecture</t>
+        </is>
+      </c>
+      <c r="K296" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L296" s="4" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M296" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N296" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O296" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P296" s="4" t="inlineStr">
+        <is>
+          <t>Two decades of local project history not converted into AI-search authority</t>
+        </is>
+      </c>
+      <c r="Q296" s="4" t="inlineStr">
+        <is>
+          <t>Portfolio-driven AEO leveraging 20 years of Teddington-area projects</t>
+        </is>
+      </c>
+      <c r="R296" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S296" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T296" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T289"/>
+  <autoFilter ref="A1:T296"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -25488,7 +26092,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B131"/>
+  <dimension ref="A1:B133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -25508,7 +26112,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>288</v>
+        <v>295</v>
       </c>
     </row>
     <row r="5">
@@ -25525,7 +26129,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7">
@@ -25535,13 +26139,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Wedding venue</t>
+          <t>Private dentist</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -25551,11 +26155,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Private dentist</t>
+          <t>Wedding venue</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10">
@@ -25631,7 +26235,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>IT support / MSP</t>
+          <t>Private dentist / implants</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -25641,17 +26245,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Mortgage broker</t>
+          <t>IT support / MSP</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Private dentist / implants</t>
+          <t>Mortgage broker</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -26775,6 +27379,26 @@
         </is>
       </c>
       <c r="B131" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Estate agent &amp; surveyors</t>
+        </is>
+      </c>
+      <c r="B132" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Independent financial adviser</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 24: +7 prospects (302 total) - Richmond/Twickenham GPs, vets, personal training
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$296</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$303</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T296"/>
+  <dimension ref="A1:T303"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -26080,8 +26080,600 @@
       </c>
       <c r="T296" s="4" t="inlineStr"/>
     </row>
+    <row r="297">
+      <c r="A297" s="3" t="inlineStr">
+        <is>
+          <t>Dr Shilpa Dave Health</t>
+        </is>
+      </c>
+      <c r="B297" s="3" t="inlineStr">
+        <is>
+          <t>Private GP</t>
+        </is>
+      </c>
+      <c r="C297" s="3" t="inlineStr">
+        <is>
+          <t>Teddington &amp; Twickenham, London</t>
+        </is>
+      </c>
+      <c r="D297" s="3" t="inlineStr">
+        <is>
+          <t>https://privategp.org</t>
+        </is>
+      </c>
+      <c r="E297" s="3" t="inlineStr">
+        <is>
+          <t>pa@privategp.org</t>
+        </is>
+      </c>
+      <c r="F297" s="3" t="inlineStr">
+        <is>
+          <t>0203 303 0326</t>
+        </is>
+      </c>
+      <c r="G297" s="3" t="inlineStr">
+        <is>
+          <t>Dr Shilpa Dave (Founder &amp; Lead GP, 15+ yrs private/20+ yrs NHS)</t>
+        </is>
+      </c>
+      <c r="H297" s="3" t="inlineStr"/>
+      <c r="I297" s="3" t="inlineStr"/>
+      <c r="J297" s="3" t="inlineStr">
+        <is>
+          <t>Two-site private GP with membership model; 6-day availability and deep dual NHS/private credentials = strong trust signal</t>
+        </is>
+      </c>
+      <c r="K297" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L297" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M297" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N297" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O297" s="3" t="inlineStr">
+        <is>
+          <t>Doctify profile; membership tiers</t>
+        </is>
+      </c>
+      <c r="P297" s="3" t="inlineStr">
+        <is>
+          <t>Membership-model private GPs increasingly compete for the same self-pay searches as hospital brands</t>
+        </is>
+      </c>
+      <c r="Q297" s="3" t="inlineStr">
+        <is>
+          <t>'20 years NHS + 15 years private - own that credibility in AI answers, not just Doctify'</t>
+        </is>
+      </c>
+      <c r="R297" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S297" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T297" s="3" t="inlineStr"/>
+    </row>
+    <row r="298">
+      <c r="A298" s="4" t="inlineStr">
+        <is>
+          <t>The Richmond Doctor</t>
+        </is>
+      </c>
+      <c r="B298" s="4" t="inlineStr">
+        <is>
+          <t>Private GP</t>
+        </is>
+      </c>
+      <c r="C298" s="4" t="inlineStr">
+        <is>
+          <t>Richmond, London</t>
+        </is>
+      </c>
+      <c r="D298" s="4" t="inlineStr">
+        <is>
+          <t>https://therichmonddoctor.com</t>
+        </is>
+      </c>
+      <c r="E298" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F298" s="4" t="inlineStr"/>
+      <c r="G298" s="4" t="inlineStr"/>
+      <c r="H298" s="4" t="inlineStr"/>
+      <c r="I298" s="4" t="inlineStr"/>
+      <c r="J298" s="4" t="inlineStr">
+        <is>
+          <t>Premium private GP serving local and international families in wealthy Richmond</t>
+        </is>
+      </c>
+      <c r="K298" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L298" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M298" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N298" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O298" s="4" t="inlineStr">
+        <is>
+          <t>International-family positioning</t>
+        </is>
+      </c>
+      <c r="P298" s="4" t="inlineStr">
+        <is>
+          <t>International-family niche is a distinct, under-optimised AEO angle vs generic private GP competitors</t>
+        </is>
+      </c>
+      <c r="Q298" s="4" t="inlineStr">
+        <is>
+          <t>Own 'private GP for international families Richmond' - genuinely specific, defensible niche</t>
+        </is>
+      </c>
+      <c r="R298" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S298" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T298" s="4" t="inlineStr"/>
+    </row>
+    <row r="299">
+      <c r="A299" s="3" t="inlineStr">
+        <is>
+          <t>King Street Vets</t>
+        </is>
+      </c>
+      <c r="B299" s="3" t="inlineStr">
+        <is>
+          <t>Independent vet</t>
+        </is>
+      </c>
+      <c r="C299" s="3" t="inlineStr">
+        <is>
+          <t>King Street, Twickenham</t>
+        </is>
+      </c>
+      <c r="D299" s="3" t="inlineStr">
+        <is>
+          <t>https://www.kingstreetvets.co.uk</t>
+        </is>
+      </c>
+      <c r="E299" s="3" t="inlineStr">
+        <is>
+          <t>contact@kingstreetvets.co.uk</t>
+        </is>
+      </c>
+      <c r="F299" s="3" t="inlineStr">
+        <is>
+          <t>020 8963 3306</t>
+        </is>
+      </c>
+      <c r="G299" s="3" t="inlineStr">
+        <is>
+          <t>Dr Karmen Webbe (Owner, MRCVS)</t>
+        </is>
+      </c>
+      <c r="H299" s="3" t="inlineStr"/>
+      <c r="I299" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/KingStreetVets</t>
+        </is>
+      </c>
+      <c r="J299" s="3" t="inlineStr">
+        <is>
+          <t>Owner-led independent small-animal practice in premium Twickenham; explicit independence positioning</t>
+        </is>
+      </c>
+      <c r="K299" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L299" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M299" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N299" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O299" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence</t>
+        </is>
+      </c>
+      <c r="P299" s="3" t="inlineStr">
+        <is>
+          <t>Corporate vet groups (Medivet, CVS) heavily outspend on Twickenham/Richmond vet search</t>
+        </is>
+      </c>
+      <c r="Q299" s="3" t="inlineStr">
+        <is>
+          <t>'Owner-led and independent - own that AI answer against the corporate vet chains'</t>
+        </is>
+      </c>
+      <c r="R299" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S299" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T299" s="3" t="inlineStr"/>
+    </row>
+    <row r="300">
+      <c r="A300" s="4" t="inlineStr">
+        <is>
+          <t>The Vet in St Margarets</t>
+        </is>
+      </c>
+      <c r="B300" s="4" t="inlineStr">
+        <is>
+          <t>Independent vet</t>
+        </is>
+      </c>
+      <c r="C300" s="4" t="inlineStr">
+        <is>
+          <t>St Margarets (serves Twickenham/Isleworth/Teddington/Richmond)</t>
+        </is>
+      </c>
+      <c r="D300" s="4" t="inlineStr">
+        <is>
+          <t>https://thevetinstmargarets.co.uk</t>
+        </is>
+      </c>
+      <c r="E300" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F300" s="4" t="inlineStr"/>
+      <c r="G300" s="4" t="inlineStr"/>
+      <c r="H300" s="4" t="inlineStr"/>
+      <c r="I300" s="4" t="inlineStr"/>
+      <c r="J300" s="4" t="inlineStr">
+        <is>
+          <t>Proudly independent, 4-town catchment from one St Margarets base</t>
+        </is>
+      </c>
+      <c r="K300" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L300" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M300" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N300" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O300" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P300" s="4" t="inlineStr">
+        <is>
+          <t>4-town claim not matched by per-town search dominance</t>
+        </is>
+      </c>
+      <c r="Q300" s="4" t="inlineStr">
+        <is>
+          <t>Per-town AEO content to actually own the claimed catchment</t>
+        </is>
+      </c>
+      <c r="R300" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S300" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T300" s="4" t="inlineStr"/>
+    </row>
+    <row r="301">
+      <c r="A301" s="3" t="inlineStr">
+        <is>
+          <t>Richmond Vets</t>
+        </is>
+      </c>
+      <c r="B301" s="3" t="inlineStr">
+        <is>
+          <t>Independent vet</t>
+        </is>
+      </c>
+      <c r="C301" s="3" t="inlineStr">
+        <is>
+          <t>Richmond, London (between Kew Gardens and Richmond)</t>
+        </is>
+      </c>
+      <c r="D301" s="3" t="inlineStr">
+        <is>
+          <t>https://www.richmond-vets.co.uk</t>
+        </is>
+      </c>
+      <c r="E301" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F301" s="3" t="inlineStr"/>
+      <c r="G301" s="3" t="inlineStr">
+        <is>
+          <t>Family-owned since the 1970s</t>
+        </is>
+      </c>
+      <c r="H301" s="3" t="inlineStr"/>
+      <c r="I301" s="3" t="inlineStr"/>
+      <c r="J301" s="3" t="inlineStr">
+        <is>
+          <t>50+ years family-owned in one of London's wealthiest boroughs - exceptional heritage for a competitive vet market</t>
+        </is>
+      </c>
+      <c r="K301" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L301" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M301" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N301" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O301" s="3" t="inlineStr">
+        <is>
+          <t>50-year heritage</t>
+        </is>
+      </c>
+      <c r="P301" s="3" t="inlineStr">
+        <is>
+          <t>Half a century of trust invisible against Medivet/CVS corporate marketing budgets</t>
+        </is>
+      </c>
+      <c r="Q301" s="3" t="inlineStr">
+        <is>
+          <t>'50 years family-owned in Richmond - the AI answer should say so, not just Google Maps'</t>
+        </is>
+      </c>
+      <c r="R301" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S301" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T301" s="3" t="inlineStr"/>
+    </row>
+    <row r="302">
+      <c r="A302" s="4" t="inlineStr">
+        <is>
+          <t>Richmond Sports Conditioning (RSC)</t>
+        </is>
+      </c>
+      <c r="B302" s="4" t="inlineStr">
+        <is>
+          <t>Personal training</t>
+        </is>
+      </c>
+      <c r="C302" s="4" t="inlineStr">
+        <is>
+          <t>Kew, Richmond, London</t>
+        </is>
+      </c>
+      <c r="D302" s="4" t="inlineStr">
+        <is>
+          <t>https://www.rsc.coach</t>
+        </is>
+      </c>
+      <c r="E302" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F302" s="4" t="inlineStr"/>
+      <c r="G302" s="4" t="inlineStr">
+        <is>
+          <t>Dan Matkin (Founder)</t>
+        </is>
+      </c>
+      <c r="H302" s="4" t="inlineStr"/>
+      <c r="I302" s="4" t="inlineStr"/>
+      <c r="J302" s="4" t="inlineStr">
+        <is>
+          <t>Strength &amp; conditioning specialist PT in affluent Kew/Richmond; ongoing client packages</t>
+        </is>
+      </c>
+      <c r="K302" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L302" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M302" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N302" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O302" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P302" s="4" t="inlineStr">
+        <is>
+          <t>Generic 'personal trainer Richmond' searches won by bigger studio brands (Foundry, nmotion)</t>
+        </is>
+      </c>
+      <c r="Q302" s="4" t="inlineStr">
+        <is>
+          <t>Own the 'strength and conditioning coach Richmond' niche specifically</t>
+        </is>
+      </c>
+      <c r="R302" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S302" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T302" s="4" t="inlineStr"/>
+    </row>
+    <row r="303">
+      <c r="A303" s="4" t="inlineStr">
+        <is>
+          <t>The Performance Works</t>
+        </is>
+      </c>
+      <c r="B303" s="4" t="inlineStr">
+        <is>
+          <t>Personal training</t>
+        </is>
+      </c>
+      <c r="C303" s="4" t="inlineStr">
+        <is>
+          <t>Richmond Rugby Club &amp; Barnes (serves SW London)</t>
+        </is>
+      </c>
+      <c r="D303" s="4" t="inlineStr">
+        <is>
+          <t>https://www.theperformanceworks-pt.com</t>
+        </is>
+      </c>
+      <c r="E303" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F303" s="4" t="inlineStr"/>
+      <c r="G303" s="4" t="inlineStr">
+        <is>
+          <t>Edward Stembridge (Founder, ex-professional rugby player)</t>
+        </is>
+      </c>
+      <c r="H303" s="4" t="inlineStr"/>
+      <c r="I303" s="4" t="inlineStr"/>
+      <c r="J303" s="4" t="inlineStr">
+        <is>
+          <t>Ex-pro rugby player credential is a rare, genuinely differentiating trust signal for a PT business</t>
+        </is>
+      </c>
+      <c r="K303" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L303" s="4" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M303" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N303" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O303" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P303" s="4" t="inlineStr">
+        <is>
+          <t>Ex-pro athlete credential not yet leveraged as the AI-cited differentiator</t>
+        </is>
+      </c>
+      <c r="Q303" s="4" t="inlineStr">
+        <is>
+          <t>'Trained by a professional rugby player' - own that exact positioning in AI answers</t>
+        </is>
+      </c>
+      <c r="R303" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S303" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T303" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T296"/>
+  <autoFilter ref="A1:T303"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -26092,7 +26684,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B133"/>
+  <dimension ref="A1:B134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -26112,7 +26704,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>295</v>
+        <v>302</v>
       </c>
     </row>
     <row r="5">
@@ -26169,7 +26761,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11">
@@ -26185,7 +26777,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Aesthetics clinic</t>
+          <t>Private GP</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -26195,17 +26787,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Physiotherapy clinic</t>
+          <t>Aesthetics clinic</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Chartered accountants</t>
+          <t>Physiotherapy clinic</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -26215,17 +26807,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Solar installer</t>
+          <t>Chartered accountants</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Private GP</t>
+          <t>Solar installer</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -26525,17 +27117,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Dentist / Orthodontics</t>
+          <t>Personal training</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Specialist dental/implant clinic</t>
+          <t>Dentist / Orthodontics</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -26545,7 +27137,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Boutique corporate law firm</t>
+          <t>Specialist dental/implant clinic</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -26555,7 +27147,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Cosmetic/aesthetics clinic</t>
+          <t>Boutique corporate law firm</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -26565,7 +27157,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Skin &amp; laser clinic</t>
+          <t>Cosmetic/aesthetics clinic</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -26575,7 +27167,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Mortgage broker / financial adviser</t>
+          <t>Skin &amp; laser clinic</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -26585,7 +27177,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Architects (RIBA chartered)</t>
+          <t>Mortgage broker / financial adviser</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -26595,7 +27187,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Recruitment agency (tech/startups)</t>
+          <t>Architects (RIBA chartered)</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -26605,7 +27197,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Recruitment agency (IT/data)</t>
+          <t>Recruitment agency (tech/startups)</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -26615,7 +27207,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Independent vet (24/7 emergency)</t>
+          <t>Recruitment agency (IT/data)</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -26625,7 +27217,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Interior design studio</t>
+          <t>Independent vet (24/7 emergency)</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -26635,7 +27227,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Letting &amp; estate agent</t>
+          <t>Interior design studio</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -26645,7 +27237,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Cosmetic clinic (injectables)</t>
+          <t>Letting &amp; estate agent</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -26655,7 +27247,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Cosmetic/anti-ageing clinic</t>
+          <t>Cosmetic clinic (injectables)</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -26665,7 +27257,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Yoga &amp; reformer pilates studio</t>
+          <t>Cosmetic/anti-ageing clinic</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -26675,7 +27267,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Reformer pilates studio</t>
+          <t>Yoga &amp; reformer pilates studio</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -26685,7 +27277,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Wealth management</t>
+          <t>Reformer pilates studio</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -26695,7 +27287,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Private tuition &amp; education consultancy</t>
+          <t>Wealth management</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -26705,7 +27297,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Osteopath</t>
+          <t>Private tuition &amp; education consultancy</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -26715,7 +27307,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Design &amp; build / home renovation</t>
+          <t>Osteopath</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -26725,7 +27317,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Builders / building contractor</t>
+          <t>Design &amp; build / home renovation</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -26735,7 +27327,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Home care / live-in care</t>
+          <t>Builders / building contractor</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -26745,7 +27337,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Private day nurseries</t>
+          <t>Home care / live-in care</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -26755,7 +27347,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Personal training &amp; wellness studio</t>
+          <t>Private day nurseries</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -26765,7 +27357,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Mortgage &amp; insurance broker</t>
+          <t>Personal training &amp; wellness studio</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -26775,7 +27367,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Business consultancy</t>
+          <t>Mortgage &amp; insurance broker</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -26785,7 +27377,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Interior designer (period homes)</t>
+          <t>Business consultancy</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -26795,7 +27387,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Landscape design &amp; build</t>
+          <t>Interior designer (period homes)</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -26805,7 +27397,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Interior designer</t>
+          <t>Landscape design &amp; build</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -26815,7 +27407,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Garden design &amp; landscaping</t>
+          <t>Interior designer</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -26825,7 +27417,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Legal recruitment</t>
+          <t>Garden design &amp; landscaping</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -26835,7 +27427,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Independent gym &amp; health club</t>
+          <t>Legal recruitment</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -26845,7 +27437,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Independent gym</t>
+          <t>Independent gym &amp; health club</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -26855,7 +27447,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Physiotherapy (sports)</t>
+          <t>Independent gym</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -26865,7 +27457,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Letting agent / property management</t>
+          <t>Physiotherapy (sports)</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -26875,7 +27467,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Skin clinic</t>
+          <t>Letting agent / property management</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -26885,7 +27477,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Tutoring company</t>
+          <t>Skin clinic</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -26895,7 +27487,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Tutorial college &amp; exam centre</t>
+          <t>Tutoring company</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -26905,7 +27497,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Employment law (disability discrimination)</t>
+          <t>Tutorial college &amp; exam centre</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -26915,7 +27507,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating</t>
+          <t>Employment law (disability discrimination)</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -26925,7 +27517,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Plumbing &amp; heating</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -26935,7 +27527,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Sports physio &amp; massage</t>
+          <t>Plumbing</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -26945,7 +27537,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Chartered surveyors (party wall/building)</t>
+          <t>Sports physio &amp; massage</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -26955,7 +27547,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Chartered surveyors</t>
+          <t>Chartered surveyors (party wall/building)</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -26965,7 +27557,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Chartered building surveyors</t>
+          <t>Chartered surveyors</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -26975,7 +27567,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Osteopathy clinics</t>
+          <t>Chartered building surveyors</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -26985,7 +27577,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Builders / renovations</t>
+          <t>Osteopathy clinics</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -26995,7 +27587,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Private nursery schools</t>
+          <t>Builders / renovations</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -27005,7 +27597,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Private day nursery</t>
+          <t>Private nursery schools</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -27015,7 +27607,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Private GP (membership model)</t>
+          <t>Private day nursery</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -27025,7 +27617,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Sash window restoration</t>
+          <t>Private GP (membership model)</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -27035,7 +27627,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Personal training (1:1)</t>
+          <t>Sash window restoration</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -27045,7 +27637,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Personal training &amp; nutrition coaching</t>
+          <t>Personal training (1:1)</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -27055,7 +27647,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Private nursery/pre-prep school</t>
+          <t>Personal training &amp; nutrition coaching</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -27065,7 +27657,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Independent nursery (Montessori)</t>
+          <t>Private nursery/pre-prep school</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -27075,7 +27667,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Live-in care agency</t>
+          <t>Independent nursery (Montessori)</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -27085,7 +27677,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Law firm (conveyancing/family)</t>
+          <t>Live-in care agency</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -27095,7 +27687,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Architect &amp; interior designer</t>
+          <t>Law firm (conveyancing/family)</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -27105,7 +27697,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Architects / project management</t>
+          <t>Architect &amp; interior designer</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -27115,7 +27707,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>IFA / wealth management</t>
+          <t>Architects / project management</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -27125,7 +27717,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Physiotherapy &amp; clinical Pilates</t>
+          <t>IFA / wealth management</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -27135,7 +27727,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Aesthetics &amp; skin clinic</t>
+          <t>Physiotherapy &amp; clinical Pilates</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -27145,7 +27737,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Wealth management / IFA</t>
+          <t>Aesthetics &amp; skin clinic</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -27155,7 +27747,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>IFA / financial planning</t>
+          <t>Wealth management / IFA</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -27165,7 +27757,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Wealth management &amp; employee benefits</t>
+          <t>IFA / financial planning</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -27175,7 +27767,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Dermatology clinic</t>
+          <t>Wealth management &amp; employee benefits</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -27185,7 +27777,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Pilates studio (multi-site)</t>
+          <t>Dermatology clinic</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -27195,7 +27787,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Private nursery (Montessori, multi-site)</t>
+          <t>Pilates studio (multi-site)</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -27205,7 +27797,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Law firm (wills &amp; probate)</t>
+          <t>Private nursery (Montessori, multi-site)</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -27215,7 +27807,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Business/technical consultancy</t>
+          <t>Law firm (wills &amp; probate)</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -27225,7 +27817,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Architects &amp; interior design</t>
+          <t>Business/technical consultancy</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -27235,7 +27827,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Private/NHS dentist</t>
+          <t>Architects &amp; interior design</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -27245,7 +27837,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Removals company</t>
+          <t>Private/NHS dentist</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -27255,7 +27847,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Driveways &amp; landscaping</t>
+          <t>Removals company</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -27265,7 +27857,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Wedding &amp; event venue</t>
+          <t>Driveways &amp; landscaping</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -27275,7 +27867,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>IFA &amp; mortgage broker</t>
+          <t>Wedding &amp; event venue</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -27285,7 +27877,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Estate agent &amp; chartered surveyors</t>
+          <t>IFA &amp; mortgage broker</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -27295,7 +27887,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Wedding photography &amp; videography</t>
+          <t>Estate agent &amp; chartered surveyors</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -27305,7 +27897,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Commercial property litigation law firm</t>
+          <t>Wedding photography &amp; videography</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -27315,7 +27907,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Recruitment agency (boutique)</t>
+          <t>Commercial property litigation law firm</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -27325,7 +27917,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Home cinema &amp; smart home installer</t>
+          <t>Recruitment agency (boutique)</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -27335,7 +27927,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Home cinema installer</t>
+          <t>Home cinema &amp; smart home installer</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -27345,7 +27937,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Curtains, blinds &amp; upholstery</t>
+          <t>Home cinema installer</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -27355,7 +27947,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Bespoke curtains &amp; soft furnishings</t>
+          <t>Curtains, blinds &amp; upholstery</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -27365,7 +27957,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Wine merchant</t>
+          <t>Bespoke curtains &amp; soft furnishings</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -27375,7 +27967,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Education consultancy (school placement)</t>
+          <t>Wine merchant</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -27385,7 +27977,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Estate agent &amp; surveyors</t>
+          <t>Education consultancy (school placement)</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -27395,10 +27987,20 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
+          <t>Estate agent &amp; surveyors</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
           <t>Independent financial adviser</t>
         </is>
       </c>
-      <c r="B133" t="n">
+      <c r="B134" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 25: +7 prospects (309 total) - Kingston upon Thames/Surbiton
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$303</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$310</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T303"/>
+  <dimension ref="A1:T310"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -26672,8 +26672,600 @@
       </c>
       <c r="T303" s="4" t="inlineStr"/>
     </row>
+    <row r="304">
+      <c r="A304" s="3" t="inlineStr">
+        <is>
+          <t>Latimer</t>
+        </is>
+      </c>
+      <c r="B304" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C304" s="3" t="inlineStr">
+        <is>
+          <t>Kingston upon Thames, London</t>
+        </is>
+      </c>
+      <c r="D304" s="3" t="inlineStr">
+        <is>
+          <t>https://www.latimerandco.com</t>
+        </is>
+      </c>
+      <c r="E304" s="3" t="inlineStr">
+        <is>
+          <t>info@latimerandco.co.uk</t>
+        </is>
+      </c>
+      <c r="F304" s="3" t="inlineStr">
+        <is>
+          <t>020 3463 0274</t>
+        </is>
+      </c>
+      <c r="G304" s="3" t="inlineStr">
+        <is>
+          <t>Carla Lester (Owner, 30+ years experience, est. 1989)</t>
+        </is>
+      </c>
+      <c r="H304" s="3" t="inlineStr"/>
+      <c r="I304" s="3" t="inlineStr"/>
+      <c r="J304" s="3" t="inlineStr">
+        <is>
+          <t>Independent since 1989, owner-run for 35 years; premium Kingston/Surbiton border property fees</t>
+        </is>
+      </c>
+      <c r="K304" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L304" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M304" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N304" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O304" s="3" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P304" s="3" t="inlineStr">
+        <is>
+          <t>Corporate brands (Hamptons, Curchods) dominate Kingston search visibility</t>
+        </is>
+      </c>
+      <c r="Q304" s="3" t="inlineStr">
+        <is>
+          <t>'35 years owner-run in Kingston - make AI say so, not just Rightmove'</t>
+        </is>
+      </c>
+      <c r="R304" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S304" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T304" s="3" t="inlineStr"/>
+    </row>
+    <row r="305">
+      <c r="A305" s="4" t="inlineStr">
+        <is>
+          <t>Saxon Kings</t>
+        </is>
+      </c>
+      <c r="B305" s="4" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C305" s="4" t="inlineStr">
+        <is>
+          <t>Kingston upon Thames, London</t>
+        </is>
+      </c>
+      <c r="D305" s="4" t="inlineStr">
+        <is>
+          <t>https://saxonkings.co.uk</t>
+        </is>
+      </c>
+      <c r="E305" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F305" s="4" t="inlineStr"/>
+      <c r="G305" s="4" t="inlineStr"/>
+      <c r="H305" s="4" t="inlineStr"/>
+      <c r="I305" s="4" t="inlineStr"/>
+      <c r="J305" s="4" t="inlineStr">
+        <is>
+          <t>Independent, owner-run since 2006; established local reputation in KT1/KT2</t>
+        </is>
+      </c>
+      <c r="K305" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L305" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M305" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N305" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O305" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P305" s="4" t="inlineStr">
+        <is>
+          <t>Newer independent competing with 100-year-old incumbents and corporate brands alike</t>
+        </is>
+      </c>
+      <c r="Q305" s="4" t="inlineStr">
+        <is>
+          <t>Ground-floor AEO investment to build search authority alongside reputation</t>
+        </is>
+      </c>
+      <c r="R305" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S305" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T305" s="4" t="inlineStr"/>
+    </row>
+    <row r="306">
+      <c r="A306" s="4" t="inlineStr">
+        <is>
+          <t>Carringtons</t>
+        </is>
+      </c>
+      <c r="B306" s="4" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C306" s="4" t="inlineStr">
+        <is>
+          <t>Kingston, Surbiton, New Malden, Kingston Vale</t>
+        </is>
+      </c>
+      <c r="D306" s="4" t="inlineStr">
+        <is>
+          <t>https://carringtonsproperty.com</t>
+        </is>
+      </c>
+      <c r="E306" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F306" s="4" t="inlineStr"/>
+      <c r="G306" s="4" t="inlineStr"/>
+      <c r="H306" s="4" t="inlineStr"/>
+      <c r="I306" s="4" t="inlineStr"/>
+      <c r="J306" s="4" t="inlineStr">
+        <is>
+          <t>Family-led independent across 4 SW London towns; broad residential coverage</t>
+        </is>
+      </c>
+      <c r="K306" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L306" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M306" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N306" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O306" s="4" t="inlineStr">
+        <is>
+          <t>Multi-town coverage</t>
+        </is>
+      </c>
+      <c r="P306" s="4" t="inlineStr">
+        <is>
+          <t>Wide catchment claim not matched by per-town search dominance</t>
+        </is>
+      </c>
+      <c r="Q306" s="4" t="inlineStr">
+        <is>
+          <t>Per-town AEO content to actually own all 4 claimed markets</t>
+        </is>
+      </c>
+      <c r="R306" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S306" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T306" s="4" t="inlineStr"/>
+    </row>
+    <row r="307">
+      <c r="A307" s="4" t="inlineStr">
+        <is>
+          <t>Thames Street Dental</t>
+        </is>
+      </c>
+      <c r="B307" s="4" t="inlineStr">
+        <is>
+          <t>Private dentist / implants</t>
+        </is>
+      </c>
+      <c r="C307" s="4" t="inlineStr">
+        <is>
+          <t>Thames Street, Kingston upon Thames</t>
+        </is>
+      </c>
+      <c r="D307" s="4" t="inlineStr">
+        <is>
+          <t>https://thames-dental.co.uk</t>
+        </is>
+      </c>
+      <c r="E307" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F307" s="4" t="inlineStr">
+        <is>
+          <t>020 8546 6546</t>
+        </is>
+      </c>
+      <c r="G307" s="4" t="inlineStr"/>
+      <c r="H307" s="4" t="inlineStr"/>
+      <c r="I307" s="4" t="inlineStr"/>
+      <c r="J307" s="4" t="inlineStr">
+        <is>
+          <t>Independent family-run clinic on Kingston's riverside high street; implant work = high per-case value</t>
+        </is>
+      </c>
+      <c r="K307" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L307" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M307" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N307" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O307" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P307" s="4" t="inlineStr">
+        <is>
+          <t>Chain dental brands and Aesthetika compete for the same Kingston implant searches</t>
+        </is>
+      </c>
+      <c r="Q307" s="4" t="inlineStr">
+        <is>
+          <t>'Family-run on the Thames - own "dental implants Kingston" before the chains do'</t>
+        </is>
+      </c>
+      <c r="R307" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S307" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T307" s="4" t="inlineStr"/>
+    </row>
+    <row r="308">
+      <c r="A308" s="4" t="inlineStr">
+        <is>
+          <t>Aesthetika Dental Studio</t>
+        </is>
+      </c>
+      <c r="B308" s="4" t="inlineStr">
+        <is>
+          <t>Private dentist</t>
+        </is>
+      </c>
+      <c r="C308" s="4" t="inlineStr">
+        <is>
+          <t>Kingston upon Thames</t>
+        </is>
+      </c>
+      <c r="D308" s="4" t="inlineStr">
+        <is>
+          <t>https://aesthetikadentalstudio.co.uk</t>
+        </is>
+      </c>
+      <c r="E308" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F308" s="4" t="inlineStr"/>
+      <c r="G308" s="4" t="inlineStr"/>
+      <c r="H308" s="4" t="inlineStr"/>
+      <c r="I308" s="4" t="inlineStr"/>
+      <c r="J308" s="4" t="inlineStr">
+        <is>
+          <t>Established since 2011, private-only positioning with dedicated implants landing page</t>
+        </is>
+      </c>
+      <c r="K308" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L308" s="4" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M308" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N308" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O308" s="4" t="inlineStr">
+        <is>
+          <t>Dedicated implants page = active SEO</t>
+        </is>
+      </c>
+      <c r="P308" s="4" t="inlineStr">
+        <is>
+          <t>Implants page exists but not yet the AI-cited answer for Kingston implant searches</t>
+        </is>
+      </c>
+      <c r="Q308" s="4" t="inlineStr">
+        <is>
+          <t>Upgrade existing implants SEO page into an AEO-optimised asset</t>
+        </is>
+      </c>
+      <c r="R308" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S308" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T308" s="4" t="inlineStr"/>
+    </row>
+    <row r="309">
+      <c r="A309" s="3" t="inlineStr">
+        <is>
+          <t>Fletcher Crane Architects</t>
+        </is>
+      </c>
+      <c r="B309" s="3" t="inlineStr">
+        <is>
+          <t>Architects</t>
+        </is>
+      </c>
+      <c r="C309" s="3" t="inlineStr">
+        <is>
+          <t>Union Street, Kingston upon Thames</t>
+        </is>
+      </c>
+      <c r="D309" s="3" t="inlineStr">
+        <is>
+          <t>https://www.fletchercranearchitects.com</t>
+        </is>
+      </c>
+      <c r="E309" s="3" t="inlineStr">
+        <is>
+          <t>info@fletchercranearchitects.com</t>
+        </is>
+      </c>
+      <c r="F309" s="3" t="inlineStr">
+        <is>
+          <t>020 8977 4693</t>
+        </is>
+      </c>
+      <c r="G309" s="3" t="inlineStr">
+        <is>
+          <t>Carmine Bassi (Founder)</t>
+        </is>
+      </c>
+      <c r="H309" s="3" t="inlineStr"/>
+      <c r="I309" s="3" t="inlineStr"/>
+      <c r="J309" s="3" t="inlineStr">
+        <is>
+          <t>RIBA award-winning practice, 20+ years across residential/education/hotel sectors - diverse high-value client base</t>
+        </is>
+      </c>
+      <c r="K309" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L309" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M309" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N309" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O309" s="3" t="inlineStr">
+        <is>
+          <t>RIBA awards</t>
+        </is>
+      </c>
+      <c r="P309" s="3" t="inlineStr">
+        <is>
+          <t>Award-winning multi-sector practice not leveraging that range as an AEO differentiator</t>
+        </is>
+      </c>
+      <c r="Q309" s="3" t="inlineStr">
+        <is>
+          <t>'From homes to hotels - own the AI answer for versatile Kingston architecture'</t>
+        </is>
+      </c>
+      <c r="R309" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S309" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T309" s="3" t="inlineStr"/>
+    </row>
+    <row r="310">
+      <c r="A310" s="4" t="inlineStr">
+        <is>
+          <t>Tax Affinity Accountants</t>
+        </is>
+      </c>
+      <c r="B310" s="4" t="inlineStr">
+        <is>
+          <t>Chartered accountants</t>
+        </is>
+      </c>
+      <c r="C310" s="4" t="inlineStr">
+        <is>
+          <t>Tolworth, Kingston upon Thames</t>
+        </is>
+      </c>
+      <c r="D310" s="4" t="inlineStr">
+        <is>
+          <t>https://www.taxaffinity.com</t>
+        </is>
+      </c>
+      <c r="E310" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F310" s="4" t="inlineStr">
+        <is>
+          <t>0800 043 4051</t>
+        </is>
+      </c>
+      <c r="G310" s="4" t="inlineStr">
+        <is>
+          <t>Founder (ex-top-tier accountancy firm advisor)</t>
+        </is>
+      </c>
+      <c r="H310" s="4" t="inlineStr">
+        <is>
+          <t>facebook.com/TaxAffinity</t>
+        </is>
+      </c>
+      <c r="I310" s="4" t="inlineStr"/>
+      <c r="J310" s="4" t="inlineStr">
+        <is>
+          <t>Independent since 2012; founder's big-firm pedigree serving SME/sole trader clients; self-described 'No 1 rated'</t>
+        </is>
+      </c>
+      <c r="K310" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L310" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M310" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N310" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O310" s="4" t="inlineStr">
+        <is>
+          <t>'Independently rated No 1' claim; Facebook presence</t>
+        </is>
+      </c>
+      <c r="P310" s="4" t="inlineStr">
+        <is>
+          <t>Rating claim not converted into the AI-cited answer for 'accountant Kingston'</t>
+        </is>
+      </c>
+      <c r="Q310" s="4" t="inlineStr">
+        <is>
+          <t>'Independently rated No 1 - make sure AI repeats that, not just the website banner'</t>
+        </is>
+      </c>
+      <c r="R310" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S310" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T310" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T303"/>
+  <autoFilter ref="A1:T310"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -26704,7 +27296,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>302</v>
+        <v>309</v>
       </c>
     </row>
     <row r="5">
@@ -26721,7 +27313,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7">
@@ -26731,7 +27323,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8">
@@ -26741,7 +27333,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9">
@@ -26777,7 +27369,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Private GP</t>
+          <t>Chartered accountants</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -26787,7 +27379,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Aesthetics clinic</t>
+          <t>Private GP</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -26797,17 +27389,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Physiotherapy clinic</t>
+          <t>Aesthetics clinic</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Chartered accountants</t>
+          <t>Physiotherapy clinic</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -26817,17 +27409,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Solar installer</t>
+          <t>Private dentist / implants</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Private dentist / implants</t>
+          <t>Solar installer</t>
         </is>
       </c>
       <c r="B17" t="n">

</xml_diff>

<commit_message>
Batch 26: +8 prospects (317 total) - Bromley/Beckenham
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$310</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$318</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T310"/>
+  <dimension ref="A1:T318"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -27264,8 +27264,712 @@
       </c>
       <c r="T310" s="4" t="inlineStr"/>
     </row>
+    <row r="311">
+      <c r="A311" s="3" t="inlineStr">
+        <is>
+          <t>Capital Estate Agents</t>
+        </is>
+      </c>
+      <c r="B311" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C311" s="3" t="inlineStr">
+        <is>
+          <t>Beckenham Lane, Bromley, Kent</t>
+        </is>
+      </c>
+      <c r="D311" s="3" t="inlineStr">
+        <is>
+          <t>https://capitalestateagents.com</t>
+        </is>
+      </c>
+      <c r="E311" s="3" t="inlineStr">
+        <is>
+          <t>info@capitalestateagents.com</t>
+        </is>
+      </c>
+      <c r="F311" s="3" t="inlineStr">
+        <is>
+          <t>020 8313 0010</t>
+        </is>
+      </c>
+      <c r="G311" s="3" t="inlineStr">
+        <is>
+          <t>Rob Tancred (Managing Director, est. 1996)</t>
+        </is>
+      </c>
+      <c r="H311" s="3" t="inlineStr"/>
+      <c r="I311" s="3" t="inlineStr"/>
+      <c r="J311" s="3" t="inlineStr">
+        <is>
+          <t>Independent since 1996, leading agent positioning in Bromley/Beckenham; premium SE London commuter-belt fees</t>
+        </is>
+      </c>
+      <c r="K311" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L311" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M311" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N311" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O311" s="3" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P311" s="3" t="inlineStr">
+        <is>
+          <t>Alan de Maid (est. 1953) and Mann corporate brands dominate Bromley search visibility</t>
+        </is>
+      </c>
+      <c r="Q311" s="3" t="inlineStr">
+        <is>
+          <t>'Leading independent agent since 1996 - make AI say so, not just Rightmove'</t>
+        </is>
+      </c>
+      <c r="R311" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S311" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T311" s="3" t="inlineStr"/>
+    </row>
+    <row r="312">
+      <c r="A312" s="4" t="inlineStr">
+        <is>
+          <t>Sinclair Hammelton</t>
+        </is>
+      </c>
+      <c r="B312" s="4" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C312" s="4" t="inlineStr">
+        <is>
+          <t>Bromley, Beckenham &amp; Hayes, Kent</t>
+        </is>
+      </c>
+      <c r="D312" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sinclairhammelton.co.uk</t>
+        </is>
+      </c>
+      <c r="E312" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F312" s="4" t="inlineStr"/>
+      <c r="G312" s="4" t="inlineStr"/>
+      <c r="H312" s="4" t="inlineStr"/>
+      <c r="I312" s="4" t="inlineStr"/>
+      <c r="J312" s="4" t="inlineStr">
+        <is>
+          <t>Independently owned across 3 SE London/Kent towns; residential sales and lettings</t>
+        </is>
+      </c>
+      <c r="K312" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L312" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M312" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N312" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O312" s="4" t="inlineStr">
+        <is>
+          <t>Multi-town coverage</t>
+        </is>
+      </c>
+      <c r="P312" s="4" t="inlineStr">
+        <is>
+          <t>3-town claim not matched by per-town search dominance</t>
+        </is>
+      </c>
+      <c r="Q312" s="4" t="inlineStr">
+        <is>
+          <t>Per-town AEO content to actually own all 3 claimed markets</t>
+        </is>
+      </c>
+      <c r="R312" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S312" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T312" s="4" t="inlineStr"/>
+    </row>
+    <row r="313">
+      <c r="A313" s="4" t="inlineStr">
+        <is>
+          <t>Grafton Estate Agents</t>
+        </is>
+      </c>
+      <c r="B313" s="4" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C313" s="4" t="inlineStr">
+        <is>
+          <t>Beckenham, Kent</t>
+        </is>
+      </c>
+      <c r="D313" s="4" t="inlineStr">
+        <is>
+          <t>https://www.graftonestateagents.co.uk</t>
+        </is>
+      </c>
+      <c r="E313" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F313" s="4" t="inlineStr"/>
+      <c r="G313" s="4" t="inlineStr">
+        <is>
+          <t>Tariq Gabr (Owner, 18+ years experience)</t>
+        </is>
+      </c>
+      <c r="H313" s="4" t="inlineStr"/>
+      <c r="I313" s="4" t="inlineStr"/>
+      <c r="J313" s="4" t="inlineStr">
+        <is>
+          <t>Proudly independent, family-run; founder-led with nearly two decades of local experience</t>
+        </is>
+      </c>
+      <c r="K313" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L313" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M313" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N313" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O313" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P313" s="4" t="inlineStr">
+        <is>
+          <t>Family-run positioning invisible against bigger Bromley-area agents in search</t>
+        </is>
+      </c>
+      <c r="Q313" s="4" t="inlineStr">
+        <is>
+          <t>'Family-run since day one - own that AEO positioning against the bigger brands'</t>
+        </is>
+      </c>
+      <c r="R313" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S313" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T313" s="4" t="inlineStr"/>
+    </row>
+    <row r="314">
+      <c r="A314" s="3" t="inlineStr">
+        <is>
+          <t>Kelsey Park Dental</t>
+        </is>
+      </c>
+      <c r="B314" s="3" t="inlineStr">
+        <is>
+          <t>Private dentist / implants</t>
+        </is>
+      </c>
+      <c r="C314" s="3" t="inlineStr">
+        <is>
+          <t>Kelsey Park Road, Beckenham, Kent</t>
+        </is>
+      </c>
+      <c r="D314" s="3" t="inlineStr">
+        <is>
+          <t>https://kelseyparkdental.co.uk</t>
+        </is>
+      </c>
+      <c r="E314" s="3" t="inlineStr">
+        <is>
+          <t>frontdesk@kelseyparkdental.co.uk</t>
+        </is>
+      </c>
+      <c r="F314" s="3" t="inlineStr">
+        <is>
+          <t>020 8650 7677</t>
+        </is>
+      </c>
+      <c r="G314" s="3" t="inlineStr">
+        <is>
+          <t>Monica Moreira De Smith (Principal Owner)</t>
+        </is>
+      </c>
+      <c r="H314" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/monica-moreira-36607673</t>
+        </is>
+      </c>
+      <c r="I314" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/kelseyparkdental</t>
+        </is>
+      </c>
+      <c r="J314" s="3" t="inlineStr">
+        <is>
+          <t>70+ years independent practice serving Beckenham/Bromley/West Wickham; named owner-principal with implant specialism</t>
+        </is>
+      </c>
+      <c r="K314" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L314" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M314" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N314" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O314" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence; LinkedIn</t>
+        </is>
+      </c>
+      <c r="P314" s="3" t="inlineStr">
+        <is>
+          <t>70 years of trust invisible against national dental chains dominating Beckenham search</t>
+        </is>
+      </c>
+      <c r="Q314" s="3" t="inlineStr">
+        <is>
+          <t>'70 years in Beckenham - the AI answer should reflect that heritage, not just Google Maps'</t>
+        </is>
+      </c>
+      <c r="R314" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S314" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T314" s="3" t="inlineStr"/>
+    </row>
+    <row r="315">
+      <c r="A315" s="3" t="inlineStr">
+        <is>
+          <t>Premier Dental Clinic</t>
+        </is>
+      </c>
+      <c r="B315" s="3" t="inlineStr">
+        <is>
+          <t>Private dentist / implants</t>
+        </is>
+      </c>
+      <c r="C315" s="3" t="inlineStr">
+        <is>
+          <t>Beckenham Lane, Bromley, Kent</t>
+        </is>
+      </c>
+      <c r="D315" s="3" t="inlineStr">
+        <is>
+          <t>https://premierdentalclinic.co.uk</t>
+        </is>
+      </c>
+      <c r="E315" s="3" t="inlineStr">
+        <is>
+          <t>reception@premierdentalclinic.co.uk</t>
+        </is>
+      </c>
+      <c r="F315" s="3" t="inlineStr">
+        <is>
+          <t>020 8460 9150</t>
+        </is>
+      </c>
+      <c r="G315" s="3" t="inlineStr">
+        <is>
+          <t>Dr Louie (Implant specialist)</t>
+        </is>
+      </c>
+      <c r="H315" s="3" t="inlineStr"/>
+      <c r="I315" s="3" t="inlineStr"/>
+      <c r="J315" s="3" t="inlineStr">
+        <is>
+          <t>Named implant specialist offering digital surgical planning and guided surgery - genuine clinical differentiation</t>
+        </is>
+      </c>
+      <c r="K315" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L315" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M315" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N315" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O315" s="3" t="inlineStr">
+        <is>
+          <t>Digital surgical planning promoted</t>
+        </is>
+      </c>
+      <c r="P315" s="3" t="inlineStr">
+        <is>
+          <t>Advanced technique not yet leveraged as the AI-cited differentiator vs generic implant clinics</t>
+        </is>
+      </c>
+      <c r="Q315" s="3" t="inlineStr">
+        <is>
+          <t>'Digital-guided implant surgery - own that specific AEO niche in Bromley'</t>
+        </is>
+      </c>
+      <c r="R315" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S315" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T315" s="3" t="inlineStr"/>
+    </row>
+    <row r="316">
+      <c r="A316" s="3" t="inlineStr">
+        <is>
+          <t>Culverhouse &amp; Co</t>
+        </is>
+      </c>
+      <c r="B316" s="3" t="inlineStr">
+        <is>
+          <t>Chartered accountants &amp; financial planners</t>
+        </is>
+      </c>
+      <c r="C316" s="3" t="inlineStr">
+        <is>
+          <t>Farnborough Village, Orpington (Bromley/Kent)</t>
+        </is>
+      </c>
+      <c r="D316" s="3" t="inlineStr">
+        <is>
+          <t>https://www.culverhouse-accountants.co.uk</t>
+        </is>
+      </c>
+      <c r="E316" s="3" t="inlineStr">
+        <is>
+          <t>info@culverhouse-accountants.co.uk</t>
+        </is>
+      </c>
+      <c r="F316" s="3" t="inlineStr">
+        <is>
+          <t>01689 862 211</t>
+        </is>
+      </c>
+      <c r="G316" s="3" t="inlineStr">
+        <is>
+          <t>John Culverhouse (Founder)</t>
+        </is>
+      </c>
+      <c r="H316" s="3" t="inlineStr"/>
+      <c r="I316" s="3" t="inlineStr"/>
+      <c r="J316" s="3" t="inlineStr">
+        <is>
+          <t>Combined accountancy + financial planning firm - two revenue lines per client relationship, high LTV</t>
+        </is>
+      </c>
+      <c r="K316" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L316" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M316" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N316" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O316" s="3" t="inlineStr">
+        <is>
+          <t>Detailed service-specific SEO pages (HMRC enquiries, savings &amp; investments)</t>
+        </is>
+      </c>
+      <c r="P316" s="3" t="inlineStr">
+        <is>
+          <t>Many individual service pages exist but AI-answer citations for specific queries still open</t>
+        </is>
+      </c>
+      <c r="Q316" s="3" t="inlineStr">
+        <is>
+          <t>'You've written pages for every service - let's make AI cite them, not just index them'</t>
+        </is>
+      </c>
+      <c r="R316" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S316" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T316" s="3" t="inlineStr"/>
+    </row>
+    <row r="317">
+      <c r="A317" s="3" t="inlineStr">
+        <is>
+          <t>Gary Arnold Architects</t>
+        </is>
+      </c>
+      <c r="B317" s="3" t="inlineStr">
+        <is>
+          <t>Architects</t>
+        </is>
+      </c>
+      <c r="C317" s="3" t="inlineStr">
+        <is>
+          <t>Bromley, Kent (serves Beckenham/Croydon)</t>
+        </is>
+      </c>
+      <c r="D317" s="3" t="inlineStr">
+        <is>
+          <t>https://garyarnoldarchitects.co.uk</t>
+        </is>
+      </c>
+      <c r="E317" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F317" s="3" t="inlineStr">
+        <is>
+          <t>07595 916 171</t>
+        </is>
+      </c>
+      <c r="G317" s="3" t="inlineStr">
+        <is>
+          <t>Gary Arnold (Founder, 15+ years)</t>
+        </is>
+      </c>
+      <c r="H317" s="3" t="inlineStr"/>
+      <c r="I317" s="3" t="inlineStr"/>
+      <c r="J317" s="3" t="inlineStr">
+        <is>
+          <t>5-star rated chartered architect, per-area landing pages (Beckenham, South Croydon) = active SEO investment</t>
+        </is>
+      </c>
+      <c r="K317" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L317" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M317" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N317" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O317" s="3" t="inlineStr">
+        <is>
+          <t>Per-area landing pages; 5-star reviews</t>
+        </is>
+      </c>
+      <c r="P317" s="3" t="inlineStr">
+        <is>
+          <t>Landing pages exist across multiple areas but AI-answer citations still open</t>
+        </is>
+      </c>
+      <c r="Q317" s="3" t="inlineStr">
+        <is>
+          <t>'You built pages for every area you serve - add the AEO layer to make AI cite them'</t>
+        </is>
+      </c>
+      <c r="R317" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S317" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T317" s="3" t="inlineStr"/>
+    </row>
+    <row r="318">
+      <c r="A318" s="3" t="inlineStr">
+        <is>
+          <t>Brouard Architects</t>
+        </is>
+      </c>
+      <c r="B318" s="3" t="inlineStr">
+        <is>
+          <t>Architects</t>
+        </is>
+      </c>
+      <c r="C318" s="3" t="inlineStr">
+        <is>
+          <t>Chislehurst, Kent (serves Bromley/Beckenham/Keston)</t>
+        </is>
+      </c>
+      <c r="D318" s="3" t="inlineStr">
+        <is>
+          <t>via directory listing</t>
+        </is>
+      </c>
+      <c r="E318" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F318" s="3" t="inlineStr">
+        <is>
+          <t>01689 857 253</t>
+        </is>
+      </c>
+      <c r="G318" s="3" t="inlineStr">
+        <is>
+          <t>Philip Brouard (Founder, est. 1999)</t>
+        </is>
+      </c>
+      <c r="H318" s="3" t="inlineStr"/>
+      <c r="I318" s="3" t="inlineStr"/>
+      <c r="J318" s="3" t="inlineStr">
+        <is>
+          <t>25-year practice across residential/education/healthcare/hotel sectors - diverse, high-value client base</t>
+        </is>
+      </c>
+      <c r="K318" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L318" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M318" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N318" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O318" s="3" t="inlineStr">
+        <is>
+          <t>Multi-sector portfolio</t>
+        </is>
+      </c>
+      <c r="P318" s="3" t="inlineStr">
+        <is>
+          <t>Diverse sector experience not leveraged as an AEO differentiator vs residential-only rivals</t>
+        </is>
+      </c>
+      <c r="Q318" s="3" t="inlineStr">
+        <is>
+          <t>'From homes to hotels - one practice, own the AI answer for every project type'</t>
+        </is>
+      </c>
+      <c r="R318" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S318" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T318" s="3" t="inlineStr">
+        <is>
+          <t>Confirm current live website before outreach</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T310"/>
+  <autoFilter ref="A1:T318"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -27276,7 +27980,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B134"/>
+  <dimension ref="A1:B135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -27296,7 +28000,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>309</v>
+        <v>317</v>
       </c>
     </row>
     <row r="5">
@@ -27313,7 +28017,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7">
@@ -27323,7 +28027,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8">
@@ -27369,17 +28073,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Chartered accountants</t>
+          <t>Private dentist / implants</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Private GP</t>
+          <t>Chartered accountants</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -27389,7 +28093,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Aesthetics clinic</t>
+          <t>Private GP</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -27399,17 +28103,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Physiotherapy clinic</t>
+          <t>Aesthetics clinic</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Private dentist / implants</t>
+          <t>Physiotherapy clinic</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -28593,6 +29297,16 @@
         </is>
       </c>
       <c r="B134" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Chartered accountants &amp; financial planners</t>
+        </is>
+      </c>
+      <c r="B135" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 27: +9 prospects (326 total) - Purley/Croydon, Bromley GPs/vets, Surrey wedding venues
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$318</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$327</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T318"/>
+  <dimension ref="A1:T327"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -27968,8 +27968,768 @@
         </is>
       </c>
     </row>
+    <row r="319">
+      <c r="A319" s="3" t="inlineStr">
+        <is>
+          <t>ShineRocks</t>
+        </is>
+      </c>
+      <c r="B319" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C319" s="3" t="inlineStr">
+        <is>
+          <t>Purley, Surrey/Croydon</t>
+        </is>
+      </c>
+      <c r="D319" s="3" t="inlineStr">
+        <is>
+          <t>https://www.shinerocks.co.uk</t>
+        </is>
+      </c>
+      <c r="E319" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F319" s="3" t="inlineStr">
+        <is>
+          <t>020 3745 3493</t>
+        </is>
+      </c>
+      <c r="G319" s="3" t="inlineStr">
+        <is>
+          <t>Paul &amp; Claire Shinerock (Family owners, 35+ yr local brand)</t>
+        </is>
+      </c>
+      <c r="H319" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/ShinerocksPurley</t>
+        </is>
+      </c>
+      <c r="I319" s="3" t="inlineStr"/>
+      <c r="J319" s="3" t="inlineStr">
+        <is>
+          <t>Family name recognised locally for 35+ years (originally soft-furnishing retail); leading independent in mid/upper Purley market</t>
+        </is>
+      </c>
+      <c r="K319" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L319" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M319" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N319" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O319" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence; 35-year local brand</t>
+        </is>
+      </c>
+      <c r="P319" s="3" t="inlineStr">
+        <is>
+          <t>Frost (est. 1862) and corporate agents also compete hard for Purley/Croydon search</t>
+        </is>
+      </c>
+      <c r="Q319" s="3" t="inlineStr">
+        <is>
+          <t>'35 years of the Shinerocks name in Purley - make AI say it, not just word of mouth'</t>
+        </is>
+      </c>
+      <c r="R319" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S319" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T319" s="3" t="inlineStr"/>
+    </row>
+    <row r="320">
+      <c r="A320" s="2" t="inlineStr">
+        <is>
+          <t>Frost Estate Agents</t>
+        </is>
+      </c>
+      <c r="B320" s="2" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C320" s="2" t="inlineStr">
+        <is>
+          <t>Purley, Surrey</t>
+        </is>
+      </c>
+      <c r="D320" s="2" t="inlineStr">
+        <is>
+          <t>https://www.frostproperty.co.uk</t>
+        </is>
+      </c>
+      <c r="E320" s="2" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F320" s="2" t="inlineStr"/>
+      <c r="G320" s="2" t="inlineStr"/>
+      <c r="H320" s="2" t="inlineStr"/>
+      <c r="I320" s="2" t="inlineStr"/>
+      <c r="J320" s="2" t="inlineStr">
+        <is>
+          <t>Independent since 1862 - extraordinary 160+ year heritage; multiple 'Best Agent in Purley' awards since 2017</t>
+        </is>
+      </c>
+      <c r="K320" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L320" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M320" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N320" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O320" s="2" t="inlineStr">
+        <is>
+          <t>Multiple industry awards</t>
+        </is>
+      </c>
+      <c r="P320" s="2" t="inlineStr">
+        <is>
+          <t>160 years of history + repeated awards not yet the AI-cited answer for Purley property search</t>
+        </is>
+      </c>
+      <c r="Q320" s="2" t="inlineStr">
+        <is>
+          <t>'160 years and multiple Best Agent awards - the AI answer should say both, not just one'</t>
+        </is>
+      </c>
+      <c r="R320" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S320" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T320" s="2" t="inlineStr">
+        <is>
+          <t>Exceptional heritage + award combination - high-value AEO opportunity</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="4" t="inlineStr">
+        <is>
+          <t>David Bright Estates</t>
+        </is>
+      </c>
+      <c r="B321" s="4" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C321" s="4" t="inlineStr">
+        <is>
+          <t>Purley/Kenley/Coulsdon/Croydon, Surrey</t>
+        </is>
+      </c>
+      <c r="D321" s="4" t="inlineStr">
+        <is>
+          <t>https://www.davidbrightestates.co.uk</t>
+        </is>
+      </c>
+      <c r="E321" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F321" s="4" t="inlineStr"/>
+      <c r="G321" s="4" t="inlineStr"/>
+      <c r="H321" s="4" t="inlineStr"/>
+      <c r="I321" s="4" t="inlineStr"/>
+      <c r="J321" s="4" t="inlineStr">
+        <is>
+          <t>35+ years combined experience across a 4-town South Croydon/Surrey catchment</t>
+        </is>
+      </c>
+      <c r="K321" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L321" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M321" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N321" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O321" s="4" t="inlineStr">
+        <is>
+          <t>Multi-town coverage</t>
+        </is>
+      </c>
+      <c r="P321" s="4" t="inlineStr">
+        <is>
+          <t>35 years' experience claim not converted into per-town AI-search dominance</t>
+        </is>
+      </c>
+      <c r="Q321" s="4" t="inlineStr">
+        <is>
+          <t>Per-town AEO content to actually own all 4 claimed markets</t>
+        </is>
+      </c>
+      <c r="R321" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S321" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T321" s="4" t="inlineStr"/>
+    </row>
+    <row r="322">
+      <c r="A322" s="3" t="inlineStr">
+        <is>
+          <t>The Artemis Clinic</t>
+        </is>
+      </c>
+      <c r="B322" s="3" t="inlineStr">
+        <is>
+          <t>Private GP</t>
+        </is>
+      </c>
+      <c r="C322" s="3" t="inlineStr">
+        <is>
+          <t>West Wickham (serves Beckenham/Bromley/Hayes/Orpington)</t>
+        </is>
+      </c>
+      <c r="D322" s="3" t="inlineStr">
+        <is>
+          <t>https://www.artemisclinic.co.uk</t>
+        </is>
+      </c>
+      <c r="E322" s="3" t="inlineStr">
+        <is>
+          <t>office@artemisclinic.co.uk</t>
+        </is>
+      </c>
+      <c r="F322" s="3" t="inlineStr">
+        <is>
+          <t>020 8777 1500</t>
+        </is>
+      </c>
+      <c r="G322" s="3" t="inlineStr"/>
+      <c r="H322" s="3" t="inlineStr"/>
+      <c r="I322" s="3" t="inlineStr"/>
+      <c r="J322" s="3" t="inlineStr">
+        <is>
+          <t>Independent private GP covering 4 SE London/Kent towns from one base; self-pay consultations</t>
+        </is>
+      </c>
+      <c r="K322" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L322" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M322" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N322" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O322" s="3" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P322" s="3" t="inlineStr">
+        <is>
+          <t>4-town catchment claim not matched by per-town search visibility</t>
+        </is>
+      </c>
+      <c r="Q322" s="3" t="inlineStr">
+        <is>
+          <t>Per-town AEO content for 'private GP' across the whole claimed service area</t>
+        </is>
+      </c>
+      <c r="R322" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S322" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T322" s="3" t="inlineStr"/>
+    </row>
+    <row r="323">
+      <c r="A323" s="3" t="inlineStr">
+        <is>
+          <t>The Blackwell Clinic</t>
+        </is>
+      </c>
+      <c r="B323" s="3" t="inlineStr">
+        <is>
+          <t>Private GP &amp; dermatology</t>
+        </is>
+      </c>
+      <c r="C323" s="3" t="inlineStr">
+        <is>
+          <t>Bromley (serves Blackheath)</t>
+        </is>
+      </c>
+      <c r="D323" s="3" t="inlineStr">
+        <is>
+          <t>https://theblackwellclinic.com</t>
+        </is>
+      </c>
+      <c r="E323" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F323" s="3" t="inlineStr">
+        <is>
+          <t>0808 189 5666</t>
+        </is>
+      </c>
+      <c r="G323" s="3" t="inlineStr"/>
+      <c r="H323" s="3" t="inlineStr"/>
+      <c r="I323" s="3" t="inlineStr"/>
+      <c r="J323" s="3" t="inlineStr">
+        <is>
+          <t>Combined GP + dermatologist + aesthetics + skin surgery under one roof - multiple revenue lines per client relationship</t>
+        </is>
+      </c>
+      <c r="K323" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L323" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M323" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N323" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O323" s="3" t="inlineStr">
+        <is>
+          <t>Circle Health booking platform integration</t>
+        </is>
+      </c>
+      <c r="P323" s="3" t="inlineStr">
+        <is>
+          <t>Multi-service offering not unified into one strong AEO strategy across all 4 service lines</t>
+        </is>
+      </c>
+      <c r="Q323" s="3" t="inlineStr">
+        <is>
+          <t>Consolidate 4 service lines into one coherent AEO content plan</t>
+        </is>
+      </c>
+      <c r="R323" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S323" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T323" s="3" t="inlineStr"/>
+    </row>
+    <row r="324">
+      <c r="A324" s="3" t="inlineStr">
+        <is>
+          <t>Anderson Veterinary Surgery</t>
+        </is>
+      </c>
+      <c r="B324" s="3" t="inlineStr">
+        <is>
+          <t>Independent vet</t>
+        </is>
+      </c>
+      <c r="C324" s="3" t="inlineStr">
+        <is>
+          <t>Burnt Ash Lane, Bromley North, Kent</t>
+        </is>
+      </c>
+      <c r="D324" s="3" t="inlineStr">
+        <is>
+          <t>https://andersonvets.co.uk</t>
+        </is>
+      </c>
+      <c r="E324" s="3" t="inlineStr">
+        <is>
+          <t>info@andersonvets.co.uk</t>
+        </is>
+      </c>
+      <c r="F324" s="3" t="inlineStr">
+        <is>
+          <t>020 8290 1698</t>
+        </is>
+      </c>
+      <c r="G324" s="3" t="inlineStr">
+        <is>
+          <t>Katie Mercer MRCVS (Managing Partner, since 2013)</t>
+        </is>
+      </c>
+      <c r="H324" s="3" t="inlineStr"/>
+      <c r="I324" s="3" t="inlineStr"/>
+      <c r="J324" s="3" t="inlineStr">
+        <is>
+          <t>Proudly independent, named managing partner since 2013; strong professionalism/care positioning</t>
+        </is>
+      </c>
+      <c r="K324" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L324" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M324" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N324" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O324" s="3" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P324" s="3" t="inlineStr">
+        <is>
+          <t>Medivet's Bromley presence (Open Saturdays branding) outspends on local vet search</t>
+        </is>
+      </c>
+      <c r="Q324" s="3" t="inlineStr">
+        <is>
+          <t>'Proudly independent, named vet you can trust - own that vs the Medivet chain in AI answers'</t>
+        </is>
+      </c>
+      <c r="R324" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S324" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T324" s="3" t="inlineStr"/>
+    </row>
+    <row r="325">
+      <c r="A325" s="4" t="inlineStr">
+        <is>
+          <t>Tender Paws Vets</t>
+        </is>
+      </c>
+      <c r="B325" s="4" t="inlineStr">
+        <is>
+          <t>Independent vet</t>
+        </is>
+      </c>
+      <c r="C325" s="4" t="inlineStr">
+        <is>
+          <t>West Wickham (Bromley/Beckenham)</t>
+        </is>
+      </c>
+      <c r="D325" s="4" t="inlineStr">
+        <is>
+          <t>https://tenderpaws.vet</t>
+        </is>
+      </c>
+      <c r="E325" s="4" t="inlineStr">
+        <is>
+          <t>mail@tenderpaws.vet</t>
+        </is>
+      </c>
+      <c r="F325" s="4" t="inlineStr"/>
+      <c r="G325" s="4" t="inlineStr"/>
+      <c r="H325" s="4" t="inlineStr"/>
+      <c r="I325" s="4" t="inlineStr"/>
+      <c r="J325" s="4" t="inlineStr">
+        <is>
+          <t>40+ years as a popular local vet - genuine multi-decade community fixture</t>
+        </is>
+      </c>
+      <c r="K325" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L325" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M325" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N325" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O325" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P325" s="4" t="inlineStr">
+        <is>
+          <t>40 years of community trust invisible against corporate vet marketing budgets</t>
+        </is>
+      </c>
+      <c r="Q325" s="4" t="inlineStr">
+        <is>
+          <t>'40 years as West Wickham's local vet - the AI answer should say so too'</t>
+        </is>
+      </c>
+      <c r="R325" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S325" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T325" s="4" t="inlineStr"/>
+    </row>
+    <row r="326">
+      <c r="A326" s="2" t="inlineStr">
+        <is>
+          <t>Great Tangley Manor</t>
+        </is>
+      </c>
+      <c r="B326" s="2" t="inlineStr">
+        <is>
+          <t>Wedding venue</t>
+        </is>
+      </c>
+      <c r="C326" s="2" t="inlineStr">
+        <is>
+          <t>Wonersh, Surrey (Surrey Hills AONB)</t>
+        </is>
+      </c>
+      <c r="D326" s="2" t="inlineStr">
+        <is>
+          <t>https://www.greattangleymanor.co.uk</t>
+        </is>
+      </c>
+      <c r="E326" s="2" t="inlineStr">
+        <is>
+          <t>info@greattangleymanor.co.uk</t>
+        </is>
+      </c>
+      <c r="F326" s="2" t="inlineStr">
+        <is>
+          <t>020 7526 4852</t>
+        </is>
+      </c>
+      <c r="G326" s="2" t="inlineStr"/>
+      <c r="H326" s="2" t="inlineStr"/>
+      <c r="I326" s="2" t="inlineStr"/>
+      <c r="J326" s="2" t="inlineStr">
+        <is>
+          <t>Grade I listed, reputedly Britain's oldest house (1,000 years) - among the most extraordinary heritage stories in the whole database</t>
+        </is>
+      </c>
+      <c r="K326" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L326" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M326" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N326" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O326" s="2" t="inlineStr">
+        <is>
+          <t>Detailed visual tour/local venues content</t>
+        </is>
+      </c>
+      <c r="P326" s="2" t="inlineStr">
+        <is>
+          <t>'Britain's oldest house' claim is an exceptional AEO asset barely leveraged beyond the website itself</t>
+        </is>
+      </c>
+      <c r="Q326" s="2" t="inlineStr">
+        <is>
+          <t>'Britain's oldest house as a wedding venue - that claim alone should dominate every AI answer for Surrey manor weddings'</t>
+        </is>
+      </c>
+      <c r="R326" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S326" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T326" s="2" t="inlineStr">
+        <is>
+          <t>Among the strongest heritage-story assets found in the whole database</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="4" t="inlineStr">
+        <is>
+          <t>Kingswood Manor</t>
+        </is>
+      </c>
+      <c r="B327" s="4" t="inlineStr">
+        <is>
+          <t>Wedding venue</t>
+        </is>
+      </c>
+      <c r="C327" s="4" t="inlineStr">
+        <is>
+          <t>Surrey Hills</t>
+        </is>
+      </c>
+      <c r="D327" s="4" t="inlineStr">
+        <is>
+          <t>https://www.kingswood-manor.co.uk</t>
+        </is>
+      </c>
+      <c r="E327" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F327" s="4" t="inlineStr"/>
+      <c r="G327" s="4" t="inlineStr"/>
+      <c r="H327" s="4" t="inlineStr"/>
+      <c r="I327" s="4" t="inlineStr"/>
+      <c r="J327" s="4" t="inlineStr">
+        <is>
+          <t>Surrey Hills setting with mature gardens; premium exclusive-use weddings</t>
+        </is>
+      </c>
+      <c r="K327" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L327" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M327" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N327" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O327" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P327" s="4" t="inlineStr">
+        <is>
+          <t>Generic 'Surrey Hills wedding venue' searches split across many similar venues</t>
+        </is>
+      </c>
+      <c r="Q327" s="4" t="inlineStr">
+        <is>
+          <t>Differentiate via specific garden/landscape AEO content vs generic rivals</t>
+        </is>
+      </c>
+      <c r="R327" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S327" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T327" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T318"/>
+  <autoFilter ref="A1:T327"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -27980,7 +28740,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B135"/>
+  <dimension ref="A1:B136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -28000,7 +28760,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>317</v>
+        <v>326</v>
       </c>
     </row>
     <row r="5">
@@ -28017,7 +28777,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7">
@@ -28033,21 +28793,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Private dentist</t>
+          <t>Wedding venue</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Wedding venue</t>
+          <t>Private dentist</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10">
@@ -28057,13 +28817,13 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Estate &amp; letting agent</t>
+          <t>Private GP</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -28073,7 +28833,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Private dentist / implants</t>
+          <t>Estate &amp; letting agent</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -28083,17 +28843,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Chartered accountants</t>
+          <t>Private dentist / implants</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Private GP</t>
+          <t>Chartered accountants</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -29307,6 +30067,16 @@
         </is>
       </c>
       <c r="B135" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Private GP &amp; dermatology</t>
+        </is>
+      </c>
+      <c r="B136" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 28: +6 prospects (332 total) - Sutton/Cheam, Berkshire recruitment, SE London mortgage broker
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$327</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$333</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T327"/>
+  <dimension ref="A1:T333"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -28728,8 +28728,528 @@
       </c>
       <c r="T327" s="4" t="inlineStr"/>
     </row>
+    <row r="328">
+      <c r="A328" s="4" t="inlineStr">
+        <is>
+          <t>Mi-Move</t>
+        </is>
+      </c>
+      <c r="B328" s="4" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C328" s="4" t="inlineStr">
+        <is>
+          <t>Sutton, Surrey</t>
+        </is>
+      </c>
+      <c r="D328" s="4" t="inlineStr">
+        <is>
+          <t>https://www.mi-move.com</t>
+        </is>
+      </c>
+      <c r="E328" s="4" t="inlineStr">
+        <is>
+          <t>info@mi-move.com</t>
+        </is>
+      </c>
+      <c r="F328" s="4" t="inlineStr">
+        <is>
+          <t>020 3538 0558</t>
+        </is>
+      </c>
+      <c r="G328" s="4" t="inlineStr"/>
+      <c r="H328" s="4" t="inlineStr"/>
+      <c r="I328" s="4" t="inlineStr"/>
+      <c r="J328" s="4" t="inlineStr">
+        <is>
+          <t>Independent covering Sutton/Cheam/Carshalton/Wallington/Banstead; 35+ years combined local sales experience</t>
+        </is>
+      </c>
+      <c r="K328" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L328" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M328" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N328" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O328" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P328" s="4" t="inlineStr">
+        <is>
+          <t>Belvoir/Cubitt &amp; West corporate brands compete for the same Sutton searches</t>
+        </is>
+      </c>
+      <c r="Q328" s="4" t="inlineStr">
+        <is>
+          <t>'35 years of local sales experience deserves to be the AI's answer for Sutton property'</t>
+        </is>
+      </c>
+      <c r="R328" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S328" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T328" s="4" t="inlineStr"/>
+    </row>
+    <row r="329">
+      <c r="A329" s="4" t="inlineStr">
+        <is>
+          <t>Cromwells Estate Agents</t>
+        </is>
+      </c>
+      <c r="B329" s="4" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C329" s="4" t="inlineStr">
+        <is>
+          <t>Wallington/Carshalton/Sutton/Croydon</t>
+        </is>
+      </c>
+      <c r="D329" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cromwellsestateagents.com</t>
+        </is>
+      </c>
+      <c r="E329" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F329" s="4" t="inlineStr"/>
+      <c r="G329" s="4" t="inlineStr"/>
+      <c r="H329" s="4" t="inlineStr"/>
+      <c r="I329" s="4" t="inlineStr"/>
+      <c r="J329" s="4" t="inlineStr">
+        <is>
+          <t>Privately owned, explicitly not bank/insurance-owned; wide 5-town South London/Surrey catchment</t>
+        </is>
+      </c>
+      <c r="K329" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L329" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M329" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N329" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O329" s="4" t="inlineStr">
+        <is>
+          <t>Independence explicitly promoted</t>
+        </is>
+      </c>
+      <c r="P329" s="4" t="inlineStr">
+        <is>
+          <t>'Not owned by a bank' positioning is a strong trust angle unused in AI-search content</t>
+        </is>
+      </c>
+      <c r="Q329" s="4" t="inlineStr">
+        <is>
+          <t>'Not owned by a bank or insurer' - own that exact independence positioning in AI answers</t>
+        </is>
+      </c>
+      <c r="R329" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S329" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T329" s="4" t="inlineStr"/>
+    </row>
+    <row r="330">
+      <c r="A330" s="4" t="inlineStr">
+        <is>
+          <t>Cheam Dental Practice</t>
+        </is>
+      </c>
+      <c r="B330" s="4" t="inlineStr">
+        <is>
+          <t>Private dentist</t>
+        </is>
+      </c>
+      <c r="C330" s="4" t="inlineStr">
+        <is>
+          <t>London Road, Sutton (Cheam)</t>
+        </is>
+      </c>
+      <c r="D330" s="4" t="inlineStr">
+        <is>
+          <t>via directory listing</t>
+        </is>
+      </c>
+      <c r="E330" s="4" t="inlineStr">
+        <is>
+          <t>cheamdental@hotmail.co.uk</t>
+        </is>
+      </c>
+      <c r="F330" s="4" t="inlineStr">
+        <is>
+          <t>020 8337 2886</t>
+        </is>
+      </c>
+      <c r="G330" s="4" t="inlineStr"/>
+      <c r="H330" s="4" t="inlineStr"/>
+      <c r="I330" s="4" t="inlineStr">
+        <is>
+          <t>facebook.com/p/Cheam-Dental-Practice-100041375306012</t>
+        </is>
+      </c>
+      <c r="J330" s="4" t="inlineStr">
+        <is>
+          <t>Long-standing local practice in affluent Cheam; Hotmail contact address signals low marketing infrastructure</t>
+        </is>
+      </c>
+      <c r="K330" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L330" s="4" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="M330" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N330" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O330" s="4" t="inlineStr">
+        <is>
+          <t>Facebook presence</t>
+        </is>
+      </c>
+      <c r="P330" s="4" t="inlineStr">
+        <is>
+          <t>Hotmail email is the classic infrastructure-gap tell seen throughout this database</t>
+        </is>
+      </c>
+      <c r="Q330" s="4" t="inlineStr">
+        <is>
+          <t>'A Hotmail address is costing you patients - let's modernise the whole digital front door'</t>
+        </is>
+      </c>
+      <c r="R330" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S330" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T330" s="4" t="inlineStr">
+        <is>
+          <t>Hotmail tell - same infrastructure-gap wedge pattern</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="4" t="inlineStr">
+        <is>
+          <t>Ninety 2 Dental</t>
+        </is>
+      </c>
+      <c r="B331" s="4" t="inlineStr">
+        <is>
+          <t>Private dentist / implants</t>
+        </is>
+      </c>
+      <c r="C331" s="4" t="inlineStr">
+        <is>
+          <t>Worcester Park (serves Sutton/Cheam/Raynes Park/Wimbledon)</t>
+        </is>
+      </c>
+      <c r="D331" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ninety2dental.co.uk</t>
+        </is>
+      </c>
+      <c r="E331" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F331" s="4" t="inlineStr">
+        <is>
+          <t>020 8337 1168</t>
+        </is>
+      </c>
+      <c r="G331" s="4" t="inlineStr"/>
+      <c r="H331" s="4" t="inlineStr"/>
+      <c r="I331" s="4" t="inlineStr"/>
+      <c r="J331" s="4" t="inlineStr">
+        <is>
+          <t>Free-consultation implant offer across 4 SW London towns; volume-oriented private model</t>
+        </is>
+      </c>
+      <c r="K331" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L331" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M331" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N331" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O331" s="4" t="inlineStr">
+        <is>
+          <t>Free-consultation offer promoted</t>
+        </is>
+      </c>
+      <c r="P331" s="4" t="inlineStr">
+        <is>
+          <t>4-town catchment claim not matched by per-town search dominance</t>
+        </is>
+      </c>
+      <c r="Q331" s="4" t="inlineStr">
+        <is>
+          <t>Per-town AEO content to actually own the 4 areas served</t>
+        </is>
+      </c>
+      <c r="R331" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S331" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T331" s="4" t="inlineStr"/>
+    </row>
+    <row r="332">
+      <c r="A332" s="4" t="inlineStr">
+        <is>
+          <t>The Recruiters Room</t>
+        </is>
+      </c>
+      <c r="B332" s="4" t="inlineStr">
+        <is>
+          <t>Recruitment agency</t>
+        </is>
+      </c>
+      <c r="C332" s="4" t="inlineStr">
+        <is>
+          <t>Bracknell, Berkshire (serves Basingstoke/Hampshire/Surrey)</t>
+        </is>
+      </c>
+      <c r="D332" s="4" t="inlineStr">
+        <is>
+          <t>https://therecruitersroom.co.uk</t>
+        </is>
+      </c>
+      <c r="E332" s="4" t="inlineStr">
+        <is>
+          <t>info@therecruitersroom.co.uk</t>
+        </is>
+      </c>
+      <c r="F332" s="4" t="inlineStr"/>
+      <c r="G332" s="4" t="inlineStr">
+        <is>
+          <t>Two founders known as 'the two Lauras' (35+ yrs combined, est. 2016)</t>
+        </is>
+      </c>
+      <c r="H332" s="4" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/the-recruiters-room</t>
+        </is>
+      </c>
+      <c r="I332" s="4" t="inlineStr"/>
+      <c r="J332" s="4" t="inlineStr">
+        <is>
+          <t>Founder-led boutique with a distinctive brand identity and 35 years' combined recruitment experience</t>
+        </is>
+      </c>
+      <c r="K332" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L332" s="4" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M332" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N332" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O332" s="4" t="inlineStr">
+        <is>
+          <t>Distinctive branding; LinkedIn presence</t>
+        </is>
+      </c>
+      <c r="P332" s="4" t="inlineStr">
+        <is>
+          <t>Distinctive brand identity not yet converted into AI-search dominance for Berkshire/Hampshire recruitment</t>
+        </is>
+      </c>
+      <c r="Q332" s="4" t="inlineStr">
+        <is>
+          <t>'The two Lauras' - own that memorable branding in AI-search answers too</t>
+        </is>
+      </c>
+      <c r="R332" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S332" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T332" s="4" t="inlineStr"/>
+    </row>
+    <row r="333">
+      <c r="A333" s="3" t="inlineStr">
+        <is>
+          <t>Olympia Finance</t>
+        </is>
+      </c>
+      <c r="B333" s="3" t="inlineStr">
+        <is>
+          <t>Mortgage broker</t>
+        </is>
+      </c>
+      <c r="C333" s="3" t="inlineStr">
+        <is>
+          <t>Covent Garden, London (serves Eltham/Sidcup/Bexley/Woolwich/Dartford/Lewisham/Essex)</t>
+        </is>
+      </c>
+      <c r="D333" s="3" t="inlineStr">
+        <is>
+          <t>https://olympiafinance.co.uk</t>
+        </is>
+      </c>
+      <c r="E333" s="3" t="inlineStr">
+        <is>
+          <t>info@olympiafinance.co.uk</t>
+        </is>
+      </c>
+      <c r="F333" s="3" t="inlineStr">
+        <is>
+          <t>0207 096 1988</t>
+        </is>
+      </c>
+      <c r="G333" s="3" t="inlineStr">
+        <is>
+          <t>Ashan Sarkar (Director)</t>
+        </is>
+      </c>
+      <c r="H333" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/olympiafinance</t>
+        </is>
+      </c>
+      <c r="I333" s="3" t="inlineStr"/>
+      <c r="J333" s="3" t="inlineStr">
+        <is>
+          <t>Whole-of-market broker with per-area landing pages across 8+ SE London/Essex towns - genuine SEO investment</t>
+        </is>
+      </c>
+      <c r="K333" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L333" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M333" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N333" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O333" s="3" t="inlineStr">
+        <is>
+          <t>Extensive per-area landing pages = active SEO strategy</t>
+        </is>
+      </c>
+      <c r="P333" s="3" t="inlineStr">
+        <is>
+          <t>Landing pages exist across 8+ areas but AI-answer citations still open for most of them</t>
+        </is>
+      </c>
+      <c r="Q333" s="3" t="inlineStr">
+        <is>
+          <t>'You've built pages for 8 areas - the AEO layer could multiply that investment overnight'</t>
+        </is>
+      </c>
+      <c r="R333" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S333" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T333" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T327"/>
+  <autoFilter ref="A1:T333"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -28760,7 +29280,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>326</v>
+        <v>332</v>
       </c>
     </row>
     <row r="5">
@@ -28777,7 +29297,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7">
@@ -28793,7 +29313,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Wedding venue</t>
+          <t>Private dentist</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -28803,11 +29323,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Private dentist</t>
+          <t>Wedding venue</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10">
@@ -28823,17 +29343,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Private GP</t>
+          <t>Private dentist / implants</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Estate &amp; letting agent</t>
+          <t>Private GP</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -28843,7 +29363,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Private dentist / implants</t>
+          <t>Estate &amp; letting agent</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -28883,7 +29403,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Solar installer</t>
+          <t>Mortgage broker</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -28893,7 +29413,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>IT support / MSP</t>
+          <t>Solar installer</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -28903,21 +29423,21 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Mortgage broker</t>
+          <t>Recruitment agency</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Recruitment agency</t>
+          <t>IT support / MSP</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
Batch 29: +7 prospects (339 total) - Reading/Wokingham (Berkshire)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$333</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$340</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T333"/>
+  <dimension ref="A1:T340"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -29248,8 +29248,604 @@
       </c>
       <c r="T333" s="3" t="inlineStr"/>
     </row>
+    <row r="334">
+      <c r="A334" s="3" t="inlineStr">
+        <is>
+          <t>Bespoke Estate Agents</t>
+        </is>
+      </c>
+      <c r="B334" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C334" s="3" t="inlineStr">
+        <is>
+          <t>Reading, Berkshire (+ South Oxfordshire)</t>
+        </is>
+      </c>
+      <c r="D334" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mybespokeagent.com</t>
+        </is>
+      </c>
+      <c r="E334" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F334" s="3" t="inlineStr"/>
+      <c r="G334" s="3" t="inlineStr">
+        <is>
+          <t>Mark Heneghan MNAEA (Founder, 30+ years)</t>
+        </is>
+      </c>
+      <c r="H334" s="3" t="inlineStr"/>
+      <c r="I334" s="3" t="inlineStr"/>
+      <c r="J334" s="3" t="inlineStr">
+        <is>
+          <t>Founder personally involved with every client for 30 years; local-knowledge positioning across Berkshire/South Oxon</t>
+        </is>
+      </c>
+      <c r="K334" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L334" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M334" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N334" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O334" s="3" t="inlineStr">
+        <is>
+          <t>Alumni/community directory presence</t>
+        </is>
+      </c>
+      <c r="P334" s="3" t="inlineStr">
+        <is>
+          <t>30 years of personal service invisible against Winkworth/Chancellors corporate brands in Reading search</t>
+        </is>
+      </c>
+      <c r="Q334" s="3" t="inlineStr">
+        <is>
+          <t>'A founder who personally guides every client for 30 years - own that story in AI answers'</t>
+        </is>
+      </c>
+      <c r="R334" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S334" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T334" s="3" t="inlineStr"/>
+    </row>
+    <row r="335">
+      <c r="A335" s="3" t="inlineStr">
+        <is>
+          <t>Quarters</t>
+        </is>
+      </c>
+      <c r="B335" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C335" s="3" t="inlineStr">
+        <is>
+          <t>Rose Street, Wokingham, Berkshire</t>
+        </is>
+      </c>
+      <c r="D335" s="3" t="inlineStr">
+        <is>
+          <t>https://www.quarters.agency</t>
+        </is>
+      </c>
+      <c r="E335" s="3" t="inlineStr">
+        <is>
+          <t>hello@quarters.agency</t>
+        </is>
+      </c>
+      <c r="F335" s="3" t="inlineStr">
+        <is>
+          <t>0118 466 0292</t>
+        </is>
+      </c>
+      <c r="G335" s="3" t="inlineStr">
+        <is>
+          <t>Co-founders with 40+ years combined experience (est. 2003)</t>
+        </is>
+      </c>
+      <c r="H335" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/QuartersResidential</t>
+        </is>
+      </c>
+      <c r="I335" s="3" t="inlineStr"/>
+      <c r="J335" s="3" t="inlineStr">
+        <is>
+          <t>Deliberately boutique - only partners with a small handful of families at a time; bespoke marketing per home</t>
+        </is>
+      </c>
+      <c r="K335" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L335" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M335" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N335" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O335" s="3" t="inlineStr">
+        <is>
+          <t>Journal/values content = active brand marketing</t>
+        </is>
+      </c>
+      <c r="P335" s="3" t="inlineStr">
+        <is>
+          <t>Boutique-by-design positioning not yet the AI-cited answer for premium Wokingham property</t>
+        </is>
+      </c>
+      <c r="Q335" s="3" t="inlineStr">
+        <is>
+          <t>'Deliberately small, deliberately bespoke - own that AEO positioning against volume agents'</t>
+        </is>
+      </c>
+      <c r="R335" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S335" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T335" s="3" t="inlineStr"/>
+    </row>
+    <row r="336">
+      <c r="A336" s="4" t="inlineStr">
+        <is>
+          <t>Wentworth Estate Agents</t>
+        </is>
+      </c>
+      <c r="B336" s="4" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C336" s="4" t="inlineStr">
+        <is>
+          <t>Twyford/Woodley (serves Reading), Berkshire</t>
+        </is>
+      </c>
+      <c r="D336" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wentworthestateagents.com</t>
+        </is>
+      </c>
+      <c r="E336" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F336" s="4" t="inlineStr"/>
+      <c r="G336" s="4" t="inlineStr">
+        <is>
+          <t>Adrian Laflin (Founder, est. 2000)</t>
+        </is>
+      </c>
+      <c r="H336" s="4" t="inlineStr"/>
+      <c r="I336" s="4" t="inlineStr"/>
+      <c r="J336" s="4" t="inlineStr">
+        <is>
+          <t>Independent since 2000, founder actively involved day-to-day across the Reading commuter belt</t>
+        </is>
+      </c>
+      <c r="K336" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L336" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M336" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N336" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O336" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P336" s="4" t="inlineStr">
+        <is>
+          <t>24 years of active founder involvement untranslated into modern search presence</t>
+        </is>
+      </c>
+      <c r="Q336" s="4" t="inlineStr">
+        <is>
+          <t>'A founder still hands-on after 24 years - own that trust story in AI answers'</t>
+        </is>
+      </c>
+      <c r="R336" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S336" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T336" s="4" t="inlineStr"/>
+    </row>
+    <row r="337">
+      <c r="A337" s="3" t="inlineStr">
+        <is>
+          <t>Reading Dental Spa</t>
+        </is>
+      </c>
+      <c r="B337" s="3" t="inlineStr">
+        <is>
+          <t>Private dentist / implants</t>
+        </is>
+      </c>
+      <c r="C337" s="3" t="inlineStr">
+        <is>
+          <t>Wokingham Road, Reading, Berkshire</t>
+        </is>
+      </c>
+      <c r="D337" s="3" t="inlineStr">
+        <is>
+          <t>https://www.readingdentalspa.co.uk</t>
+        </is>
+      </c>
+      <c r="E337" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F337" s="3" t="inlineStr">
+        <is>
+          <t>01183 272 322</t>
+        </is>
+      </c>
+      <c r="G337" s="3" t="inlineStr"/>
+      <c r="H337" s="3" t="inlineStr"/>
+      <c r="I337" s="3" t="inlineStr"/>
+      <c r="J337" s="3" t="inlineStr">
+        <is>
+          <t>Dedicated implant-offer landing page shows active SEO investment; spa-style premium positioning</t>
+        </is>
+      </c>
+      <c r="K337" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L337" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M337" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N337" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O337" s="3" t="inlineStr">
+        <is>
+          <t>Dedicated implant-offer page = active SEO</t>
+        </is>
+      </c>
+      <c r="P337" s="3" t="inlineStr">
+        <is>
+          <t>Implant offer page exists but AI-answer citations for 'dental implants Reading' still open</t>
+        </is>
+      </c>
+      <c r="Q337" s="3" t="inlineStr">
+        <is>
+          <t>Upgrade the existing implant-offer SEO page into an AEO-optimised asset</t>
+        </is>
+      </c>
+      <c r="R337" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S337" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T337" s="3" t="inlineStr"/>
+    </row>
+    <row r="338">
+      <c r="A338" s="4" t="inlineStr">
+        <is>
+          <t>Earley Dental Practice</t>
+        </is>
+      </c>
+      <c r="B338" s="4" t="inlineStr">
+        <is>
+          <t>Private dentist / implants</t>
+        </is>
+      </c>
+      <c r="C338" s="4" t="inlineStr">
+        <is>
+          <t>Earley, Reading, Berkshire</t>
+        </is>
+      </c>
+      <c r="D338" s="4" t="inlineStr">
+        <is>
+          <t>https://earleydentist.co.uk</t>
+        </is>
+      </c>
+      <c r="E338" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F338" s="4" t="inlineStr"/>
+      <c r="G338" s="4" t="inlineStr"/>
+      <c r="H338" s="4" t="inlineStr"/>
+      <c r="I338" s="4" t="inlineStr"/>
+      <c r="J338" s="4" t="inlineStr">
+        <is>
+          <t>Well-established private practice with dedicated implants category page</t>
+        </is>
+      </c>
+      <c r="K338" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L338" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M338" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N338" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O338" s="4" t="inlineStr">
+        <is>
+          <t>Dedicated implants category page</t>
+        </is>
+      </c>
+      <c r="P338" s="4" t="inlineStr">
+        <is>
+          <t>Reading Dental Spa and Puresmile Earley compete for the same implant searches</t>
+        </is>
+      </c>
+      <c r="Q338" s="4" t="inlineStr">
+        <is>
+          <t>Differentiate via specific implant-technique AEO content vs generic rivals</t>
+        </is>
+      </c>
+      <c r="R338" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S338" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T338" s="4" t="inlineStr"/>
+    </row>
+    <row r="339">
+      <c r="A339" s="3" t="inlineStr">
+        <is>
+          <t>Heritage Revival</t>
+        </is>
+      </c>
+      <c r="B339" s="3" t="inlineStr">
+        <is>
+          <t>Architects (heritage specialism)</t>
+        </is>
+      </c>
+      <c r="C339" s="3" t="inlineStr">
+        <is>
+          <t>Broad Street, Wokingham, Berkshire</t>
+        </is>
+      </c>
+      <c r="D339" s="3" t="inlineStr">
+        <is>
+          <t>https://heritagerevival.uk</t>
+        </is>
+      </c>
+      <c r="E339" s="3" t="inlineStr">
+        <is>
+          <t>info@heritagerevival.uk</t>
+        </is>
+      </c>
+      <c r="F339" s="3" t="inlineStr">
+        <is>
+          <t>0118 403 2885</t>
+        </is>
+      </c>
+      <c r="G339" s="3" t="inlineStr"/>
+      <c r="H339" s="3" t="inlineStr"/>
+      <c r="I339" s="3" t="inlineStr"/>
+      <c r="J339" s="3" t="inlineStr">
+        <is>
+          <t>Heritage/listed-building architecture specialism - genuinely defensible niche vs generic residential architects</t>
+        </is>
+      </c>
+      <c r="K339" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L339" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M339" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N339" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O339" s="3" t="inlineStr">
+        <is>
+          <t>Niche name/positioning ('Heritage Revival')</t>
+        </is>
+      </c>
+      <c r="P339" s="3" t="inlineStr">
+        <is>
+          <t>Heritage specialism is a strong AEO niche barely contested in Berkshire search</t>
+        </is>
+      </c>
+      <c r="Q339" s="3" t="inlineStr">
+        <is>
+          <t>Own 'listed building architect Berkshire' - a specific, low-competition AEO target</t>
+        </is>
+      </c>
+      <c r="R339" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S339" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T339" s="3" t="inlineStr"/>
+    </row>
+    <row r="340">
+      <c r="A340" s="4" t="inlineStr">
+        <is>
+          <t>Millward, May &amp; Co</t>
+        </is>
+      </c>
+      <c r="B340" s="4" t="inlineStr">
+        <is>
+          <t>Chartered accountants</t>
+        </is>
+      </c>
+      <c r="C340" s="4" t="inlineStr">
+        <is>
+          <t>Peach Street, Wokingham, Berkshire</t>
+        </is>
+      </c>
+      <c r="D340" s="4" t="inlineStr">
+        <is>
+          <t>https://www.millwardmay.co.uk</t>
+        </is>
+      </c>
+      <c r="E340" s="4" t="inlineStr">
+        <is>
+          <t>emma@millwardmay.co.uk</t>
+        </is>
+      </c>
+      <c r="F340" s="4" t="inlineStr">
+        <is>
+          <t>0118 380 0363</t>
+        </is>
+      </c>
+      <c r="G340" s="4" t="inlineStr">
+        <is>
+          <t>Emma May &amp; Ben Hicks (Partners)</t>
+        </is>
+      </c>
+      <c r="H340" s="4" t="inlineStr"/>
+      <c r="I340" s="4" t="inlineStr"/>
+      <c r="J340" s="4" t="inlineStr">
+        <is>
+          <t>Independent firm for business owners; named partners with direct emails; recurring-fee SME client base</t>
+        </is>
+      </c>
+      <c r="K340" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L340" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M340" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N340" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O340" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P340" s="4" t="inlineStr">
+        <is>
+          <t>Generic 'accountant Wokingham' searches won by TaxAssist/national franchise brands</t>
+        </is>
+      </c>
+      <c r="Q340" s="4" t="inlineStr">
+        <is>
+          <t>'For business owners' positioning - own that specific AEO angle vs generic accountancy search</t>
+        </is>
+      </c>
+      <c r="R340" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S340" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T340" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T333"/>
+  <autoFilter ref="A1:T340"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -29260,7 +29856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B136"/>
+  <dimension ref="A1:B137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -29280,7 +29876,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>332</v>
+        <v>339</v>
       </c>
     </row>
     <row r="5">
@@ -29297,7 +29893,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="7">
@@ -29347,13 +29943,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Private GP</t>
+          <t>Chartered accountants</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -29363,7 +29959,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Estate &amp; letting agent</t>
+          <t>Private GP</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -29373,11 +29969,11 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Chartered accountants</t>
+          <t>Estate &amp; letting agent</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15">
@@ -30597,6 +31193,16 @@
         </is>
       </c>
       <c r="B136" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Architects (heritage specialism)</t>
+        </is>
+      </c>
+      <c r="B137" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 30: +8 prospects (347 total) - Basingstoke, Wokingham solar, Reading heating
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$340</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$348</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T340"/>
+  <dimension ref="A1:T348"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -29844,8 +29844,708 @@
       </c>
       <c r="T340" s="4" t="inlineStr"/>
     </row>
+    <row r="341">
+      <c r="A341" s="4" t="inlineStr">
+        <is>
+          <t>Jacobs Properties</t>
+        </is>
+      </c>
+      <c r="B341" s="4" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C341" s="4" t="inlineStr">
+        <is>
+          <t>Basingstoke, Hampshire</t>
+        </is>
+      </c>
+      <c r="D341" s="4" t="inlineStr">
+        <is>
+          <t>https://www.jacobs.properties</t>
+        </is>
+      </c>
+      <c r="E341" s="4" t="inlineStr">
+        <is>
+          <t>info@jacobs.properties</t>
+        </is>
+      </c>
+      <c r="F341" s="4" t="inlineStr">
+        <is>
+          <t>01256 781 300</t>
+        </is>
+      </c>
+      <c r="G341" s="4" t="inlineStr">
+        <is>
+          <t>Jon Coombs (Owner, est. 1999)</t>
+        </is>
+      </c>
+      <c r="H341" s="4" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/jon-coombs</t>
+        </is>
+      </c>
+      <c r="I341" s="4" t="inlineStr"/>
+      <c r="J341" s="4" t="inlineStr">
+        <is>
+          <t>Independent since 1999, self-described 'people's estate agent'; friendly-service positioning in Basingstoke commuter belt</t>
+        </is>
+      </c>
+      <c r="K341" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L341" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M341" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N341" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O341" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P341" s="4" t="inlineStr">
+        <is>
+          <t>'People's estate agent' branding not yet the AI-cited answer for Basingstoke property search</t>
+        </is>
+      </c>
+      <c r="Q341" s="4" t="inlineStr">
+        <is>
+          <t>Own the friendly/people-first AEO positioning against corporate Basingstoke rivals</t>
+        </is>
+      </c>
+      <c r="R341" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S341" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T341" s="4" t="inlineStr"/>
+    </row>
+    <row r="342">
+      <c r="A342" s="4" t="inlineStr">
+        <is>
+          <t>Barons Estate Agents</t>
+        </is>
+      </c>
+      <c r="B342" s="4" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C342" s="4" t="inlineStr">
+        <is>
+          <t>Winton Square, Basingstoke, Hampshire</t>
+        </is>
+      </c>
+      <c r="D342" s="4" t="inlineStr">
+        <is>
+          <t>https://www.viewagents.com/estate-agent/Basingstoke/Barons-Estate-Agents</t>
+        </is>
+      </c>
+      <c r="E342" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F342" s="4" t="inlineStr"/>
+      <c r="G342" s="4" t="inlineStr">
+        <is>
+          <t>Kevin Penfold &amp; Trevor Lee (Founders, est. 1988)</t>
+        </is>
+      </c>
+      <c r="H342" s="4" t="inlineStr"/>
+      <c r="I342" s="4" t="inlineStr"/>
+      <c r="J342" s="4" t="inlineStr">
+        <is>
+          <t>36-year independent firm still trading from its original office; long local heritage</t>
+        </is>
+      </c>
+      <c r="K342" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L342" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M342" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N342" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O342" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P342" s="4" t="inlineStr">
+        <is>
+          <t>36 years of continuous trading undersold as an AEO trust signal</t>
+        </is>
+      </c>
+      <c r="Q342" s="4" t="inlineStr">
+        <is>
+          <t>'Same office, same name, 36 years - make AI say so, not just Companies House'</t>
+        </is>
+      </c>
+      <c r="R342" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S342" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T342" s="4" t="inlineStr"/>
+    </row>
+    <row r="343">
+      <c r="A343" s="4" t="inlineStr">
+        <is>
+          <t>Sansome and George</t>
+        </is>
+      </c>
+      <c r="B343" s="4" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C343" s="4" t="inlineStr">
+        <is>
+          <t>Basingstoke, Hampshire</t>
+        </is>
+      </c>
+      <c r="D343" s="4" t="inlineStr">
+        <is>
+          <t>https://www.sansomeandgeorge.co.uk</t>
+        </is>
+      </c>
+      <c r="E343" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F343" s="4" t="inlineStr"/>
+      <c r="G343" s="4" t="inlineStr"/>
+      <c r="H343" s="4" t="inlineStr"/>
+      <c r="I343" s="4" t="inlineStr"/>
+      <c r="J343" s="4" t="inlineStr">
+        <is>
+          <t>Family-run independent providing personal service across Basingstoke</t>
+        </is>
+      </c>
+      <c r="K343" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L343" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M343" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N343" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O343" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P343" s="4" t="inlineStr">
+        <is>
+          <t>Family-run positioning invisible against Fine &amp; Country/corporate rivals in Basingstoke search</t>
+        </is>
+      </c>
+      <c r="Q343" s="4" t="inlineStr">
+        <is>
+          <t>Own the family-run/personal-service AEO positioning outright</t>
+        </is>
+      </c>
+      <c r="R343" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S343" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T343" s="4" t="inlineStr"/>
+    </row>
+    <row r="344">
+      <c r="A344" s="4" t="inlineStr">
+        <is>
+          <t>Bounty Road Dental</t>
+        </is>
+      </c>
+      <c r="B344" s="4" t="inlineStr">
+        <is>
+          <t>Private dentist / implants</t>
+        </is>
+      </c>
+      <c r="C344" s="4" t="inlineStr">
+        <is>
+          <t>Basingstoke, Hampshire</t>
+        </is>
+      </c>
+      <c r="D344" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bountyroaddental.co.uk</t>
+        </is>
+      </c>
+      <c r="E344" s="4" t="inlineStr">
+        <is>
+          <t>info@bountyroaddental.co.uk</t>
+        </is>
+      </c>
+      <c r="F344" s="4" t="inlineStr">
+        <is>
+          <t>01256 465 764</t>
+        </is>
+      </c>
+      <c r="G344" s="4" t="inlineStr"/>
+      <c r="H344" s="4" t="inlineStr"/>
+      <c r="I344" s="4" t="inlineStr"/>
+      <c r="J344" s="4" t="inlineStr">
+        <is>
+          <t>Friendly, affordable-positioned implant/cosmetic private practice in Basingstoke</t>
+        </is>
+      </c>
+      <c r="K344" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L344" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M344" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N344" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O344" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P344" s="4" t="inlineStr">
+        <is>
+          <t>'Affordable + high-quality' positioning not yet the AI-cited local answer</t>
+        </is>
+      </c>
+      <c r="Q344" s="4" t="inlineStr">
+        <is>
+          <t>Own the value-conscious implant-patient AEO segment in Basingstoke</t>
+        </is>
+      </c>
+      <c r="R344" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S344" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T344" s="4" t="inlineStr"/>
+    </row>
+    <row r="345">
+      <c r="A345" s="3" t="inlineStr">
+        <is>
+          <t>Gwynne Dental</t>
+        </is>
+      </c>
+      <c r="B345" s="3" t="inlineStr">
+        <is>
+          <t>Private cosmetic dentist / implants</t>
+        </is>
+      </c>
+      <c r="C345" s="3" t="inlineStr">
+        <is>
+          <t>Basingstoke, Hampshire</t>
+        </is>
+      </c>
+      <c r="D345" s="3" t="inlineStr">
+        <is>
+          <t>https://gwynnedental.co.uk</t>
+        </is>
+      </c>
+      <c r="E345" s="3" t="inlineStr">
+        <is>
+          <t>office@gwynnedental.co.uk</t>
+        </is>
+      </c>
+      <c r="F345" s="3" t="inlineStr">
+        <is>
+          <t>01256 321 945</t>
+        </is>
+      </c>
+      <c r="G345" s="3" t="inlineStr">
+        <is>
+          <t>Dr Sophie Clark-Lipscomb (Oral Surgeon)</t>
+        </is>
+      </c>
+      <c r="H345" s="3" t="inlineStr"/>
+      <c r="I345" s="3" t="inlineStr"/>
+      <c r="J345" s="3" t="inlineStr">
+        <is>
+          <t>Named oral surgeon providing implant treatment; leading private cosmetic dentist positioning</t>
+        </is>
+      </c>
+      <c r="K345" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L345" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M345" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N345" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O345" s="3" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P345" s="3" t="inlineStr">
+        <is>
+          <t>Named-surgeon credential not leveraged as the AI-cited trust signal for implant searches</t>
+        </is>
+      </c>
+      <c r="Q345" s="3" t="inlineStr">
+        <is>
+          <t>'A named oral surgeon doing your implants' - own that credibility angle in AEO content</t>
+        </is>
+      </c>
+      <c r="R345" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S345" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T345" s="3" t="inlineStr"/>
+    </row>
+    <row r="346">
+      <c r="A346" s="3" t="inlineStr">
+        <is>
+          <t>The Hampshire Vet</t>
+        </is>
+      </c>
+      <c r="B346" s="3" t="inlineStr">
+        <is>
+          <t>Independent vet</t>
+        </is>
+      </c>
+      <c r="C346" s="3" t="inlineStr">
+        <is>
+          <t>Beggarwood, Basingstoke, Hampshire</t>
+        </is>
+      </c>
+      <c r="D346" s="3" t="inlineStr">
+        <is>
+          <t>https://www.thehampshirevet.co.uk</t>
+        </is>
+      </c>
+      <c r="E346" s="3" t="inlineStr">
+        <is>
+          <t>info@thehampshirevet.co.uk</t>
+        </is>
+      </c>
+      <c r="F346" s="3" t="inlineStr">
+        <is>
+          <t>01256 639 707</t>
+        </is>
+      </c>
+      <c r="G346" s="3" t="inlineStr">
+        <is>
+          <t>Emily &amp; Jamie (Founders, both head vets)</t>
+        </is>
+      </c>
+      <c r="H346" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/thehampshirevet</t>
+        </is>
+      </c>
+      <c r="I346" s="3" t="inlineStr"/>
+      <c r="J346" s="3" t="inlineStr">
+        <is>
+          <t>New independent practice with onsite overnight care - genuine differentiator vs corporate day-only branches</t>
+        </is>
+      </c>
+      <c r="K346" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L346" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M346" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N346" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O346" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence; onsite-care positioning</t>
+        </is>
+      </c>
+      <c r="P346" s="3" t="inlineStr">
+        <is>
+          <t>New practice needs fast search-authority building against established corporate Basingstoke vets</t>
+        </is>
+      </c>
+      <c r="Q346" s="3" t="inlineStr">
+        <is>
+          <t>'Overnight care onsite - own that AEO differentiator before corporate chains copy it'</t>
+        </is>
+      </c>
+      <c r="R346" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S346" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T346" s="3" t="inlineStr"/>
+    </row>
+    <row r="347">
+      <c r="A347" s="3" t="inlineStr">
+        <is>
+          <t>Wokingham Solar</t>
+        </is>
+      </c>
+      <c r="B347" s="3" t="inlineStr">
+        <is>
+          <t>Solar installer</t>
+        </is>
+      </c>
+      <c r="C347" s="3" t="inlineStr">
+        <is>
+          <t>Wokingham, Berkshire</t>
+        </is>
+      </c>
+      <c r="D347" s="3" t="inlineStr">
+        <is>
+          <t>https://www.wokinghamsolar.co.uk</t>
+        </is>
+      </c>
+      <c r="E347" s="3" t="inlineStr">
+        <is>
+          <t>hello@wokinghamsolar.co.uk</t>
+        </is>
+      </c>
+      <c r="F347" s="3" t="inlineStr">
+        <is>
+          <t>0118 449 2824</t>
+        </is>
+      </c>
+      <c r="G347" s="3" t="inlineStr">
+        <is>
+          <t>Paul &amp; Simon (Founders)</t>
+        </is>
+      </c>
+      <c r="H347" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/p/Wokingham-Solar-61568618596545</t>
+        </is>
+      </c>
+      <c r="I347" s="3" t="inlineStr"/>
+      <c r="J347" s="3" t="inlineStr">
+        <is>
+          <t>MCS installer with dedicated case-studies page - active SEO/proof-point investment</t>
+        </is>
+      </c>
+      <c r="K347" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L347" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M347" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N347" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O347" s="3" t="inlineStr">
+        <is>
+          <t>Case studies page = active content marketing</t>
+        </is>
+      </c>
+      <c r="P347" s="3" t="inlineStr">
+        <is>
+          <t>Case studies exist but AI-answer citations for 'solar installer Wokingham' still open</t>
+        </is>
+      </c>
+      <c r="Q347" s="3" t="inlineStr">
+        <is>
+          <t>Turn existing case studies into AEO-optimised proof-point content</t>
+        </is>
+      </c>
+      <c r="R347" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S347" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T347" s="3" t="inlineStr"/>
+    </row>
+    <row r="348">
+      <c r="A348" s="4" t="inlineStr">
+        <is>
+          <t>FlexiFlame</t>
+        </is>
+      </c>
+      <c r="B348" s="4" t="inlineStr">
+        <is>
+          <t>Heating engineer / plumbing</t>
+        </is>
+      </c>
+      <c r="C348" s="4" t="inlineStr">
+        <is>
+          <t>Tilehurst, Reading (serves Berkshire)</t>
+        </is>
+      </c>
+      <c r="D348" s="4" t="inlineStr">
+        <is>
+          <t>https://www.flexiflame.co.uk</t>
+        </is>
+      </c>
+      <c r="E348" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F348" s="4" t="inlineStr">
+        <is>
+          <t>0118 945 1999</t>
+        </is>
+      </c>
+      <c r="G348" s="4" t="inlineStr">
+        <is>
+          <t>Michael Pearse (Founder, 20+ years, Gas Safe)</t>
+        </is>
+      </c>
+      <c r="H348" s="4" t="inlineStr"/>
+      <c r="I348" s="4" t="inlineStr"/>
+      <c r="J348" s="4" t="inlineStr">
+        <is>
+          <t>20-year independent Gas Safe engineer; boiler/appliance repairs across Berkshire homes and businesses</t>
+        </is>
+      </c>
+      <c r="K348" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L348" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M348" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N348" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O348" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P348" s="4" t="inlineStr">
+        <is>
+          <t>MyBuilder/Checkatrade intercept heating-engineer searches before independents are found directly</t>
+        </is>
+      </c>
+      <c r="Q348" s="4" t="inlineStr">
+        <is>
+          <t>'20 years Gas Safe registered - stop paying Checkatrade for leads to your own patch'</t>
+        </is>
+      </c>
+      <c r="R348" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S348" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T348" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T340"/>
+  <autoFilter ref="A1:T348"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -29856,7 +30556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B137"/>
+  <dimension ref="A1:B139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -29876,7 +30576,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>339</v>
+        <v>347</v>
       </c>
     </row>
     <row r="5">
@@ -29893,7 +30593,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7">
@@ -29919,7 +30619,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Wedding venue</t>
+          <t>Independent vet</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -29929,11 +30629,11 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Independent vet</t>
+          <t>Wedding venue</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11">
@@ -29943,7 +30643,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12">
@@ -29999,17 +30699,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Mortgage broker</t>
+          <t>Solar installer</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Solar installer</t>
+          <t>Mortgage broker</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -31203,6 +31903,26 @@
         </is>
       </c>
       <c r="B137" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Private cosmetic dentist / implants</t>
+        </is>
+      </c>
+      <c r="B138" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Heating engineer / plumbing</t>
+        </is>
+      </c>
+      <c r="B139" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 31: +8 prospects (355 total) - Newbury, Berkshire wedding venues, Berkshire GP
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$348</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$356</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T348"/>
+  <dimension ref="A1:T356"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -30544,8 +30544,692 @@
       </c>
       <c r="T348" s="4" t="inlineStr"/>
     </row>
+    <row r="349">
+      <c r="A349" s="3" t="inlineStr">
+        <is>
+          <t>Downer &amp; Co</t>
+        </is>
+      </c>
+      <c r="B349" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C349" s="3" t="inlineStr">
+        <is>
+          <t>Cheap Street, Newbury, Berkshire</t>
+        </is>
+      </c>
+      <c r="D349" s="3" t="inlineStr">
+        <is>
+          <t>https://www.downer.co.uk</t>
+        </is>
+      </c>
+      <c r="E349" s="3" t="inlineStr">
+        <is>
+          <t>simon.downer@downer.co.uk</t>
+        </is>
+      </c>
+      <c r="F349" s="3" t="inlineStr">
+        <is>
+          <t>01635 523 777</t>
+        </is>
+      </c>
+      <c r="G349" s="3" t="inlineStr">
+        <is>
+          <t>Simon Downer (Founder, est. 1988)</t>
+        </is>
+      </c>
+      <c r="H349" s="3" t="inlineStr"/>
+      <c r="I349" s="3" t="inlineStr"/>
+      <c r="J349" s="3" t="inlineStr">
+        <is>
+          <t>36-year entirely independent firm; founder still directly contactable; premium West Berkshire property fees</t>
+        </is>
+      </c>
+      <c r="K349" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L349" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M349" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N349" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O349" s="3" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P349" s="3" t="inlineStr">
+        <is>
+          <t>Savills/Carter Jonas corporate brands dominate Newbury premium search</t>
+        </is>
+      </c>
+      <c r="Q349" s="3" t="inlineStr">
+        <is>
+          <t>'36 years independent, founder still answering emails - own that AEO trust story'</t>
+        </is>
+      </c>
+      <c r="R349" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S349" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T349" s="3" t="inlineStr"/>
+    </row>
+    <row r="350">
+      <c r="A350" s="4" t="inlineStr">
+        <is>
+          <t>Cricketts Estate Agent</t>
+        </is>
+      </c>
+      <c r="B350" s="4" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C350" s="4" t="inlineStr">
+        <is>
+          <t>Newbury, West Berkshire</t>
+        </is>
+      </c>
+      <c r="D350" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cricketts.co.uk</t>
+        </is>
+      </c>
+      <c r="E350" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F350" s="4" t="inlineStr"/>
+      <c r="G350" s="4" t="inlineStr"/>
+      <c r="H350" s="4" t="inlineStr"/>
+      <c r="I350" s="4" t="inlineStr"/>
+      <c r="J350" s="4" t="inlineStr">
+        <is>
+          <t>60+ years combined team experience, dedicated property manager per client - genuine service differentiator</t>
+        </is>
+      </c>
+      <c r="K350" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L350" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M350" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N350" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O350" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P350" s="4" t="inlineStr">
+        <is>
+          <t>'Dedicated property manager' positioning invisible in generic Newbury agent searches</t>
+        </is>
+      </c>
+      <c r="Q350" s="4" t="inlineStr">
+        <is>
+          <t>Own that specific personal-service AEO angle vs volume-focused rivals</t>
+        </is>
+      </c>
+      <c r="R350" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S350" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T350" s="4" t="inlineStr"/>
+    </row>
+    <row r="351">
+      <c r="A351" s="4" t="inlineStr">
+        <is>
+          <t>Emmett Bloom</t>
+        </is>
+      </c>
+      <c r="B351" s="4" t="inlineStr">
+        <is>
+          <t>Estate agent (boutique)</t>
+        </is>
+      </c>
+      <c r="C351" s="4" t="inlineStr">
+        <is>
+          <t>West Berkshire</t>
+        </is>
+      </c>
+      <c r="D351" s="4" t="inlineStr">
+        <is>
+          <t>via directory listing</t>
+        </is>
+      </c>
+      <c r="E351" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F351" s="4" t="inlineStr"/>
+      <c r="G351" s="4" t="inlineStr"/>
+      <c r="H351" s="4" t="inlineStr"/>
+      <c r="I351" s="4" t="inlineStr"/>
+      <c r="J351" s="4" t="inlineStr">
+        <is>
+          <t>Boutique independent with bespoke marketing for distinctive homes - premium niche positioning</t>
+        </is>
+      </c>
+      <c r="K351" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L351" s="4" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M351" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N351" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O351" s="4" t="inlineStr">
+        <is>
+          <t>Bespoke-marketing positioning</t>
+        </is>
+      </c>
+      <c r="P351" s="4" t="inlineStr">
+        <is>
+          <t>Boutique/bespoke claim not yet the AI-cited answer for premium West Berkshire property</t>
+        </is>
+      </c>
+      <c r="Q351" s="4" t="inlineStr">
+        <is>
+          <t>Own 'boutique estate agent West Berkshire' - a specific, defensible niche</t>
+        </is>
+      </c>
+      <c r="R351" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S351" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T351" s="4" t="inlineStr">
+        <is>
+          <t>Confirm live website before outreach</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="2" t="inlineStr">
+        <is>
+          <t>Combe Manor</t>
+        </is>
+      </c>
+      <c r="B352" s="2" t="inlineStr">
+        <is>
+          <t>Wedding venue</t>
+        </is>
+      </c>
+      <c r="C352" s="2" t="inlineStr">
+        <is>
+          <t>Hungerford, West Berkshire</t>
+        </is>
+      </c>
+      <c r="D352" s="2" t="inlineStr">
+        <is>
+          <t>https://www.combemanor.com</t>
+        </is>
+      </c>
+      <c r="E352" s="2" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F352" s="2" t="inlineStr">
+        <is>
+          <t>01488 668 931</t>
+        </is>
+      </c>
+      <c r="G352" s="2" t="inlineStr">
+        <is>
+          <t>Sybille Russell (Family owner, since 1960s)</t>
+        </is>
+      </c>
+      <c r="H352" s="2" t="inlineStr"/>
+      <c r="I352" s="2" t="inlineStr"/>
+      <c r="J352" s="2" t="inlineStr">
+        <is>
+          <t>Russell family estate for 60+ years, 30 years running weddings from the barns - deep, genuine multi-generation story</t>
+        </is>
+      </c>
+      <c r="K352" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L352" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M352" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N352" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O352" s="2" t="inlineStr">
+        <is>
+          <t>Multiple directory listings (Guides for Brides, Bridebook, Cvent)</t>
+        </is>
+      </c>
+      <c r="P352" s="2" t="inlineStr">
+        <is>
+          <t>60-year family story is an exceptional AEO asset barely used beyond directory blurbs</t>
+        </is>
+      </c>
+      <c r="Q352" s="2" t="inlineStr">
+        <is>
+          <t>'One family, one estate, 60 years - own that story in every AI answer for Berkshire barn weddings'</t>
+        </is>
+      </c>
+      <c r="R352" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S352" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T352" s="2" t="inlineStr">
+        <is>
+          <t>Strong multi-generational heritage story - high-value AEO opportunity</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="4" t="inlineStr">
+        <is>
+          <t>The Post Barn</t>
+        </is>
+      </c>
+      <c r="B353" s="4" t="inlineStr">
+        <is>
+          <t>Wedding venue</t>
+        </is>
+      </c>
+      <c r="C353" s="4" t="inlineStr">
+        <is>
+          <t>Snelsmore Common, Newbury, Berkshire</t>
+        </is>
+      </c>
+      <c r="D353" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thepostbarn.co.uk</t>
+        </is>
+      </c>
+      <c r="E353" s="4" t="inlineStr">
+        <is>
+          <t>info@thepostbarn.co.uk</t>
+        </is>
+      </c>
+      <c r="F353" s="4" t="inlineStr">
+        <is>
+          <t>01635 881 800</t>
+        </is>
+      </c>
+      <c r="G353" s="4" t="inlineStr"/>
+      <c r="H353" s="4" t="inlineStr"/>
+      <c r="I353" s="4" t="inlineStr"/>
+      <c r="J353" s="4" t="inlineStr">
+        <is>
+          <t>Barn venue set within Snelsmore Common's protected countryside - distinctive natural setting</t>
+        </is>
+      </c>
+      <c r="K353" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L353" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M353" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N353" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O353" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P353" s="4" t="inlineStr">
+        <is>
+          <t>Protected-countryside setting undersold as a differentiator vs generic Berkshire barn venues</t>
+        </is>
+      </c>
+      <c r="Q353" s="4" t="inlineStr">
+        <is>
+          <t>'Weddings on protected common land' - own that unusual, specific AEO positioning</t>
+        </is>
+      </c>
+      <c r="R353" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S353" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T353" s="4" t="inlineStr"/>
+    </row>
+    <row r="354">
+      <c r="A354" s="4" t="inlineStr">
+        <is>
+          <t>Lillibrooke Manor</t>
+        </is>
+      </c>
+      <c r="B354" s="4" t="inlineStr">
+        <is>
+          <t>Wedding venue</t>
+        </is>
+      </c>
+      <c r="C354" s="4" t="inlineStr">
+        <is>
+          <t>Maidenhead, Berkshire</t>
+        </is>
+      </c>
+      <c r="D354" s="4" t="inlineStr">
+        <is>
+          <t>https://lillibrookemanor.co.uk</t>
+        </is>
+      </c>
+      <c r="E354" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F354" s="4" t="inlineStr"/>
+      <c r="G354" s="4" t="inlineStr"/>
+      <c r="H354" s="4" t="inlineStr"/>
+      <c r="I354" s="4" t="inlineStr"/>
+      <c r="J354" s="4" t="inlineStr">
+        <is>
+          <t>Family-run barn wedding venue in Berkshire's Maidenhead commuter belt</t>
+        </is>
+      </c>
+      <c r="K354" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L354" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M354" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N354" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O354" s="4" t="inlineStr">
+        <is>
+          <t>Dedicated estate/venue content pages</t>
+        </is>
+      </c>
+      <c r="P354" s="4" t="inlineStr">
+        <is>
+          <t>Family-run story not yet leveraged as the AI-cited local differentiator</t>
+        </is>
+      </c>
+      <c r="Q354" s="4" t="inlineStr">
+        <is>
+          <t>Turn the family-run story into AEO content vs corporate-feeling rivals</t>
+        </is>
+      </c>
+      <c r="R354" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S354" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T354" s="4" t="inlineStr"/>
+    </row>
+    <row r="355">
+      <c r="A355" s="3" t="inlineStr">
+        <is>
+          <t>The Berkshire Clinic</t>
+        </is>
+      </c>
+      <c r="B355" s="3" t="inlineStr">
+        <is>
+          <t>Private GP</t>
+        </is>
+      </c>
+      <c r="C355" s="3" t="inlineStr">
+        <is>
+          <t>Reading &amp; Wokingham, Berkshire</t>
+        </is>
+      </c>
+      <c r="D355" s="3" t="inlineStr">
+        <is>
+          <t>https://theberkshireclinic.com</t>
+        </is>
+      </c>
+      <c r="E355" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F355" s="3" t="inlineStr">
+        <is>
+          <t>0118 304 5920</t>
+        </is>
+      </c>
+      <c r="G355" s="3" t="inlineStr"/>
+      <c r="H355" s="3" t="inlineStr"/>
+      <c r="I355" s="3" t="inlineStr"/>
+      <c r="J355" s="3" t="inlineStr">
+        <is>
+          <t>Two-town private GP with urgent-consultation phone line - convenience differentiator</t>
+        </is>
+      </c>
+      <c r="K355" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L355" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M355" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N355" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O355" s="3" t="inlineStr">
+        <is>
+          <t>Urgent-line promoted</t>
+        </is>
+      </c>
+      <c r="P355" s="3" t="inlineStr">
+        <is>
+          <t>Two-town coverage claim not matched by per-town search dominance</t>
+        </is>
+      </c>
+      <c r="Q355" s="3" t="inlineStr">
+        <is>
+          <t>Per-town AEO content for both Reading and Wokingham private GP searches</t>
+        </is>
+      </c>
+      <c r="R355" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S355" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T355" s="3" t="inlineStr"/>
+    </row>
+    <row r="356">
+      <c r="A356" s="3" t="inlineStr">
+        <is>
+          <t>Absolute Architecture</t>
+        </is>
+      </c>
+      <c r="B356" s="3" t="inlineStr">
+        <is>
+          <t>Architects &amp; interior design</t>
+        </is>
+      </c>
+      <c r="C356" s="3" t="inlineStr">
+        <is>
+          <t>Newbury, Berkshire (40-mile radius)</t>
+        </is>
+      </c>
+      <c r="D356" s="3" t="inlineStr">
+        <is>
+          <t>https://absolute-architecture.co.uk</t>
+        </is>
+      </c>
+      <c r="E356" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F356" s="3" t="inlineStr">
+        <is>
+          <t>01635 528 188</t>
+        </is>
+      </c>
+      <c r="G356" s="3" t="inlineStr">
+        <is>
+          <t>Kate Cooper &amp; Jennie Lunn (Directors, est. 2008)</t>
+        </is>
+      </c>
+      <c r="H356" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/kate-cooper-a92a1420</t>
+        </is>
+      </c>
+      <c r="I356" s="3" t="inlineStr"/>
+      <c r="J356" s="3" t="inlineStr">
+        <is>
+          <t>Combined architecture + interior design for a 40-mile radius across 4 counties; named studio manager for client onboarding</t>
+        </is>
+      </c>
+      <c r="K356" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L356" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M356" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N356" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O356" s="3" t="inlineStr">
+        <is>
+          <t>Press coverage (Hamptons brochure feature)</t>
+        </is>
+      </c>
+      <c r="P356" s="3" t="inlineStr">
+        <is>
+          <t>Press feature exists but not yet converted into AI-search citation authority</t>
+        </is>
+      </c>
+      <c r="Q356" s="3" t="inlineStr">
+        <is>
+          <t>Turn existing press coverage into the AI-cited authority for Berkshire/Hampshire residential architecture</t>
+        </is>
+      </c>
+      <c r="R356" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S356" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T356" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T348"/>
+  <autoFilter ref="A1:T356"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -30556,7 +31240,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B139"/>
+  <dimension ref="A1:B140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -30576,7 +31260,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>347</v>
+        <v>355</v>
       </c>
     </row>
     <row r="5">
@@ -30593,13 +31277,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Architects</t>
+          <t>Wedding venue</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -30609,17 +31293,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Private dentist</t>
+          <t>Architects</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Independent vet</t>
+          <t>Private dentist</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -30629,7 +31313,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Wedding venue</t>
+          <t>Independent vet</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -30649,17 +31333,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Chartered accountants</t>
+          <t>Private GP</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Private GP</t>
+          <t>Chartered accountants</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -30949,7 +31633,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Funeral directors</t>
+          <t>Architects &amp; interior design</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -30959,7 +31643,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Garden rooms / outbuildings</t>
+          <t>Funeral directors</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -30969,7 +31653,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Personal training gym</t>
+          <t>Garden rooms / outbuildings</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -30979,7 +31663,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Wedding &amp; event caterer</t>
+          <t>Personal training gym</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -30989,7 +31673,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Personal training</t>
+          <t>Wedding &amp; event caterer</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -30999,17 +31683,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Dentist / Orthodontics</t>
+          <t>Personal training</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Specialist dental/implant clinic</t>
+          <t>Dentist / Orthodontics</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -31019,7 +31703,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Boutique corporate law firm</t>
+          <t>Specialist dental/implant clinic</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -31029,7 +31713,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Cosmetic/aesthetics clinic</t>
+          <t>Boutique corporate law firm</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -31039,7 +31723,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Skin &amp; laser clinic</t>
+          <t>Cosmetic/aesthetics clinic</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -31049,7 +31733,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Mortgage broker / financial adviser</t>
+          <t>Skin &amp; laser clinic</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -31059,7 +31743,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Architects (RIBA chartered)</t>
+          <t>Mortgage broker / financial adviser</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -31069,7 +31753,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Recruitment agency (tech/startups)</t>
+          <t>Architects (RIBA chartered)</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -31079,7 +31763,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Recruitment agency (IT/data)</t>
+          <t>Recruitment agency (tech/startups)</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -31089,7 +31773,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Independent vet (24/7 emergency)</t>
+          <t>Recruitment agency (IT/data)</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -31099,7 +31783,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Interior design studio</t>
+          <t>Independent vet (24/7 emergency)</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -31109,7 +31793,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Letting &amp; estate agent</t>
+          <t>Interior design studio</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -31119,7 +31803,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Cosmetic clinic (injectables)</t>
+          <t>Letting &amp; estate agent</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -31129,7 +31813,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Cosmetic/anti-ageing clinic</t>
+          <t>Cosmetic clinic (injectables)</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -31139,7 +31823,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Yoga &amp; reformer pilates studio</t>
+          <t>Cosmetic/anti-ageing clinic</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -31149,7 +31833,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Reformer pilates studio</t>
+          <t>Yoga &amp; reformer pilates studio</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -31159,7 +31843,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Wealth management</t>
+          <t>Reformer pilates studio</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -31169,7 +31853,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Private tuition &amp; education consultancy</t>
+          <t>Wealth management</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -31179,7 +31863,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Osteopath</t>
+          <t>Private tuition &amp; education consultancy</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -31189,7 +31873,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Design &amp; build / home renovation</t>
+          <t>Osteopath</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -31199,7 +31883,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Builders / building contractor</t>
+          <t>Design &amp; build / home renovation</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -31209,7 +31893,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Home care / live-in care</t>
+          <t>Builders / building contractor</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -31219,7 +31903,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Private day nurseries</t>
+          <t>Home care / live-in care</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -31229,7 +31913,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Personal training &amp; wellness studio</t>
+          <t>Private day nurseries</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -31239,7 +31923,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Mortgage &amp; insurance broker</t>
+          <t>Personal training &amp; wellness studio</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -31249,7 +31933,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Business consultancy</t>
+          <t>Mortgage &amp; insurance broker</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -31259,7 +31943,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Interior designer (period homes)</t>
+          <t>Business consultancy</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -31269,7 +31953,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Landscape design &amp; build</t>
+          <t>Interior designer (period homes)</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -31279,7 +31963,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Interior designer</t>
+          <t>Landscape design &amp; build</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -31289,7 +31973,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Garden design &amp; landscaping</t>
+          <t>Interior designer</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -31299,7 +31983,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Legal recruitment</t>
+          <t>Garden design &amp; landscaping</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -31309,7 +31993,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Independent gym &amp; health club</t>
+          <t>Legal recruitment</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -31319,7 +32003,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Independent gym</t>
+          <t>Independent gym &amp; health club</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -31329,7 +32013,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Physiotherapy (sports)</t>
+          <t>Independent gym</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -31339,7 +32023,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Letting agent / property management</t>
+          <t>Physiotherapy (sports)</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -31349,7 +32033,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Skin clinic</t>
+          <t>Letting agent / property management</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -31359,7 +32043,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Tutoring company</t>
+          <t>Skin clinic</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -31369,7 +32053,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Tutorial college &amp; exam centre</t>
+          <t>Tutoring company</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -31379,7 +32063,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Employment law (disability discrimination)</t>
+          <t>Tutorial college &amp; exam centre</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -31389,7 +32073,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating</t>
+          <t>Employment law (disability discrimination)</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -31399,7 +32083,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Plumbing &amp; heating</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -31409,7 +32093,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Sports physio &amp; massage</t>
+          <t>Plumbing</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -31419,7 +32103,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Chartered surveyors (party wall/building)</t>
+          <t>Sports physio &amp; massage</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -31429,7 +32113,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Chartered surveyors</t>
+          <t>Chartered surveyors (party wall/building)</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -31439,7 +32123,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Chartered building surveyors</t>
+          <t>Chartered surveyors</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -31449,7 +32133,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Osteopathy clinics</t>
+          <t>Chartered building surveyors</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -31459,7 +32143,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Builders / renovations</t>
+          <t>Osteopathy clinics</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -31469,7 +32153,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Private nursery schools</t>
+          <t>Builders / renovations</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -31479,7 +32163,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Private day nursery</t>
+          <t>Private nursery schools</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -31489,7 +32173,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Private GP (membership model)</t>
+          <t>Private day nursery</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -31499,7 +32183,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Sash window restoration</t>
+          <t>Private GP (membership model)</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -31509,7 +32193,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Personal training (1:1)</t>
+          <t>Sash window restoration</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -31519,7 +32203,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Personal training &amp; nutrition coaching</t>
+          <t>Personal training (1:1)</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -31529,7 +32213,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Private nursery/pre-prep school</t>
+          <t>Personal training &amp; nutrition coaching</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -31539,7 +32223,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Independent nursery (Montessori)</t>
+          <t>Private nursery/pre-prep school</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -31549,7 +32233,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Live-in care agency</t>
+          <t>Independent nursery (Montessori)</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -31559,7 +32243,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Law firm (conveyancing/family)</t>
+          <t>Live-in care agency</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -31569,7 +32253,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Architect &amp; interior designer</t>
+          <t>Law firm (conveyancing/family)</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -31579,7 +32263,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Architects / project management</t>
+          <t>Architect &amp; interior designer</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -31589,7 +32273,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>IFA / wealth management</t>
+          <t>Architects / project management</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -31599,7 +32283,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Physiotherapy &amp; clinical Pilates</t>
+          <t>IFA / wealth management</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -31609,7 +32293,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Aesthetics &amp; skin clinic</t>
+          <t>Physiotherapy &amp; clinical Pilates</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -31619,7 +32303,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Wealth management / IFA</t>
+          <t>Aesthetics &amp; skin clinic</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -31629,7 +32313,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>IFA / financial planning</t>
+          <t>Wealth management / IFA</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -31639,7 +32323,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Wealth management &amp; employee benefits</t>
+          <t>IFA / financial planning</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -31649,7 +32333,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Dermatology clinic</t>
+          <t>Wealth management &amp; employee benefits</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -31659,7 +32343,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Pilates studio (multi-site)</t>
+          <t>Dermatology clinic</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -31669,7 +32353,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Private nursery (Montessori, multi-site)</t>
+          <t>Pilates studio (multi-site)</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -31679,7 +32363,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Law firm (wills &amp; probate)</t>
+          <t>Private nursery (Montessori, multi-site)</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -31689,7 +32373,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Business/technical consultancy</t>
+          <t>Law firm (wills &amp; probate)</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -31699,7 +32383,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Architects &amp; interior design</t>
+          <t>Business/technical consultancy</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -31923,6 +32607,16 @@
         </is>
       </c>
       <c r="B139" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Estate agent (boutique)</t>
+        </is>
+      </c>
+      <c r="B140" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 32: +8 prospects (363 total) - Witney, Abingdon, Oxford
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$356</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$364</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T356"/>
+  <dimension ref="A1:T364"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -31228,8 +31228,712 @@
       </c>
       <c r="T356" s="3" t="inlineStr"/>
     </row>
+    <row r="357">
+      <c r="A357" s="3" t="inlineStr">
+        <is>
+          <t>Martyn Cox &amp; Company</t>
+        </is>
+      </c>
+      <c r="B357" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C357" s="3" t="inlineStr">
+        <is>
+          <t>Corn Street, Witney, Oxfordshire</t>
+        </is>
+      </c>
+      <c r="D357" s="3" t="inlineStr">
+        <is>
+          <t>https://www.martyncox.com</t>
+        </is>
+      </c>
+      <c r="E357" s="3" t="inlineStr">
+        <is>
+          <t>property@martyncox.com</t>
+        </is>
+      </c>
+      <c r="F357" s="3" t="inlineStr">
+        <is>
+          <t>01993 779 020</t>
+        </is>
+      </c>
+      <c r="G357" s="3" t="inlineStr">
+        <is>
+          <t>Martyn Cox (Founder, est. 1988)</t>
+        </is>
+      </c>
+      <c r="H357" s="3" t="inlineStr"/>
+      <c r="I357" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/martyncoxco</t>
+        </is>
+      </c>
+      <c r="J357" s="3" t="inlineStr">
+        <is>
+          <t>36-year independent in West Oxfordshire's market towns; town &amp; country property specialism</t>
+        </is>
+      </c>
+      <c r="K357" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L357" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M357" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N357" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O357" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence</t>
+        </is>
+      </c>
+      <c r="P357" s="3" t="inlineStr">
+        <is>
+          <t>Corporate brands (scottfraser, Hamptons) compete for the same Witney searches</t>
+        </is>
+      </c>
+      <c r="Q357" s="3" t="inlineStr">
+        <is>
+          <t>'36 years of Witney town &amp; country property - own the AI answer, not just Rightmove'</t>
+        </is>
+      </c>
+      <c r="R357" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S357" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T357" s="3" t="inlineStr"/>
+    </row>
+    <row r="358">
+      <c r="A358" s="3" t="inlineStr">
+        <is>
+          <t>Thomas Merrifield</t>
+        </is>
+      </c>
+      <c r="B358" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C358" s="3" t="inlineStr">
+        <is>
+          <t>Witney/Abingdon/Wantage, Oxfordshire (8 offices)</t>
+        </is>
+      </c>
+      <c r="D358" s="3" t="inlineStr">
+        <is>
+          <t>via directory listing</t>
+        </is>
+      </c>
+      <c r="E358" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F358" s="3" t="inlineStr"/>
+      <c r="G358" s="3" t="inlineStr">
+        <is>
+          <t>Philip Miller &amp; Stuart Wallsworth (Directors, 30+ years each)</t>
+        </is>
+      </c>
+      <c r="H358" s="3" t="inlineStr"/>
+      <c r="I358" s="3" t="inlineStr"/>
+      <c r="J358" s="3" t="inlineStr">
+        <is>
+          <t>8-office independent group across West Oxfordshire market towns; high-energy proactive positioning</t>
+        </is>
+      </c>
+      <c r="K358" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L358" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M358" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N358" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O358" s="3" t="inlineStr">
+        <is>
+          <t>Multi-office scale</t>
+        </is>
+      </c>
+      <c r="P358" s="3" t="inlineStr">
+        <is>
+          <t>8-office claim not matched by per-town search dominance</t>
+        </is>
+      </c>
+      <c r="Q358" s="3" t="inlineStr">
+        <is>
+          <t>Per-town AEO content to actually own all 8 claimed markets</t>
+        </is>
+      </c>
+      <c r="R358" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S358" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T358" s="3" t="inlineStr">
+        <is>
+          <t>Confirm live website before outreach</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="4" t="inlineStr">
+        <is>
+          <t>Simpsons Property</t>
+        </is>
+      </c>
+      <c r="B359" s="4" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C359" s="4" t="inlineStr">
+        <is>
+          <t>Witney (+ Abingdon), Oxfordshire</t>
+        </is>
+      </c>
+      <c r="D359" s="4" t="inlineStr">
+        <is>
+          <t>https://www.simpsonsproperty.com</t>
+        </is>
+      </c>
+      <c r="E359" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F359" s="4" t="inlineStr"/>
+      <c r="G359" s="4" t="inlineStr">
+        <is>
+          <t>Tom Mizen (Witney branch manager)</t>
+        </is>
+      </c>
+      <c r="H359" s="4" t="inlineStr"/>
+      <c r="I359" s="4" t="inlineStr"/>
+      <c r="J359" s="4" t="inlineStr">
+        <is>
+          <t>60 years combined team experience across Witney/Abingdon offices</t>
+        </is>
+      </c>
+      <c r="K359" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L359" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M359" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N359" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O359" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P359" s="4" t="inlineStr">
+        <is>
+          <t>60 years' combined experience untranslated into modern AI-search visibility</t>
+        </is>
+      </c>
+      <c r="Q359" s="4" t="inlineStr">
+        <is>
+          <t>'60 years combined experience - the AI answer should reflect it, not just staff bios'</t>
+        </is>
+      </c>
+      <c r="R359" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S359" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T359" s="4" t="inlineStr"/>
+    </row>
+    <row r="360">
+      <c r="A360" s="4" t="inlineStr">
+        <is>
+          <t>Rejoice Dental Care</t>
+        </is>
+      </c>
+      <c r="B360" s="4" t="inlineStr">
+        <is>
+          <t>Private dentist / implants</t>
+        </is>
+      </c>
+      <c r="C360" s="4" t="inlineStr">
+        <is>
+          <t>Ock Street, Abingdon, Oxfordshire</t>
+        </is>
+      </c>
+      <c r="D360" s="4" t="inlineStr">
+        <is>
+          <t>https://rejoicedental.co.uk</t>
+        </is>
+      </c>
+      <c r="E360" s="4" t="inlineStr">
+        <is>
+          <t>info@rejoicedental.co.uk</t>
+        </is>
+      </c>
+      <c r="F360" s="4" t="inlineStr">
+        <is>
+          <t>01235 550 855</t>
+        </is>
+      </c>
+      <c r="G360" s="4" t="inlineStr">
+        <is>
+          <t>Grace Addanki (Principal Dentist)</t>
+        </is>
+      </c>
+      <c r="H360" s="4" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/grace-addanki-94325b203</t>
+        </is>
+      </c>
+      <c r="I360" s="4" t="inlineStr">
+        <is>
+          <t>facebook.com/rejoicedc.sm</t>
+        </is>
+      </c>
+      <c r="J360" s="4" t="inlineStr">
+        <is>
+          <t>Named principal dentist, welcomes patients across South Oxfordshire including Witney; implant + whitening services</t>
+        </is>
+      </c>
+      <c r="K360" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L360" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M360" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N360" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O360" s="4" t="inlineStr">
+        <is>
+          <t>Facebook presence; LinkedIn</t>
+        </is>
+      </c>
+      <c r="P360" s="4" t="inlineStr">
+        <is>
+          <t>Wide catchment claim (South Oxon + Witney) not matched by per-area search dominance</t>
+        </is>
+      </c>
+      <c r="Q360" s="4" t="inlineStr">
+        <is>
+          <t>Per-area AEO content to actually own the wider claimed catchment</t>
+        </is>
+      </c>
+      <c r="R360" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S360" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T360" s="4" t="inlineStr"/>
+    </row>
+    <row r="361">
+      <c r="A361" s="4" t="inlineStr">
+        <is>
+          <t>Buttercross Dental Practice</t>
+        </is>
+      </c>
+      <c r="B361" s="4" t="inlineStr">
+        <is>
+          <t>Private dentist / implants</t>
+        </is>
+      </c>
+      <c r="C361" s="4" t="inlineStr">
+        <is>
+          <t>Corn Street, Witney, Oxfordshire</t>
+        </is>
+      </c>
+      <c r="D361" s="4" t="inlineStr">
+        <is>
+          <t>https://www.buttercrossdp.co.uk</t>
+        </is>
+      </c>
+      <c r="E361" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F361" s="4" t="inlineStr">
+        <is>
+          <t>01993 402 402</t>
+        </is>
+      </c>
+      <c r="G361" s="4" t="inlineStr"/>
+      <c r="H361" s="4" t="inlineStr"/>
+      <c r="I361" s="4" t="inlineStr"/>
+      <c r="J361" s="4" t="inlineStr">
+        <is>
+          <t>Advanced dentistry with dedicated implants treatment page in Witney town centre</t>
+        </is>
+      </c>
+      <c r="K361" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L361" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M361" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N361" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O361" s="4" t="inlineStr">
+        <is>
+          <t>Dedicated implants page = active SEO</t>
+        </is>
+      </c>
+      <c r="P361" s="4" t="inlineStr">
+        <is>
+          <t>Implants page exists but AI-answer citations for 'dental implants Witney' still open</t>
+        </is>
+      </c>
+      <c r="Q361" s="4" t="inlineStr">
+        <is>
+          <t>Upgrade existing implants SEO page into an AEO-optimised asset</t>
+        </is>
+      </c>
+      <c r="R361" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S361" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T361" s="4" t="inlineStr"/>
+    </row>
+    <row r="362">
+      <c r="A362" s="3" t="inlineStr">
+        <is>
+          <t>Anderson Orr Architects</t>
+        </is>
+      </c>
+      <c r="B362" s="3" t="inlineStr">
+        <is>
+          <t>Architects</t>
+        </is>
+      </c>
+      <c r="C362" s="3" t="inlineStr">
+        <is>
+          <t>Oxfordshire (+ London/Cotswolds)</t>
+        </is>
+      </c>
+      <c r="D362" s="3" t="inlineStr">
+        <is>
+          <t>https://www.andersonorr.com</t>
+        </is>
+      </c>
+      <c r="E362" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F362" s="3" t="inlineStr"/>
+      <c r="G362" s="3" t="inlineStr">
+        <is>
+          <t>Est. 2000, 4th-generation design-led practice</t>
+        </is>
+      </c>
+      <c r="H362" s="3" t="inlineStr"/>
+      <c r="I362" s="3" t="inlineStr"/>
+      <c r="J362" s="3" t="inlineStr">
+        <is>
+          <t>High-end private residential + developer + commercial work spanning London to the Cotswolds - very high project values</t>
+        </is>
+      </c>
+      <c r="K362" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L362" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M362" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N362" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O362" s="3" t="inlineStr">
+        <is>
+          <t>Multi-region portfolio</t>
+        </is>
+      </c>
+      <c r="P362" s="3" t="inlineStr">
+        <is>
+          <t>Broad geographic reach not matched by per-region AEO dominance</t>
+        </is>
+      </c>
+      <c r="Q362" s="3" t="inlineStr">
+        <is>
+          <t>Per-region AEO content leveraging the 4th-generation design pedigree</t>
+        </is>
+      </c>
+      <c r="R362" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S362" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T362" s="3" t="inlineStr"/>
+    </row>
+    <row r="363">
+      <c r="A363" s="4" t="inlineStr">
+        <is>
+          <t>SWA Architects</t>
+        </is>
+      </c>
+      <c r="B363" s="4" t="inlineStr">
+        <is>
+          <t>Architects</t>
+        </is>
+      </c>
+      <c r="C363" s="4" t="inlineStr">
+        <is>
+          <t>Eynsham, near Oxford, Oxfordshire</t>
+        </is>
+      </c>
+      <c r="D363" s="4" t="inlineStr">
+        <is>
+          <t>http://www.swa-architects.co.uk</t>
+        </is>
+      </c>
+      <c r="E363" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F363" s="4" t="inlineStr"/>
+      <c r="G363" s="4" t="inlineStr">
+        <is>
+          <t>Est. 1985 (Stanhope Wilkinson Associates)</t>
+        </is>
+      </c>
+      <c r="H363" s="4" t="inlineStr"/>
+      <c r="I363" s="4" t="inlineStr"/>
+      <c r="J363" s="4" t="inlineStr">
+        <is>
+          <t>40-year established practice near Oxford; efficient, value-for-money positioning</t>
+        </is>
+      </c>
+      <c r="K363" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L363" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M363" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N363" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O363" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P363" s="4" t="inlineStr">
+        <is>
+          <t>40 years of trust untranslated into modern AI-search visibility</t>
+        </is>
+      </c>
+      <c r="Q363" s="4" t="inlineStr">
+        <is>
+          <t>'40 years near Oxford - the AI answer should reflect that heritage'</t>
+        </is>
+      </c>
+      <c r="R363" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S363" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T363" s="4" t="inlineStr"/>
+    </row>
+    <row r="364">
+      <c r="A364" s="3" t="inlineStr">
+        <is>
+          <t>Ridgefield Consulting</t>
+        </is>
+      </c>
+      <c r="B364" s="3" t="inlineStr">
+        <is>
+          <t>Chartered accountants</t>
+        </is>
+      </c>
+      <c r="C364" s="3" t="inlineStr">
+        <is>
+          <t>Oxford (Church Way)</t>
+        </is>
+      </c>
+      <c r="D364" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ridgefieldconsulting.co.uk</t>
+        </is>
+      </c>
+      <c r="E364" s="3" t="inlineStr">
+        <is>
+          <t>simon@ridgefieldconsulting.co.uk</t>
+        </is>
+      </c>
+      <c r="F364" s="3" t="inlineStr">
+        <is>
+          <t>01491 578 207</t>
+        </is>
+      </c>
+      <c r="G364" s="3" t="inlineStr">
+        <is>
+          <t>Simon Thomas (Founder &amp; MD) &amp; Brian Thomas (Director, father-son)</t>
+        </is>
+      </c>
+      <c r="H364" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/simonthomasoxford</t>
+        </is>
+      </c>
+      <c r="I364" s="3" t="inlineStr"/>
+      <c r="J364" s="3" t="inlineStr">
+        <is>
+          <t>Father-son independent firm since 2010; press-featured (Independent Oxford interview) - marketing-aware</t>
+        </is>
+      </c>
+      <c r="K364" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L364" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M364" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N364" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O364" s="3" t="inlineStr">
+        <is>
+          <t>Press interview coverage; detailed team page</t>
+        </is>
+      </c>
+      <c r="P364" s="3" t="inlineStr">
+        <is>
+          <t>Press coverage exists but not yet converted into AI-search citation authority</t>
+        </is>
+      </c>
+      <c r="Q364" s="3" t="inlineStr">
+        <is>
+          <t>Turn the Independent Oxford press feature into AI-cited local authority content</t>
+        </is>
+      </c>
+      <c r="R364" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S364" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T364" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T356"/>
+  <autoFilter ref="A1:T364"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -31260,7 +31964,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>355</v>
+        <v>363</v>
       </c>
     </row>
     <row r="5">
@@ -31277,23 +31981,23 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Wedding venue</t>
+          <t>Architects</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Architects</t>
+          <t>Wedding venue</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -31327,13 +32031,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Private GP</t>
+          <t>Chartered accountants</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -31343,11 +32047,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Chartered accountants</t>
+          <t>Private GP</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14">

</xml_diff>

<commit_message>
Batch 33: +8 prospects (371 total) - Banbury, Bicester, Oxfordshire vets
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$364</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$372</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T364"/>
+  <dimension ref="A1:T372"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -31932,8 +31932,696 @@
       </c>
       <c r="T364" s="3" t="inlineStr"/>
     </row>
+    <row r="365">
+      <c r="A365" s="3" t="inlineStr">
+        <is>
+          <t>Anker and Partners</t>
+        </is>
+      </c>
+      <c r="B365" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent &amp; chartered surveyors</t>
+        </is>
+      </c>
+      <c r="C365" s="3" t="inlineStr">
+        <is>
+          <t>High Street, Banbury, Oxfordshire</t>
+        </is>
+      </c>
+      <c r="D365" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ankerandpartners.co.uk</t>
+        </is>
+      </c>
+      <c r="E365" s="3" t="inlineStr">
+        <is>
+          <t>post@ankerandpartners.co.uk</t>
+        </is>
+      </c>
+      <c r="F365" s="3" t="inlineStr">
+        <is>
+          <t>01295 271 414</t>
+        </is>
+      </c>
+      <c r="G365" s="3" t="inlineStr">
+        <is>
+          <t>Est. 1984</t>
+        </is>
+      </c>
+      <c r="H365" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/anker-and-partners</t>
+        </is>
+      </c>
+      <c r="I365" s="3" t="inlineStr"/>
+      <c r="J365" s="3" t="inlineStr">
+        <is>
+          <t>40-year independent covering sales/lettings/surveying in North Oxfordshire; surveying arm adds a second revenue line</t>
+        </is>
+      </c>
+      <c r="K365" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L365" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M365" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N365" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O365" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn presence</t>
+        </is>
+      </c>
+      <c r="P365" s="3" t="inlineStr">
+        <is>
+          <t>Fine &amp; Country and Chancellors corporate brands compete for Banbury premium search</t>
+        </is>
+      </c>
+      <c r="Q365" s="3" t="inlineStr">
+        <is>
+          <t>'40 years in Banbury property - own the AI answer, not just the high street presence'</t>
+        </is>
+      </c>
+      <c r="R365" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S365" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T365" s="3" t="inlineStr"/>
+    </row>
+    <row r="366">
+      <c r="A366" s="3" t="inlineStr">
+        <is>
+          <t>Mark David Estate Agents</t>
+        </is>
+      </c>
+      <c r="B366" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C366" s="3" t="inlineStr">
+        <is>
+          <t>North Oxfordshire &amp; Cotswolds</t>
+        </is>
+      </c>
+      <c r="D366" s="3" t="inlineStr">
+        <is>
+          <t>via directory listing</t>
+        </is>
+      </c>
+      <c r="E366" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F366" s="3" t="inlineStr"/>
+      <c r="G366" s="3" t="inlineStr"/>
+      <c r="H366" s="3" t="inlineStr"/>
+      <c r="I366" s="3" t="inlineStr"/>
+      <c r="J366" s="3" t="inlineStr">
+        <is>
+          <t>Leading independent for village/country/equestrian homes in North Oxfordshire and the Cotswolds - high-value niche stock</t>
+        </is>
+      </c>
+      <c r="K366" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L366" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M366" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N366" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O366" s="3" t="inlineStr">
+        <is>
+          <t>Equestrian/country-home niche positioning</t>
+        </is>
+      </c>
+      <c r="P366" s="3" t="inlineStr">
+        <is>
+          <t>Niche property type (equestrian/country) is a strong AEO angle barely contested</t>
+        </is>
+      </c>
+      <c r="Q366" s="3" t="inlineStr">
+        <is>
+          <t>Own 'equestrian property agent Oxfordshire' - a specific, high-value niche</t>
+        </is>
+      </c>
+      <c r="R366" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S366" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T366" s="3" t="inlineStr">
+        <is>
+          <t>Confirm live website before outreach</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="3" t="inlineStr">
+        <is>
+          <t>41 South Bar Dental Practice</t>
+        </is>
+      </c>
+      <c r="B367" s="3" t="inlineStr">
+        <is>
+          <t>Private dentist / implants</t>
+        </is>
+      </c>
+      <c r="C367" s="3" t="inlineStr">
+        <is>
+          <t>South Bar, Banbury, Oxfordshire</t>
+        </is>
+      </c>
+      <c r="D367" s="3" t="inlineStr">
+        <is>
+          <t>https://www.41southbar.com</t>
+        </is>
+      </c>
+      <c r="E367" s="3" t="inlineStr">
+        <is>
+          <t>info@41southbar.com</t>
+        </is>
+      </c>
+      <c r="F367" s="3" t="inlineStr">
+        <is>
+          <t>01295 262 008</t>
+        </is>
+      </c>
+      <c r="G367" s="3" t="inlineStr">
+        <is>
+          <t>Dr Tom Donnelly (Owner since 1989)</t>
+        </is>
+      </c>
+      <c r="H367" s="3" t="inlineStr"/>
+      <c r="I367" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/41southbar</t>
+        </is>
+      </c>
+      <c r="J367" s="3" t="inlineStr">
+        <is>
+          <t>Award-winning practice, same owner for 35+ years; deep local reputation for implants/cosmetic dentistry</t>
+        </is>
+      </c>
+      <c r="K367" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L367" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M367" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N367" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O367" s="3" t="inlineStr">
+        <is>
+          <t>Award-winning branding; Facebook presence</t>
+        </is>
+      </c>
+      <c r="P367" s="3" t="inlineStr">
+        <is>
+          <t>35 years of ownership continuity is a strong AEO trust signal currently underused</t>
+        </is>
+      </c>
+      <c r="Q367" s="3" t="inlineStr">
+        <is>
+          <t>'Same owner, 35 years, award-winning - own that continuity story in AI answers'</t>
+        </is>
+      </c>
+      <c r="R367" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S367" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T367" s="3" t="inlineStr"/>
+    </row>
+    <row r="368">
+      <c r="A368" s="4" t="inlineStr">
+        <is>
+          <t>Bicester Dental Care &amp; Implant Centre</t>
+        </is>
+      </c>
+      <c r="B368" s="4" t="inlineStr">
+        <is>
+          <t>Private dentist / implants</t>
+        </is>
+      </c>
+      <c r="C368" s="4" t="inlineStr">
+        <is>
+          <t>Sheep Street, Bicester, Oxfordshire</t>
+        </is>
+      </c>
+      <c r="D368" s="4" t="inlineStr">
+        <is>
+          <t>via directory listing</t>
+        </is>
+      </c>
+      <c r="E368" s="4" t="inlineStr">
+        <is>
+          <t>bicesterdental@gmail.com</t>
+        </is>
+      </c>
+      <c r="F368" s="4" t="inlineStr">
+        <is>
+          <t>01869 252 788</t>
+        </is>
+      </c>
+      <c r="G368" s="4" t="inlineStr"/>
+      <c r="H368" s="4" t="inlineStr"/>
+      <c r="I368" s="4" t="inlineStr"/>
+      <c r="J368" s="4" t="inlineStr">
+        <is>
+          <t>Free implant consultation offer in a growing Oxfordshire commuter town</t>
+        </is>
+      </c>
+      <c r="K368" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L368" s="4" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="M368" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N368" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O368" s="4" t="inlineStr">
+        <is>
+          <t>Gmail contact address - low marketing infrastructure</t>
+        </is>
+      </c>
+      <c r="P368" s="4" t="inlineStr">
+        <is>
+          <t>Gmail address signals minimal digital marketing investment despite Bicester's fast-growing population</t>
+        </is>
+      </c>
+      <c r="Q368" s="4" t="inlineStr">
+        <is>
+          <t>'Bicester is growing fast - a Gmail address won't win the new-resident dental searches'</t>
+        </is>
+      </c>
+      <c r="R368" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S368" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T368" s="4" t="inlineStr">
+        <is>
+          <t>Gmail tell - same infrastructure-gap wedge pattern</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="4" t="inlineStr">
+        <is>
+          <t>Hilltop Vets</t>
+        </is>
+      </c>
+      <c r="B369" s="4" t="inlineStr">
+        <is>
+          <t>Independent vet</t>
+        </is>
+      </c>
+      <c r="C369" s="4" t="inlineStr">
+        <is>
+          <t>Hinksey Heights, Oxford</t>
+        </is>
+      </c>
+      <c r="D369" s="4" t="inlineStr">
+        <is>
+          <t>https://hilltopvets.co.uk</t>
+        </is>
+      </c>
+      <c r="E369" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F369" s="4" t="inlineStr"/>
+      <c r="G369" s="4" t="inlineStr"/>
+      <c r="H369" s="4" t="inlineStr"/>
+      <c r="I369" s="4" t="inlineStr"/>
+      <c r="J369" s="4" t="inlineStr">
+        <is>
+          <t>Proudly independent, distinctive 'The Barn' setting on Oxford's southern bypass</t>
+        </is>
+      </c>
+      <c r="K369" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L369" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M369" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N369" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O369" s="4" t="inlineStr">
+        <is>
+          <t>Distinctive branding ('proudly independent')</t>
+        </is>
+      </c>
+      <c r="P369" s="4" t="inlineStr">
+        <is>
+          <t>'Proudly independent' positioning not yet the AI-cited answer for Oxford vet search</t>
+        </is>
+      </c>
+      <c r="Q369" s="4" t="inlineStr">
+        <is>
+          <t>Own that exact independence positioning as the AEO target</t>
+        </is>
+      </c>
+      <c r="R369" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S369" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T369" s="4" t="inlineStr"/>
+    </row>
+    <row r="370">
+      <c r="A370" s="4" t="inlineStr">
+        <is>
+          <t>Boundary Vets</t>
+        </is>
+      </c>
+      <c r="B370" s="4" t="inlineStr">
+        <is>
+          <t>Independent vet</t>
+        </is>
+      </c>
+      <c r="C370" s="4" t="inlineStr">
+        <is>
+          <t>Oxford Road, Abingdon, Oxfordshire</t>
+        </is>
+      </c>
+      <c r="D370" s="4" t="inlineStr">
+        <is>
+          <t>via directory listing</t>
+        </is>
+      </c>
+      <c r="E370" s="4" t="inlineStr">
+        <is>
+          <t>info@boundaryvets.co.uk</t>
+        </is>
+      </c>
+      <c r="F370" s="4" t="inlineStr">
+        <is>
+          <t>01235 538 721</t>
+        </is>
+      </c>
+      <c r="G370" s="4" t="inlineStr"/>
+      <c r="H370" s="4" t="inlineStr"/>
+      <c r="I370" s="4" t="inlineStr"/>
+      <c r="J370" s="4" t="inlineStr">
+        <is>
+          <t>Independent Abingdon practice serving a fast-growing Oxfordshire commuter town</t>
+        </is>
+      </c>
+      <c r="K370" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L370" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M370" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N370" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O370" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P370" s="4" t="inlineStr">
+        <is>
+          <t>Corporate vet chains outspend on Abingdon-area vet search</t>
+        </is>
+      </c>
+      <c r="Q370" s="4" t="inlineStr">
+        <is>
+          <t>'Independent in a growing town - own the AI answer before the chains do'</t>
+        </is>
+      </c>
+      <c r="R370" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S370" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T370" s="4" t="inlineStr"/>
+    </row>
+    <row r="371">
+      <c r="A371" s="4" t="inlineStr">
+        <is>
+          <t>Larkmead Veterinary Group</t>
+        </is>
+      </c>
+      <c r="B371" s="4" t="inlineStr">
+        <is>
+          <t>Independent vet (mixed practice)</t>
+        </is>
+      </c>
+      <c r="C371" s="4" t="inlineStr">
+        <is>
+          <t>Didcot, Oxfordshire</t>
+        </is>
+      </c>
+      <c r="D371" s="4" t="inlineStr">
+        <is>
+          <t>via directory listing</t>
+        </is>
+      </c>
+      <c r="E371" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F371" s="4" t="inlineStr"/>
+      <c r="G371" s="4" t="inlineStr"/>
+      <c r="H371" s="4" t="inlineStr"/>
+      <c r="I371" s="4" t="inlineStr"/>
+      <c r="J371" s="4" t="inlineStr">
+        <is>
+          <t>Independent 24/7 emergency practice covering pets, farm animals and equines - unusually broad mixed-practice model</t>
+        </is>
+      </c>
+      <c r="K371" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L371" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M371" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N371" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O371" s="4" t="inlineStr">
+        <is>
+          <t>24/7 emergency service</t>
+        </is>
+      </c>
+      <c r="P371" s="4" t="inlineStr">
+        <is>
+          <t>Mixed-practice (farm + equine + pets) breadth undersold as an AEO differentiator</t>
+        </is>
+      </c>
+      <c r="Q371" s="4" t="inlineStr">
+        <is>
+          <t>Own 'mixed animal vet Didcot' - a broader, less-contested niche than small-animal-only rivals</t>
+        </is>
+      </c>
+      <c r="R371" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S371" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T371" s="4" t="inlineStr">
+        <is>
+          <t>Confirm live website before outreach</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" s="3" t="inlineStr">
+        <is>
+          <t>The Great Barn</t>
+        </is>
+      </c>
+      <c r="B372" s="3" t="inlineStr">
+        <is>
+          <t>Wedding venue</t>
+        </is>
+      </c>
+      <c r="C372" s="3" t="inlineStr">
+        <is>
+          <t>Aynho, Oxfordshire/Northamptonshire border</t>
+        </is>
+      </c>
+      <c r="D372" s="3" t="inlineStr">
+        <is>
+          <t>https://thegreatbarn.net</t>
+        </is>
+      </c>
+      <c r="E372" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F372" s="3" t="inlineStr"/>
+      <c r="G372" s="3" t="inlineStr">
+        <is>
+          <t>Stephenson family (converted the barns in 1986)</t>
+        </is>
+      </c>
+      <c r="H372" s="3" t="inlineStr"/>
+      <c r="I372" s="3" t="inlineStr"/>
+      <c r="J372" s="3" t="inlineStr">
+        <is>
+          <t>18th-century barn converted for weddings by the founding family in 1986; recently professionalised operations via The Venue Group partnership</t>
+        </is>
+      </c>
+      <c r="K372" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L372" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M372" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N372" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O372" s="3" t="inlineStr">
+        <is>
+          <t>Multiple wedding-directory listings; professional venue-management partnership</t>
+        </is>
+      </c>
+      <c r="P372" s="3" t="inlineStr">
+        <is>
+          <t>New operational partnership is an opportunity to refresh the AEO strategy alongside it</t>
+        </is>
+      </c>
+      <c r="Q372" s="3" t="inlineStr">
+        <is>
+          <t>'Since the family converted it in 1986' - own that heritage story as the AI-cited differentiator</t>
+        </is>
+      </c>
+      <c r="R372" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S372" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T372" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T364"/>
+  <autoFilter ref="A1:T372"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -31944,7 +32632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B140"/>
+  <dimension ref="A1:B141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -31964,7 +32652,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>363</v>
+        <v>371</v>
       </c>
     </row>
     <row r="5">
@@ -31981,7 +32669,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="7">
@@ -32001,37 +32689,37 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Private dentist</t>
+          <t>Independent vet</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Independent vet</t>
+          <t>Private dentist / implants</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Private dentist / implants</t>
+          <t>Private dentist</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12">
@@ -32377,7 +33065,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Wedding &amp; event caterer</t>
+          <t>Estate agent &amp; chartered surveyors</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -32387,7 +33075,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Personal training</t>
+          <t>Wedding &amp; event caterer</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -32397,17 +33085,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Dentist / Orthodontics</t>
+          <t>Personal training</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Specialist dental/implant clinic</t>
+          <t>Dentist / Orthodontics</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -32417,7 +33105,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Boutique corporate law firm</t>
+          <t>Specialist dental/implant clinic</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -32427,7 +33115,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Cosmetic/aesthetics clinic</t>
+          <t>Boutique corporate law firm</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -32437,7 +33125,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Skin &amp; laser clinic</t>
+          <t>Cosmetic/aesthetics clinic</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -32447,7 +33135,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Mortgage broker / financial adviser</t>
+          <t>Skin &amp; laser clinic</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -32457,7 +33145,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Architects (RIBA chartered)</t>
+          <t>Mortgage broker / financial adviser</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -32467,7 +33155,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Recruitment agency (tech/startups)</t>
+          <t>Architects (RIBA chartered)</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -32477,7 +33165,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Recruitment agency (IT/data)</t>
+          <t>Recruitment agency (tech/startups)</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -32487,7 +33175,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Independent vet (24/7 emergency)</t>
+          <t>Recruitment agency (IT/data)</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -32497,7 +33185,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Interior design studio</t>
+          <t>Independent vet (24/7 emergency)</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -32507,7 +33195,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Letting &amp; estate agent</t>
+          <t>Interior design studio</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -32517,7 +33205,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Cosmetic clinic (injectables)</t>
+          <t>Letting &amp; estate agent</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -32527,7 +33215,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Cosmetic/anti-ageing clinic</t>
+          <t>Cosmetic clinic (injectables)</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -32537,7 +33225,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Yoga &amp; reformer pilates studio</t>
+          <t>Cosmetic/anti-ageing clinic</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -32547,7 +33235,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Reformer pilates studio</t>
+          <t>Yoga &amp; reformer pilates studio</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -32557,7 +33245,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Wealth management</t>
+          <t>Reformer pilates studio</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -32567,7 +33255,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Private tuition &amp; education consultancy</t>
+          <t>Wealth management</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -32577,7 +33265,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Osteopath</t>
+          <t>Private tuition &amp; education consultancy</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -32587,7 +33275,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Design &amp; build / home renovation</t>
+          <t>Osteopath</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -32597,7 +33285,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Builders / building contractor</t>
+          <t>Design &amp; build / home renovation</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -32607,7 +33295,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Home care / live-in care</t>
+          <t>Builders / building contractor</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -32617,7 +33305,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Private day nurseries</t>
+          <t>Home care / live-in care</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -32627,7 +33315,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Personal training &amp; wellness studio</t>
+          <t>Private day nurseries</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -32637,7 +33325,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Mortgage &amp; insurance broker</t>
+          <t>Personal training &amp; wellness studio</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -32647,7 +33335,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Business consultancy</t>
+          <t>Mortgage &amp; insurance broker</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -32657,7 +33345,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Interior designer (period homes)</t>
+          <t>Business consultancy</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -32667,7 +33355,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Landscape design &amp; build</t>
+          <t>Interior designer (period homes)</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -32677,7 +33365,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Interior designer</t>
+          <t>Landscape design &amp; build</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -32687,7 +33375,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Garden design &amp; landscaping</t>
+          <t>Interior designer</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -32697,7 +33385,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Legal recruitment</t>
+          <t>Garden design &amp; landscaping</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -32707,7 +33395,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Independent gym &amp; health club</t>
+          <t>Legal recruitment</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -32717,7 +33405,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Independent gym</t>
+          <t>Independent gym &amp; health club</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -32727,7 +33415,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Physiotherapy (sports)</t>
+          <t>Independent gym</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -32737,7 +33425,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Letting agent / property management</t>
+          <t>Physiotherapy (sports)</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -32747,7 +33435,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Skin clinic</t>
+          <t>Letting agent / property management</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -32757,7 +33445,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Tutoring company</t>
+          <t>Skin clinic</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -32767,7 +33455,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Tutorial college &amp; exam centre</t>
+          <t>Tutoring company</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -32777,7 +33465,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Employment law (disability discrimination)</t>
+          <t>Tutorial college &amp; exam centre</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -32787,7 +33475,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating</t>
+          <t>Employment law (disability discrimination)</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -32797,7 +33485,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Plumbing &amp; heating</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -32807,7 +33495,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Sports physio &amp; massage</t>
+          <t>Plumbing</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -32817,7 +33505,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Chartered surveyors (party wall/building)</t>
+          <t>Sports physio &amp; massage</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -32827,7 +33515,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Chartered surveyors</t>
+          <t>Chartered surveyors (party wall/building)</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -32837,7 +33525,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Chartered building surveyors</t>
+          <t>Chartered surveyors</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -32847,7 +33535,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Osteopathy clinics</t>
+          <t>Chartered building surveyors</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -32857,7 +33545,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Builders / renovations</t>
+          <t>Osteopathy clinics</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -32867,7 +33555,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Private nursery schools</t>
+          <t>Builders / renovations</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -32877,7 +33565,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Private day nursery</t>
+          <t>Private nursery schools</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -32887,7 +33575,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Private GP (membership model)</t>
+          <t>Private day nursery</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -32897,7 +33585,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Sash window restoration</t>
+          <t>Private GP (membership model)</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -32907,7 +33595,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Personal training (1:1)</t>
+          <t>Sash window restoration</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -32917,7 +33605,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Personal training &amp; nutrition coaching</t>
+          <t>Personal training (1:1)</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -32927,7 +33615,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Private nursery/pre-prep school</t>
+          <t>Personal training &amp; nutrition coaching</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -32937,7 +33625,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Independent nursery (Montessori)</t>
+          <t>Private nursery/pre-prep school</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -32947,7 +33635,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Live-in care agency</t>
+          <t>Independent nursery (Montessori)</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -32957,7 +33645,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Law firm (conveyancing/family)</t>
+          <t>Live-in care agency</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -32967,7 +33655,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Architect &amp; interior designer</t>
+          <t>Law firm (conveyancing/family)</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -32977,7 +33665,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Architects / project management</t>
+          <t>Architect &amp; interior designer</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -32987,7 +33675,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>IFA / wealth management</t>
+          <t>Architects / project management</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -32997,7 +33685,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Physiotherapy &amp; clinical Pilates</t>
+          <t>IFA / wealth management</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -33007,7 +33695,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Aesthetics &amp; skin clinic</t>
+          <t>Physiotherapy &amp; clinical Pilates</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -33017,7 +33705,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Wealth management / IFA</t>
+          <t>Aesthetics &amp; skin clinic</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -33027,7 +33715,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>IFA / financial planning</t>
+          <t>Wealth management / IFA</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -33037,7 +33725,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Wealth management &amp; employee benefits</t>
+          <t>IFA / financial planning</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -33047,7 +33735,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Dermatology clinic</t>
+          <t>Wealth management &amp; employee benefits</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -33057,7 +33745,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Pilates studio (multi-site)</t>
+          <t>Dermatology clinic</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -33067,7 +33755,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Private nursery (Montessori, multi-site)</t>
+          <t>Pilates studio (multi-site)</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -33077,7 +33765,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Law firm (wills &amp; probate)</t>
+          <t>Private nursery (Montessori, multi-site)</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -33087,7 +33775,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Business/technical consultancy</t>
+          <t>Law firm (wills &amp; probate)</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -33097,7 +33785,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Private/NHS dentist</t>
+          <t>Business/technical consultancy</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -33107,7 +33795,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Removals company</t>
+          <t>Private/NHS dentist</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -33117,7 +33805,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Driveways &amp; landscaping</t>
+          <t>Removals company</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -33127,7 +33815,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Wedding &amp; event venue</t>
+          <t>Driveways &amp; landscaping</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -33137,7 +33825,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>IFA &amp; mortgage broker</t>
+          <t>Wedding &amp; event venue</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -33147,7 +33835,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Estate agent &amp; chartered surveyors</t>
+          <t>IFA &amp; mortgage broker</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -33321,6 +34009,16 @@
         </is>
       </c>
       <c r="B140" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Independent vet (mixed practice)</t>
+        </is>
+      </c>
+      <c r="B141" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 34: +8 prospects (379 total) - Windsor, Maidenhead, Ascot
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$372</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$380</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T372"/>
+  <dimension ref="A1:T380"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -32620,8 +32620,692 @@
       </c>
       <c r="T372" s="3" t="inlineStr"/>
     </row>
+    <row r="373">
+      <c r="A373" s="3" t="inlineStr">
+        <is>
+          <t>SLM Property</t>
+        </is>
+      </c>
+      <c r="B373" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C373" s="3" t="inlineStr">
+        <is>
+          <t>Windsor Town Centre, Berkshire</t>
+        </is>
+      </c>
+      <c r="D373" s="3" t="inlineStr">
+        <is>
+          <t>https://www.slmproperty.com</t>
+        </is>
+      </c>
+      <c r="E373" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F373" s="3" t="inlineStr"/>
+      <c r="G373" s="3" t="inlineStr">
+        <is>
+          <t>Lance Mordant &amp; Sophie Potter-Mordant (Father-daughter owners)</t>
+        </is>
+      </c>
+      <c r="H373" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/sophie-potter-mordant-09585a55</t>
+        </is>
+      </c>
+      <c r="I373" s="3" t="inlineStr"/>
+      <c r="J373" s="3" t="inlineStr">
+        <is>
+          <t>Family firm with 90 years of Central London property reputation now serving Windsor; ultra-premium royal-town property fees</t>
+        </is>
+      </c>
+      <c r="K373" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L373" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M373" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N373" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O373" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn presence</t>
+        </is>
+      </c>
+      <c r="P373" s="3" t="inlineStr">
+        <is>
+          <t>90-year family reputation not yet converted into AI-search dominance for Windsor property searches</t>
+        </is>
+      </c>
+      <c r="Q373" s="3" t="inlineStr">
+        <is>
+          <t>'90 years of family reputation, now in Windsor - own that story in AI answers, not just testimonials'</t>
+        </is>
+      </c>
+      <c r="R373" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S373" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T373" s="3" t="inlineStr"/>
+    </row>
+    <row r="374">
+      <c r="A374" s="4" t="inlineStr">
+        <is>
+          <t>Barker Stone</t>
+        </is>
+      </c>
+      <c r="B374" s="4" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C374" s="4" t="inlineStr">
+        <is>
+          <t>Cookham, Maidenhead, Berkshire</t>
+        </is>
+      </c>
+      <c r="D374" s="4" t="inlineStr">
+        <is>
+          <t>https://barkerstone.co.uk</t>
+        </is>
+      </c>
+      <c r="E374" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F374" s="4" t="inlineStr"/>
+      <c r="G374" s="4" t="inlineStr">
+        <is>
+          <t>Simon Stone (Director)</t>
+        </is>
+      </c>
+      <c r="H374" s="4" t="inlineStr">
+        <is>
+          <t>facebook.com/BarkerStoneUK</t>
+        </is>
+      </c>
+      <c r="I374" s="4" t="inlineStr"/>
+      <c r="J374" s="4" t="inlineStr">
+        <is>
+          <t>Bespoke personal service across Berkshire/Bucks/Surrey/London - wide, premium multi-county coverage</t>
+        </is>
+      </c>
+      <c r="K374" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L374" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M374" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N374" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O374" s="4" t="inlineStr">
+        <is>
+          <t>Facebook presence</t>
+        </is>
+      </c>
+      <c r="P374" s="4" t="inlineStr">
+        <is>
+          <t>Wide multi-county claim not matched by per-area search dominance</t>
+        </is>
+      </c>
+      <c r="Q374" s="4" t="inlineStr">
+        <is>
+          <t>Per-town AEO content to actually own the claimed multi-county footprint</t>
+        </is>
+      </c>
+      <c r="R374" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S374" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T374" s="4" t="inlineStr"/>
+    </row>
+    <row r="375">
+      <c r="A375" s="4" t="inlineStr">
+        <is>
+          <t>Marshalls Property Services</t>
+        </is>
+      </c>
+      <c r="B375" s="4" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C375" s="4" t="inlineStr">
+        <is>
+          <t>Windsor, Berkshire</t>
+        </is>
+      </c>
+      <c r="D375" s="4" t="inlineStr">
+        <is>
+          <t>via directory listing</t>
+        </is>
+      </c>
+      <c r="E375" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F375" s="4" t="inlineStr"/>
+      <c r="G375" s="4" t="inlineStr">
+        <is>
+          <t>Est. 1995</t>
+        </is>
+      </c>
+      <c r="H375" s="4" t="inlineStr"/>
+      <c r="I375" s="4" t="inlineStr"/>
+      <c r="J375" s="4" t="inlineStr">
+        <is>
+          <t>Family-owned since 1995, full estate management service in Windsor and surrounding villages</t>
+        </is>
+      </c>
+      <c r="K375" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L375" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M375" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N375" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O375" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P375" s="4" t="inlineStr">
+        <is>
+          <t>30 years of trust untranslated into modern AI-search visibility</t>
+        </is>
+      </c>
+      <c r="Q375" s="4" t="inlineStr">
+        <is>
+          <t>'30 years managing Windsor estates - the AI answer should reflect that heritage'</t>
+        </is>
+      </c>
+      <c r="R375" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S375" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T375" s="4" t="inlineStr">
+        <is>
+          <t>Confirm live website before outreach</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" s="4" t="inlineStr">
+        <is>
+          <t>Optima Dental Care</t>
+        </is>
+      </c>
+      <c r="B376" s="4" t="inlineStr">
+        <is>
+          <t>Private dentist / cosmetic</t>
+        </is>
+      </c>
+      <c r="C376" s="4" t="inlineStr">
+        <is>
+          <t>Boyn Valley Road, Maidenhead, Berkshire</t>
+        </is>
+      </c>
+      <c r="D376" s="4" t="inlineStr">
+        <is>
+          <t>https://optimadentalcare.co.uk</t>
+        </is>
+      </c>
+      <c r="E376" s="4" t="inlineStr">
+        <is>
+          <t>info@optimadentalcare.co.uk</t>
+        </is>
+      </c>
+      <c r="F376" s="4" t="inlineStr">
+        <is>
+          <t>01628 777 552</t>
+        </is>
+      </c>
+      <c r="G376" s="4" t="inlineStr"/>
+      <c r="H376" s="4" t="inlineStr"/>
+      <c r="I376" s="4" t="inlineStr"/>
+      <c r="J376" s="4" t="inlineStr">
+        <is>
+          <t>Private + NHS cosmetic/implant practice also serving High Wycombe - two-town reach</t>
+        </is>
+      </c>
+      <c r="K376" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L376" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M376" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N376" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O376" s="4" t="inlineStr">
+        <is>
+          <t>Two-town service pages (Maidenhead + High Wycombe)</t>
+        </is>
+      </c>
+      <c r="P376" s="4" t="inlineStr">
+        <is>
+          <t>Two-town pages exist but AI-answer citations for either town still open</t>
+        </is>
+      </c>
+      <c r="Q376" s="4" t="inlineStr">
+        <is>
+          <t>Upgrade the existing two-town SEO pages into AEO-optimised assets</t>
+        </is>
+      </c>
+      <c r="R376" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S376" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T376" s="4" t="inlineStr"/>
+    </row>
+    <row r="377">
+      <c r="A377" s="4" t="inlineStr">
+        <is>
+          <t>Portman Dental &amp; Implant Clinic</t>
+        </is>
+      </c>
+      <c r="B377" s="4" t="inlineStr">
+        <is>
+          <t>Private dentist / implants</t>
+        </is>
+      </c>
+      <c r="C377" s="4" t="inlineStr">
+        <is>
+          <t>Maidenhead, Berkshire</t>
+        </is>
+      </c>
+      <c r="D377" s="4" t="inlineStr">
+        <is>
+          <t>https://www.dentists-maidenhead.co.uk</t>
+        </is>
+      </c>
+      <c r="E377" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F377" s="4" t="inlineStr"/>
+      <c r="G377" s="4" t="inlineStr">
+        <is>
+          <t>Est. 2006</t>
+        </is>
+      </c>
+      <c r="H377" s="4" t="inlineStr"/>
+      <c r="I377" s="4" t="inlineStr"/>
+      <c r="J377" s="4" t="inlineStr">
+        <is>
+          <t>Specialist implant clinic playing a central Maidenhead role for nearly 20 years</t>
+        </is>
+      </c>
+      <c r="K377" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L377" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M377" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N377" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O377" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P377" s="4" t="inlineStr">
+        <is>
+          <t>20 years of specialist reputation untranslated into modern AI-search visibility</t>
+        </is>
+      </c>
+      <c r="Q377" s="4" t="inlineStr">
+        <is>
+          <t>'Nearly 20 years of specialist implant care - own that AEO trust signal in Maidenhead'</t>
+        </is>
+      </c>
+      <c r="R377" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S377" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T377" s="4" t="inlineStr"/>
+    </row>
+    <row r="378">
+      <c r="A378" s="3" t="inlineStr">
+        <is>
+          <t>Philip Wadge Architecture Studio</t>
+        </is>
+      </c>
+      <c r="B378" s="3" t="inlineStr">
+        <is>
+          <t>Architects</t>
+        </is>
+      </c>
+      <c r="C378" s="3" t="inlineStr">
+        <is>
+          <t>Berkshire (Ascot/Sunningdale/Windsor/Maidenhead/Newbury)</t>
+        </is>
+      </c>
+      <c r="D378" s="3" t="inlineStr">
+        <is>
+          <t>https://www.philipwadge.co.uk</t>
+        </is>
+      </c>
+      <c r="E378" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F378" s="3" t="inlineStr"/>
+      <c r="G378" s="3" t="inlineStr">
+        <is>
+          <t>Philip Wadge (Founder)</t>
+        </is>
+      </c>
+      <c r="H378" s="3" t="inlineStr"/>
+      <c r="I378" s="3" t="inlineStr"/>
+      <c r="J378" s="3" t="inlineStr">
+        <is>
+          <t>Extremely wide Berkshire coverage across 8+ named towns - genuinely broad reach for a single-founder practice</t>
+        </is>
+      </c>
+      <c r="K378" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L378" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M378" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N378" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O378" s="3" t="inlineStr">
+        <is>
+          <t>Per-town landing pages across many towns = major SEO investment</t>
+        </is>
+      </c>
+      <c r="P378" s="3" t="inlineStr">
+        <is>
+          <t>Landing pages exist for 8+ towns but AI-answer citations remain open across most of them</t>
+        </is>
+      </c>
+      <c r="Q378" s="3" t="inlineStr">
+        <is>
+          <t>'You built pages for 8 towns - the AEO layer could multiply that investment several times over'</t>
+        </is>
+      </c>
+      <c r="R378" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S378" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T378" s="3" t="inlineStr"/>
+    </row>
+    <row r="379">
+      <c r="A379" s="4" t="inlineStr">
+        <is>
+          <t>TPA Studio</t>
+        </is>
+      </c>
+      <c r="B379" s="4" t="inlineStr">
+        <is>
+          <t>Architects</t>
+        </is>
+      </c>
+      <c r="C379" s="4" t="inlineStr">
+        <is>
+          <t>Maidenhead &amp; Thames Valley, Berkshire</t>
+        </is>
+      </c>
+      <c r="D379" s="4" t="inlineStr">
+        <is>
+          <t>https://tpa.studio</t>
+        </is>
+      </c>
+      <c r="E379" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F379" s="4" t="inlineStr"/>
+      <c r="G379" s="4" t="inlineStr">
+        <is>
+          <t>Natasha Gandhi, Ed Drysdale &amp; Peter Thomas (Partners, 30+ yrs combined)</t>
+        </is>
+      </c>
+      <c r="H379" s="4" t="inlineStr"/>
+      <c r="I379" s="4" t="inlineStr"/>
+      <c r="J379" s="4" t="inlineStr">
+        <is>
+          <t>Three-partner practice with 30+ years combined expertise across the Thames Valley</t>
+        </is>
+      </c>
+      <c r="K379" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L379" s="4" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M379" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N379" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O379" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P379" s="4" t="inlineStr">
+        <is>
+          <t>30 years' combined partner expertise untranslated into modern AI-search visibility</t>
+        </is>
+      </c>
+      <c r="Q379" s="4" t="inlineStr">
+        <is>
+          <t>Portfolio-driven AEO content leveraging the partners' combined decades of experience</t>
+        </is>
+      </c>
+      <c r="R379" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S379" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T379" s="4" t="inlineStr"/>
+    </row>
+    <row r="380">
+      <c r="A380" s="3" t="inlineStr">
+        <is>
+          <t>SMA Wealth (Steven Mufti &amp; Associates)</t>
+        </is>
+      </c>
+      <c r="B380" s="3" t="inlineStr">
+        <is>
+          <t>Wealth management / IFA</t>
+        </is>
+      </c>
+      <c r="C380" s="3" t="inlineStr">
+        <is>
+          <t>Ascot, Berkshire</t>
+        </is>
+      </c>
+      <c r="D380" s="3" t="inlineStr">
+        <is>
+          <t>https://www.smawm.co.uk</t>
+        </is>
+      </c>
+      <c r="E380" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F380" s="3" t="inlineStr"/>
+      <c r="G380" s="3" t="inlineStr">
+        <is>
+          <t>Steven Mufti (Founder, Chartered Financial Planner, est. 2013)</t>
+        </is>
+      </c>
+      <c r="H380" s="3" t="inlineStr"/>
+      <c r="I380" s="3" t="inlineStr"/>
+      <c r="J380" s="3" t="inlineStr">
+        <is>
+          <t>Chartered founder serving the Home Counties from Ascot; detailed service-specific content (family wealth, professionals, corporate)</t>
+        </is>
+      </c>
+      <c r="K380" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L380" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M380" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N380" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O380" s="3" t="inlineStr">
+        <is>
+          <t>Multiple detailed service pages = active content marketing</t>
+        </is>
+      </c>
+      <c r="P380" s="3" t="inlineStr">
+        <is>
+          <t>Detailed service content exists but AI-answer citations for specific queries still open</t>
+        </is>
+      </c>
+      <c r="Q380" s="3" t="inlineStr">
+        <is>
+          <t>'You've written pages for every client type - let's make AI cite them, not just index them'</t>
+        </is>
+      </c>
+      <c r="R380" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S380" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T380" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T372"/>
+  <autoFilter ref="A1:T380"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -32632,7 +33316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B141"/>
+  <dimension ref="A1:B142"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -32652,7 +33336,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>371</v>
+        <v>379</v>
       </c>
     </row>
     <row r="5">
@@ -32669,7 +33353,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7">
@@ -32679,7 +33363,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8">
@@ -32709,7 +33393,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11">
@@ -33025,7 +33709,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Architects &amp; interior design</t>
+          <t>Wealth management / IFA</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -33035,7 +33719,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Funeral directors</t>
+          <t>Architects &amp; interior design</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -33045,7 +33729,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Garden rooms / outbuildings</t>
+          <t>Funeral directors</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -33055,7 +33739,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Personal training gym</t>
+          <t>Garden rooms / outbuildings</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -33065,7 +33749,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Estate agent &amp; chartered surveyors</t>
+          <t>Personal training gym</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -33075,7 +33759,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Wedding &amp; event caterer</t>
+          <t>Estate agent &amp; chartered surveyors</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -33085,7 +33769,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Personal training</t>
+          <t>Wedding &amp; event caterer</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -33095,17 +33779,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Dentist / Orthodontics</t>
+          <t>Personal training</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Specialist dental/implant clinic</t>
+          <t>Dentist / Orthodontics</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -33115,7 +33799,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Boutique corporate law firm</t>
+          <t>Specialist dental/implant clinic</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -33125,7 +33809,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Cosmetic/aesthetics clinic</t>
+          <t>Boutique corporate law firm</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -33135,7 +33819,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Skin &amp; laser clinic</t>
+          <t>Cosmetic/aesthetics clinic</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -33145,7 +33829,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Mortgage broker / financial adviser</t>
+          <t>Skin &amp; laser clinic</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -33155,7 +33839,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Architects (RIBA chartered)</t>
+          <t>Mortgage broker / financial adviser</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -33165,7 +33849,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Recruitment agency (tech/startups)</t>
+          <t>Architects (RIBA chartered)</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -33175,7 +33859,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Recruitment agency (IT/data)</t>
+          <t>Recruitment agency (tech/startups)</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -33185,7 +33869,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Independent vet (24/7 emergency)</t>
+          <t>Recruitment agency (IT/data)</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -33195,7 +33879,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Interior design studio</t>
+          <t>Independent vet (24/7 emergency)</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -33205,7 +33889,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Letting &amp; estate agent</t>
+          <t>Interior design studio</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -33215,7 +33899,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Cosmetic clinic (injectables)</t>
+          <t>Letting &amp; estate agent</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -33225,7 +33909,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Cosmetic/anti-ageing clinic</t>
+          <t>Cosmetic clinic (injectables)</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -33235,7 +33919,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Yoga &amp; reformer pilates studio</t>
+          <t>Cosmetic/anti-ageing clinic</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -33245,7 +33929,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Reformer pilates studio</t>
+          <t>Yoga &amp; reformer pilates studio</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -33255,7 +33939,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Wealth management</t>
+          <t>Reformer pilates studio</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -33265,7 +33949,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Private tuition &amp; education consultancy</t>
+          <t>Wealth management</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -33275,7 +33959,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Osteopath</t>
+          <t>Private tuition &amp; education consultancy</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -33285,7 +33969,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Design &amp; build / home renovation</t>
+          <t>Osteopath</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -33295,7 +33979,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Builders / building contractor</t>
+          <t>Design &amp; build / home renovation</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -33305,7 +33989,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Home care / live-in care</t>
+          <t>Builders / building contractor</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -33315,7 +33999,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Private day nurseries</t>
+          <t>Home care / live-in care</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -33325,7 +34009,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Personal training &amp; wellness studio</t>
+          <t>Private day nurseries</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -33335,7 +34019,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Mortgage &amp; insurance broker</t>
+          <t>Personal training &amp; wellness studio</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -33345,7 +34029,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Business consultancy</t>
+          <t>Mortgage &amp; insurance broker</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -33355,7 +34039,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Interior designer (period homes)</t>
+          <t>Business consultancy</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -33365,7 +34049,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Landscape design &amp; build</t>
+          <t>Interior designer (period homes)</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -33375,7 +34059,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Interior designer</t>
+          <t>Landscape design &amp; build</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -33385,7 +34069,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Garden design &amp; landscaping</t>
+          <t>Interior designer</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -33395,7 +34079,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Legal recruitment</t>
+          <t>Garden design &amp; landscaping</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -33405,7 +34089,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Independent gym &amp; health club</t>
+          <t>Legal recruitment</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -33415,7 +34099,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Independent gym</t>
+          <t>Independent gym &amp; health club</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -33425,7 +34109,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Physiotherapy (sports)</t>
+          <t>Independent gym</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -33435,7 +34119,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Letting agent / property management</t>
+          <t>Physiotherapy (sports)</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -33445,7 +34129,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Skin clinic</t>
+          <t>Letting agent / property management</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -33455,7 +34139,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Tutoring company</t>
+          <t>Skin clinic</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -33465,7 +34149,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Tutorial college &amp; exam centre</t>
+          <t>Tutoring company</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -33475,7 +34159,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Employment law (disability discrimination)</t>
+          <t>Tutorial college &amp; exam centre</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -33485,7 +34169,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating</t>
+          <t>Employment law (disability discrimination)</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -33495,7 +34179,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Plumbing &amp; heating</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -33505,7 +34189,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Sports physio &amp; massage</t>
+          <t>Plumbing</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -33515,7 +34199,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Chartered surveyors (party wall/building)</t>
+          <t>Sports physio &amp; massage</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -33525,7 +34209,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Chartered surveyors</t>
+          <t>Chartered surveyors (party wall/building)</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -33535,7 +34219,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Chartered building surveyors</t>
+          <t>Chartered surveyors</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -33545,7 +34229,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Osteopathy clinics</t>
+          <t>Chartered building surveyors</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -33555,7 +34239,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Builders / renovations</t>
+          <t>Osteopathy clinics</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -33565,7 +34249,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Private nursery schools</t>
+          <t>Builders / renovations</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -33575,7 +34259,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Private day nursery</t>
+          <t>Private nursery schools</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -33585,7 +34269,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Private GP (membership model)</t>
+          <t>Private day nursery</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -33595,7 +34279,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Sash window restoration</t>
+          <t>Private GP (membership model)</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -33605,7 +34289,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Personal training (1:1)</t>
+          <t>Sash window restoration</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -33615,7 +34299,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Personal training &amp; nutrition coaching</t>
+          <t>Personal training (1:1)</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -33625,7 +34309,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Private nursery/pre-prep school</t>
+          <t>Personal training &amp; nutrition coaching</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -33635,7 +34319,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Independent nursery (Montessori)</t>
+          <t>Private nursery/pre-prep school</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -33645,7 +34329,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Live-in care agency</t>
+          <t>Independent nursery (Montessori)</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -33655,7 +34339,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Law firm (conveyancing/family)</t>
+          <t>Live-in care agency</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -33665,7 +34349,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Architect &amp; interior designer</t>
+          <t>Law firm (conveyancing/family)</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -33675,7 +34359,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Architects / project management</t>
+          <t>Architect &amp; interior designer</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -33685,7 +34369,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>IFA / wealth management</t>
+          <t>Architects / project management</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -33695,7 +34379,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Physiotherapy &amp; clinical Pilates</t>
+          <t>IFA / wealth management</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -33705,7 +34389,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Aesthetics &amp; skin clinic</t>
+          <t>Physiotherapy &amp; clinical Pilates</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -33715,7 +34399,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Wealth management / IFA</t>
+          <t>Aesthetics &amp; skin clinic</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -34019,6 +34703,16 @@
         </is>
       </c>
       <c r="B141" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Private dentist / cosmetic</t>
+        </is>
+      </c>
+      <c r="B142" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 35: +7 prospects (386 total) - Amersham, Chesham, Ashford
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$380</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$387</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T380"/>
+  <dimension ref="A1:T387"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -33304,8 +33304,616 @@
       </c>
       <c r="T380" s="3" t="inlineStr"/>
     </row>
+    <row r="381">
+      <c r="A381" s="3" t="inlineStr">
+        <is>
+          <t>Robsons Estate Agents</t>
+        </is>
+      </c>
+      <c r="B381" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C381" s="3" t="inlineStr">
+        <is>
+          <t>Amersham &amp; Chesham, Buckinghamshire</t>
+        </is>
+      </c>
+      <c r="D381" s="3" t="inlineStr">
+        <is>
+          <t>https://robsonsweb.com</t>
+        </is>
+      </c>
+      <c r="E381" s="3" t="inlineStr">
+        <is>
+          <t>Property@robsonsbucks.com</t>
+        </is>
+      </c>
+      <c r="F381" s="3" t="inlineStr">
+        <is>
+          <t>01494 724 999</t>
+        </is>
+      </c>
+      <c r="G381" s="3" t="inlineStr">
+        <is>
+          <t>Est. 1962, 9-office independent group</t>
+        </is>
+      </c>
+      <c r="H381" s="3" t="inlineStr"/>
+      <c r="I381" s="3" t="inlineStr"/>
+      <c r="J381" s="3" t="inlineStr">
+        <is>
+          <t>63-year independent group along the Metropolitan Line; 9-office scale gives serious cross-market fee volume</t>
+        </is>
+      </c>
+      <c r="K381" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L381" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M381" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N381" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O381" s="3" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P381" s="3" t="inlineStr">
+        <is>
+          <t>63 years of heritage across 9 offices untranslated into modern per-office AI-search visibility</t>
+        </is>
+      </c>
+      <c r="Q381" s="3" t="inlineStr">
+        <is>
+          <t>'63 years along the Met Line - own the AI answer for every office, not just Rightmove'</t>
+        </is>
+      </c>
+      <c r="R381" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S381" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T381" s="3" t="inlineStr"/>
+    </row>
+    <row r="382">
+      <c r="A382" s="4" t="inlineStr">
+        <is>
+          <t>Binks Estate Agents</t>
+        </is>
+      </c>
+      <c r="B382" s="4" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C382" s="4" t="inlineStr">
+        <is>
+          <t>Amersham/Chorleywood (Northwood to Chesham corridor)</t>
+        </is>
+      </c>
+      <c r="D382" s="4" t="inlineStr">
+        <is>
+          <t>https://binksweb.com</t>
+        </is>
+      </c>
+      <c r="E382" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F382" s="4" t="inlineStr"/>
+      <c r="G382" s="4" t="inlineStr">
+        <is>
+          <t>Est. 1994</t>
+        </is>
+      </c>
+      <c r="H382" s="4" t="inlineStr"/>
+      <c r="I382" s="4" t="inlineStr"/>
+      <c r="J382" s="4" t="inlineStr">
+        <is>
+          <t>31-year independent along the Metropolitan Line corridor; premium lettings/management specialism</t>
+        </is>
+      </c>
+      <c r="K382" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L382" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M382" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N382" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O382" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P382" s="4" t="inlineStr">
+        <is>
+          <t>Corporate rivals (Savills, Knight Frank) compete for the same Met Line searches</t>
+        </is>
+      </c>
+      <c r="Q382" s="4" t="inlineStr">
+        <is>
+          <t>'31 years along the Met Line - own the AI answer for Amersham/Chorleywood property'</t>
+        </is>
+      </c>
+      <c r="R382" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S382" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T382" s="4" t="inlineStr"/>
+    </row>
+    <row r="383">
+      <c r="A383" s="3" t="inlineStr">
+        <is>
+          <t>Chess House Dental Practice</t>
+        </is>
+      </c>
+      <c r="B383" s="3" t="inlineStr">
+        <is>
+          <t>Private dentist / implants</t>
+        </is>
+      </c>
+      <c r="C383" s="3" t="inlineStr">
+        <is>
+          <t>High Street, Chesham, Buckinghamshire</t>
+        </is>
+      </c>
+      <c r="D383" s="3" t="inlineStr">
+        <is>
+          <t>https://www.chesshousedental.com</t>
+        </is>
+      </c>
+      <c r="E383" s="3" t="inlineStr">
+        <is>
+          <t>info@chesshousedental.com</t>
+        </is>
+      </c>
+      <c r="F383" s="3" t="inlineStr">
+        <is>
+          <t>01494 977 140</t>
+        </is>
+      </c>
+      <c r="G383" s="3" t="inlineStr">
+        <is>
+          <t>Dr Yash Ghevaria &amp; Dr Devang Patel (Implantology team)</t>
+        </is>
+      </c>
+      <c r="H383" s="3" t="inlineStr"/>
+      <c r="I383" s="3" t="inlineStr"/>
+      <c r="J383" s="3" t="inlineStr">
+        <is>
+          <t>Named implant specialists serving 4 Bucks towns (Chesham/Amersham/Chalfont/Bovingdon) from one practice</t>
+        </is>
+      </c>
+      <c r="K383" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L383" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M383" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N383" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O383" s="3" t="inlineStr">
+        <is>
+          <t>Dedicated implants page = active SEO</t>
+        </is>
+      </c>
+      <c r="P383" s="3" t="inlineStr">
+        <is>
+          <t>4-town claim not matched by per-town search dominance for implant searches</t>
+        </is>
+      </c>
+      <c r="Q383" s="3" t="inlineStr">
+        <is>
+          <t>Per-town AEO content for 'dental implants' across all 4 claimed towns</t>
+        </is>
+      </c>
+      <c r="R383" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S383" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T383" s="3" t="inlineStr"/>
+    </row>
+    <row r="384">
+      <c r="A384" s="4" t="inlineStr">
+        <is>
+          <t>The Dental &amp; Implant Centre</t>
+        </is>
+      </c>
+      <c r="B384" s="4" t="inlineStr">
+        <is>
+          <t>Private dentist / implants</t>
+        </is>
+      </c>
+      <c r="C384" s="4" t="inlineStr">
+        <is>
+          <t>Hill Avenue, Amersham, Buckinghamshire</t>
+        </is>
+      </c>
+      <c r="D384" s="4" t="inlineStr">
+        <is>
+          <t>https://www.dentalandimplant.co.uk</t>
+        </is>
+      </c>
+      <c r="E384" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F384" s="4" t="inlineStr">
+        <is>
+          <t>01494 854 053</t>
+        </is>
+      </c>
+      <c r="G384" s="4" t="inlineStr"/>
+      <c r="H384" s="4" t="inlineStr"/>
+      <c r="I384" s="4" t="inlineStr"/>
+      <c r="J384" s="4" t="inlineStr">
+        <is>
+          <t>Affordable-positioned implant specialist in Amersham; value-conscious implant patient segment</t>
+        </is>
+      </c>
+      <c r="K384" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L384" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M384" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N384" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O384" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P384" s="4" t="inlineStr">
+        <is>
+          <t>'Affordable' positioning not yet the AI-cited local answer for value-conscious implant searches</t>
+        </is>
+      </c>
+      <c r="Q384" s="4" t="inlineStr">
+        <is>
+          <t>Own the value-conscious implant-patient AEO segment in Amersham</t>
+        </is>
+      </c>
+      <c r="R384" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S384" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T384" s="4" t="inlineStr"/>
+    </row>
+    <row r="385">
+      <c r="A385" s="2" t="inlineStr">
+        <is>
+          <t>Evolution Properties</t>
+        </is>
+      </c>
+      <c r="B385" s="2" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C385" s="2" t="inlineStr">
+        <is>
+          <t>Ashford (+ Folkestone/Maidstone), Kent</t>
+        </is>
+      </c>
+      <c r="D385" s="2" t="inlineStr">
+        <is>
+          <t>https://evolutionproperties.co.uk</t>
+        </is>
+      </c>
+      <c r="E385" s="2" t="inlineStr">
+        <is>
+          <t>ashford@evolutionproperties.co.uk</t>
+        </is>
+      </c>
+      <c r="F385" s="2" t="inlineStr">
+        <is>
+          <t>01233 501 601</t>
+        </is>
+      </c>
+      <c r="G385" s="2" t="inlineStr">
+        <is>
+          <t>Sharron (Founder, est. 2012)</t>
+        </is>
+      </c>
+      <c r="H385" s="2" t="inlineStr"/>
+      <c r="I385" s="2" t="inlineStr"/>
+      <c r="J385" s="2" t="inlineStr">
+        <is>
+          <t>Gold Award-winning independent, invitation-only industry recognition, 130+ years combined staff experience</t>
+        </is>
+      </c>
+      <c r="K385" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L385" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M385" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N385" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O385" s="2" t="inlineStr">
+        <is>
+          <t>Gold Award status; polished agent-profile pages</t>
+        </is>
+      </c>
+      <c r="P385" s="2" t="inlineStr">
+        <is>
+          <t>Award status is a strong AEO trust signal not yet the AI-cited answer for Ashford property</t>
+        </is>
+      </c>
+      <c r="Q385" s="2" t="inlineStr">
+        <is>
+          <t>'Gold Award-winning, invitation-only recognition - own that exact AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R385" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S385" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T385" s="2" t="inlineStr">
+        <is>
+          <t>Award pedigree + founder story = strong AEO opportunity</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" s="3" t="inlineStr">
+        <is>
+          <t>Geering &amp; Colyer</t>
+        </is>
+      </c>
+      <c r="B386" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C386" s="3" t="inlineStr">
+        <is>
+          <t>Ashford, Kent</t>
+        </is>
+      </c>
+      <c r="D386" s="3" t="inlineStr">
+        <is>
+          <t>https://www.geeringandcolyer.co.uk</t>
+        </is>
+      </c>
+      <c r="E386" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F386" s="3" t="inlineStr"/>
+      <c r="G386" s="3" t="inlineStr">
+        <is>
+          <t>Est. 1800s (Robert Geering &amp; Frank Colyer)</t>
+        </is>
+      </c>
+      <c r="H386" s="3" t="inlineStr"/>
+      <c r="I386" s="3" t="inlineStr"/>
+      <c r="J386" s="3" t="inlineStr">
+        <is>
+          <t>115+ year heritage firm - one of the oldest independent names in Kent property</t>
+        </is>
+      </c>
+      <c r="K386" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L386" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M386" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N386" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O386" s="3" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P386" s="3" t="inlineStr">
+        <is>
+          <t>115 years of history vastly underused as an AI-search trust signal</t>
+        </is>
+      </c>
+      <c r="Q386" s="3" t="inlineStr">
+        <is>
+          <t>'115 years in Kent property - the AI answer should say so, not just the company history page'</t>
+        </is>
+      </c>
+      <c r="R386" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S386" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T386" s="3" t="inlineStr"/>
+    </row>
+    <row r="387">
+      <c r="A387" s="4" t="inlineStr">
+        <is>
+          <t>Cansdales</t>
+        </is>
+      </c>
+      <c r="B387" s="4" t="inlineStr">
+        <is>
+          <t>Chartered accountants &amp; financial advisers</t>
+        </is>
+      </c>
+      <c r="C387" s="4" t="inlineStr">
+        <is>
+          <t>Little Chalfont &amp; Old Amersham, Buckinghamshire</t>
+        </is>
+      </c>
+      <c r="D387" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cansdales.co.uk</t>
+        </is>
+      </c>
+      <c r="E387" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F387" s="4" t="inlineStr">
+        <is>
+          <t>01494 924 417</t>
+        </is>
+      </c>
+      <c r="G387" s="4" t="inlineStr">
+        <is>
+          <t>John Thornton (Director)</t>
+        </is>
+      </c>
+      <c r="H387" s="4" t="inlineStr"/>
+      <c r="I387" s="4" t="inlineStr"/>
+      <c r="J387" s="4" t="inlineStr">
+        <is>
+          <t>Combined accountancy + IFA firm across two Amersham-area offices - two revenue lines per client relationship</t>
+        </is>
+      </c>
+      <c r="K387" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L387" s="4" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M387" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N387" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O387" s="4" t="inlineStr">
+        <is>
+          <t>Two-office presence; SKS network member</t>
+        </is>
+      </c>
+      <c r="P387" s="4" t="inlineStr">
+        <is>
+          <t>Combined-service model not unified into one coherent AEO strategy across accountancy and IFA searches</t>
+        </is>
+      </c>
+      <c r="Q387" s="4" t="inlineStr">
+        <is>
+          <t>Consolidate accountancy + IFA services into one coherent local AEO content plan</t>
+        </is>
+      </c>
+      <c r="R387" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S387" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T387" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T380"/>
+  <autoFilter ref="A1:T387"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -33316,7 +33924,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B142"/>
+  <dimension ref="A1:B143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -33336,7 +33944,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>379</v>
+        <v>386</v>
       </c>
     </row>
     <row r="5">
@@ -33353,7 +33961,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
     </row>
     <row r="7">
@@ -33379,17 +33987,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Independent vet</t>
+          <t>Private dentist / implants</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Private dentist / implants</t>
+          <t>Independent vet</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -34713,6 +35321,16 @@
         </is>
       </c>
       <c r="B142" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Chartered accountants &amp; financial advisers</t>
+        </is>
+      </c>
+      <c r="B143" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 36: +8 prospects (394 total) - recruitment/education/training push begins
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$387</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$395</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T387"/>
+  <dimension ref="A1:T395"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -33912,8 +33912,724 @@
       </c>
       <c r="T387" s="4" t="inlineStr"/>
     </row>
+    <row r="388">
+      <c r="A388" s="3" t="inlineStr">
+        <is>
+          <t>Safehands Recruitment (Bristol)</t>
+        </is>
+      </c>
+      <c r="B388" s="3" t="inlineStr">
+        <is>
+          <t>Healthcare recruitment agency</t>
+        </is>
+      </c>
+      <c r="C388" s="3" t="inlineStr">
+        <is>
+          <t>Castlemead, Bristol</t>
+        </is>
+      </c>
+      <c r="D388" s="3" t="inlineStr">
+        <is>
+          <t>https://www.safehandsrecruitment.co.uk/office/bristol/</t>
+        </is>
+      </c>
+      <c r="E388" s="3" t="inlineStr">
+        <is>
+          <t>info@safehandsrecruitment.co.uk</t>
+        </is>
+      </c>
+      <c r="F388" s="3" t="inlineStr">
+        <is>
+          <t>0117 917 5777</t>
+        </is>
+      </c>
+      <c r="G388" s="3" t="inlineStr">
+        <is>
+          <t>Oli Yuille (Franchise owner, 25+ yrs recruitment experience)</t>
+        </is>
+      </c>
+      <c r="H388" s="3" t="inlineStr"/>
+      <c r="I388" s="3" t="inlineStr"/>
+      <c r="J388" s="3" t="inlineStr">
+        <is>
+          <t>Interim/permanent/temp staffing for social care and healthcare sector; care homes and NHS trusts pay premium day rates per placement</t>
+        </is>
+      </c>
+      <c r="K388" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L388" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M388" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N388" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O388" s="3" t="inlineStr">
+        <is>
+          <t>Franchise brand with national marketing support</t>
+        </is>
+      </c>
+      <c r="P388" s="3" t="inlineStr">
+        <is>
+          <t>Franchise model means local search visibility competes with sister branches for the same brand terms</t>
+        </is>
+      </c>
+      <c r="Q388" s="3" t="inlineStr">
+        <is>
+          <t>'Bristol's own Safehands - own the local AI answer, not just the national franchise site'</t>
+        </is>
+      </c>
+      <c r="R388" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S388" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T388" s="3" t="inlineStr"/>
+    </row>
+    <row r="389">
+      <c r="A389" s="3" t="inlineStr">
+        <is>
+          <t>Moon Executive Search</t>
+        </is>
+      </c>
+      <c r="B389" s="3" t="inlineStr">
+        <is>
+          <t>Executive search / headhunting</t>
+        </is>
+      </c>
+      <c r="C389" s="3" t="inlineStr">
+        <is>
+          <t>Bristol &amp; London</t>
+        </is>
+      </c>
+      <c r="D389" s="3" t="inlineStr">
+        <is>
+          <t>https://www.moonexecsearch.com</t>
+        </is>
+      </c>
+      <c r="E389" s="3" t="inlineStr">
+        <is>
+          <t>recruit@moonexecsearch.com</t>
+        </is>
+      </c>
+      <c r="F389" s="3" t="inlineStr">
+        <is>
+          <t>01275 371 200</t>
+        </is>
+      </c>
+      <c r="G389" s="3" t="inlineStr">
+        <is>
+          <t>Vanessa Moon &amp; Simon Quinn (Principals)</t>
+        </is>
+      </c>
+      <c r="H389" s="3" t="inlineStr"/>
+      <c r="I389" s="3" t="inlineStr"/>
+      <c r="J389" s="3" t="inlineStr">
+        <is>
+          <t>20+ years senior/board-level search; single placement fees run into tens of thousands; charity/corporate client mix</t>
+        </is>
+      </c>
+      <c r="K389" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L389" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M389" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N389" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O389" s="3" t="inlineStr">
+        <is>
+          <t>Press coverage (charity appointments)</t>
+        </is>
+      </c>
+      <c r="P389" s="3" t="inlineStr">
+        <is>
+          <t>High-value senior search queries increasingly researched via AI before a headhunter is contacted directly</t>
+        </is>
+      </c>
+      <c r="Q389" s="3" t="inlineStr">
+        <is>
+          <t>'When boards ask ChatGPT who handles senior search in the South West, be the answer'</t>
+        </is>
+      </c>
+      <c r="R389" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S389" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T389" s="3" t="inlineStr"/>
+    </row>
+    <row r="390">
+      <c r="A390" s="3" t="inlineStr">
+        <is>
+          <t>Safe Haven Training</t>
+        </is>
+      </c>
+      <c r="B390" s="3" t="inlineStr">
+        <is>
+          <t>First aid &amp; health &amp; safety training</t>
+        </is>
+      </c>
+      <c r="C390" s="3" t="inlineStr">
+        <is>
+          <t>Cannock (nationwide UK delivery)</t>
+        </is>
+      </c>
+      <c r="D390" s="3" t="inlineStr">
+        <is>
+          <t>https://www.safehaventraining.co.uk</t>
+        </is>
+      </c>
+      <c r="E390" s="3" t="inlineStr">
+        <is>
+          <t>info@safehaventraining.co.uk</t>
+        </is>
+      </c>
+      <c r="F390" s="3" t="inlineStr">
+        <is>
+          <t>0800 260 6942</t>
+        </is>
+      </c>
+      <c r="G390" s="3" t="inlineStr">
+        <is>
+          <t>Ian Bryan (Founder, ex-NHS paramedic, est. 2012)</t>
+        </is>
+      </c>
+      <c r="H390" s="3" t="inlineStr"/>
+      <c r="I390" s="3" t="inlineStr"/>
+      <c r="J390" s="3" t="inlineStr">
+        <is>
+          <t>Nationwide certified first aid/H&amp;S training for businesses; corporate training contracts recur annually per client</t>
+        </is>
+      </c>
+      <c r="K390" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L390" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M390" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N390" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O390" s="3" t="inlineStr">
+        <is>
+          <t>Nationwide coverage claim; paramedic-credential branding</t>
+        </is>
+      </c>
+      <c r="P390" s="3" t="inlineStr">
+        <is>
+          <t>Nationwide reach means competing with dozens of similarly-positioned training providers in generic search</t>
+        </is>
+      </c>
+      <c r="Q390" s="3" t="inlineStr">
+        <is>
+          <t>'An ex-NHS paramedic teaching your team first aid' - own that credibility angle in AEO content</t>
+        </is>
+      </c>
+      <c r="R390" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S390" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T390" s="3" t="inlineStr"/>
+    </row>
+    <row r="391">
+      <c r="A391" s="3" t="inlineStr">
+        <is>
+          <t>Education People</t>
+        </is>
+      </c>
+      <c r="B391" s="3" t="inlineStr">
+        <is>
+          <t>Teaching &amp; education recruitment agency</t>
+        </is>
+      </c>
+      <c r="C391" s="3" t="inlineStr">
+        <is>
+          <t>Bristol (South West England)</t>
+        </is>
+      </c>
+      <c r="D391" s="3" t="inlineStr">
+        <is>
+          <t>https://educationpeopleltd.com</t>
+        </is>
+      </c>
+      <c r="E391" s="3" t="inlineStr">
+        <is>
+          <t>nicole@educationpeopleltd.com</t>
+        </is>
+      </c>
+      <c r="F391" s="3" t="inlineStr">
+        <is>
+          <t>0117 325 2516</t>
+        </is>
+      </c>
+      <c r="G391" s="3" t="inlineStr">
+        <is>
+          <t>Nicole Dommett (Founder &amp; Director, est. 2008)</t>
+        </is>
+      </c>
+      <c r="H391" s="3" t="inlineStr"/>
+      <c r="I391" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/educationpeople</t>
+        </is>
+      </c>
+      <c r="J391" s="3" t="inlineStr">
+        <is>
+          <t>17-year independent education recruiter covering Bristol/BANES/Somerset/Gloucestershire; schools pay per-placement fees repeatedly each term</t>
+        </is>
+      </c>
+      <c r="K391" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L391" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M391" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N391" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O391" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence; established regional brand</t>
+        </is>
+      </c>
+      <c r="P391" s="3" t="inlineStr">
+        <is>
+          <t>TeacherActive/Tradewind/Prospero national brands with bigger budgets dominate 'teaching agency Bristol' search</t>
+        </is>
+      </c>
+      <c r="Q391" s="3" t="inlineStr">
+        <is>
+          <t>'17 years placing South West teachers - own that AEO answer against the national chains'</t>
+        </is>
+      </c>
+      <c r="R391" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S391" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T391" s="3" t="inlineStr"/>
+    </row>
+    <row r="392">
+      <c r="A392" s="3" t="inlineStr">
+        <is>
+          <t>Supply Education Alliance</t>
+        </is>
+      </c>
+      <c r="B392" s="3" t="inlineStr">
+        <is>
+          <t>Supply teaching agency</t>
+        </is>
+      </c>
+      <c r="C392" s="3" t="inlineStr">
+        <is>
+          <t>Taunton (serves Bristol/Bath/Somerset/Wiltshire)</t>
+        </is>
+      </c>
+      <c r="D392" s="3" t="inlineStr">
+        <is>
+          <t>https://supply-education-alliance.co.uk</t>
+        </is>
+      </c>
+      <c r="E392" s="3" t="inlineStr">
+        <is>
+          <t>admin@supply-education-alliance.co.uk</t>
+        </is>
+      </c>
+      <c r="F392" s="3" t="inlineStr">
+        <is>
+          <t>0117 990 3481</t>
+        </is>
+      </c>
+      <c r="G392" s="3" t="inlineStr">
+        <is>
+          <t>Marie &amp; Emma (Co-founders, 17+ yrs combined)</t>
+        </is>
+      </c>
+      <c r="H392" s="3" t="inlineStr">
+        <is>
+          <t>instagram.com/supplyeducationalliance</t>
+        </is>
+      </c>
+      <c r="I392" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/somerseteducationallianceltd</t>
+        </is>
+      </c>
+      <c r="J392" s="3" t="inlineStr">
+        <is>
+          <t>Independent supply-teaching specialist across 3 counties from a Somerset base; recurring termly school placements</t>
+        </is>
+      </c>
+      <c r="K392" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L392" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M392" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N392" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O392" s="3" t="inlineStr">
+        <is>
+          <t>Instagram/Facebook presence</t>
+        </is>
+      </c>
+      <c r="P392" s="3" t="inlineStr">
+        <is>
+          <t>3-county claim not matched by per-county search dominance vs bigger agencies</t>
+        </is>
+      </c>
+      <c r="Q392" s="3" t="inlineStr">
+        <is>
+          <t>Per-county AEO content to actually own Bristol/Bath/Wiltshire searches separately</t>
+        </is>
+      </c>
+      <c r="R392" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S392" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T392" s="3" t="inlineStr"/>
+    </row>
+    <row r="393">
+      <c r="A393" s="4" t="inlineStr">
+        <is>
+          <t>Harper Construction Recruitment</t>
+        </is>
+      </c>
+      <c r="B393" s="4" t="inlineStr">
+        <is>
+          <t>Construction recruitment agency</t>
+        </is>
+      </c>
+      <c r="C393" s="4" t="inlineStr">
+        <is>
+          <t>Clevedon, Bristol (South West)</t>
+        </is>
+      </c>
+      <c r="D393" s="4" t="inlineStr">
+        <is>
+          <t>https://harperconstructionrecruitment.co.uk</t>
+        </is>
+      </c>
+      <c r="E393" s="4" t="inlineStr">
+        <is>
+          <t>info@harpercr.co.uk</t>
+        </is>
+      </c>
+      <c r="F393" s="4" t="inlineStr">
+        <is>
+          <t>01275 873 664</t>
+        </is>
+      </c>
+      <c r="G393" s="4" t="inlineStr">
+        <is>
+          <t>Family-run, est. ~2006 (nearly 20 years)</t>
+        </is>
+      </c>
+      <c r="H393" s="4" t="inlineStr"/>
+      <c r="I393" s="4" t="inlineStr"/>
+      <c r="J393" s="4" t="inlineStr">
+        <is>
+          <t>Independent trades/labour supplier to South West building sites; placement fees plus ongoing temp-labour margin per worker per week</t>
+        </is>
+      </c>
+      <c r="K393" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L393" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M393" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N393" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O393" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P393" s="4" t="inlineStr">
+        <is>
+          <t>Time4Recruitment/national construction agencies compete for the same South West site-labour searches</t>
+        </is>
+      </c>
+      <c r="Q393" s="4" t="inlineStr">
+        <is>
+          <t>'20 years supplying South West sites - own the AI answer for "construction recruitment Bristol"'</t>
+        </is>
+      </c>
+      <c r="R393" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S393" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T393" s="4" t="inlineStr"/>
+    </row>
+    <row r="394">
+      <c r="A394" s="4" t="inlineStr">
+        <is>
+          <t>Drayton Fox</t>
+        </is>
+      </c>
+      <c r="B394" s="4" t="inlineStr">
+        <is>
+          <t>Construction recruitment agency</t>
+        </is>
+      </c>
+      <c r="C394" s="4" t="inlineStr">
+        <is>
+          <t>Bristol (South West England)</t>
+        </is>
+      </c>
+      <c r="D394" s="4" t="inlineStr">
+        <is>
+          <t>https://www.draytonfox.com</t>
+        </is>
+      </c>
+      <c r="E394" s="4" t="inlineStr">
+        <is>
+          <t>alex.wyatt@draytonfox.com</t>
+        </is>
+      </c>
+      <c r="F394" s="4" t="inlineStr">
+        <is>
+          <t>07498 154 635</t>
+        </is>
+      </c>
+      <c r="G394" s="4" t="inlineStr"/>
+      <c r="H394" s="4" t="inlineStr"/>
+      <c r="I394" s="4" t="inlineStr"/>
+      <c r="J394" s="4" t="inlineStr">
+        <is>
+          <t>Independent built-environment recruiter; permanent/temp/contract placements across the South West construction sector</t>
+        </is>
+      </c>
+      <c r="K394" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L394" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M394" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N394" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O394" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P394" s="4" t="inlineStr">
+        <is>
+          <t>Generic 'construction recruitment Bristol' searches split across several similar independents</t>
+        </is>
+      </c>
+      <c r="Q394" s="4" t="inlineStr">
+        <is>
+          <t>Own a specific built-environment sub-niche (e.g. quantity surveyors, site managers) in AEO content</t>
+        </is>
+      </c>
+      <c r="R394" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S394" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T394" s="4" t="inlineStr"/>
+    </row>
+    <row r="395">
+      <c r="A395" s="4" t="inlineStr">
+        <is>
+          <t>Evolve Hospitality Recruitment</t>
+        </is>
+      </c>
+      <c r="B395" s="4" t="inlineStr">
+        <is>
+          <t>Hospitality staffing agency</t>
+        </is>
+      </c>
+      <c r="C395" s="4" t="inlineStr">
+        <is>
+          <t>City of London (nationwide)</t>
+        </is>
+      </c>
+      <c r="D395" s="4" t="inlineStr">
+        <is>
+          <t>https://evolvehospitality.co.uk</t>
+        </is>
+      </c>
+      <c r="E395" s="4" t="inlineStr">
+        <is>
+          <t>london@evolvehospitality.co.uk</t>
+        </is>
+      </c>
+      <c r="F395" s="4" t="inlineStr">
+        <is>
+          <t>0207 397 1260</t>
+        </is>
+      </c>
+      <c r="G395" s="4" t="inlineStr">
+        <is>
+          <t>Ed Vokes (Director, est. 2011)</t>
+        </is>
+      </c>
+      <c r="H395" s="4" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/ed-vokes-9a113433</t>
+        </is>
+      </c>
+      <c r="I395" s="4" t="inlineStr"/>
+      <c r="J395" s="4" t="inlineStr">
+        <is>
+          <t>14-year specialist hospitality staffing firm; caterers/hotels/venues pay recurring temp-staffing margins for events and shifts</t>
+        </is>
+      </c>
+      <c r="K395" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L395" s="4" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M395" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N395" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O395" s="4" t="inlineStr">
+        <is>
+          <t>Established multi-year brand</t>
+        </is>
+      </c>
+      <c r="P395" s="4" t="inlineStr">
+        <is>
+          <t>Crowded London hospitality-staffing market with many similarly-positioned independents</t>
+        </is>
+      </c>
+      <c r="Q395" s="4" t="inlineStr">
+        <is>
+          <t>Own a specific hospitality-staffing niche (e.g. Michelin-standard chefs, prestige events) in AEO content</t>
+        </is>
+      </c>
+      <c r="R395" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S395" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T395" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T387"/>
+  <autoFilter ref="A1:T395"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -33924,7 +34640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B143"/>
+  <dimension ref="A1:B150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -33944,7 +34660,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>386</v>
+        <v>394</v>
       </c>
     </row>
     <row r="5">
@@ -34397,17 +35113,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Dentist / Orthodontics</t>
+          <t>Construction recruitment agency</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Specialist dental/implant clinic</t>
+          <t>Dentist / Orthodontics</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -34417,7 +35133,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Boutique corporate law firm</t>
+          <t>Specialist dental/implant clinic</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -34427,7 +35143,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Cosmetic/aesthetics clinic</t>
+          <t>Boutique corporate law firm</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -34437,7 +35153,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Skin &amp; laser clinic</t>
+          <t>Cosmetic/aesthetics clinic</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -34447,7 +35163,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Mortgage broker / financial adviser</t>
+          <t>Skin &amp; laser clinic</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -34457,7 +35173,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Architects (RIBA chartered)</t>
+          <t>Mortgage broker / financial adviser</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -34467,7 +35183,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Recruitment agency (tech/startups)</t>
+          <t>Architects (RIBA chartered)</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -34477,7 +35193,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Recruitment agency (IT/data)</t>
+          <t>Recruitment agency (tech/startups)</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -34487,7 +35203,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Independent vet (24/7 emergency)</t>
+          <t>Recruitment agency (IT/data)</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -34497,7 +35213,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Interior design studio</t>
+          <t>Independent vet (24/7 emergency)</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -34507,7 +35223,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Letting &amp; estate agent</t>
+          <t>Interior design studio</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -34517,7 +35233,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Cosmetic clinic (injectables)</t>
+          <t>Letting &amp; estate agent</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -34527,7 +35243,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Cosmetic/anti-ageing clinic</t>
+          <t>Cosmetic clinic (injectables)</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -34537,7 +35253,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Yoga &amp; reformer pilates studio</t>
+          <t>Cosmetic/anti-ageing clinic</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -34547,7 +35263,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Reformer pilates studio</t>
+          <t>Yoga &amp; reformer pilates studio</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -34557,7 +35273,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Wealth management</t>
+          <t>Reformer pilates studio</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -34567,7 +35283,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Private tuition &amp; education consultancy</t>
+          <t>Wealth management</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -34577,7 +35293,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Osteopath</t>
+          <t>Private tuition &amp; education consultancy</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -34587,7 +35303,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Design &amp; build / home renovation</t>
+          <t>Osteopath</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -34597,7 +35313,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Builders / building contractor</t>
+          <t>Design &amp; build / home renovation</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -34607,7 +35323,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Home care / live-in care</t>
+          <t>Builders / building contractor</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -34617,7 +35333,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Private day nurseries</t>
+          <t>Home care / live-in care</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -34627,7 +35343,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Personal training &amp; wellness studio</t>
+          <t>Private day nurseries</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -34637,7 +35353,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Mortgage &amp; insurance broker</t>
+          <t>Personal training &amp; wellness studio</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -34647,7 +35363,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Business consultancy</t>
+          <t>Mortgage &amp; insurance broker</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -34657,7 +35373,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Interior designer (period homes)</t>
+          <t>Business consultancy</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -34667,7 +35383,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Landscape design &amp; build</t>
+          <t>Interior designer (period homes)</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -34677,7 +35393,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Interior designer</t>
+          <t>Landscape design &amp; build</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -34687,7 +35403,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Garden design &amp; landscaping</t>
+          <t>Interior designer</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -34697,7 +35413,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Legal recruitment</t>
+          <t>Garden design &amp; landscaping</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -34707,7 +35423,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Independent gym &amp; health club</t>
+          <t>Legal recruitment</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -34717,7 +35433,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Independent gym</t>
+          <t>Independent gym &amp; health club</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -34727,7 +35443,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Physiotherapy (sports)</t>
+          <t>Independent gym</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -34737,7 +35453,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Letting agent / property management</t>
+          <t>Physiotherapy (sports)</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -34747,7 +35463,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Skin clinic</t>
+          <t>Letting agent / property management</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -34757,7 +35473,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Tutoring company</t>
+          <t>Skin clinic</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -34767,7 +35483,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Tutorial college &amp; exam centre</t>
+          <t>Tutoring company</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -34777,7 +35493,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Employment law (disability discrimination)</t>
+          <t>Tutorial college &amp; exam centre</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -34787,7 +35503,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating</t>
+          <t>Employment law (disability discrimination)</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -34797,7 +35513,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Plumbing &amp; heating</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -34807,7 +35523,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Sports physio &amp; massage</t>
+          <t>Plumbing</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -34817,7 +35533,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Chartered surveyors (party wall/building)</t>
+          <t>Sports physio &amp; massage</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -34827,7 +35543,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Chartered surveyors</t>
+          <t>Chartered surveyors (party wall/building)</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -34837,7 +35553,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Chartered building surveyors</t>
+          <t>Chartered surveyors</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -34847,7 +35563,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Osteopathy clinics</t>
+          <t>Chartered building surveyors</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -34857,7 +35573,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Builders / renovations</t>
+          <t>Osteopathy clinics</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -34867,7 +35583,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Private nursery schools</t>
+          <t>Builders / renovations</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -34877,7 +35593,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Private day nursery</t>
+          <t>Private nursery schools</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -34887,7 +35603,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Private GP (membership model)</t>
+          <t>Private day nursery</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -34897,7 +35613,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Sash window restoration</t>
+          <t>Private GP (membership model)</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -34907,7 +35623,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Personal training (1:1)</t>
+          <t>Sash window restoration</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -34917,7 +35633,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Personal training &amp; nutrition coaching</t>
+          <t>Personal training (1:1)</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -34927,7 +35643,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Private nursery/pre-prep school</t>
+          <t>Personal training &amp; nutrition coaching</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -34937,7 +35653,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Independent nursery (Montessori)</t>
+          <t>Private nursery/pre-prep school</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -34947,7 +35663,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Live-in care agency</t>
+          <t>Independent nursery (Montessori)</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -34957,7 +35673,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Law firm (conveyancing/family)</t>
+          <t>Live-in care agency</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -34967,7 +35683,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Architect &amp; interior designer</t>
+          <t>Law firm (conveyancing/family)</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -34977,7 +35693,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Architects / project management</t>
+          <t>Architect &amp; interior designer</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -34987,7 +35703,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>IFA / wealth management</t>
+          <t>Architects / project management</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -34997,7 +35713,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Physiotherapy &amp; clinical Pilates</t>
+          <t>IFA / wealth management</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -35007,7 +35723,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Aesthetics &amp; skin clinic</t>
+          <t>Physiotherapy &amp; clinical Pilates</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -35017,7 +35733,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>IFA / financial planning</t>
+          <t>Aesthetics &amp; skin clinic</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -35027,7 +35743,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Wealth management &amp; employee benefits</t>
+          <t>IFA / financial planning</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -35037,7 +35753,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Dermatology clinic</t>
+          <t>Wealth management &amp; employee benefits</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -35047,7 +35763,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Pilates studio (multi-site)</t>
+          <t>Dermatology clinic</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -35057,7 +35773,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Private nursery (Montessori, multi-site)</t>
+          <t>Pilates studio (multi-site)</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -35067,7 +35783,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Law firm (wills &amp; probate)</t>
+          <t>Private nursery (Montessori, multi-site)</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -35077,7 +35793,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Business/technical consultancy</t>
+          <t>Law firm (wills &amp; probate)</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -35087,7 +35803,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Private/NHS dentist</t>
+          <t>Business/technical consultancy</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -35097,7 +35813,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Removals company</t>
+          <t>Private/NHS dentist</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -35107,7 +35823,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Driveways &amp; landscaping</t>
+          <t>Removals company</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -35117,7 +35833,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Wedding &amp; event venue</t>
+          <t>Driveways &amp; landscaping</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -35127,7 +35843,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>IFA &amp; mortgage broker</t>
+          <t>Wedding &amp; event venue</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -35137,7 +35853,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Wedding photography &amp; videography</t>
+          <t>IFA &amp; mortgage broker</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -35147,7 +35863,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Commercial property litigation law firm</t>
+          <t>Wedding photography &amp; videography</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -35157,7 +35873,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Recruitment agency (boutique)</t>
+          <t>Commercial property litigation law firm</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -35167,7 +35883,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Home cinema &amp; smart home installer</t>
+          <t>Recruitment agency (boutique)</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -35177,7 +35893,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Home cinema installer</t>
+          <t>Home cinema &amp; smart home installer</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -35187,7 +35903,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Curtains, blinds &amp; upholstery</t>
+          <t>Home cinema installer</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -35197,7 +35913,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Bespoke curtains &amp; soft furnishings</t>
+          <t>Curtains, blinds &amp; upholstery</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -35207,7 +35923,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Wine merchant</t>
+          <t>Bespoke curtains &amp; soft furnishings</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -35217,7 +35933,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Education consultancy (school placement)</t>
+          <t>Wine merchant</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -35227,7 +35943,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Estate agent &amp; surveyors</t>
+          <t>Education consultancy (school placement)</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -35237,7 +35953,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Independent financial adviser</t>
+          <t>Estate agent &amp; surveyors</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -35247,7 +35963,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Chartered accountants &amp; financial planners</t>
+          <t>Independent financial adviser</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -35257,7 +35973,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Private GP &amp; dermatology</t>
+          <t>Chartered accountants &amp; financial planners</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -35267,7 +35983,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Architects (heritage specialism)</t>
+          <t>Private GP &amp; dermatology</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -35277,7 +35993,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Private cosmetic dentist / implants</t>
+          <t>Architects (heritage specialism)</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -35287,7 +36003,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Heating engineer / plumbing</t>
+          <t>Private cosmetic dentist / implants</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -35297,7 +36013,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Estate agent (boutique)</t>
+          <t>Heating engineer / plumbing</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -35307,7 +36023,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Independent vet (mixed practice)</t>
+          <t>Estate agent (boutique)</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -35317,7 +36033,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Private dentist / cosmetic</t>
+          <t>Independent vet (mixed practice)</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -35327,10 +36043,80 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
+          <t>Private dentist / cosmetic</t>
+        </is>
+      </c>
+      <c r="B143" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
           <t>Chartered accountants &amp; financial advisers</t>
         </is>
       </c>
-      <c r="B143" t="n">
+      <c r="B144" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Healthcare recruitment agency</t>
+        </is>
+      </c>
+      <c r="B145" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Executive search / headhunting</t>
+        </is>
+      </c>
+      <c r="B146" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>First aid &amp; health &amp; safety training</t>
+        </is>
+      </c>
+      <c r="B147" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Teaching &amp; education recruitment agency</t>
+        </is>
+      </c>
+      <c r="B148" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Supply teaching agency</t>
+        </is>
+      </c>
+      <c r="B149" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Hospitality staffing agency</t>
+        </is>
+      </c>
+      <c r="B150" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 37: +6 prospects (400 total) - finance/legal recruitment, forklift training
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$395</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$401</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T395"/>
+  <dimension ref="A1:T401"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -34628,8 +34628,532 @@
       </c>
       <c r="T395" s="4" t="inlineStr"/>
     </row>
+    <row r="396">
+      <c r="A396" s="3" t="inlineStr">
+        <is>
+          <t>Ashley Rees Associates</t>
+        </is>
+      </c>
+      <c r="B396" s="3" t="inlineStr">
+        <is>
+          <t>Finance &amp; accountancy recruitment agency</t>
+        </is>
+      </c>
+      <c r="C396" s="3" t="inlineStr">
+        <is>
+          <t>Henbury Road, Bristol</t>
+        </is>
+      </c>
+      <c r="D396" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ashleyreesassociates.co.uk</t>
+        </is>
+      </c>
+      <c r="E396" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F396" s="3" t="inlineStr"/>
+      <c r="G396" s="3" t="inlineStr">
+        <is>
+          <t>20-year independent South West specialist</t>
+        </is>
+      </c>
+      <c r="H396" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/p/Ashley-Rees-Associates-100070959433536</t>
+        </is>
+      </c>
+      <c r="I396" s="3" t="inlineStr"/>
+      <c r="J396" s="3" t="inlineStr">
+        <is>
+          <t>REC-member independent recruiter for finance roles across SW England; placement fees on management-accountant-to-CFO roles are substantial</t>
+        </is>
+      </c>
+      <c r="K396" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L396" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M396" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N396" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O396" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence; REC membership</t>
+        </is>
+      </c>
+      <c r="P396" s="3" t="inlineStr">
+        <is>
+          <t>Core3/national brands (Robert Walters, Morgan McKinley) dominate 'finance recruitment Bristol' search</t>
+        </is>
+      </c>
+      <c r="Q396" s="3" t="inlineStr">
+        <is>
+          <t>'20 years placing SW finance talent - own that AEO answer against the national brands'</t>
+        </is>
+      </c>
+      <c r="R396" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S396" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T396" s="3" t="inlineStr"/>
+    </row>
+    <row r="397">
+      <c r="A397" s="4" t="inlineStr">
+        <is>
+          <t>Core3</t>
+        </is>
+      </c>
+      <c r="B397" s="4" t="inlineStr">
+        <is>
+          <t>Accounting &amp; finance recruitment agency</t>
+        </is>
+      </c>
+      <c r="C397" s="4" t="inlineStr">
+        <is>
+          <t>Bristol</t>
+        </is>
+      </c>
+      <c r="D397" s="4" t="inlineStr">
+        <is>
+          <t>via directory listing</t>
+        </is>
+      </c>
+      <c r="E397" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F397" s="4" t="inlineStr"/>
+      <c r="G397" s="4" t="inlineStr"/>
+      <c r="H397" s="4" t="inlineStr"/>
+      <c r="I397" s="4" t="inlineStr"/>
+      <c r="J397" s="4" t="inlineStr">
+        <is>
+          <t>Bristol-headquartered specialist covering management accountants through to CFO placements</t>
+        </is>
+      </c>
+      <c r="K397" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L397" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M397" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N397" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O397" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P397" s="4" t="inlineStr">
+        <is>
+          <t>Same national-brand squeeze as other Bristol finance recruiters</t>
+        </is>
+      </c>
+      <c r="Q397" s="4" t="inlineStr">
+        <is>
+          <t>Own a specific finance sub-niche (e.g. CFO/interim finance) in AEO content</t>
+        </is>
+      </c>
+      <c r="R397" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S397" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T397" s="4" t="inlineStr">
+        <is>
+          <t>Confirm live website before outreach</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" s="3" t="inlineStr">
+        <is>
+          <t>HL Training Services</t>
+        </is>
+      </c>
+      <c r="B398" s="3" t="inlineStr">
+        <is>
+          <t>Forklift &amp; plant operator training</t>
+        </is>
+      </c>
+      <c r="C398" s="3" t="inlineStr">
+        <is>
+          <t>Barton Hill, Bristol</t>
+        </is>
+      </c>
+      <c r="D398" s="3" t="inlineStr">
+        <is>
+          <t>https://www.hltraining.co.uk</t>
+        </is>
+      </c>
+      <c r="E398" s="3" t="inlineStr">
+        <is>
+          <t>sales@hltraining.co.uk</t>
+        </is>
+      </c>
+      <c r="F398" s="3" t="inlineStr">
+        <is>
+          <t>0117 952 5625</t>
+        </is>
+      </c>
+      <c r="G398" s="3" t="inlineStr">
+        <is>
+          <t>Vince Hueston Jr &amp; Angela Hueston (Family, est. 1988)</t>
+        </is>
+      </c>
+      <c r="H398" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/hl-training-services</t>
+        </is>
+      </c>
+      <c r="I398" s="3" t="inlineStr"/>
+      <c r="J398" s="3" t="inlineStr">
+        <is>
+          <t>37-year family business delivering RTITB/ITSSAR-accredited forklift and plant training on-site across the South West; corporate H&amp;S contracts recur</t>
+        </is>
+      </c>
+      <c r="K398" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L398" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M398" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N398" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O398" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn presence; long trading history</t>
+        </is>
+      </c>
+      <c r="P398" s="3" t="inlineStr">
+        <is>
+          <t>National forklift-training franchises (Wallace School, Pegasus) outspend on generic 'forklift training Bristol' search</t>
+        </is>
+      </c>
+      <c r="Q398" s="3" t="inlineStr">
+        <is>
+          <t>'37 years training Bristol's forklift operators - own that AEO trust signal against national franchises'</t>
+        </is>
+      </c>
+      <c r="R398" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S398" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T398" s="3" t="inlineStr"/>
+    </row>
+    <row r="399">
+      <c r="A399" s="3" t="inlineStr">
+        <is>
+          <t>Cuff Jones</t>
+        </is>
+      </c>
+      <c r="B399" s="3" t="inlineStr">
+        <is>
+          <t>Legal recruitment agency</t>
+        </is>
+      </c>
+      <c r="C399" s="3" t="inlineStr">
+        <is>
+          <t>Clerkenwell, London</t>
+        </is>
+      </c>
+      <c r="D399" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cuffjones.co.uk</t>
+        </is>
+      </c>
+      <c r="E399" s="3" t="inlineStr">
+        <is>
+          <t>steph@cuffjones.com</t>
+        </is>
+      </c>
+      <c r="F399" s="3" t="inlineStr"/>
+      <c r="G399" s="3" t="inlineStr">
+        <is>
+          <t>Jonathan Cuff (Director, est. 2010)</t>
+        </is>
+      </c>
+      <c r="H399" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/jonathancuff1</t>
+        </is>
+      </c>
+      <c r="I399" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/p/Cuff-Jones-Expert-Legal-Recruitment-100076873250336</t>
+        </is>
+      </c>
+      <c r="J399" s="3" t="inlineStr">
+        <is>
+          <t>Boutique legal recruiter to top law firms globally; single senior-solicitor placement fees run into tens of thousands</t>
+        </is>
+      </c>
+      <c r="K399" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L399" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M399" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N399" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O399" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence; international client base</t>
+        </is>
+      </c>
+      <c r="P399" s="3" t="inlineStr">
+        <is>
+          <t>Boutique positioning invisible against Taylor Root/SSQ/Robert Walters in generic legal-recruitment search</t>
+        </is>
+      </c>
+      <c r="Q399" s="3" t="inlineStr">
+        <is>
+          <t>'Dedicated, personable legal recruitment vs a corporate agency conveyor belt - own that AEO positioning'</t>
+        </is>
+      </c>
+      <c r="R399" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S399" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T399" s="3" t="inlineStr"/>
+    </row>
+    <row r="400">
+      <c r="A400" s="4" t="inlineStr">
+        <is>
+          <t>EJ Legal</t>
+        </is>
+      </c>
+      <c r="B400" s="4" t="inlineStr">
+        <is>
+          <t>Legal recruitment agency</t>
+        </is>
+      </c>
+      <c r="C400" s="4" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D400" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ejlegal.co.uk</t>
+        </is>
+      </c>
+      <c r="E400" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F400" s="4" t="inlineStr"/>
+      <c r="G400" s="4" t="inlineStr"/>
+      <c r="H400" s="4" t="inlineStr"/>
+      <c r="I400" s="4" t="inlineStr"/>
+      <c r="J400" s="4" t="inlineStr">
+        <is>
+          <t>London legal recruitment specialist placing solicitors/paralegals into law firms</t>
+        </is>
+      </c>
+      <c r="K400" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L400" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M400" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N400" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O400" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P400" s="4" t="inlineStr">
+        <is>
+          <t>Crowded London legal-recruitment market with many similarly-positioned boutiques</t>
+        </is>
+      </c>
+      <c r="Q400" s="4" t="inlineStr">
+        <is>
+          <t>Own a specific legal practice-area niche (e.g. private client, litigation) in AEO content</t>
+        </is>
+      </c>
+      <c r="R400" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S400" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T400" s="4" t="inlineStr">
+        <is>
+          <t>Confirm live website before outreach</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" s="4" t="inlineStr">
+        <is>
+          <t>Pegasus Lift Truck Training</t>
+        </is>
+      </c>
+      <c r="B401" s="4" t="inlineStr">
+        <is>
+          <t>Forklift training</t>
+        </is>
+      </c>
+      <c r="C401" s="4" t="inlineStr">
+        <is>
+          <t>UK-wide (on-site delivery)</t>
+        </is>
+      </c>
+      <c r="D401" s="4" t="inlineStr">
+        <is>
+          <t>https://pegasuslifttrucktraining.co.uk</t>
+        </is>
+      </c>
+      <c r="E401" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F401" s="4" t="inlineStr"/>
+      <c r="G401" s="4" t="inlineStr">
+        <is>
+          <t>Dawn &amp; Giuseppe Girardi (Founders, 25+ yrs experience)</t>
+        </is>
+      </c>
+      <c r="H401" s="4" t="inlineStr"/>
+      <c r="I401" s="4" t="inlineStr"/>
+      <c r="J401" s="4" t="inlineStr">
+        <is>
+          <t>ITSSAR-accredited nationwide on-site training; corporate clients need repeat annual certification renewals</t>
+        </is>
+      </c>
+      <c r="K401" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L401" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M401" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N401" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O401" s="4" t="inlineStr">
+        <is>
+          <t>25-year trading history</t>
+        </is>
+      </c>
+      <c r="P401" s="4" t="inlineStr">
+        <is>
+          <t>National reach means competing with many similarly-positioned forklift trainers for the same generic searches</t>
+        </is>
+      </c>
+      <c r="Q401" s="4" t="inlineStr">
+        <is>
+          <t>'25 years of ITSSAR-accredited training - own the AEO answer for corporate renewal searches'</t>
+        </is>
+      </c>
+      <c r="R401" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S401" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T401" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T395"/>
+  <autoFilter ref="A1:T401"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -34640,7 +35164,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B150"/>
+  <dimension ref="A1:B155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -34660,7 +35184,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>394</v>
+        <v>400</v>
       </c>
     </row>
     <row r="5">
@@ -35123,17 +35647,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Dentist / Orthodontics</t>
+          <t>Legal recruitment agency</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Specialist dental/implant clinic</t>
+          <t>Dentist / Orthodontics</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -35143,7 +35667,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Boutique corporate law firm</t>
+          <t>Specialist dental/implant clinic</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -35153,7 +35677,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Cosmetic/aesthetics clinic</t>
+          <t>Boutique corporate law firm</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -35163,7 +35687,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Skin &amp; laser clinic</t>
+          <t>Cosmetic/aesthetics clinic</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -35173,7 +35697,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Mortgage broker / financial adviser</t>
+          <t>Skin &amp; laser clinic</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -35183,7 +35707,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Architects (RIBA chartered)</t>
+          <t>Mortgage broker / financial adviser</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -35193,7 +35717,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Recruitment agency (tech/startups)</t>
+          <t>Architects (RIBA chartered)</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -35203,7 +35727,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Recruitment agency (IT/data)</t>
+          <t>Recruitment agency (tech/startups)</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -35213,7 +35737,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Independent vet (24/7 emergency)</t>
+          <t>Recruitment agency (IT/data)</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -35223,7 +35747,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Interior design studio</t>
+          <t>Independent vet (24/7 emergency)</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -35233,7 +35757,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Letting &amp; estate agent</t>
+          <t>Interior design studio</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -35243,7 +35767,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Cosmetic clinic (injectables)</t>
+          <t>Letting &amp; estate agent</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -35253,7 +35777,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Cosmetic/anti-ageing clinic</t>
+          <t>Cosmetic clinic (injectables)</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -35263,7 +35787,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Yoga &amp; reformer pilates studio</t>
+          <t>Cosmetic/anti-ageing clinic</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -35273,7 +35797,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Reformer pilates studio</t>
+          <t>Yoga &amp; reformer pilates studio</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -35283,7 +35807,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Wealth management</t>
+          <t>Reformer pilates studio</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -35293,7 +35817,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Private tuition &amp; education consultancy</t>
+          <t>Wealth management</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -35303,7 +35827,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Osteopath</t>
+          <t>Private tuition &amp; education consultancy</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -35313,7 +35837,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Design &amp; build / home renovation</t>
+          <t>Osteopath</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -35323,7 +35847,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Builders / building contractor</t>
+          <t>Design &amp; build / home renovation</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -35333,7 +35857,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Home care / live-in care</t>
+          <t>Builders / building contractor</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -35343,7 +35867,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Private day nurseries</t>
+          <t>Home care / live-in care</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -35353,7 +35877,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Personal training &amp; wellness studio</t>
+          <t>Private day nurseries</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -35363,7 +35887,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Mortgage &amp; insurance broker</t>
+          <t>Personal training &amp; wellness studio</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -35373,7 +35897,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Business consultancy</t>
+          <t>Mortgage &amp; insurance broker</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -35383,7 +35907,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Interior designer (period homes)</t>
+          <t>Business consultancy</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -35393,7 +35917,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Landscape design &amp; build</t>
+          <t>Interior designer (period homes)</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -35403,7 +35927,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Interior designer</t>
+          <t>Landscape design &amp; build</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -35413,7 +35937,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Garden design &amp; landscaping</t>
+          <t>Interior designer</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -35423,7 +35947,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Legal recruitment</t>
+          <t>Garden design &amp; landscaping</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -35433,7 +35957,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Independent gym &amp; health club</t>
+          <t>Legal recruitment</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -35443,7 +35967,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Independent gym</t>
+          <t>Independent gym &amp; health club</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -35453,7 +35977,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Physiotherapy (sports)</t>
+          <t>Independent gym</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -35463,7 +35987,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Letting agent / property management</t>
+          <t>Physiotherapy (sports)</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -35473,7 +35997,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Skin clinic</t>
+          <t>Letting agent / property management</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -35483,7 +36007,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Tutoring company</t>
+          <t>Skin clinic</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -35493,7 +36017,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Tutorial college &amp; exam centre</t>
+          <t>Tutoring company</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -35503,7 +36027,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Employment law (disability discrimination)</t>
+          <t>Tutorial college &amp; exam centre</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -35513,7 +36037,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating</t>
+          <t>Employment law (disability discrimination)</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -35523,7 +36047,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Plumbing &amp; heating</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -35533,7 +36057,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Sports physio &amp; massage</t>
+          <t>Plumbing</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -35543,7 +36067,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Chartered surveyors (party wall/building)</t>
+          <t>Sports physio &amp; massage</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -35553,7 +36077,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Chartered surveyors</t>
+          <t>Chartered surveyors (party wall/building)</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -35563,7 +36087,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Chartered building surveyors</t>
+          <t>Chartered surveyors</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -35573,7 +36097,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Osteopathy clinics</t>
+          <t>Chartered building surveyors</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -35583,7 +36107,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Builders / renovations</t>
+          <t>Osteopathy clinics</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -35593,7 +36117,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Private nursery schools</t>
+          <t>Builders / renovations</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -35603,7 +36127,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Private day nursery</t>
+          <t>Private nursery schools</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -35613,7 +36137,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Private GP (membership model)</t>
+          <t>Private day nursery</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -35623,7 +36147,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Sash window restoration</t>
+          <t>Private GP (membership model)</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -35633,7 +36157,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Personal training (1:1)</t>
+          <t>Sash window restoration</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -35643,7 +36167,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Personal training &amp; nutrition coaching</t>
+          <t>Personal training (1:1)</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -35653,7 +36177,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Private nursery/pre-prep school</t>
+          <t>Personal training &amp; nutrition coaching</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -35663,7 +36187,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Independent nursery (Montessori)</t>
+          <t>Private nursery/pre-prep school</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -35673,7 +36197,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Live-in care agency</t>
+          <t>Independent nursery (Montessori)</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -35683,7 +36207,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Law firm (conveyancing/family)</t>
+          <t>Live-in care agency</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -35693,7 +36217,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Architect &amp; interior designer</t>
+          <t>Law firm (conveyancing/family)</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -35703,7 +36227,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Architects / project management</t>
+          <t>Architect &amp; interior designer</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -35713,7 +36237,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>IFA / wealth management</t>
+          <t>Architects / project management</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -35723,7 +36247,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Physiotherapy &amp; clinical Pilates</t>
+          <t>IFA / wealth management</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -35733,7 +36257,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Aesthetics &amp; skin clinic</t>
+          <t>Physiotherapy &amp; clinical Pilates</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -35743,7 +36267,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>IFA / financial planning</t>
+          <t>Aesthetics &amp; skin clinic</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -35753,7 +36277,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Wealth management &amp; employee benefits</t>
+          <t>IFA / financial planning</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -35763,7 +36287,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Dermatology clinic</t>
+          <t>Wealth management &amp; employee benefits</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -35773,7 +36297,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Pilates studio (multi-site)</t>
+          <t>Dermatology clinic</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -35783,7 +36307,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Private nursery (Montessori, multi-site)</t>
+          <t>Pilates studio (multi-site)</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -35793,7 +36317,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Law firm (wills &amp; probate)</t>
+          <t>Private nursery (Montessori, multi-site)</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -35803,7 +36327,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Business/technical consultancy</t>
+          <t>Law firm (wills &amp; probate)</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -35813,7 +36337,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Private/NHS dentist</t>
+          <t>Business/technical consultancy</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -35823,7 +36347,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Removals company</t>
+          <t>Private/NHS dentist</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -35833,7 +36357,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Driveways &amp; landscaping</t>
+          <t>Removals company</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -35843,7 +36367,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Wedding &amp; event venue</t>
+          <t>Driveways &amp; landscaping</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -35853,7 +36377,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>IFA &amp; mortgage broker</t>
+          <t>Wedding &amp; event venue</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -35863,7 +36387,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Wedding photography &amp; videography</t>
+          <t>IFA &amp; mortgage broker</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -35873,7 +36397,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Commercial property litigation law firm</t>
+          <t>Wedding photography &amp; videography</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -35883,7 +36407,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Recruitment agency (boutique)</t>
+          <t>Commercial property litigation law firm</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -35893,7 +36417,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Home cinema &amp; smart home installer</t>
+          <t>Recruitment agency (boutique)</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -35903,7 +36427,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Home cinema installer</t>
+          <t>Home cinema &amp; smart home installer</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -35913,7 +36437,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Curtains, blinds &amp; upholstery</t>
+          <t>Home cinema installer</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -35923,7 +36447,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Bespoke curtains &amp; soft furnishings</t>
+          <t>Curtains, blinds &amp; upholstery</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -35933,7 +36457,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Wine merchant</t>
+          <t>Bespoke curtains &amp; soft furnishings</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -35943,7 +36467,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Education consultancy (school placement)</t>
+          <t>Wine merchant</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -35953,7 +36477,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Estate agent &amp; surveyors</t>
+          <t>Education consultancy (school placement)</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -35963,7 +36487,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Independent financial adviser</t>
+          <t>Estate agent &amp; surveyors</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -35973,7 +36497,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Chartered accountants &amp; financial planners</t>
+          <t>Independent financial adviser</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -35983,7 +36507,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Private GP &amp; dermatology</t>
+          <t>Chartered accountants &amp; financial planners</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -35993,7 +36517,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Architects (heritage specialism)</t>
+          <t>Private GP &amp; dermatology</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -36003,7 +36527,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Private cosmetic dentist / implants</t>
+          <t>Architects (heritage specialism)</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -36013,7 +36537,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Heating engineer / plumbing</t>
+          <t>Private cosmetic dentist / implants</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -36023,7 +36547,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Estate agent (boutique)</t>
+          <t>Heating engineer / plumbing</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -36033,7 +36557,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Independent vet (mixed practice)</t>
+          <t>Estate agent (boutique)</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -36043,7 +36567,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Private dentist / cosmetic</t>
+          <t>Independent vet (mixed practice)</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -36053,7 +36577,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Chartered accountants &amp; financial advisers</t>
+          <t>Private dentist / cosmetic</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -36063,7 +36587,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Healthcare recruitment agency</t>
+          <t>Chartered accountants &amp; financial advisers</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -36073,7 +36597,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Executive search / headhunting</t>
+          <t>Healthcare recruitment agency</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -36083,7 +36607,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>First aid &amp; health &amp; safety training</t>
+          <t>Executive search / headhunting</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -36093,7 +36617,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Teaching &amp; education recruitment agency</t>
+          <t>First aid &amp; health &amp; safety training</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -36103,7 +36627,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Supply teaching agency</t>
+          <t>Teaching &amp; education recruitment agency</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -36113,10 +36637,60 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
+          <t>Supply teaching agency</t>
+        </is>
+      </c>
+      <c r="B150" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
           <t>Hospitality staffing agency</t>
         </is>
       </c>
-      <c r="B150" t="n">
+      <c r="B151" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Finance &amp; accountancy recruitment agency</t>
+        </is>
+      </c>
+      <c r="B152" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Accounting &amp; finance recruitment agency</t>
+        </is>
+      </c>
+      <c r="B153" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Forklift &amp; plant operator training</t>
+        </is>
+      </c>
+      <c r="B154" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Forklift training</t>
+        </is>
+      </c>
+      <c r="B155" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 38: +6 prospects (406 total) - language school, engineering recruitment, coaching, HGV training
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$401</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$407</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T401"/>
+  <dimension ref="A1:T407"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -35152,8 +35152,540 @@
       </c>
       <c r="T401" s="4" t="inlineStr"/>
     </row>
+    <row r="402">
+      <c r="A402" s="3" t="inlineStr">
+        <is>
+          <t>Lewis School of English</t>
+        </is>
+      </c>
+      <c r="B402" s="3" t="inlineStr">
+        <is>
+          <t>Language school</t>
+        </is>
+      </c>
+      <c r="C402" s="3" t="inlineStr">
+        <is>
+          <t>Southampton (+ juniors/online)</t>
+        </is>
+      </c>
+      <c r="D402" s="3" t="inlineStr">
+        <is>
+          <t>https://lewis-school.co.uk</t>
+        </is>
+      </c>
+      <c r="E402" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F402" s="3" t="inlineStr">
+        <is>
+          <t>023 8022 8203</t>
+        </is>
+      </c>
+      <c r="G402" s="3" t="inlineStr">
+        <is>
+          <t>Alistair Walker MA (Director); est. 1976, 50th anniversary 2026</t>
+        </is>
+      </c>
+      <c r="H402" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/lewisschool</t>
+        </is>
+      </c>
+      <c r="I402" s="3" t="inlineStr"/>
+      <c r="J402" s="3" t="inlineStr">
+        <is>
+          <t>50-year independent language school; international students pay per-course/term fees, high LTV per enrolment</t>
+        </is>
+      </c>
+      <c r="K402" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L402" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M402" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N402" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O402" s="3" t="inlineStr">
+        <is>
+          <t>Established multi-decade brand; LinkedIn presence</t>
+        </is>
+      </c>
+      <c r="P402" s="3" t="inlineStr">
+        <is>
+          <t>50th-anniversary milestone is a strong AEO/PR hook not yet leveraged for AI-search visibility</t>
+        </is>
+      </c>
+      <c r="Q402" s="3" t="inlineStr">
+        <is>
+          <t>'Celebrating 50 years - turn the anniversary into the AI-cited answer for English language schools in the UK'</t>
+        </is>
+      </c>
+      <c r="R402" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S402" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T402" s="3" t="inlineStr"/>
+    </row>
+    <row r="403">
+      <c r="A403" s="3" t="inlineStr">
+        <is>
+          <t>Sigma Recruitment</t>
+        </is>
+      </c>
+      <c r="B403" s="3" t="inlineStr">
+        <is>
+          <t>Engineering &amp; manufacturing recruitment</t>
+        </is>
+      </c>
+      <c r="C403" s="3" t="inlineStr">
+        <is>
+          <t>Cardiff (serves Bristol/Bath/South West)</t>
+        </is>
+      </c>
+      <c r="D403" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sigmarecruitment.co.uk</t>
+        </is>
+      </c>
+      <c r="E403" s="3" t="inlineStr">
+        <is>
+          <t>rhys@sigmarecruitment.co.uk</t>
+        </is>
+      </c>
+      <c r="F403" s="3" t="inlineStr">
+        <is>
+          <t>029 2010 0790</t>
+        </is>
+      </c>
+      <c r="G403" s="3" t="inlineStr">
+        <is>
+          <t>Rhys Williams (Founder, est. 2005)</t>
+        </is>
+      </c>
+      <c r="H403" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/rhyswilliamsigma</t>
+        </is>
+      </c>
+      <c r="I403" s="3" t="inlineStr"/>
+      <c r="J403" s="3" t="inlineStr">
+        <is>
+          <t>20-year independent engineering recruiter with a dedicated Bristol-market landing page - active SEO investment reaching into the South West despite a Cardiff HQ</t>
+        </is>
+      </c>
+      <c r="K403" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L403" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M403" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N403" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O403" s="3" t="inlineStr">
+        <is>
+          <t>Dedicated Bristol/Bath location landing pages = active SEO</t>
+        </is>
+      </c>
+      <c r="P403" s="3" t="inlineStr">
+        <is>
+          <t>Bristol landing page exists but AI-answer citations for 'engineering recruitment Bristol' still open</t>
+        </is>
+      </c>
+      <c r="Q403" s="3" t="inlineStr">
+        <is>
+          <t>'You built the Bristol page - let's make sure AI cites it, not just Google'</t>
+        </is>
+      </c>
+      <c r="R403" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S403" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T403" s="3" t="inlineStr">
+        <is>
+          <t>HQ is Cardiff; targets Bristol/Bath market via dedicated pages</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="3" t="inlineStr">
+        <is>
+          <t>Kieran Perry</t>
+        </is>
+      </c>
+      <c r="B404" s="3" t="inlineStr">
+        <is>
+          <t>Business &amp; sales coaching</t>
+        </is>
+      </c>
+      <c r="C404" s="3" t="inlineStr">
+        <is>
+          <t>Sandbach/London (serves UK-wide)</t>
+        </is>
+      </c>
+      <c r="D404" s="3" t="inlineStr">
+        <is>
+          <t>https://www.kieranperry.com</t>
+        </is>
+      </c>
+      <c r="E404" s="3" t="inlineStr">
+        <is>
+          <t>info@kieranperry.com</t>
+        </is>
+      </c>
+      <c r="F404" s="3" t="inlineStr">
+        <is>
+          <t>07912 846 492</t>
+        </is>
+      </c>
+      <c r="G404" s="3" t="inlineStr">
+        <is>
+          <t>Kieran Perry (Founder, 25+ yrs experience)</t>
+        </is>
+      </c>
+      <c r="H404" s="3" t="inlineStr"/>
+      <c r="I404" s="3" t="inlineStr"/>
+      <c r="J404" s="3" t="inlineStr">
+        <is>
+          <t>Solo executive/sales coach with published book and blog-driven content strategy; corporate coaching retainers worth thousands per client</t>
+        </is>
+      </c>
+      <c r="K404" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L404" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M404" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N404" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O404" s="3" t="inlineStr">
+        <is>
+          <t>Extensive blog/SEO content across many coaching topics = active SEO investment</t>
+        </is>
+      </c>
+      <c r="P404" s="3" t="inlineStr">
+        <is>
+          <t>Large content library exists but AI-answer citations for specific coaching queries still open</t>
+        </is>
+      </c>
+      <c r="Q404" s="3" t="inlineStr">
+        <is>
+          <t>'You've written the definitive guides - let's make AI cite them, not just index them'</t>
+        </is>
+      </c>
+      <c r="R404" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S404" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T404" s="3" t="inlineStr"/>
+    </row>
+    <row r="405">
+      <c r="A405" s="4" t="inlineStr">
+        <is>
+          <t>Nolan Recruitment</t>
+        </is>
+      </c>
+      <c r="B405" s="4" t="inlineStr">
+        <is>
+          <t>Engineering &amp; energy recruitment</t>
+        </is>
+      </c>
+      <c r="C405" s="4" t="inlineStr">
+        <is>
+          <t>UK-wide</t>
+        </is>
+      </c>
+      <c r="D405" s="4" t="inlineStr">
+        <is>
+          <t>https://www.nolanrecruitment.com</t>
+        </is>
+      </c>
+      <c r="E405" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F405" s="4" t="inlineStr"/>
+      <c r="G405" s="4" t="inlineStr">
+        <is>
+          <t>Sean Neary (Managing Director, est. 2016)</t>
+        </is>
+      </c>
+      <c r="H405" s="4" t="inlineStr"/>
+      <c r="I405" s="4" t="inlineStr"/>
+      <c r="J405" s="4" t="inlineStr">
+        <is>
+          <t>Independent specialist in engineering/energy sector placements since 2016; high-value technical placements</t>
+        </is>
+      </c>
+      <c r="K405" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L405" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M405" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N405" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O405" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P405" s="4" t="inlineStr">
+        <is>
+          <t>Crowded engineering-recruitment market with many similarly-positioned independents</t>
+        </is>
+      </c>
+      <c r="Q405" s="4" t="inlineStr">
+        <is>
+          <t>Own a specific energy-sector sub-niche in AEO content vs generalist engineering recruiters</t>
+        </is>
+      </c>
+      <c r="R405" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S405" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T405" s="4" t="inlineStr"/>
+    </row>
+    <row r="406">
+      <c r="A406" s="3" t="inlineStr">
+        <is>
+          <t>Hughes Driver Training</t>
+        </is>
+      </c>
+      <c r="B406" s="3" t="inlineStr">
+        <is>
+          <t>HGV driver training</t>
+        </is>
+      </c>
+      <c r="C406" s="3" t="inlineStr">
+        <is>
+          <t>Leicester (nationwide delivery)</t>
+        </is>
+      </c>
+      <c r="D406" s="3" t="inlineStr">
+        <is>
+          <t>https://www.hughesdrivertraining.co.uk</t>
+        </is>
+      </c>
+      <c r="E406" s="3" t="inlineStr">
+        <is>
+          <t>info@hughesdrivertraining.co.uk</t>
+        </is>
+      </c>
+      <c r="F406" s="3" t="inlineStr">
+        <is>
+          <t>0800 177 7447</t>
+        </is>
+      </c>
+      <c r="G406" s="3" t="inlineStr">
+        <is>
+          <t>Bill Hughes (Founder); now 3rd generation family-run</t>
+        </is>
+      </c>
+      <c r="H406" s="3" t="inlineStr"/>
+      <c r="I406" s="3" t="inlineStr"/>
+      <c r="J406" s="3" t="inlineStr">
+        <is>
+          <t>Multi-generation family HGV training business; logistics firms need repeat driver certification and CPC training</t>
+        </is>
+      </c>
+      <c r="K406" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L406" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M406" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N406" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O406" s="3" t="inlineStr">
+        <is>
+          <t>Family-story branding ('Our Story' page)</t>
+        </is>
+      </c>
+      <c r="P406" s="3" t="inlineStr">
+        <is>
+          <t>3-generation family story is a strong AEO trust asset not yet leveraged against national franchises</t>
+        </is>
+      </c>
+      <c r="Q406" s="3" t="inlineStr">
+        <is>
+          <t>'3 generations training HGV drivers - own that family-trust story in AI answers'</t>
+        </is>
+      </c>
+      <c r="R406" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S406" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T406" s="3" t="inlineStr"/>
+    </row>
+    <row r="407">
+      <c r="A407" s="4" t="inlineStr">
+        <is>
+          <t>Hartlip HGV Driving School</t>
+        </is>
+      </c>
+      <c r="B407" s="4" t="inlineStr">
+        <is>
+          <t>HGV driver training</t>
+        </is>
+      </c>
+      <c r="C407" s="4" t="inlineStr">
+        <is>
+          <t>Kent</t>
+        </is>
+      </c>
+      <c r="D407" s="4" t="inlineStr">
+        <is>
+          <t>https://www.hartliphgv.co.uk</t>
+        </is>
+      </c>
+      <c r="E407" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F407" s="4" t="inlineStr"/>
+      <c r="G407" s="4" t="inlineStr">
+        <is>
+          <t>Family-run</t>
+        </is>
+      </c>
+      <c r="H407" s="4" t="inlineStr"/>
+      <c r="I407" s="4" t="inlineStr"/>
+      <c r="J407" s="4" t="inlineStr">
+        <is>
+          <t>Independent family-run HGV school in Kent; affordable, tailored training for career-changers and logistics firms</t>
+        </is>
+      </c>
+      <c r="K407" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L407" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M407" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N407" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O407" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P407" s="4" t="inlineStr">
+        <is>
+          <t>National HGV training brands with bigger ad budgets dominate generic 'HGV training Kent' search</t>
+        </is>
+      </c>
+      <c r="Q407" s="4" t="inlineStr">
+        <is>
+          <t>'Family-run and affordable' - own that exact AEO positioning vs national franchises</t>
+        </is>
+      </c>
+      <c r="R407" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S407" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T407" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T401"/>
+  <autoFilter ref="A1:T407"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -35164,7 +35696,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B155"/>
+  <dimension ref="A1:B160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -35184,7 +35716,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>400</v>
+        <v>406</v>
       </c>
     </row>
     <row r="5">
@@ -35657,17 +36189,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Dentist / Orthodontics</t>
+          <t>HGV driver training</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Specialist dental/implant clinic</t>
+          <t>Dentist / Orthodontics</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -35677,7 +36209,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Boutique corporate law firm</t>
+          <t>Specialist dental/implant clinic</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -35687,7 +36219,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Cosmetic/aesthetics clinic</t>
+          <t>Boutique corporate law firm</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -35697,7 +36229,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Skin &amp; laser clinic</t>
+          <t>Cosmetic/aesthetics clinic</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -35707,7 +36239,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Mortgage broker / financial adviser</t>
+          <t>Skin &amp; laser clinic</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -35717,7 +36249,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Architects (RIBA chartered)</t>
+          <t>Mortgage broker / financial adviser</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -35727,7 +36259,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Recruitment agency (tech/startups)</t>
+          <t>Architects (RIBA chartered)</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -35737,7 +36269,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Recruitment agency (IT/data)</t>
+          <t>Recruitment agency (tech/startups)</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -35747,7 +36279,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Independent vet (24/7 emergency)</t>
+          <t>Recruitment agency (IT/data)</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -35757,7 +36289,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Interior design studio</t>
+          <t>Independent vet (24/7 emergency)</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -35767,7 +36299,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Letting &amp; estate agent</t>
+          <t>Interior design studio</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -35777,7 +36309,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Cosmetic clinic (injectables)</t>
+          <t>Letting &amp; estate agent</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -35787,7 +36319,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Cosmetic/anti-ageing clinic</t>
+          <t>Cosmetic clinic (injectables)</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -35797,7 +36329,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Yoga &amp; reformer pilates studio</t>
+          <t>Cosmetic/anti-ageing clinic</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -35807,7 +36339,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Reformer pilates studio</t>
+          <t>Yoga &amp; reformer pilates studio</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -35817,7 +36349,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Wealth management</t>
+          <t>Reformer pilates studio</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -35827,7 +36359,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Private tuition &amp; education consultancy</t>
+          <t>Wealth management</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -35837,7 +36369,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Osteopath</t>
+          <t>Private tuition &amp; education consultancy</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -35847,7 +36379,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Design &amp; build / home renovation</t>
+          <t>Osteopath</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -35857,7 +36389,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Builders / building contractor</t>
+          <t>Design &amp; build / home renovation</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -35867,7 +36399,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Home care / live-in care</t>
+          <t>Builders / building contractor</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -35877,7 +36409,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Private day nurseries</t>
+          <t>Home care / live-in care</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -35887,7 +36419,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Personal training &amp; wellness studio</t>
+          <t>Private day nurseries</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -35897,7 +36429,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Mortgage &amp; insurance broker</t>
+          <t>Personal training &amp; wellness studio</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -35907,7 +36439,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Business consultancy</t>
+          <t>Mortgage &amp; insurance broker</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -35917,7 +36449,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Interior designer (period homes)</t>
+          <t>Business consultancy</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -35927,7 +36459,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Landscape design &amp; build</t>
+          <t>Interior designer (period homes)</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -35937,7 +36469,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Interior designer</t>
+          <t>Landscape design &amp; build</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -35947,7 +36479,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Garden design &amp; landscaping</t>
+          <t>Interior designer</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -35957,7 +36489,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Legal recruitment</t>
+          <t>Garden design &amp; landscaping</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -35967,7 +36499,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Independent gym &amp; health club</t>
+          <t>Legal recruitment</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -35977,7 +36509,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Independent gym</t>
+          <t>Independent gym &amp; health club</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -35987,7 +36519,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Physiotherapy (sports)</t>
+          <t>Independent gym</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -35997,7 +36529,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Letting agent / property management</t>
+          <t>Physiotherapy (sports)</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -36007,7 +36539,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Skin clinic</t>
+          <t>Letting agent / property management</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -36017,7 +36549,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Tutoring company</t>
+          <t>Skin clinic</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -36027,7 +36559,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Tutorial college &amp; exam centre</t>
+          <t>Tutoring company</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -36037,7 +36569,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Employment law (disability discrimination)</t>
+          <t>Tutorial college &amp; exam centre</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -36047,7 +36579,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating</t>
+          <t>Employment law (disability discrimination)</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -36057,7 +36589,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Plumbing &amp; heating</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -36067,7 +36599,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Sports physio &amp; massage</t>
+          <t>Plumbing</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -36077,7 +36609,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Chartered surveyors (party wall/building)</t>
+          <t>Sports physio &amp; massage</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -36087,7 +36619,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Chartered surveyors</t>
+          <t>Chartered surveyors (party wall/building)</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -36097,7 +36629,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Chartered building surveyors</t>
+          <t>Chartered surveyors</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -36107,7 +36639,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Osteopathy clinics</t>
+          <t>Chartered building surveyors</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -36117,7 +36649,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Builders / renovations</t>
+          <t>Osteopathy clinics</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -36127,7 +36659,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Private nursery schools</t>
+          <t>Builders / renovations</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -36137,7 +36669,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Private day nursery</t>
+          <t>Private nursery schools</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -36147,7 +36679,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Private GP (membership model)</t>
+          <t>Private day nursery</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -36157,7 +36689,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Sash window restoration</t>
+          <t>Private GP (membership model)</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -36167,7 +36699,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Personal training (1:1)</t>
+          <t>Sash window restoration</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -36177,7 +36709,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Personal training &amp; nutrition coaching</t>
+          <t>Personal training (1:1)</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -36187,7 +36719,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Private nursery/pre-prep school</t>
+          <t>Personal training &amp; nutrition coaching</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -36197,7 +36729,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Independent nursery (Montessori)</t>
+          <t>Private nursery/pre-prep school</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -36207,7 +36739,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Live-in care agency</t>
+          <t>Independent nursery (Montessori)</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -36217,7 +36749,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Law firm (conveyancing/family)</t>
+          <t>Live-in care agency</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -36227,7 +36759,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Architect &amp; interior designer</t>
+          <t>Law firm (conveyancing/family)</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -36237,7 +36769,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Architects / project management</t>
+          <t>Architect &amp; interior designer</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -36247,7 +36779,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>IFA / wealth management</t>
+          <t>Architects / project management</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -36257,7 +36789,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Physiotherapy &amp; clinical Pilates</t>
+          <t>IFA / wealth management</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -36267,7 +36799,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Aesthetics &amp; skin clinic</t>
+          <t>Physiotherapy &amp; clinical Pilates</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -36277,7 +36809,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>IFA / financial planning</t>
+          <t>Aesthetics &amp; skin clinic</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -36287,7 +36819,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Wealth management &amp; employee benefits</t>
+          <t>IFA / financial planning</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -36297,7 +36829,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Dermatology clinic</t>
+          <t>Wealth management &amp; employee benefits</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -36307,7 +36839,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Pilates studio (multi-site)</t>
+          <t>Dermatology clinic</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -36317,7 +36849,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Private nursery (Montessori, multi-site)</t>
+          <t>Pilates studio (multi-site)</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -36327,7 +36859,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Law firm (wills &amp; probate)</t>
+          <t>Private nursery (Montessori, multi-site)</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -36337,7 +36869,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Business/technical consultancy</t>
+          <t>Law firm (wills &amp; probate)</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -36347,7 +36879,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Private/NHS dentist</t>
+          <t>Business/technical consultancy</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -36357,7 +36889,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Removals company</t>
+          <t>Private/NHS dentist</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -36367,7 +36899,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Driveways &amp; landscaping</t>
+          <t>Removals company</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -36377,7 +36909,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Wedding &amp; event venue</t>
+          <t>Driveways &amp; landscaping</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -36387,7 +36919,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>IFA &amp; mortgage broker</t>
+          <t>Wedding &amp; event venue</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -36397,7 +36929,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Wedding photography &amp; videography</t>
+          <t>IFA &amp; mortgage broker</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -36407,7 +36939,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Commercial property litigation law firm</t>
+          <t>Wedding photography &amp; videography</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -36417,7 +36949,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Recruitment agency (boutique)</t>
+          <t>Commercial property litigation law firm</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -36427,7 +36959,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Home cinema &amp; smart home installer</t>
+          <t>Recruitment agency (boutique)</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -36437,7 +36969,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Home cinema installer</t>
+          <t>Home cinema &amp; smart home installer</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -36447,7 +36979,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Curtains, blinds &amp; upholstery</t>
+          <t>Home cinema installer</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -36457,7 +36989,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Bespoke curtains &amp; soft furnishings</t>
+          <t>Curtains, blinds &amp; upholstery</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -36467,7 +36999,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Wine merchant</t>
+          <t>Bespoke curtains &amp; soft furnishings</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -36477,7 +37009,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Education consultancy (school placement)</t>
+          <t>Wine merchant</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -36487,7 +37019,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Estate agent &amp; surveyors</t>
+          <t>Education consultancy (school placement)</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -36497,7 +37029,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Independent financial adviser</t>
+          <t>Estate agent &amp; surveyors</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -36507,7 +37039,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Chartered accountants &amp; financial planners</t>
+          <t>Independent financial adviser</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -36517,7 +37049,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Private GP &amp; dermatology</t>
+          <t>Chartered accountants &amp; financial planners</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -36527,7 +37059,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Architects (heritage specialism)</t>
+          <t>Private GP &amp; dermatology</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -36537,7 +37069,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Private cosmetic dentist / implants</t>
+          <t>Architects (heritage specialism)</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -36547,7 +37079,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Heating engineer / plumbing</t>
+          <t>Private cosmetic dentist / implants</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -36557,7 +37089,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Estate agent (boutique)</t>
+          <t>Heating engineer / plumbing</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -36567,7 +37099,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Independent vet (mixed practice)</t>
+          <t>Estate agent (boutique)</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -36577,7 +37109,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Private dentist / cosmetic</t>
+          <t>Independent vet (mixed practice)</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -36587,7 +37119,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Chartered accountants &amp; financial advisers</t>
+          <t>Private dentist / cosmetic</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -36597,7 +37129,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Healthcare recruitment agency</t>
+          <t>Chartered accountants &amp; financial advisers</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -36607,7 +37139,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Executive search / headhunting</t>
+          <t>Healthcare recruitment agency</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -36617,7 +37149,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>First aid &amp; health &amp; safety training</t>
+          <t>Executive search / headhunting</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -36627,7 +37159,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Teaching &amp; education recruitment agency</t>
+          <t>First aid &amp; health &amp; safety training</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -36637,7 +37169,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Supply teaching agency</t>
+          <t>Teaching &amp; education recruitment agency</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -36647,7 +37179,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Hospitality staffing agency</t>
+          <t>Supply teaching agency</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -36657,7 +37189,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Finance &amp; accountancy recruitment agency</t>
+          <t>Hospitality staffing agency</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -36667,7 +37199,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Accounting &amp; finance recruitment agency</t>
+          <t>Finance &amp; accountancy recruitment agency</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -36677,7 +37209,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Forklift &amp; plant operator training</t>
+          <t>Accounting &amp; finance recruitment agency</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -36687,10 +37219,60 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
+          <t>Forklift &amp; plant operator training</t>
+        </is>
+      </c>
+      <c r="B155" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
           <t>Forklift training</t>
         </is>
       </c>
-      <c r="B155" t="n">
+      <c r="B156" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Language school</t>
+        </is>
+      </c>
+      <c r="B157" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Engineering &amp; manufacturing recruitment</t>
+        </is>
+      </c>
+      <c r="B158" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Business &amp; sales coaching</t>
+        </is>
+      </c>
+      <c r="B159" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Engineering &amp; energy recruitment</t>
+        </is>
+      </c>
+      <c r="B160" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 39: +4 prospects (410 total) - Bristol tech recruitment, beauty training academies
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$407</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$411</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T407"/>
+  <dimension ref="A1:T411"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -35684,8 +35684,380 @@
       </c>
       <c r="T407" s="4" t="inlineStr"/>
     </row>
+    <row r="408">
+      <c r="A408" s="3" t="inlineStr">
+        <is>
+          <t>TRIA Recruitment</t>
+        </is>
+      </c>
+      <c r="B408" s="3" t="inlineStr">
+        <is>
+          <t>Tech recruitment agency</t>
+        </is>
+      </c>
+      <c r="C408" s="3" t="inlineStr">
+        <is>
+          <t>Colston Tower, Bristol</t>
+        </is>
+      </c>
+      <c r="D408" s="3" t="inlineStr">
+        <is>
+          <t>https://www.triarecruitment.com</t>
+        </is>
+      </c>
+      <c r="E408" s="3" t="inlineStr">
+        <is>
+          <t>info@triarecruitment.com</t>
+        </is>
+      </c>
+      <c r="F408" s="3" t="inlineStr">
+        <is>
+          <t>0117 332 7000</t>
+        </is>
+      </c>
+      <c r="G408" s="3" t="inlineStr">
+        <is>
+          <t>Harriet Kirkpatrick, Lara Webb &amp; David Kirkpatrick (Co-founders, est. 2015)</t>
+        </is>
+      </c>
+      <c r="H408" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/tria-recruitment</t>
+        </is>
+      </c>
+      <c r="I408" s="3" t="inlineStr"/>
+      <c r="J408" s="3" t="inlineStr">
+        <is>
+          <t>Majority women-owned independent tech recruiter; placement fees on developer/engineering roles run into thousands per hire</t>
+        </is>
+      </c>
+      <c r="K408" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L408" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M408" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N408" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O408" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn presence; established multi-founder brand</t>
+        </is>
+      </c>
+      <c r="P408" s="3" t="inlineStr">
+        <is>
+          <t>Peaple Talent/ISL Talent/Xist4 all compete for the same Bristol tech-recruitment searches</t>
+        </is>
+      </c>
+      <c r="Q408" s="3" t="inlineStr">
+        <is>
+          <t>'Majority women-owned, independent tech recruiter - own that distinct AEO positioning in Bristol'</t>
+        </is>
+      </c>
+      <c r="R408" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S408" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T408" s="3" t="inlineStr"/>
+    </row>
+    <row r="409">
+      <c r="A409" s="3" t="inlineStr">
+        <is>
+          <t>Xist4</t>
+        </is>
+      </c>
+      <c r="B409" s="3" t="inlineStr">
+        <is>
+          <t>Data/tech/AI recruitment agency</t>
+        </is>
+      </c>
+      <c r="C409" s="3" t="inlineStr">
+        <is>
+          <t>Bristol &amp; London</t>
+        </is>
+      </c>
+      <c r="D409" s="3" t="inlineStr">
+        <is>
+          <t>https://www.xist4.com</t>
+        </is>
+      </c>
+      <c r="E409" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F409" s="3" t="inlineStr"/>
+      <c r="G409" s="3" t="inlineStr">
+        <is>
+          <t>26 years combined sector experience</t>
+        </is>
+      </c>
+      <c r="H409" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/xist4-it-recruitment</t>
+        </is>
+      </c>
+      <c r="I409" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/XIST4</t>
+        </is>
+      </c>
+      <c r="J409" s="3" t="inlineStr">
+        <is>
+          <t>Specialist data/cyber/AI recruiter across 2 major cities; placement fees on senior tech/leadership roles are substantial</t>
+        </is>
+      </c>
+      <c r="K409" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L409" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M409" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N409" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O409" s="3" t="inlineStr">
+        <is>
+          <t>Sector-specific landing pages (fintech, startups, cyber) = active SEO</t>
+        </is>
+      </c>
+      <c r="P409" s="3" t="inlineStr">
+        <is>
+          <t>Sector pages exist but AI-answer citations for specific niche tech-recruitment queries still open</t>
+        </is>
+      </c>
+      <c r="Q409" s="3" t="inlineStr">
+        <is>
+          <t>'You built pages for fintech, cyber and AI recruitment - let's make AI cite them'</t>
+        </is>
+      </c>
+      <c r="R409" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S409" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T409" s="3" t="inlineStr"/>
+    </row>
+    <row r="410">
+      <c r="A410" s="2" t="inlineStr">
+        <is>
+          <t>Ray Cochrane Beauty Aesthetics Academy</t>
+        </is>
+      </c>
+      <c r="B410" s="2" t="inlineStr">
+        <is>
+          <t>Beauty/aesthetics training academy</t>
+        </is>
+      </c>
+      <c r="C410" s="2" t="inlineStr">
+        <is>
+          <t>Baker Street, London W1</t>
+        </is>
+      </c>
+      <c r="D410" s="2" t="inlineStr">
+        <is>
+          <t>https://www.raycochrane.co.uk</t>
+        </is>
+      </c>
+      <c r="E410" s="2" t="inlineStr">
+        <is>
+          <t>admission@raycochrane.co.uk</t>
+        </is>
+      </c>
+      <c r="F410" s="2" t="inlineStr">
+        <is>
+          <t>020 7486 6291</t>
+        </is>
+      </c>
+      <c r="G410" s="2" t="inlineStr">
+        <is>
+          <t>Founded 1954 by Mrs Ray Cochrane; longest-established CIDESCO school in the UK</t>
+        </is>
+      </c>
+      <c r="H410" s="2" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/raycochranebeautyaestheticsacademy</t>
+        </is>
+      </c>
+      <c r="I410" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/raycochraneacademy</t>
+        </is>
+      </c>
+      <c r="J410" s="2" t="inlineStr">
+        <is>
+          <t>71-year heritage academy training beauty therapists who go on to open their own high-value clinics; course fees run into thousands per student</t>
+        </is>
+      </c>
+      <c r="K410" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L410" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M410" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N410" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O410" s="2" t="inlineStr">
+        <is>
+          <t>CIDESCO prestige accreditation promoted</t>
+        </is>
+      </c>
+      <c r="P410" s="2" t="inlineStr">
+        <is>
+          <t>71 years of heritage + prestigious accreditation not yet the AI-cited answer for 'beauty academy London'</t>
+        </is>
+      </c>
+      <c r="Q410" s="2" t="inlineStr">
+        <is>
+          <t>'The UK's longest-established CIDESCO school - own that exact AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R410" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S410" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T410" s="2" t="inlineStr">
+        <is>
+          <t>Exceptional 71-year heritage story - high-value AEO opportunity</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" s="4" t="inlineStr">
+        <is>
+          <t>Omni Academy of Hair, Beauty &amp; Aesthetics</t>
+        </is>
+      </c>
+      <c r="B411" s="4" t="inlineStr">
+        <is>
+          <t>Beauty/hair training academy</t>
+        </is>
+      </c>
+      <c r="C411" s="4" t="inlineStr">
+        <is>
+          <t>Walton-on-Thames, Surrey</t>
+        </is>
+      </c>
+      <c r="D411" s="4" t="inlineStr">
+        <is>
+          <t>https://www.omniacademy.co.uk</t>
+        </is>
+      </c>
+      <c r="E411" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F411" s="4" t="inlineStr"/>
+      <c r="G411" s="4" t="inlineStr">
+        <is>
+          <t>Carolyne Cross (Founder, est. 2008); Rianna (current lead, since 2022)</t>
+        </is>
+      </c>
+      <c r="H411" s="4" t="inlineStr">
+        <is>
+          <t>instagram.com/omniacademy1</t>
+        </is>
+      </c>
+      <c r="I411" s="4" t="inlineStr"/>
+      <c r="J411" s="4" t="inlineStr">
+        <is>
+          <t>17-year independent academy in wealthy Surrey; students pay course fees for hair/beauty/aesthetics/massage qualifications</t>
+        </is>
+      </c>
+      <c r="K411" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L411" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M411" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N411" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O411" s="4" t="inlineStr">
+        <is>
+          <t>Instagram presence</t>
+        </is>
+      </c>
+      <c r="P411" s="4" t="inlineStr">
+        <is>
+          <t>Local Surrey students search generically for 'beauty course near me' - academy not yet the AI-cited local answer</t>
+        </is>
+      </c>
+      <c r="Q411" s="4" t="inlineStr">
+        <is>
+          <t>Own 'beauty training course Surrey' - a specific, winnable local AEO target</t>
+        </is>
+      </c>
+      <c r="R411" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S411" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="T411" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T407"/>
+  <autoFilter ref="A1:T411"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -35696,7 +36068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B160"/>
+  <dimension ref="A1:B164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -35716,7 +36088,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>406</v>
+        <v>410</v>
       </c>
     </row>
     <row r="5">
@@ -37273,6 +37645,46 @@
         </is>
       </c>
       <c r="B160" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Tech recruitment agency</t>
+        </is>
+      </c>
+      <c r="B161" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Data/tech/AI recruitment agency</t>
+        </is>
+      </c>
+      <c r="B162" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Beauty/aesthetics training academy</t>
+        </is>
+      </c>
+      <c r="B163" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Beauty/hair training academy</t>
+        </is>
+      </c>
+      <c r="B164" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 40: +3 prospects (413 total) - medical aesthetics training, yoga teacher training, creative recruitment
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$411</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$414</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T411"/>
+  <dimension ref="A1:T414"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -36056,8 +36056,276 @@
       </c>
       <c r="T411" s="4" t="inlineStr"/>
     </row>
+    <row r="412">
+      <c r="A412" s="2" t="inlineStr">
+        <is>
+          <t>Interface Aesthetics</t>
+        </is>
+      </c>
+      <c r="B412" s="2" t="inlineStr">
+        <is>
+          <t>Medical aesthetics/injectable training academy</t>
+        </is>
+      </c>
+      <c r="C412" s="2" t="inlineStr">
+        <is>
+          <t>Westminster Bridge Road, London SE1</t>
+        </is>
+      </c>
+      <c r="D412" s="2" t="inlineStr">
+        <is>
+          <t>https://www.interfaceaesthetics.co.uk</t>
+        </is>
+      </c>
+      <c r="E412" s="2" t="inlineStr">
+        <is>
+          <t>contact@interfaceaesthetics.co.uk</t>
+        </is>
+      </c>
+      <c r="F412" s="2" t="inlineStr">
+        <is>
+          <t>07944 543113</t>
+        </is>
+      </c>
+      <c r="G412" s="2" t="inlineStr">
+        <is>
+          <t>Dr James Olding (Founder/Lead Trainer; Senior Specialist Registrar in Oral &amp; Maxillofacial Surgery, GetHarley Medical Aesthetic Practitioner of the Year 2025)</t>
+        </is>
+      </c>
+      <c r="H412" s="2" t="inlineStr"/>
+      <c r="I412" s="2" t="inlineStr"/>
+      <c r="J412" s="2" t="inlineStr">
+        <is>
+          <t>Award-winning consultant-led injectables training academy for medical professionals; course fees run into thousands per delegate, repeat cohorts</t>
+        </is>
+      </c>
+      <c r="K412" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L412" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M412" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N412" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O412" s="2" t="inlineStr">
+        <is>
+          <t>Award win (GetHarley 2025) = active PR/marketing investment</t>
+        </is>
+      </c>
+      <c r="P412" s="2" t="inlineStr">
+        <is>
+          <t>Award-winning credentials not yet the AI-cited answer for 'medical aesthetics training London'</t>
+        </is>
+      </c>
+      <c r="Q412" s="2" t="inlineStr">
+        <is>
+          <t>'2025 Practitioner of the Year - own that exact AEO trust signal in AI-search answers'</t>
+        </is>
+      </c>
+      <c r="R412" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S412" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T412" s="2" t="inlineStr">
+        <is>
+          <t>Strong credentialed-founder story, high-value course fees</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" s="4" t="inlineStr">
+        <is>
+          <t>Bristol School of Yoga</t>
+        </is>
+      </c>
+      <c r="B413" s="4" t="inlineStr">
+        <is>
+          <t>Yoga teacher training school</t>
+        </is>
+      </c>
+      <c r="C413" s="4" t="inlineStr">
+        <is>
+          <t>Backfields Lane, Bristol BS2</t>
+        </is>
+      </c>
+      <c r="D413" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bristolschoolofyoga.co.uk</t>
+        </is>
+      </c>
+      <c r="E413" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F413" s="4" t="inlineStr"/>
+      <c r="G413" s="4" t="inlineStr">
+        <is>
+          <t>Laura Gilmore (Founder/Director)</t>
+        </is>
+      </c>
+      <c r="H413" s="4" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/lauragilmoreyoga</t>
+        </is>
+      </c>
+      <c r="I413" s="4" t="inlineStr"/>
+      <c r="J413" s="4" t="inlineStr">
+        <is>
+          <t>Independent 200hr/300hr yoga teacher-training provider; trainee fees run into thousands per cohort, repeat intakes</t>
+        </is>
+      </c>
+      <c r="K413" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L413" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M413" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N413" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O413" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn presence</t>
+        </is>
+      </c>
+      <c r="P413" s="4" t="inlineStr">
+        <is>
+          <t>Generic 'yoga teacher training Bristol' searches not yet AI-answer dominated by this school</t>
+        </is>
+      </c>
+      <c r="Q413" s="4" t="inlineStr">
+        <is>
+          <t>'Own the AI-cited answer for yoga teacher training in Bristol - not just another studio timetable'</t>
+        </is>
+      </c>
+      <c r="R413" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S413" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T413" s="4" t="inlineStr"/>
+    </row>
+    <row r="414">
+      <c r="A414" s="3" t="inlineStr">
+        <is>
+          <t>Creative Crowd</t>
+        </is>
+      </c>
+      <c r="B414" s="3" t="inlineStr">
+        <is>
+          <t>Creative &amp; marketing recruitment agency</t>
+        </is>
+      </c>
+      <c r="C414" s="3" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="D414" s="3" t="inlineStr">
+        <is>
+          <t>https://www.creativecrowd.london</t>
+        </is>
+      </c>
+      <c r="E414" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F414" s="3" t="inlineStr"/>
+      <c r="G414" s="3" t="inlineStr">
+        <is>
+          <t>Surfraz Alam &amp; Daniel Levy (Co-founders)</t>
+        </is>
+      </c>
+      <c r="H414" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/creative-crowd-recruitment</t>
+        </is>
+      </c>
+      <c r="I414" s="3" t="inlineStr"/>
+      <c r="J414" s="3" t="inlineStr">
+        <is>
+          <t>Independent specialist recruiter placing creative/marketing/digital talent into agencies and brands; placement fees on mid-senior creative roles are substantial</t>
+        </is>
+      </c>
+      <c r="K414" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L414" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M414" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N414" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O414" s="3" t="inlineStr">
+        <is>
+          <t>Dedicated department landing pages = active SEO investment</t>
+        </is>
+      </c>
+      <c r="P414" s="3" t="inlineStr">
+        <is>
+          <t>Crowded London creative-recruitment market with many similarly-positioned boutiques</t>
+        </is>
+      </c>
+      <c r="Q414" s="3" t="inlineStr">
+        <is>
+          <t>'You built pages for every creative discipline - let's make AI cite them, not just index them'</t>
+        </is>
+      </c>
+      <c r="R414" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S414" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T414" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T411"/>
+  <autoFilter ref="A1:T414"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -36068,7 +36336,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B164"/>
+  <dimension ref="A1:B167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -36088,7 +36356,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>410</v>
+        <v>413</v>
       </c>
     </row>
     <row r="5">
@@ -37685,6 +37953,36 @@
         </is>
       </c>
       <c r="B164" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Medical aesthetics/injectable training academy</t>
+        </is>
+      </c>
+      <c r="B165" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Yoga teacher training school</t>
+        </is>
+      </c>
+      <c r="B166" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Creative &amp; marketing recruitment agency</t>
+        </is>
+      </c>
+      <c r="B167" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batches 41-44: +17 prospects (430 total) - Cotswolds/Kent architects & interiors, Cheltenham/Oxford healthcare, Cheltenham/Oxford/Windsor estate agents, ADI driving instructor training
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$414</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$431</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T414"/>
+  <dimension ref="A1:T431"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -36324,8 +36324,1588 @@
       </c>
       <c r="T414" s="3" t="inlineStr"/>
     </row>
+    <row r="415">
+      <c r="A415" s="3" t="inlineStr">
+        <is>
+          <t>Blake Architects</t>
+        </is>
+      </c>
+      <c r="B415" s="3" t="inlineStr">
+        <is>
+          <t>Architecture practice</t>
+        </is>
+      </c>
+      <c r="C415" s="3" t="inlineStr">
+        <is>
+          <t>Winstone, Cirencester, Cotswolds</t>
+        </is>
+      </c>
+      <c r="D415" s="3" t="inlineStr">
+        <is>
+          <t>https://www.blakearchitects.co.uk</t>
+        </is>
+      </c>
+      <c r="E415" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F415" s="3" t="inlineStr">
+        <is>
+          <t>01285 841407</t>
+        </is>
+      </c>
+      <c r="G415" s="3" t="inlineStr">
+        <is>
+          <t>Jonathan Nettleton (Founder, est. 2011)</t>
+        </is>
+      </c>
+      <c r="H415" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/blake-architects-limited</t>
+        </is>
+      </c>
+      <c r="I415" s="3" t="inlineStr">
+        <is>
+          <t>instagram.com/blakearchitects; facebook.com/BlakeArchitectsLimited</t>
+        </is>
+      </c>
+      <c r="J415" s="3" t="inlineStr">
+        <is>
+          <t>RIBA Chartered practice specialising in barn conversions to listed manors; single-site independent studio in a converted Cotswold barn, project fees run into tens of thousands</t>
+        </is>
+      </c>
+      <c r="K415" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L415" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M415" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N415" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O415" s="3" t="inlineStr">
+        <is>
+          <t>Instagram (3.9k followers) + Green Register membership = active marketing investment</t>
+        </is>
+      </c>
+      <c r="P415" s="3" t="inlineStr">
+        <is>
+          <t>Niche listed-building/barn-conversion expertise not yet the AI-cited answer for Cotswolds architects</t>
+        </is>
+      </c>
+      <c r="Q415" s="3" t="inlineStr">
+        <is>
+          <t>'RIBA-chartered barn-conversion specialists - own that exact AEO niche in the Cotswolds'</t>
+        </is>
+      </c>
+      <c r="R415" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S415" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T415" s="3" t="inlineStr"/>
+    </row>
+    <row r="416">
+      <c r="A416" s="3" t="inlineStr">
+        <is>
+          <t>Studio Bellord (Camilla Bellord Interiors)</t>
+        </is>
+      </c>
+      <c r="B416" s="3" t="inlineStr">
+        <is>
+          <t>Interior design studio</t>
+        </is>
+      </c>
+      <c r="C416" s="3" t="inlineStr">
+        <is>
+          <t>Great Rissington, nr Bourton-on-the-Water, Cotswolds</t>
+        </is>
+      </c>
+      <c r="D416" s="3" t="inlineStr">
+        <is>
+          <t>https://www.studiobellord.com</t>
+        </is>
+      </c>
+      <c r="E416" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F416" s="3" t="inlineStr">
+        <is>
+          <t>07584 044052</t>
+        </is>
+      </c>
+      <c r="G416" s="3" t="inlineStr">
+        <is>
+          <t>Camilla Bellord &amp; Tom Bellord (Husband-and-wife owners)</t>
+        </is>
+      </c>
+      <c r="H416" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/camilla-bellord-b40b9563</t>
+        </is>
+      </c>
+      <c r="I416" s="3" t="inlineStr"/>
+      <c r="J416" s="3" t="inlineStr">
+        <is>
+          <t>Bespoke private residential interior design across the Cotswolds; KLC-trained founder with 20+ years experience, project fees run into tens of thousands</t>
+        </is>
+      </c>
+      <c r="K416" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L416" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M416" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N416" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O416" s="3" t="inlineStr">
+        <is>
+          <t>Featured on Houzz and industry blogs = active PR/marketing</t>
+        </is>
+      </c>
+      <c r="P416" s="3" t="inlineStr">
+        <is>
+          <t>Houzz features not yet converted into AI-cited answers for 'interior designer Cotswolds'</t>
+        </is>
+      </c>
+      <c r="Q416" s="3" t="inlineStr">
+        <is>
+          <t>'Featured on Houzz - let's make AI cite you the same way for search'</t>
+        </is>
+      </c>
+      <c r="R416" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S416" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T416" s="3" t="inlineStr"/>
+    </row>
+    <row r="417">
+      <c r="A417" s="3" t="inlineStr">
+        <is>
+          <t>Studio Hudson Architects</t>
+        </is>
+      </c>
+      <c r="B417" s="3" t="inlineStr">
+        <is>
+          <t>Architecture practice</t>
+        </is>
+      </c>
+      <c r="C417" s="3" t="inlineStr">
+        <is>
+          <t>Royal Tunbridge Wells, Kent</t>
+        </is>
+      </c>
+      <c r="D417" s="3" t="inlineStr">
+        <is>
+          <t>https://www.studio-hudson.co.uk</t>
+        </is>
+      </c>
+      <c r="E417" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F417" s="3" t="inlineStr"/>
+      <c r="G417" s="3" t="inlineStr">
+        <is>
+          <t>Ian Hudson (Founder/Principal Architect, est. 2012)</t>
+        </is>
+      </c>
+      <c r="H417" s="3" t="inlineStr"/>
+      <c r="I417" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/studiohudson1</t>
+        </is>
+      </c>
+      <c r="J417" s="3" t="inlineStr">
+        <is>
+          <t>RIBA Chartered residential practice covering Sevenoaks/Tonbridge/Maidstone; award-winning one-founder studio, project fees run into tens of thousands</t>
+        </is>
+      </c>
+      <c r="K417" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L417" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M417" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N417" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O417" s="3" t="inlineStr">
+        <is>
+          <t>Two industry awards (2017, 2021) = active reputation-building</t>
+        </is>
+      </c>
+      <c r="P417" s="3" t="inlineStr">
+        <is>
+          <t>Award wins not yet the AI-cited trust signal for 'architect Tunbridge Wells'</t>
+        </is>
+      </c>
+      <c r="Q417" s="3" t="inlineStr">
+        <is>
+          <t>'Award-winning since 2017 - own that AEO trust signal against bigger multi-office practices'</t>
+        </is>
+      </c>
+      <c r="R417" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S417" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T417" s="3" t="inlineStr"/>
+    </row>
+    <row r="418">
+      <c r="A418" s="3" t="inlineStr">
+        <is>
+          <t>Barkerdesign</t>
+        </is>
+      </c>
+      <c r="B418" s="3" t="inlineStr">
+        <is>
+          <t>Interior design studio</t>
+        </is>
+      </c>
+      <c r="C418" s="3" t="inlineStr">
+        <is>
+          <t>Tunbridge Wells, Kent</t>
+        </is>
+      </c>
+      <c r="D418" s="3" t="inlineStr">
+        <is>
+          <t>https://www.barker-design.com</t>
+        </is>
+      </c>
+      <c r="E418" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F418" s="3" t="inlineStr">
+        <is>
+          <t>07788 581928</t>
+        </is>
+      </c>
+      <c r="G418" s="3" t="inlineStr">
+        <is>
+          <t>Justine Hodgson-Barker (Founder, BIID-accredited)</t>
+        </is>
+      </c>
+      <c r="H418" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/justine-hodgson-barker-8626a4107</t>
+        </is>
+      </c>
+      <c r="I418" s="3" t="inlineStr">
+        <is>
+          <t>instagram.com/barker_design</t>
+        </is>
+      </c>
+      <c r="J418" s="3" t="inlineStr">
+        <is>
+          <t>High-end interior design for period/character homes across Kent and East Sussex; BIID accreditation and House &amp; Garden Directory membership signal premium positioning, project fees run into tens of thousands</t>
+        </is>
+      </c>
+      <c r="K418" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L418" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M418" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N418" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O418" s="3" t="inlineStr">
+        <is>
+          <t>House &amp; Garden Directory + press features (Great British Life, Priceless) = active PR</t>
+        </is>
+      </c>
+      <c r="P418" s="3" t="inlineStr">
+        <is>
+          <t>Press features not yet the AI-cited answer for 'interior designer Tunbridge Wells'</t>
+        </is>
+      </c>
+      <c r="Q418" s="3" t="inlineStr">
+        <is>
+          <t>'House &amp; Garden Directory listed - own that exact AEO credibility signal'</t>
+        </is>
+      </c>
+      <c r="R418" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S418" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T418" s="3" t="inlineStr"/>
+    </row>
+    <row r="419">
+      <c r="A419" s="3" t="inlineStr">
+        <is>
+          <t>Wyatt Glass Chartered Architects</t>
+        </is>
+      </c>
+      <c r="B419" s="3" t="inlineStr">
+        <is>
+          <t>Architecture practice</t>
+        </is>
+      </c>
+      <c r="C419" s="3" t="inlineStr">
+        <is>
+          <t>Sevenoaks, Kent</t>
+        </is>
+      </c>
+      <c r="D419" s="3" t="inlineStr">
+        <is>
+          <t>https://www.wyattglass.co.uk</t>
+        </is>
+      </c>
+      <c r="E419" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F419" s="3" t="inlineStr">
+        <is>
+          <t>01732 746600</t>
+        </is>
+      </c>
+      <c r="G419" s="3" t="inlineStr">
+        <is>
+          <t>Wyatt Glass (Founder, est. 1992)</t>
+        </is>
+      </c>
+      <c r="H419" s="3" t="inlineStr"/>
+      <c r="I419" s="3" t="inlineStr"/>
+      <c r="J419" s="3" t="inlineStr">
+        <is>
+          <t>33-year RIBA Chartered practice for extensions, conversions, new builds and listed buildings; one of the longest-running independents in the area, project fees run into tens of thousands</t>
+        </is>
+      </c>
+      <c r="K419" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L419" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M419" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N419" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O419" s="3" t="inlineStr">
+        <is>
+          <t>33-year trading history = established local reputation</t>
+        </is>
+      </c>
+      <c r="P419" s="3" t="inlineStr">
+        <is>
+          <t>Long heritage not yet leveraged as an AEO trust signal against newer competitors</t>
+        </is>
+      </c>
+      <c r="Q419" s="3" t="inlineStr">
+        <is>
+          <t>'33 years designing Sevenoaks homes - own that AEO trust signal in AI-search answers'</t>
+        </is>
+      </c>
+      <c r="R419" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S419" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T419" s="3" t="inlineStr"/>
+    </row>
+    <row r="420">
+      <c r="A420" s="4" t="inlineStr">
+        <is>
+          <t>Catherine Westoby Interior Design</t>
+        </is>
+      </c>
+      <c r="B420" s="4" t="inlineStr">
+        <is>
+          <t>Interior design studio</t>
+        </is>
+      </c>
+      <c r="C420" s="4" t="inlineStr">
+        <is>
+          <t>Tonbridge, Kent</t>
+        </is>
+      </c>
+      <c r="D420" s="4" t="inlineStr">
+        <is>
+          <t>https://www.catherinewestobyinteriordesign.co.uk</t>
+        </is>
+      </c>
+      <c r="E420" s="4" t="inlineStr">
+        <is>
+          <t>catherinewestoby.interiordesign@gmail.com</t>
+        </is>
+      </c>
+      <c r="F420" s="4" t="inlineStr"/>
+      <c r="G420" s="4" t="inlineStr">
+        <is>
+          <t>Catherine Westoby (Founder)</t>
+        </is>
+      </c>
+      <c r="H420" s="4" t="inlineStr"/>
+      <c r="I420" s="4" t="inlineStr">
+        <is>
+          <t>facebook.com/catherinewestobyinteriordesign</t>
+        </is>
+      </c>
+      <c r="J420" s="4" t="inlineStr">
+        <is>
+          <t>Solo-practitioner residential interior designer across Sevenoaks/Tunbridge Wells/Tonbridge; Houzz-listed, project fees run into thousands per client</t>
+        </is>
+      </c>
+      <c r="K420" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L420" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M420" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N420" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O420" s="4" t="inlineStr">
+        <is>
+          <t>Houzz listing</t>
+        </is>
+      </c>
+      <c r="P420" s="4" t="inlineStr">
+        <is>
+          <t>Solo practitioner needs to compete with larger studios for AI-search visibility</t>
+        </is>
+      </c>
+      <c r="Q420" s="4" t="inlineStr">
+        <is>
+          <t>Own a specific Kent-market AEO niche (e.g. period-home interiors) vs bigger studios</t>
+        </is>
+      </c>
+      <c r="R420" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S420" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T420" s="4" t="inlineStr"/>
+    </row>
+    <row r="421">
+      <c r="A421" s="3" t="inlineStr">
+        <is>
+          <t>Montpellier Medical</t>
+        </is>
+      </c>
+      <c r="B421" s="3" t="inlineStr">
+        <is>
+          <t>Private GP practice</t>
+        </is>
+      </c>
+      <c r="C421" s="3" t="inlineStr">
+        <is>
+          <t>Montpellier Parade, Cheltenham</t>
+        </is>
+      </c>
+      <c r="D421" s="3" t="inlineStr">
+        <is>
+          <t>https://www.montpelliermedical.co.uk</t>
+        </is>
+      </c>
+      <c r="E421" s="3" t="inlineStr">
+        <is>
+          <t>admin@montpelliermedical.co.uk</t>
+        </is>
+      </c>
+      <c r="F421" s="3" t="inlineStr">
+        <is>
+          <t>01242 379 138</t>
+        </is>
+      </c>
+      <c r="G421" s="3" t="inlineStr">
+        <is>
+          <t>Dr Laura O'Loghlen &amp; Dr Justin Forbes (Co-founders, opened 2025)</t>
+        </is>
+      </c>
+      <c r="H421" s="3" t="inlineStr"/>
+      <c r="I421" s="3" t="inlineStr"/>
+      <c r="J421" s="3" t="inlineStr">
+        <is>
+          <t>New two-doctor private GP practice offering 30-min appointments/health checks/blood tests; private consultation fees run into hundreds per visit, repeat annual health-check clients</t>
+        </is>
+      </c>
+      <c r="K421" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L421" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M421" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N421" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O421" s="3" t="inlineStr">
+        <is>
+          <t>None visible - newly opened 2025</t>
+        </is>
+      </c>
+      <c r="P421" s="3" t="inlineStr">
+        <is>
+          <t>Brand-new practice with no AI-search presence yet - ground-floor opportunity</t>
+        </is>
+      </c>
+      <c r="Q421" s="3" t="inlineStr">
+        <is>
+          <t>'You're brand new in Cheltenham - be the AI-cited answer before competitors are'</t>
+        </is>
+      </c>
+      <c r="R421" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S421" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T421" s="3" t="inlineStr">
+        <is>
+          <t>Opened March 2025, CQC-registered - very new, high AEO upside</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" s="3" t="inlineStr">
+        <is>
+          <t>Cotswold Private GP Service</t>
+        </is>
+      </c>
+      <c r="B422" s="3" t="inlineStr">
+        <is>
+          <t>Private GP practice</t>
+        </is>
+      </c>
+      <c r="C422" s="3" t="inlineStr">
+        <is>
+          <t>Hatherley Lane, Cheltenham</t>
+        </is>
+      </c>
+      <c r="D422" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cotswoldprivategp.co.uk</t>
+        </is>
+      </c>
+      <c r="E422" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F422" s="3" t="inlineStr">
+        <is>
+          <t>01242 700350</t>
+        </is>
+      </c>
+      <c r="G422" s="3" t="inlineStr">
+        <is>
+          <t>Dr Hosur, Dr Meenakshi Raina, Dr Junemani (Clinical team, 20+ yrs NHS experience each)</t>
+        </is>
+      </c>
+      <c r="H422" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/cotswold-private-gp</t>
+        </is>
+      </c>
+      <c r="I422" s="3" t="inlineStr">
+        <is>
+          <t>instagram.com/cotswoldprivategp; facebook.com/p/Cotswold-Private-GP-Service</t>
+        </is>
+      </c>
+      <c r="J422" s="3" t="inlineStr">
+        <is>
+          <t>Same-day private GP consultations across Cheltenham/Cotswolds; private consultation fees run into hundreds per visit with repeat patients</t>
+        </is>
+      </c>
+      <c r="K422" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L422" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M422" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N422" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O422" s="3" t="inlineStr">
+        <is>
+          <t>Instagram/Facebook/LinkedIn presence = active marketing</t>
+        </is>
+      </c>
+      <c r="P422" s="3" t="inlineStr">
+        <is>
+          <t>Multi-channel social presence not yet converted into AI-cited answers for 'private GP Cheltenham'</t>
+        </is>
+      </c>
+      <c r="Q422" s="3" t="inlineStr">
+        <is>
+          <t>'You're already posting on 3 platforms - let's make AI cite you too'</t>
+        </is>
+      </c>
+      <c r="R422" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S422" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T422" s="3" t="inlineStr"/>
+    </row>
+    <row r="423">
+      <c r="A423" s="2" t="inlineStr">
+        <is>
+          <t>Ruth Jackson Aesthetics</t>
+        </is>
+      </c>
+      <c r="B423" s="2" t="inlineStr">
+        <is>
+          <t>Aesthetics clinic (non-surgical)</t>
+        </is>
+      </c>
+      <c r="C423" s="2" t="inlineStr">
+        <is>
+          <t>St George's Road, Cheltenham</t>
+        </is>
+      </c>
+      <c r="D423" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ruthjacksonaesthetics.co.uk</t>
+        </is>
+      </c>
+      <c r="E423" s="2" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F423" s="2" t="inlineStr">
+        <is>
+          <t>07804 432426</t>
+        </is>
+      </c>
+      <c r="G423" s="2" t="inlineStr">
+        <is>
+          <t>Ruth Jackson (Founder, nurse prescriber)</t>
+        </is>
+      </c>
+      <c r="H423" s="2" t="inlineStr"/>
+      <c r="I423" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/p/Ruth-Jackson-Aesthetics-100093995566592</t>
+        </is>
+      </c>
+      <c r="J423" s="2" t="inlineStr">
+        <is>
+          <t>Award-winning nurse-led non-surgical aesthetics clinic (fillers, HIFU, facials) plus mobile service; repeat treatment clients, premium per-session fees</t>
+        </is>
+      </c>
+      <c r="K423" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L423" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M423" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N423" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O423" s="2" t="inlineStr">
+        <is>
+          <t>2025 National Winner, Best Aesthetics Business in England award</t>
+        </is>
+      </c>
+      <c r="P423" s="2" t="inlineStr">
+        <is>
+          <t>National award win not yet the AI-cited trust signal for 'aesthetics clinic Cheltenham'</t>
+        </is>
+      </c>
+      <c r="Q423" s="2" t="inlineStr">
+        <is>
+          <t>'National award winner 2025 - own that exact AEO trust signal in AI-search answers'</t>
+        </is>
+      </c>
+      <c r="R423" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S423" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T423" s="2" t="inlineStr">
+        <is>
+          <t>National award win = strong AEO hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" s="3" t="inlineStr">
+        <is>
+          <t>Oxona Healthcare</t>
+        </is>
+      </c>
+      <c r="B424" s="3" t="inlineStr">
+        <is>
+          <t>Private dermatology &amp; women's health clinics</t>
+        </is>
+      </c>
+      <c r="C424" s="3" t="inlineStr">
+        <is>
+          <t>Headington, Oxford (+ Chipping Norton, Didcot, Henley, St Albans)</t>
+        </is>
+      </c>
+      <c r="D424" s="3" t="inlineStr">
+        <is>
+          <t>https://www.oxonahealth.co.uk</t>
+        </is>
+      </c>
+      <c r="E424" s="3" t="inlineStr">
+        <is>
+          <t>reception@oxonahealth.co.uk</t>
+        </is>
+      </c>
+      <c r="F424" s="3" t="inlineStr">
+        <is>
+          <t>01865 965 027</t>
+        </is>
+      </c>
+      <c r="G424" s="3" t="inlineStr">
+        <is>
+          <t>Megan (Co-founder, Business Development)</t>
+        </is>
+      </c>
+      <c r="H424" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/oxonahealthcare</t>
+        </is>
+      </c>
+      <c r="I424" s="3" t="inlineStr">
+        <is>
+          <t>instagram.com/oxona_health; facebook.com/Oxonahealthcare</t>
+        </is>
+      </c>
+      <c r="J424" s="3" t="inlineStr">
+        <is>
+          <t>Independent multi-site dermatology/women's health group across 5 Home Counties towns; consultant-led private appointments run into hundreds per visit, repeat patients</t>
+        </is>
+      </c>
+      <c r="K424" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L424" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M424" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N424" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O424" s="3" t="inlineStr">
+        <is>
+          <t>Multi-channel social presence + multi-site expansion = active marketing investment</t>
+        </is>
+      </c>
+      <c r="P424" s="3" t="inlineStr">
+        <is>
+          <t>5-site footprint not matched by 5-location AI-search dominance</t>
+        </is>
+      </c>
+      <c r="Q424" s="3" t="inlineStr">
+        <is>
+          <t>Per-location AEO content to own each town's 'private dermatologist near me' AI answer separately</t>
+        </is>
+      </c>
+      <c r="R424" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S424" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T424" s="3" t="inlineStr"/>
+    </row>
+    <row r="425">
+      <c r="A425" s="2" t="inlineStr">
+        <is>
+          <t>My Dermatologist (Dr Jonathan Bowling)</t>
+        </is>
+      </c>
+      <c r="B425" s="2" t="inlineStr">
+        <is>
+          <t>Private dermatology practice</t>
+        </is>
+      </c>
+      <c r="C425" s="2" t="inlineStr">
+        <is>
+          <t>Headington, Oxford</t>
+        </is>
+      </c>
+      <c r="D425" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mydermatologist.co.uk</t>
+        </is>
+      </c>
+      <c r="E425" s="2" t="inlineStr">
+        <is>
+          <t>info@mydermatologist.co.uk</t>
+        </is>
+      </c>
+      <c r="F425" s="2" t="inlineStr">
+        <is>
+          <t>01865 861577</t>
+        </is>
+      </c>
+      <c r="G425" s="2" t="inlineStr">
+        <is>
+          <t>Dr Jonathan Bowling (Consultant Dermatologist, FRCP, ex-Oxford Univ. Hospitals lecturer)</t>
+        </is>
+      </c>
+      <c r="H425" s="2" t="inlineStr"/>
+      <c r="I425" s="2" t="inlineStr"/>
+      <c r="J425" s="2" t="inlineStr">
+        <is>
+          <t>Solo-consultant skin cancer/mole screening practice; author of an award-winning dermoscopy textbook, trained 4,000+ clinicians - premium per-consultation fees</t>
+        </is>
+      </c>
+      <c r="K425" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L425" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M425" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N425" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O425" s="2" t="inlineStr">
+        <is>
+          <t>Published award-winning textbook = strong authority/credibility asset</t>
+        </is>
+      </c>
+      <c r="P425" s="2" t="inlineStr">
+        <is>
+          <t>Exceptional published-authority credential not yet the AI-cited answer for 'private dermatologist Oxford'</t>
+        </is>
+      </c>
+      <c r="Q425" s="2" t="inlineStr">
+        <is>
+          <t>'You wrote the textbook other dermatologists train from - own that AEO authority signal'</t>
+        </is>
+      </c>
+      <c r="R425" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S425" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T425" s="2" t="inlineStr">
+        <is>
+          <t>Textbook author + 4,000 clinicians trained - exceptional authority story</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" s="4" t="inlineStr">
+        <is>
+          <t>Town House Face &amp; Body Clinic</t>
+        </is>
+      </c>
+      <c r="B426" s="4" t="inlineStr">
+        <is>
+          <t>Aesthetics clinic (non-surgical)</t>
+        </is>
+      </c>
+      <c r="C426" s="4" t="inlineStr">
+        <is>
+          <t>Albany Road, Cheltenham</t>
+        </is>
+      </c>
+      <c r="D426" s="4" t="inlineStr">
+        <is>
+          <t>https://www.townhousefaceandbodyclinic.co.uk</t>
+        </is>
+      </c>
+      <c r="E426" s="4" t="inlineStr">
+        <is>
+          <t>enquiries@townhousefaceandbodyclinic.co.uk</t>
+        </is>
+      </c>
+      <c r="F426" s="4" t="inlineStr">
+        <is>
+          <t>01242 303785</t>
+        </is>
+      </c>
+      <c r="G426" s="4" t="inlineStr">
+        <is>
+          <t>Eliza (Founder, 30+ yrs NHS nursing background, est. 2011)</t>
+        </is>
+      </c>
+      <c r="H426" s="4" t="inlineStr"/>
+      <c r="I426" s="4" t="inlineStr"/>
+      <c r="J426" s="4" t="inlineStr">
+        <is>
+          <t>14-year independent non-surgical aesthetics clinic with natural-results focus; repeat treatment clients, premium per-session fees</t>
+        </is>
+      </c>
+      <c r="K426" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L426" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M426" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N426" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O426" s="4" t="inlineStr">
+        <is>
+          <t>14-year trading history</t>
+        </is>
+      </c>
+      <c r="P426" s="4" t="inlineStr">
+        <is>
+          <t>Long heritage not yet leveraged as an AEO trust signal against newer Cheltenham aesthetics clinics</t>
+        </is>
+      </c>
+      <c r="Q426" s="4" t="inlineStr">
+        <is>
+          <t>'14 years of natural-results aesthetics in Cheltenham - own that AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R426" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S426" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T426" s="4" t="inlineStr"/>
+    </row>
+    <row r="427">
+      <c r="A427" s="2" t="inlineStr">
+        <is>
+          <t>Charles Lear &amp; Co</t>
+        </is>
+      </c>
+      <c r="B427" s="2" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C427" s="2" t="inlineStr">
+        <is>
+          <t>The Promenade, Cheltenham</t>
+        </is>
+      </c>
+      <c r="D427" s="2" t="inlineStr">
+        <is>
+          <t>https://www.charleslear.co.uk</t>
+        </is>
+      </c>
+      <c r="E427" s="2" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F427" s="2" t="inlineStr">
+        <is>
+          <t>01242 222722</t>
+        </is>
+      </c>
+      <c r="G427" s="2" t="inlineStr">
+        <is>
+          <t>Tom Hatcher (Director/Owner); founded 1992 by Charles Lear, trading roots to 1947</t>
+        </is>
+      </c>
+      <c r="H427" s="2" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/tom-hatcher-b045aa30</t>
+        </is>
+      </c>
+      <c r="I427" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/CharlesLearCo; instagram.com/charleslearco</t>
+        </is>
+      </c>
+      <c r="J427" s="2" t="inlineStr">
+        <is>
+          <t>Cheltenham's longest-established estate agent (roots to 1947), International Property Award winner; sales commissions on premium property are substantial</t>
+        </is>
+      </c>
+      <c r="K427" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L427" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M427" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N427" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O427" s="2" t="inlineStr">
+        <is>
+          <t>Facebook/Instagram presence; International Property Award win</t>
+        </is>
+      </c>
+      <c r="P427" s="2" t="inlineStr">
+        <is>
+          <t>Award-winning heritage brand not yet the AI-cited answer for 'estate agent Cheltenham'</t>
+        </is>
+      </c>
+      <c r="Q427" s="2" t="inlineStr">
+        <is>
+          <t>'International Property Award winner, trading since 1947 - own that AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R427" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S427" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T427" s="2" t="inlineStr">
+        <is>
+          <t>Strong heritage + award story, high-value AEO target</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" s="3" t="inlineStr">
+        <is>
+          <t>Osborne Heath</t>
+        </is>
+      </c>
+      <c r="B428" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C428" s="3" t="inlineStr">
+        <is>
+          <t>Sunninghill, Ascot &amp; Windsor</t>
+        </is>
+      </c>
+      <c r="D428" s="3" t="inlineStr">
+        <is>
+          <t>https://www.osborneheath.co.uk</t>
+        </is>
+      </c>
+      <c r="E428" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F428" s="3" t="inlineStr">
+        <is>
+          <t>01344 627777</t>
+        </is>
+      </c>
+      <c r="G428" s="3" t="inlineStr">
+        <is>
+          <t>James Niknejad (Founding Director, est. 2016)</t>
+        </is>
+      </c>
+      <c r="H428" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/james-niknejad-mnaea-038109117</t>
+        </is>
+      </c>
+      <c r="I428" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/osborneheathltd; instagram.com/osborneheath</t>
+        </is>
+      </c>
+      <c r="J428" s="3" t="inlineStr">
+        <is>
+          <t>Multi-award-winning independent luxury-homes agent in Ascot/Windsor; commissions on high-value property sales are substantial</t>
+        </is>
+      </c>
+      <c r="K428" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L428" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M428" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N428" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O428" s="3" t="inlineStr">
+        <is>
+          <t>Facebook/Instagram presence; multiple industry awards</t>
+        </is>
+      </c>
+      <c r="P428" s="3" t="inlineStr">
+        <is>
+          <t>Award-winning credentials not yet the AI-cited answer for 'estate agent Ascot'</t>
+        </is>
+      </c>
+      <c r="Q428" s="3" t="inlineStr">
+        <is>
+          <t>'Multi-award-winning luxury agent - own that AEO trust signal in Ascot/Windsor'</t>
+        </is>
+      </c>
+      <c r="R428" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S428" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T428" s="3" t="inlineStr"/>
+    </row>
+    <row r="429">
+      <c r="A429" s="3" t="inlineStr">
+        <is>
+          <t>Duncan Yeardley</t>
+        </is>
+      </c>
+      <c r="B429" s="3" t="inlineStr">
+        <is>
+          <t>Estate &amp; lettings agent</t>
+        </is>
+      </c>
+      <c r="C429" s="3" t="inlineStr">
+        <is>
+          <t>Sunninghill, Ascot (Ascot/Bracknell)</t>
+        </is>
+      </c>
+      <c r="D429" s="3" t="inlineStr">
+        <is>
+          <t>https://www.duncanyeardley.co.uk</t>
+        </is>
+      </c>
+      <c r="E429" s="3" t="inlineStr">
+        <is>
+          <t>nick@duncanyeardley.co.uk</t>
+        </is>
+      </c>
+      <c r="F429" s="3" t="inlineStr">
+        <is>
+          <t>01344 874300</t>
+        </is>
+      </c>
+      <c r="G429" s="3" t="inlineStr">
+        <is>
+          <t>Nick Thring (Owner, took over 2012; family affair with sister Helen &amp; wife Charlotte)</t>
+        </is>
+      </c>
+      <c r="H429" s="3" t="inlineStr"/>
+      <c r="I429" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/duncan.yeardley.estate.agent</t>
+        </is>
+      </c>
+      <c r="J429" s="3" t="inlineStr">
+        <is>
+          <t>38-year family-run estate agent trading since 1987 in Ascot/Bracknell; commissions on premium property sales recur</t>
+        </is>
+      </c>
+      <c r="K429" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L429" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M429" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N429" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O429" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence; long family-run history</t>
+        </is>
+      </c>
+      <c r="P429" s="3" t="inlineStr">
+        <is>
+          <t>'Real family affair' story not yet leveraged as an AEO trust signal</t>
+        </is>
+      </c>
+      <c r="Q429" s="3" t="inlineStr">
+        <is>
+          <t>'A real family affair since 1987 - own that AEO trust signal against corporate agents'</t>
+        </is>
+      </c>
+      <c r="R429" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S429" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T429" s="3" t="inlineStr"/>
+    </row>
+    <row r="430">
+      <c r="A430" s="4" t="inlineStr">
+        <is>
+          <t>The Bristol Driving School</t>
+        </is>
+      </c>
+      <c r="B430" s="4" t="inlineStr">
+        <is>
+          <t>Driving school &amp; ADI instructor training</t>
+        </is>
+      </c>
+      <c r="C430" s="4" t="inlineStr">
+        <is>
+          <t>Coombe Dingle, Bristol</t>
+        </is>
+      </c>
+      <c r="D430" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thebristoldrivingschool.com</t>
+        </is>
+      </c>
+      <c r="E430" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F430" s="4" t="inlineStr">
+        <is>
+          <t>0117 968 3344</t>
+        </is>
+      </c>
+      <c r="G430" s="4" t="inlineStr">
+        <is>
+          <t>Long-established, ORDIT founder member</t>
+        </is>
+      </c>
+      <c r="H430" s="4" t="inlineStr"/>
+      <c r="I430" s="4" t="inlineStr"/>
+      <c r="J430" s="4" t="inlineStr">
+        <is>
+          <t>~30-year Bristol driving school with a dedicated ADI (instructor) training arm; ORDIT/MSA-accredited, trainee-instructor course fees run into thousands per cohort</t>
+        </is>
+      </c>
+      <c r="K430" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L430" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M430" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N430" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O430" s="4" t="inlineStr">
+        <is>
+          <t>ORDIT founder-member status = established industry credibility</t>
+        </is>
+      </c>
+      <c r="P430" s="4" t="inlineStr">
+        <is>
+          <t>30-year heritage and ORDIT pedigree not yet the AI-cited answer for 'become a driving instructor Bristol'</t>
+        </is>
+      </c>
+      <c r="Q430" s="4" t="inlineStr">
+        <is>
+          <t>'A founder member of ORDIT - own that exact AEO trust signal for ADI training in Bristol'</t>
+        </is>
+      </c>
+      <c r="R430" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S430" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T430" s="4" t="inlineStr">
+        <is>
+          <t>Founder name unconfirmed via public search - verify before outreach</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" s="4" t="inlineStr">
+        <is>
+          <t>Sapphire Driving Academy</t>
+        </is>
+      </c>
+      <c r="B431" s="4" t="inlineStr">
+        <is>
+          <t>Driving school &amp; ADI instructor training</t>
+        </is>
+      </c>
+      <c r="C431" s="4" t="inlineStr">
+        <is>
+          <t>Harlington, Hayes, West London</t>
+        </is>
+      </c>
+      <c r="D431" s="4" t="inlineStr">
+        <is>
+          <t>https://sapphiredrivingacademy.co.uk</t>
+        </is>
+      </c>
+      <c r="E431" s="4" t="inlineStr">
+        <is>
+          <t>sapphiredrivingacademy@gmail.com</t>
+        </is>
+      </c>
+      <c r="F431" s="4" t="inlineStr">
+        <is>
+          <t>07596 786786</t>
+        </is>
+      </c>
+      <c r="G431" s="4" t="inlineStr">
+        <is>
+          <t>Nadia (Founder/Lead Trainer, ex-DVSA driving examiner)</t>
+        </is>
+      </c>
+      <c r="H431" s="4" t="inlineStr"/>
+      <c r="I431" s="4" t="inlineStr">
+        <is>
+          <t>facebook.com/p/Sapphire-Driving-Academy-100089952324304; instagram.com/sapphiredrivingacademy_</t>
+        </is>
+      </c>
+      <c r="J431" s="4" t="inlineStr">
+        <is>
+          <t>West London driving school with an ADI instructor-training arm led by an ex-DVSA examiner; ~100 instructors qualified to date, trainee course fees run into thousands per cohort</t>
+        </is>
+      </c>
+      <c r="K431" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L431" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M431" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N431" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O431" s="4" t="inlineStr">
+        <is>
+          <t>Facebook/Instagram presence</t>
+        </is>
+      </c>
+      <c r="P431" s="4" t="inlineStr">
+        <is>
+          <t>Ex-DVSA-examiner credential not yet the AI-cited trust signal for 'ADI training West London'</t>
+        </is>
+      </c>
+      <c r="Q431" s="4" t="inlineStr">
+        <is>
+          <t>'Trained by an ex-DVSA examiner - own that exact AEO credibility signal'</t>
+        </is>
+      </c>
+      <c r="R431" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S431" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T431" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T414"/>
+  <autoFilter ref="A1:T431"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -36336,7 +37916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B167"/>
+  <dimension ref="A1:B174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -36356,7 +37936,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>413</v>
+        <v>430</v>
       </c>
     </row>
     <row r="5">
@@ -36373,7 +37953,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7">
@@ -36519,17 +38099,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Law firm</t>
+          <t>Interior design studio</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Letting agent</t>
+          <t>Law firm</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -36539,7 +38119,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Private tuition agency</t>
+          <t>Letting agent</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -36549,7 +38129,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Osteopathy clinic</t>
+          <t>Private tuition agency</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -36559,7 +38139,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Electrician</t>
+          <t>Osteopathy clinic</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -36569,7 +38149,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Personal training studio</t>
+          <t>Electrician</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -36579,7 +38159,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Family law firm</t>
+          <t>Personal training studio</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -36589,7 +38169,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Chiropractor</t>
+          <t>Family law firm</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -36599,7 +38179,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Immigration law firm</t>
+          <t>Chiropractor</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -36609,7 +38189,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Independent optician</t>
+          <t>Immigration law firm</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -36619,7 +38199,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Pilates studio</t>
+          <t>Independent optician</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -36629,7 +38209,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Kitchen &amp; bathroom design</t>
+          <t>Pilates studio</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -36639,27 +38219,27 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Financial adviser / wealth management</t>
+          <t>Kitchen &amp; bathroom design</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Roofer</t>
+          <t>Architecture practice</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating / boilers</t>
+          <t>Financial adviser / wealth management</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -36669,7 +38249,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Event &amp; wedding caterer</t>
+          <t>Roofer</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -36679,7 +38259,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Estate agent (premium)</t>
+          <t>Plumbing &amp; heating / boilers</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -36689,7 +38269,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Orthodontist</t>
+          <t>Event &amp; wedding caterer</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -36699,7 +38279,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Employment law firm</t>
+          <t>Estate agent (premium)</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -36709,7 +38289,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Event management agency</t>
+          <t>Orthodontist</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -36719,7 +38299,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Design &amp; build</t>
+          <t>Employment law firm</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -36729,7 +38309,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Wealth management / IFA</t>
+          <t>Event management agency</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -36739,7 +38319,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Architects &amp; interior design</t>
+          <t>Design &amp; build</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -36749,7 +38329,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Funeral directors</t>
+          <t>Wealth management / IFA</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -36759,7 +38339,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Garden rooms / outbuildings</t>
+          <t>Architects &amp; interior design</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -36769,7 +38349,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Personal training gym</t>
+          <t>Funeral directors</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -36779,7 +38359,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Estate agent &amp; chartered surveyors</t>
+          <t>Garden rooms / outbuildings</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -36789,7 +38369,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Wedding &amp; event caterer</t>
+          <t>Personal training gym</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -36799,7 +38379,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Personal training</t>
+          <t>Estate agent &amp; chartered surveyors</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -36809,7 +38389,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Construction recruitment agency</t>
+          <t>Wedding &amp; event caterer</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -36819,7 +38399,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Legal recruitment agency</t>
+          <t>Personal training</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -36829,7 +38409,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>HGV driver training</t>
+          <t>Construction recruitment agency</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -36839,57 +38419,57 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Dentist / Orthodontics</t>
+          <t>Legal recruitment agency</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Specialist dental/implant clinic</t>
+          <t>HGV driver training</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Boutique corporate law firm</t>
+          <t>Private GP practice</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Cosmetic/aesthetics clinic</t>
+          <t>Aesthetics clinic (non-surgical)</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Skin &amp; laser clinic</t>
+          <t>Driving school &amp; ADI instructor training</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Mortgage broker / financial adviser</t>
+          <t>Dentist / Orthodontics</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -36899,7 +38479,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Architects (RIBA chartered)</t>
+          <t>Specialist dental/implant clinic</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -36909,7 +38489,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Recruitment agency (tech/startups)</t>
+          <t>Boutique corporate law firm</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -36919,7 +38499,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Recruitment agency (IT/data)</t>
+          <t>Cosmetic/aesthetics clinic</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -36929,7 +38509,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Independent vet (24/7 emergency)</t>
+          <t>Skin &amp; laser clinic</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -36939,7 +38519,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Interior design studio</t>
+          <t>Mortgage broker / financial adviser</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -36949,7 +38529,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Letting &amp; estate agent</t>
+          <t>Architects (RIBA chartered)</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -36959,7 +38539,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Cosmetic clinic (injectables)</t>
+          <t>Recruitment agency (tech/startups)</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -36969,7 +38549,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Cosmetic/anti-ageing clinic</t>
+          <t>Recruitment agency (IT/data)</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -36979,7 +38559,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Yoga &amp; reformer pilates studio</t>
+          <t>Independent vet (24/7 emergency)</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -36989,7 +38569,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Reformer pilates studio</t>
+          <t>Letting &amp; estate agent</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -36999,7 +38579,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Wealth management</t>
+          <t>Cosmetic clinic (injectables)</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -37009,7 +38589,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Private tuition &amp; education consultancy</t>
+          <t>Cosmetic/anti-ageing clinic</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -37019,7 +38599,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Osteopath</t>
+          <t>Yoga &amp; reformer pilates studio</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -37029,7 +38609,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Design &amp; build / home renovation</t>
+          <t>Reformer pilates studio</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -37039,7 +38619,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Builders / building contractor</t>
+          <t>Wealth management</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -37049,7 +38629,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Home care / live-in care</t>
+          <t>Private tuition &amp; education consultancy</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -37059,7 +38639,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Private day nurseries</t>
+          <t>Osteopath</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -37069,7 +38649,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Personal training &amp; wellness studio</t>
+          <t>Design &amp; build / home renovation</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -37079,7 +38659,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Mortgage &amp; insurance broker</t>
+          <t>Builders / building contractor</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -37089,7 +38669,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Business consultancy</t>
+          <t>Home care / live-in care</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -37099,7 +38679,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Interior designer (period homes)</t>
+          <t>Private day nurseries</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -37109,7 +38689,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Landscape design &amp; build</t>
+          <t>Personal training &amp; wellness studio</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -37119,7 +38699,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Interior designer</t>
+          <t>Mortgage &amp; insurance broker</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -37129,7 +38709,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Garden design &amp; landscaping</t>
+          <t>Business consultancy</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -37139,7 +38719,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Legal recruitment</t>
+          <t>Interior designer (period homes)</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -37149,7 +38729,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Independent gym &amp; health club</t>
+          <t>Landscape design &amp; build</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -37159,7 +38739,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Independent gym</t>
+          <t>Interior designer</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -37169,7 +38749,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Physiotherapy (sports)</t>
+          <t>Garden design &amp; landscaping</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -37179,7 +38759,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Letting agent / property management</t>
+          <t>Legal recruitment</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -37189,7 +38769,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Skin clinic</t>
+          <t>Independent gym &amp; health club</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -37199,7 +38779,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Tutoring company</t>
+          <t>Independent gym</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -37209,7 +38789,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Tutorial college &amp; exam centre</t>
+          <t>Physiotherapy (sports)</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -37219,7 +38799,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Employment law (disability discrimination)</t>
+          <t>Letting agent / property management</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -37229,7 +38809,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating</t>
+          <t>Skin clinic</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -37239,7 +38819,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Tutoring company</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -37249,7 +38829,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Sports physio &amp; massage</t>
+          <t>Tutorial college &amp; exam centre</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -37259,7 +38839,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Chartered surveyors (party wall/building)</t>
+          <t>Employment law (disability discrimination)</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -37269,7 +38849,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Chartered surveyors</t>
+          <t>Plumbing &amp; heating</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -37279,7 +38859,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Chartered building surveyors</t>
+          <t>Plumbing</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -37289,7 +38869,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Osteopathy clinics</t>
+          <t>Sports physio &amp; massage</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -37299,7 +38879,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Builders / renovations</t>
+          <t>Chartered surveyors (party wall/building)</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -37309,7 +38889,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Private nursery schools</t>
+          <t>Chartered surveyors</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -37319,7 +38899,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Private day nursery</t>
+          <t>Chartered building surveyors</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -37329,7 +38909,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Private GP (membership model)</t>
+          <t>Osteopathy clinics</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -37339,7 +38919,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Sash window restoration</t>
+          <t>Builders / renovations</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -37349,7 +38929,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Personal training (1:1)</t>
+          <t>Private nursery schools</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -37359,7 +38939,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Personal training &amp; nutrition coaching</t>
+          <t>Private day nursery</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -37369,7 +38949,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Private nursery/pre-prep school</t>
+          <t>Private GP (membership model)</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -37379,7 +38959,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Independent nursery (Montessori)</t>
+          <t>Sash window restoration</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -37389,7 +38969,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Live-in care agency</t>
+          <t>Personal training (1:1)</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -37399,7 +38979,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Law firm (conveyancing/family)</t>
+          <t>Personal training &amp; nutrition coaching</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -37409,7 +38989,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Architect &amp; interior designer</t>
+          <t>Private nursery/pre-prep school</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -37419,7 +38999,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Architects / project management</t>
+          <t>Independent nursery (Montessori)</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -37429,7 +39009,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>IFA / wealth management</t>
+          <t>Live-in care agency</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -37439,7 +39019,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Physiotherapy &amp; clinical Pilates</t>
+          <t>Law firm (conveyancing/family)</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -37449,7 +39029,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Aesthetics &amp; skin clinic</t>
+          <t>Architect &amp; interior designer</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -37459,7 +39039,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>IFA / financial planning</t>
+          <t>Architects / project management</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -37469,7 +39049,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Wealth management &amp; employee benefits</t>
+          <t>IFA / wealth management</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -37479,7 +39059,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Dermatology clinic</t>
+          <t>Physiotherapy &amp; clinical Pilates</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -37489,7 +39069,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Pilates studio (multi-site)</t>
+          <t>Aesthetics &amp; skin clinic</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -37499,7 +39079,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Private nursery (Montessori, multi-site)</t>
+          <t>IFA / financial planning</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -37509,7 +39089,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Law firm (wills &amp; probate)</t>
+          <t>Wealth management &amp; employee benefits</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -37519,7 +39099,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Business/technical consultancy</t>
+          <t>Dermatology clinic</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -37529,7 +39109,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Private/NHS dentist</t>
+          <t>Pilates studio (multi-site)</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -37539,7 +39119,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Removals company</t>
+          <t>Private nursery (Montessori, multi-site)</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -37549,7 +39129,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Driveways &amp; landscaping</t>
+          <t>Law firm (wills &amp; probate)</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -37559,7 +39139,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Wedding &amp; event venue</t>
+          <t>Business/technical consultancy</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -37569,7 +39149,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>IFA &amp; mortgage broker</t>
+          <t>Private/NHS dentist</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -37579,7 +39159,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Wedding photography &amp; videography</t>
+          <t>Removals company</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -37589,7 +39169,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Commercial property litigation law firm</t>
+          <t>Driveways &amp; landscaping</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -37599,7 +39179,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Recruitment agency (boutique)</t>
+          <t>Wedding &amp; event venue</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -37609,7 +39189,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Home cinema &amp; smart home installer</t>
+          <t>IFA &amp; mortgage broker</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -37619,7 +39199,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Home cinema installer</t>
+          <t>Wedding photography &amp; videography</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -37629,7 +39209,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Curtains, blinds &amp; upholstery</t>
+          <t>Commercial property litigation law firm</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -37639,7 +39219,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Bespoke curtains &amp; soft furnishings</t>
+          <t>Recruitment agency (boutique)</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -37649,7 +39229,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Wine merchant</t>
+          <t>Home cinema &amp; smart home installer</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -37659,7 +39239,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Education consultancy (school placement)</t>
+          <t>Home cinema installer</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -37669,7 +39249,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Estate agent &amp; surveyors</t>
+          <t>Curtains, blinds &amp; upholstery</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -37679,7 +39259,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Independent financial adviser</t>
+          <t>Bespoke curtains &amp; soft furnishings</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -37689,7 +39269,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Chartered accountants &amp; financial planners</t>
+          <t>Wine merchant</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -37699,7 +39279,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Private GP &amp; dermatology</t>
+          <t>Education consultancy (school placement)</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -37709,7 +39289,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Architects (heritage specialism)</t>
+          <t>Estate agent &amp; surveyors</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -37719,7 +39299,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Private cosmetic dentist / implants</t>
+          <t>Independent financial adviser</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -37729,7 +39309,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Heating engineer / plumbing</t>
+          <t>Chartered accountants &amp; financial planners</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -37739,7 +39319,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Estate agent (boutique)</t>
+          <t>Private GP &amp; dermatology</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -37749,7 +39329,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Independent vet (mixed practice)</t>
+          <t>Architects (heritage specialism)</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -37759,7 +39339,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Private dentist / cosmetic</t>
+          <t>Private cosmetic dentist / implants</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -37769,7 +39349,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Chartered accountants &amp; financial advisers</t>
+          <t>Heating engineer / plumbing</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -37779,7 +39359,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Healthcare recruitment agency</t>
+          <t>Estate agent (boutique)</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -37789,7 +39369,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Executive search / headhunting</t>
+          <t>Independent vet (mixed practice)</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -37799,7 +39379,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>First aid &amp; health &amp; safety training</t>
+          <t>Private dentist / cosmetic</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -37809,7 +39389,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Teaching &amp; education recruitment agency</t>
+          <t>Chartered accountants &amp; financial advisers</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -37819,7 +39399,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Supply teaching agency</t>
+          <t>Healthcare recruitment agency</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -37829,7 +39409,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Hospitality staffing agency</t>
+          <t>Executive search / headhunting</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -37839,7 +39419,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Finance &amp; accountancy recruitment agency</t>
+          <t>First aid &amp; health &amp; safety training</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -37849,7 +39429,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Accounting &amp; finance recruitment agency</t>
+          <t>Teaching &amp; education recruitment agency</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -37859,7 +39439,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Forklift &amp; plant operator training</t>
+          <t>Supply teaching agency</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -37869,7 +39449,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Forklift training</t>
+          <t>Hospitality staffing agency</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -37879,7 +39459,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Language school</t>
+          <t>Finance &amp; accountancy recruitment agency</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -37889,7 +39469,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Engineering &amp; manufacturing recruitment</t>
+          <t>Accounting &amp; finance recruitment agency</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -37899,7 +39479,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Business &amp; sales coaching</t>
+          <t>Forklift &amp; plant operator training</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -37909,7 +39489,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Engineering &amp; energy recruitment</t>
+          <t>Forklift training</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -37919,7 +39499,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Tech recruitment agency</t>
+          <t>Language school</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -37929,7 +39509,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Data/tech/AI recruitment agency</t>
+          <t>Engineering &amp; manufacturing recruitment</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -37939,7 +39519,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Beauty/aesthetics training academy</t>
+          <t>Business &amp; sales coaching</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -37949,7 +39529,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Beauty/hair training academy</t>
+          <t>Engineering &amp; energy recruitment</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -37959,7 +39539,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Medical aesthetics/injectable training academy</t>
+          <t>Tech recruitment agency</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -37969,7 +39549,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Yoga teacher training school</t>
+          <t>Data/tech/AI recruitment agency</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -37979,10 +39559,80 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
+          <t>Beauty/aesthetics training academy</t>
+        </is>
+      </c>
+      <c r="B167" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Beauty/hair training academy</t>
+        </is>
+      </c>
+      <c r="B168" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Medical aesthetics/injectable training academy</t>
+        </is>
+      </c>
+      <c r="B169" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Yoga teacher training school</t>
+        </is>
+      </c>
+      <c r="B170" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
           <t>Creative &amp; marketing recruitment agency</t>
         </is>
       </c>
-      <c r="B167" t="n">
+      <c r="B171" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Private dermatology &amp; women's health clinics</t>
+        </is>
+      </c>
+      <c r="B172" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Private dermatology practice</t>
+        </is>
+      </c>
+      <c r="B173" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Estate &amp; lettings agent</t>
+        </is>
+      </c>
+      <c r="B174" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batches 45-48: +17 prospects (447 total) - wedding venues, IFAs/mortgage brokers, vets, conveyancing solicitors
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$431</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$448</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T431"/>
+  <dimension ref="A1:T448"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -37904,8 +37904,1600 @@
       </c>
       <c r="T431" s="4" t="inlineStr"/>
     </row>
+    <row r="432">
+      <c r="A432" s="3" t="inlineStr">
+        <is>
+          <t>Jack's Barn</t>
+        </is>
+      </c>
+      <c r="B432" s="3" t="inlineStr">
+        <is>
+          <t>Wedding venue (converted barn)</t>
+        </is>
+      </c>
+      <c r="C432" s="3" t="inlineStr">
+        <is>
+          <t>Aldington, Ashford, Kent</t>
+        </is>
+      </c>
+      <c r="D432" s="3" t="inlineStr">
+        <is>
+          <t>https://www.jacksbarnkent.co.uk</t>
+        </is>
+      </c>
+      <c r="E432" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F432" s="3" t="inlineStr">
+        <is>
+          <t>07966 525067</t>
+        </is>
+      </c>
+      <c r="G432" s="3" t="inlineStr">
+        <is>
+          <t>Wanstall family (100+ years farming the land)</t>
+        </is>
+      </c>
+      <c r="H432" s="3" t="inlineStr"/>
+      <c r="I432" s="3" t="inlineStr">
+        <is>
+          <t>instagram.com/jacksbarnkent; facebook.com/jacksbarnkent</t>
+        </is>
+      </c>
+      <c r="J432" s="3" t="inlineStr">
+        <is>
+          <t>14th-century converted barn on a century-old family farm; wedding bookings run into thousands to tens of thousands per event</t>
+        </is>
+      </c>
+      <c r="K432" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L432" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M432" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N432" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O432" s="3" t="inlineStr">
+        <is>
+          <t>Instagram/Facebook presence = active marketing</t>
+        </is>
+      </c>
+      <c r="P432" s="3" t="inlineStr">
+        <is>
+          <t>Century-old family farm story not yet the AI-cited answer for 'barn wedding venue Kent'</t>
+        </is>
+      </c>
+      <c r="Q432" s="3" t="inlineStr">
+        <is>
+          <t>'A family farm for 100+ years, now Kent's most characterful barn wedding venue - own that AEO story'</t>
+        </is>
+      </c>
+      <c r="R432" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S432" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T432" s="3" t="inlineStr"/>
+    </row>
+    <row r="433">
+      <c r="A433" s="2" t="inlineStr">
+        <is>
+          <t>The Harty Estate</t>
+        </is>
+      </c>
+      <c r="B433" s="2" t="inlineStr">
+        <is>
+          <t>Wedding venue (waterside barn &amp; estate)</t>
+        </is>
+      </c>
+      <c r="C433" s="2" t="inlineStr">
+        <is>
+          <t>Isle of Sheppey, nr Faversham, Kent</t>
+        </is>
+      </c>
+      <c r="D433" s="2" t="inlineStr">
+        <is>
+          <t>https://www.thehartyestate.co.uk</t>
+        </is>
+      </c>
+      <c r="E433" s="2" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F433" s="2" t="inlineStr"/>
+      <c r="G433" s="2" t="inlineStr">
+        <is>
+          <t>Alex &amp; Victoria Burden (Third-generation family farm since 1960s)</t>
+        </is>
+      </c>
+      <c r="H433" s="2" t="inlineStr"/>
+      <c r="I433" s="2" t="inlineStr">
+        <is>
+          <t>instagram.com/thehartyestate; facebook.com/thehartyestate</t>
+        </is>
+      </c>
+      <c r="J433" s="2" t="inlineStr">
+        <is>
+          <t>Award-winning waterside estuary wedding venue on a third-generation family farm; bookings run into thousands to tens of thousands per event</t>
+        </is>
+      </c>
+      <c r="K433" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L433" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M433" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N433" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O433" s="2" t="inlineStr">
+        <is>
+          <t>2025 Kent Wedding Awards winner ('Wedding Venue of the Year') = active PR/marketing</t>
+        </is>
+      </c>
+      <c r="P433" s="2" t="inlineStr">
+        <is>
+          <t>Award win not yet the AI-cited trust signal for 'wedding venue Kent'</t>
+        </is>
+      </c>
+      <c r="Q433" s="2" t="inlineStr">
+        <is>
+          <t>'2025 Kent Wedding Venue of the Year - own that exact AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R433" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S433" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T433" s="2" t="inlineStr">
+        <is>
+          <t>Recent award win = strong AEO hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" s="3" t="inlineStr">
+        <is>
+          <t>Clock Barn</t>
+        </is>
+      </c>
+      <c r="B434" s="3" t="inlineStr">
+        <is>
+          <t>Wedding venue (thatched barn on working farm)</t>
+        </is>
+      </c>
+      <c r="C434" s="3" t="inlineStr">
+        <is>
+          <t>Whitchurch, Hampshire</t>
+        </is>
+      </c>
+      <c r="D434" s="3" t="inlineStr">
+        <is>
+          <t>https://www.clockbarn.co.uk</t>
+        </is>
+      </c>
+      <c r="E434" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F434" s="3" t="inlineStr">
+        <is>
+          <t>01256 630199</t>
+        </is>
+      </c>
+      <c r="G434" s="3" t="inlineStr">
+        <is>
+          <t>Family-run since 1997</t>
+        </is>
+      </c>
+      <c r="H434" s="3" t="inlineStr"/>
+      <c r="I434" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/ClockBarn</t>
+        </is>
+      </c>
+      <c r="J434" s="3" t="inlineStr">
+        <is>
+          <t>19th-century thatched barn venue on a working farm, hosting weddings since 2004; bookings run into thousands to tens of thousands per event</t>
+        </is>
+      </c>
+      <c r="K434" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L434" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M434" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N434" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O434" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence; 20+ year trading history</t>
+        </is>
+      </c>
+      <c r="P434" s="3" t="inlineStr">
+        <is>
+          <t>20-year heritage not yet the AI-cited answer for 'barn wedding venue Hampshire'</t>
+        </is>
+      </c>
+      <c r="Q434" s="3" t="inlineStr">
+        <is>
+          <t>'Hosting weddings since 2004 in our iconic thatched barn - own that AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R434" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S434" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T434" s="3" t="inlineStr"/>
+    </row>
+    <row r="435">
+      <c r="A435" s="3" t="inlineStr">
+        <is>
+          <t>Hollands Farm Weddings &amp; Events</t>
+        </is>
+      </c>
+      <c r="B435" s="3" t="inlineStr">
+        <is>
+          <t>Wedding venue (working farm)</t>
+        </is>
+      </c>
+      <c r="C435" s="3" t="inlineStr">
+        <is>
+          <t>Great Milton, Oxford</t>
+        </is>
+      </c>
+      <c r="D435" s="3" t="inlineStr">
+        <is>
+          <t>https://www.hollandsfarmevents.com</t>
+        </is>
+      </c>
+      <c r="E435" s="3" t="inlineStr">
+        <is>
+          <t>laura@hollandsfarmevents.com</t>
+        </is>
+      </c>
+      <c r="F435" s="3" t="inlineStr">
+        <is>
+          <t>07889 703791</t>
+        </is>
+      </c>
+      <c r="G435" s="3" t="inlineStr">
+        <is>
+          <t>Family-run (Laura, contact)</t>
+        </is>
+      </c>
+      <c r="H435" s="3" t="inlineStr"/>
+      <c r="I435" s="3" t="inlineStr">
+        <is>
+          <t>instagram.com/hollandsfarmevents</t>
+        </is>
+      </c>
+      <c r="J435" s="3" t="inlineStr">
+        <is>
+          <t>Family-owned rural wedding venue on a 500-acre working farm near the M40; bookings run into thousands to tens of thousands per event</t>
+        </is>
+      </c>
+      <c r="K435" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L435" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M435" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N435" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O435" s="3" t="inlineStr">
+        <is>
+          <t>Instagram presence</t>
+        </is>
+      </c>
+      <c r="P435" s="3" t="inlineStr">
+        <is>
+          <t>Working-farm setting not yet the AI-cited answer for 'wedding venue Oxfordshire'</t>
+        </is>
+      </c>
+      <c r="Q435" s="3" t="inlineStr">
+        <is>
+          <t>'A 500-acre working farm wedding venue - own that AEO story in Oxfordshire'</t>
+        </is>
+      </c>
+      <c r="R435" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S435" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T435" s="3" t="inlineStr"/>
+    </row>
+    <row r="436">
+      <c r="A436" s="3" t="inlineStr">
+        <is>
+          <t>Lains Barn</t>
+        </is>
+      </c>
+      <c r="B436" s="3" t="inlineStr">
+        <is>
+          <t>Wedding venue (restored historic barn)</t>
+        </is>
+      </c>
+      <c r="C436" s="3" t="inlineStr">
+        <is>
+          <t>Ardington, Wantage, Oxfordshire</t>
+        </is>
+      </c>
+      <c r="D436" s="3" t="inlineStr">
+        <is>
+          <t>https://www.lainsbarn.co.uk</t>
+        </is>
+      </c>
+      <c r="E436" s="3" t="inlineStr">
+        <is>
+          <t>events@lainsbarn.co.uk</t>
+        </is>
+      </c>
+      <c r="F436" s="3" t="inlineStr">
+        <is>
+          <t>01235 832745</t>
+        </is>
+      </c>
+      <c r="G436" s="3" t="inlineStr">
+        <is>
+          <t>Sherry family (Tom Sherry, Michelin-trained executive chef; 50+ yrs combined catering experience)</t>
+        </is>
+      </c>
+      <c r="H436" s="3" t="inlineStr"/>
+      <c r="I436" s="3" t="inlineStr">
+        <is>
+          <t>instagram.com/lainsbarn; facebook.com/lainsbarnoxfordshire</t>
+        </is>
+      </c>
+      <c r="J436" s="3" t="inlineStr">
+        <is>
+          <t>Award-winning restored barn venue with in-house Michelin-trained catering; bookings run into thousands to tens of thousands per event</t>
+        </is>
+      </c>
+      <c r="K436" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L436" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M436" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N436" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O436" s="3" t="inlineStr">
+        <is>
+          <t>Instagram (5.4k followers); Michelin-trained chef credential = strong PR asset</t>
+        </is>
+      </c>
+      <c r="P436" s="3" t="inlineStr">
+        <is>
+          <t>Michelin-trained chef story not yet the AI-cited answer for 'wedding venue Oxfordshire'</t>
+        </is>
+      </c>
+      <c r="Q436" s="3" t="inlineStr">
+        <is>
+          <t>'Michelin-trained catering at an award-winning barn venue - own that AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R436" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S436" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T436" s="3" t="inlineStr"/>
+    </row>
+    <row r="437">
+      <c r="A437" s="2" t="inlineStr">
+        <is>
+          <t>Partridge Muir &amp; Warren (PMW)</t>
+        </is>
+      </c>
+      <c r="B437" s="2" t="inlineStr">
+        <is>
+          <t>Chartered IFA / wealth management</t>
+        </is>
+      </c>
+      <c r="C437" s="2" t="inlineStr">
+        <is>
+          <t>Esher, Surrey</t>
+        </is>
+      </c>
+      <c r="D437" s="2" t="inlineStr">
+        <is>
+          <t>https://www.pmw.co.uk</t>
+        </is>
+      </c>
+      <c r="E437" s="2" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F437" s="2" t="inlineStr">
+        <is>
+          <t>01372 471550</t>
+        </is>
+      </c>
+      <c r="G437" s="2" t="inlineStr">
+        <is>
+          <t>Simon Lewis (CEO)</t>
+        </is>
+      </c>
+      <c r="H437" s="2" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/partridge-muir-&amp;-warren-ltd</t>
+        </is>
+      </c>
+      <c r="I437" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/pmwesher; instagram.com/pmwesher</t>
+        </is>
+      </c>
+      <c r="J437" s="2" t="inlineStr">
+        <is>
+          <t>Chartered financial planning firm trading since 1969 with generational family-client relationships; ongoing wealth-management fees run into thousands annually per client</t>
+        </is>
+      </c>
+      <c r="K437" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L437" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M437" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N437" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O437" s="2" t="inlineStr">
+        <is>
+          <t>Facebook/Instagram presence; Chartered status; 55+ year heritage</t>
+        </is>
+      </c>
+      <c r="P437" s="2" t="inlineStr">
+        <is>
+          <t>55-year heritage not yet the AI-cited answer for 'financial planner Esher'</t>
+        </is>
+      </c>
+      <c r="Q437" s="2" t="inlineStr">
+        <is>
+          <t>'Advising Esher families since 1969, now into the second generation - own that AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R437" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S437" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T437" s="2" t="inlineStr">
+        <is>
+          <t>Exceptional heritage (56 yrs) - high-value AEO opportunity</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" s="3" t="inlineStr">
+        <is>
+          <t>Heritage Independent Mortgage Advisers</t>
+        </is>
+      </c>
+      <c r="B438" s="3" t="inlineStr">
+        <is>
+          <t>Independent mortgage broker</t>
+        </is>
+      </c>
+      <c r="C438" s="3" t="inlineStr">
+        <is>
+          <t>Guildford, Surrey</t>
+        </is>
+      </c>
+      <c r="D438" s="3" t="inlineStr">
+        <is>
+          <t>https://www.heritageima.com</t>
+        </is>
+      </c>
+      <c r="E438" s="3" t="inlineStr">
+        <is>
+          <t>info@heritageima.com</t>
+        </is>
+      </c>
+      <c r="F438" s="3" t="inlineStr">
+        <is>
+          <t>01483 531025</t>
+        </is>
+      </c>
+      <c r="G438" s="3" t="inlineStr">
+        <is>
+          <t>Paul Glover (Director)</t>
+        </is>
+      </c>
+      <c r="H438" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/heritage-independent-mortgage-advisers</t>
+        </is>
+      </c>
+      <c r="I438" s="3" t="inlineStr"/>
+      <c r="J438" s="3" t="inlineStr">
+        <is>
+          <t>Whole-of-market independent mortgage broker (residential/BTL/equity release/specialist lending) since 2000; commission per completed mortgage recurs with remortgage clients</t>
+        </is>
+      </c>
+      <c r="K438" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L438" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M438" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N438" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O438" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn presence; 25-year trading history</t>
+        </is>
+      </c>
+      <c r="P438" s="3" t="inlineStr">
+        <is>
+          <t>25-year heritage not yet the AI-cited answer for 'mortgage broker Guildford'</t>
+        </is>
+      </c>
+      <c r="Q438" s="3" t="inlineStr">
+        <is>
+          <t>'25 years of whole-of-market mortgage advice in Guildford - own that AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R438" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S438" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T438" s="3" t="inlineStr"/>
+    </row>
+    <row r="439">
+      <c r="A439" s="4" t="inlineStr">
+        <is>
+          <t>C A Financial Services</t>
+        </is>
+      </c>
+      <c r="B439" s="4" t="inlineStr">
+        <is>
+          <t>Independent financial planning</t>
+        </is>
+      </c>
+      <c r="C439" s="4" t="inlineStr">
+        <is>
+          <t>Kemsing, Sevenoaks, Kent</t>
+        </is>
+      </c>
+      <c r="D439" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cafinancialservices.co.uk</t>
+        </is>
+      </c>
+      <c r="E439" s="4" t="inlineStr">
+        <is>
+          <t>craig.atkins@cafinancialservices.co.uk</t>
+        </is>
+      </c>
+      <c r="F439" s="4" t="inlineStr">
+        <is>
+          <t>01732 617950</t>
+        </is>
+      </c>
+      <c r="G439" s="4" t="inlineStr">
+        <is>
+          <t>Craig Atkins (Founder/Owner, est. 2007)</t>
+        </is>
+      </c>
+      <c r="H439" s="4" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/c-a-financial-services</t>
+        </is>
+      </c>
+      <c r="I439" s="4" t="inlineStr">
+        <is>
+          <t>facebook.com/cafsuk</t>
+        </is>
+      </c>
+      <c r="J439" s="4" t="inlineStr">
+        <is>
+          <t>Sole-owned independent financial planning practice (pensions/investments/tax/protection/estate planning); ongoing wealth-management fees run into thousands annually per client</t>
+        </is>
+      </c>
+      <c r="K439" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L439" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M439" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N439" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O439" s="4" t="inlineStr">
+        <is>
+          <t>Facebook/LinkedIn presence; 18-year trading history</t>
+        </is>
+      </c>
+      <c r="P439" s="4" t="inlineStr">
+        <is>
+          <t>18-year sole-practitioner heritage not yet the AI-cited answer for 'financial adviser Sevenoaks'</t>
+        </is>
+      </c>
+      <c r="Q439" s="4" t="inlineStr">
+        <is>
+          <t>'18 years of independent financial planning in Sevenoaks - own that AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R439" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S439" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T439" s="4" t="inlineStr"/>
+    </row>
+    <row r="440">
+      <c r="A440" s="3" t="inlineStr">
+        <is>
+          <t>Isis Financial Planners</t>
+        </is>
+      </c>
+      <c r="B440" s="3" t="inlineStr">
+        <is>
+          <t>Chartered independent financial planners</t>
+        </is>
+      </c>
+      <c r="C440" s="3" t="inlineStr">
+        <is>
+          <t>Farmoor, Oxford</t>
+        </is>
+      </c>
+      <c r="D440" s="3" t="inlineStr">
+        <is>
+          <t>https://www.isisfp.co.uk</t>
+        </is>
+      </c>
+      <c r="E440" s="3" t="inlineStr">
+        <is>
+          <t>postbox@isisfp.co.uk</t>
+        </is>
+      </c>
+      <c r="F440" s="3" t="inlineStr">
+        <is>
+          <t>01865 655980</t>
+        </is>
+      </c>
+      <c r="G440" s="3" t="inlineStr">
+        <is>
+          <t>Louis Letourneau (Founder, Chartered Financial Planner, est. 2002)</t>
+        </is>
+      </c>
+      <c r="H440" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/isis-financial-planners-limited</t>
+        </is>
+      </c>
+      <c r="I440" s="3" t="inlineStr"/>
+      <c r="J440" s="3" t="inlineStr">
+        <is>
+          <t>Chartered wealth-management/retirement-planning firm trading since 2002; ongoing wealth-management fees run into thousands annually per client</t>
+        </is>
+      </c>
+      <c r="K440" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L440" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M440" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N440" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O440" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn presence; Chartered status; 23-year heritage</t>
+        </is>
+      </c>
+      <c r="P440" s="3" t="inlineStr">
+        <is>
+          <t>23-year heritage not yet the AI-cited answer for 'financial planner Oxford'</t>
+        </is>
+      </c>
+      <c r="Q440" s="3" t="inlineStr">
+        <is>
+          <t>'23 years of Chartered financial planning in Oxford - own that AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R440" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S440" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T440" s="3" t="inlineStr"/>
+    </row>
+    <row r="441">
+      <c r="A441" s="3" t="inlineStr">
+        <is>
+          <t>Pattenden Vets</t>
+        </is>
+      </c>
+      <c r="B441" s="3" t="inlineStr">
+        <is>
+          <t>Veterinary practice</t>
+        </is>
+      </c>
+      <c r="C441" s="3" t="inlineStr">
+        <is>
+          <t>Marden, Kent</t>
+        </is>
+      </c>
+      <c r="D441" s="3" t="inlineStr">
+        <is>
+          <t>https://www.pattendenvets.com</t>
+        </is>
+      </c>
+      <c r="E441" s="3" t="inlineStr">
+        <is>
+          <t>info@pattendenvets.com</t>
+        </is>
+      </c>
+      <c r="F441" s="3" t="inlineStr">
+        <is>
+          <t>01622 397900</t>
+        </is>
+      </c>
+      <c r="G441" s="3" t="inlineStr">
+        <is>
+          <t>Dr Lara Hummel, Robert Everitt, Dr Laura Heasman &amp; Dr Vanessa Martin MRCVS (Directors, est. 2018)</t>
+        </is>
+      </c>
+      <c r="H441" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/pattenden-vets</t>
+        </is>
+      </c>
+      <c r="I441" s="3" t="inlineStr">
+        <is>
+          <t>instagram.com/pattendenvets; facebook.com/pattendenvets</t>
+        </is>
+      </c>
+      <c r="J441" s="3" t="inlineStr">
+        <is>
+          <t>Independent small-animal/exotic practice recently celebrating its 7th anniversary; consultation/treatment fees plus repeat annual health-plan clients</t>
+        </is>
+      </c>
+      <c r="K441" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L441" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M441" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N441" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O441" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn/Instagram/Facebook presence = active marketing investment</t>
+        </is>
+      </c>
+      <c r="P441" s="3" t="inlineStr">
+        <is>
+          <t>Multi-channel social presence not yet converted into AI-cited answers for 'vet Marden'</t>
+        </is>
+      </c>
+      <c r="Q441" s="3" t="inlineStr">
+        <is>
+          <t>'You're already active on 3 platforms - let's make AI cite you for local vet searches too'</t>
+        </is>
+      </c>
+      <c r="R441" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S441" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T441" s="3" t="inlineStr"/>
+    </row>
+    <row r="442">
+      <c r="A442" s="4" t="inlineStr">
+        <is>
+          <t>Surrey Family Vets</t>
+        </is>
+      </c>
+      <c r="B442" s="4" t="inlineStr">
+        <is>
+          <t>Veterinary practice</t>
+        </is>
+      </c>
+      <c r="C442" s="4" t="inlineStr">
+        <is>
+          <t>Jacobs Well, Guildford, Surrey</t>
+        </is>
+      </c>
+      <c r="D442" s="4" t="inlineStr">
+        <is>
+          <t>https://www.surreyfamilyvets.co.uk</t>
+        </is>
+      </c>
+      <c r="E442" s="4" t="inlineStr">
+        <is>
+          <t>hello@surreyfamilyvets.co.uk</t>
+        </is>
+      </c>
+      <c r="F442" s="4" t="inlineStr">
+        <is>
+          <t>01483 322023</t>
+        </is>
+      </c>
+      <c r="G442" s="4" t="inlineStr">
+        <is>
+          <t>Natalia &amp; Marcos (Husband-and-wife founders)</t>
+        </is>
+      </c>
+      <c r="H442" s="4" t="inlineStr"/>
+      <c r="I442" s="4" t="inlineStr">
+        <is>
+          <t>instagram.com/surreyfamilyvets; facebook.com/SurreyFamilyVets</t>
+        </is>
+      </c>
+      <c r="J442" s="4" t="inlineStr">
+        <is>
+          <t>Husband-and-wife independent practice with on-site diagnostics and keyhole surgery; consultation/treatment fees plus repeat annual health-plan clients</t>
+        </is>
+      </c>
+      <c r="K442" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L442" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M442" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N442" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O442" s="4" t="inlineStr">
+        <is>
+          <t>Instagram/Facebook presence</t>
+        </is>
+      </c>
+      <c r="P442" s="4" t="inlineStr">
+        <is>
+          <t>Husband-and-wife story not yet the AI-cited trust signal for 'vet Guildford'</t>
+        </is>
+      </c>
+      <c r="Q442" s="4" t="inlineStr">
+        <is>
+          <t>'A husband-and-wife vet team you can trust - own that AEO story in Guildford'</t>
+        </is>
+      </c>
+      <c r="R442" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S442" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T442" s="4" t="inlineStr">
+        <is>
+          <t>Confirm Companies House entry before outreach</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" s="3" t="inlineStr">
+        <is>
+          <t>Iffley Vets</t>
+        </is>
+      </c>
+      <c r="B443" s="3" t="inlineStr">
+        <is>
+          <t>Veterinary practice (small independent group)</t>
+        </is>
+      </c>
+      <c r="C443" s="3" t="inlineStr">
+        <is>
+          <t>Oxford &amp; Wheatley, Oxfordshire</t>
+        </is>
+      </c>
+      <c r="D443" s="3" t="inlineStr">
+        <is>
+          <t>https://www.iffleyvets.com</t>
+        </is>
+      </c>
+      <c r="E443" s="3" t="inlineStr">
+        <is>
+          <t>info@iffleyvets.com</t>
+        </is>
+      </c>
+      <c r="F443" s="3" t="inlineStr">
+        <is>
+          <t>01865 242600</t>
+        </is>
+      </c>
+      <c r="G443" s="3" t="inlineStr">
+        <is>
+          <t>Andrew Bartholomew, Katharine Morrison &amp; Cameron Forbes MRCVS (Vet-owner directors, part of DNA Vetcare)</t>
+        </is>
+      </c>
+      <c r="H443" s="3" t="inlineStr"/>
+      <c r="I443" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/p/Iffley-Vets-Oxford-Wheatley</t>
+        </is>
+      </c>
+      <c r="J443" s="3" t="inlineStr">
+        <is>
+          <t>Vet-owned two-site independent group (not PE/corporate-backed) named 'Best Vets in Oxfordshire 2026'; consultation/treatment fees plus repeat annual health-plan clients</t>
+        </is>
+      </c>
+      <c r="K443" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L443" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M443" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N443" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O443" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence; recent 'Best Vets in Oxfordshire 2026' award</t>
+        </is>
+      </c>
+      <c r="P443" s="3" t="inlineStr">
+        <is>
+          <t>Award win not yet the AI-cited trust signal for 'vet Oxford'</t>
+        </is>
+      </c>
+      <c r="Q443" s="3" t="inlineStr">
+        <is>
+          <t>'Best Vets in Oxfordshire 2026 - own that exact AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R443" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S443" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T443" s="3" t="inlineStr">
+        <is>
+          <t>Small owner-vet group (DNA Vetcare), not corporate-chain owned</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" s="3" t="inlineStr">
+        <is>
+          <t>Capstone Solicitors</t>
+        </is>
+      </c>
+      <c r="B444" s="3" t="inlineStr">
+        <is>
+          <t>Law firm (conveyancing, family, private client)</t>
+        </is>
+      </c>
+      <c r="C444" s="3" t="inlineStr">
+        <is>
+          <t>Bishopston, Bristol</t>
+        </is>
+      </c>
+      <c r="D444" s="3" t="inlineStr">
+        <is>
+          <t>https://www.capstonelaw.co.uk</t>
+        </is>
+      </c>
+      <c r="E444" s="3" t="inlineStr">
+        <is>
+          <t>enquiries@capstonelaw.co.uk</t>
+        </is>
+      </c>
+      <c r="F444" s="3" t="inlineStr">
+        <is>
+          <t>0117 942 8214</t>
+        </is>
+      </c>
+      <c r="G444" s="3" t="inlineStr">
+        <is>
+          <t>Richard Vooght &amp; Rob Wilson (Partners; office trading continuously since 1973)</t>
+        </is>
+      </c>
+      <c r="H444" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/capstone-solicitors</t>
+        </is>
+      </c>
+      <c r="I444" s="3" t="inlineStr"/>
+      <c r="J444" s="3" t="inlineStr">
+        <is>
+          <t>Independent Bristol firm with roots to 1973 (rebranded 2013), grows entirely by referral with no third-party lead-buying; conveyancing fees plus private-client work recur</t>
+        </is>
+      </c>
+      <c r="K444" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L444" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M444" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N444" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O444" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn presence; 50+ year trading roots</t>
+        </is>
+      </c>
+      <c r="P444" s="3" t="inlineStr">
+        <is>
+          <t>50-year heritage not yet the AI-cited answer for 'solicitor Bristol'</t>
+        </is>
+      </c>
+      <c r="Q444" s="3" t="inlineStr">
+        <is>
+          <t>'Trading since 1973, no lead-buying, pure reputation - own that AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R444" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S444" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T444" s="3" t="inlineStr"/>
+    </row>
+    <row r="445">
+      <c r="A445" s="4" t="inlineStr">
+        <is>
+          <t>Beaufort Montague Harris (BMH Solicitors)</t>
+        </is>
+      </c>
+      <c r="B445" s="4" t="inlineStr">
+        <is>
+          <t>Law firm (conveyancing, private client)</t>
+        </is>
+      </c>
+      <c r="C445" s="4" t="inlineStr">
+        <is>
+          <t>Bath</t>
+        </is>
+      </c>
+      <c r="D445" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bmhsolicitors.co.uk</t>
+        </is>
+      </c>
+      <c r="E445" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F445" s="4" t="inlineStr">
+        <is>
+          <t>01225 667648</t>
+        </is>
+      </c>
+      <c r="G445" s="4" t="inlineStr">
+        <is>
+          <t>Geraint James (Owner)</t>
+        </is>
+      </c>
+      <c r="H445" s="4" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/geraint-james-8b9b6414</t>
+        </is>
+      </c>
+      <c r="I445" s="4" t="inlineStr"/>
+      <c r="J445" s="4" t="inlineStr">
+        <is>
+          <t>Single-office Bath firm formed via 2019 merger of two established local practices; conveyancing fees plus private-client work recur</t>
+        </is>
+      </c>
+      <c r="K445" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L445" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M445" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N445" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O445" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P445" s="4" t="inlineStr">
+        <is>
+          <t>Merger of two established firms not yet leveraged as an AEO trust signal</t>
+        </is>
+      </c>
+      <c r="Q445" s="4" t="inlineStr">
+        <is>
+          <t>'Two established Bath firms, now one - own that combined-heritage AEO story'</t>
+        </is>
+      </c>
+      <c r="R445" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S445" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T445" s="4" t="inlineStr"/>
+    </row>
+    <row r="446">
+      <c r="A446" s="4" t="inlineStr">
+        <is>
+          <t>Surrey Property Lawyers</t>
+        </is>
+      </c>
+      <c r="B446" s="4" t="inlineStr">
+        <is>
+          <t>Conveyancing solicitors</t>
+        </is>
+      </c>
+      <c r="C446" s="4" t="inlineStr">
+        <is>
+          <t>Onslow Village, Guildford, Surrey</t>
+        </is>
+      </c>
+      <c r="D446" s="4" t="inlineStr">
+        <is>
+          <t>https://www.surreypropertylawyers.co.uk</t>
+        </is>
+      </c>
+      <c r="E446" s="4" t="inlineStr">
+        <is>
+          <t>info@surreypropertylawyers.co.uk</t>
+        </is>
+      </c>
+      <c r="F446" s="4" t="inlineStr">
+        <is>
+          <t>01483 485800</t>
+        </is>
+      </c>
+      <c r="G446" s="4" t="inlineStr">
+        <is>
+          <t>Catherine Fewings &amp; Amanda (Team)</t>
+        </is>
+      </c>
+      <c r="H446" s="4" t="inlineStr"/>
+      <c r="I446" s="4" t="inlineStr">
+        <is>
+          <t>facebook.com/SurreyPropertyLawyers</t>
+        </is>
+      </c>
+      <c r="J446" s="4" t="inlineStr">
+        <is>
+          <t>Boutique conveyancing-only specialist built on client reviews/local reputation rather than volume; conveyancing fees per transaction, repeat referral clients</t>
+        </is>
+      </c>
+      <c r="K446" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L446" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M446" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N446" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O446" s="4" t="inlineStr">
+        <is>
+          <t>Facebook presence</t>
+        </is>
+      </c>
+      <c r="P446" s="4" t="inlineStr">
+        <is>
+          <t>Review-driven growth not yet converted into AI-cited answers for 'conveyancing solicitor Guildford'</t>
+        </is>
+      </c>
+      <c r="Q446" s="4" t="inlineStr">
+        <is>
+          <t>'Built on 5-star reviews, not volume - let's make AI cite those reviews too'</t>
+        </is>
+      </c>
+      <c r="R446" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S446" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T446" s="4" t="inlineStr"/>
+    </row>
+    <row r="447">
+      <c r="A447" s="4" t="inlineStr">
+        <is>
+          <t>Hunter Peddell Property Law</t>
+        </is>
+      </c>
+      <c r="B447" s="4" t="inlineStr">
+        <is>
+          <t>Law firm (residential &amp; commercial property)</t>
+        </is>
+      </c>
+      <c r="C447" s="4" t="inlineStr">
+        <is>
+          <t>Claygate, Esher, Surrey</t>
+        </is>
+      </c>
+      <c r="D447" s="4" t="inlineStr">
+        <is>
+          <t>via directory listing</t>
+        </is>
+      </c>
+      <c r="E447" s="4" t="inlineStr">
+        <is>
+          <t>ihunter@hpplaw.co.uk</t>
+        </is>
+      </c>
+      <c r="F447" s="4" t="inlineStr">
+        <is>
+          <t>01372 477900</t>
+        </is>
+      </c>
+      <c r="G447" s="4" t="inlineStr">
+        <is>
+          <t>Ian Hunter (Partner, solicitor since 1980) &amp; Loretta Peddell (Partner, 35+ yrs experience)</t>
+        </is>
+      </c>
+      <c r="H447" s="4" t="inlineStr"/>
+      <c r="I447" s="4" t="inlineStr"/>
+      <c r="J447" s="4" t="inlineStr">
+        <is>
+          <t>Long-standing two-partner practice with 40+ years combined local experience serving Esher/Claygate/Cobham; conveyancing fees per transaction, repeat local-client referrals</t>
+        </is>
+      </c>
+      <c r="K447" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L447" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M447" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N447" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O447" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P447" s="4" t="inlineStr">
+        <is>
+          <t>40+ years combined experience not yet leveraged as an AEO trust signal in a no-website/no-social firm</t>
+        </is>
+      </c>
+      <c r="Q447" s="4" t="inlineStr">
+        <is>
+          <t>'40+ years of combined Esher property law experience - own that AEO trust signal, starting with a stronger web presence'</t>
+        </is>
+      </c>
+      <c r="R447" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S447" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T447" s="4" t="inlineStr">
+        <is>
+          <t>No website/social presence found - verify a live site exists before outreach</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" s="3" t="inlineStr">
+        <is>
+          <t>Cunningham Eves Solicitors</t>
+        </is>
+      </c>
+      <c r="B448" s="3" t="inlineStr">
+        <is>
+          <t>Law firm (conveyancing, private client, family)</t>
+        </is>
+      </c>
+      <c r="C448" s="3" t="inlineStr">
+        <is>
+          <t>Leatherhead &amp; Dorking, Surrey</t>
+        </is>
+      </c>
+      <c r="D448" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cunninghameves.com</t>
+        </is>
+      </c>
+      <c r="E448" s="3" t="inlineStr">
+        <is>
+          <t>info@cunninghameves.com</t>
+        </is>
+      </c>
+      <c r="F448" s="3" t="inlineStr">
+        <is>
+          <t>01372 897857</t>
+        </is>
+      </c>
+      <c r="G448" s="3" t="inlineStr">
+        <is>
+          <t>Richard Cunningham (Managing Partner) &amp; Christine Eves (Senior Partner); founded 2020/21 by 4 partners</t>
+        </is>
+      </c>
+      <c r="H448" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/cunningham-eves-solicitors</t>
+        </is>
+      </c>
+      <c r="I448" s="3" t="inlineStr">
+        <is>
+          <t>instagram.com/cunninghamevessolicitors; facebook.com/CunninghamEvesSolicitors</t>
+        </is>
+      </c>
+      <c r="J448" s="3" t="inlineStr">
+        <is>
+          <t>Fast-growing two-office firm founded by 4 partners with a decade+ working together previously; conveyancing/private-client/family fees recur across the Cobham/Leatherhead/Dorking corridor</t>
+        </is>
+      </c>
+      <c r="K448" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L448" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M448" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N448" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O448" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn/Instagram/Facebook presence = active marketing investment</t>
+        </is>
+      </c>
+      <c r="P448" s="3" t="inlineStr">
+        <is>
+          <t>Rapid organic growth not yet matched by AI-search dominance across 2 offices</t>
+        </is>
+      </c>
+      <c r="Q448" s="3" t="inlineStr">
+        <is>
+          <t>'You grew from 4 partners to 2 offices by reputation - let's make AI cite you the same way'</t>
+        </is>
+      </c>
+      <c r="R448" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S448" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T448" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T431"/>
+  <autoFilter ref="A1:T448"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -37916,7 +39508,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B174"/>
+  <dimension ref="A1:B190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -37936,7 +39528,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>430</v>
+        <v>447</v>
       </c>
     </row>
     <row r="5">
@@ -38469,17 +40061,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Dentist / Orthodontics</t>
+          <t>Veterinary practice</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Specialist dental/implant clinic</t>
+          <t>Dentist / Orthodontics</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -38489,7 +40081,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Boutique corporate law firm</t>
+          <t>Specialist dental/implant clinic</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -38499,7 +40091,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Cosmetic/aesthetics clinic</t>
+          <t>Boutique corporate law firm</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -38509,7 +40101,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Skin &amp; laser clinic</t>
+          <t>Cosmetic/aesthetics clinic</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -38519,7 +40111,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Mortgage broker / financial adviser</t>
+          <t>Skin &amp; laser clinic</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -38529,7 +40121,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Architects (RIBA chartered)</t>
+          <t>Mortgage broker / financial adviser</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -38539,7 +40131,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Recruitment agency (tech/startups)</t>
+          <t>Architects (RIBA chartered)</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -38549,7 +40141,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Recruitment agency (IT/data)</t>
+          <t>Recruitment agency (tech/startups)</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -38559,7 +40151,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Independent vet (24/7 emergency)</t>
+          <t>Recruitment agency (IT/data)</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -38569,7 +40161,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Letting &amp; estate agent</t>
+          <t>Independent vet (24/7 emergency)</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -38579,7 +40171,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Cosmetic clinic (injectables)</t>
+          <t>Letting &amp; estate agent</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -38589,7 +40181,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Cosmetic/anti-ageing clinic</t>
+          <t>Cosmetic clinic (injectables)</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -38599,7 +40191,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Yoga &amp; reformer pilates studio</t>
+          <t>Cosmetic/anti-ageing clinic</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -38609,7 +40201,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Reformer pilates studio</t>
+          <t>Yoga &amp; reformer pilates studio</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -38619,7 +40211,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Wealth management</t>
+          <t>Reformer pilates studio</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -38629,7 +40221,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Private tuition &amp; education consultancy</t>
+          <t>Wealth management</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -38639,7 +40231,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Osteopath</t>
+          <t>Private tuition &amp; education consultancy</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -38649,7 +40241,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Design &amp; build / home renovation</t>
+          <t>Osteopath</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -38659,7 +40251,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Builders / building contractor</t>
+          <t>Design &amp; build / home renovation</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -38669,7 +40261,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Home care / live-in care</t>
+          <t>Builders / building contractor</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -38679,7 +40271,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Private day nurseries</t>
+          <t>Home care / live-in care</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -38689,7 +40281,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Personal training &amp; wellness studio</t>
+          <t>Private day nurseries</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -38699,7 +40291,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Mortgage &amp; insurance broker</t>
+          <t>Personal training &amp; wellness studio</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -38709,7 +40301,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Business consultancy</t>
+          <t>Mortgage &amp; insurance broker</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -38719,7 +40311,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Interior designer (period homes)</t>
+          <t>Business consultancy</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -38729,7 +40321,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Landscape design &amp; build</t>
+          <t>Interior designer (period homes)</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -38739,7 +40331,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Interior designer</t>
+          <t>Landscape design &amp; build</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -38749,7 +40341,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Garden design &amp; landscaping</t>
+          <t>Interior designer</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -38759,7 +40351,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Legal recruitment</t>
+          <t>Garden design &amp; landscaping</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -38769,7 +40361,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Independent gym &amp; health club</t>
+          <t>Legal recruitment</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -38779,7 +40371,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Independent gym</t>
+          <t>Independent gym &amp; health club</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -38789,7 +40381,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Physiotherapy (sports)</t>
+          <t>Independent gym</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -38799,7 +40391,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Letting agent / property management</t>
+          <t>Physiotherapy (sports)</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -38809,7 +40401,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Skin clinic</t>
+          <t>Letting agent / property management</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -38819,7 +40411,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Tutoring company</t>
+          <t>Skin clinic</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -38829,7 +40421,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Tutorial college &amp; exam centre</t>
+          <t>Tutoring company</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -38839,7 +40431,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Employment law (disability discrimination)</t>
+          <t>Tutorial college &amp; exam centre</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -38849,7 +40441,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating</t>
+          <t>Employment law (disability discrimination)</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -38859,7 +40451,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Plumbing &amp; heating</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -38869,7 +40461,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Sports physio &amp; massage</t>
+          <t>Plumbing</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -38879,7 +40471,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Chartered surveyors (party wall/building)</t>
+          <t>Sports physio &amp; massage</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -38889,7 +40481,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Chartered surveyors</t>
+          <t>Chartered surveyors (party wall/building)</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -38899,7 +40491,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Chartered building surveyors</t>
+          <t>Chartered surveyors</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -38909,7 +40501,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Osteopathy clinics</t>
+          <t>Chartered building surveyors</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -38919,7 +40511,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Builders / renovations</t>
+          <t>Osteopathy clinics</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -38929,7 +40521,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Private nursery schools</t>
+          <t>Builders / renovations</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -38939,7 +40531,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Private day nursery</t>
+          <t>Private nursery schools</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -38949,7 +40541,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Private GP (membership model)</t>
+          <t>Private day nursery</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -38959,7 +40551,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Sash window restoration</t>
+          <t>Private GP (membership model)</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -38969,7 +40561,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Personal training (1:1)</t>
+          <t>Sash window restoration</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -38979,7 +40571,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Personal training &amp; nutrition coaching</t>
+          <t>Personal training (1:1)</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -38989,7 +40581,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Private nursery/pre-prep school</t>
+          <t>Personal training &amp; nutrition coaching</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -38999,7 +40591,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Independent nursery (Montessori)</t>
+          <t>Private nursery/pre-prep school</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -39009,7 +40601,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Live-in care agency</t>
+          <t>Independent nursery (Montessori)</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -39019,7 +40611,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Law firm (conveyancing/family)</t>
+          <t>Live-in care agency</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -39029,7 +40621,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Architect &amp; interior designer</t>
+          <t>Law firm (conveyancing/family)</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -39039,7 +40631,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Architects / project management</t>
+          <t>Architect &amp; interior designer</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -39049,7 +40641,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>IFA / wealth management</t>
+          <t>Architects / project management</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -39059,7 +40651,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Physiotherapy &amp; clinical Pilates</t>
+          <t>IFA / wealth management</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -39069,7 +40661,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Aesthetics &amp; skin clinic</t>
+          <t>Physiotherapy &amp; clinical Pilates</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -39079,7 +40671,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>IFA / financial planning</t>
+          <t>Aesthetics &amp; skin clinic</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -39089,7 +40681,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Wealth management &amp; employee benefits</t>
+          <t>IFA / financial planning</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -39099,7 +40691,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Dermatology clinic</t>
+          <t>Wealth management &amp; employee benefits</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -39109,7 +40701,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Pilates studio (multi-site)</t>
+          <t>Dermatology clinic</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -39119,7 +40711,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Private nursery (Montessori, multi-site)</t>
+          <t>Pilates studio (multi-site)</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -39129,7 +40721,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Law firm (wills &amp; probate)</t>
+          <t>Private nursery (Montessori, multi-site)</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -39139,7 +40731,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Business/technical consultancy</t>
+          <t>Law firm (wills &amp; probate)</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -39149,7 +40741,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Private/NHS dentist</t>
+          <t>Business/technical consultancy</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -39159,7 +40751,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Removals company</t>
+          <t>Private/NHS dentist</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -39169,7 +40761,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Driveways &amp; landscaping</t>
+          <t>Removals company</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -39179,7 +40771,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Wedding &amp; event venue</t>
+          <t>Driveways &amp; landscaping</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -39189,7 +40781,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>IFA &amp; mortgage broker</t>
+          <t>Wedding &amp; event venue</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -39199,7 +40791,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Wedding photography &amp; videography</t>
+          <t>IFA &amp; mortgage broker</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -39209,7 +40801,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Commercial property litigation law firm</t>
+          <t>Wedding photography &amp; videography</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -39219,7 +40811,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Recruitment agency (boutique)</t>
+          <t>Commercial property litigation law firm</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -39229,7 +40821,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Home cinema &amp; smart home installer</t>
+          <t>Recruitment agency (boutique)</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -39239,7 +40831,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Home cinema installer</t>
+          <t>Home cinema &amp; smart home installer</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -39249,7 +40841,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Curtains, blinds &amp; upholstery</t>
+          <t>Home cinema installer</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -39259,7 +40851,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Bespoke curtains &amp; soft furnishings</t>
+          <t>Curtains, blinds &amp; upholstery</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -39269,7 +40861,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Wine merchant</t>
+          <t>Bespoke curtains &amp; soft furnishings</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -39279,7 +40871,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Education consultancy (school placement)</t>
+          <t>Wine merchant</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -39289,7 +40881,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Estate agent &amp; surveyors</t>
+          <t>Education consultancy (school placement)</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -39299,7 +40891,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Independent financial adviser</t>
+          <t>Estate agent &amp; surveyors</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -39309,7 +40901,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Chartered accountants &amp; financial planners</t>
+          <t>Independent financial adviser</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -39319,7 +40911,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Private GP &amp; dermatology</t>
+          <t>Chartered accountants &amp; financial planners</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -39329,7 +40921,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Architects (heritage specialism)</t>
+          <t>Private GP &amp; dermatology</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -39339,7 +40931,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Private cosmetic dentist / implants</t>
+          <t>Architects (heritage specialism)</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -39349,7 +40941,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Heating engineer / plumbing</t>
+          <t>Private cosmetic dentist / implants</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -39359,7 +40951,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Estate agent (boutique)</t>
+          <t>Heating engineer / plumbing</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -39369,7 +40961,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Independent vet (mixed practice)</t>
+          <t>Estate agent (boutique)</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -39379,7 +40971,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Private dentist / cosmetic</t>
+          <t>Independent vet (mixed practice)</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -39389,7 +40981,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Chartered accountants &amp; financial advisers</t>
+          <t>Private dentist / cosmetic</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -39399,7 +40991,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Healthcare recruitment agency</t>
+          <t>Chartered accountants &amp; financial advisers</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -39409,7 +41001,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Executive search / headhunting</t>
+          <t>Healthcare recruitment agency</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -39419,7 +41011,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>First aid &amp; health &amp; safety training</t>
+          <t>Executive search / headhunting</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -39429,7 +41021,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Teaching &amp; education recruitment agency</t>
+          <t>First aid &amp; health &amp; safety training</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -39439,7 +41031,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Supply teaching agency</t>
+          <t>Teaching &amp; education recruitment agency</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -39449,7 +41041,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Hospitality staffing agency</t>
+          <t>Supply teaching agency</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -39459,7 +41051,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Finance &amp; accountancy recruitment agency</t>
+          <t>Hospitality staffing agency</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -39469,7 +41061,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Accounting &amp; finance recruitment agency</t>
+          <t>Finance &amp; accountancy recruitment agency</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -39479,7 +41071,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Forklift &amp; plant operator training</t>
+          <t>Accounting &amp; finance recruitment agency</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -39489,7 +41081,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Forklift training</t>
+          <t>Forklift &amp; plant operator training</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -39499,7 +41091,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Language school</t>
+          <t>Forklift training</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -39509,7 +41101,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Engineering &amp; manufacturing recruitment</t>
+          <t>Language school</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -39519,7 +41111,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Business &amp; sales coaching</t>
+          <t>Engineering &amp; manufacturing recruitment</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -39529,7 +41121,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Engineering &amp; energy recruitment</t>
+          <t>Business &amp; sales coaching</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -39539,7 +41131,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Tech recruitment agency</t>
+          <t>Engineering &amp; energy recruitment</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -39549,7 +41141,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Data/tech/AI recruitment agency</t>
+          <t>Tech recruitment agency</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -39559,7 +41151,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Beauty/aesthetics training academy</t>
+          <t>Data/tech/AI recruitment agency</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -39569,7 +41161,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Beauty/hair training academy</t>
+          <t>Beauty/aesthetics training academy</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -39579,7 +41171,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Medical aesthetics/injectable training academy</t>
+          <t>Beauty/hair training academy</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -39589,7 +41181,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Yoga teacher training school</t>
+          <t>Medical aesthetics/injectable training academy</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -39599,7 +41191,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Creative &amp; marketing recruitment agency</t>
+          <t>Yoga teacher training school</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -39609,7 +41201,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Private dermatology &amp; women's health clinics</t>
+          <t>Creative &amp; marketing recruitment agency</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -39619,7 +41211,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Private dermatology practice</t>
+          <t>Private dermatology &amp; women's health clinics</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -39629,10 +41221,170 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
+          <t>Private dermatology practice</t>
+        </is>
+      </c>
+      <c r="B174" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
           <t>Estate &amp; lettings agent</t>
         </is>
       </c>
-      <c r="B174" t="n">
+      <c r="B175" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Wedding venue (converted barn)</t>
+        </is>
+      </c>
+      <c r="B176" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Wedding venue (waterside barn &amp; estate)</t>
+        </is>
+      </c>
+      <c r="B177" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Wedding venue (thatched barn on working farm)</t>
+        </is>
+      </c>
+      <c r="B178" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Wedding venue (working farm)</t>
+        </is>
+      </c>
+      <c r="B179" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Wedding venue (restored historic barn)</t>
+        </is>
+      </c>
+      <c r="B180" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Chartered IFA / wealth management</t>
+        </is>
+      </c>
+      <c r="B181" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Independent mortgage broker</t>
+        </is>
+      </c>
+      <c r="B182" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Independent financial planning</t>
+        </is>
+      </c>
+      <c r="B183" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Chartered independent financial planners</t>
+        </is>
+      </c>
+      <c r="B184" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Veterinary practice (small independent group)</t>
+        </is>
+      </c>
+      <c r="B185" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>Law firm (conveyancing, family, private client)</t>
+        </is>
+      </c>
+      <c r="B186" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Law firm (conveyancing, private client)</t>
+        </is>
+      </c>
+      <c r="B187" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>Conveyancing solicitors</t>
+        </is>
+      </c>
+      <c r="B188" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>Law firm (residential &amp; commercial property)</t>
+        </is>
+      </c>
+      <c r="B189" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>Law firm (conveyancing, private client, family)</t>
+        </is>
+      </c>
+      <c r="B190" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batches 49-52: +23 prospects (470 total) - solar/heat pump installers, fitness studios, immigration/private-client law, home care providers
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$448</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$471</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T448"/>
+  <dimension ref="A1:T471"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -39496,8 +39496,2156 @@
       </c>
       <c r="T448" s="3" t="inlineStr"/>
     </row>
+    <row r="449">
+      <c r="A449" s="3" t="inlineStr">
+        <is>
+          <t>Solar Age UK</t>
+        </is>
+      </c>
+      <c r="B449" s="3" t="inlineStr">
+        <is>
+          <t>Solar &amp; heat pump installer</t>
+        </is>
+      </c>
+      <c r="C449" s="3" t="inlineStr">
+        <is>
+          <t>Barham, Canterbury, Kent</t>
+        </is>
+      </c>
+      <c r="D449" s="3" t="inlineStr">
+        <is>
+          <t>https://www.solarage.co.uk</t>
+        </is>
+      </c>
+      <c r="E449" s="3" t="inlineStr">
+        <is>
+          <t>info@solarage.co.uk</t>
+        </is>
+      </c>
+      <c r="F449" s="3" t="inlineStr">
+        <is>
+          <t>01227 832299</t>
+        </is>
+      </c>
+      <c r="G449" s="3" t="inlineStr">
+        <is>
+          <t>Piotr Bojda (Director)</t>
+        </is>
+      </c>
+      <c r="H449" s="3" t="inlineStr"/>
+      <c r="I449" s="3" t="inlineStr"/>
+      <c r="J449" s="3" t="inlineStr">
+        <is>
+          <t>Family-run MCS-accredited installer since October 2009 (16-year track record) covering solar PV/thermal and ground/air/water-source heat pumps; installation jobs worth thousands to tens of thousands each</t>
+        </is>
+      </c>
+      <c r="K449" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L449" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M449" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N449" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O449" s="3" t="inlineStr">
+        <is>
+          <t>16-year MCS accreditation + RECC membership = established credibility</t>
+        </is>
+      </c>
+      <c r="P449" s="3" t="inlineStr">
+        <is>
+          <t>16-year heritage not yet the AI-cited answer for 'solar installer Kent'</t>
+        </is>
+      </c>
+      <c r="Q449" s="3" t="inlineStr">
+        <is>
+          <t>'MCS-accredited since 2009 - own that exact AEO trust signal in AI-search answers'</t>
+        </is>
+      </c>
+      <c r="R449" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S449" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T449" s="3" t="inlineStr"/>
+    </row>
+    <row r="450">
+      <c r="A450" s="4" t="inlineStr">
+        <is>
+          <t>South East Solar &amp; Electrical</t>
+        </is>
+      </c>
+      <c r="B450" s="4" t="inlineStr">
+        <is>
+          <t>Solar PV &amp; electrical installer</t>
+        </is>
+      </c>
+      <c r="C450" s="4" t="inlineStr">
+        <is>
+          <t>Rochester, Kent (also Sevenoaks)</t>
+        </is>
+      </c>
+      <c r="D450" s="4" t="inlineStr">
+        <is>
+          <t>https://www.southeastsolar.co.uk</t>
+        </is>
+      </c>
+      <c r="E450" s="4" t="inlineStr">
+        <is>
+          <t>office@southeastsolar.co.uk</t>
+        </is>
+      </c>
+      <c r="F450" s="4" t="inlineStr">
+        <is>
+          <t>01634 553422</t>
+        </is>
+      </c>
+      <c r="G450" s="4" t="inlineStr">
+        <is>
+          <t>Director details not public - verify via Companies House #09345242</t>
+        </is>
+      </c>
+      <c r="H450" s="4" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/south-east-solar-and-electrical-limited</t>
+        </is>
+      </c>
+      <c r="I450" s="4" t="inlineStr"/>
+      <c r="J450" s="4" t="inlineStr">
+        <is>
+          <t>11-year residential/commercial solar &amp; electrical installer; installation jobs worth thousands to tens of thousands each</t>
+        </is>
+      </c>
+      <c r="K450" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L450" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M450" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N450" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O450" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn presence; 11-year trading history</t>
+        </is>
+      </c>
+      <c r="P450" s="4" t="inlineStr">
+        <is>
+          <t>11-year heritage not yet the AI-cited answer for 'solar installer Kent'</t>
+        </is>
+      </c>
+      <c r="Q450" s="4" t="inlineStr">
+        <is>
+          <t>'11 years installing solar across Kent - own that AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R450" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S450" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T450" s="4" t="inlineStr">
+        <is>
+          <t>Confirm director name via Companies House before outreach</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" s="2" t="inlineStr">
+        <is>
+          <t>Cinergi</t>
+        </is>
+      </c>
+      <c r="B451" s="2" t="inlineStr">
+        <is>
+          <t>Heat pump &amp; EV charger installer</t>
+        </is>
+      </c>
+      <c r="C451" s="2" t="inlineStr">
+        <is>
+          <t>Romsey, Hampshire (covers Hants/Dorset/Wilts/Oxon/Surrey)</t>
+        </is>
+      </c>
+      <c r="D451" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cinergi.co.uk</t>
+        </is>
+      </c>
+      <c r="E451" s="2" t="inlineStr">
+        <is>
+          <t>info@cinergi.co.uk</t>
+        </is>
+      </c>
+      <c r="F451" s="2" t="inlineStr">
+        <is>
+          <t>0800 321 3142</t>
+        </is>
+      </c>
+      <c r="G451" s="2" t="inlineStr">
+        <is>
+          <t>Dan Loveridge (Founder/Managing Director)</t>
+        </is>
+      </c>
+      <c r="H451" s="2" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/cinergi-ltd</t>
+        </is>
+      </c>
+      <c r="I451" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/CinergiUK; instagram.com/cinergi_</t>
+        </is>
+      </c>
+      <c r="J451" s="2" t="inlineStr">
+        <is>
+          <t>Ranked in Ofgem's top 1% of heat pump installers nationally, uses only in-house engineers (no subcontracting); installation jobs worth thousands to tens of thousands each</t>
+        </is>
+      </c>
+      <c r="K451" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L451" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M451" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N451" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O451" s="2" t="inlineStr">
+        <is>
+          <t>Facebook/Instagram presence; Ofgem top 1% ranking = exceptional credibility asset</t>
+        </is>
+      </c>
+      <c r="P451" s="2" t="inlineStr">
+        <is>
+          <t>Ofgem top 1% ranking not yet the AI-cited trust signal for 'heat pump installer Hampshire'</t>
+        </is>
+      </c>
+      <c r="Q451" s="2" t="inlineStr">
+        <is>
+          <t>'Ranked in Ofgem's top 1% of heat pump installers - own that exact AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R451" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S451" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T451" s="2" t="inlineStr">
+        <is>
+          <t>Ofgem top 1% credential is an exceptional AEO hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" s="4" t="inlineStr">
+        <is>
+          <t>Volts Waggon</t>
+        </is>
+      </c>
+      <c r="B452" s="4" t="inlineStr">
+        <is>
+          <t>Solar PV &amp; EV charger installer</t>
+        </is>
+      </c>
+      <c r="C452" s="4" t="inlineStr">
+        <is>
+          <t>Hedge End, Southampton, Hampshire</t>
+        </is>
+      </c>
+      <c r="D452" s="4" t="inlineStr">
+        <is>
+          <t>https://www.voltswaggon.co.uk</t>
+        </is>
+      </c>
+      <c r="E452" s="4" t="inlineStr">
+        <is>
+          <t>john@voltswaggon.co.uk</t>
+        </is>
+      </c>
+      <c r="F452" s="4" t="inlineStr">
+        <is>
+          <t>07585 306346</t>
+        </is>
+      </c>
+      <c r="G452" s="4" t="inlineStr">
+        <is>
+          <t>John Wood (Founder, certified electrician, est. 2022)</t>
+        </is>
+      </c>
+      <c r="H452" s="4" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/woodster; linkedin.com/company/volts-waggon</t>
+        </is>
+      </c>
+      <c r="I452" s="4" t="inlineStr"/>
+      <c r="J452" s="4" t="inlineStr">
+        <is>
+          <t>Growing bespoke residential solar/battery/EV-charger installer with 50+ installations across Hampshire/East Dorset; installation jobs worth thousands to tens of thousands each</t>
+        </is>
+      </c>
+      <c r="K452" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L452" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M452" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N452" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O452" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn presence</t>
+        </is>
+      </c>
+      <c r="P452" s="4" t="inlineStr">
+        <is>
+          <t>Early-stage growth business - ground-floor opportunity to own local AEO search before bigger installers do</t>
+        </is>
+      </c>
+      <c r="Q452" s="4" t="inlineStr">
+        <is>
+          <t>'50+ installations and growing - be the AI-cited answer before the bigger installers catch on'</t>
+        </is>
+      </c>
+      <c r="R452" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S452" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T452" s="4" t="inlineStr"/>
+    </row>
+    <row r="453">
+      <c r="A453" s="4" t="inlineStr">
+        <is>
+          <t>Justin Bucknell Electrical</t>
+        </is>
+      </c>
+      <c r="B453" s="4" t="inlineStr">
+        <is>
+          <t>Electrical contractor &amp; solar installer</t>
+        </is>
+      </c>
+      <c r="C453" s="4" t="inlineStr">
+        <is>
+          <t>Bicester, Oxfordshire</t>
+        </is>
+      </c>
+      <c r="D453" s="4" t="inlineStr">
+        <is>
+          <t>https://www.justinbucknellelectrical.co.uk</t>
+        </is>
+      </c>
+      <c r="E453" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F453" s="4" t="inlineStr"/>
+      <c r="G453" s="4" t="inlineStr">
+        <is>
+          <t>Justin Bucknell (Founder, ~20 years trading)</t>
+        </is>
+      </c>
+      <c r="H453" s="4" t="inlineStr"/>
+      <c r="I453" s="4" t="inlineStr">
+        <is>
+          <t>facebook.com/justinbucknellelectrical</t>
+        </is>
+      </c>
+      <c r="J453" s="4" t="inlineStr">
+        <is>
+          <t>20-year local electrical contractor with MCS-accredited solar installation arm; Which? Trusted Trader listed, installation jobs worth thousands each</t>
+        </is>
+      </c>
+      <c r="K453" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L453" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M453" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N453" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O453" s="4" t="inlineStr">
+        <is>
+          <t>Facebook presence; Which? Trusted Trader listing; 20-year trading history</t>
+        </is>
+      </c>
+      <c r="P453" s="4" t="inlineStr">
+        <is>
+          <t>20-year heritage and trusted-trader status not yet the AI-cited answer for 'solar installer Bicester'</t>
+        </is>
+      </c>
+      <c r="Q453" s="4" t="inlineStr">
+        <is>
+          <t>'Which? Trusted Trader for 20 years - own that AEO trust signal in Oxfordshire'</t>
+        </is>
+      </c>
+      <c r="R453" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S453" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T453" s="4" t="inlineStr"/>
+    </row>
+    <row r="454">
+      <c r="A454" s="4" t="inlineStr">
+        <is>
+          <t>Capital Solar</t>
+        </is>
+      </c>
+      <c r="B454" s="4" t="inlineStr">
+        <is>
+          <t>Solar PV installer</t>
+        </is>
+      </c>
+      <c r="C454" s="4" t="inlineStr">
+        <is>
+          <t>Abingdon, Oxfordshire (Oxfordshire-wide)</t>
+        </is>
+      </c>
+      <c r="D454" s="4" t="inlineStr">
+        <is>
+          <t>https://www.capitalsolar.co.uk</t>
+        </is>
+      </c>
+      <c r="E454" s="4" t="inlineStr">
+        <is>
+          <t>dan@capitalsolar.co.uk</t>
+        </is>
+      </c>
+      <c r="F454" s="4" t="inlineStr">
+        <is>
+          <t>07931 957447</t>
+        </is>
+      </c>
+      <c r="G454" s="4" t="inlineStr">
+        <is>
+          <t>Dan (Director) - surname unconfirmed, verify via Companies House #11850466</t>
+        </is>
+      </c>
+      <c r="H454" s="4" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/capital-electrical-and-solar</t>
+        </is>
+      </c>
+      <c r="I454" s="4" t="inlineStr">
+        <is>
+          <t>facebook.com/capitalelectricalandsolar</t>
+        </is>
+      </c>
+      <c r="J454" s="4" t="inlineStr">
+        <is>
+          <t>Oxfordshire-wide solar PV installer; installation jobs worth thousands to tens of thousands each</t>
+        </is>
+      </c>
+      <c r="K454" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L454" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M454" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N454" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O454" s="4" t="inlineStr">
+        <is>
+          <t>Facebook/LinkedIn presence</t>
+        </is>
+      </c>
+      <c r="P454" s="4" t="inlineStr">
+        <is>
+          <t>Generic 'solar installer Oxfordshire' searches not yet AI-answer dominated by this installer</t>
+        </is>
+      </c>
+      <c r="Q454" s="4" t="inlineStr">
+        <is>
+          <t>Own a specific Oxfordshire-town AEO niche vs bigger regional installers</t>
+        </is>
+      </c>
+      <c r="R454" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S454" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T454" s="4" t="inlineStr">
+        <is>
+          <t>Confirm director surname via Companies House before outreach</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" s="4" t="inlineStr">
+        <is>
+          <t>The Pilates Sphere</t>
+        </is>
+      </c>
+      <c r="B455" s="4" t="inlineStr">
+        <is>
+          <t>Reformer Pilates studio</t>
+        </is>
+      </c>
+      <c r="C455" s="4" t="inlineStr">
+        <is>
+          <t>Richmond, London TW9</t>
+        </is>
+      </c>
+      <c r="D455" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thepilatessphere.co.uk</t>
+        </is>
+      </c>
+      <c r="E455" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F455" s="4" t="inlineStr"/>
+      <c r="G455" s="4" t="inlineStr">
+        <is>
+          <t>Charlotte Faul (Owner, rebranded/relaunched summer 2024)</t>
+        </is>
+      </c>
+      <c r="H455" s="4" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/charlotte-faul</t>
+        </is>
+      </c>
+      <c r="I455" s="4" t="inlineStr">
+        <is>
+          <t>instagram.com/thepilatessphere.richmond; facebook.com/61573085375104</t>
+        </is>
+      </c>
+      <c r="J455" s="4" t="inlineStr">
+        <is>
+          <t>Independent boutique reformer Pilates studio serving Richmond/Kew/Twickenham/Kingston; class packages and memberships worth hundreds to thousands per client per year</t>
+        </is>
+      </c>
+      <c r="K455" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L455" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M455" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N455" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O455" s="4" t="inlineStr">
+        <is>
+          <t>Instagram/Facebook presence = active marketing</t>
+        </is>
+      </c>
+      <c r="P455" s="4" t="inlineStr">
+        <is>
+          <t>Recent rebrand not yet the AI-cited answer for 'reformer Pilates Richmond'</t>
+        </is>
+      </c>
+      <c r="Q455" s="4" t="inlineStr">
+        <is>
+          <t>'Just relaunched - be the AI-cited answer before the old brand's search history fades'</t>
+        </is>
+      </c>
+      <c r="R455" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S455" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T455" s="4" t="inlineStr"/>
+    </row>
+    <row r="456">
+      <c r="A456" s="4" t="inlineStr">
+        <is>
+          <t>Victoria Hinds Pilates</t>
+        </is>
+      </c>
+      <c r="B456" s="4" t="inlineStr">
+        <is>
+          <t>Classical Pilates studio</t>
+        </is>
+      </c>
+      <c r="C456" s="4" t="inlineStr">
+        <is>
+          <t>St Margarets/East Twickenham (serving Richmond)</t>
+        </is>
+      </c>
+      <c r="D456" s="4" t="inlineStr">
+        <is>
+          <t>https://www.victoriahindspilates.co.uk</t>
+        </is>
+      </c>
+      <c r="E456" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F456" s="4" t="inlineStr">
+        <is>
+          <t>07853 902032</t>
+        </is>
+      </c>
+      <c r="G456" s="4" t="inlineStr">
+        <is>
+          <t>Victoria Hinds (Founder, Body Control Pilates-certified, est. 2011)</t>
+        </is>
+      </c>
+      <c r="H456" s="4" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/victoria-hinds-99938648</t>
+        </is>
+      </c>
+      <c r="I456" s="4" t="inlineStr">
+        <is>
+          <t>instagram.com/victoria_hindspilates</t>
+        </is>
+      </c>
+      <c r="J456" s="4" t="inlineStr">
+        <is>
+          <t>14-year solo-owner classical Pilates studio (mat &amp; reformer, private and small-group); class packages worth hundreds to thousands per client per year</t>
+        </is>
+      </c>
+      <c r="K456" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L456" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M456" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N456" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O456" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn/Instagram presence; 14-year trading history</t>
+        </is>
+      </c>
+      <c r="P456" s="4" t="inlineStr">
+        <is>
+          <t>14-year heritage not yet the AI-cited answer for 'Pilates Richmond'</t>
+        </is>
+      </c>
+      <c r="Q456" s="4" t="inlineStr">
+        <is>
+          <t>'14 years teaching classical Pilates in Richmond - own that AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R456" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S456" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T456" s="4" t="inlineStr"/>
+    </row>
+    <row r="457">
+      <c r="A457" s="4" t="inlineStr">
+        <is>
+          <t>Cheltenham Pilates &amp; Yoga Studios</t>
+        </is>
+      </c>
+      <c r="B457" s="4" t="inlineStr">
+        <is>
+          <t>Pilates &amp; yoga studio (+ teacher training)</t>
+        </is>
+      </c>
+      <c r="C457" s="4" t="inlineStr">
+        <is>
+          <t>Cheltenham</t>
+        </is>
+      </c>
+      <c r="D457" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cheltenhampilatesandyoga.co.uk</t>
+        </is>
+      </c>
+      <c r="E457" s="4" t="inlineStr">
+        <is>
+          <t>nicky@cheltenhampilatesandyoga.co.uk</t>
+        </is>
+      </c>
+      <c r="F457" s="4" t="inlineStr"/>
+      <c r="G457" s="4" t="inlineStr">
+        <is>
+          <t>Nicky Gladman (Founder, 20 years teaching Pilates, studio est. 2009)</t>
+        </is>
+      </c>
+      <c r="H457" s="4" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/nicky-gladman-7683b9153</t>
+        </is>
+      </c>
+      <c r="I457" s="4" t="inlineStr"/>
+      <c r="J457" s="4" t="inlineStr">
+        <is>
+          <t>One of Cheltenham's most established independent studios (15+ years at current site) offering classes and teacher training; class packages and trainee course fees recur</t>
+        </is>
+      </c>
+      <c r="K457" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L457" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M457" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N457" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O457" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn presence; 15+ year trading history</t>
+        </is>
+      </c>
+      <c r="P457" s="4" t="inlineStr">
+        <is>
+          <t>15-year heritage not yet the AI-cited answer for 'Pilates Cheltenham'</t>
+        </is>
+      </c>
+      <c r="Q457" s="4" t="inlineStr">
+        <is>
+          <t>'15 years at the same Cheltenham studio - own that AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R457" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S457" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T457" s="4" t="inlineStr"/>
+    </row>
+    <row r="458">
+      <c r="A458" s="3" t="inlineStr">
+        <is>
+          <t>The Studio Cheltenham</t>
+        </is>
+      </c>
+      <c r="B458" s="3" t="inlineStr">
+        <is>
+          <t>Reformer Pilates studio</t>
+        </is>
+      </c>
+      <c r="C458" s="3" t="inlineStr">
+        <is>
+          <t>The Brewery Quarter, Cheltenham</t>
+        </is>
+      </c>
+      <c r="D458" s="3" t="inlineStr">
+        <is>
+          <t>https://www.thestudiocheltenham.com</t>
+        </is>
+      </c>
+      <c r="E458" s="3" t="inlineStr">
+        <is>
+          <t>hello@thestudiocheltenham.com</t>
+        </is>
+      </c>
+      <c r="F458" s="3" t="inlineStr"/>
+      <c r="G458" s="3" t="inlineStr">
+        <is>
+          <t>Fontaine Wright (Co-founder, former Team GB badminton player) &amp; Harry (Co-founder, launched Oct 2024)</t>
+        </is>
+      </c>
+      <c r="H458" s="3" t="inlineStr"/>
+      <c r="I458" s="3" t="inlineStr">
+        <is>
+          <t>instagram.com/thestudiocheltenham; facebook.com/p/The-Studio-Cheltenham-61561700947780</t>
+        </is>
+      </c>
+      <c r="J458" s="3" t="inlineStr">
+        <is>
+          <t>New strength-focused dynamic reformer Pilates studio from a former Team GB athlete, with press coverage in SoGlos; class packages and memberships worth hundreds to thousands per client per year</t>
+        </is>
+      </c>
+      <c r="K458" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L458" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M458" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N458" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O458" s="3" t="inlineStr">
+        <is>
+          <t>Instagram/Facebook presence; press coverage (SoGlos) = active PR</t>
+        </is>
+      </c>
+      <c r="P458" s="3" t="inlineStr">
+        <is>
+          <t>Team GB founder story and press coverage not yet the AI-cited answer for 'Pilates Cheltenham'</t>
+        </is>
+      </c>
+      <c r="Q458" s="3" t="inlineStr">
+        <is>
+          <t>'Founded by a former Team GB athlete - own that exact AEO story before competitors catch on'</t>
+        </is>
+      </c>
+      <c r="R458" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S458" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T458" s="3" t="inlineStr">
+        <is>
+          <t>New studio (Oct 2024), explicitly markets as 'proudly independent'</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" s="4" t="inlineStr">
+        <is>
+          <t>Every Body Studio</t>
+        </is>
+      </c>
+      <c r="B459" s="4" t="inlineStr">
+        <is>
+          <t>Yoga, barre &amp; Pilates studio (+ teacher training)</t>
+        </is>
+      </c>
+      <c r="C459" s="4" t="inlineStr">
+        <is>
+          <t>St Clements/Magdalen Road, Oxford</t>
+        </is>
+      </c>
+      <c r="D459" s="4" t="inlineStr">
+        <is>
+          <t>https://www.everybodystudio.co.uk</t>
+        </is>
+      </c>
+      <c r="E459" s="4" t="inlineStr">
+        <is>
+          <t>hello@everybodystudio.co.uk</t>
+        </is>
+      </c>
+      <c r="F459" s="4" t="inlineStr">
+        <is>
+          <t>07813 691906</t>
+        </is>
+      </c>
+      <c r="G459" s="4" t="inlineStr">
+        <is>
+          <t>Katie Gordon (Founder)</t>
+        </is>
+      </c>
+      <c r="H459" s="4" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/katie-gordon-73702253</t>
+        </is>
+      </c>
+      <c r="I459" s="4" t="inlineStr">
+        <is>
+          <t>facebook.com/EverybodyStudioOxford</t>
+        </is>
+      </c>
+      <c r="J459" s="4" t="inlineStr">
+        <is>
+          <t>Inclusive independent movement studio running its own yoga teacher-training programme, listed on the Independent Oxford directory; class packages and trainee course fees recur</t>
+        </is>
+      </c>
+      <c r="K459" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L459" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M459" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N459" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O459" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn/Facebook presence; Independent Oxford directory listing</t>
+        </is>
+      </c>
+      <c r="P459" s="4" t="inlineStr">
+        <is>
+          <t>Independent Oxford listing not yet converted into AI-cited answers for 'yoga studio Oxford'</t>
+        </is>
+      </c>
+      <c r="Q459" s="4" t="inlineStr">
+        <is>
+          <t>'Listed on Independent Oxford - let's make AI cite you too'</t>
+        </is>
+      </c>
+      <c r="R459" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S459" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T459" s="4" t="inlineStr"/>
+    </row>
+    <row r="460">
+      <c r="A460" s="3" t="inlineStr">
+        <is>
+          <t>TUFFCORE</t>
+        </is>
+      </c>
+      <c r="B460" s="3" t="inlineStr">
+        <is>
+          <t>Women-only strength &amp; personal training studio</t>
+        </is>
+      </c>
+      <c r="C460" s="3" t="inlineStr">
+        <is>
+          <t>Cowley, Oxford</t>
+        </is>
+      </c>
+      <c r="D460" s="3" t="inlineStr">
+        <is>
+          <t>https://www.teamtuffcore.com</t>
+        </is>
+      </c>
+      <c r="E460" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F460" s="3" t="inlineStr">
+        <is>
+          <t>07904 122815</t>
+        </is>
+      </c>
+      <c r="G460" s="3" t="inlineStr">
+        <is>
+          <t>Igor (Founder, martial arts/combat sports background) &amp; Agata (Coach)</t>
+        </is>
+      </c>
+      <c r="H460" s="3" t="inlineStr"/>
+      <c r="I460" s="3" t="inlineStr">
+        <is>
+          <t>instagram.com/tuffcorefitness_ox</t>
+        </is>
+      </c>
+      <c r="J460" s="3" t="inlineStr">
+        <is>
+          <t>Largest women-only small-group strength/PT studio in Oxford, niche-focused on women 30+; membership and PT packages worth thousands per client per year</t>
+        </is>
+      </c>
+      <c r="K460" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L460" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M460" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N460" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O460" s="3" t="inlineStr">
+        <is>
+          <t>Instagram presence; strong niche positioning</t>
+        </is>
+      </c>
+      <c r="P460" s="3" t="inlineStr">
+        <is>
+          <t>Niche positioning not yet the AI-cited answer for 'women's strength training Oxford'</t>
+        </is>
+      </c>
+      <c r="Q460" s="3" t="inlineStr">
+        <is>
+          <t>'The largest women-only strength studio in Oxford - own that exact AEO niche'</t>
+        </is>
+      </c>
+      <c r="R460" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S460" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T460" s="3" t="inlineStr"/>
+    </row>
+    <row r="461">
+      <c r="A461" s="3" t="inlineStr">
+        <is>
+          <t>Edmans &amp; Co</t>
+        </is>
+      </c>
+      <c r="B461" s="3" t="inlineStr">
+        <is>
+          <t>Immigration &amp; commercial law firm</t>
+        </is>
+      </c>
+      <c r="C461" s="3" t="inlineStr">
+        <is>
+          <t>Chancery Lane, London</t>
+        </is>
+      </c>
+      <c r="D461" s="3" t="inlineStr">
+        <is>
+          <t>https://www.edmansco.com</t>
+        </is>
+      </c>
+      <c r="E461" s="3" t="inlineStr">
+        <is>
+          <t>info@edmansco.com</t>
+        </is>
+      </c>
+      <c r="F461" s="3" t="inlineStr">
+        <is>
+          <t>020 8935 5205</t>
+        </is>
+      </c>
+      <c r="G461" s="3" t="inlineStr">
+        <is>
+          <t>David Manasyan &amp; Emil Manasyan (Founding brothers)</t>
+        </is>
+      </c>
+      <c r="H461" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/edmans; linkedin.com/in/emilmanasyan</t>
+        </is>
+      </c>
+      <c r="I461" s="3" t="inlineStr"/>
+      <c r="J461" s="3" t="inlineStr">
+        <is>
+          <t>Boutique OISC Level 3 immigration/commercial firm founded by immigrants who experienced the visa process firsthand; single-case fees run into thousands</t>
+        </is>
+      </c>
+      <c r="K461" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L461" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M461" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N461" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O461" s="3" t="inlineStr">
+        <is>
+          <t>Tech-forward 'modern law firm' positioning = active marketing investment</t>
+        </is>
+      </c>
+      <c r="P461" s="3" t="inlineStr">
+        <is>
+          <t>Founder-story angle not yet the AI-cited trust signal for 'immigration solicitor London'</t>
+        </is>
+      </c>
+      <c r="Q461" s="3" t="inlineStr">
+        <is>
+          <t>'Founded by immigrants who lived the visa process - own that authentic AEO story'</t>
+        </is>
+      </c>
+      <c r="R461" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S461" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T461" s="3" t="inlineStr"/>
+    </row>
+    <row r="462">
+      <c r="A462" s="2" t="inlineStr">
+        <is>
+          <t>Laura Devine Immigration</t>
+        </is>
+      </c>
+      <c r="B462" s="2" t="inlineStr">
+        <is>
+          <t>Immigration law firm (UK/US)</t>
+        </is>
+      </c>
+      <c r="C462" s="2" t="inlineStr">
+        <is>
+          <t>Cannon Street, London (+ New York)</t>
+        </is>
+      </c>
+      <c r="D462" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lauradevine.com</t>
+        </is>
+      </c>
+      <c r="E462" s="2" t="inlineStr">
+        <is>
+          <t>enquiries@lauradevine.com</t>
+        </is>
+      </c>
+      <c r="F462" s="2" t="inlineStr">
+        <is>
+          <t>020 7469 6460</t>
+        </is>
+      </c>
+      <c r="G462" s="2" t="inlineStr">
+        <is>
+          <t>Laura Devine (Founder, est. 2003) &amp; Sophie Barrett-Brown (Senior Partner)</t>
+        </is>
+      </c>
+      <c r="H462" s="2" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/laura-devine-immigration; linkedin.com/in/lauradevineimmigration</t>
+        </is>
+      </c>
+      <c r="I462" s="2" t="inlineStr"/>
+      <c r="J462" s="2" t="inlineStr">
+        <is>
+          <t>Top-tier boutique transatlantic immigration firm, Legal 500 Hall of Fame and Chambers 'Eminent Practitioner' ranked; single-case fees run into thousands to tens of thousands</t>
+        </is>
+      </c>
+      <c r="K462" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L462" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M462" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N462" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O462" s="2" t="inlineStr">
+        <is>
+          <t>2,400+ LinkedIn followers; top-tier legal directory rankings</t>
+        </is>
+      </c>
+      <c r="P462" s="2" t="inlineStr">
+        <is>
+          <t>Elite rankings not yet the AI-cited answer for 'immigration lawyer London'</t>
+        </is>
+      </c>
+      <c r="Q462" s="2" t="inlineStr">
+        <is>
+          <t>'Legal 500 Hall of Fame - own that exact AEO trust signal against bigger immigration firms'</t>
+        </is>
+      </c>
+      <c r="R462" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S462" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T462" s="2" t="inlineStr">
+        <is>
+          <t>Elite rankings + transatlantic reach - high-value AEO opportunity</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" s="2" t="inlineStr">
+        <is>
+          <t>Currey &amp; Co</t>
+        </is>
+      </c>
+      <c r="B463" s="2" t="inlineStr">
+        <is>
+          <t>Private client law firm (wills, trusts, estates)</t>
+        </is>
+      </c>
+      <c r="C463" s="2" t="inlineStr">
+        <is>
+          <t>Marylebone, London</t>
+        </is>
+      </c>
+      <c r="D463" s="2" t="inlineStr">
+        <is>
+          <t>https://www.curreyandco.co.uk</t>
+        </is>
+      </c>
+      <c r="E463" s="2" t="inlineStr">
+        <is>
+          <t>enquiries@curreyandco.co.uk</t>
+        </is>
+      </c>
+      <c r="F463" s="2" t="inlineStr">
+        <is>
+          <t>020 7802 2700</t>
+        </is>
+      </c>
+      <c r="G463" s="2" t="inlineStr">
+        <is>
+          <t>Robert Currey (Chairman); founded 1812 by Benjamin Currey</t>
+        </is>
+      </c>
+      <c r="H463" s="2" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/currey-&amp;-co-llp</t>
+        </is>
+      </c>
+      <c r="I463" s="2" t="inlineStr"/>
+      <c r="J463" s="2" t="inlineStr">
+        <is>
+          <t>213-year boutique private-client firm for landed-estate and HNW families, deliberately kept small and partner-led; estate-planning fees run into tens of thousands per family</t>
+        </is>
+      </c>
+      <c r="K463" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L463" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M463" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N463" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O463" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn presence; Chambers High Net Worth ranking; 200+ year heritage</t>
+        </is>
+      </c>
+      <c r="P463" s="2" t="inlineStr">
+        <is>
+          <t>Exceptional 213-year heritage not yet the AI-cited answer for 'private client solicitor London'</t>
+        </is>
+      </c>
+      <c r="Q463" s="2" t="inlineStr">
+        <is>
+          <t>'Advising families since 1812 - own that exact AEO trust signal, unmatched by any competitor'</t>
+        </is>
+      </c>
+      <c r="R463" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S463" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T463" s="2" t="inlineStr">
+        <is>
+          <t>Exceptional 213-year heritage - among the strongest AEO trust stories in the whole database</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" s="3" t="inlineStr">
+        <is>
+          <t>Maurice Turnor Gardner</t>
+        </is>
+      </c>
+      <c r="B464" s="3" t="inlineStr">
+        <is>
+          <t>Private wealth &amp; estate planning law firm</t>
+        </is>
+      </c>
+      <c r="C464" s="3" t="inlineStr">
+        <is>
+          <t>City of London</t>
+        </is>
+      </c>
+      <c r="D464" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mauriceturnorgardner.com</t>
+        </is>
+      </c>
+      <c r="E464" s="3" t="inlineStr">
+        <is>
+          <t>enquiries@mauriceturnorgardner.com</t>
+        </is>
+      </c>
+      <c r="F464" s="3" t="inlineStr">
+        <is>
+          <t>020 7786 8710</t>
+        </is>
+      </c>
+      <c r="G464" s="3" t="inlineStr">
+        <is>
+          <t>Clare Maurice (Senior Partner, first female partner at Allen &amp; Overy 1985); founded 2009</t>
+        </is>
+      </c>
+      <c r="H464" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/maurice-turnor-gardner-llp</t>
+        </is>
+      </c>
+      <c r="I464" s="3" t="inlineStr"/>
+      <c r="J464" s="3" t="inlineStr">
+        <is>
+          <t>Boutique private wealth firm for complex HNW estates, demerged from Allen &amp; Overy in 2009; estate-planning fees run into tens of thousands per family</t>
+        </is>
+      </c>
+      <c r="K464" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L464" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M464" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N464" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O464" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn presence; Lifetime Achievement award (British Legal Awards 2023)</t>
+        </is>
+      </c>
+      <c r="P464" s="3" t="inlineStr">
+        <is>
+          <t>Senior partner's award and A&amp;O pedigree not yet the AI-cited trust signal</t>
+        </is>
+      </c>
+      <c r="Q464" s="3" t="inlineStr">
+        <is>
+          <t>'Founded by A&amp;O's first female partner - own that exact AEO credibility signal'</t>
+        </is>
+      </c>
+      <c r="R464" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S464" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T464" s="3" t="inlineStr"/>
+    </row>
+    <row r="465">
+      <c r="A465" s="3" t="inlineStr">
+        <is>
+          <t>RMW Law</t>
+        </is>
+      </c>
+      <c r="B465" s="3" t="inlineStr">
+        <is>
+          <t>Private wealth law firm (UHNW)</t>
+        </is>
+      </c>
+      <c r="C465" s="3" t="inlineStr">
+        <is>
+          <t>Old Bailey, London</t>
+        </is>
+      </c>
+      <c r="D465" s="3" t="inlineStr">
+        <is>
+          <t>https://www.rmwlaw.co.uk</t>
+        </is>
+      </c>
+      <c r="E465" s="3" t="inlineStr">
+        <is>
+          <t>mail@rmwlaw.co.uk</t>
+        </is>
+      </c>
+      <c r="F465" s="3" t="inlineStr">
+        <is>
+          <t>020 7597 6416</t>
+        </is>
+      </c>
+      <c r="G465" s="3" t="inlineStr">
+        <is>
+          <t>John Riches &amp; Samantha Morgan (Founders, ex-Withers, est. 2011)</t>
+        </is>
+      </c>
+      <c r="H465" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/rmw-law-llp; linkedin.com/in/john-riches-93014415</t>
+        </is>
+      </c>
+      <c r="I465" s="3" t="inlineStr"/>
+      <c r="J465" s="3" t="inlineStr">
+        <is>
+          <t>Boutique UHNW private wealth firm (trusts, foundations, succession); estate-planning fees run into tens of thousands per family</t>
+        </is>
+      </c>
+      <c r="K465" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L465" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M465" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N465" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O465" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn presence; Chambers HNW ranking, top-tier global recognition for founder</t>
+        </is>
+      </c>
+      <c r="P465" s="3" t="inlineStr">
+        <is>
+          <t>Founder's global top-tier ranking not yet the AI-cited answer for 'private wealth lawyer London'</t>
+        </is>
+      </c>
+      <c r="Q465" s="3" t="inlineStr">
+        <is>
+          <t>'Globally top-ranked for private wealth work - own that exact AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R465" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S465" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T465" s="3" t="inlineStr"/>
+    </row>
+    <row r="466">
+      <c r="A466" s="2" t="inlineStr">
+        <is>
+          <t>Home Counties Carers</t>
+        </is>
+      </c>
+      <c r="B466" s="2" t="inlineStr">
+        <is>
+          <t>Home care &amp; live-in care agency</t>
+        </is>
+      </c>
+      <c r="C466" s="2" t="inlineStr">
+        <is>
+          <t>Ripley, Surrey</t>
+        </is>
+      </c>
+      <c r="D466" s="2" t="inlineStr">
+        <is>
+          <t>https://www.homecountiescarers.co.uk</t>
+        </is>
+      </c>
+      <c r="E466" s="2" t="inlineStr">
+        <is>
+          <t>mkalupka@homecountiescarers.co.uk</t>
+        </is>
+      </c>
+      <c r="F466" s="2" t="inlineStr">
+        <is>
+          <t>01483 224985</t>
+        </is>
+      </c>
+      <c r="G466" s="2" t="inlineStr">
+        <is>
+          <t>Family-run (verify via Companies House #07647044)</t>
+        </is>
+      </c>
+      <c r="H466" s="2" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/home-counties-carers</t>
+        </is>
+      </c>
+      <c r="I466" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/HomeCountiesCarers</t>
+        </is>
+      </c>
+      <c r="J466" s="2" t="inlineStr">
+        <is>
+          <t>CQC Outstanding-rated home/live-in/dementia care agency and Surrey Care Provider of the Year winner; care packages worth thousands per month per client</t>
+        </is>
+      </c>
+      <c r="K466" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L466" s="2" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M466" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N466" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O466" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn/Facebook presence; CQC Outstanding + regional award</t>
+        </is>
+      </c>
+      <c r="P466" s="2" t="inlineStr">
+        <is>
+          <t>CQC Outstanding rating and award win not yet the AI-cited trust signal for 'home care Surrey'</t>
+        </is>
+      </c>
+      <c r="Q466" s="2" t="inlineStr">
+        <is>
+          <t>'CQC Outstanding and Surrey Care Provider of the Year - own that exact AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R466" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S466" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T466" s="2" t="inlineStr">
+        <is>
+          <t>CQC Outstanding + award win - strong AEO hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" s="2" t="inlineStr">
+        <is>
+          <t>All About Home Care</t>
+        </is>
+      </c>
+      <c r="B467" s="2" t="inlineStr">
+        <is>
+          <t>Home care agency</t>
+        </is>
+      </c>
+      <c r="C467" s="2" t="inlineStr">
+        <is>
+          <t>Tunbridge Wells/Tonbridge/Sevenoaks/Maidstone, Kent</t>
+        </is>
+      </c>
+      <c r="D467" s="2" t="inlineStr">
+        <is>
+          <t>https://www.allabouthomecare.co.uk</t>
+        </is>
+      </c>
+      <c r="E467" s="2" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F467" s="2" t="inlineStr">
+        <is>
+          <t>01732 447 055</t>
+        </is>
+      </c>
+      <c r="G467" s="2" t="inlineStr">
+        <is>
+          <t>Kieron Brennan &amp; David Barrett (Co-founders, est. 2014)</t>
+        </is>
+      </c>
+      <c r="H467" s="2" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/davidrlbarrett</t>
+        </is>
+      </c>
+      <c r="I467" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/allabouthomecareHQ; instagram.com/allabouthomecarehq</t>
+        </is>
+      </c>
+      <c r="J467" s="2" t="inlineStr">
+        <is>
+          <t>CQC Outstanding-rated community home care provider, 'Top 20 Recommended Home Care Provider (South East)' three years running; care packages worth thousands per month per client</t>
+        </is>
+      </c>
+      <c r="K467" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L467" s="2" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M467" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N467" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O467" s="2" t="inlineStr">
+        <is>
+          <t>Multi-channel social presence; CQC Outstanding + 3-year 'Top 20' recognition</t>
+        </is>
+      </c>
+      <c r="P467" s="2" t="inlineStr">
+        <is>
+          <t>3 years of 'Top 20' recognition not yet the AI-cited answer for 'home care Tunbridge Wells'</t>
+        </is>
+      </c>
+      <c r="Q467" s="2" t="inlineStr">
+        <is>
+          <t>'Top 20 Recommended Home Care Provider, 3 years running - own that AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R467" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S467" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T467" s="2" t="inlineStr">
+        <is>
+          <t>CQC Outstanding + repeat regional recognition - strong AEO hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" s="3" t="inlineStr">
+        <is>
+          <t>Gardiner's Homecare</t>
+        </is>
+      </c>
+      <c r="B468" s="3" t="inlineStr">
+        <is>
+          <t>Home care agency</t>
+        </is>
+      </c>
+      <c r="C468" s="3" t="inlineStr">
+        <is>
+          <t>Caversham, Reading (Berkshire/South Oxfordshire)</t>
+        </is>
+      </c>
+      <c r="D468" s="3" t="inlineStr">
+        <is>
+          <t>https://www.gardinershomecare.co.uk</t>
+        </is>
+      </c>
+      <c r="E468" s="3" t="inlineStr">
+        <is>
+          <t>simon@gardinershomecare.co.uk</t>
+        </is>
+      </c>
+      <c r="F468" s="3" t="inlineStr">
+        <is>
+          <t>0118 334 7474</t>
+        </is>
+      </c>
+      <c r="G468" s="3" t="inlineStr">
+        <is>
+          <t>Simon Mahony (Director, third-generation family ownership, est. 1968)</t>
+        </is>
+      </c>
+      <c r="H468" s="3" t="inlineStr"/>
+      <c r="I468" s="3" t="inlineStr"/>
+      <c r="J468" s="3" t="inlineStr">
+        <is>
+          <t>57-year, third-generation family home care agency; CQC rated Good overall, Outstanding for Responsiveness; care packages worth thousands per month per client</t>
+        </is>
+      </c>
+      <c r="K468" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L468" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M468" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N468" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O468" s="3" t="inlineStr">
+        <is>
+          <t>CQC Outstanding-for-Responsiveness rating; 57-year heritage</t>
+        </is>
+      </c>
+      <c r="P468" s="3" t="inlineStr">
+        <is>
+          <t>57 years of family heritage not yet the AI-cited answer for 'home care Reading'</t>
+        </is>
+      </c>
+      <c r="Q468" s="3" t="inlineStr">
+        <is>
+          <t>'Three generations of family care since 1968 - own that AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R468" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S468" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T468" s="3" t="inlineStr"/>
+    </row>
+    <row r="469">
+      <c r="A469" s="4" t="inlineStr">
+        <is>
+          <t>1 to 1 Care</t>
+        </is>
+      </c>
+      <c r="B469" s="4" t="inlineStr">
+        <is>
+          <t>Home care agency</t>
+        </is>
+      </c>
+      <c r="C469" s="4" t="inlineStr">
+        <is>
+          <t>Chalgrove, South Oxfordshire</t>
+        </is>
+      </c>
+      <c r="D469" s="4" t="inlineStr">
+        <is>
+          <t>https://www.1to1care.co.uk</t>
+        </is>
+      </c>
+      <c r="E469" s="4" t="inlineStr">
+        <is>
+          <t>care@1to1care.co.uk</t>
+        </is>
+      </c>
+      <c r="F469" s="4" t="inlineStr">
+        <is>
+          <t>01865 343134</t>
+        </is>
+      </c>
+      <c r="G469" s="4" t="inlineStr">
+        <is>
+          <t>Family-owned, est. 2004; Sheena (Care Manager, 15 years)</t>
+        </is>
+      </c>
+      <c r="H469" s="4" t="inlineStr"/>
+      <c r="I469" s="4" t="inlineStr"/>
+      <c r="J469" s="4" t="inlineStr">
+        <is>
+          <t>21-year family-owned home care agency, CQC Good across all five categories; care packages worth thousands per month per client</t>
+        </is>
+      </c>
+      <c r="K469" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L469" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M469" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N469" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O469" s="4" t="inlineStr">
+        <is>
+          <t>CQC Good across all categories; 21-year trading history</t>
+        </is>
+      </c>
+      <c r="P469" s="4" t="inlineStr">
+        <is>
+          <t>21-year heritage and consistent CQC ratings not yet the AI-cited answer for 'home care Oxfordshire'</t>
+        </is>
+      </c>
+      <c r="Q469" s="4" t="inlineStr">
+        <is>
+          <t>'21 years of consistent 5-star CQC ratings - own that AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R469" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S469" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T469" s="4" t="inlineStr"/>
+    </row>
+    <row r="470">
+      <c r="A470" s="4" t="inlineStr">
+        <is>
+          <t>Amily Homecare</t>
+        </is>
+      </c>
+      <c r="B470" s="4" t="inlineStr">
+        <is>
+          <t>Home care &amp; live-in care agency</t>
+        </is>
+      </c>
+      <c r="C470" s="4" t="inlineStr">
+        <is>
+          <t>Walton-on-Thames, Surrey</t>
+        </is>
+      </c>
+      <c r="D470" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amily.co.uk</t>
+        </is>
+      </c>
+      <c r="E470" s="4" t="inlineStr">
+        <is>
+          <t>admin@amily.co.uk</t>
+        </is>
+      </c>
+      <c r="F470" s="4" t="inlineStr">
+        <is>
+          <t>01932 259613</t>
+        </is>
+      </c>
+      <c r="G470" s="4" t="inlineStr">
+        <is>
+          <t>Suvendu 'Butch' Seal (Owner/CEO)</t>
+        </is>
+      </c>
+      <c r="H470" s="4" t="inlineStr"/>
+      <c r="I470" s="4" t="inlineStr"/>
+      <c r="J470" s="4" t="inlineStr">
+        <is>
+          <t>CQC Good-rated family-run home and live-in care agency in Walton-on-Thames; care packages worth thousands per month per client</t>
+        </is>
+      </c>
+      <c r="K470" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L470" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M470" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N470" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O470" s="4" t="inlineStr">
+        <is>
+          <t>CQC Good rating</t>
+        </is>
+      </c>
+      <c r="P470" s="4" t="inlineStr">
+        <is>
+          <t>Generic 'home care Walton-on-Thames' searches not yet AI-answer dominated by this agency</t>
+        </is>
+      </c>
+      <c r="Q470" s="4" t="inlineStr">
+        <is>
+          <t>Own a specific Surrey-town AEO niche vs bigger regional care agencies</t>
+        </is>
+      </c>
+      <c r="R470" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S470" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T470" s="4" t="inlineStr"/>
+    </row>
+    <row r="471">
+      <c r="A471" s="3" t="inlineStr">
+        <is>
+          <t>County Carers</t>
+        </is>
+      </c>
+      <c r="B471" s="3" t="inlineStr">
+        <is>
+          <t>Residential &amp; domiciliary care provider</t>
+        </is>
+      </c>
+      <c r="C471" s="3" t="inlineStr">
+        <is>
+          <t>Crowthorne, Berkshire (Wokingham/Bracknell area)</t>
+        </is>
+      </c>
+      <c r="D471" s="3" t="inlineStr">
+        <is>
+          <t>https://www.countycarers.com</t>
+        </is>
+      </c>
+      <c r="E471" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F471" s="3" t="inlineStr">
+        <is>
+          <t>0118 973 3302</t>
+        </is>
+      </c>
+      <c r="G471" s="3" t="inlineStr">
+        <is>
+          <t>Eloise Wakeford (Founder &amp; Proprietor/CEO, CQC-registered since age 19, est. 2014)</t>
+        </is>
+      </c>
+      <c r="H471" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/eloise-wakeford-981460138; linkedin.com/company/county-carers-ltd</t>
+        </is>
+      </c>
+      <c r="I471" s="3" t="inlineStr"/>
+      <c r="J471" s="3" t="inlineStr">
+        <is>
+          <t>11-year care provider serving 100+ clients, founded by a CQC-registered manager since age 19; care packages worth thousands per month per client</t>
+        </is>
+      </c>
+      <c r="K471" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L471" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M471" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N471" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O471" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn presence; young-founder credibility story</t>
+        </is>
+      </c>
+      <c r="P471" s="3" t="inlineStr">
+        <is>
+          <t>Founder's early-CQC-registration story not yet the AI-cited trust signal for 'care provider Berkshire'</t>
+        </is>
+      </c>
+      <c r="Q471" s="3" t="inlineStr">
+        <is>
+          <t>'CQC-registered at 19, now serving 100+ families - own that exact AEO founder story'</t>
+        </is>
+      </c>
+      <c r="R471" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S471" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T471" s="3" t="inlineStr">
+        <is>
+          <t>Distinct from similarly-named 'County Care Berkshire Ltd' - do not conflate</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T448"/>
+  <autoFilter ref="A1:T471"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -39508,7 +41656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B190"/>
+  <dimension ref="A1:B209"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -39528,7 +41676,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>447</v>
+        <v>470</v>
       </c>
     </row>
     <row r="5">
@@ -39831,17 +41979,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Financial adviser / wealth management</t>
+          <t>Home care agency</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Roofer</t>
+          <t>Financial adviser / wealth management</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -39851,7 +41999,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating / boilers</t>
+          <t>Roofer</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -39861,7 +42009,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Event &amp; wedding caterer</t>
+          <t>Plumbing &amp; heating / boilers</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -39871,7 +42019,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Estate agent (premium)</t>
+          <t>Event &amp; wedding caterer</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -39881,7 +42029,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Orthodontist</t>
+          <t>Estate agent (premium)</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -39891,7 +42039,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Employment law firm</t>
+          <t>Orthodontist</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -39901,7 +42049,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Event management agency</t>
+          <t>Employment law firm</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -39911,7 +42059,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Design &amp; build</t>
+          <t>Event management agency</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -39921,7 +42069,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Wealth management / IFA</t>
+          <t>Design &amp; build</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -39931,7 +42079,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Architects &amp; interior design</t>
+          <t>Wealth management / IFA</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -39941,7 +42089,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Funeral directors</t>
+          <t>Architects &amp; interior design</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -39951,7 +42099,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Garden rooms / outbuildings</t>
+          <t>Funeral directors</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -39961,7 +42109,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Personal training gym</t>
+          <t>Garden rooms / outbuildings</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -39971,7 +42119,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Estate agent &amp; chartered surveyors</t>
+          <t>Personal training gym</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -39981,7 +42129,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Wedding &amp; event caterer</t>
+          <t>Estate agent &amp; chartered surveyors</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -39991,7 +42139,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Personal training</t>
+          <t>Wedding &amp; event caterer</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -40001,7 +42149,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Construction recruitment agency</t>
+          <t>Personal training</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -40011,7 +42159,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Legal recruitment agency</t>
+          <t>Construction recruitment agency</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -40021,7 +42169,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>HGV driver training</t>
+          <t>Legal recruitment agency</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -40031,7 +42179,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Private GP practice</t>
+          <t>HGV driver training</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -40041,7 +42189,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Aesthetics clinic (non-surgical)</t>
+          <t>Private GP practice</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -40051,7 +42199,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Driving school &amp; ADI instructor training</t>
+          <t>Aesthetics clinic (non-surgical)</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -40061,7 +42209,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Veterinary practice</t>
+          <t>Driving school &amp; ADI instructor training</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -40071,37 +42219,37 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Dentist / Orthodontics</t>
+          <t>Veterinary practice</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Specialist dental/implant clinic</t>
+          <t>Reformer Pilates studio</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Boutique corporate law firm</t>
+          <t>Home care &amp; live-in care agency</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Cosmetic/aesthetics clinic</t>
+          <t>Dentist / Orthodontics</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -40111,7 +42259,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Skin &amp; laser clinic</t>
+          <t>Specialist dental/implant clinic</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -40121,7 +42269,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Mortgage broker / financial adviser</t>
+          <t>Boutique corporate law firm</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -40131,7 +42279,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Architects (RIBA chartered)</t>
+          <t>Cosmetic/aesthetics clinic</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -40141,7 +42289,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Recruitment agency (tech/startups)</t>
+          <t>Skin &amp; laser clinic</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -40151,7 +42299,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Recruitment agency (IT/data)</t>
+          <t>Mortgage broker / financial adviser</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -40161,7 +42309,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Independent vet (24/7 emergency)</t>
+          <t>Architects (RIBA chartered)</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -40171,7 +42319,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Letting &amp; estate agent</t>
+          <t>Recruitment agency (tech/startups)</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -40181,7 +42329,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Cosmetic clinic (injectables)</t>
+          <t>Recruitment agency (IT/data)</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -40191,7 +42339,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Cosmetic/anti-ageing clinic</t>
+          <t>Independent vet (24/7 emergency)</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -40201,7 +42349,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Yoga &amp; reformer pilates studio</t>
+          <t>Letting &amp; estate agent</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -40211,7 +42359,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Reformer pilates studio</t>
+          <t>Cosmetic clinic (injectables)</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -40221,7 +42369,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Wealth management</t>
+          <t>Cosmetic/anti-ageing clinic</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -40231,7 +42379,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Private tuition &amp; education consultancy</t>
+          <t>Yoga &amp; reformer pilates studio</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -40241,7 +42389,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Osteopath</t>
+          <t>Reformer pilates studio</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -40251,7 +42399,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Design &amp; build / home renovation</t>
+          <t>Wealth management</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -40261,7 +42409,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Builders / building contractor</t>
+          <t>Private tuition &amp; education consultancy</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -40271,7 +42419,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Home care / live-in care</t>
+          <t>Osteopath</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -40281,7 +42429,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Private day nurseries</t>
+          <t>Design &amp; build / home renovation</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -40291,7 +42439,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Personal training &amp; wellness studio</t>
+          <t>Builders / building contractor</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -40301,7 +42449,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Mortgage &amp; insurance broker</t>
+          <t>Home care / live-in care</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -40311,7 +42459,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Business consultancy</t>
+          <t>Private day nurseries</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -40321,7 +42469,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Interior designer (period homes)</t>
+          <t>Personal training &amp; wellness studio</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -40331,7 +42479,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Landscape design &amp; build</t>
+          <t>Mortgage &amp; insurance broker</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -40341,7 +42489,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Interior designer</t>
+          <t>Business consultancy</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -40351,7 +42499,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Garden design &amp; landscaping</t>
+          <t>Interior designer (period homes)</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -40361,7 +42509,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Legal recruitment</t>
+          <t>Landscape design &amp; build</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -40371,7 +42519,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Independent gym &amp; health club</t>
+          <t>Interior designer</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -40381,7 +42529,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Independent gym</t>
+          <t>Garden design &amp; landscaping</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -40391,7 +42539,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Physiotherapy (sports)</t>
+          <t>Legal recruitment</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -40401,7 +42549,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Letting agent / property management</t>
+          <t>Independent gym &amp; health club</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -40411,7 +42559,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Skin clinic</t>
+          <t>Independent gym</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -40421,7 +42569,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Tutoring company</t>
+          <t>Physiotherapy (sports)</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -40431,7 +42579,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Tutorial college &amp; exam centre</t>
+          <t>Letting agent / property management</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -40441,7 +42589,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Employment law (disability discrimination)</t>
+          <t>Skin clinic</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -40451,7 +42599,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating</t>
+          <t>Tutoring company</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -40461,7 +42609,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Tutorial college &amp; exam centre</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -40471,7 +42619,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Sports physio &amp; massage</t>
+          <t>Employment law (disability discrimination)</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -40481,7 +42629,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Chartered surveyors (party wall/building)</t>
+          <t>Plumbing &amp; heating</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -40491,7 +42639,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Chartered surveyors</t>
+          <t>Plumbing</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -40501,7 +42649,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Chartered building surveyors</t>
+          <t>Sports physio &amp; massage</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -40511,7 +42659,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Osteopathy clinics</t>
+          <t>Chartered surveyors (party wall/building)</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -40521,7 +42669,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Builders / renovations</t>
+          <t>Chartered surveyors</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -40531,7 +42679,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Private nursery schools</t>
+          <t>Chartered building surveyors</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -40541,7 +42689,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Private day nursery</t>
+          <t>Osteopathy clinics</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -40551,7 +42699,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Private GP (membership model)</t>
+          <t>Builders / renovations</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -40561,7 +42709,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Sash window restoration</t>
+          <t>Private nursery schools</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -40571,7 +42719,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Personal training (1:1)</t>
+          <t>Private day nursery</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -40581,7 +42729,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Personal training &amp; nutrition coaching</t>
+          <t>Private GP (membership model)</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -40591,7 +42739,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Private nursery/pre-prep school</t>
+          <t>Sash window restoration</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -40601,7 +42749,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Independent nursery (Montessori)</t>
+          <t>Personal training (1:1)</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -40611,7 +42759,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Live-in care agency</t>
+          <t>Personal training &amp; nutrition coaching</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -40621,7 +42769,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Law firm (conveyancing/family)</t>
+          <t>Private nursery/pre-prep school</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -40631,7 +42779,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Architect &amp; interior designer</t>
+          <t>Independent nursery (Montessori)</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -40641,7 +42789,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Architects / project management</t>
+          <t>Live-in care agency</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -40651,7 +42799,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>IFA / wealth management</t>
+          <t>Law firm (conveyancing/family)</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -40661,7 +42809,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Physiotherapy &amp; clinical Pilates</t>
+          <t>Architect &amp; interior designer</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -40671,7 +42819,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Aesthetics &amp; skin clinic</t>
+          <t>Architects / project management</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -40681,7 +42829,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>IFA / financial planning</t>
+          <t>IFA / wealth management</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -40691,7 +42839,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Wealth management &amp; employee benefits</t>
+          <t>Physiotherapy &amp; clinical Pilates</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -40701,7 +42849,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Dermatology clinic</t>
+          <t>Aesthetics &amp; skin clinic</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -40711,7 +42859,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Pilates studio (multi-site)</t>
+          <t>IFA / financial planning</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -40721,7 +42869,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Private nursery (Montessori, multi-site)</t>
+          <t>Wealth management &amp; employee benefits</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -40731,7 +42879,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Law firm (wills &amp; probate)</t>
+          <t>Dermatology clinic</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -40741,7 +42889,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Business/technical consultancy</t>
+          <t>Pilates studio (multi-site)</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -40751,7 +42899,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Private/NHS dentist</t>
+          <t>Private nursery (Montessori, multi-site)</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -40761,7 +42909,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Removals company</t>
+          <t>Law firm (wills &amp; probate)</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -40771,7 +42919,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Driveways &amp; landscaping</t>
+          <t>Business/technical consultancy</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -40781,7 +42929,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Wedding &amp; event venue</t>
+          <t>Private/NHS dentist</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -40791,7 +42939,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>IFA &amp; mortgage broker</t>
+          <t>Removals company</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -40801,7 +42949,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Wedding photography &amp; videography</t>
+          <t>Driveways &amp; landscaping</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -40811,7 +42959,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Commercial property litigation law firm</t>
+          <t>Wedding &amp; event venue</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -40821,7 +42969,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Recruitment agency (boutique)</t>
+          <t>IFA &amp; mortgage broker</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -40831,7 +42979,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Home cinema &amp; smart home installer</t>
+          <t>Wedding photography &amp; videography</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -40841,7 +42989,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Home cinema installer</t>
+          <t>Commercial property litigation law firm</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -40851,7 +42999,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Curtains, blinds &amp; upholstery</t>
+          <t>Recruitment agency (boutique)</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -40861,7 +43009,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Bespoke curtains &amp; soft furnishings</t>
+          <t>Home cinema &amp; smart home installer</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -40871,7 +43019,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Wine merchant</t>
+          <t>Home cinema installer</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -40881,7 +43029,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Education consultancy (school placement)</t>
+          <t>Curtains, blinds &amp; upholstery</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -40891,7 +43039,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Estate agent &amp; surveyors</t>
+          <t>Bespoke curtains &amp; soft furnishings</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -40901,7 +43049,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Independent financial adviser</t>
+          <t>Wine merchant</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -40911,7 +43059,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Chartered accountants &amp; financial planners</t>
+          <t>Education consultancy (school placement)</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -40921,7 +43069,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Private GP &amp; dermatology</t>
+          <t>Estate agent &amp; surveyors</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -40931,7 +43079,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Architects (heritage specialism)</t>
+          <t>Independent financial adviser</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -40941,7 +43089,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Private cosmetic dentist / implants</t>
+          <t>Chartered accountants &amp; financial planners</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -40951,7 +43099,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Heating engineer / plumbing</t>
+          <t>Private GP &amp; dermatology</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -40961,7 +43109,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Estate agent (boutique)</t>
+          <t>Architects (heritage specialism)</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -40971,7 +43119,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Independent vet (mixed practice)</t>
+          <t>Private cosmetic dentist / implants</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -40981,7 +43129,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Private dentist / cosmetic</t>
+          <t>Heating engineer / plumbing</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -40991,7 +43139,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Chartered accountants &amp; financial advisers</t>
+          <t>Estate agent (boutique)</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -41001,7 +43149,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Healthcare recruitment agency</t>
+          <t>Independent vet (mixed practice)</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -41011,7 +43159,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Executive search / headhunting</t>
+          <t>Private dentist / cosmetic</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -41021,7 +43169,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>First aid &amp; health &amp; safety training</t>
+          <t>Chartered accountants &amp; financial advisers</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -41031,7 +43179,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Teaching &amp; education recruitment agency</t>
+          <t>Healthcare recruitment agency</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -41041,7 +43189,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Supply teaching agency</t>
+          <t>Executive search / headhunting</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -41051,7 +43199,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Hospitality staffing agency</t>
+          <t>First aid &amp; health &amp; safety training</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -41061,7 +43209,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Finance &amp; accountancy recruitment agency</t>
+          <t>Teaching &amp; education recruitment agency</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -41071,7 +43219,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Accounting &amp; finance recruitment agency</t>
+          <t>Supply teaching agency</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -41081,7 +43229,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Forklift &amp; plant operator training</t>
+          <t>Hospitality staffing agency</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -41091,7 +43239,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Forklift training</t>
+          <t>Finance &amp; accountancy recruitment agency</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -41101,7 +43249,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Language school</t>
+          <t>Accounting &amp; finance recruitment agency</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -41111,7 +43259,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Engineering &amp; manufacturing recruitment</t>
+          <t>Forklift &amp; plant operator training</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -41121,7 +43269,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Business &amp; sales coaching</t>
+          <t>Forklift training</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -41131,7 +43279,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Engineering &amp; energy recruitment</t>
+          <t>Language school</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -41141,7 +43289,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Tech recruitment agency</t>
+          <t>Engineering &amp; manufacturing recruitment</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -41151,7 +43299,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Data/tech/AI recruitment agency</t>
+          <t>Business &amp; sales coaching</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -41161,7 +43309,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Beauty/aesthetics training academy</t>
+          <t>Engineering &amp; energy recruitment</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -41171,7 +43319,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Beauty/hair training academy</t>
+          <t>Tech recruitment agency</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -41181,7 +43329,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Medical aesthetics/injectable training academy</t>
+          <t>Data/tech/AI recruitment agency</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -41191,7 +43339,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Yoga teacher training school</t>
+          <t>Beauty/aesthetics training academy</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -41201,7 +43349,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Creative &amp; marketing recruitment agency</t>
+          <t>Beauty/hair training academy</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -41211,7 +43359,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Private dermatology &amp; women's health clinics</t>
+          <t>Medical aesthetics/injectable training academy</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -41221,7 +43369,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Private dermatology practice</t>
+          <t>Yoga teacher training school</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -41231,7 +43379,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>Estate &amp; lettings agent</t>
+          <t>Creative &amp; marketing recruitment agency</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -41241,7 +43389,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Wedding venue (converted barn)</t>
+          <t>Private dermatology &amp; women's health clinics</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -41251,7 +43399,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Wedding venue (waterside barn &amp; estate)</t>
+          <t>Private dermatology practice</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -41261,7 +43409,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Wedding venue (thatched barn on working farm)</t>
+          <t>Estate &amp; lettings agent</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -41271,7 +43419,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>Wedding venue (working farm)</t>
+          <t>Wedding venue (converted barn)</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -41281,7 +43429,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>Wedding venue (restored historic barn)</t>
+          <t>Wedding venue (waterside barn &amp; estate)</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -41291,7 +43439,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>Chartered IFA / wealth management</t>
+          <t>Wedding venue (thatched barn on working farm)</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -41301,7 +43449,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>Independent mortgage broker</t>
+          <t>Wedding venue (working farm)</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -41311,7 +43459,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>Independent financial planning</t>
+          <t>Wedding venue (restored historic barn)</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -41321,7 +43469,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>Chartered independent financial planners</t>
+          <t>Chartered IFA / wealth management</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -41331,7 +43479,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>Veterinary practice (small independent group)</t>
+          <t>Independent mortgage broker</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -41341,7 +43489,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Law firm (conveyancing, family, private client)</t>
+          <t>Independent financial planning</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -41351,7 +43499,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Law firm (conveyancing, private client)</t>
+          <t>Chartered independent financial planners</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -41361,7 +43509,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Conveyancing solicitors</t>
+          <t>Veterinary practice (small independent group)</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -41371,7 +43519,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Law firm (residential &amp; commercial property)</t>
+          <t>Law firm (conveyancing, family, private client)</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -41381,10 +43529,200 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
+          <t>Law firm (conveyancing, private client)</t>
+        </is>
+      </c>
+      <c r="B190" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Conveyancing solicitors</t>
+        </is>
+      </c>
+      <c r="B191" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>Law firm (residential &amp; commercial property)</t>
+        </is>
+      </c>
+      <c r="B192" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
           <t>Law firm (conveyancing, private client, family)</t>
         </is>
       </c>
-      <c r="B190" t="n">
+      <c r="B193" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Solar &amp; heat pump installer</t>
+        </is>
+      </c>
+      <c r="B194" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>Solar PV &amp; electrical installer</t>
+        </is>
+      </c>
+      <c r="B195" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Heat pump &amp; EV charger installer</t>
+        </is>
+      </c>
+      <c r="B196" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Solar PV &amp; EV charger installer</t>
+        </is>
+      </c>
+      <c r="B197" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>Electrical contractor &amp; solar installer</t>
+        </is>
+      </c>
+      <c r="B198" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Solar PV installer</t>
+        </is>
+      </c>
+      <c r="B199" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Classical Pilates studio</t>
+        </is>
+      </c>
+      <c r="B200" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Pilates &amp; yoga studio (+ teacher training)</t>
+        </is>
+      </c>
+      <c r="B201" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>Yoga, barre &amp; Pilates studio (+ teacher training)</t>
+        </is>
+      </c>
+      <c r="B202" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>Women-only strength &amp; personal training studio</t>
+        </is>
+      </c>
+      <c r="B203" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>Immigration &amp; commercial law firm</t>
+        </is>
+      </c>
+      <c r="B204" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>Immigration law firm (UK/US)</t>
+        </is>
+      </c>
+      <c r="B205" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>Private client law firm (wills, trusts, estates)</t>
+        </is>
+      </c>
+      <c r="B206" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>Private wealth &amp; estate planning law firm</t>
+        </is>
+      </c>
+      <c r="B207" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>Private wealth law firm (UHNW)</t>
+        </is>
+      </c>
+      <c r="B208" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>Residential &amp; domiciliary care provider</t>
+        </is>
+      </c>
+      <c r="B209" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batches 53-56: +21 prospects (491 total) - nurseries/tutors, wealth managers, IT MSPs/consultants, Bath/Cotswolds heritage trades
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$471</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$492</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T471"/>
+  <dimension ref="A1:T492"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -41644,8 +41644,1984 @@
         </is>
       </c>
     </row>
+    <row r="472">
+      <c r="A472" s="4" t="inlineStr">
+        <is>
+          <t>Byrne's Tuition (Islington Maths &amp; English)</t>
+        </is>
+      </c>
+      <c r="B472" s="4" t="inlineStr">
+        <is>
+          <t>Private tuition (primary/11+)</t>
+        </is>
+      </c>
+      <c r="C472" s="4" t="inlineStr">
+        <is>
+          <t>Islington, North London</t>
+        </is>
+      </c>
+      <c r="D472" s="4" t="inlineStr">
+        <is>
+          <t>https://www.islingtonmathsandenglish.co.uk</t>
+        </is>
+      </c>
+      <c r="E472" s="4" t="inlineStr">
+        <is>
+          <t>denisegbyrne@hotmail.com</t>
+        </is>
+      </c>
+      <c r="F472" s="4" t="inlineStr">
+        <is>
+          <t>07949 669275</t>
+        </is>
+      </c>
+      <c r="G472" s="4" t="inlineStr">
+        <is>
+          <t>Denise Byrne (Founder, PGCE Primary &amp; English, est. 2008)</t>
+        </is>
+      </c>
+      <c r="H472" s="4" t="inlineStr"/>
+      <c r="I472" s="4" t="inlineStr"/>
+      <c r="J472" s="4" t="inlineStr">
+        <is>
+          <t>17-year sole-practitioner tutor with 26+ years' teaching experience; per-session tuition fees recur weekly across a family's school years</t>
+        </is>
+      </c>
+      <c r="K472" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L472" s="4" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="M472" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N472" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O472" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P472" s="4" t="inlineStr">
+        <is>
+          <t>No website polish/social presence - relies entirely on word-of-mouth and testimonials</t>
+        </is>
+      </c>
+      <c r="Q472" s="4" t="inlineStr">
+        <is>
+          <t>'26 years of trusted local tutoring - let's build the AEO presence to match your reputation'</t>
+        </is>
+      </c>
+      <c r="R472" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S472" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T472" s="4" t="inlineStr"/>
+    </row>
+    <row r="473">
+      <c r="A473" s="2" t="inlineStr">
+        <is>
+          <t>Into The Woods Outdoor Nursery</t>
+        </is>
+      </c>
+      <c r="B473" s="2" t="inlineStr">
+        <is>
+          <t>Outdoor 'Forest School' nursery</t>
+        </is>
+      </c>
+      <c r="C473" s="2" t="inlineStr">
+        <is>
+          <t>Highgate &amp; Hampstead Heath, North London</t>
+        </is>
+      </c>
+      <c r="D473" s="2" t="inlineStr">
+        <is>
+          <t>https://www.intothewoodsnursery.co.uk</t>
+        </is>
+      </c>
+      <c r="E473" s="2" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F473" s="2" t="inlineStr"/>
+      <c r="G473" s="2" t="inlineStr">
+        <is>
+          <t>Emma Shaw (Founder, ex-primary teacher)</t>
+        </is>
+      </c>
+      <c r="H473" s="2" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/into-the-woods-outdoor-nursery-ltd</t>
+        </is>
+      </c>
+      <c r="I473" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/intothewoodsnursery; instagram.com/intothewoodsnursery</t>
+        </is>
+      </c>
+      <c r="J473" s="2" t="inlineStr">
+        <is>
+          <t>North London's first full-time outdoor 'Forest School' nursery concept, Ofsted-registered; nursery fees run into thousands per year per child</t>
+        </is>
+      </c>
+      <c r="K473" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L473" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M473" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N473" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O473" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn/Facebook/Instagram presence = active marketing</t>
+        </is>
+      </c>
+      <c r="P473" s="2" t="inlineStr">
+        <is>
+          <t>Genuinely unique 'first outdoor nursery' positioning not yet the AI-cited answer for 'outdoor nursery North London'</t>
+        </is>
+      </c>
+      <c r="Q473" s="2" t="inlineStr">
+        <is>
+          <t>'North London's first outdoor nursery - own that exact AEO category-creator positioning'</t>
+        </is>
+      </c>
+      <c r="R473" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S473" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T473" s="2" t="inlineStr">
+        <is>
+          <t>Genuine category-first positioning - strong AEO differentiation</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" s="3" t="inlineStr">
+        <is>
+          <t>Shapes Day Nurseries</t>
+        </is>
+      </c>
+      <c r="B474" s="3" t="inlineStr">
+        <is>
+          <t>Day nursery group (3 sites)</t>
+        </is>
+      </c>
+      <c r="C474" s="3" t="inlineStr">
+        <is>
+          <t>Reigate, Epsom &amp; Banstead, Surrey</t>
+        </is>
+      </c>
+      <c r="D474" s="3" t="inlineStr">
+        <is>
+          <t>https://www.shapesdaynursery.co.uk</t>
+        </is>
+      </c>
+      <c r="E474" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F474" s="3" t="inlineStr">
+        <is>
+          <t>01737 221441</t>
+        </is>
+      </c>
+      <c r="G474" s="3" t="inlineStr">
+        <is>
+          <t>Owner-operated (started in childcare aged 16); verify name via Companies House #07450220</t>
+        </is>
+      </c>
+      <c r="H474" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/shapes-day-nurseries-ltd</t>
+        </is>
+      </c>
+      <c r="I474" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/shapesdaynurseriesltd; instagram.com/shapesdaynurseriesltd</t>
+        </is>
+      </c>
+      <c r="J474" s="3" t="inlineStr">
+        <is>
+          <t>Independently owned 3-site nursery group personally run by its founder; nursery fees run into thousands per year per child across 3 locations</t>
+        </is>
+      </c>
+      <c r="K474" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L474" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M474" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N474" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O474" s="3" t="inlineStr">
+        <is>
+          <t>Multi-channel social presence = active marketing investment</t>
+        </is>
+      </c>
+      <c r="P474" s="3" t="inlineStr">
+        <is>
+          <t>3-site footprint not matched by 3-location AI-search dominance</t>
+        </is>
+      </c>
+      <c r="Q474" s="3" t="inlineStr">
+        <is>
+          <t>Per-site AEO content to own Reigate/Epsom/Banstead 'nursery near me' searches separately</t>
+        </is>
+      </c>
+      <c r="R474" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S474" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T474" s="3" t="inlineStr"/>
+    </row>
+    <row r="475">
+      <c r="A475" s="4" t="inlineStr">
+        <is>
+          <t>Eden Tutors</t>
+        </is>
+      </c>
+      <c r="B475" s="4" t="inlineStr">
+        <is>
+          <t>Private tuition (primary/11+)</t>
+        </is>
+      </c>
+      <c r="C475" s="4" t="inlineStr">
+        <is>
+          <t>Virginia Water, Surrey (Ascot/Windsor border)</t>
+        </is>
+      </c>
+      <c r="D475" s="4" t="inlineStr">
+        <is>
+          <t>https://www.eden-tutors.co.uk</t>
+        </is>
+      </c>
+      <c r="E475" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F475" s="4" t="inlineStr">
+        <is>
+          <t>01344 508077</t>
+        </is>
+      </c>
+      <c r="G475" s="4" t="inlineStr">
+        <is>
+          <t>Hannah Nuthall &amp; Rebecca Nuthall (Sister co-founders, both PGCE/QTS)</t>
+        </is>
+      </c>
+      <c r="H475" s="4" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/eden-tutors</t>
+        </is>
+      </c>
+      <c r="I475" s="4" t="inlineStr"/>
+      <c r="J475" s="4" t="inlineStr">
+        <is>
+          <t>Sister-founded tutoring practice covering the Virginia Water/Ascot/Windsor corridor; per-session tuition fees recur weekly across a family's school years, especially around 11+ exams</t>
+        </is>
+      </c>
+      <c r="K475" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L475" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M475" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N475" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O475" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn presence</t>
+        </is>
+      </c>
+      <c r="P475" s="4" t="inlineStr">
+        <is>
+          <t>11+ exam-prep demand in a wealthy catchment not yet the AI-cited answer for this practice</t>
+        </is>
+      </c>
+      <c r="Q475" s="4" t="inlineStr">
+        <is>
+          <t>'Own the AI-cited answer for 11+ tutoring in the Ascot/Virginia Water corridor'</t>
+        </is>
+      </c>
+      <c r="R475" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S475" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T475" s="4" t="inlineStr"/>
+    </row>
+    <row r="476">
+      <c r="A476" s="2" t="inlineStr">
+        <is>
+          <t>Archfield House Nursery</t>
+        </is>
+      </c>
+      <c r="B476" s="2" t="inlineStr">
+        <is>
+          <t>Day nursery &amp; pre-school</t>
+        </is>
+      </c>
+      <c r="C476" s="2" t="inlineStr">
+        <is>
+          <t>Cotham, Bristol</t>
+        </is>
+      </c>
+      <c r="D476" s="2" t="inlineStr">
+        <is>
+          <t>https://www.archfieldhousenursery.co.uk</t>
+        </is>
+      </c>
+      <c r="E476" s="2" t="inlineStr">
+        <is>
+          <t>accounts@archfieldhousenursery.co.uk</t>
+        </is>
+      </c>
+      <c r="F476" s="2" t="inlineStr">
+        <is>
+          <t>0117 942 2120</t>
+        </is>
+      </c>
+      <c r="G476" s="2" t="inlineStr">
+        <is>
+          <t>Rebecca Clevett (Nursery Head); privately owned since 1986</t>
+        </is>
+      </c>
+      <c r="H476" s="2" t="inlineStr"/>
+      <c r="I476" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/archfieldhousenursery; instagram.com/archfieldhousenursery</t>
+        </is>
+      </c>
+      <c r="J476" s="2" t="inlineStr">
+        <is>
+          <t>Nearly 40-year Ofsted Outstanding-rated independent Bristol nursery; nursery fees run into thousands per year per child</t>
+        </is>
+      </c>
+      <c r="K476" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L476" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M476" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N476" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O476" s="2" t="inlineStr">
+        <is>
+          <t>Facebook/Instagram presence; Ofsted Outstanding rating; 39-year heritage</t>
+        </is>
+      </c>
+      <c r="P476" s="2" t="inlineStr">
+        <is>
+          <t>39-year heritage and Outstanding Ofsted rating not yet the AI-cited answer for 'nursery Bristol'</t>
+        </is>
+      </c>
+      <c r="Q476" s="2" t="inlineStr">
+        <is>
+          <t>'Ofsted Outstanding for nearly 40 years - own that exact AEO trust signal in Bristol'</t>
+        </is>
+      </c>
+      <c r="R476" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S476" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T476" s="2" t="inlineStr">
+        <is>
+          <t>Ofsted Outstanding + 39-year heritage - strong AEO hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" s="2" t="inlineStr">
+        <is>
+          <t>MLP Wealth</t>
+        </is>
+      </c>
+      <c r="B477" s="2" t="inlineStr">
+        <is>
+          <t>IFA / wealth management</t>
+        </is>
+      </c>
+      <c r="C477" s="2" t="inlineStr">
+        <is>
+          <t>Banstead, Surrey</t>
+        </is>
+      </c>
+      <c r="D477" s="2" t="inlineStr">
+        <is>
+          <t>https://www.mlpwealth.co.uk</t>
+        </is>
+      </c>
+      <c r="E477" s="2" t="inlineStr">
+        <is>
+          <t>info@mlpwealth.co.uk</t>
+        </is>
+      </c>
+      <c r="F477" s="2" t="inlineStr">
+        <is>
+          <t>020 8296 1799</t>
+        </is>
+      </c>
+      <c r="G477" s="2" t="inlineStr">
+        <is>
+          <t>Paul Standerwick &amp; Seán Standerwick (2nd-generation, father Paolo founded 1983)</t>
+        </is>
+      </c>
+      <c r="H477" s="2" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/seanstanderwick</t>
+        </is>
+      </c>
+      <c r="I477" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/MLPWealth</t>
+        </is>
+      </c>
+      <c r="J477" s="2" t="inlineStr">
+        <is>
+          <t>42-year family-run Chartered IFA, featured in FT Adviser Top 50 Boutique Advisers and VouchedFor Top Rated Guide every year since inception; ongoing wealth-management fees run into thousands annually per client</t>
+        </is>
+      </c>
+      <c r="K477" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L477" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M477" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N477" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O477" s="2" t="inlineStr">
+        <is>
+          <t>Facebook presence; FT Adviser Top 50 + VouchedFor recognition every year since 1983</t>
+        </is>
+      </c>
+      <c r="P477" s="2" t="inlineStr">
+        <is>
+          <t>Consistent multi-decade press recognition not yet the AI-cited answer for 'IFA Banstead'</t>
+        </is>
+      </c>
+      <c r="Q477" s="2" t="inlineStr">
+        <is>
+          <t>'FT Adviser Top 50 every year since 1983 - own that exact AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R477" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S477" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T477" s="2" t="inlineStr">
+        <is>
+          <t>Exceptional consistent-recognition heritage - strong AEO opportunity</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" s="2" t="inlineStr">
+        <is>
+          <t>GPFM (Gerald Pepper Financial Management)</t>
+        </is>
+      </c>
+      <c r="B478" s="2" t="inlineStr">
+        <is>
+          <t>Chartered lifestyle financial planning</t>
+        </is>
+      </c>
+      <c r="C478" s="2" t="inlineStr">
+        <is>
+          <t>Hertford, Hertfordshire</t>
+        </is>
+      </c>
+      <c r="D478" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gpfm.co.uk</t>
+        </is>
+      </c>
+      <c r="E478" s="2" t="inlineStr">
+        <is>
+          <t>enquiries@gpfm.co.uk</t>
+        </is>
+      </c>
+      <c r="F478" s="2" t="inlineStr">
+        <is>
+          <t>01992 500 261</t>
+        </is>
+      </c>
+      <c r="G478" s="2" t="inlineStr">
+        <is>
+          <t>Simon Frost &amp; Scott Atkinson (Co-Managing Directors)</t>
+        </is>
+      </c>
+      <c r="H478" s="2" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/gp-financial-management</t>
+        </is>
+      </c>
+      <c r="I478" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/gpfmfinancial</t>
+        </is>
+      </c>
+      <c r="J478" s="2" t="inlineStr">
+        <is>
+          <t>Chartered 'lifestyle financial planning' firm voted #1 Boutique Adviser in FT Adviser Top 50, won VouchedFor Client Trust Award 2025; ongoing wealth-management fees run into thousands annually per client</t>
+        </is>
+      </c>
+      <c r="K478" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L478" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M478" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N478" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O478" s="2" t="inlineStr">
+        <is>
+          <t>Facebook presence; #1 Boutique Adviser ranking + 2025 award win</t>
+        </is>
+      </c>
+      <c r="P478" s="2" t="inlineStr">
+        <is>
+          <t>#1 ranking and recent award not yet the AI-cited trust signal for 'financial planner Hertford'</t>
+        </is>
+      </c>
+      <c r="Q478" s="2" t="inlineStr">
+        <is>
+          <t>'Voted #1 Boutique Adviser in the UK - own that exact AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R478" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S478" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T478" s="2" t="inlineStr">
+        <is>
+          <t>#1 national ranking + 2025 award - exceptional AEO hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" s="3" t="inlineStr">
+        <is>
+          <t>Jane Smith Financial Planning</t>
+        </is>
+      </c>
+      <c r="B479" s="3" t="inlineStr">
+        <is>
+          <t>Chartered independent financial planning</t>
+        </is>
+      </c>
+      <c r="C479" s="3" t="inlineStr">
+        <is>
+          <t>Olney, Buckinghamshire</t>
+        </is>
+      </c>
+      <c r="D479" s="3" t="inlineStr">
+        <is>
+          <t>https://www.janesmithfinancial.com</t>
+        </is>
+      </c>
+      <c r="E479" s="3" t="inlineStr">
+        <is>
+          <t>info@janesmithfinancial.com</t>
+        </is>
+      </c>
+      <c r="F479" s="3" t="inlineStr">
+        <is>
+          <t>01234 713131</t>
+        </is>
+      </c>
+      <c r="G479" s="3" t="inlineStr">
+        <is>
+          <t>Nicola Watts (Director, 2nd-generation; founded 1994 by mother Jane Smith)</t>
+        </is>
+      </c>
+      <c r="H479" s="3" t="inlineStr"/>
+      <c r="I479" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/IFAinOlney</t>
+        </is>
+      </c>
+      <c r="J479" s="3" t="inlineStr">
+        <is>
+          <t>31-year two-generation family Chartered IFA practice; ongoing wealth-management fees run into thousands annually per client</t>
+        </is>
+      </c>
+      <c r="K479" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L479" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M479" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N479" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O479" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence; Chartered/Accredited status</t>
+        </is>
+      </c>
+      <c r="P479" s="3" t="inlineStr">
+        <is>
+          <t>31-year family heritage not yet the AI-cited answer for 'financial planner Olney'</t>
+        </is>
+      </c>
+      <c r="Q479" s="3" t="inlineStr">
+        <is>
+          <t>'Two generations of Chartered financial planning in Olney - own that AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R479" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S479" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T479" s="3" t="inlineStr"/>
+    </row>
+    <row r="480">
+      <c r="A480" s="3" t="inlineStr">
+        <is>
+          <t>Financial Planning Partners (FPP)</t>
+        </is>
+      </c>
+      <c r="B480" s="3" t="inlineStr">
+        <is>
+          <t>Independent Chartered financial planning</t>
+        </is>
+      </c>
+      <c r="C480" s="3" t="inlineStr">
+        <is>
+          <t>Crowthorne, Berkshire</t>
+        </is>
+      </c>
+      <c r="D480" s="3" t="inlineStr">
+        <is>
+          <t>https://www.fpp-ifa.co.uk</t>
+        </is>
+      </c>
+      <c r="E480" s="3" t="inlineStr">
+        <is>
+          <t>info@fpp-ifa.co.uk</t>
+        </is>
+      </c>
+      <c r="F480" s="3" t="inlineStr">
+        <is>
+          <t>01344 778990</t>
+        </is>
+      </c>
+      <c r="G480" s="3" t="inlineStr">
+        <is>
+          <t>David Hearne (CISI 'CFP Professional of the Year' 2022) &amp; Andrew Hearne (Chartered Financial Planner)</t>
+        </is>
+      </c>
+      <c r="H480" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/davidjhearne; linkedin.com/company/financial-planning-partners-ltd</t>
+        </is>
+      </c>
+      <c r="I480" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/fppifa</t>
+        </is>
+      </c>
+      <c r="J480" s="3" t="inlineStr">
+        <is>
+          <t>Chartered wealth-management firm led by a national award-winning adviser; ongoing wealth-management fees run into thousands annually per client</t>
+        </is>
+      </c>
+      <c r="K480" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L480" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M480" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N480" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O480" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn/Facebook presence; CISI national award win (2022)</t>
+        </is>
+      </c>
+      <c r="P480" s="3" t="inlineStr">
+        <is>
+          <t>National award win not yet the AI-cited trust signal for 'financial planner Berkshire'</t>
+        </is>
+      </c>
+      <c r="Q480" s="3" t="inlineStr">
+        <is>
+          <t>'CFP Professional of the Year 2022 - own that exact AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R480" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S480" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T480" s="3" t="inlineStr"/>
+    </row>
+    <row r="481">
+      <c r="A481" s="3" t="inlineStr">
+        <is>
+          <t>Chapters Financial</t>
+        </is>
+      </c>
+      <c r="B481" s="3" t="inlineStr">
+        <is>
+          <t>Independent Chartered financial planning</t>
+        </is>
+      </c>
+      <c r="C481" s="3" t="inlineStr">
+        <is>
+          <t>Guildford, Surrey</t>
+        </is>
+      </c>
+      <c r="D481" s="3" t="inlineStr">
+        <is>
+          <t>https://www.chaptersfinancial.com</t>
+        </is>
+      </c>
+      <c r="E481" s="3" t="inlineStr">
+        <is>
+          <t>info@chaptersfinancial.com</t>
+        </is>
+      </c>
+      <c r="F481" s="3" t="inlineStr">
+        <is>
+          <t>01483 578 800</t>
+        </is>
+      </c>
+      <c r="G481" s="3" t="inlineStr">
+        <is>
+          <t>Keith Churchouse (Director, CFP) with Esther Dadswell &amp; Vicky Fulcher</t>
+        </is>
+      </c>
+      <c r="H481" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/chapters-financial-limited</t>
+        </is>
+      </c>
+      <c r="I481" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/chaptersfinancial</t>
+        </is>
+      </c>
+      <c r="J481" s="3" t="inlineStr">
+        <is>
+          <t>20-year Chartered financial planning firm serving Surrey/South East individuals; ongoing wealth-management fees run into thousands annually per client</t>
+        </is>
+      </c>
+      <c r="K481" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L481" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M481" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N481" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O481" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn/Facebook presence; 20-year client-service milestone (2024)</t>
+        </is>
+      </c>
+      <c r="P481" s="3" t="inlineStr">
+        <is>
+          <t>20-year milestone not yet the AI-cited answer for 'financial planner Guildford'</t>
+        </is>
+      </c>
+      <c r="Q481" s="3" t="inlineStr">
+        <is>
+          <t>'20 years of client service in Guildford - own that AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R481" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S481" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T481" s="3" t="inlineStr"/>
+    </row>
+    <row r="482">
+      <c r="A482" s="3" t="inlineStr">
+        <is>
+          <t>Dial A Geek</t>
+        </is>
+      </c>
+      <c r="B482" s="3" t="inlineStr">
+        <is>
+          <t>IT support &amp; managed services (MSP)</t>
+        </is>
+      </c>
+      <c r="C482" s="3" t="inlineStr">
+        <is>
+          <t>Bristol</t>
+        </is>
+      </c>
+      <c r="D482" s="3" t="inlineStr">
+        <is>
+          <t>https://www.dialageek.co.uk</t>
+        </is>
+      </c>
+      <c r="E482" s="3" t="inlineStr">
+        <is>
+          <t>dialageek2018@gmail.com</t>
+        </is>
+      </c>
+      <c r="F482" s="3" t="inlineStr">
+        <is>
+          <t>0117 369 4335</t>
+        </is>
+      </c>
+      <c r="G482" s="3" t="inlineStr">
+        <is>
+          <t>Gildas Jones ('Chief Geek', Founder, est. 2006)</t>
+        </is>
+      </c>
+      <c r="H482" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/dialageek</t>
+        </is>
+      </c>
+      <c r="I482" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/dialageek</t>
+        </is>
+      </c>
+      <c r="J482" s="3" t="inlineStr">
+        <is>
+          <t>18-year founder-led Bristol MSP serving 1,000+ businesses with IT support/cyber security/managed AI services; monthly support contracts recur across all clients</t>
+        </is>
+      </c>
+      <c r="K482" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L482" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M482" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N482" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O482" s="3" t="inlineStr">
+        <is>
+          <t>Facebook/LinkedIn presence; press coverage (Bristol247 18th-anniversary feature)</t>
+        </is>
+      </c>
+      <c r="P482" s="3" t="inlineStr">
+        <is>
+          <t>18-year milestone and press coverage not yet the AI-cited answer for 'IT support Bristol'</t>
+        </is>
+      </c>
+      <c r="Q482" s="3" t="inlineStr">
+        <is>
+          <t>'18 years, 1,000+ businesses helped - own that exact AEO trust signal in Bristol IT support'</t>
+        </is>
+      </c>
+      <c r="R482" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S482" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T482" s="3" t="inlineStr"/>
+    </row>
+    <row r="483">
+      <c r="A483" s="3" t="inlineStr">
+        <is>
+          <t>Business Control</t>
+        </is>
+      </c>
+      <c r="B483" s="3" t="inlineStr">
+        <is>
+          <t>Outsourced finance &amp; business consultancy</t>
+        </is>
+      </c>
+      <c r="C483" s="3" t="inlineStr">
+        <is>
+          <t>Odd Down, Bath</t>
+        </is>
+      </c>
+      <c r="D483" s="3" t="inlineStr">
+        <is>
+          <t>https://www.businesscontrol.co.uk</t>
+        </is>
+      </c>
+      <c r="E483" s="3" t="inlineStr">
+        <is>
+          <t>hello@businesscontrol.co.uk</t>
+        </is>
+      </c>
+      <c r="F483" s="3" t="inlineStr">
+        <is>
+          <t>01225 840538</t>
+        </is>
+      </c>
+      <c r="G483" s="3" t="inlineStr">
+        <is>
+          <t>Richard Starkey ACMA (Founder/Managing Director, est. 1990)</t>
+        </is>
+      </c>
+      <c r="H483" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/businesscontrol</t>
+        </is>
+      </c>
+      <c r="I483" s="3" t="inlineStr"/>
+      <c r="J483" s="3" t="inlineStr">
+        <is>
+          <t>36-year Bath outsourced-finance consultancy for SMEs and start-ups; monthly retained finance/consultancy fees recur across a client's growth</t>
+        </is>
+      </c>
+      <c r="K483" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L483" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M483" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N483" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O483" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn presence; 36-year trading history; strong client testimonials</t>
+        </is>
+      </c>
+      <c r="P483" s="3" t="inlineStr">
+        <is>
+          <t>36-year heritage not yet the AI-cited answer for 'outsourced finance Bath'</t>
+        </is>
+      </c>
+      <c r="Q483" s="3" t="inlineStr">
+        <is>
+          <t>'36 years as Bath's outsourced finance team - own that AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R483" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S483" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T483" s="3" t="inlineStr"/>
+    </row>
+    <row r="484">
+      <c r="A484" s="3" t="inlineStr">
+        <is>
+          <t>Oscura</t>
+        </is>
+      </c>
+      <c r="B484" s="3" t="inlineStr">
+        <is>
+          <t>IT support, hosting &amp; web development (MSP)</t>
+        </is>
+      </c>
+      <c r="C484" s="3" t="inlineStr">
+        <is>
+          <t>Reading, Berkshire</t>
+        </is>
+      </c>
+      <c r="D484" s="3" t="inlineStr">
+        <is>
+          <t>https://www.oscura.co.uk</t>
+        </is>
+      </c>
+      <c r="E484" s="3" t="inlineStr">
+        <is>
+          <t>support@oscura.co.uk</t>
+        </is>
+      </c>
+      <c r="F484" s="3" t="inlineStr">
+        <is>
+          <t>0118 959 7600</t>
+        </is>
+      </c>
+      <c r="G484" s="3" t="inlineStr">
+        <is>
+          <t>Stephen John Leitch &amp; Graham Andrew Loader (Directors, ISP roots to 1997)</t>
+        </is>
+      </c>
+      <c r="H484" s="3" t="inlineStr"/>
+      <c r="I484" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/oscuraltd</t>
+        </is>
+      </c>
+      <c r="J484" s="3" t="inlineStr">
+        <is>
+          <t>28-year Reading IT/hosting/web MSP with a low digital footprint (29 LinkedIn followers) despite deep trading history - strong SEO/AEO upside; monthly support/hosting contracts recur</t>
+        </is>
+      </c>
+      <c r="K484" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L484" s="3" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="M484" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N484" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O484" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence; long trading history but thin digital marketing</t>
+        </is>
+      </c>
+      <c r="P484" s="3" t="inlineStr">
+        <is>
+          <t>Low digital footprint despite 28 years trading = clear AEO upside opportunity</t>
+        </is>
+      </c>
+      <c r="Q484" s="3" t="inlineStr">
+        <is>
+          <t>'28 years trading but almost invisible online - massive AEO upside waiting to be unlocked'</t>
+        </is>
+      </c>
+      <c r="R484" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S484" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T484" s="3" t="inlineStr">
+        <is>
+          <t>Low online footprint despite long heritage = strong AEO opportunity</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" s="4" t="inlineStr">
+        <is>
+          <t>Oxford IT Solutions</t>
+        </is>
+      </c>
+      <c r="B485" s="4" t="inlineStr">
+        <is>
+          <t>IT support (MSP)</t>
+        </is>
+      </c>
+      <c r="C485" s="4" t="inlineStr">
+        <is>
+          <t>Kidlington, Oxford</t>
+        </is>
+      </c>
+      <c r="D485" s="4" t="inlineStr">
+        <is>
+          <t>https://www.oxforditsolutions.com</t>
+        </is>
+      </c>
+      <c r="E485" s="4" t="inlineStr">
+        <is>
+          <t>hello@oxforditsolutions.com</t>
+        </is>
+      </c>
+      <c r="F485" s="4" t="inlineStr">
+        <is>
+          <t>01865 364995</t>
+        </is>
+      </c>
+      <c r="G485" s="4" t="inlineStr">
+        <is>
+          <t>Rob Williams (Founder, running with wife Jenny since 2010)</t>
+        </is>
+      </c>
+      <c r="H485" s="4" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/rob-williams-873b2412; linkedin.com/company/oxford-it-solutions</t>
+        </is>
+      </c>
+      <c r="I485" s="4" t="inlineStr"/>
+      <c r="J485" s="4" t="inlineStr">
+        <is>
+          <t>15-year husband-and-wife-run MSP serving 450+ clients (SMEs, schools, home users) with a Cyber Essentials focus; monthly support contracts recur</t>
+        </is>
+      </c>
+      <c r="K485" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L485" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M485" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N485" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O485" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn presence; 450+ clients served</t>
+        </is>
+      </c>
+      <c r="P485" s="4" t="inlineStr">
+        <is>
+          <t>450+ clients served not yet the AI-cited trust signal for 'IT support Oxford'</t>
+        </is>
+      </c>
+      <c r="Q485" s="4" t="inlineStr">
+        <is>
+          <t>'450+ clients trust us with their IT - own that exact AEO trust signal in Oxford'</t>
+        </is>
+      </c>
+      <c r="R485" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S485" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T485" s="4" t="inlineStr"/>
+    </row>
+    <row r="486">
+      <c r="A486" s="3" t="inlineStr">
+        <is>
+          <t>Jo Richings Business &amp; Executive Coaching</t>
+        </is>
+      </c>
+      <c r="B486" s="3" t="inlineStr">
+        <is>
+          <t>Executive coaching &amp; leadership training</t>
+        </is>
+      </c>
+      <c r="C486" s="3" t="inlineStr">
+        <is>
+          <t>Bristol</t>
+        </is>
+      </c>
+      <c r="D486" s="3" t="inlineStr">
+        <is>
+          <t>https://www.jorichings.com</t>
+        </is>
+      </c>
+      <c r="E486" s="3" t="inlineStr">
+        <is>
+          <t>jo@jorichings.co.uk</t>
+        </is>
+      </c>
+      <c r="F486" s="3" t="inlineStr">
+        <is>
+          <t>07813 963523</t>
+        </is>
+      </c>
+      <c r="G486" s="3" t="inlineStr">
+        <is>
+          <t>Jo Richings (Founder)</t>
+        </is>
+      </c>
+      <c r="H486" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/jorichingsbusinesscoach</t>
+        </is>
+      </c>
+      <c r="I486" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/jorichings2018</t>
+        </is>
+      </c>
+      <c r="J486" s="3" t="inlineStr">
+        <is>
+          <t>Solo executive/leadership coach who also runs a training arm with ~18 associate trainers and founded the 3,000+ member Bristol Small Business Network; corporate coaching/training retainers recur</t>
+        </is>
+      </c>
+      <c r="K486" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L486" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M486" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N486" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O486" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn/Facebook presence; founded a 3,000+ member local business network</t>
+        </is>
+      </c>
+      <c r="P486" s="3" t="inlineStr">
+        <is>
+          <t>Community-builder reputation (3,000+ member network) not yet the AI-cited trust signal for 'business coach Bristol'</t>
+        </is>
+      </c>
+      <c r="Q486" s="3" t="inlineStr">
+        <is>
+          <t>'Founded Bristol's 3,000+ member Small Business Network - own that exact AEO community-trust signal'</t>
+        </is>
+      </c>
+      <c r="R486" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S486" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T486" s="3" t="inlineStr"/>
+    </row>
+    <row r="487">
+      <c r="A487" s="3" t="inlineStr">
+        <is>
+          <t>Cotswold Lime Works</t>
+        </is>
+      </c>
+      <c r="B487" s="3" t="inlineStr">
+        <is>
+          <t>Lime plastering/render conservation specialist</t>
+        </is>
+      </c>
+      <c r="C487" s="3" t="inlineStr">
+        <is>
+          <t>Coln St Aldwyns/Aldsworth, Cotswolds</t>
+        </is>
+      </c>
+      <c r="D487" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cotswoldlimeworks.co.uk</t>
+        </is>
+      </c>
+      <c r="E487" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F487" s="3" t="inlineStr">
+        <is>
+          <t>07944 746947</t>
+        </is>
+      </c>
+      <c r="G487" s="3" t="inlineStr">
+        <is>
+          <t>Callum David (Owner)</t>
+        </is>
+      </c>
+      <c r="H487" s="3" t="inlineStr"/>
+      <c r="I487" s="3" t="inlineStr">
+        <is>
+          <t>instagram.com/cotswoldlimework; facebook.com/cotswoldlime</t>
+        </is>
+      </c>
+      <c r="J487" s="3" t="inlineStr">
+        <is>
+          <t>12-year sole-trader conservation lime plasterer with Grade I/II listed-building project experience (churches, manor houses, schools); project fees run into thousands each</t>
+        </is>
+      </c>
+      <c r="K487" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L487" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M487" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N487" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O487" s="3" t="inlineStr">
+        <is>
+          <t>Instagram/Facebook presence</t>
+        </is>
+      </c>
+      <c r="P487" s="3" t="inlineStr">
+        <is>
+          <t>Grade I/II listed-building project portfolio not yet the AI-cited answer for 'lime plasterer Cotswolds'</t>
+        </is>
+      </c>
+      <c r="Q487" s="3" t="inlineStr">
+        <is>
+          <t>'Trusted on Grade I listed churches and manor houses - own that exact AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R487" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S487" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T487" s="3" t="inlineStr"/>
+    </row>
+    <row r="488">
+      <c r="A488" s="4" t="inlineStr">
+        <is>
+          <t>Lime Plasterers</t>
+        </is>
+      </c>
+      <c r="B488" s="4" t="inlineStr">
+        <is>
+          <t>Lime plastering &amp; traditional render specialist</t>
+        </is>
+      </c>
+      <c r="C488" s="4" t="inlineStr">
+        <is>
+          <t>Benhall, Cheltenham</t>
+        </is>
+      </c>
+      <c r="D488" s="4" t="inlineStr">
+        <is>
+          <t>https://www.lime-plasterers.co.uk</t>
+        </is>
+      </c>
+      <c r="E488" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F488" s="4" t="inlineStr">
+        <is>
+          <t>01242 701237</t>
+        </is>
+      </c>
+      <c r="G488" s="4" t="inlineStr">
+        <is>
+          <t>Thomas Campbell (Contact); team with 50+ years combined experience</t>
+        </is>
+      </c>
+      <c r="H488" s="4" t="inlineStr"/>
+      <c r="I488" s="4" t="inlineStr"/>
+      <c r="J488" s="4" t="inlineStr">
+        <is>
+          <t>Small skilled team focused on Cheltenham/Cotswolds heritage-property lime plastering and pointing; project fees run into thousands each</t>
+        </is>
+      </c>
+      <c r="K488" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L488" s="4" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="M488" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N488" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O488" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P488" s="4" t="inlineStr">
+        <is>
+          <t>50+ years combined experience not yet the AI-cited answer for 'lime plasterer Cheltenham'</t>
+        </is>
+      </c>
+      <c r="Q488" s="4" t="inlineStr">
+        <is>
+          <t>'50+ years of combined heritage-plastering experience - own that AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R488" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S488" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T488" s="4" t="inlineStr"/>
+    </row>
+    <row r="489">
+      <c r="A489" s="2" t="inlineStr">
+        <is>
+          <t>Bath Bespoke</t>
+        </is>
+      </c>
+      <c r="B489" s="2" t="inlineStr">
+        <is>
+          <t>Sash window manufacture &amp; restoration</t>
+        </is>
+      </c>
+      <c r="C489" s="2" t="inlineStr">
+        <is>
+          <t>Winsley, nr Bath</t>
+        </is>
+      </c>
+      <c r="D489" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bathbespoke.co.uk</t>
+        </is>
+      </c>
+      <c r="E489" s="2" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F489" s="2" t="inlineStr">
+        <is>
+          <t>01225 920900</t>
+        </is>
+      </c>
+      <c r="G489" s="2" t="inlineStr">
+        <is>
+          <t>James Etheridge &amp; Tom Jones-Marquez (Founders, est. 2009)</t>
+        </is>
+      </c>
+      <c r="H489" s="2" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/bath-bespoke-limited</t>
+        </is>
+      </c>
+      <c r="I489" s="2" t="inlineStr"/>
+      <c r="J489" s="2" t="inlineStr">
+        <is>
+          <t>15-year bespoke sash-window joinery firm with Royal Crescent project experience and up to 50-year timber guarantees; project fees run into thousands per property</t>
+        </is>
+      </c>
+      <c r="K489" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L489" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M489" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N489" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O489" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn presence; Royal Crescent project credential; 50-year guarantee marketing</t>
+        </is>
+      </c>
+      <c r="P489" s="2" t="inlineStr">
+        <is>
+          <t>Royal Crescent project credential not yet the AI-cited answer for 'sash window restoration Bath'</t>
+        </is>
+      </c>
+      <c r="Q489" s="2" t="inlineStr">
+        <is>
+          <t>'Restored windows on the Royal Crescent - own that exact AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R489" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S489" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T489" s="2" t="inlineStr">
+        <is>
+          <t>Royal Crescent project credential - exceptional AEO hook for Bath heritage market</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" s="3" t="inlineStr">
+        <is>
+          <t>K Pitman Joinery</t>
+        </is>
+      </c>
+      <c r="B490" s="3" t="inlineStr">
+        <is>
+          <t>Bespoke joinery (sash windows, doors, cabinetry)</t>
+        </is>
+      </c>
+      <c r="C490" s="3" t="inlineStr">
+        <is>
+          <t>Norton St Philip, nr Bath</t>
+        </is>
+      </c>
+      <c r="D490" s="3" t="inlineStr">
+        <is>
+          <t>https://www.kpitmanjoinery.co.uk</t>
+        </is>
+      </c>
+      <c r="E490" s="3" t="inlineStr">
+        <is>
+          <t>enquiries@kpitmanjoinery.co.uk</t>
+        </is>
+      </c>
+      <c r="F490" s="3" t="inlineStr">
+        <is>
+          <t>01373 384742</t>
+        </is>
+      </c>
+      <c r="G490" s="3" t="inlineStr">
+        <is>
+          <t>Ken Pitman (Founder, est. 1968) &amp; Andrew Pitman (2nd generation)</t>
+        </is>
+      </c>
+      <c r="H490" s="3" t="inlineStr"/>
+      <c r="I490" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/kpitmanjoinery</t>
+        </is>
+      </c>
+      <c r="J490" s="3" t="inlineStr">
+        <is>
+          <t>57-year two-generation family joinery workshop serving Bath/Frome/South West; project fees run into thousands per property</t>
+        </is>
+      </c>
+      <c r="K490" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L490" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M490" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N490" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O490" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence; 57-year trading history</t>
+        </is>
+      </c>
+      <c r="P490" s="3" t="inlineStr">
+        <is>
+          <t>57-year family heritage not yet the AI-cited answer for 'bespoke joinery Bath'</t>
+        </is>
+      </c>
+      <c r="Q490" s="3" t="inlineStr">
+        <is>
+          <t>'57 years of family joinery craftsmanship - own that AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R490" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S490" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T490" s="3" t="inlineStr"/>
+    </row>
+    <row r="491">
+      <c r="A491" s="4" t="inlineStr">
+        <is>
+          <t>Simon Watts Joinery</t>
+        </is>
+      </c>
+      <c r="B491" s="4" t="inlineStr">
+        <is>
+          <t>Bespoke joinery for listed/conservation buildings</t>
+        </is>
+      </c>
+      <c r="C491" s="4" t="inlineStr">
+        <is>
+          <t>Evesham, Vale of Evesham (edge of Cotswolds)</t>
+        </is>
+      </c>
+      <c r="D491" s="4" t="inlineStr">
+        <is>
+          <t>https://www.simonwattsjoinery.com</t>
+        </is>
+      </c>
+      <c r="E491" s="4" t="inlineStr">
+        <is>
+          <t>info@simonwattsjoinery.com</t>
+        </is>
+      </c>
+      <c r="F491" s="4" t="inlineStr">
+        <is>
+          <t>01386 765429</t>
+        </is>
+      </c>
+      <c r="G491" s="4" t="inlineStr">
+        <is>
+          <t>Dan &amp; Lyndsey Gregory (Successors, continuing founder Simon Watts's legacy since his 2021 passing)</t>
+        </is>
+      </c>
+      <c r="H491" s="4" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/simon-watts-joinery-limited</t>
+        </is>
+      </c>
+      <c r="I491" s="4" t="inlineStr">
+        <is>
+          <t>facebook.com/simonwattsjoinery</t>
+        </is>
+      </c>
+      <c r="J491" s="4" t="inlineStr">
+        <is>
+          <t>Listed-building/conservation-area joinery specialist with a strong continuity story across the Cotswolds; project fees run into thousands per property</t>
+        </is>
+      </c>
+      <c r="K491" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L491" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M491" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N491" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O491" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn/Facebook presence</t>
+        </is>
+      </c>
+      <c r="P491" s="4" t="inlineStr">
+        <is>
+          <t>Founder-legacy continuity story not yet the AI-cited trust signal for 'conservation joinery Cotswolds'</t>
+        </is>
+      </c>
+      <c r="Q491" s="4" t="inlineStr">
+        <is>
+          <t>'Carrying forward a founder's legacy of listed-building craftsmanship - own that AEO story'</t>
+        </is>
+      </c>
+      <c r="R491" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S491" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T491" s="4" t="inlineStr"/>
+    </row>
+    <row r="492">
+      <c r="A492" s="4" t="inlineStr">
+        <is>
+          <t>J E Righton Builders</t>
+        </is>
+      </c>
+      <c r="B492" s="4" t="inlineStr">
+        <is>
+          <t>Conservation/heritage builder</t>
+        </is>
+      </c>
+      <c r="C492" s="4" t="inlineStr">
+        <is>
+          <t>Mickleton, Chipping Campden, Cotswolds</t>
+        </is>
+      </c>
+      <c r="D492" s="4" t="inlineStr">
+        <is>
+          <t>https://www.jebuildright.co.uk</t>
+        </is>
+      </c>
+      <c r="E492" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F492" s="4" t="inlineStr">
+        <is>
+          <t>01789 430240</t>
+        </is>
+      </c>
+      <c r="G492" s="4" t="inlineStr">
+        <is>
+          <t>James Righton (Founder, 20+ years hands-on experience, 30+ years firm history)</t>
+        </is>
+      </c>
+      <c r="H492" s="4" t="inlineStr"/>
+      <c r="I492" s="4" t="inlineStr"/>
+      <c r="J492" s="4" t="inlineStr">
+        <is>
+          <t>FMB member since 2012, NHBC-registered heritage builder specialising in sympathetic period/listed-property restoration across Chipping Campden/Broadway/Stow-on-the-Wold/Stratford; project fees run into tens of thousands each</t>
+        </is>
+      </c>
+      <c r="K492" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L492" s="4" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="M492" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N492" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O492" s="4" t="inlineStr">
+        <is>
+          <t>FMB membership; NHBC registration</t>
+        </is>
+      </c>
+      <c r="P492" s="4" t="inlineStr">
+        <is>
+          <t>FMB/NHBC credentials not yet the AI-cited answer for 'heritage builder Cotswolds'</t>
+        </is>
+      </c>
+      <c r="Q492" s="4" t="inlineStr">
+        <is>
+          <t>'FMB member since 2012, NHBC-registered - own that exact AEO trust signal in the Cotswolds'</t>
+        </is>
+      </c>
+      <c r="R492" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S492" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T492" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T471"/>
+  <autoFilter ref="A1:T492"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -41656,7 +43632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B209"/>
+  <dimension ref="A1:B227"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -41676,7 +43652,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>470</v>
+        <v>491</v>
       </c>
     </row>
     <row r="5">
@@ -42079,7 +44055,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Wealth management / IFA</t>
+          <t>IFA / wealth management</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -42089,7 +44065,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Architects &amp; interior design</t>
+          <t>Wealth management / IFA</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -42099,7 +44075,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Funeral directors</t>
+          <t>Architects &amp; interior design</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -42109,7 +44085,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Garden rooms / outbuildings</t>
+          <t>Funeral directors</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -42119,7 +44095,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Personal training gym</t>
+          <t>Garden rooms / outbuildings</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -42129,7 +44105,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Estate agent &amp; chartered surveyors</t>
+          <t>Personal training gym</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -42139,7 +44115,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Wedding &amp; event caterer</t>
+          <t>Estate agent &amp; chartered surveyors</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -42149,7 +44125,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Personal training</t>
+          <t>Wedding &amp; event caterer</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -42159,7 +44135,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Construction recruitment agency</t>
+          <t>Personal training</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -42169,7 +44145,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Legal recruitment agency</t>
+          <t>Construction recruitment agency</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -42179,7 +44155,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>HGV driver training</t>
+          <t>Legal recruitment agency</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -42189,7 +44165,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Private GP practice</t>
+          <t>HGV driver training</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -42199,7 +44175,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Aesthetics clinic (non-surgical)</t>
+          <t>Private GP practice</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -42209,7 +44185,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Driving school &amp; ADI instructor training</t>
+          <t>Aesthetics clinic (non-surgical)</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -42219,7 +44195,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Veterinary practice</t>
+          <t>Driving school &amp; ADI instructor training</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -42229,7 +44205,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Reformer Pilates studio</t>
+          <t>Veterinary practice</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -42239,7 +44215,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Home care &amp; live-in care agency</t>
+          <t>Reformer Pilates studio</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -42249,37 +44225,37 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Dentist / Orthodontics</t>
+          <t>Home care &amp; live-in care agency</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Specialist dental/implant clinic</t>
+          <t>Private tuition (primary/11+)</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Boutique corporate law firm</t>
+          <t>Independent Chartered financial planning</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Cosmetic/aesthetics clinic</t>
+          <t>Dentist / Orthodontics</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -42289,7 +44265,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Skin &amp; laser clinic</t>
+          <t>Specialist dental/implant clinic</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -42299,7 +44275,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Mortgage broker / financial adviser</t>
+          <t>Boutique corporate law firm</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -42309,7 +44285,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Architects (RIBA chartered)</t>
+          <t>Cosmetic/aesthetics clinic</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -42319,7 +44295,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Recruitment agency (tech/startups)</t>
+          <t>Skin &amp; laser clinic</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -42329,7 +44305,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Recruitment agency (IT/data)</t>
+          <t>Mortgage broker / financial adviser</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -42339,7 +44315,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Independent vet (24/7 emergency)</t>
+          <t>Architects (RIBA chartered)</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -42349,7 +44325,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Letting &amp; estate agent</t>
+          <t>Recruitment agency (tech/startups)</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -42359,7 +44335,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Cosmetic clinic (injectables)</t>
+          <t>Recruitment agency (IT/data)</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -42369,7 +44345,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Cosmetic/anti-ageing clinic</t>
+          <t>Independent vet (24/7 emergency)</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -42379,7 +44355,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Yoga &amp; reformer pilates studio</t>
+          <t>Letting &amp; estate agent</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -42389,7 +44365,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Reformer pilates studio</t>
+          <t>Cosmetic clinic (injectables)</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -42399,7 +44375,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Wealth management</t>
+          <t>Cosmetic/anti-ageing clinic</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -42409,7 +44385,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Private tuition &amp; education consultancy</t>
+          <t>Yoga &amp; reformer pilates studio</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -42419,7 +44395,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Osteopath</t>
+          <t>Reformer pilates studio</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -42429,7 +44405,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Design &amp; build / home renovation</t>
+          <t>Wealth management</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -42439,7 +44415,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Builders / building contractor</t>
+          <t>Private tuition &amp; education consultancy</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -42449,7 +44425,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Home care / live-in care</t>
+          <t>Osteopath</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -42459,7 +44435,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Private day nurseries</t>
+          <t>Design &amp; build / home renovation</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -42469,7 +44445,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Personal training &amp; wellness studio</t>
+          <t>Builders / building contractor</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -42479,7 +44455,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Mortgage &amp; insurance broker</t>
+          <t>Home care / live-in care</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -42489,7 +44465,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Business consultancy</t>
+          <t>Private day nurseries</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -42499,7 +44475,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Interior designer (period homes)</t>
+          <t>Personal training &amp; wellness studio</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -42509,7 +44485,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Landscape design &amp; build</t>
+          <t>Mortgage &amp; insurance broker</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -42519,7 +44495,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Interior designer</t>
+          <t>Business consultancy</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -42529,7 +44505,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Garden design &amp; landscaping</t>
+          <t>Interior designer (period homes)</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -42539,7 +44515,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Legal recruitment</t>
+          <t>Landscape design &amp; build</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -42549,7 +44525,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Independent gym &amp; health club</t>
+          <t>Interior designer</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -42559,7 +44535,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Independent gym</t>
+          <t>Garden design &amp; landscaping</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -42569,7 +44545,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Physiotherapy (sports)</t>
+          <t>Legal recruitment</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -42579,7 +44555,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Letting agent / property management</t>
+          <t>Independent gym &amp; health club</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -42589,7 +44565,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Skin clinic</t>
+          <t>Independent gym</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -42599,7 +44575,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Tutoring company</t>
+          <t>Physiotherapy (sports)</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -42609,7 +44585,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Tutorial college &amp; exam centre</t>
+          <t>Letting agent / property management</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -42619,7 +44595,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Employment law (disability discrimination)</t>
+          <t>Skin clinic</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -42629,7 +44605,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating</t>
+          <t>Tutoring company</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -42639,7 +44615,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Tutorial college &amp; exam centre</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -42649,7 +44625,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Sports physio &amp; massage</t>
+          <t>Employment law (disability discrimination)</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -42659,7 +44635,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Chartered surveyors (party wall/building)</t>
+          <t>Plumbing &amp; heating</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -42669,7 +44645,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Chartered surveyors</t>
+          <t>Plumbing</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -42679,7 +44655,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Chartered building surveyors</t>
+          <t>Sports physio &amp; massage</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -42689,7 +44665,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Osteopathy clinics</t>
+          <t>Chartered surveyors (party wall/building)</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -42699,7 +44675,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Builders / renovations</t>
+          <t>Chartered surveyors</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -42709,7 +44685,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Private nursery schools</t>
+          <t>Chartered building surveyors</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -42719,7 +44695,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Private day nursery</t>
+          <t>Osteopathy clinics</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -42729,7 +44705,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Private GP (membership model)</t>
+          <t>Builders / renovations</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -42739,7 +44715,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Sash window restoration</t>
+          <t>Private nursery schools</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -42749,7 +44725,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Personal training (1:1)</t>
+          <t>Private day nursery</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -42759,7 +44735,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Personal training &amp; nutrition coaching</t>
+          <t>Private GP (membership model)</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -42769,7 +44745,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Private nursery/pre-prep school</t>
+          <t>Sash window restoration</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -42779,7 +44755,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Independent nursery (Montessori)</t>
+          <t>Personal training (1:1)</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -42789,7 +44765,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Live-in care agency</t>
+          <t>Personal training &amp; nutrition coaching</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -42799,7 +44775,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Law firm (conveyancing/family)</t>
+          <t>Private nursery/pre-prep school</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -42809,7 +44785,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Architect &amp; interior designer</t>
+          <t>Independent nursery (Montessori)</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -42819,7 +44795,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Architects / project management</t>
+          <t>Live-in care agency</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -42829,7 +44805,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>IFA / wealth management</t>
+          <t>Law firm (conveyancing/family)</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -42839,7 +44815,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Physiotherapy &amp; clinical Pilates</t>
+          <t>Architect &amp; interior designer</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -42849,7 +44825,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Aesthetics &amp; skin clinic</t>
+          <t>Architects / project management</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -42859,7 +44835,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>IFA / financial planning</t>
+          <t>Physiotherapy &amp; clinical Pilates</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -42869,7 +44845,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Wealth management &amp; employee benefits</t>
+          <t>Aesthetics &amp; skin clinic</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -42879,7 +44855,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Dermatology clinic</t>
+          <t>IFA / financial planning</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -42889,7 +44865,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Pilates studio (multi-site)</t>
+          <t>Wealth management &amp; employee benefits</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -42899,7 +44875,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Private nursery (Montessori, multi-site)</t>
+          <t>Dermatology clinic</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -42909,7 +44885,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Law firm (wills &amp; probate)</t>
+          <t>Pilates studio (multi-site)</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -42919,7 +44895,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Business/technical consultancy</t>
+          <t>Private nursery (Montessori, multi-site)</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -42929,7 +44905,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Private/NHS dentist</t>
+          <t>Law firm (wills &amp; probate)</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -42939,7 +44915,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Removals company</t>
+          <t>Business/technical consultancy</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -42949,7 +44925,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Driveways &amp; landscaping</t>
+          <t>Private/NHS dentist</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -42959,7 +44935,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Wedding &amp; event venue</t>
+          <t>Removals company</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -42969,7 +44945,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>IFA &amp; mortgage broker</t>
+          <t>Driveways &amp; landscaping</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -42979,7 +44955,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Wedding photography &amp; videography</t>
+          <t>Wedding &amp; event venue</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -42989,7 +44965,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Commercial property litigation law firm</t>
+          <t>IFA &amp; mortgage broker</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -42999,7 +44975,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Recruitment agency (boutique)</t>
+          <t>Wedding photography &amp; videography</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -43009,7 +44985,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Home cinema &amp; smart home installer</t>
+          <t>Commercial property litigation law firm</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -43019,7 +44995,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Home cinema installer</t>
+          <t>Recruitment agency (boutique)</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -43029,7 +45005,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Curtains, blinds &amp; upholstery</t>
+          <t>Home cinema &amp; smart home installer</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -43039,7 +45015,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Bespoke curtains &amp; soft furnishings</t>
+          <t>Home cinema installer</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -43049,7 +45025,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Wine merchant</t>
+          <t>Curtains, blinds &amp; upholstery</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -43059,7 +45035,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Education consultancy (school placement)</t>
+          <t>Bespoke curtains &amp; soft furnishings</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -43069,7 +45045,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Estate agent &amp; surveyors</t>
+          <t>Wine merchant</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -43079,7 +45055,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Independent financial adviser</t>
+          <t>Education consultancy (school placement)</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -43089,7 +45065,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Chartered accountants &amp; financial planners</t>
+          <t>Estate agent &amp; surveyors</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -43099,7 +45075,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Private GP &amp; dermatology</t>
+          <t>Independent financial adviser</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -43109,7 +45085,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Architects (heritage specialism)</t>
+          <t>Chartered accountants &amp; financial planners</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -43119,7 +45095,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Private cosmetic dentist / implants</t>
+          <t>Private GP &amp; dermatology</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -43129,7 +45105,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Heating engineer / plumbing</t>
+          <t>Architects (heritage specialism)</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -43139,7 +45115,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Estate agent (boutique)</t>
+          <t>Private cosmetic dentist / implants</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -43149,7 +45125,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Independent vet (mixed practice)</t>
+          <t>Heating engineer / plumbing</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -43159,7 +45135,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Private dentist / cosmetic</t>
+          <t>Estate agent (boutique)</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -43169,7 +45145,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Chartered accountants &amp; financial advisers</t>
+          <t>Independent vet (mixed practice)</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -43179,7 +45155,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Healthcare recruitment agency</t>
+          <t>Private dentist / cosmetic</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -43189,7 +45165,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Executive search / headhunting</t>
+          <t>Chartered accountants &amp; financial advisers</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -43199,7 +45175,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>First aid &amp; health &amp; safety training</t>
+          <t>Healthcare recruitment agency</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -43209,7 +45185,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Teaching &amp; education recruitment agency</t>
+          <t>Executive search / headhunting</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -43219,7 +45195,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Supply teaching agency</t>
+          <t>First aid &amp; health &amp; safety training</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -43229,7 +45205,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Hospitality staffing agency</t>
+          <t>Teaching &amp; education recruitment agency</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -43239,7 +45215,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Finance &amp; accountancy recruitment agency</t>
+          <t>Supply teaching agency</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -43249,7 +45225,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Accounting &amp; finance recruitment agency</t>
+          <t>Hospitality staffing agency</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -43259,7 +45235,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Forklift &amp; plant operator training</t>
+          <t>Finance &amp; accountancy recruitment agency</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -43269,7 +45245,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Forklift training</t>
+          <t>Accounting &amp; finance recruitment agency</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -43279,7 +45255,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Language school</t>
+          <t>Forklift &amp; plant operator training</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -43289,7 +45265,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Engineering &amp; manufacturing recruitment</t>
+          <t>Forklift training</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -43299,7 +45275,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Business &amp; sales coaching</t>
+          <t>Language school</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -43309,7 +45285,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Engineering &amp; energy recruitment</t>
+          <t>Engineering &amp; manufacturing recruitment</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -43319,7 +45295,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Tech recruitment agency</t>
+          <t>Business &amp; sales coaching</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -43329,7 +45305,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Data/tech/AI recruitment agency</t>
+          <t>Engineering &amp; energy recruitment</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -43339,7 +45315,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Beauty/aesthetics training academy</t>
+          <t>Tech recruitment agency</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -43349,7 +45325,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Beauty/hair training academy</t>
+          <t>Data/tech/AI recruitment agency</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -43359,7 +45335,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Medical aesthetics/injectable training academy</t>
+          <t>Beauty/aesthetics training academy</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -43369,7 +45345,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Yoga teacher training school</t>
+          <t>Beauty/hair training academy</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -43379,7 +45355,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>Creative &amp; marketing recruitment agency</t>
+          <t>Medical aesthetics/injectable training academy</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -43389,7 +45365,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Private dermatology &amp; women's health clinics</t>
+          <t>Yoga teacher training school</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -43399,7 +45375,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Private dermatology practice</t>
+          <t>Creative &amp; marketing recruitment agency</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -43409,7 +45385,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Estate &amp; lettings agent</t>
+          <t>Private dermatology &amp; women's health clinics</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -43419,7 +45395,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>Wedding venue (converted barn)</t>
+          <t>Private dermatology practice</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -43429,7 +45405,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>Wedding venue (waterside barn &amp; estate)</t>
+          <t>Estate &amp; lettings agent</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -43439,7 +45415,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>Wedding venue (thatched barn on working farm)</t>
+          <t>Wedding venue (converted barn)</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -43449,7 +45425,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>Wedding venue (working farm)</t>
+          <t>Wedding venue (waterside barn &amp; estate)</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -43459,7 +45435,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>Wedding venue (restored historic barn)</t>
+          <t>Wedding venue (thatched barn on working farm)</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -43469,7 +45445,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>Chartered IFA / wealth management</t>
+          <t>Wedding venue (working farm)</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -43479,7 +45455,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>Independent mortgage broker</t>
+          <t>Wedding venue (restored historic barn)</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -43489,7 +45465,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Independent financial planning</t>
+          <t>Chartered IFA / wealth management</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -43499,7 +45475,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Chartered independent financial planners</t>
+          <t>Independent mortgage broker</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -43509,7 +45485,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Veterinary practice (small independent group)</t>
+          <t>Independent financial planning</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -43519,7 +45495,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Law firm (conveyancing, family, private client)</t>
+          <t>Chartered independent financial planners</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -43529,7 +45505,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>Law firm (conveyancing, private client)</t>
+          <t>Veterinary practice (small independent group)</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -43539,7 +45515,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>Conveyancing solicitors</t>
+          <t>Law firm (conveyancing, family, private client)</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -43549,7 +45525,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>Law firm (residential &amp; commercial property)</t>
+          <t>Law firm (conveyancing, private client)</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -43559,7 +45535,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>Law firm (conveyancing, private client, family)</t>
+          <t>Conveyancing solicitors</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -43569,7 +45545,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>Solar &amp; heat pump installer</t>
+          <t>Law firm (residential &amp; commercial property)</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -43579,7 +45555,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>Solar PV &amp; electrical installer</t>
+          <t>Law firm (conveyancing, private client, family)</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -43589,7 +45565,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>Heat pump &amp; EV charger installer</t>
+          <t>Solar &amp; heat pump installer</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -43599,7 +45575,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>Solar PV &amp; EV charger installer</t>
+          <t>Solar PV &amp; electrical installer</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -43609,7 +45585,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>Electrical contractor &amp; solar installer</t>
+          <t>Heat pump &amp; EV charger installer</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -43619,7 +45595,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>Solar PV installer</t>
+          <t>Solar PV &amp; EV charger installer</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -43629,7 +45605,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>Classical Pilates studio</t>
+          <t>Electrical contractor &amp; solar installer</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -43639,7 +45615,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>Pilates &amp; yoga studio (+ teacher training)</t>
+          <t>Solar PV installer</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -43649,7 +45625,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>Yoga, barre &amp; Pilates studio (+ teacher training)</t>
+          <t>Classical Pilates studio</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -43659,7 +45635,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>Women-only strength &amp; personal training studio</t>
+          <t>Pilates &amp; yoga studio (+ teacher training)</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -43669,7 +45645,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>Immigration &amp; commercial law firm</t>
+          <t>Yoga, barre &amp; Pilates studio (+ teacher training)</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -43679,7 +45655,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>Immigration law firm (UK/US)</t>
+          <t>Women-only strength &amp; personal training studio</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -43689,7 +45665,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>Private client law firm (wills, trusts, estates)</t>
+          <t>Immigration &amp; commercial law firm</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -43699,7 +45675,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>Private wealth &amp; estate planning law firm</t>
+          <t>Immigration law firm (UK/US)</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -43709,7 +45685,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>Private wealth law firm (UHNW)</t>
+          <t>Private client law firm (wills, trusts, estates)</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -43719,10 +45695,190 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
+          <t>Private wealth &amp; estate planning law firm</t>
+        </is>
+      </c>
+      <c r="B209" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>Private wealth law firm (UHNW)</t>
+        </is>
+      </c>
+      <c r="B210" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
           <t>Residential &amp; domiciliary care provider</t>
         </is>
       </c>
-      <c r="B209" t="n">
+      <c r="B211" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>Outdoor 'Forest School' nursery</t>
+        </is>
+      </c>
+      <c r="B212" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>Day nursery group (3 sites)</t>
+        </is>
+      </c>
+      <c r="B213" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>Day nursery &amp; pre-school</t>
+        </is>
+      </c>
+      <c r="B214" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>Chartered lifestyle financial planning</t>
+        </is>
+      </c>
+      <c r="B215" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>Chartered independent financial planning</t>
+        </is>
+      </c>
+      <c r="B216" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>IT support &amp; managed services (MSP)</t>
+        </is>
+      </c>
+      <c r="B217" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>Outsourced finance &amp; business consultancy</t>
+        </is>
+      </c>
+      <c r="B218" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>IT support, hosting &amp; web development (MSP)</t>
+        </is>
+      </c>
+      <c r="B219" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>IT support (MSP)</t>
+        </is>
+      </c>
+      <c r="B220" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>Executive coaching &amp; leadership training</t>
+        </is>
+      </c>
+      <c r="B221" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>Lime plastering/render conservation specialist</t>
+        </is>
+      </c>
+      <c r="B222" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>Lime plastering &amp; traditional render specialist</t>
+        </is>
+      </c>
+      <c r="B223" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>Sash window manufacture &amp; restoration</t>
+        </is>
+      </c>
+      <c r="B224" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>Bespoke joinery (sash windows, doors, cabinetry)</t>
+        </is>
+      </c>
+      <c r="B225" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>Bespoke joinery for listed/conservation buildings</t>
+        </is>
+      </c>
+      <c r="B226" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>Conservation/heritage builder</t>
+        </is>
+      </c>
+      <c r="B227" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batches 57-60: +16 prospects (507 total) - chiropractors/osteopaths/physios, builders/roofers/electricians, dentists, Winchester/Henley/Marlow businesses
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$492</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$508</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T492"/>
+  <dimension ref="A1:T508"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -43620,8 +43620,1460 @@
       </c>
       <c r="T492" s="4" t="inlineStr"/>
     </row>
+    <row r="493">
+      <c r="A493" s="3" t="inlineStr">
+        <is>
+          <t>The Guildford Spine Centre</t>
+        </is>
+      </c>
+      <c r="B493" s="3" t="inlineStr">
+        <is>
+          <t>Chiropractic clinic</t>
+        </is>
+      </c>
+      <c r="C493" s="3" t="inlineStr">
+        <is>
+          <t>Guildford, Surrey</t>
+        </is>
+      </c>
+      <c r="D493" s="3" t="inlineStr">
+        <is>
+          <t>https://www.spinecentreguildford.co.uk</t>
+        </is>
+      </c>
+      <c r="E493" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F493" s="3" t="inlineStr">
+        <is>
+          <t>01483 808868</t>
+        </is>
+      </c>
+      <c r="G493" s="3" t="inlineStr">
+        <is>
+          <t>Alex Symington (Founder, est. 2014)</t>
+        </is>
+      </c>
+      <c r="H493" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/alex-spinecentreguildford-3192a5290</t>
+        </is>
+      </c>
+      <c r="I493" s="3" t="inlineStr">
+        <is>
+          <t>instagram.com/guildfordspinecentre</t>
+        </is>
+      </c>
+      <c r="J493" s="3" t="inlineStr">
+        <is>
+          <t>11-year independent chiropractic clinic founded by a former busy London practitioner; private treatment packages worth hundreds to thousands per patient</t>
+        </is>
+      </c>
+      <c r="K493" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L493" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M493" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N493" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O493" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn/Instagram presence; 11-year trading history</t>
+        </is>
+      </c>
+      <c r="P493" s="3" t="inlineStr">
+        <is>
+          <t>11-year heritage not yet the AI-cited answer for 'chiropractor Guildford'</t>
+        </is>
+      </c>
+      <c r="Q493" s="3" t="inlineStr">
+        <is>
+          <t>'From a busy London practice to Guildford's trusted chiropractor - own that AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R493" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S493" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T493" s="3" t="inlineStr"/>
+    </row>
+    <row r="494">
+      <c r="A494" s="3" t="inlineStr">
+        <is>
+          <t>The Atman Clinic</t>
+        </is>
+      </c>
+      <c r="B494" s="3" t="inlineStr">
+        <is>
+          <t>Osteopathy clinic</t>
+        </is>
+      </c>
+      <c r="C494" s="3" t="inlineStr">
+        <is>
+          <t>Southborough, Tunbridge Wells, Kent</t>
+        </is>
+      </c>
+      <c r="D494" s="3" t="inlineStr">
+        <is>
+          <t>https://www.atmanclinic.co.uk</t>
+        </is>
+      </c>
+      <c r="E494" s="3" t="inlineStr">
+        <is>
+          <t>info@atmanclinic.co.uk</t>
+        </is>
+      </c>
+      <c r="F494" s="3" t="inlineStr">
+        <is>
+          <t>01892 544 783</t>
+        </is>
+      </c>
+      <c r="G494" s="3" t="inlineStr">
+        <is>
+          <t>Geoffrey Montague-Smith D.O. (Founder, est. 1994)</t>
+        </is>
+      </c>
+      <c r="H494" s="3" t="inlineStr"/>
+      <c r="I494" s="3" t="inlineStr"/>
+      <c r="J494" s="3" t="inlineStr">
+        <is>
+          <t>31-year established osteopathy clinic offering structural/cranial osteopathy and sports injury treatment; private treatment packages worth hundreds to thousands per patient</t>
+        </is>
+      </c>
+      <c r="K494" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L494" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M494" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N494" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O494" s="3" t="inlineStr">
+        <is>
+          <t>31-year trading history</t>
+        </is>
+      </c>
+      <c r="P494" s="3" t="inlineStr">
+        <is>
+          <t>31-year heritage not yet the AI-cited answer for 'osteopath Tunbridge Wells'</t>
+        </is>
+      </c>
+      <c r="Q494" s="3" t="inlineStr">
+        <is>
+          <t>'31 years of osteopathic care in Tunbridge Wells - own that AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R494" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S494" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T494" s="3" t="inlineStr"/>
+    </row>
+    <row r="495">
+      <c r="A495" s="4" t="inlineStr">
+        <is>
+          <t>CJ Osteopathy</t>
+        </is>
+      </c>
+      <c r="B495" s="4" t="inlineStr">
+        <is>
+          <t>Osteopathy clinic</t>
+        </is>
+      </c>
+      <c r="C495" s="4" t="inlineStr">
+        <is>
+          <t>Tunbridge Wells, Kent</t>
+        </is>
+      </c>
+      <c r="D495" s="4" t="inlineStr">
+        <is>
+          <t>https://cjosteopathy.co.uk</t>
+        </is>
+      </c>
+      <c r="E495" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F495" s="4" t="inlineStr"/>
+      <c r="G495" s="4" t="inlineStr">
+        <is>
+          <t>Caroline Jack (Founder/Principal Osteopath, est. 2009)</t>
+        </is>
+      </c>
+      <c r="H495" s="4" t="inlineStr"/>
+      <c r="I495" s="4" t="inlineStr">
+        <is>
+          <t>facebook.com/osteopathyCJ</t>
+        </is>
+      </c>
+      <c r="J495" s="4" t="inlineStr">
+        <is>
+          <t>16-year solo-practitioner osteopathy clinic in central Tunbridge Wells with 50+ patient reviews; private treatment packages worth hundreds to thousands per patient</t>
+        </is>
+      </c>
+      <c r="K495" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L495" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M495" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N495" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O495" s="4" t="inlineStr">
+        <is>
+          <t>Facebook presence; 52 reviews on Birdeye</t>
+        </is>
+      </c>
+      <c r="P495" s="4" t="inlineStr">
+        <is>
+          <t>Strong review base not yet converted into AI-cited answers for 'osteopath Tunbridge Wells'</t>
+        </is>
+      </c>
+      <c r="Q495" s="4" t="inlineStr">
+        <is>
+          <t>'52+ patient reviews - let's make AI cite those, not just Google'</t>
+        </is>
+      </c>
+      <c r="R495" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S495" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T495" s="4" t="inlineStr"/>
+    </row>
+    <row r="496">
+      <c r="A496" s="3" t="inlineStr">
+        <is>
+          <t>Weybridge &amp; Walton Physiotherapy</t>
+        </is>
+      </c>
+      <c r="B496" s="3" t="inlineStr">
+        <is>
+          <t>Physiotherapy clinic (3 locations)</t>
+        </is>
+      </c>
+      <c r="C496" s="3" t="inlineStr">
+        <is>
+          <t>Weybridge, Walton-on-Thames &amp; Brooklands, Surrey</t>
+        </is>
+      </c>
+      <c r="D496" s="3" t="inlineStr">
+        <is>
+          <t>https://www.weybridgephysio.co.uk</t>
+        </is>
+      </c>
+      <c r="E496" s="3" t="inlineStr">
+        <is>
+          <t>info@weybridgephysio.co.uk</t>
+        </is>
+      </c>
+      <c r="F496" s="3" t="inlineStr">
+        <is>
+          <t>01932 847 900</t>
+        </is>
+      </c>
+      <c r="G496" s="3" t="inlineStr">
+        <is>
+          <t>Michael O'Reilly (Founder, est. 2005)</t>
+        </is>
+      </c>
+      <c r="H496" s="3" t="inlineStr"/>
+      <c r="I496" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/WeybridgeWaltonPhysiotherapy</t>
+        </is>
+      </c>
+      <c r="J496" s="3" t="inlineStr">
+        <is>
+          <t>20-year independent physiotherapy practice across 3 Surrey locations; private treatment packages worth hundreds to thousands per patient</t>
+        </is>
+      </c>
+      <c r="K496" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L496" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M496" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N496" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O496" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence; 3-location expansion; 20-year trading history</t>
+        </is>
+      </c>
+      <c r="P496" s="3" t="inlineStr">
+        <is>
+          <t>3-location footprint not matched by 3-location AI-search dominance</t>
+        </is>
+      </c>
+      <c r="Q496" s="3" t="inlineStr">
+        <is>
+          <t>Per-location AEO content to own Weybridge/Walton/Brooklands 'physio near me' searches separately</t>
+        </is>
+      </c>
+      <c r="R496" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S496" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T496" s="3" t="inlineStr"/>
+    </row>
+    <row r="497">
+      <c r="A497" s="4" t="inlineStr">
+        <is>
+          <t>Vitality Physiotherapy</t>
+        </is>
+      </c>
+      <c r="B497" s="4" t="inlineStr">
+        <is>
+          <t>Physiotherapy clinic</t>
+        </is>
+      </c>
+      <c r="C497" s="4" t="inlineStr">
+        <is>
+          <t>Esher, Surrey (+ Southwark, London)</t>
+        </is>
+      </c>
+      <c r="D497" s="4" t="inlineStr">
+        <is>
+          <t>https://www.vitality-physio.co.uk</t>
+        </is>
+      </c>
+      <c r="E497" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F497" s="4" t="inlineStr">
+        <is>
+          <t>020 7193 9928</t>
+        </is>
+      </c>
+      <c r="G497" s="4" t="inlineStr">
+        <is>
+          <t>Janine Enoch (Founder/Clinical Director)</t>
+        </is>
+      </c>
+      <c r="H497" s="4" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/vitalityphysio</t>
+        </is>
+      </c>
+      <c r="I497" s="4" t="inlineStr"/>
+      <c r="J497" s="4" t="inlineStr">
+        <is>
+          <t>Two-location physiotherapy practice with a shoulder/respiratory/running specialist founder; private treatment packages worth hundreds to thousands per patient</t>
+        </is>
+      </c>
+      <c r="K497" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L497" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M497" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N497" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O497" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn presence</t>
+        </is>
+      </c>
+      <c r="P497" s="4" t="inlineStr">
+        <is>
+          <t>New Esher location not yet the AI-cited answer for 'physiotherapist Esher'</t>
+        </is>
+      </c>
+      <c r="Q497" s="4" t="inlineStr">
+        <is>
+          <t>'New to Esher - be the AI-cited answer before competitors are'</t>
+        </is>
+      </c>
+      <c r="R497" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S497" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T497" s="4" t="inlineStr">
+        <is>
+          <t>Recently opened Esher location per LinkedIn post</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" s="2" t="inlineStr">
+        <is>
+          <t>EAB Homes</t>
+        </is>
+      </c>
+      <c r="B498" s="2" t="inlineStr">
+        <is>
+          <t>Luxury home builder &amp; developer</t>
+        </is>
+      </c>
+      <c r="C498" s="2" t="inlineStr">
+        <is>
+          <t>Beaconsfield, Buckinghamshire</t>
+        </is>
+      </c>
+      <c r="D498" s="2" t="inlineStr">
+        <is>
+          <t>https://www.eabhomes.co.uk</t>
+        </is>
+      </c>
+      <c r="E498" s="2" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F498" s="2" t="inlineStr"/>
+      <c r="G498" s="2" t="inlineStr">
+        <is>
+          <t>Paul (Founder, started 1986) &amp; Julia (Partner)</t>
+        </is>
+      </c>
+      <c r="H498" s="2" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/eab-homes</t>
+        </is>
+      </c>
+      <c r="I498" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/eabhomes</t>
+        </is>
+      </c>
+      <c r="J498" s="2" t="inlineStr">
+        <is>
+          <t>39-year bespoke luxury new-build and extension specialist serving Beaconsfield/Marlow; project fees run into hundreds of thousands per build</t>
+        </is>
+      </c>
+      <c r="K498" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L498" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M498" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N498" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O498" s="2" t="inlineStr">
+        <is>
+          <t>Facebook/LinkedIn presence; 39-year trading history</t>
+        </is>
+      </c>
+      <c r="P498" s="2" t="inlineStr">
+        <is>
+          <t>39-year heritage not yet the AI-cited answer for 'luxury home builder Beaconsfield'</t>
+        </is>
+      </c>
+      <c r="Q498" s="2" t="inlineStr">
+        <is>
+          <t>'39 years building Beaconsfield's finest homes - own that exact AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R498" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S498" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T498" s="2" t="inlineStr">
+        <is>
+          <t>39-year heritage + very high-value builds - strong AEO opportunity</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" s="4" t="inlineStr">
+        <is>
+          <t>G R Regan &amp; Son</t>
+        </is>
+      </c>
+      <c r="B499" s="4" t="inlineStr">
+        <is>
+          <t>Roofing contractor</t>
+        </is>
+      </c>
+      <c r="C499" s="4" t="inlineStr">
+        <is>
+          <t>Sevenoaks, Kent</t>
+        </is>
+      </c>
+      <c r="D499" s="4" t="inlineStr">
+        <is>
+          <t>https://www.grreganroofing.com</t>
+        </is>
+      </c>
+      <c r="E499" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F499" s="4" t="inlineStr">
+        <is>
+          <t>01732 463 156</t>
+        </is>
+      </c>
+      <c r="G499" s="4" t="inlineStr">
+        <is>
+          <t>Family-owned, est. ~1994 (30 years trading)</t>
+        </is>
+      </c>
+      <c r="H499" s="4" t="inlineStr"/>
+      <c r="I499" s="4" t="inlineStr"/>
+      <c r="J499" s="4" t="inlineStr">
+        <is>
+          <t>30-year family-owned roofing business serving Sevenoaks and the South East; project fees run into thousands per roof</t>
+        </is>
+      </c>
+      <c r="K499" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L499" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M499" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N499" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O499" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P499" s="4" t="inlineStr">
+        <is>
+          <t>30-year heritage not yet the AI-cited answer for 'roofer Sevenoaks'</t>
+        </is>
+      </c>
+      <c r="Q499" s="4" t="inlineStr">
+        <is>
+          <t>'30 years of family roofing in Sevenoaks - own that AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R499" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S499" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T499" s="4" t="inlineStr"/>
+    </row>
+    <row r="500">
+      <c r="A500" s="3" t="inlineStr">
+        <is>
+          <t>Weatherall Roofing</t>
+        </is>
+      </c>
+      <c r="B500" s="3" t="inlineStr">
+        <is>
+          <t>Roofing contractor</t>
+        </is>
+      </c>
+      <c r="C500" s="3" t="inlineStr">
+        <is>
+          <t>Southborough, Tunbridge Wells, Kent</t>
+        </is>
+      </c>
+      <c r="D500" s="3" t="inlineStr">
+        <is>
+          <t>https://www.weatherallroofing.co.uk</t>
+        </is>
+      </c>
+      <c r="E500" s="3" t="inlineStr">
+        <is>
+          <t>enquiry@weatherallroofing.co.uk</t>
+        </is>
+      </c>
+      <c r="F500" s="3" t="inlineStr">
+        <is>
+          <t>01892 535478</t>
+        </is>
+      </c>
+      <c r="G500" s="3" t="inlineStr">
+        <is>
+          <t>Clive Berry (Founder)</t>
+        </is>
+      </c>
+      <c r="H500" s="3" t="inlineStr"/>
+      <c r="I500" s="3" t="inlineStr"/>
+      <c r="J500" s="3" t="inlineStr">
+        <is>
+          <t>40+ year family-run roofing firm covering all aspects of roofing (incl. EPDM/green/slate) across Tunbridge Wells/Tonbridge/Sevenoaks; project fees run into thousands per roof</t>
+        </is>
+      </c>
+      <c r="K500" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L500" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M500" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N500" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O500" s="3" t="inlineStr">
+        <is>
+          <t>TrustMark accreditation; 40+ year trading history</t>
+        </is>
+      </c>
+      <c r="P500" s="3" t="inlineStr">
+        <is>
+          <t>40-year heritage not yet the AI-cited answer for 'roofer Tunbridge Wells'</t>
+        </is>
+      </c>
+      <c r="Q500" s="3" t="inlineStr">
+        <is>
+          <t>'40+ years of family roofing expertise - own that exact AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R500" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S500" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T500" s="3" t="inlineStr"/>
+    </row>
+    <row r="501">
+      <c r="A501" s="4" t="inlineStr">
+        <is>
+          <t>Nixon Electrical Contractors</t>
+        </is>
+      </c>
+      <c r="B501" s="4" t="inlineStr">
+        <is>
+          <t>Electrical contractor</t>
+        </is>
+      </c>
+      <c r="C501" s="4" t="inlineStr">
+        <is>
+          <t>Chesham, Buckinghamshire (Amersham/Beaconsfield/Chalfonts)</t>
+        </is>
+      </c>
+      <c r="D501" s="4" t="inlineStr">
+        <is>
+          <t>https://www.cheshamelectrician.co.uk</t>
+        </is>
+      </c>
+      <c r="E501" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F501" s="4" t="inlineStr">
+        <is>
+          <t>07973 660552</t>
+        </is>
+      </c>
+      <c r="G501" s="4" t="inlineStr">
+        <is>
+          <t>Martin Nixon (Founder, est. 1996)</t>
+        </is>
+      </c>
+      <c r="H501" s="4" t="inlineStr"/>
+      <c r="I501" s="4" t="inlineStr">
+        <is>
+          <t>facebook.com/nixonelectricalcontractors</t>
+        </is>
+      </c>
+      <c r="J501" s="4" t="inlineStr">
+        <is>
+          <t>29-year NICEIC-approved, City &amp; Guilds-qualified electrical contractor serving Chesham/Amersham/Beaconsfield/Chalfont St Giles; project fees run into thousands per job with repeat commercial clients</t>
+        </is>
+      </c>
+      <c r="K501" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L501" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M501" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N501" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O501" s="4" t="inlineStr">
+        <is>
+          <t>Facebook presence; NICEIC accreditation; 29-year trading history</t>
+        </is>
+      </c>
+      <c r="P501" s="4" t="inlineStr">
+        <is>
+          <t>29-year NICEIC-approved heritage not yet the AI-cited answer for 'electrician Chesham'</t>
+        </is>
+      </c>
+      <c r="Q501" s="4" t="inlineStr">
+        <is>
+          <t>'29 years NICEIC-approved in Chesham and Amersham - own that AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R501" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S501" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T501" s="4" t="inlineStr"/>
+    </row>
+    <row r="502">
+      <c r="A502" s="3" t="inlineStr">
+        <is>
+          <t>Lovat House Dental Practice</t>
+        </is>
+      </c>
+      <c r="B502" s="3" t="inlineStr">
+        <is>
+          <t>Dental practice (specialist, implants, aesthetics)</t>
+        </is>
+      </c>
+      <c r="C502" s="3" t="inlineStr">
+        <is>
+          <t>Cheltenham</t>
+        </is>
+      </c>
+      <c r="D502" s="3" t="inlineStr">
+        <is>
+          <t>https://lovathousedental.co.uk</t>
+        </is>
+      </c>
+      <c r="E502" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F502" s="3" t="inlineStr">
+        <is>
+          <t>01242 522841</t>
+        </is>
+      </c>
+      <c r="G502" s="3" t="inlineStr">
+        <is>
+          <t>James Barber &amp; Andrew Barber (Brothers, Principal Dental Surgeons)</t>
+        </is>
+      </c>
+      <c r="H502" s="3" t="inlineStr"/>
+      <c r="I502" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/lovathousedentalcheltenham</t>
+        </is>
+      </c>
+      <c r="J502" s="3" t="inlineStr">
+        <is>
+          <t>Independent brother-owned specialist dental practice offering implants and aesthetic dentistry; private treatment fees run into thousands per patient</t>
+        </is>
+      </c>
+      <c r="K502" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L502" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M502" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N502" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O502" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence</t>
+        </is>
+      </c>
+      <c r="P502" s="3" t="inlineStr">
+        <is>
+          <t>Brother-owned specialist practice not yet the AI-cited answer for 'dental implants Cheltenham'</t>
+        </is>
+      </c>
+      <c r="Q502" s="3" t="inlineStr">
+        <is>
+          <t>'Two brothers, one specialist dental practice - own that AEO trust story'</t>
+        </is>
+      </c>
+      <c r="R502" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S502" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T502" s="3" t="inlineStr"/>
+    </row>
+    <row r="503">
+      <c r="A503" s="3" t="inlineStr">
+        <is>
+          <t>17 Dental</t>
+        </is>
+      </c>
+      <c r="B503" s="3" t="inlineStr">
+        <is>
+          <t>Dental practice (general, cosmetic, surgical)</t>
+        </is>
+      </c>
+      <c r="C503" s="3" t="inlineStr">
+        <is>
+          <t>Guildford, Surrey</t>
+        </is>
+      </c>
+      <c r="D503" s="3" t="inlineStr">
+        <is>
+          <t>https://www.17dental.com</t>
+        </is>
+      </c>
+      <c r="E503" s="3" t="inlineStr">
+        <is>
+          <t>17dental@gmail.com</t>
+        </is>
+      </c>
+      <c r="F503" s="3" t="inlineStr">
+        <is>
+          <t>01483 575908</t>
+        </is>
+      </c>
+      <c r="G503" s="3" t="inlineStr">
+        <is>
+          <t>Dr Waseem Akhtar &amp; Associates</t>
+        </is>
+      </c>
+      <c r="H503" s="3" t="inlineStr"/>
+      <c r="I503" s="3" t="inlineStr">
+        <is>
+          <t>instagram.com/17.dental</t>
+        </is>
+      </c>
+      <c r="J503" s="3" t="inlineStr">
+        <is>
+          <t>Long-established independent Guildford practice offering minor oral surgery and dental implants; private treatment fees run into thousands per patient</t>
+        </is>
+      </c>
+      <c r="K503" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L503" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M503" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N503" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O503" s="3" t="inlineStr">
+        <is>
+          <t>Instagram presence</t>
+        </is>
+      </c>
+      <c r="P503" s="3" t="inlineStr">
+        <is>
+          <t>Long-established local reputation not yet the AI-cited answer for 'dentist Guildford'</t>
+        </is>
+      </c>
+      <c r="Q503" s="3" t="inlineStr">
+        <is>
+          <t>'Long-established and independent - own that exact AEO trust signal in Guildford'</t>
+        </is>
+      </c>
+      <c r="R503" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S503" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T503" s="3" t="inlineStr"/>
+    </row>
+    <row r="504">
+      <c r="A504" s="2" t="inlineStr">
+        <is>
+          <t>The Neem Tree Dental Practice (Esher)</t>
+        </is>
+      </c>
+      <c r="B504" s="2" t="inlineStr">
+        <is>
+          <t>Dental practice (holistic, implants, orthodontics)</t>
+        </is>
+      </c>
+      <c r="C504" s="2" t="inlineStr">
+        <is>
+          <t>Esher High Street, Surrey</t>
+        </is>
+      </c>
+      <c r="D504" s="2" t="inlineStr">
+        <is>
+          <t>https://theneemtree.co.uk</t>
+        </is>
+      </c>
+      <c r="E504" s="2" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F504" s="2" t="inlineStr">
+        <is>
+          <t>01372 464 000</t>
+        </is>
+      </c>
+      <c r="G504" s="2" t="inlineStr">
+        <is>
+          <t>Dr Smita (Founder, opened first practice 2004; Esher site since 2006)</t>
+        </is>
+      </c>
+      <c r="H504" s="2" t="inlineStr"/>
+      <c r="I504" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/the.neem.tree.dental.group</t>
+        </is>
+      </c>
+      <c r="J504" s="2" t="inlineStr">
+        <is>
+          <t>One of Surrey's most established dental practices (19 years on Esher High Street), handling complex cases other practices refer out; private treatment fees run into thousands per patient</t>
+        </is>
+      </c>
+      <c r="K504" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L504" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M504" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N504" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O504" s="2" t="inlineStr">
+        <is>
+          <t>Facebook presence; 19-year trading history; complex-referral reputation</t>
+        </is>
+      </c>
+      <c r="P504" s="2" t="inlineStr">
+        <is>
+          <t>19-year heritage and complex-case reputation not yet the AI-cited answer for 'dentist Esher'</t>
+        </is>
+      </c>
+      <c r="Q504" s="2" t="inlineStr">
+        <is>
+          <t>'The practice other dentists refer complex cases to - own that exact AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R504" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S504" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T504" s="2" t="inlineStr">
+        <is>
+          <t>19-year heritage + referral-of-choice reputation - strong AEO hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" s="3" t="inlineStr">
+        <is>
+          <t>Belgarum</t>
+        </is>
+      </c>
+      <c r="B505" s="3" t="inlineStr">
+        <is>
+          <t>Estate &amp; lettings agent</t>
+        </is>
+      </c>
+      <c r="C505" s="3" t="inlineStr">
+        <is>
+          <t>Winchester, Hampshire</t>
+        </is>
+      </c>
+      <c r="D505" s="3" t="inlineStr">
+        <is>
+          <t>https://www.belgarum.com</t>
+        </is>
+      </c>
+      <c r="E505" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F505" s="3" t="inlineStr">
+        <is>
+          <t>01962 844 460</t>
+        </is>
+      </c>
+      <c r="G505" s="3" t="inlineStr">
+        <is>
+          <t>Family-owned (est. 1989 as a letting agent, sales dept. added 2003)</t>
+        </is>
+      </c>
+      <c r="H505" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/belgarum-estate-agents-limited</t>
+        </is>
+      </c>
+      <c r="I505" s="3" t="inlineStr"/>
+      <c r="J505" s="3" t="inlineStr">
+        <is>
+          <t>36-year family-owned independent Winchester agent with an explicit 'anti-corporate ethos'; sales commissions on premium Winchester property are substantial</t>
+        </is>
+      </c>
+      <c r="K505" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L505" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M505" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N505" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O505" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn presence; explicit 'independent, anti-corporate' marketing message; 36-year heritage</t>
+        </is>
+      </c>
+      <c r="P505" s="3" t="inlineStr">
+        <is>
+          <t>'Anti-corporate' positioning not yet the AI-cited answer for 'estate agent Winchester'</t>
+        </is>
+      </c>
+      <c r="Q505" s="3" t="inlineStr">
+        <is>
+          <t>'36 years of anti-corporate, independent service - own that exact AEO positioning'</t>
+        </is>
+      </c>
+      <c r="R505" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S505" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T505" s="3" t="inlineStr"/>
+    </row>
+    <row r="506">
+      <c r="A506" s="3" t="inlineStr">
+        <is>
+          <t>HÁM Interiors</t>
+        </is>
+      </c>
+      <c r="B506" s="3" t="inlineStr">
+        <is>
+          <t>Architecture, interior design &amp; build practice</t>
+        </is>
+      </c>
+      <c r="C506" s="3" t="inlineStr">
+        <is>
+          <t>Hambleden Valley, nr Henley-on-Thames</t>
+        </is>
+      </c>
+      <c r="D506" s="3" t="inlineStr">
+        <is>
+          <t>https://www.haminteriors.com</t>
+        </is>
+      </c>
+      <c r="E506" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F506" s="3" t="inlineStr"/>
+      <c r="G506" s="3" t="inlineStr">
+        <is>
+          <t>Nick, Pamela, Kate &amp; Tom Cox (Family founders, est. 2011)</t>
+        </is>
+      </c>
+      <c r="H506" s="3" t="inlineStr"/>
+      <c r="I506" s="3" t="inlineStr"/>
+      <c r="J506" s="3" t="inlineStr">
+        <is>
+          <t>14-year family-run architecture/interiors/build practice in the Hambleden Valley; project fees run into tens of thousands per client</t>
+        </is>
+      </c>
+      <c r="K506" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L506" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M506" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N506" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O506" s="3" t="inlineStr">
+        <is>
+          <t>14-year family-run trading history</t>
+        </is>
+      </c>
+      <c r="P506" s="3" t="inlineStr">
+        <is>
+          <t>Family-run, full-service (design + build) positioning not yet the AI-cited answer for 'interior design Henley'</t>
+        </is>
+      </c>
+      <c r="Q506" s="3" t="inlineStr">
+        <is>
+          <t>'One family, design through to build - own that exact AEO full-service positioning'</t>
+        </is>
+      </c>
+      <c r="R506" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S506" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T506" s="3" t="inlineStr"/>
+    </row>
+    <row r="507">
+      <c r="A507" s="4" t="inlineStr">
+        <is>
+          <t>Marlow Face &amp; Body</t>
+        </is>
+      </c>
+      <c r="B507" s="4" t="inlineStr">
+        <is>
+          <t>Aesthetics clinic (face, body, skin)</t>
+        </is>
+      </c>
+      <c r="C507" s="4" t="inlineStr">
+        <is>
+          <t>Marlow, Buckinghamshire</t>
+        </is>
+      </c>
+      <c r="D507" s="4" t="inlineStr">
+        <is>
+          <t>https://marlowfaceandbody.com</t>
+        </is>
+      </c>
+      <c r="E507" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F507" s="4" t="inlineStr"/>
+      <c r="G507" s="4" t="inlineStr">
+        <is>
+          <t>Elisabeth Bester (Founder, est. 2014)</t>
+        </is>
+      </c>
+      <c r="H507" s="4" t="inlineStr"/>
+      <c r="I507" s="4" t="inlineStr">
+        <is>
+          <t>instagram.com/marlowfaceandbody (handle per site posts)</t>
+        </is>
+      </c>
+      <c r="J507" s="4" t="inlineStr">
+        <is>
+          <t>11-year independent aesthetics clinic (cryolipolysis, radiofrequency, LED photon therapy); repeat treatment clients, premium per-session fees</t>
+        </is>
+      </c>
+      <c r="K507" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L507" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M507" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N507" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O507" s="4" t="inlineStr">
+        <is>
+          <t>Instagram presence; 11-year trading history</t>
+        </is>
+      </c>
+      <c r="P507" s="4" t="inlineStr">
+        <is>
+          <t>11-year heritage not yet the AI-cited answer for 'aesthetics clinic Marlow'</t>
+        </is>
+      </c>
+      <c r="Q507" s="4" t="inlineStr">
+        <is>
+          <t>'11 years of trusted aesthetics treatments in Marlow - own that AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R507" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S507" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T507" s="4" t="inlineStr"/>
+    </row>
+    <row r="508">
+      <c r="A508" s="3" t="inlineStr">
+        <is>
+          <t>Appearance Based Medicine (AB Med)</t>
+        </is>
+      </c>
+      <c r="B508" s="3" t="inlineStr">
+        <is>
+          <t>Medical aesthetics clinic</t>
+        </is>
+      </c>
+      <c r="C508" s="3" t="inlineStr">
+        <is>
+          <t>Marlow, Buckinghamshire</t>
+        </is>
+      </c>
+      <c r="D508" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ab-med.co.uk</t>
+        </is>
+      </c>
+      <c r="E508" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F508" s="3" t="inlineStr"/>
+      <c r="G508" s="3" t="inlineStr">
+        <is>
+          <t>Clare McLoughlin RGN INP (Founder, pioneering medical aesthetics since 1999)</t>
+        </is>
+      </c>
+      <c r="H508" s="3" t="inlineStr"/>
+      <c r="I508" s="3" t="inlineStr"/>
+      <c r="J508" s="3" t="inlineStr">
+        <is>
+          <t>Founded by a pioneering nurse prescriber with 25+ years in medical aesthetics; repeat treatment clients, premium per-session fees</t>
+        </is>
+      </c>
+      <c r="K508" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L508" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M508" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N508" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O508" s="3" t="inlineStr">
+        <is>
+          <t>25+ year pioneer credential = strong authority asset</t>
+        </is>
+      </c>
+      <c r="P508" s="3" t="inlineStr">
+        <is>
+          <t>Pioneer-since-1999 story not yet the AI-cited trust signal for 'medical aesthetics Marlow'</t>
+        </is>
+      </c>
+      <c r="Q508" s="3" t="inlineStr">
+        <is>
+          <t>'A pioneer in medical aesthetics since 1999 - own that exact AEO authority signal'</t>
+        </is>
+      </c>
+      <c r="R508" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S508" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T508" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T492"/>
+  <autoFilter ref="A1:T508"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -43632,7 +45084,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B227"/>
+  <dimension ref="A1:B238"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -43652,7 +45104,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>491</v>
+        <v>507</v>
       </c>
     </row>
     <row r="5">
@@ -43755,7 +45207,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Aesthetics clinic</t>
+          <t>Physiotherapy clinic</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -43765,11 +45217,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Physiotherapy clinic</t>
+          <t>Aesthetics clinic</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="17">
@@ -43795,7 +45247,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Recruitment agency</t>
+          <t>Osteopathy clinic</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -43805,7 +45257,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>IT support / MSP</t>
+          <t>Recruitment agency</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -43815,27 +45267,27 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Interior design studio</t>
+          <t>IT support / MSP</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Law firm</t>
+          <t>Interior design studio</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Letting agent</t>
+          <t>Law firm</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -43845,7 +45297,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Private tuition agency</t>
+          <t>Letting agent</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -43855,7 +45307,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Osteopathy clinic</t>
+          <t>Private tuition agency</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -44195,7 +45647,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Driving school &amp; ADI instructor training</t>
+          <t>Estate &amp; lettings agent</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -44205,7 +45657,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Veterinary practice</t>
+          <t>Driving school &amp; ADI instructor training</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -44215,7 +45667,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Reformer Pilates studio</t>
+          <t>Veterinary practice</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -44225,7 +45677,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Home care &amp; live-in care agency</t>
+          <t>Reformer Pilates studio</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -44235,7 +45687,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Private tuition (primary/11+)</t>
+          <t>Home care &amp; live-in care agency</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -44245,7 +45697,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Independent Chartered financial planning</t>
+          <t>Private tuition (primary/11+)</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -44255,27 +45707,27 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Dentist / Orthodontics</t>
+          <t>Independent Chartered financial planning</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Specialist dental/implant clinic</t>
+          <t>Roofing contractor</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Boutique corporate law firm</t>
+          <t>Dentist / Orthodontics</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -44285,7 +45737,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Cosmetic/aesthetics clinic</t>
+          <t>Specialist dental/implant clinic</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -44295,7 +45747,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Skin &amp; laser clinic</t>
+          <t>Boutique corporate law firm</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -44305,7 +45757,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Mortgage broker / financial adviser</t>
+          <t>Cosmetic/aesthetics clinic</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -44315,7 +45767,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Architects (RIBA chartered)</t>
+          <t>Skin &amp; laser clinic</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -44325,7 +45777,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Recruitment agency (tech/startups)</t>
+          <t>Mortgage broker / financial adviser</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -44335,7 +45787,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Recruitment agency (IT/data)</t>
+          <t>Architects (RIBA chartered)</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -44345,7 +45797,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Independent vet (24/7 emergency)</t>
+          <t>Recruitment agency (tech/startups)</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -44355,7 +45807,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Letting &amp; estate agent</t>
+          <t>Recruitment agency (IT/data)</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -44365,7 +45817,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Cosmetic clinic (injectables)</t>
+          <t>Independent vet (24/7 emergency)</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -44375,7 +45827,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Cosmetic/anti-ageing clinic</t>
+          <t>Letting &amp; estate agent</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -44385,7 +45837,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Yoga &amp; reformer pilates studio</t>
+          <t>Cosmetic clinic (injectables)</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -44395,7 +45847,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Reformer pilates studio</t>
+          <t>Cosmetic/anti-ageing clinic</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -44405,7 +45857,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Wealth management</t>
+          <t>Yoga &amp; reformer pilates studio</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -44415,7 +45867,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Private tuition &amp; education consultancy</t>
+          <t>Reformer pilates studio</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -44425,7 +45877,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Osteopath</t>
+          <t>Wealth management</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -44435,7 +45887,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Design &amp; build / home renovation</t>
+          <t>Private tuition &amp; education consultancy</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -44445,7 +45897,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Builders / building contractor</t>
+          <t>Osteopath</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -44455,7 +45907,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Home care / live-in care</t>
+          <t>Design &amp; build / home renovation</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -44465,7 +45917,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Private day nurseries</t>
+          <t>Builders / building contractor</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -44475,7 +45927,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Personal training &amp; wellness studio</t>
+          <t>Home care / live-in care</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -44485,7 +45937,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Mortgage &amp; insurance broker</t>
+          <t>Private day nurseries</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -44495,7 +45947,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Business consultancy</t>
+          <t>Personal training &amp; wellness studio</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -44505,7 +45957,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Interior designer (period homes)</t>
+          <t>Mortgage &amp; insurance broker</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -44515,7 +45967,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Landscape design &amp; build</t>
+          <t>Business consultancy</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -44525,7 +45977,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Interior designer</t>
+          <t>Interior designer (period homes)</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -44535,7 +45987,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Garden design &amp; landscaping</t>
+          <t>Landscape design &amp; build</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -44545,7 +45997,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Legal recruitment</t>
+          <t>Interior designer</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -44555,7 +46007,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Independent gym &amp; health club</t>
+          <t>Garden design &amp; landscaping</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -44565,7 +46017,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Independent gym</t>
+          <t>Legal recruitment</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -44575,7 +46027,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Physiotherapy (sports)</t>
+          <t>Independent gym &amp; health club</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -44585,7 +46037,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Letting agent / property management</t>
+          <t>Independent gym</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -44595,7 +46047,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Skin clinic</t>
+          <t>Physiotherapy (sports)</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -44605,7 +46057,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Tutoring company</t>
+          <t>Letting agent / property management</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -44615,7 +46067,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Tutorial college &amp; exam centre</t>
+          <t>Skin clinic</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -44625,7 +46077,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Employment law (disability discrimination)</t>
+          <t>Tutoring company</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -44635,7 +46087,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating</t>
+          <t>Tutorial college &amp; exam centre</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -44645,7 +46097,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Employment law (disability discrimination)</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -44655,7 +46107,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Sports physio &amp; massage</t>
+          <t>Plumbing &amp; heating</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -44665,7 +46117,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Chartered surveyors (party wall/building)</t>
+          <t>Plumbing</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -44675,7 +46127,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Chartered surveyors</t>
+          <t>Sports physio &amp; massage</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -44685,7 +46137,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Chartered building surveyors</t>
+          <t>Chartered surveyors (party wall/building)</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -44695,7 +46147,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Osteopathy clinics</t>
+          <t>Chartered surveyors</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -44705,7 +46157,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Builders / renovations</t>
+          <t>Chartered building surveyors</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -44715,7 +46167,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Private nursery schools</t>
+          <t>Osteopathy clinics</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -44725,7 +46177,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Private day nursery</t>
+          <t>Builders / renovations</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -44735,7 +46187,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Private GP (membership model)</t>
+          <t>Private nursery schools</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -44745,7 +46197,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Sash window restoration</t>
+          <t>Private day nursery</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -44755,7 +46207,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Personal training (1:1)</t>
+          <t>Private GP (membership model)</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -44765,7 +46217,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Personal training &amp; nutrition coaching</t>
+          <t>Sash window restoration</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -44775,7 +46227,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Private nursery/pre-prep school</t>
+          <t>Personal training (1:1)</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -44785,7 +46237,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Independent nursery (Montessori)</t>
+          <t>Personal training &amp; nutrition coaching</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -44795,7 +46247,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Live-in care agency</t>
+          <t>Private nursery/pre-prep school</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -44805,7 +46257,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Law firm (conveyancing/family)</t>
+          <t>Independent nursery (Montessori)</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -44815,7 +46267,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Architect &amp; interior designer</t>
+          <t>Live-in care agency</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -44825,7 +46277,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Architects / project management</t>
+          <t>Law firm (conveyancing/family)</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -44835,7 +46287,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Physiotherapy &amp; clinical Pilates</t>
+          <t>Architect &amp; interior designer</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -44845,7 +46297,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Aesthetics &amp; skin clinic</t>
+          <t>Architects / project management</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -44855,7 +46307,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>IFA / financial planning</t>
+          <t>Physiotherapy &amp; clinical Pilates</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -44865,7 +46317,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Wealth management &amp; employee benefits</t>
+          <t>Aesthetics &amp; skin clinic</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -44875,7 +46327,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Dermatology clinic</t>
+          <t>IFA / financial planning</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -44885,7 +46337,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Pilates studio (multi-site)</t>
+          <t>Wealth management &amp; employee benefits</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -44895,7 +46347,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Private nursery (Montessori, multi-site)</t>
+          <t>Dermatology clinic</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -44905,7 +46357,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Law firm (wills &amp; probate)</t>
+          <t>Pilates studio (multi-site)</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -44915,7 +46367,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Business/technical consultancy</t>
+          <t>Private nursery (Montessori, multi-site)</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -44925,7 +46377,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Private/NHS dentist</t>
+          <t>Law firm (wills &amp; probate)</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -44935,7 +46387,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Removals company</t>
+          <t>Business/technical consultancy</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -44945,7 +46397,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Driveways &amp; landscaping</t>
+          <t>Private/NHS dentist</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -44955,7 +46407,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Wedding &amp; event venue</t>
+          <t>Removals company</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -44965,7 +46417,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>IFA &amp; mortgage broker</t>
+          <t>Driveways &amp; landscaping</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -44975,7 +46427,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Wedding photography &amp; videography</t>
+          <t>Wedding &amp; event venue</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -44985,7 +46437,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Commercial property litigation law firm</t>
+          <t>IFA &amp; mortgage broker</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -44995,7 +46447,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Recruitment agency (boutique)</t>
+          <t>Wedding photography &amp; videography</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -45005,7 +46457,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Home cinema &amp; smart home installer</t>
+          <t>Commercial property litigation law firm</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -45015,7 +46467,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Home cinema installer</t>
+          <t>Recruitment agency (boutique)</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -45025,7 +46477,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Curtains, blinds &amp; upholstery</t>
+          <t>Home cinema &amp; smart home installer</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -45035,7 +46487,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Bespoke curtains &amp; soft furnishings</t>
+          <t>Home cinema installer</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -45045,7 +46497,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Wine merchant</t>
+          <t>Curtains, blinds &amp; upholstery</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -45055,7 +46507,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Education consultancy (school placement)</t>
+          <t>Bespoke curtains &amp; soft furnishings</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -45065,7 +46517,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Estate agent &amp; surveyors</t>
+          <t>Wine merchant</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -45075,7 +46527,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Independent financial adviser</t>
+          <t>Education consultancy (school placement)</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -45085,7 +46537,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Chartered accountants &amp; financial planners</t>
+          <t>Estate agent &amp; surveyors</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -45095,7 +46547,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Private GP &amp; dermatology</t>
+          <t>Independent financial adviser</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -45105,7 +46557,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Architects (heritage specialism)</t>
+          <t>Chartered accountants &amp; financial planners</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -45115,7 +46567,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Private cosmetic dentist / implants</t>
+          <t>Private GP &amp; dermatology</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -45125,7 +46577,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Heating engineer / plumbing</t>
+          <t>Architects (heritage specialism)</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -45135,7 +46587,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Estate agent (boutique)</t>
+          <t>Private cosmetic dentist / implants</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -45145,7 +46597,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Independent vet (mixed practice)</t>
+          <t>Heating engineer / plumbing</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -45155,7 +46607,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Private dentist / cosmetic</t>
+          <t>Estate agent (boutique)</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -45165,7 +46617,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Chartered accountants &amp; financial advisers</t>
+          <t>Independent vet (mixed practice)</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -45175,7 +46627,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Healthcare recruitment agency</t>
+          <t>Private dentist / cosmetic</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -45185,7 +46637,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Executive search / headhunting</t>
+          <t>Chartered accountants &amp; financial advisers</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -45195,7 +46647,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>First aid &amp; health &amp; safety training</t>
+          <t>Healthcare recruitment agency</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -45205,7 +46657,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Teaching &amp; education recruitment agency</t>
+          <t>Executive search / headhunting</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -45215,7 +46667,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Supply teaching agency</t>
+          <t>First aid &amp; health &amp; safety training</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -45225,7 +46677,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Hospitality staffing agency</t>
+          <t>Teaching &amp; education recruitment agency</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -45235,7 +46687,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Finance &amp; accountancy recruitment agency</t>
+          <t>Supply teaching agency</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -45245,7 +46697,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Accounting &amp; finance recruitment agency</t>
+          <t>Hospitality staffing agency</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -45255,7 +46707,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Forklift &amp; plant operator training</t>
+          <t>Finance &amp; accountancy recruitment agency</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -45265,7 +46717,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Forklift training</t>
+          <t>Accounting &amp; finance recruitment agency</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -45275,7 +46727,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Language school</t>
+          <t>Forklift &amp; plant operator training</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -45285,7 +46737,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Engineering &amp; manufacturing recruitment</t>
+          <t>Forklift training</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -45295,7 +46747,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Business &amp; sales coaching</t>
+          <t>Language school</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -45305,7 +46757,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Engineering &amp; energy recruitment</t>
+          <t>Engineering &amp; manufacturing recruitment</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -45315,7 +46767,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Tech recruitment agency</t>
+          <t>Business &amp; sales coaching</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -45325,7 +46777,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Data/tech/AI recruitment agency</t>
+          <t>Engineering &amp; energy recruitment</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -45335,7 +46787,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Beauty/aesthetics training academy</t>
+          <t>Tech recruitment agency</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -45345,7 +46797,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Beauty/hair training academy</t>
+          <t>Data/tech/AI recruitment agency</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -45355,7 +46807,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>Medical aesthetics/injectable training academy</t>
+          <t>Beauty/aesthetics training academy</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -45365,7 +46817,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Yoga teacher training school</t>
+          <t>Beauty/hair training academy</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -45375,7 +46827,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Creative &amp; marketing recruitment agency</t>
+          <t>Medical aesthetics/injectable training academy</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -45385,7 +46837,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Private dermatology &amp; women's health clinics</t>
+          <t>Yoga teacher training school</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -45395,7 +46847,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>Private dermatology practice</t>
+          <t>Creative &amp; marketing recruitment agency</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -45405,7 +46857,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>Estate &amp; lettings agent</t>
+          <t>Private dermatology &amp; women's health clinics</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -45415,7 +46867,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>Wedding venue (converted barn)</t>
+          <t>Private dermatology practice</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -45425,7 +46877,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>Wedding venue (waterside barn &amp; estate)</t>
+          <t>Wedding venue (converted barn)</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -45435,7 +46887,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>Wedding venue (thatched barn on working farm)</t>
+          <t>Wedding venue (waterside barn &amp; estate)</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -45445,7 +46897,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>Wedding venue (working farm)</t>
+          <t>Wedding venue (thatched barn on working farm)</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -45455,7 +46907,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>Wedding venue (restored historic barn)</t>
+          <t>Wedding venue (working farm)</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -45465,7 +46917,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Chartered IFA / wealth management</t>
+          <t>Wedding venue (restored historic barn)</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -45475,7 +46927,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Independent mortgage broker</t>
+          <t>Chartered IFA / wealth management</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -45485,7 +46937,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Independent financial planning</t>
+          <t>Independent mortgage broker</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -45495,7 +46947,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Chartered independent financial planners</t>
+          <t>Independent financial planning</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -45505,7 +46957,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>Veterinary practice (small independent group)</t>
+          <t>Chartered independent financial planners</t>
         </is>
       </c>
       <c r="B190" t="n">
@@ -45515,7 +46967,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>Law firm (conveyancing, family, private client)</t>
+          <t>Veterinary practice (small independent group)</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -45525,7 +46977,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>Law firm (conveyancing, private client)</t>
+          <t>Law firm (conveyancing, family, private client)</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -45535,7 +46987,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>Conveyancing solicitors</t>
+          <t>Law firm (conveyancing, private client)</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -45545,7 +46997,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>Law firm (residential &amp; commercial property)</t>
+          <t>Conveyancing solicitors</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -45555,7 +47007,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>Law firm (conveyancing, private client, family)</t>
+          <t>Law firm (residential &amp; commercial property)</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -45565,7 +47017,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>Solar &amp; heat pump installer</t>
+          <t>Law firm (conveyancing, private client, family)</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -45575,7 +47027,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>Solar PV &amp; electrical installer</t>
+          <t>Solar &amp; heat pump installer</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -45585,7 +47037,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>Heat pump &amp; EV charger installer</t>
+          <t>Solar PV &amp; electrical installer</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -45595,7 +47047,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>Solar PV &amp; EV charger installer</t>
+          <t>Heat pump &amp; EV charger installer</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -45605,7 +47057,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>Electrical contractor &amp; solar installer</t>
+          <t>Solar PV &amp; EV charger installer</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -45615,7 +47067,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>Solar PV installer</t>
+          <t>Electrical contractor &amp; solar installer</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -45625,7 +47077,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>Classical Pilates studio</t>
+          <t>Solar PV installer</t>
         </is>
       </c>
       <c r="B202" t="n">
@@ -45635,7 +47087,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>Pilates &amp; yoga studio (+ teacher training)</t>
+          <t>Classical Pilates studio</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -45645,7 +47097,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>Yoga, barre &amp; Pilates studio (+ teacher training)</t>
+          <t>Pilates &amp; yoga studio (+ teacher training)</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -45655,7 +47107,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>Women-only strength &amp; personal training studio</t>
+          <t>Yoga, barre &amp; Pilates studio (+ teacher training)</t>
         </is>
       </c>
       <c r="B205" t="n">
@@ -45665,7 +47117,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>Immigration &amp; commercial law firm</t>
+          <t>Women-only strength &amp; personal training studio</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -45675,7 +47127,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>Immigration law firm (UK/US)</t>
+          <t>Immigration &amp; commercial law firm</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -45685,7 +47137,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>Private client law firm (wills, trusts, estates)</t>
+          <t>Immigration law firm (UK/US)</t>
         </is>
       </c>
       <c r="B208" t="n">
@@ -45695,7 +47147,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>Private wealth &amp; estate planning law firm</t>
+          <t>Private client law firm (wills, trusts, estates)</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -45705,7 +47157,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>Private wealth law firm (UHNW)</t>
+          <t>Private wealth &amp; estate planning law firm</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -45715,7 +47167,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>Residential &amp; domiciliary care provider</t>
+          <t>Private wealth law firm (UHNW)</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -45725,7 +47177,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>Outdoor 'Forest School' nursery</t>
+          <t>Residential &amp; domiciliary care provider</t>
         </is>
       </c>
       <c r="B212" t="n">
@@ -45735,7 +47187,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>Day nursery group (3 sites)</t>
+          <t>Outdoor 'Forest School' nursery</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -45745,7 +47197,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>Day nursery &amp; pre-school</t>
+          <t>Day nursery group (3 sites)</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -45755,7 +47207,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>Chartered lifestyle financial planning</t>
+          <t>Day nursery &amp; pre-school</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -45765,7 +47217,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>Chartered independent financial planning</t>
+          <t>Chartered lifestyle financial planning</t>
         </is>
       </c>
       <c r="B216" t="n">
@@ -45775,7 +47227,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>IT support &amp; managed services (MSP)</t>
+          <t>Chartered independent financial planning</t>
         </is>
       </c>
       <c r="B217" t="n">
@@ -45785,7 +47237,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>Outsourced finance &amp; business consultancy</t>
+          <t>IT support &amp; managed services (MSP)</t>
         </is>
       </c>
       <c r="B218" t="n">
@@ -45795,7 +47247,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>IT support, hosting &amp; web development (MSP)</t>
+          <t>Outsourced finance &amp; business consultancy</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -45805,7 +47257,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>IT support (MSP)</t>
+          <t>IT support, hosting &amp; web development (MSP)</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -45815,7 +47267,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>Executive coaching &amp; leadership training</t>
+          <t>IT support (MSP)</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -45825,7 +47277,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>Lime plastering/render conservation specialist</t>
+          <t>Executive coaching &amp; leadership training</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -45835,7 +47287,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>Lime plastering &amp; traditional render specialist</t>
+          <t>Lime plastering/render conservation specialist</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -45845,7 +47297,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>Sash window manufacture &amp; restoration</t>
+          <t>Lime plastering &amp; traditional render specialist</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -45855,7 +47307,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>Bespoke joinery (sash windows, doors, cabinetry)</t>
+          <t>Sash window manufacture &amp; restoration</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -45865,7 +47317,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>Bespoke joinery for listed/conservation buildings</t>
+          <t>Bespoke joinery (sash windows, doors, cabinetry)</t>
         </is>
       </c>
       <c r="B226" t="n">
@@ -45875,10 +47327,120 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
+          <t>Bespoke joinery for listed/conservation buildings</t>
+        </is>
+      </c>
+      <c r="B227" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
           <t>Conservation/heritage builder</t>
         </is>
       </c>
-      <c r="B227" t="n">
+      <c r="B228" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>Chiropractic clinic</t>
+        </is>
+      </c>
+      <c r="B229" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>Physiotherapy clinic (3 locations)</t>
+        </is>
+      </c>
+      <c r="B230" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>Luxury home builder &amp; developer</t>
+        </is>
+      </c>
+      <c r="B231" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>Electrical contractor</t>
+        </is>
+      </c>
+      <c r="B232" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>Dental practice (specialist, implants, aesthetics)</t>
+        </is>
+      </c>
+      <c r="B233" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>Dental practice (general, cosmetic, surgical)</t>
+        </is>
+      </c>
+      <c r="B234" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>Dental practice (holistic, implants, orthodontics)</t>
+        </is>
+      </c>
+      <c r="B235" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>Architecture, interior design &amp; build practice</t>
+        </is>
+      </c>
+      <c r="B236" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>Aesthetics clinic (face, body, skin)</t>
+        </is>
+      </c>
+      <c r="B237" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>Medical aesthetics clinic</t>
+        </is>
+      </c>
+      <c r="B238" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batches 61-62: +6 prospects (513 total) - Hampstead/Highgate/Notting Hill/Greenwich independent businesses
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$508</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$514</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T508"/>
+  <dimension ref="A1:T514"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -45072,8 +45072,548 @@
       </c>
       <c r="T508" s="3" t="inlineStr"/>
     </row>
+    <row r="509">
+      <c r="A509" s="3" t="inlineStr">
+        <is>
+          <t>Litchfields</t>
+        </is>
+      </c>
+      <c r="B509" s="3" t="inlineStr">
+        <is>
+          <t>Estate &amp; lettings agent</t>
+        </is>
+      </c>
+      <c r="C509" s="3" t="inlineStr">
+        <is>
+          <t>Highgate &amp; Hampstead Garden Suburb, London</t>
+        </is>
+      </c>
+      <c r="D509" s="3" t="inlineStr">
+        <is>
+          <t>https://www.litchfields.com</t>
+        </is>
+      </c>
+      <c r="E509" s="3" t="inlineStr">
+        <is>
+          <t>highgate@litchfields.com</t>
+        </is>
+      </c>
+      <c r="F509" s="3" t="inlineStr">
+        <is>
+          <t>020 8348 8000</t>
+        </is>
+      </c>
+      <c r="G509" s="3" t="inlineStr">
+        <is>
+          <t>Independent, privately owned (est. 1989)</t>
+        </is>
+      </c>
+      <c r="H509" s="3" t="inlineStr"/>
+      <c r="I509" s="3" t="inlineStr"/>
+      <c r="J509" s="3" t="inlineStr">
+        <is>
+          <t>36-year independent multi-office agent covering Highgate/Hampstead Garden Suburb/Crouch End; commissions on premium North London property sales are substantial</t>
+        </is>
+      </c>
+      <c r="K509" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L509" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M509" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N509" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O509" s="3" t="inlineStr">
+        <is>
+          <t>36-year trading history; multi-office expansion</t>
+        </is>
+      </c>
+      <c r="P509" s="3" t="inlineStr">
+        <is>
+          <t>36-year heritage not yet the AI-cited answer for 'estate agent Highgate'</t>
+        </is>
+      </c>
+      <c r="Q509" s="3" t="inlineStr">
+        <is>
+          <t>'36 years, run like a family business - own that exact AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R509" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S509" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T509" s="3" t="inlineStr"/>
+    </row>
+    <row r="510">
+      <c r="A510" s="3" t="inlineStr">
+        <is>
+          <t>Day Morris Estate Agents</t>
+        </is>
+      </c>
+      <c r="B510" s="3" t="inlineStr">
+        <is>
+          <t>Estate &amp; lettings agent</t>
+        </is>
+      </c>
+      <c r="C510" s="3" t="inlineStr">
+        <is>
+          <t>Hampstead &amp; Highgate, London</t>
+        </is>
+      </c>
+      <c r="D510" s="3" t="inlineStr">
+        <is>
+          <t>https://daymorris.co.uk</t>
+        </is>
+      </c>
+      <c r="E510" s="3" t="inlineStr">
+        <is>
+          <t>hampstead@daymorris.co.uk</t>
+        </is>
+      </c>
+      <c r="F510" s="3" t="inlineStr">
+        <is>
+          <t>020 7482 4282</t>
+        </is>
+      </c>
+      <c r="G510" s="3" t="inlineStr">
+        <is>
+          <t>Steven Day &amp; John Morris (Founders, est. 1989)</t>
+        </is>
+      </c>
+      <c r="H510" s="3" t="inlineStr"/>
+      <c r="I510" s="3" t="inlineStr"/>
+      <c r="J510" s="3" t="inlineStr">
+        <is>
+          <t>36-year independent agency founded by two of Hampstead's most respected property professionals; commissions on premium North London property sales are substantial</t>
+        </is>
+      </c>
+      <c r="K510" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L510" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M510" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N510" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O510" s="3" t="inlineStr">
+        <is>
+          <t>36-year heritage; founders' local reputation</t>
+        </is>
+      </c>
+      <c r="P510" s="3" t="inlineStr">
+        <is>
+          <t>36-year founder reputation not yet the AI-cited answer for 'estate agent Hampstead'</t>
+        </is>
+      </c>
+      <c r="Q510" s="3" t="inlineStr">
+        <is>
+          <t>'Founded by two of Hampstead's most respected agents - own that AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R510" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S510" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T510" s="3" t="inlineStr"/>
+    </row>
+    <row r="511">
+      <c r="A511" s="3" t="inlineStr">
+        <is>
+          <t>Pembridge Dental</t>
+        </is>
+      </c>
+      <c r="B511" s="3" t="inlineStr">
+        <is>
+          <t>Dental practice (general, cosmetic, implants)</t>
+        </is>
+      </c>
+      <c r="C511" s="3" t="inlineStr">
+        <is>
+          <t>Notting Hill, West London</t>
+        </is>
+      </c>
+      <c r="D511" s="3" t="inlineStr">
+        <is>
+          <t>https://pembridgedental.co.uk</t>
+        </is>
+      </c>
+      <c r="E511" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F511" s="3" t="inlineStr"/>
+      <c r="G511" s="3" t="inlineStr">
+        <is>
+          <t>Dr Ardalan Eghtedar BDS MFDS RCS(Edin) (Principal Dentist, practice est. 1986)</t>
+        </is>
+      </c>
+      <c r="H511" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/aeghtedar</t>
+        </is>
+      </c>
+      <c r="I511" s="3" t="inlineStr"/>
+      <c r="J511" s="3" t="inlineStr">
+        <is>
+          <t>39-year long-established private dental practice serving Kensington/Holland Park/Bayswater/Chelsea; private treatment fees run into thousands per patient, especially implants</t>
+        </is>
+      </c>
+      <c r="K511" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L511" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M511" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N511" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O511" s="3" t="inlineStr">
+        <is>
+          <t>39-year trading history; extensive patient reviews</t>
+        </is>
+      </c>
+      <c r="P511" s="3" t="inlineStr">
+        <is>
+          <t>39-year heritage not yet the AI-cited answer for 'dentist Notting Hill'</t>
+        </is>
+      </c>
+      <c r="Q511" s="3" t="inlineStr">
+        <is>
+          <t>'39 years serving Notting Hill and Kensington - own that exact AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R511" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S511" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T511" s="3" t="inlineStr"/>
+    </row>
+    <row r="512">
+      <c r="A512" s="3" t="inlineStr">
+        <is>
+          <t>Pilates Plus London</t>
+        </is>
+      </c>
+      <c r="B512" s="3" t="inlineStr">
+        <is>
+          <t>Pilates, osteopathy &amp; functional medicine clinic</t>
+        </is>
+      </c>
+      <c r="C512" s="3" t="inlineStr">
+        <is>
+          <t>Blackheath &amp; Greenwich, London</t>
+        </is>
+      </c>
+      <c r="D512" s="3" t="inlineStr">
+        <is>
+          <t>https://www.pilatespluslondon.co.uk</t>
+        </is>
+      </c>
+      <c r="E512" s="3" t="inlineStr">
+        <is>
+          <t>pilatespluss@hotmail.co.uk</t>
+        </is>
+      </c>
+      <c r="F512" s="3" t="inlineStr">
+        <is>
+          <t>020 3305 5563</t>
+        </is>
+      </c>
+      <c r="G512" s="3" t="inlineStr">
+        <is>
+          <t>Galina Bell (Founder, Registered Osteopath, est. 20+ years ago)</t>
+        </is>
+      </c>
+      <c r="H512" s="3" t="inlineStr"/>
+      <c r="I512" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/pilatespluslondon</t>
+        </is>
+      </c>
+      <c r="J512" s="3" t="inlineStr">
+        <is>
+          <t>20+ year multi-discipline clinic combining Pilates, osteopathy, acupuncture and functional medicine; class packages and treatment fees worth hundreds to thousands per client per year</t>
+        </is>
+      </c>
+      <c r="K512" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L512" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M512" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N512" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O512" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence; 20+ year trading history; multi-discipline offering</t>
+        </is>
+      </c>
+      <c r="P512" s="3" t="inlineStr">
+        <is>
+          <t>Multi-discipline offering (Pilates + osteopathy + functional medicine) not yet the AI-cited answer for 'Pilates Blackheath'</t>
+        </is>
+      </c>
+      <c r="Q512" s="3" t="inlineStr">
+        <is>
+          <t>'One clinic for Pilates, osteopathy and functional medicine - own that exact AEO multi-discipline positioning'</t>
+        </is>
+      </c>
+      <c r="R512" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S512" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T512" s="3" t="inlineStr"/>
+    </row>
+    <row r="513">
+      <c r="A513" s="3" t="inlineStr">
+        <is>
+          <t>Godfrey &amp; Barr</t>
+        </is>
+      </c>
+      <c r="B513" s="3" t="inlineStr">
+        <is>
+          <t>Estate agent</t>
+        </is>
+      </c>
+      <c r="C513" s="3" t="inlineStr">
+        <is>
+          <t>Hampstead Garden Suburb, London</t>
+        </is>
+      </c>
+      <c r="D513" s="3" t="inlineStr">
+        <is>
+          <t>https://www.godfreyandbarr.com</t>
+        </is>
+      </c>
+      <c r="E513" s="3" t="inlineStr">
+        <is>
+          <t>enquire@godfreyandbarr.com</t>
+        </is>
+      </c>
+      <c r="F513" s="3" t="inlineStr">
+        <is>
+          <t>020 8458 9119</t>
+        </is>
+      </c>
+      <c r="G513" s="3" t="inlineStr">
+        <is>
+          <t>Ian Godfrey &amp; Jonathan Barr (Founders, est. 1991)</t>
+        </is>
+      </c>
+      <c r="H513" s="3" t="inlineStr"/>
+      <c r="I513" s="3" t="inlineStr"/>
+      <c r="J513" s="3" t="inlineStr">
+        <is>
+          <t>34-year fully independent residential estate agent covering Hampstead Garden Suburb; commissions on premium North London property sales are substantial</t>
+        </is>
+      </c>
+      <c r="K513" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L513" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M513" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N513" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O513" s="3" t="inlineStr">
+        <is>
+          <t>34-year trading history; press features (Fabric Magazine)</t>
+        </is>
+      </c>
+      <c r="P513" s="3" t="inlineStr">
+        <is>
+          <t>34-year heritage and press coverage not yet the AI-cited answer for 'estate agent Hampstead Garden Suburb'</t>
+        </is>
+      </c>
+      <c r="Q513" s="3" t="inlineStr">
+        <is>
+          <t>'34 years, fully independent, featured in Fabric Magazine - own that exact AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R513" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S513" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T513" s="3" t="inlineStr"/>
+    </row>
+    <row r="514">
+      <c r="A514" s="3" t="inlineStr">
+        <is>
+          <t>Studio Duggan</t>
+        </is>
+      </c>
+      <c r="B514" s="3" t="inlineStr">
+        <is>
+          <t>Interior design studio</t>
+        </is>
+      </c>
+      <c r="C514" s="3" t="inlineStr">
+        <is>
+          <t>Notting Hill, London (projects incl. Islington)</t>
+        </is>
+      </c>
+      <c r="D514" s="3" t="inlineStr">
+        <is>
+          <t>https://www.studioduggan.com</t>
+        </is>
+      </c>
+      <c r="E514" s="3" t="inlineStr">
+        <is>
+          <t>info@studioduggan.com</t>
+        </is>
+      </c>
+      <c r="F514" s="3" t="inlineStr">
+        <is>
+          <t>020 3642 3120</t>
+        </is>
+      </c>
+      <c r="G514" s="3" t="inlineStr">
+        <is>
+          <t>Tiffany Duggan (Founder, est. 2011, ex-Elle Decoration/Livingetc stylist)</t>
+        </is>
+      </c>
+      <c r="H514" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/tiffany-duggan-b97bb148</t>
+        </is>
+      </c>
+      <c r="I514" s="3" t="inlineStr">
+        <is>
+          <t>instagram.com/studioduggan</t>
+        </is>
+      </c>
+      <c r="J514" s="3" t="inlineStr">
+        <is>
+          <t>14-year high-end residential/boutique-commercial interior design studio founded by a former Elle Decoration/Livingetc stylist; project fees run into tens of thousands per client</t>
+        </is>
+      </c>
+      <c r="K514" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L514" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M514" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N514" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O514" s="3" t="inlineStr">
+        <is>
+          <t>Instagram presence; press-editorial founder background = strong PR asset</t>
+        </is>
+      </c>
+      <c r="P514" s="3" t="inlineStr">
+        <is>
+          <t>Editorial-press founder pedigree not yet the AI-cited answer for 'interior designer Notting Hill'</t>
+        </is>
+      </c>
+      <c r="Q514" s="3" t="inlineStr">
+        <is>
+          <t>'Founded by a former Elle Decoration stylist - own that exact AEO credibility signal'</t>
+        </is>
+      </c>
+      <c r="R514" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S514" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T514" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T508"/>
+  <autoFilter ref="A1:T514"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -45084,7 +45624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B238"/>
+  <dimension ref="A1:B240"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -45104,7 +45644,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>507</v>
+        <v>513</v>
       </c>
     </row>
     <row r="5">
@@ -45121,7 +45661,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="7">
@@ -45247,7 +45787,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Osteopathy clinic</t>
+          <t>Interior design studio</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -45257,7 +45797,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Recruitment agency</t>
+          <t>Osteopathy clinic</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -45267,7 +45807,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>IT support / MSP</t>
+          <t>Recruitment agency</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -45277,27 +45817,27 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Interior design studio</t>
+          <t>IT support / MSP</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Law firm</t>
+          <t>Estate &amp; lettings agent</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Letting agent</t>
+          <t>Law firm</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -45307,7 +45847,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Private tuition agency</t>
+          <t>Letting agent</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -45317,7 +45857,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Electrician</t>
+          <t>Private tuition agency</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -45327,7 +45867,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Personal training studio</t>
+          <t>Electrician</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -45337,7 +45877,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Family law firm</t>
+          <t>Personal training studio</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -45347,7 +45887,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Chiropractor</t>
+          <t>Family law firm</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -45357,7 +45897,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Immigration law firm</t>
+          <t>Chiropractor</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -45367,7 +45907,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Independent optician</t>
+          <t>Immigration law firm</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -45377,7 +45917,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Pilates studio</t>
+          <t>Independent optician</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -45387,7 +45927,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Kitchen &amp; bathroom design</t>
+          <t>Pilates studio</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -45397,7 +45937,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Architecture practice</t>
+          <t>Kitchen &amp; bathroom design</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -45407,7 +45947,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Home care agency</t>
+          <t>Architecture practice</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -45417,17 +45957,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Financial adviser / wealth management</t>
+          <t>Home care agency</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Roofer</t>
+          <t>Financial adviser / wealth management</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -45437,7 +45977,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating / boilers</t>
+          <t>Roofer</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -45447,7 +45987,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Event &amp; wedding caterer</t>
+          <t>Plumbing &amp; heating / boilers</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -45457,7 +45997,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Estate agent (premium)</t>
+          <t>Event &amp; wedding caterer</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -45467,7 +46007,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Orthodontist</t>
+          <t>Estate agent (premium)</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -45477,7 +46017,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Employment law firm</t>
+          <t>Orthodontist</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -45487,7 +46027,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Event management agency</t>
+          <t>Employment law firm</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -45497,7 +46037,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Design &amp; build</t>
+          <t>Event management agency</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -45507,7 +46047,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>IFA / wealth management</t>
+          <t>Design &amp; build</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -45517,7 +46057,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Wealth management / IFA</t>
+          <t>IFA / wealth management</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -45527,7 +46067,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Architects &amp; interior design</t>
+          <t>Wealth management / IFA</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -45537,7 +46077,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Funeral directors</t>
+          <t>Architects &amp; interior design</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -45547,7 +46087,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Garden rooms / outbuildings</t>
+          <t>Funeral directors</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -45557,7 +46097,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Personal training gym</t>
+          <t>Garden rooms / outbuildings</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -45567,7 +46107,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Estate agent &amp; chartered surveyors</t>
+          <t>Personal training gym</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -45577,7 +46117,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Wedding &amp; event caterer</t>
+          <t>Estate agent &amp; chartered surveyors</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -45587,7 +46127,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Personal training</t>
+          <t>Wedding &amp; event caterer</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -45597,7 +46137,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Construction recruitment agency</t>
+          <t>Personal training</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -45607,7 +46147,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Legal recruitment agency</t>
+          <t>Construction recruitment agency</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -45617,7 +46157,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>HGV driver training</t>
+          <t>Legal recruitment agency</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -45627,7 +46167,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Private GP practice</t>
+          <t>HGV driver training</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -45637,7 +46177,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Aesthetics clinic (non-surgical)</t>
+          <t>Private GP practice</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -45647,7 +46187,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Estate &amp; lettings agent</t>
+          <t>Aesthetics clinic (non-surgical)</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -47441,6 +47981,26 @@
         </is>
       </c>
       <c r="B238" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>Dental practice (general, cosmetic, implants)</t>
+        </is>
+      </c>
+      <c r="B239" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>Pilates, osteopathy &amp; functional medicine clinic</t>
+        </is>
+      </c>
+      <c r="B240" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batches 63-64: +4 prospects (517 total) - Bristol vets, Bath mortgage broker, Richmond private GP, wedding barns
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$514</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$518</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T514"/>
+  <dimension ref="A1:T518"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -45612,8 +45612,360 @@
       </c>
       <c r="T514" s="3" t="inlineStr"/>
     </row>
+    <row r="515">
+      <c r="A515" s="3" t="inlineStr">
+        <is>
+          <t>The Grove Vets</t>
+        </is>
+      </c>
+      <c r="B515" s="3" t="inlineStr">
+        <is>
+          <t>Veterinary practice</t>
+        </is>
+      </c>
+      <c r="C515" s="3" t="inlineStr">
+        <is>
+          <t>Henleaze, Bristol</t>
+        </is>
+      </c>
+      <c r="D515" s="3" t="inlineStr">
+        <is>
+          <t>https://www.thegrovevet.com</t>
+        </is>
+      </c>
+      <c r="E515" s="3" t="inlineStr">
+        <is>
+          <t>info@thegrovevet.com</t>
+        </is>
+      </c>
+      <c r="F515" s="3" t="inlineStr">
+        <is>
+          <t>0117 252 0545</t>
+        </is>
+      </c>
+      <c r="G515" s="3" t="inlineStr">
+        <is>
+          <t>Andy Valenzia &amp; Amy Valenzia (Founders, vets since 2008)</t>
+        </is>
+      </c>
+      <c r="H515" s="3" t="inlineStr"/>
+      <c r="I515" s="3" t="inlineStr">
+        <is>
+          <t>instagram.com/grovevetbristol; facebook.com/grovevetbristol</t>
+        </is>
+      </c>
+      <c r="J515" s="3" t="inlineStr">
+        <is>
+          <t>Vet-owned family-run practice explicitly marketed as independent; consultation/treatment fees plus repeat annual health-plan clients</t>
+        </is>
+      </c>
+      <c r="K515" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L515" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M515" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N515" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O515" s="3" t="inlineStr">
+        <is>
+          <t>Instagram/Facebook presence</t>
+        </is>
+      </c>
+      <c r="P515" s="3" t="inlineStr">
+        <is>
+          <t>'Independent veterinary centre' positioning not yet the AI-cited trust signal for 'vet Bristol'</t>
+        </is>
+      </c>
+      <c r="Q515" s="3" t="inlineStr">
+        <is>
+          <t>'Vet-owned, family-run, proudly independent - own that exact AEO trust signal in Bristol'</t>
+        </is>
+      </c>
+      <c r="R515" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S515" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T515" s="3" t="inlineStr"/>
+    </row>
+    <row r="516">
+      <c r="A516" s="4" t="inlineStr">
+        <is>
+          <t>Mortgage Gold</t>
+        </is>
+      </c>
+      <c r="B516" s="4" t="inlineStr">
+        <is>
+          <t>Independent mortgage broker</t>
+        </is>
+      </c>
+      <c r="C516" s="4" t="inlineStr">
+        <is>
+          <t>Bath (+ Bristol)</t>
+        </is>
+      </c>
+      <c r="D516" s="4" t="inlineStr">
+        <is>
+          <t>https://www.mortgagegold.co.uk</t>
+        </is>
+      </c>
+      <c r="E516" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F516" s="4" t="inlineStr"/>
+      <c r="G516" s="4" t="inlineStr">
+        <is>
+          <t>Guy Maloney &amp; Clarissa Bellavia (Founders)</t>
+        </is>
+      </c>
+      <c r="H516" s="4" t="inlineStr"/>
+      <c r="I516" s="4" t="inlineStr"/>
+      <c r="J516" s="4" t="inlineStr">
+        <is>
+          <t>Fees-free, whole-of-market independent mortgage broker serving Bath and Bristol; commission per completed mortgage recurs with remortgage clients</t>
+        </is>
+      </c>
+      <c r="K516" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L516" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M516" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N516" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O516" s="4" t="inlineStr">
+        <is>
+          <t>'Fees-free' whole-of-market marketing positioning</t>
+        </is>
+      </c>
+      <c r="P516" s="4" t="inlineStr">
+        <is>
+          <t>'Fees-free' positioning not yet the AI-cited answer for 'mortgage broker Bath'</t>
+        </is>
+      </c>
+      <c r="Q516" s="4" t="inlineStr">
+        <is>
+          <t>'Fees-free, whole-of-market - own that exact AEO trust signal in Bath'</t>
+        </is>
+      </c>
+      <c r="R516" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S516" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T516" s="4" t="inlineStr"/>
+    </row>
+    <row r="517">
+      <c r="A517" s="3" t="inlineStr">
+        <is>
+          <t>Gate Street Barn</t>
+        </is>
+      </c>
+      <c r="B517" s="3" t="inlineStr">
+        <is>
+          <t>Wedding venue (barn on working farm)</t>
+        </is>
+      </c>
+      <c r="C517" s="3" t="inlineStr">
+        <is>
+          <t>Bramley, nr Guildford, Surrey</t>
+        </is>
+      </c>
+      <c r="D517" s="3" t="inlineStr">
+        <is>
+          <t>https://gatestreet.co.uk</t>
+        </is>
+      </c>
+      <c r="E517" s="3" t="inlineStr">
+        <is>
+          <t>info@gatestreetbarn.com</t>
+        </is>
+      </c>
+      <c r="F517" s="3" t="inlineStr"/>
+      <c r="G517" s="3" t="inlineStr">
+        <is>
+          <t>Third-generation family farm owners</t>
+        </is>
+      </c>
+      <c r="H517" s="3" t="inlineStr"/>
+      <c r="I517" s="3" t="inlineStr"/>
+      <c r="J517" s="3" t="inlineStr">
+        <is>
+          <t>180-acre third-generation family-run regenerative farm hosting countryside weddings; bookings run into thousands to tens of thousands per event</t>
+        </is>
+      </c>
+      <c r="K517" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L517" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M517" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N517" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O517" s="3" t="inlineStr">
+        <is>
+          <t>Regenerative-farming/biodiversity marketing angle = active PR positioning</t>
+        </is>
+      </c>
+      <c r="P517" s="3" t="inlineStr">
+        <is>
+          <t>Third-generation regenerative-farm story not yet the AI-cited answer for 'barn wedding venue Surrey'</t>
+        </is>
+      </c>
+      <c r="Q517" s="3" t="inlineStr">
+        <is>
+          <t>'A third-generation regenerative farm - own that exact AEO story in Surrey weddings'</t>
+        </is>
+      </c>
+      <c r="R517" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S517" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T517" s="3" t="inlineStr"/>
+    </row>
+    <row r="518">
+      <c r="A518" s="3" t="inlineStr">
+        <is>
+          <t>Jenners Barn</t>
+        </is>
+      </c>
+      <c r="B518" s="3" t="inlineStr">
+        <is>
+          <t>Wedding venue (Cotswold stone barn)</t>
+        </is>
+      </c>
+      <c r="C518" s="3" t="inlineStr">
+        <is>
+          <t>Whelford, nr Fairford, Cotswolds</t>
+        </is>
+      </c>
+      <c r="D518" s="3" t="inlineStr">
+        <is>
+          <t>https://jennersbarn.co.uk</t>
+        </is>
+      </c>
+      <c r="E518" s="3" t="inlineStr">
+        <is>
+          <t>hello@jennersbarn.co.uk</t>
+        </is>
+      </c>
+      <c r="F518" s="3" t="inlineStr">
+        <is>
+          <t>07886 037224</t>
+        </is>
+      </c>
+      <c r="G518" s="3" t="inlineStr">
+        <is>
+          <t>Family-owned and run</t>
+        </is>
+      </c>
+      <c r="H518" s="3" t="inlineStr"/>
+      <c r="I518" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/Jennersbarn</t>
+        </is>
+      </c>
+      <c r="J518" s="3" t="inlineStr">
+        <is>
+          <t>Family-owned Cotswold stone barn venue near Fairford/Lechlade/Cirencester with flexible planning freedom; bookings run into thousands to tens of thousands per event</t>
+        </is>
+      </c>
+      <c r="K518" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L518" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M518" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N518" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O518" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence</t>
+        </is>
+      </c>
+      <c r="P518" s="3" t="inlineStr">
+        <is>
+          <t>Flexible-planning positioning not yet the AI-cited answer for 'barn wedding venue Cotswolds'</t>
+        </is>
+      </c>
+      <c r="Q518" s="3" t="inlineStr">
+        <is>
+          <t>'Freedom to plan your own unique day - own that exact AEO positioning in the Cotswolds'</t>
+        </is>
+      </c>
+      <c r="R518" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S518" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T518" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T514"/>
+  <autoFilter ref="A1:T518"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -45624,7 +45976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B240"/>
+  <dimension ref="A1:B242"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -45644,7 +45996,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>513</v>
+        <v>517</v>
       </c>
     </row>
     <row r="5">
@@ -45957,7 +46309,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Home care agency</t>
+          <t>Veterinary practice</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -45967,17 +46319,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Financial adviser / wealth management</t>
+          <t>Home care agency</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Roofer</t>
+          <t>Financial adviser / wealth management</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -45987,7 +46339,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating / boilers</t>
+          <t>Roofer</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -45997,7 +46349,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Event &amp; wedding caterer</t>
+          <t>Plumbing &amp; heating / boilers</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -46007,7 +46359,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Estate agent (premium)</t>
+          <t>Event &amp; wedding caterer</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -46017,7 +46369,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Orthodontist</t>
+          <t>Estate agent (premium)</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -46027,7 +46379,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Employment law firm</t>
+          <t>Orthodontist</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -46037,7 +46389,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Event management agency</t>
+          <t>Employment law firm</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -46047,7 +46399,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Design &amp; build</t>
+          <t>Event management agency</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -46057,7 +46409,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>IFA / wealth management</t>
+          <t>Design &amp; build</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -46067,7 +46419,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Wealth management / IFA</t>
+          <t>IFA / wealth management</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -46077,7 +46429,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Architects &amp; interior design</t>
+          <t>Wealth management / IFA</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -46087,7 +46439,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Funeral directors</t>
+          <t>Architects &amp; interior design</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -46097,7 +46449,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Garden rooms / outbuildings</t>
+          <t>Funeral directors</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -46107,7 +46459,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Personal training gym</t>
+          <t>Garden rooms / outbuildings</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -46117,7 +46469,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Estate agent &amp; chartered surveyors</t>
+          <t>Personal training gym</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -46127,7 +46479,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Wedding &amp; event caterer</t>
+          <t>Estate agent &amp; chartered surveyors</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -46137,7 +46489,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Personal training</t>
+          <t>Wedding &amp; event caterer</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -46147,7 +46499,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Construction recruitment agency</t>
+          <t>Personal training</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -46157,7 +46509,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Legal recruitment agency</t>
+          <t>Construction recruitment agency</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -46167,7 +46519,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>HGV driver training</t>
+          <t>Legal recruitment agency</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -46177,7 +46529,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Private GP practice</t>
+          <t>HGV driver training</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -46187,7 +46539,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Aesthetics clinic (non-surgical)</t>
+          <t>Private GP practice</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -46197,7 +46549,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Driving school &amp; ADI instructor training</t>
+          <t>Aesthetics clinic (non-surgical)</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -46207,7 +46559,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Veterinary practice</t>
+          <t>Driving school &amp; ADI instructor training</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -46217,7 +46569,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Reformer Pilates studio</t>
+          <t>Independent mortgage broker</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -46227,7 +46579,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Home care &amp; live-in care agency</t>
+          <t>Reformer Pilates studio</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -46237,7 +46589,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Private tuition (primary/11+)</t>
+          <t>Home care &amp; live-in care agency</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -46247,7 +46599,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Independent Chartered financial planning</t>
+          <t>Private tuition (primary/11+)</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -46257,7 +46609,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Roofing contractor</t>
+          <t>Independent Chartered financial planning</t>
         </is>
       </c>
       <c r="B66" t="n">
@@ -46267,17 +46619,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Dentist / Orthodontics</t>
+          <t>Roofing contractor</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Specialist dental/implant clinic</t>
+          <t>Dentist / Orthodontics</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -46287,7 +46639,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Boutique corporate law firm</t>
+          <t>Specialist dental/implant clinic</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -46297,7 +46649,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Cosmetic/aesthetics clinic</t>
+          <t>Boutique corporate law firm</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -46307,7 +46659,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Skin &amp; laser clinic</t>
+          <t>Cosmetic/aesthetics clinic</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -46317,7 +46669,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Mortgage broker / financial adviser</t>
+          <t>Skin &amp; laser clinic</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -46327,7 +46679,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Architects (RIBA chartered)</t>
+          <t>Mortgage broker / financial adviser</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -46337,7 +46689,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Recruitment agency (tech/startups)</t>
+          <t>Architects (RIBA chartered)</t>
         </is>
       </c>
       <c r="B74" t="n">
@@ -46347,7 +46699,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Recruitment agency (IT/data)</t>
+          <t>Recruitment agency (tech/startups)</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -46357,7 +46709,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Independent vet (24/7 emergency)</t>
+          <t>Recruitment agency (IT/data)</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -46367,7 +46719,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Letting &amp; estate agent</t>
+          <t>Independent vet (24/7 emergency)</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -46377,7 +46729,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Cosmetic clinic (injectables)</t>
+          <t>Letting &amp; estate agent</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -46387,7 +46739,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Cosmetic/anti-ageing clinic</t>
+          <t>Cosmetic clinic (injectables)</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -46397,7 +46749,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Yoga &amp; reformer pilates studio</t>
+          <t>Cosmetic/anti-ageing clinic</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -46407,7 +46759,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Reformer pilates studio</t>
+          <t>Yoga &amp; reformer pilates studio</t>
         </is>
       </c>
       <c r="B81" t="n">
@@ -46417,7 +46769,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Wealth management</t>
+          <t>Reformer pilates studio</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -46427,7 +46779,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Private tuition &amp; education consultancy</t>
+          <t>Wealth management</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -46437,7 +46789,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Osteopath</t>
+          <t>Private tuition &amp; education consultancy</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -46447,7 +46799,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Design &amp; build / home renovation</t>
+          <t>Osteopath</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -46457,7 +46809,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Builders / building contractor</t>
+          <t>Design &amp; build / home renovation</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -46467,7 +46819,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Home care / live-in care</t>
+          <t>Builders / building contractor</t>
         </is>
       </c>
       <c r="B87" t="n">
@@ -46477,7 +46829,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Private day nurseries</t>
+          <t>Home care / live-in care</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -46487,7 +46839,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Personal training &amp; wellness studio</t>
+          <t>Private day nurseries</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -46497,7 +46849,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Mortgage &amp; insurance broker</t>
+          <t>Personal training &amp; wellness studio</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -46507,7 +46859,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Business consultancy</t>
+          <t>Mortgage &amp; insurance broker</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -46517,7 +46869,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Interior designer (period homes)</t>
+          <t>Business consultancy</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -46527,7 +46879,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Landscape design &amp; build</t>
+          <t>Interior designer (period homes)</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -46537,7 +46889,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Interior designer</t>
+          <t>Landscape design &amp; build</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -46547,7 +46899,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Garden design &amp; landscaping</t>
+          <t>Interior designer</t>
         </is>
       </c>
       <c r="B95" t="n">
@@ -46557,7 +46909,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Legal recruitment</t>
+          <t>Garden design &amp; landscaping</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -46567,7 +46919,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Independent gym &amp; health club</t>
+          <t>Legal recruitment</t>
         </is>
       </c>
       <c r="B97" t="n">
@@ -46577,7 +46929,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Independent gym</t>
+          <t>Independent gym &amp; health club</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -46587,7 +46939,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Physiotherapy (sports)</t>
+          <t>Independent gym</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -46597,7 +46949,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Letting agent / property management</t>
+          <t>Physiotherapy (sports)</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -46607,7 +46959,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Skin clinic</t>
+          <t>Letting agent / property management</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -46617,7 +46969,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Tutoring company</t>
+          <t>Skin clinic</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -46627,7 +46979,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Tutorial college &amp; exam centre</t>
+          <t>Tutoring company</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -46637,7 +46989,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Employment law (disability discrimination)</t>
+          <t>Tutorial college &amp; exam centre</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -46647,7 +46999,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Plumbing &amp; heating</t>
+          <t>Employment law (disability discrimination)</t>
         </is>
       </c>
       <c r="B105" t="n">
@@ -46657,7 +47009,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Plumbing &amp; heating</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -46667,7 +47019,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Sports physio &amp; massage</t>
+          <t>Plumbing</t>
         </is>
       </c>
       <c r="B107" t="n">
@@ -46677,7 +47029,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Chartered surveyors (party wall/building)</t>
+          <t>Sports physio &amp; massage</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -46687,7 +47039,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Chartered surveyors</t>
+          <t>Chartered surveyors (party wall/building)</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -46697,7 +47049,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Chartered building surveyors</t>
+          <t>Chartered surveyors</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -46707,7 +47059,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Osteopathy clinics</t>
+          <t>Chartered building surveyors</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -46717,7 +47069,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Builders / renovations</t>
+          <t>Osteopathy clinics</t>
         </is>
       </c>
       <c r="B112" t="n">
@@ -46727,7 +47079,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Private nursery schools</t>
+          <t>Builders / renovations</t>
         </is>
       </c>
       <c r="B113" t="n">
@@ -46737,7 +47089,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Private day nursery</t>
+          <t>Private nursery schools</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -46747,7 +47099,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Private GP (membership model)</t>
+          <t>Private day nursery</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -46757,7 +47109,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Sash window restoration</t>
+          <t>Private GP (membership model)</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -46767,7 +47119,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Personal training (1:1)</t>
+          <t>Sash window restoration</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -46777,7 +47129,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Personal training &amp; nutrition coaching</t>
+          <t>Personal training (1:1)</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -46787,7 +47139,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Private nursery/pre-prep school</t>
+          <t>Personal training &amp; nutrition coaching</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -46797,7 +47149,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Independent nursery (Montessori)</t>
+          <t>Private nursery/pre-prep school</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -46807,7 +47159,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Live-in care agency</t>
+          <t>Independent nursery (Montessori)</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -46817,7 +47169,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Law firm (conveyancing/family)</t>
+          <t>Live-in care agency</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -46827,7 +47179,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Architect &amp; interior designer</t>
+          <t>Law firm (conveyancing/family)</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -46837,7 +47189,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Architects / project management</t>
+          <t>Architect &amp; interior designer</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -46847,7 +47199,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Physiotherapy &amp; clinical Pilates</t>
+          <t>Architects / project management</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -46857,7 +47209,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Aesthetics &amp; skin clinic</t>
+          <t>Physiotherapy &amp; clinical Pilates</t>
         </is>
       </c>
       <c r="B126" t="n">
@@ -46867,7 +47219,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>IFA / financial planning</t>
+          <t>Aesthetics &amp; skin clinic</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -46877,7 +47229,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Wealth management &amp; employee benefits</t>
+          <t>IFA / financial planning</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -46887,7 +47239,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Dermatology clinic</t>
+          <t>Wealth management &amp; employee benefits</t>
         </is>
       </c>
       <c r="B129" t="n">
@@ -46897,7 +47249,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Pilates studio (multi-site)</t>
+          <t>Dermatology clinic</t>
         </is>
       </c>
       <c r="B130" t="n">
@@ -46907,7 +47259,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Private nursery (Montessori, multi-site)</t>
+          <t>Pilates studio (multi-site)</t>
         </is>
       </c>
       <c r="B131" t="n">
@@ -46917,7 +47269,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Law firm (wills &amp; probate)</t>
+          <t>Private nursery (Montessori, multi-site)</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -46927,7 +47279,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Business/technical consultancy</t>
+          <t>Law firm (wills &amp; probate)</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -46937,7 +47289,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Private/NHS dentist</t>
+          <t>Business/technical consultancy</t>
         </is>
       </c>
       <c r="B134" t="n">
@@ -46947,7 +47299,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Removals company</t>
+          <t>Private/NHS dentist</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -46957,7 +47309,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Driveways &amp; landscaping</t>
+          <t>Removals company</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -46967,7 +47319,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Wedding &amp; event venue</t>
+          <t>Driveways &amp; landscaping</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -46977,7 +47329,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>IFA &amp; mortgage broker</t>
+          <t>Wedding &amp; event venue</t>
         </is>
       </c>
       <c r="B138" t="n">
@@ -46987,7 +47339,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Wedding photography &amp; videography</t>
+          <t>IFA &amp; mortgage broker</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -46997,7 +47349,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Commercial property litigation law firm</t>
+          <t>Wedding photography &amp; videography</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -47007,7 +47359,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Recruitment agency (boutique)</t>
+          <t>Commercial property litigation law firm</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -47017,7 +47369,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Home cinema &amp; smart home installer</t>
+          <t>Recruitment agency (boutique)</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -47027,7 +47379,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Home cinema installer</t>
+          <t>Home cinema &amp; smart home installer</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -47037,7 +47389,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Curtains, blinds &amp; upholstery</t>
+          <t>Home cinema installer</t>
         </is>
       </c>
       <c r="B144" t="n">
@@ -47047,7 +47399,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Bespoke curtains &amp; soft furnishings</t>
+          <t>Curtains, blinds &amp; upholstery</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -47057,7 +47409,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Wine merchant</t>
+          <t>Bespoke curtains &amp; soft furnishings</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -47067,7 +47419,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Education consultancy (school placement)</t>
+          <t>Wine merchant</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -47077,7 +47429,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Estate agent &amp; surveyors</t>
+          <t>Education consultancy (school placement)</t>
         </is>
       </c>
       <c r="B148" t="n">
@@ -47087,7 +47439,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Independent financial adviser</t>
+          <t>Estate agent &amp; surveyors</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -47097,7 +47449,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Chartered accountants &amp; financial planners</t>
+          <t>Independent financial adviser</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -47107,7 +47459,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Private GP &amp; dermatology</t>
+          <t>Chartered accountants &amp; financial planners</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -47117,7 +47469,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Architects (heritage specialism)</t>
+          <t>Private GP &amp; dermatology</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -47127,7 +47479,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Private cosmetic dentist / implants</t>
+          <t>Architects (heritage specialism)</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -47137,7 +47489,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Heating engineer / plumbing</t>
+          <t>Private cosmetic dentist / implants</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -47147,7 +47499,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Estate agent (boutique)</t>
+          <t>Heating engineer / plumbing</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -47157,7 +47509,7 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Independent vet (mixed practice)</t>
+          <t>Estate agent (boutique)</t>
         </is>
       </c>
       <c r="B156" t="n">
@@ -47167,7 +47519,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Private dentist / cosmetic</t>
+          <t>Independent vet (mixed practice)</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -47177,7 +47529,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Chartered accountants &amp; financial advisers</t>
+          <t>Private dentist / cosmetic</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -47187,7 +47539,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Healthcare recruitment agency</t>
+          <t>Chartered accountants &amp; financial advisers</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -47197,7 +47549,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Executive search / headhunting</t>
+          <t>Healthcare recruitment agency</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -47207,7 +47559,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>First aid &amp; health &amp; safety training</t>
+          <t>Executive search / headhunting</t>
         </is>
       </c>
       <c r="B161" t="n">
@@ -47217,7 +47569,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Teaching &amp; education recruitment agency</t>
+          <t>First aid &amp; health &amp; safety training</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -47227,7 +47579,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Supply teaching agency</t>
+          <t>Teaching &amp; education recruitment agency</t>
         </is>
       </c>
       <c r="B163" t="n">
@@ -47237,7 +47589,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Hospitality staffing agency</t>
+          <t>Supply teaching agency</t>
         </is>
       </c>
       <c r="B164" t="n">
@@ -47247,7 +47599,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Finance &amp; accountancy recruitment agency</t>
+          <t>Hospitality staffing agency</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -47257,7 +47609,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Accounting &amp; finance recruitment agency</t>
+          <t>Finance &amp; accountancy recruitment agency</t>
         </is>
       </c>
       <c r="B166" t="n">
@@ -47267,7 +47619,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Forklift &amp; plant operator training</t>
+          <t>Accounting &amp; finance recruitment agency</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -47277,7 +47629,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Forklift training</t>
+          <t>Forklift &amp; plant operator training</t>
         </is>
       </c>
       <c r="B168" t="n">
@@ -47287,7 +47639,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Language school</t>
+          <t>Forklift training</t>
         </is>
       </c>
       <c r="B169" t="n">
@@ -47297,7 +47649,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Engineering &amp; manufacturing recruitment</t>
+          <t>Language school</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -47307,7 +47659,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Business &amp; sales coaching</t>
+          <t>Engineering &amp; manufacturing recruitment</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -47317,7 +47669,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Engineering &amp; energy recruitment</t>
+          <t>Business &amp; sales coaching</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -47327,7 +47679,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Tech recruitment agency</t>
+          <t>Engineering &amp; energy recruitment</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -47337,7 +47689,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Data/tech/AI recruitment agency</t>
+          <t>Tech recruitment agency</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -47347,7 +47699,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>Beauty/aesthetics training academy</t>
+          <t>Data/tech/AI recruitment agency</t>
         </is>
       </c>
       <c r="B175" t="n">
@@ -47357,7 +47709,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Beauty/hair training academy</t>
+          <t>Beauty/aesthetics training academy</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -47367,7 +47719,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Medical aesthetics/injectable training academy</t>
+          <t>Beauty/hair training academy</t>
         </is>
       </c>
       <c r="B177" t="n">
@@ -47377,7 +47729,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Yoga teacher training school</t>
+          <t>Medical aesthetics/injectable training academy</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -47387,7 +47739,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>Creative &amp; marketing recruitment agency</t>
+          <t>Yoga teacher training school</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -47397,7 +47749,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>Private dermatology &amp; women's health clinics</t>
+          <t>Creative &amp; marketing recruitment agency</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -47407,7 +47759,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>Private dermatology practice</t>
+          <t>Private dermatology &amp; women's health clinics</t>
         </is>
       </c>
       <c r="B181" t="n">
@@ -47417,7 +47769,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>Wedding venue (converted barn)</t>
+          <t>Private dermatology practice</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -47427,7 +47779,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>Wedding venue (waterside barn &amp; estate)</t>
+          <t>Wedding venue (converted barn)</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -47437,7 +47789,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>Wedding venue (thatched barn on working farm)</t>
+          <t>Wedding venue (waterside barn &amp; estate)</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -47447,7 +47799,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>Wedding venue (working farm)</t>
+          <t>Wedding venue (thatched barn on working farm)</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -47457,7 +47809,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Wedding venue (restored historic barn)</t>
+          <t>Wedding venue (working farm)</t>
         </is>
       </c>
       <c r="B186" t="n">
@@ -47467,7 +47819,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Chartered IFA / wealth management</t>
+          <t>Wedding venue (restored historic barn)</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -47477,7 +47829,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Independent mortgage broker</t>
+          <t>Chartered IFA / wealth management</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -48001,6 +48353,26 @@
         </is>
       </c>
       <c r="B240" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>Wedding venue (barn on working farm)</t>
+        </is>
+      </c>
+      <c r="B241" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>Wedding venue (Cotswold stone barn)</t>
+        </is>
+      </c>
+      <c r="B242" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 65: +4 prospects (521 total) - Cotswolds/Cheltenham care homes, Guildford business consultancy
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$518</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$522</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T518"/>
+  <dimension ref="A1:T522"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -45964,8 +45964,368 @@
       </c>
       <c r="T518" s="3" t="inlineStr"/>
     </row>
+    <row r="519">
+      <c r="A519" s="3" t="inlineStr">
+        <is>
+          <t>Cedar Trust Care Homes</t>
+        </is>
+      </c>
+      <c r="B519" s="3" t="inlineStr">
+        <is>
+          <t>Care home group (residential, nursing, dementia)</t>
+        </is>
+      </c>
+      <c r="C519" s="3" t="inlineStr">
+        <is>
+          <t>Cheltenham, Tewkesbury &amp; Gloucester (5 homes)</t>
+        </is>
+      </c>
+      <c r="D519" s="3" t="inlineStr">
+        <is>
+          <t>https://www.cedartrust.co.uk</t>
+        </is>
+      </c>
+      <c r="E519" s="3" t="inlineStr">
+        <is>
+          <t>info@cedartrust.co.uk</t>
+        </is>
+      </c>
+      <c r="F519" s="3" t="inlineStr">
+        <is>
+          <t>01242 525 087</t>
+        </is>
+      </c>
+      <c r="G519" s="3" t="inlineStr">
+        <is>
+          <t>Antony D. Cronk (Managing Director, opened first home 1986)</t>
+        </is>
+      </c>
+      <c r="H519" s="3" t="inlineStr"/>
+      <c r="I519" s="3" t="inlineStr"/>
+      <c r="J519" s="3" t="inlineStr">
+        <is>
+          <t>39-year family-owned care home group with 5 homes across Gloucestershire; care fees run into thousands per month per resident, recurring</t>
+        </is>
+      </c>
+      <c r="K519" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L519" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M519" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N519" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O519" s="3" t="inlineStr">
+        <is>
+          <t>39-year trading history; 5-site regional footprint</t>
+        </is>
+      </c>
+      <c r="P519" s="3" t="inlineStr">
+        <is>
+          <t>5-site footprint not matched by per-town AI-search dominance</t>
+        </is>
+      </c>
+      <c r="Q519" s="3" t="inlineStr">
+        <is>
+          <t>Per-site AEO content to own Cheltenham/Tewkesbury/Gloucester 'care home near me' searches separately</t>
+        </is>
+      </c>
+      <c r="R519" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S519" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T519" s="3" t="inlineStr"/>
+    </row>
+    <row r="520">
+      <c r="A520" s="4" t="inlineStr">
+        <is>
+          <t>Northleach Court Care Home</t>
+        </is>
+      </c>
+      <c r="B520" s="4" t="inlineStr">
+        <is>
+          <t>Care home (nursing, dementia, residential)</t>
+        </is>
+      </c>
+      <c r="C520" s="4" t="inlineStr">
+        <is>
+          <t>Northleach, nr Cheltenham &amp; Cirencester</t>
+        </is>
+      </c>
+      <c r="D520" s="4" t="inlineStr">
+        <is>
+          <t>https://www.northleachcourtcarehome.com</t>
+        </is>
+      </c>
+      <c r="E520" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F520" s="4" t="inlineStr">
+        <is>
+          <t>01451 861447</t>
+        </is>
+      </c>
+      <c r="G520" s="4" t="inlineStr">
+        <is>
+          <t>Family-run, independently owned</t>
+        </is>
+      </c>
+      <c r="H520" s="4" t="inlineStr"/>
+      <c r="I520" s="4" t="inlineStr"/>
+      <c r="J520" s="4" t="inlineStr">
+        <is>
+          <t>Family-run independent Cotswolds care home with CQC Good rating, 'home from home' positioning; care fees run into thousands per month per resident, recurring</t>
+        </is>
+      </c>
+      <c r="K520" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L520" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M520" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N520" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O520" s="4" t="inlineStr">
+        <is>
+          <t>CQC Good rating</t>
+        </is>
+      </c>
+      <c r="P520" s="4" t="inlineStr">
+        <is>
+          <t>'Home from home' family positioning not yet the AI-cited answer for 'care home Cotswolds'</t>
+        </is>
+      </c>
+      <c r="Q520" s="4" t="inlineStr">
+        <is>
+          <t>'A true home from home, family-run - own that exact AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R520" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S520" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T520" s="4" t="inlineStr"/>
+    </row>
+    <row r="521">
+      <c r="A521" s="3" t="inlineStr">
+        <is>
+          <t>Newlands Care (Newlands of Stow)</t>
+        </is>
+      </c>
+      <c r="B521" s="3" t="inlineStr">
+        <is>
+          <t>Care home (exclusive residential care)</t>
+        </is>
+      </c>
+      <c r="C521" s="3" t="inlineStr">
+        <is>
+          <t>Stow-on-the-Wold, Cotswolds</t>
+        </is>
+      </c>
+      <c r="D521" s="3" t="inlineStr">
+        <is>
+          <t>https://newlands.care</t>
+        </is>
+      </c>
+      <c r="E521" s="3" t="inlineStr">
+        <is>
+          <t>enquiries@newlandsofstow.co.uk</t>
+        </is>
+      </c>
+      <c r="F521" s="3" t="inlineStr">
+        <is>
+          <t>01451 885277</t>
+        </is>
+      </c>
+      <c r="G521" s="3" t="inlineStr">
+        <is>
+          <t>Amar Sheikh (Founder, family ties spanning 30+ years)</t>
+        </is>
+      </c>
+      <c r="H521" s="3" t="inlineStr"/>
+      <c r="I521" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/NewlandsofStow</t>
+        </is>
+      </c>
+      <c r="J521" s="3" t="inlineStr">
+        <is>
+          <t>Exclusive Cotswolds care residence built on 30+ years of family history in care; care fees run into thousands per month per resident, recurring</t>
+        </is>
+      </c>
+      <c r="K521" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L521" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M521" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N521" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O521" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence; 30+ year family heritage; 'exclusive' premium positioning</t>
+        </is>
+      </c>
+      <c r="P521" s="3" t="inlineStr">
+        <is>
+          <t>Premium/exclusive positioning and family heritage not yet the AI-cited answer for 'care home Cotswolds'</t>
+        </is>
+      </c>
+      <c r="Q521" s="3" t="inlineStr">
+        <is>
+          <t>'30+ years of family care history, now an exclusive Cotswold residence - own that AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R521" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S521" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T521" s="3" t="inlineStr"/>
+    </row>
+    <row r="522">
+      <c r="A522" s="4" t="inlineStr">
+        <is>
+          <t>Jolley Consultancy</t>
+        </is>
+      </c>
+      <c r="B522" s="4" t="inlineStr">
+        <is>
+          <t>Business consultancy (small business support)</t>
+        </is>
+      </c>
+      <c r="C522" s="4" t="inlineStr">
+        <is>
+          <t>Guildford, Surrey</t>
+        </is>
+      </c>
+      <c r="D522" s="4" t="inlineStr">
+        <is>
+          <t>https://jolleyconsultancy.com</t>
+        </is>
+      </c>
+      <c r="E522" s="4" t="inlineStr">
+        <is>
+          <t>jolley.consultancy@gmail.com</t>
+        </is>
+      </c>
+      <c r="F522" s="4" t="inlineStr">
+        <is>
+          <t>07718 587 526</t>
+        </is>
+      </c>
+      <c r="G522" s="4" t="inlineStr">
+        <is>
+          <t>Anna Jolley (Founder)</t>
+        </is>
+      </c>
+      <c r="H522" s="4" t="inlineStr"/>
+      <c r="I522" s="4" t="inlineStr">
+        <is>
+          <t>instagram.com/jolleyconsultancy; facebook.com/Jolley.Consultancy</t>
+        </is>
+      </c>
+      <c r="J522" s="4" t="inlineStr">
+        <is>
+          <t>Affordable one-to-one business consultancy for small, local Guildford businesses; monthly retained consultancy fees recur across a client's growth</t>
+        </is>
+      </c>
+      <c r="K522" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L522" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M522" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N522" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O522" s="4" t="inlineStr">
+        <is>
+          <t>Instagram/Facebook presence</t>
+        </is>
+      </c>
+      <c r="P522" s="4" t="inlineStr">
+        <is>
+          <t>Generic 'business consultant Guildford' searches not yet AI-answer dominated by this consultancy</t>
+        </is>
+      </c>
+      <c r="Q522" s="4" t="inlineStr">
+        <is>
+          <t>'Own the AI-cited answer for small-business support in Guildford'</t>
+        </is>
+      </c>
+      <c r="R522" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S522" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T522" s="4" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T518"/>
+  <autoFilter ref="A1:T522"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -45976,7 +46336,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B242"/>
+  <dimension ref="A1:B246"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -45996,7 +46356,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>517</v>
+        <v>521</v>
       </c>
     </row>
     <row r="5">
@@ -48373,6 +48733,46 @@
         </is>
       </c>
       <c r="B242" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>Care home group (residential, nursing, dementia)</t>
+        </is>
+      </c>
+      <c r="B243" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>Care home (nursing, dementia, residential)</t>
+        </is>
+      </c>
+      <c r="B244" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>Care home (exclusive residential care)</t>
+        </is>
+      </c>
+      <c r="B245" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>Business consultancy (small business support)</t>
+        </is>
+      </c>
+      <c r="B246" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batch 66: +2 prospects (523 total) - Cheltenham/Oxfordshire chartered accountants
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$522</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$524</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T522"/>
+  <dimension ref="A1:T524"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -46324,8 +46324,184 @@
       </c>
       <c r="T522" s="4" t="inlineStr"/>
     </row>
+    <row r="523">
+      <c r="A523" s="3" t="inlineStr">
+        <is>
+          <t>Randall &amp; Payne</t>
+        </is>
+      </c>
+      <c r="B523" s="3" t="inlineStr">
+        <is>
+          <t>Chartered accountants &amp; tax advisers</t>
+        </is>
+      </c>
+      <c r="C523" s="3" t="inlineStr">
+        <is>
+          <t>Shurdington, Cheltenham</t>
+        </is>
+      </c>
+      <c r="D523" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randall-payne.co.uk</t>
+        </is>
+      </c>
+      <c r="E523" s="3" t="inlineStr">
+        <is>
+          <t>info@randall-payne.co.uk</t>
+        </is>
+      </c>
+      <c r="F523" s="3" t="inlineStr">
+        <is>
+          <t>01242 776000</t>
+        </is>
+      </c>
+      <c r="G523" s="3" t="inlineStr">
+        <is>
+          <t>Independently owned LLP</t>
+        </is>
+      </c>
+      <c r="H523" s="3" t="inlineStr"/>
+      <c r="I523" s="3" t="inlineStr"/>
+      <c r="J523" s="3" t="inlineStr">
+        <is>
+          <t>Independently owned chartered accountancy and tax advisory firm working with clients across Gloucestershire and internationally; ongoing accountancy/advisory retainers recur across a client's business lifetime</t>
+        </is>
+      </c>
+      <c r="K523" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L523" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M523" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N523" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O523" s="3" t="inlineStr">
+        <is>
+          <t>ICAEW listing; established multi-decade regional reputation</t>
+        </is>
+      </c>
+      <c r="P523" s="3" t="inlineStr">
+        <is>
+          <t>Established reputation not yet the AI-cited answer for 'accountant Cheltenham'</t>
+        </is>
+      </c>
+      <c r="Q523" s="3" t="inlineStr">
+        <is>
+          <t>'Independently owned chartered accountants serving Gloucestershire - own that exact AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R523" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S523" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T523" s="3" t="inlineStr"/>
+    </row>
+    <row r="524">
+      <c r="A524" s="4" t="inlineStr">
+        <is>
+          <t>Andy Walton &amp; Co</t>
+        </is>
+      </c>
+      <c r="B524" s="4" t="inlineStr">
+        <is>
+          <t>Chartered accountants (small business)</t>
+        </is>
+      </c>
+      <c r="C524" s="4" t="inlineStr">
+        <is>
+          <t>Dorchester-on-Thames, nr Wallingford, Oxfordshire</t>
+        </is>
+      </c>
+      <c r="D524" s="4" t="inlineStr">
+        <is>
+          <t>https://www.oxford-accountant.co.uk</t>
+        </is>
+      </c>
+      <c r="E524" s="4" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F524" s="4" t="inlineStr"/>
+      <c r="G524" s="4" t="inlineStr">
+        <is>
+          <t>Andy Walton (Founder, est. 2005)</t>
+        </is>
+      </c>
+      <c r="H524" s="4" t="inlineStr"/>
+      <c r="I524" s="4" t="inlineStr"/>
+      <c r="J524" s="4" t="inlineStr">
+        <is>
+          <t>20-year small-business chartered accountancy practice founded as an alternative to expensive high-street accountants; ongoing accountancy/tax retainers recur across a client's business lifetime</t>
+        </is>
+      </c>
+      <c r="K524" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L524" s="4" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="M524" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N524" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O524" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P524" s="4" t="inlineStr">
+        <is>
+          <t>20-year affordable-alternative positioning not yet the AI-cited answer for 'small business accountant Oxfordshire'</t>
+        </is>
+      </c>
+      <c r="Q524" s="4" t="inlineStr">
+        <is>
+          <t>'The affordable alternative to expensive high-street accountants for 20 years - own that AEO positioning'</t>
+        </is>
+      </c>
+      <c r="R524" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S524" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T524" s="4" t="inlineStr">
+        <is>
+          <t>Phone number removed from site due to nuisance calls - use contact form</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T522"/>
+  <autoFilter ref="A1:T524"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -46336,7 +46512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B246"/>
+  <dimension ref="A1:B248"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -46356,7 +46532,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>521</v>
+        <v>523</v>
       </c>
     </row>
     <row r="5">
@@ -48773,6 +48949,26 @@
         </is>
       </c>
       <c r="B246" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>Chartered accountants &amp; tax advisers</t>
+        </is>
+      </c>
+      <c r="B247" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>Chartered accountants (small business)</t>
+        </is>
+      </c>
+      <c r="B248" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batches 67-68: +8 prospects (531 total) - landscape designers, solar installer, Wimbledon/Dulwich tutors and nurseries
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$524</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$532</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T524"/>
+  <dimension ref="A1:T532"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -46500,8 +46500,732 @@
         </is>
       </c>
     </row>
+    <row r="525">
+      <c r="A525" s="3" t="inlineStr">
+        <is>
+          <t>Fern &amp; Pine Garden Design Studio</t>
+        </is>
+      </c>
+      <c r="B525" s="3" t="inlineStr">
+        <is>
+          <t>Garden &amp; landscape design studio</t>
+        </is>
+      </c>
+      <c r="C525" s="3" t="inlineStr">
+        <is>
+          <t>Brighton/Sussex (+ Surrey, Kent, Cotswolds)</t>
+        </is>
+      </c>
+      <c r="D525" s="3" t="inlineStr">
+        <is>
+          <t>https://www.fernandpine.com</t>
+        </is>
+      </c>
+      <c r="E525" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F525" s="3" t="inlineStr">
+        <is>
+          <t>01273 906 912</t>
+        </is>
+      </c>
+      <c r="G525" s="3" t="inlineStr">
+        <is>
+          <t>Alick Nee (Founder, Society of Garden Designers Pre-Registered Member)</t>
+        </is>
+      </c>
+      <c r="H525" s="3" t="inlineStr"/>
+      <c r="I525" s="3" t="inlineStr"/>
+      <c r="J525" s="3" t="inlineStr">
+        <is>
+          <t>Boutique garden design/landscape architecture studio working on £25k-£250k+ project budgets across Sussex/Surrey/Kent/Cotswolds; project fees run into tens of thousands to hundreds of thousands</t>
+        </is>
+      </c>
+      <c r="K525" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L525" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M525" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N525" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O525" s="3" t="inlineStr">
+        <is>
+          <t>Houzz presence; wide multi-county coverage</t>
+        </is>
+      </c>
+      <c r="P525" s="3" t="inlineStr">
+        <is>
+          <t>Wide geographic coverage not matched by per-region AI-search dominance</t>
+        </is>
+      </c>
+      <c r="Q525" s="3" t="inlineStr">
+        <is>
+          <t>Per-region AEO content to own Sussex/Surrey/Kent/Cotswolds 'garden designer' searches separately</t>
+        </is>
+      </c>
+      <c r="R525" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S525" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T525" s="3" t="inlineStr">
+        <is>
+          <t>High project budgets (£25k-£250k+) - strong AEO opportunity</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" s="4" t="inlineStr">
+        <is>
+          <t>The Landscape Design Studio</t>
+        </is>
+      </c>
+      <c r="B526" s="4" t="inlineStr">
+        <is>
+          <t>Landscape &amp; garden design studio</t>
+        </is>
+      </c>
+      <c r="C526" s="4" t="inlineStr">
+        <is>
+          <t>Bromley, Kent (serving South London/Surrey)</t>
+        </is>
+      </c>
+      <c r="D526" s="4" t="inlineStr">
+        <is>
+          <t>https://thelandscapedesignstudio.co.uk</t>
+        </is>
+      </c>
+      <c r="E526" s="4" t="inlineStr">
+        <is>
+          <t>info@thelandscapedesignstudio.com</t>
+        </is>
+      </c>
+      <c r="F526" s="4" t="inlineStr">
+        <is>
+          <t>0203 538 8655</t>
+        </is>
+      </c>
+      <c r="G526" s="4" t="inlineStr">
+        <is>
+          <t>Chris Benson (Founder)</t>
+        </is>
+      </c>
+      <c r="H526" s="4" t="inlineStr"/>
+      <c r="I526" s="4" t="inlineStr"/>
+      <c r="J526" s="4" t="inlineStr">
+        <is>
+          <t>Independent landscape design studio serving Kent/South London/Surrey; project fees run into tens of thousands per client</t>
+        </is>
+      </c>
+      <c r="K526" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L526" s="4" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M526" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N526" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O526" s="4" t="inlineStr">
+        <is>
+          <t>Houzz presence</t>
+        </is>
+      </c>
+      <c r="P526" s="4" t="inlineStr">
+        <is>
+          <t>Generic 'garden designer Kent' searches not yet AI-answer dominated by this studio</t>
+        </is>
+      </c>
+      <c r="Q526" s="4" t="inlineStr">
+        <is>
+          <t>Own a specific Kent/South London AEO niche vs bigger regional landscape firms</t>
+        </is>
+      </c>
+      <c r="R526" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S526" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T526" s="4" t="inlineStr"/>
+    </row>
+    <row r="527">
+      <c r="A527" s="3" t="inlineStr">
+        <is>
+          <t>Wimbledon Tutors</t>
+        </is>
+      </c>
+      <c r="B527" s="3" t="inlineStr">
+        <is>
+          <t>Private tuition (A-Level/IB/GCSE/KS3)</t>
+        </is>
+      </c>
+      <c r="C527" s="3" t="inlineStr">
+        <is>
+          <t>Wimbledon, SW London</t>
+        </is>
+      </c>
+      <c r="D527" s="3" t="inlineStr">
+        <is>
+          <t>https://www.wimbledon-tutors.co.uk</t>
+        </is>
+      </c>
+      <c r="E527" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F527" s="3" t="inlineStr"/>
+      <c r="G527" s="3" t="inlineStr">
+        <is>
+          <t>Sara, Tom, Win &amp; Jacki Davis (Partner-led team, ex-independent-school teachers/examiners)</t>
+        </is>
+      </c>
+      <c r="H527" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/jacki-davis-9518738a</t>
+        </is>
+      </c>
+      <c r="I527" s="3" t="inlineStr"/>
+      <c r="J527" s="3" t="inlineStr">
+        <is>
+          <t>Small partner-led tutoring practice staffed entirely by former top independent-school teachers and examiners; per-session tuition fees recur weekly across a family's school years</t>
+        </is>
+      </c>
+      <c r="K527" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L527" s="3" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="M527" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N527" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O527" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn presence</t>
+        </is>
+      </c>
+      <c r="P527" s="3" t="inlineStr">
+        <is>
+          <t>Elite ex-teacher credentials not yet the AI-cited answer for 'tutor Wimbledon'</t>
+        </is>
+      </c>
+      <c r="Q527" s="3" t="inlineStr">
+        <is>
+          <t>'Every tutor is a former top independent-school teacher or examiner - own that exact AEO credibility signal'</t>
+        </is>
+      </c>
+      <c r="R527" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S527" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T527" s="3" t="inlineStr"/>
+    </row>
+    <row r="528">
+      <c r="A528" s="2" t="inlineStr">
+        <is>
+          <t>Apstar Tutoring</t>
+        </is>
+      </c>
+      <c r="B528" s="2" t="inlineStr">
+        <is>
+          <t>Private tuition (maths, 7+ to Oxbridge entry)</t>
+        </is>
+      </c>
+      <c r="C528" s="2" t="inlineStr">
+        <is>
+          <t>Dulwich, South London</t>
+        </is>
+      </c>
+      <c r="D528" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apstartutoring.com</t>
+        </is>
+      </c>
+      <c r="E528" s="2" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F528" s="2" t="inlineStr"/>
+      <c r="G528" s="2" t="inlineStr">
+        <is>
+          <t>Aidin &amp; Jonathan (Co-founders, current Dulwich College maths teachers &amp; exam board examiners, est. 2023)</t>
+        </is>
+      </c>
+      <c r="H528" s="2" t="inlineStr"/>
+      <c r="I528" s="2" t="inlineStr"/>
+      <c r="J528" s="2" t="inlineStr">
+        <is>
+          <t>New tutoring practice founded by two working Dulwich College teachers/AQA-Pearson examiners, already claiming 2,000+ students; per-session tuition fees recur weekly, especially around exam season</t>
+        </is>
+      </c>
+      <c r="K528" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L528" s="2" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M528" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N528" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O528" s="2" t="inlineStr">
+        <is>
+          <t>Founders are working exam-board examiners = exceptional credibility asset</t>
+        </is>
+      </c>
+      <c r="P528" s="2" t="inlineStr">
+        <is>
+          <t>New but rapidly-growing (2,000+ students) practice not yet the AI-cited answer for 'maths tutor Dulwich'</t>
+        </is>
+      </c>
+      <c r="Q528" s="2" t="inlineStr">
+        <is>
+          <t>'Taught by working Dulwich College teachers and exam board examiners - own that exact AEO credibility signal'</t>
+        </is>
+      </c>
+      <c r="R528" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S528" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T528" s="2" t="inlineStr">
+        <is>
+          <t>Founders are practising exam-board examiners - exceptional AEO credibility hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" s="4" t="inlineStr">
+        <is>
+          <t>Dulwich Tutor</t>
+        </is>
+      </c>
+      <c r="B529" s="4" t="inlineStr">
+        <is>
+          <t>Private tuition (ages 3-16)</t>
+        </is>
+      </c>
+      <c r="C529" s="4" t="inlineStr">
+        <is>
+          <t>Dulwich Village, South London</t>
+        </is>
+      </c>
+      <c r="D529" s="4" t="inlineStr">
+        <is>
+          <t>https://dulwich-tutor.co.uk</t>
+        </is>
+      </c>
+      <c r="E529" s="4" t="inlineStr">
+        <is>
+          <t>info@dulwichtutors.com</t>
+        </is>
+      </c>
+      <c r="F529" s="4" t="inlineStr">
+        <is>
+          <t>0208 653 3502</t>
+        </is>
+      </c>
+      <c r="G529" s="4" t="inlineStr">
+        <is>
+          <t>Female founder, 14+ years teaching experience (name not publicly disclosed)</t>
+        </is>
+      </c>
+      <c r="H529" s="4" t="inlineStr"/>
+      <c r="I529" s="4" t="inlineStr"/>
+      <c r="J529" s="4" t="inlineStr">
+        <is>
+          <t>Long-standing owner-operated tutoring agency for maths/English/exam prep across independent and state school curricula; per-session tuition fees recur weekly across a family's school years</t>
+        </is>
+      </c>
+      <c r="K529" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L529" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M529" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N529" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="O529" s="4" t="inlineStr">
+        <is>
+          <t>None visible</t>
+        </is>
+      </c>
+      <c r="P529" s="4" t="inlineStr">
+        <is>
+          <t>14+ years of experience not yet the AI-cited answer for 'tutor Dulwich'</t>
+        </is>
+      </c>
+      <c r="Q529" s="4" t="inlineStr">
+        <is>
+          <t>'14+ years of trusted local tutoring in Dulwich - own that AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R529" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S529" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T529" s="4" t="inlineStr"/>
+    </row>
+    <row r="530">
+      <c r="A530" s="3" t="inlineStr">
+        <is>
+          <t>Crown Kindergartens</t>
+        </is>
+      </c>
+      <c r="B530" s="3" t="inlineStr">
+        <is>
+          <t>Day nursery</t>
+        </is>
+      </c>
+      <c r="C530" s="3" t="inlineStr">
+        <is>
+          <t>Wimbledon, SW19</t>
+        </is>
+      </c>
+      <c r="D530" s="3" t="inlineStr">
+        <is>
+          <t>https://www.crownkindergartens.co.uk</t>
+        </is>
+      </c>
+      <c r="E530" s="3" t="inlineStr">
+        <is>
+          <t>info@crownkindergartens.co.uk</t>
+        </is>
+      </c>
+      <c r="F530" s="3" t="inlineStr">
+        <is>
+          <t>020 8540 8820</t>
+        </is>
+      </c>
+      <c r="G530" s="3" t="inlineStr">
+        <is>
+          <t>Family-run since 1974</t>
+        </is>
+      </c>
+      <c r="H530" s="3" t="inlineStr"/>
+      <c r="I530" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/CrownKindergarten</t>
+        </is>
+      </c>
+      <c r="J530" s="3" t="inlineStr">
+        <is>
+          <t>51-year family-run Wimbledon nursery with a rare large private garden, Ofsted Good in all areas; nursery fees run into thousands per year per child</t>
+        </is>
+      </c>
+      <c r="K530" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L530" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M530" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N530" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O530" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence; 51-year trading history; Ofsted Good across all areas</t>
+        </is>
+      </c>
+      <c r="P530" s="3" t="inlineStr">
+        <is>
+          <t>51-year heritage not yet the AI-cited answer for 'nursery Wimbledon'</t>
+        </is>
+      </c>
+      <c r="Q530" s="3" t="inlineStr">
+        <is>
+          <t>'51 years and Ofsted Good in every area - own that exact AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R530" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S530" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T530" s="3" t="inlineStr"/>
+    </row>
+    <row r="531">
+      <c r="A531" s="3" t="inlineStr">
+        <is>
+          <t>Under the Willow</t>
+        </is>
+      </c>
+      <c r="B531" s="3" t="inlineStr">
+        <is>
+          <t>Montessori-inspired day nursery</t>
+        </is>
+      </c>
+      <c r="C531" s="3" t="inlineStr">
+        <is>
+          <t>Dulwich/Herne Hill, SE21</t>
+        </is>
+      </c>
+      <c r="D531" s="3" t="inlineStr">
+        <is>
+          <t>https://www.underthewillow.co.uk</t>
+        </is>
+      </c>
+      <c r="E531" s="3" t="inlineStr">
+        <is>
+          <t>headteacher@underthewillow.co.uk</t>
+        </is>
+      </c>
+      <c r="F531" s="3" t="inlineStr">
+        <is>
+          <t>020 8761 7972</t>
+        </is>
+      </c>
+      <c r="G531" s="3" t="inlineStr">
+        <is>
+          <t>Mary Haynes (Founder/Owner, est. 2012)</t>
+        </is>
+      </c>
+      <c r="H531" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/maryhaynes</t>
+        </is>
+      </c>
+      <c r="I531" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/Under-The-Willow-163852547114079</t>
+        </is>
+      </c>
+      <c r="J531" s="3" t="inlineStr">
+        <is>
+          <t>13-year eco-friendly Montessori nursery, Ofsted Good (2022); nursery fees run into thousands per year per child</t>
+        </is>
+      </c>
+      <c r="K531" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L531" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M531" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N531" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O531" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn/Facebook presence; Montessori niche positioning; Ofsted Good</t>
+        </is>
+      </c>
+      <c r="P531" s="3" t="inlineStr">
+        <is>
+          <t>Montessori/eco-friendly niche positioning not yet the AI-cited answer for 'Montessori nursery Dulwich'</t>
+        </is>
+      </c>
+      <c r="Q531" s="3" t="inlineStr">
+        <is>
+          <t>'The eco-friendly Montessori choice in Dulwich - own that exact AEO niche positioning'</t>
+        </is>
+      </c>
+      <c r="R531" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S531" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T531" s="3" t="inlineStr"/>
+    </row>
+    <row r="532">
+      <c r="A532" s="3" t="inlineStr">
+        <is>
+          <t>Alexander House Nursery</t>
+        </is>
+      </c>
+      <c r="B532" s="3" t="inlineStr">
+        <is>
+          <t>Day nursery (STEAM-focused, 3 sites)</t>
+        </is>
+      </c>
+      <c r="C532" s="3" t="inlineStr">
+        <is>
+          <t>Wimbledon, Wandsworth &amp; Battersea Reach, SW London</t>
+        </is>
+      </c>
+      <c r="D532" s="3" t="inlineStr">
+        <is>
+          <t>https://www.alexanderhousenursery.com</t>
+        </is>
+      </c>
+      <c r="E532" s="3" t="inlineStr">
+        <is>
+          <t>Wimbledon@alexanderhousenursery.com</t>
+        </is>
+      </c>
+      <c r="F532" s="3" t="inlineStr">
+        <is>
+          <t>0208 240 0299</t>
+        </is>
+      </c>
+      <c r="G532" s="3" t="inlineStr">
+        <is>
+          <t>Family-run, founder has 30+ years' childcare experience</t>
+        </is>
+      </c>
+      <c r="H532" s="3" t="inlineStr"/>
+      <c r="I532" s="3" t="inlineStr">
+        <is>
+          <t>instagram.com/alexanderhousenursery; facebook.com/alexanderhousenursery</t>
+        </is>
+      </c>
+      <c r="J532" s="3" t="inlineStr">
+        <is>
+          <t>3-site independent family-run nursery group with a STEAM curriculum niche; nursery fees run into thousands per year per child across 3 locations</t>
+        </is>
+      </c>
+      <c r="K532" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L532" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M532" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N532" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O532" s="3" t="inlineStr">
+        <is>
+          <t>Instagram/Facebook/TikTok presence = active marketing; STEAM niche positioning</t>
+        </is>
+      </c>
+      <c r="P532" s="3" t="inlineStr">
+        <is>
+          <t>3-site footprint and STEAM niche not matched by per-site AI-search dominance</t>
+        </is>
+      </c>
+      <c r="Q532" s="3" t="inlineStr">
+        <is>
+          <t>Per-site AEO content to own Wimbledon/Wandsworth/Battersea 'STEAM nursery' searches separately</t>
+        </is>
+      </c>
+      <c r="R532" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S532" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T532" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T524"/>
+  <autoFilter ref="A1:T532"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -46512,7 +47236,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B248"/>
+  <dimension ref="A1:B256"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -46532,7 +47256,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>523</v>
+        <v>531</v>
       </c>
     </row>
     <row r="5">
@@ -48969,6 +49693,86 @@
         </is>
       </c>
       <c r="B248" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>Garden &amp; landscape design studio</t>
+        </is>
+      </c>
+      <c r="B249" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>Landscape &amp; garden design studio</t>
+        </is>
+      </c>
+      <c r="B250" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>Private tuition (A-Level/IB/GCSE/KS3)</t>
+        </is>
+      </c>
+      <c r="B251" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>Private tuition (maths, 7+ to Oxbridge entry)</t>
+        </is>
+      </c>
+      <c r="B252" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>Private tuition (ages 3-16)</t>
+        </is>
+      </c>
+      <c r="B253" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>Day nursery</t>
+        </is>
+      </c>
+      <c r="B254" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>Montessori-inspired day nursery</t>
+        </is>
+      </c>
+      <c r="B255" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>Day nursery (STEAM-focused, 3 sites)</t>
+        </is>
+      </c>
+      <c r="B256" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Batches 69-72: +20 prospects (551 total) - Richmond/Wimbledon architects & interior designers, Guildford/Sevenoaks aesthetics, Bristol/Bath wealth managers, Surrey/Kent care homes
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XcaH9h2fjheAYYUkyNFEfe
</commit_message>
<xml_diff>
--- a/prospects/aeora_prospects.xlsx
+++ b/prospects/aeora_prospects.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$532</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$T$552</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T532"/>
+  <dimension ref="A1:T552"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -47224,8 +47224,1896 @@
       </c>
       <c r="T532" s="3" t="inlineStr"/>
     </row>
+    <row r="533">
+      <c r="A533" s="3" t="inlineStr">
+        <is>
+          <t>Michael Jones Architects</t>
+        </is>
+      </c>
+      <c r="B533" s="3" t="inlineStr">
+        <is>
+          <t>Architecture practice (residential/commercial)</t>
+        </is>
+      </c>
+      <c r="C533" s="3" t="inlineStr">
+        <is>
+          <t>Richmond, Surrey</t>
+        </is>
+      </c>
+      <c r="D533" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mjarchitects.co.uk</t>
+        </is>
+      </c>
+      <c r="E533" s="3" t="inlineStr">
+        <is>
+          <t>studio@mjarchitects.co.uk</t>
+        </is>
+      </c>
+      <c r="F533" s="3" t="inlineStr">
+        <is>
+          <t>020 8948 1863</t>
+        </is>
+      </c>
+      <c r="G533" s="3" t="inlineStr">
+        <is>
+          <t>Michael Jones (Founder, est. 1990)</t>
+        </is>
+      </c>
+      <c r="H533" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/michael-jones-architects-limited</t>
+        </is>
+      </c>
+      <c r="I533" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/MJArchitectsLtd</t>
+        </is>
+      </c>
+      <c r="J533" s="3" t="inlineStr">
+        <is>
+          <t>35-year established RIBA chartered Richmond practice spanning private residences to commercial developments; project fees run into tens of thousands per client</t>
+        </is>
+      </c>
+      <c r="K533" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L533" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M533" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N533" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O533" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn/Facebook presence; 35-year trading history; award-winning portfolio</t>
+        </is>
+      </c>
+      <c r="P533" s="3" t="inlineStr">
+        <is>
+          <t>35-year heritage not yet the AI-cited answer for 'architect Richmond'</t>
+        </is>
+      </c>
+      <c r="Q533" s="3" t="inlineStr">
+        <is>
+          <t>'35 years of award-winning architecture in Richmond - own that exact AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R533" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S533" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T533" s="3" t="inlineStr"/>
+    </row>
+    <row r="534">
+      <c r="A534" s="2" t="inlineStr">
+        <is>
+          <t>50 Degrees North Architects</t>
+        </is>
+      </c>
+      <c r="B534" s="2" t="inlineStr">
+        <is>
+          <t>Architecture practice (residential extensions/retrofit)</t>
+        </is>
+      </c>
+      <c r="C534" s="2" t="inlineStr">
+        <is>
+          <t>Richmond, Surrey</t>
+        </is>
+      </c>
+      <c r="D534" s="2" t="inlineStr">
+        <is>
+          <t>https://www.50degrees.co.uk</t>
+        </is>
+      </c>
+      <c r="E534" s="2" t="inlineStr">
+        <is>
+          <t>info@50degrees.co.uk</t>
+        </is>
+      </c>
+      <c r="F534" s="2" t="inlineStr">
+        <is>
+          <t>020 8744 2337</t>
+        </is>
+      </c>
+      <c r="G534" s="2" t="inlineStr">
+        <is>
+          <t>Leigh Bowen (Founder, ARB/RIBA, est. ~2006, worked on BedZED zero-carbon housing)</t>
+        </is>
+      </c>
+      <c r="H534" s="2" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/50-degrees-north-design-consultants-ltd</t>
+        </is>
+      </c>
+      <c r="I534" s="2" t="inlineStr">
+        <is>
+          <t>instagram.com/50degreesnortharchitects</t>
+        </is>
+      </c>
+      <c r="J534" s="2" t="inlineStr">
+        <is>
+          <t>19-year RIBA chartered practice founded by a pioneer of the BedZED zero-carbon housing project; project fees run into tens of thousands per client</t>
+        </is>
+      </c>
+      <c r="K534" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L534" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M534" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N534" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O534" s="2" t="inlineStr">
+        <is>
+          <t>Instagram (3,100+ followers); LinkedIn presence; BedZED pioneer credential = strong authority asset</t>
+        </is>
+      </c>
+      <c r="P534" s="2" t="inlineStr">
+        <is>
+          <t>BedZED pioneer credential not yet the AI-cited answer for 'sustainable architect Richmond'</t>
+        </is>
+      </c>
+      <c r="Q534" s="2" t="inlineStr">
+        <is>
+          <t>'Worked on the pioneering BedZED zero-carbon project - own that exact AEO authority signal'</t>
+        </is>
+      </c>
+      <c r="R534" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S534" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T534" s="2" t="inlineStr">
+        <is>
+          <t>BedZED pioneer credential - exceptional AEO hook for sustainability-focused clients</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" s="2" t="inlineStr">
+        <is>
+          <t>Tania Azadian Interiors</t>
+        </is>
+      </c>
+      <c r="B535" s="2" t="inlineStr">
+        <is>
+          <t>Luxury interior design</t>
+        </is>
+      </c>
+      <c r="C535" s="2" t="inlineStr">
+        <is>
+          <t>Wimbledon Village, London</t>
+        </is>
+      </c>
+      <c r="D535" s="2" t="inlineStr">
+        <is>
+          <t>https://www.taniaazadianinteriors.com</t>
+        </is>
+      </c>
+      <c r="E535" s="2" t="inlineStr">
+        <is>
+          <t>info@taniaazadianinteriors.com</t>
+        </is>
+      </c>
+      <c r="F535" s="2" t="inlineStr">
+        <is>
+          <t>07946 533380</t>
+        </is>
+      </c>
+      <c r="G535" s="2" t="inlineStr">
+        <is>
+          <t>Tania Azadian (Founder, ex-Kelly Hoppen Senior Designer, est. 2016)</t>
+        </is>
+      </c>
+      <c r="H535" s="2" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/tania-azadian; linkedin.com/company/tania-azadian-interiors-ltd</t>
+        </is>
+      </c>
+      <c r="I535" s="2" t="inlineStr">
+        <is>
+          <t>instagram.com/tania_azadian_interiors; facebook.com/taniaazadianinteriors</t>
+        </is>
+      </c>
+      <c r="J535" s="2" t="inlineStr">
+        <is>
+          <t>One of only a few BIID Registered designers in Wimbledon, founder sits on the BIID council; project fees run into tens of thousands per client</t>
+        </is>
+      </c>
+      <c r="K535" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L535" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M535" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N535" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O535" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn/Instagram/Facebook presence; BIID council position; ex-Kelly Hoppen pedigree</t>
+        </is>
+      </c>
+      <c r="P535" s="2" t="inlineStr">
+        <is>
+          <t>BIID council position and Kelly Hoppen pedigree not yet the AI-cited trust signal for 'interior designer Wimbledon'</t>
+        </is>
+      </c>
+      <c r="Q535" s="2" t="inlineStr">
+        <is>
+          <t>'A BIID council member and ex-Kelly Hoppen designer - own that exact AEO credibility signal'</t>
+        </is>
+      </c>
+      <c r="R535" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S535" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T535" s="2" t="inlineStr">
+        <is>
+          <t>BIID council position + Kelly Hoppen pedigree - exceptional AEO credibility hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" s="3" t="inlineStr">
+        <is>
+          <t>Gomm Studio</t>
+        </is>
+      </c>
+      <c r="B536" s="3" t="inlineStr">
+        <is>
+          <t>Boutique interior design</t>
+        </is>
+      </c>
+      <c r="C536" s="3" t="inlineStr">
+        <is>
+          <t>Wimbledon Village, London</t>
+        </is>
+      </c>
+      <c r="D536" s="3" t="inlineStr">
+        <is>
+          <t>https://www.gommstudio.com</t>
+        </is>
+      </c>
+      <c r="E536" s="3" t="inlineStr">
+        <is>
+          <t>office@gommstudio.com</t>
+        </is>
+      </c>
+      <c r="F536" s="3" t="inlineStr"/>
+      <c r="G536" s="3" t="inlineStr">
+        <is>
+          <t>Louise Gomm (Founder, BIID registered, KLC-trained, est. 2015)</t>
+        </is>
+      </c>
+      <c r="H536" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/louise-gomm-86507152</t>
+        </is>
+      </c>
+      <c r="I536" s="3" t="inlineStr">
+        <is>
+          <t>facebook.com/gommstudio</t>
+        </is>
+      </c>
+      <c r="J536" s="3" t="inlineStr">
+        <is>
+          <t>10-year award-winning family-run boutique studio for residential/commercial clients; project fees run into tens of thousands per client</t>
+        </is>
+      </c>
+      <c r="K536" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L536" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M536" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N536" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O536" s="3" t="inlineStr">
+        <is>
+          <t>Facebook presence; press feature (Humphrey Munson Q&amp;A); award-winning</t>
+        </is>
+      </c>
+      <c r="P536" s="3" t="inlineStr">
+        <is>
+          <t>Press feature and award-winning status not yet the AI-cited answer for 'interior designer Wimbledon'</t>
+        </is>
+      </c>
+      <c r="Q536" s="3" t="inlineStr">
+        <is>
+          <t>'Award-winning and featured in the press - own that exact AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R536" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S536" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T536" s="3" t="inlineStr"/>
+    </row>
+    <row r="537">
+      <c r="A537" s="3" t="inlineStr">
+        <is>
+          <t>Anna Auzins Interiors</t>
+        </is>
+      </c>
+      <c r="B537" s="3" t="inlineStr">
+        <is>
+          <t>Boutique residential interior design</t>
+        </is>
+      </c>
+      <c r="C537" s="3" t="inlineStr">
+        <is>
+          <t>Wimbledon, London</t>
+        </is>
+      </c>
+      <c r="D537" s="3" t="inlineStr">
+        <is>
+          <t>https://www.annaauzins.co.uk</t>
+        </is>
+      </c>
+      <c r="E537" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F537" s="3" t="inlineStr"/>
+      <c r="G537" s="3" t="inlineStr">
+        <is>
+          <t>Anna Auzins (Founder, KLC-trained, est. 2008)</t>
+        </is>
+      </c>
+      <c r="H537" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/anna-auzins-0a590b14</t>
+        </is>
+      </c>
+      <c r="I537" s="3" t="inlineStr">
+        <is>
+          <t>instagram.com/annaauzins; facebook.com/AnnaAuzinsInteriors</t>
+        </is>
+      </c>
+      <c r="J537" s="3" t="inlineStr">
+        <is>
+          <t>17-year boutique interior design studio with a distinctive people-first design approach, press-featured (Hayche/H Furniture); project fees run into tens of thousands per client</t>
+        </is>
+      </c>
+      <c r="K537" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L537" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M537" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N537" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O537" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn/Instagram/Facebook presence; 17-year trading history; press feature</t>
+        </is>
+      </c>
+      <c r="P537" s="3" t="inlineStr">
+        <is>
+          <t>17-year heritage and press feature not yet the AI-cited answer for 'interior designer Wimbledon'</t>
+        </is>
+      </c>
+      <c r="Q537" s="3" t="inlineStr">
+        <is>
+          <t>'17 years of people-first interior design in Wimbledon - own that AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R537" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S537" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T537" s="3" t="inlineStr"/>
+    </row>
+    <row r="538">
+      <c r="A538" s="4" t="inlineStr">
+        <is>
+          <t>Studio Belle Interior Design</t>
+        </is>
+      </c>
+      <c r="B538" s="4" t="inlineStr">
+        <is>
+          <t>High-end interior design</t>
+        </is>
+      </c>
+      <c r="C538" s="4" t="inlineStr">
+        <is>
+          <t>Wimbledon Village, London</t>
+        </is>
+      </c>
+      <c r="D538" s="4" t="inlineStr">
+        <is>
+          <t>https://www.studiobelle.co.uk</t>
+        </is>
+      </c>
+      <c r="E538" s="4" t="inlineStr">
+        <is>
+          <t>jessica@studiobelle.co.uk</t>
+        </is>
+      </c>
+      <c r="F538" s="4" t="inlineStr"/>
+      <c r="G538" s="4" t="inlineStr">
+        <is>
+          <t>Jessica Bell (Founder, est. 2021)</t>
+        </is>
+      </c>
+      <c r="H538" s="4" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/jessica-bell-5b722290</t>
+        </is>
+      </c>
+      <c r="I538" s="4" t="inlineStr"/>
+      <c r="J538" s="4" t="inlineStr">
+        <is>
+          <t>Growing independent studio for high-end London residential/commercial projects; project fees run into tens of thousands per client</t>
+        </is>
+      </c>
+      <c r="K538" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L538" s="4" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M538" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N538" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O538" s="4" t="inlineStr">
+        <is>
+          <t>LinkedIn presence</t>
+        </is>
+      </c>
+      <c r="P538" s="4" t="inlineStr">
+        <is>
+          <t>New but growing studio - ground-floor opportunity to own local AEO search before bigger studios do</t>
+        </is>
+      </c>
+      <c r="Q538" s="4" t="inlineStr">
+        <is>
+          <t>'A rising name in Wimbledon interior design - be the AI-cited answer before competitors catch on'</t>
+        </is>
+      </c>
+      <c r="R538" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="S538" s="4" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T538" s="4" t="inlineStr"/>
+    </row>
+    <row r="539">
+      <c r="A539" s="3" t="inlineStr">
+        <is>
+          <t>Verse Medical Aesthetics</t>
+        </is>
+      </c>
+      <c r="B539" s="3" t="inlineStr">
+        <is>
+          <t>Aesthetics clinic (injectables, skin)</t>
+        </is>
+      </c>
+      <c r="C539" s="3" t="inlineStr">
+        <is>
+          <t>Guildford, Surrey</t>
+        </is>
+      </c>
+      <c r="D539" s="3" t="inlineStr">
+        <is>
+          <t>https://www.versemedicalaesthetics.com</t>
+        </is>
+      </c>
+      <c r="E539" s="3" t="inlineStr">
+        <is>
+          <t>marta@versemedicalaesthetics.com</t>
+        </is>
+      </c>
+      <c r="F539" s="3" t="inlineStr">
+        <is>
+          <t>07476 695696</t>
+        </is>
+      </c>
+      <c r="G539" s="3" t="inlineStr">
+        <is>
+          <t>Marta (Founder, NMC-registered nurse, V300 Independent Prescriber, ex-lawyer)</t>
+        </is>
+      </c>
+      <c r="H539" s="3" t="inlineStr"/>
+      <c r="I539" s="3" t="inlineStr"/>
+      <c r="J539" s="3" t="inlineStr">
+        <is>
+          <t>Nurse-led injectables/skin clinic founded by a former Polish lawyer/barrister who retrained as a nurse prescriber; repeat treatment clients, premium per-session fees</t>
+        </is>
+      </c>
+      <c r="K539" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L539" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M539" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N539" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O539" s="3" t="inlineStr">
+        <is>
+          <t>Unusual ex-lawyer founder story = strong PR asset</t>
+        </is>
+      </c>
+      <c r="P539" s="3" t="inlineStr">
+        <is>
+          <t>Unique career-change founder story not yet the AI-cited answer for 'aesthetics clinic Guildford'</t>
+        </is>
+      </c>
+      <c r="Q539" s="3" t="inlineStr">
+        <is>
+          <t>'From barrister to nurse prescriber - own that exact AEO founder story'</t>
+        </is>
+      </c>
+      <c r="R539" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S539" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T539" s="3" t="inlineStr"/>
+    </row>
+    <row r="540">
+      <c r="A540" s="2" t="inlineStr">
+        <is>
+          <t>Optimise Aesthetics</t>
+        </is>
+      </c>
+      <c r="B540" s="2" t="inlineStr">
+        <is>
+          <t>Aesthetics, wellness &amp; weight-loss clinic</t>
+        </is>
+      </c>
+      <c r="C540" s="2" t="inlineStr">
+        <is>
+          <t>Guildford, Surrey</t>
+        </is>
+      </c>
+      <c r="D540" s="2" t="inlineStr">
+        <is>
+          <t>https://www.optimiseaesthetics.com</t>
+        </is>
+      </c>
+      <c r="E540" s="2" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F540" s="2" t="inlineStr">
+        <is>
+          <t>07581 375192</t>
+        </is>
+      </c>
+      <c r="G540" s="2" t="inlineStr">
+        <is>
+          <t>Dr Louise Bye (Founder, GP/eye surgeon, est. 2019)</t>
+        </is>
+      </c>
+      <c r="H540" s="2" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/dr-louise-bye-235bbb330</t>
+        </is>
+      </c>
+      <c r="I540" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/optimiseaesthetics</t>
+        </is>
+      </c>
+      <c r="J540" s="2" t="inlineStr">
+        <is>
+          <t>CQC-registered, award-winning doctor-led clinic founded by a dual-qualified GP and eye surgeon; repeat treatment clients, premium per-session fees</t>
+        </is>
+      </c>
+      <c r="K540" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L540" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M540" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N540" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O540" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn/Facebook presence; CQC registration; award-winning</t>
+        </is>
+      </c>
+      <c r="P540" s="2" t="inlineStr">
+        <is>
+          <t>Dual-qualification founder credential not yet the AI-cited trust signal for 'aesthetics clinic Guildford'</t>
+        </is>
+      </c>
+      <c r="Q540" s="2" t="inlineStr">
+        <is>
+          <t>'Led by a GP and eye surgeon, CQC-registered - own that exact AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R540" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S540" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T540" s="2" t="inlineStr">
+        <is>
+          <t>Dual medical qualification founder - exceptional AEO credibility hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" s="3" t="inlineStr">
+        <is>
+          <t>First Aesthetics (Guildford)</t>
+        </is>
+      </c>
+      <c r="B541" s="3" t="inlineStr">
+        <is>
+          <t>Aesthetics &amp; skin clinic</t>
+        </is>
+      </c>
+      <c r="C541" s="3" t="inlineStr">
+        <is>
+          <t>Guildford, Surrey</t>
+        </is>
+      </c>
+      <c r="D541" s="3" t="inlineStr">
+        <is>
+          <t>https://firstaesthetics.co.uk</t>
+        </is>
+      </c>
+      <c r="E541" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F541" s="3" t="inlineStr"/>
+      <c r="G541" s="3" t="inlineStr">
+        <is>
+          <t>Dr Bib &amp; Dr Shova (Co-founders, Harley Street-trained, 40+ yrs combined experience)</t>
+        </is>
+      </c>
+      <c r="H541" s="3" t="inlineStr"/>
+      <c r="I541" s="3" t="inlineStr">
+        <is>
+          <t>instagram.com/dr.bib.guildford</t>
+        </is>
+      </c>
+      <c r="J541" s="3" t="inlineStr">
+        <is>
+          <t>Harley Street-trained doctor-led clinic with a co-founder holding both a medical and law degree; repeat treatment clients, premium per-session fees</t>
+        </is>
+      </c>
+      <c r="K541" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L541" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M541" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N541" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O541" s="3" t="inlineStr">
+        <is>
+          <t>Instagram presence; Harley Street training pedigree</t>
+        </is>
+      </c>
+      <c r="P541" s="3" t="inlineStr">
+        <is>
+          <t>Harley Street pedigree not yet the AI-cited answer for 'Botox clinic Guildford'</t>
+        </is>
+      </c>
+      <c r="Q541" s="3" t="inlineStr">
+        <is>
+          <t>'Harley Street-trained doctors, now in Guildford - own that exact AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R541" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S541" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T541" s="3" t="inlineStr"/>
+    </row>
+    <row r="542">
+      <c r="A542" s="2" t="inlineStr">
+        <is>
+          <t>Dr Paulina Charlesworth Aesthetics</t>
+        </is>
+      </c>
+      <c r="B542" s="2" t="inlineStr">
+        <is>
+          <t>GP-led aesthetics &amp; longevity clinic</t>
+        </is>
+      </c>
+      <c r="C542" s="2" t="inlineStr">
+        <is>
+          <t>Underriver, Sevenoaks, Kent</t>
+        </is>
+      </c>
+      <c r="D542" s="2" t="inlineStr">
+        <is>
+          <t>https://drcharlesworth.co.uk</t>
+        </is>
+      </c>
+      <c r="E542" s="2" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F542" s="2" t="inlineStr">
+        <is>
+          <t>01732 682439</t>
+        </is>
+      </c>
+      <c r="G542" s="2" t="inlineStr">
+        <is>
+          <t>Dr Paulina Charlesworth MBBS MRCGP (Founder, ~10 years trading)</t>
+        </is>
+      </c>
+      <c r="H542" s="2" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/dr-paulina-charlesworth-mbbs-mrcgp-9b748a296</t>
+        </is>
+      </c>
+      <c r="I542" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/charlesworthclinic</t>
+        </is>
+      </c>
+      <c r="J542" s="2" t="inlineStr">
+        <is>
+          <t>American Board Certified GP-led aesthetics/anti-ageing clinic trained across UK/California/Paris; repeat treatment clients, premium per-session fees</t>
+        </is>
+      </c>
+      <c r="K542" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L542" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M542" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N542" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O542" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn/Facebook presence; American Board Certification; ~10-year trading history</t>
+        </is>
+      </c>
+      <c r="P542" s="2" t="inlineStr">
+        <is>
+          <t>International board certification not yet the AI-cited trust signal for 'aesthetics clinic Sevenoaks'</t>
+        </is>
+      </c>
+      <c r="Q542" s="2" t="inlineStr">
+        <is>
+          <t>'American Board Certified in Anti-Ageing Medicine - own that exact AEO credibility signal'</t>
+        </is>
+      </c>
+      <c r="R542" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S542" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T542" s="2" t="inlineStr">
+        <is>
+          <t>International board certification - exceptional AEO credibility hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" s="3" t="inlineStr">
+        <is>
+          <t>Greenhouse Aesthetics</t>
+        </is>
+      </c>
+      <c r="B543" s="3" t="inlineStr">
+        <is>
+          <t>Aesthetics clinic (30+ treatments)</t>
+        </is>
+      </c>
+      <c r="C543" s="3" t="inlineStr">
+        <is>
+          <t>Sevenoaks, Kent</t>
+        </is>
+      </c>
+      <c r="D543" s="3" t="inlineStr">
+        <is>
+          <t>https://www.greenhouseaesthetics.com</t>
+        </is>
+      </c>
+      <c r="E543" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F543" s="3" t="inlineStr"/>
+      <c r="G543" s="3" t="inlineStr">
+        <is>
+          <t>Tanya Garcia (Owner/Clinical Director, ex-Guy's Hospital dental training, ~5 years trading)</t>
+        </is>
+      </c>
+      <c r="H543" s="3" t="inlineStr"/>
+      <c r="I543" s="3" t="inlineStr">
+        <is>
+          <t>instagram.com/thegreenhouseaesthetics; facebook.com/thegreenhouseaesthetics</t>
+        </is>
+      </c>
+      <c r="J543" s="3" t="inlineStr">
+        <is>
+          <t>5-star rated clinic offering 30+ treatments, founded by a Guy's Hospital-trained practitioner; repeat treatment clients, premium per-session fees</t>
+        </is>
+      </c>
+      <c r="K543" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L543" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M543" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N543" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O543" s="3" t="inlineStr">
+        <is>
+          <t>Instagram/Facebook presence; 5-star rating</t>
+        </is>
+      </c>
+      <c r="P543" s="3" t="inlineStr">
+        <is>
+          <t>5-star rating not yet the AI-cited trust signal for 'aesthetics clinic Sevenoaks'</t>
+        </is>
+      </c>
+      <c r="Q543" s="3" t="inlineStr">
+        <is>
+          <t>'5-star rated across 30+ treatments - own that exact AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R543" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S543" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T543" s="3" t="inlineStr"/>
+    </row>
+    <row r="544">
+      <c r="A544" s="3" t="inlineStr">
+        <is>
+          <t>Lumen Skin Clinic</t>
+        </is>
+      </c>
+      <c r="B544" s="3" t="inlineStr">
+        <is>
+          <t>Aesthetics &amp; functional medicine clinic</t>
+        </is>
+      </c>
+      <c r="C544" s="3" t="inlineStr">
+        <is>
+          <t>Sevenoaks, Kent</t>
+        </is>
+      </c>
+      <c r="D544" s="3" t="inlineStr">
+        <is>
+          <t>https://lumenskinclinic.co.uk</t>
+        </is>
+      </c>
+      <c r="E544" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F544" s="3" t="inlineStr">
+        <is>
+          <t>01732 252770</t>
+        </is>
+      </c>
+      <c r="G544" s="3" t="inlineStr">
+        <is>
+          <t>Iwona Taylor (Founder, Registered Nurse Prescriber, dermatology-trained at Guy's &amp; St Thomas's)</t>
+        </is>
+      </c>
+      <c r="H544" s="3" t="inlineStr"/>
+      <c r="I544" s="3" t="inlineStr">
+        <is>
+          <t>instagram.com/lumen_skin_clinic; facebook.com/Lumenskinclinic</t>
+        </is>
+      </c>
+      <c r="J544" s="3" t="inlineStr">
+        <is>
+          <t>Nurse-led clinic combining aesthetic treatments with functional medicine, trained under a renowned Harley Street dermatologist; repeat treatment clients, premium per-session fees</t>
+        </is>
+      </c>
+      <c r="K544" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L544" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M544" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N544" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O544" s="3" t="inlineStr">
+        <is>
+          <t>Instagram/Facebook presence; dermatology + functional medicine dual specialism</t>
+        </is>
+      </c>
+      <c r="P544" s="3" t="inlineStr">
+        <is>
+          <t>Dual dermatology/functional-medicine specialism not yet the AI-cited answer for 'skin clinic Sevenoaks'</t>
+        </is>
+      </c>
+      <c r="Q544" s="3" t="inlineStr">
+        <is>
+          <t>'Dermatology training plus functional medicine - own that exact AEO dual-specialism positioning'</t>
+        </is>
+      </c>
+      <c r="R544" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S544" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T544" s="3" t="inlineStr"/>
+    </row>
+    <row r="545">
+      <c r="A545" s="3" t="inlineStr">
+        <is>
+          <t>Brigstow Independent Financial Planning</t>
+        </is>
+      </c>
+      <c r="B545" s="3" t="inlineStr">
+        <is>
+          <t>IFA / financial planning</t>
+        </is>
+      </c>
+      <c r="C545" s="3" t="inlineStr">
+        <is>
+          <t>Downend, Bristol</t>
+        </is>
+      </c>
+      <c r="D545" s="3" t="inlineStr">
+        <is>
+          <t>https://www.brigstowifp.co.uk</t>
+        </is>
+      </c>
+      <c r="E545" s="3" t="inlineStr">
+        <is>
+          <t>info@brigstowifp.co.uk</t>
+        </is>
+      </c>
+      <c r="F545" s="3" t="inlineStr">
+        <is>
+          <t>07894 708855</t>
+        </is>
+      </c>
+      <c r="G545" s="3" t="inlineStr">
+        <is>
+          <t>Giles &amp; Dean (Co-founders, Chartered Financial Planners, 25+ yrs experience, left Close Brothers-owned network in 2024)</t>
+        </is>
+      </c>
+      <c r="H545" s="3" t="inlineStr"/>
+      <c r="I545" s="3" t="inlineStr"/>
+      <c r="J545" s="3" t="inlineStr">
+        <is>
+          <t>Founders deliberately left a bank-owned advice network to return to true independence, naming the firm after Bristol's Old English name; ongoing wealth-management fees run into thousands annually per client</t>
+        </is>
+      </c>
+      <c r="K545" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L545" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M545" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N545" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O545" s="3" t="inlineStr">
+        <is>
+          <t>Deliberate 'return to independence' founder story = strong trust narrative</t>
+        </is>
+      </c>
+      <c r="P545" s="3" t="inlineStr">
+        <is>
+          <t>'Left a bank-owned network to go independent' story not yet the AI-cited answer for 'IFA Bristol'</t>
+        </is>
+      </c>
+      <c r="Q545" s="3" t="inlineStr">
+        <is>
+          <t>'We left a bank-owned network to be truly independent again - own that exact AEO trust story'</t>
+        </is>
+      </c>
+      <c r="R545" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S545" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T545" s="3" t="inlineStr"/>
+    </row>
+    <row r="546">
+      <c r="A546" s="3" t="inlineStr">
+        <is>
+          <t>Sunrise Independent Financial Advisers</t>
+        </is>
+      </c>
+      <c r="B546" s="3" t="inlineStr">
+        <is>
+          <t>IFA / ethical &amp; sustainable investment advice</t>
+        </is>
+      </c>
+      <c r="C546" s="3" t="inlineStr">
+        <is>
+          <t>Clifton, Bristol</t>
+        </is>
+      </c>
+      <c r="D546" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sunrise-ifa.co.uk</t>
+        </is>
+      </c>
+      <c r="E546" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F546" s="3" t="inlineStr">
+        <is>
+          <t>0117 244 3862</t>
+        </is>
+      </c>
+      <c r="G546" s="3" t="inlineStr">
+        <is>
+          <t>Guy Roper FPFS (Founder, Fellow of the Personal Finance Society - PFS's highest qualification level, est. 2019)</t>
+        </is>
+      </c>
+      <c r="H546" s="3" t="inlineStr"/>
+      <c r="I546" s="3" t="inlineStr"/>
+      <c r="J546" s="3" t="inlineStr">
+        <is>
+          <t>Ethical/sustainable-investment focused IFA led by a Fellow of the PFS (the profession's top qualification tier); ongoing wealth-management fees run into thousands annually per client</t>
+        </is>
+      </c>
+      <c r="K546" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L546" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M546" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N546" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O546" s="3" t="inlineStr">
+        <is>
+          <t>PFS Fellowship = highest national qualification tier; ethical-investment niche</t>
+        </is>
+      </c>
+      <c r="P546" s="3" t="inlineStr">
+        <is>
+          <t>PFS Fellowship and ethical-investment niche not yet the AI-cited answer for 'ethical IFA Bristol'</t>
+        </is>
+      </c>
+      <c r="Q546" s="3" t="inlineStr">
+        <is>
+          <t>'A Fellow of the Personal Finance Society specialising in ethical investing - own that exact AEO niche'</t>
+        </is>
+      </c>
+      <c r="R546" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S546" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T546" s="3" t="inlineStr"/>
+    </row>
+    <row r="547">
+      <c r="A547" s="2" t="inlineStr">
+        <is>
+          <t>Combined Financial Strategies (CFS)</t>
+        </is>
+      </c>
+      <c r="B547" s="2" t="inlineStr">
+        <is>
+          <t>IFA / financial planning</t>
+        </is>
+      </c>
+      <c r="C547" s="2" t="inlineStr">
+        <is>
+          <t>Bath</t>
+        </is>
+      </c>
+      <c r="D547" s="2" t="inlineStr">
+        <is>
+          <t>https://www.cfsorg.com</t>
+        </is>
+      </c>
+      <c r="E547" s="2" t="inlineStr">
+        <is>
+          <t>info@cfsorg.com</t>
+        </is>
+      </c>
+      <c r="F547" s="2" t="inlineStr">
+        <is>
+          <t>01225 471462</t>
+        </is>
+      </c>
+      <c r="G547" s="2" t="inlineStr">
+        <is>
+          <t>Jonothan McColgan (Founder, Chartered Financial Planner, UK Financial Adviser of the Year winner)</t>
+        </is>
+      </c>
+      <c r="H547" s="2" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/jonothanmccolgan</t>
+        </is>
+      </c>
+      <c r="I547" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/combinedfinancialstrategies</t>
+        </is>
+      </c>
+      <c r="J547" s="2" t="inlineStr">
+        <is>
+          <t>Founder is a national award-winning adviser and regular FT/Times/Telegraph/Mail on Sunday commentator; ongoing wealth-management fees run into thousands annually per client</t>
+        </is>
+      </c>
+      <c r="K547" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L547" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M547" s="2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="N547" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O547" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn/Facebook presence; national press commentator status; UK Adviser of the Year award</t>
+        </is>
+      </c>
+      <c r="P547" s="2" t="inlineStr">
+        <is>
+          <t>National press-commentator status not yet the AI-cited answer for 'financial adviser Bath'</t>
+        </is>
+      </c>
+      <c r="Q547" s="2" t="inlineStr">
+        <is>
+          <t>'Quoted in the FT and the Times, UK Adviser of the Year - own that exact AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R547" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S547" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T547" s="2" t="inlineStr">
+        <is>
+          <t>National press commentator + top industry award - exceptional AEO hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" s="3" t="inlineStr">
+        <is>
+          <t>Mhairi Cameron Consulting</t>
+        </is>
+      </c>
+      <c r="B548" s="3" t="inlineStr">
+        <is>
+          <t>Leadership &amp; organisational development consultancy</t>
+        </is>
+      </c>
+      <c r="C548" s="3" t="inlineStr">
+        <is>
+          <t>Bristol</t>
+        </is>
+      </c>
+      <c r="D548" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mhairicameronconsulting.co.uk</t>
+        </is>
+      </c>
+      <c r="E548" s="3" t="inlineStr">
+        <is>
+          <t>via website contact form</t>
+        </is>
+      </c>
+      <c r="F548" s="3" t="inlineStr">
+        <is>
+          <t>07711 764128</t>
+        </is>
+      </c>
+      <c r="G548" s="3" t="inlineStr">
+        <is>
+          <t>Mhairi Cameron (Founder/Director, est. 2003, ICF member)</t>
+        </is>
+      </c>
+      <c r="H548" s="3" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/mhairi-cameron-13426010</t>
+        </is>
+      </c>
+      <c r="I548" s="3" t="inlineStr"/>
+      <c r="J548" s="3" t="inlineStr">
+        <is>
+          <t>22-year executive coaching/organisational-change consultancy with UK, Europe, Africa and Australia client experience; monthly retained consultancy fees recur across a client's leadership development</t>
+        </is>
+      </c>
+      <c r="K548" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L548" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M548" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="N548" s="3" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O548" s="3" t="inlineStr">
+        <is>
+          <t>LinkedIn presence; 22-year trading history; international client base</t>
+        </is>
+      </c>
+      <c r="P548" s="3" t="inlineStr">
+        <is>
+          <t>22-year international track record not yet the AI-cited answer for 'executive coach Bristol'</t>
+        </is>
+      </c>
+      <c r="Q548" s="3" t="inlineStr">
+        <is>
+          <t>'22 years coaching leaders across 4 continents - own that AEO trust signal in Bristol'</t>
+        </is>
+      </c>
+      <c r="R548" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="S548" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T548" s="3" t="inlineStr"/>
+    </row>
+    <row r="549">
+      <c r="A549" s="2" t="inlineStr">
+        <is>
+          <t>Huntington &amp; Langham Estate</t>
+        </is>
+      </c>
+      <c r="B549" s="2" t="inlineStr">
+        <is>
+          <t>Care home group (residential, nursing, dementia)</t>
+        </is>
+      </c>
+      <c r="C549" s="2" t="inlineStr">
+        <is>
+          <t>Hindhead, Surrey (2 homes on a 30-acre estate)</t>
+        </is>
+      </c>
+      <c r="D549" s="2" t="inlineStr">
+        <is>
+          <t>https://www.huntingtonlangham.estate</t>
+        </is>
+      </c>
+      <c r="E549" s="2" t="inlineStr">
+        <is>
+          <t>enquiries@huntingtonhouse.co.uk</t>
+        </is>
+      </c>
+      <c r="F549" s="2" t="inlineStr">
+        <is>
+          <t>01428 604600</t>
+        </is>
+      </c>
+      <c r="G549" s="2" t="inlineStr">
+        <is>
+          <t>Hoare family (4th generation, Charlie &amp; Sarah Hoare, since 1977)</t>
+        </is>
+      </c>
+      <c r="H549" s="2" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/huntington-langham</t>
+        </is>
+      </c>
+      <c r="I549" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/huntingtonandlangham; instagram.com/huntingtonlanghamestate</t>
+        </is>
+      </c>
+      <c r="J549" s="2" t="inlineStr">
+        <is>
+          <t>48-year, four-generation family-owned care estate with 2 CQC Good-rated homes on 30 acres; care fees run into thousands per month per resident, recurring</t>
+        </is>
+      </c>
+      <c r="K549" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L549" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="M549" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N549" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O549" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn/Facebook/Instagram presence; 48-year 4-generation family history; CQC Good x2</t>
+        </is>
+      </c>
+      <c r="P549" s="2" t="inlineStr">
+        <is>
+          <t>48-year, 4-generation family story not yet the AI-cited answer for 'care home Surrey'</t>
+        </is>
+      </c>
+      <c r="Q549" s="2" t="inlineStr">
+        <is>
+          <t>'Four generations of the same family, 48 years of care - own that exact AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R549" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S549" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T549" s="2" t="inlineStr">
+        <is>
+          <t>4-generation family heritage on a 30-acre estate - exceptional AEO hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" s="2" t="inlineStr">
+        <is>
+          <t>Everycare Central Surrey</t>
+        </is>
+      </c>
+      <c r="B550" s="2" t="inlineStr">
+        <is>
+          <t>Home care agency</t>
+        </is>
+      </c>
+      <c r="C550" s="2" t="inlineStr">
+        <is>
+          <t>Merrow, Guildford, Surrey (Guildford/Woking/Leatherhead/Bookham/Godalming)</t>
+        </is>
+      </c>
+      <c r="D550" s="2" t="inlineStr">
+        <is>
+          <t>https://www.everycare.co.uk/centralsurrey</t>
+        </is>
+      </c>
+      <c r="E550" s="2" t="inlineStr">
+        <is>
+          <t>centralsurrey@everycare.co.uk</t>
+        </is>
+      </c>
+      <c r="F550" s="2" t="inlineStr">
+        <is>
+          <t>01483 536266</t>
+        </is>
+      </c>
+      <c r="G550" s="2" t="inlineStr">
+        <is>
+          <t>Pauline Herring (Founder, est. 2012), now run by daughter Serena Coates</t>
+        </is>
+      </c>
+      <c r="H550" s="2" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/everycare-central-surrey-ltd</t>
+        </is>
+      </c>
+      <c r="I550" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/EverycareCentralSurrey</t>
+        </is>
+      </c>
+      <c r="J550" s="2" t="inlineStr">
+        <is>
+          <t>13-year mother-to-daughter family care agency, CQC Good, finalist and 'Most Trusted Home Care Provider - Surrey' award winner; care packages worth thousands per month per client</t>
+        </is>
+      </c>
+      <c r="K550" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L550" s="2" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M550" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N550" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O550" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn/Facebook presence; national award win; CQC Good</t>
+        </is>
+      </c>
+      <c r="P550" s="2" t="inlineStr">
+        <is>
+          <t>'Most Trusted' award win not yet the AI-cited answer for 'home care Guildford'</t>
+        </is>
+      </c>
+      <c r="Q550" s="2" t="inlineStr">
+        <is>
+          <t>'Voted Surrey's Most Trusted Home Care Provider - own that exact AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R550" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S550" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T550" s="2" t="inlineStr">
+        <is>
+          <t>National 'Most Trusted' award - strong AEO hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" s="2" t="inlineStr">
+        <is>
+          <t>Azure Care</t>
+        </is>
+      </c>
+      <c r="B551" s="2" t="inlineStr">
+        <is>
+          <t>Home care &amp; live-in care agency</t>
+        </is>
+      </c>
+      <c r="C551" s="2" t="inlineStr">
+        <is>
+          <t>Chatham, Kent (Medway)</t>
+        </is>
+      </c>
+      <c r="D551" s="2" t="inlineStr">
+        <is>
+          <t>https://www.azurecare.co.uk</t>
+        </is>
+      </c>
+      <c r="E551" s="2" t="inlineStr">
+        <is>
+          <t>hello@azurecare.co.uk</t>
+        </is>
+      </c>
+      <c r="F551" s="2" t="inlineStr">
+        <is>
+          <t>01634 968300</t>
+        </is>
+      </c>
+      <c r="G551" s="2" t="inlineStr">
+        <is>
+          <t>Kiran Gill &amp; Parvinder Dusanj (Co-founders, est. 2019)</t>
+        </is>
+      </c>
+      <c r="H551" s="2" t="inlineStr">
+        <is>
+          <t>linkedin.com/company/azurecare</t>
+        </is>
+      </c>
+      <c r="I551" s="2" t="inlineStr">
+        <is>
+          <t>facebook.com/AzureCareLtd</t>
+        </is>
+      </c>
+      <c r="J551" s="2" t="inlineStr">
+        <is>
+          <t>The only CQC Outstanding-rated home care provider in Medway; care packages worth thousands per month per client</t>
+        </is>
+      </c>
+      <c r="K551" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L551" s="2" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="M551" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N551" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="O551" s="2" t="inlineStr">
+        <is>
+          <t>LinkedIn/Facebook presence; sole CQC Outstanding rating in Medway; local press coverage (Kent Online)</t>
+        </is>
+      </c>
+      <c r="P551" s="2" t="inlineStr">
+        <is>
+          <t>Sole-Outstanding-in-Medway status not yet the AI-cited trust signal for 'home care Medway'</t>
+        </is>
+      </c>
+      <c r="Q551" s="2" t="inlineStr">
+        <is>
+          <t>'The only Outstanding-rated home care provider in Medway - own that exact AEO trust signal'</t>
+        </is>
+      </c>
+      <c r="R551" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="S551" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="T551" s="2" t="inlineStr">
+        <is>
+          <t>Sole CQC Outstanding rating in the entire Medway area - exceptional AEO hook</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" s="4" t="inlineStr">
+        <is>
+          <t>Birchwood House &amp; Birchwood Care Services</t>
+        </is>
+      </c>
+      <c r="B552" s="4" t="inlineStr">
+        <is>
+          <t>Residential care home + domicili